<commit_message>
Stage 1 re-entry: correct F-001..F-010 from Stage 2 pass 002
BA task BA-001-04 (author subagent a5bb18013a4f4d2f8, PM-verified):
- analysis/stages/stage-01/stage-02-pass-002-dispositions.md: all ten
  findings accepted (F-002 and F-007 extended by sweeps, F-009 narrowed),
  with CHK-002/003/004 sweep row lists
- analysis/legacy_reconnaissance.md: sysadmin grant/revoke rule, social and
  import rows, GAP-001/003/007/009/011, Q3 facts, regenerated figures
- analysis/legacy_user_flows.xlsx: 193 -> 202 rows (Yes 111, Inferred 71,
  Partial 19, No 1), all static-only and open
- analysis/error-prevention-checklist.md: CHK-005 (form validation keys),
  CHK-006 (full delete data effect), CHK-007 (figures regenerated after
  correction) admitted by PM from confirmed findings
- analysis/migration_status.yaml: awaiting new Stage 2 pass 003

Not yet independently verified; the next fresh blind Stage 2 pass does that.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1349" uniqueCount="924">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1403" uniqueCount="960">
   <si>
     <t>Legacy Project - User Flows from Golden Code</t>
   </si>
@@ -22,7 +22,7 @@
     <t>Source columns contain legacy-code evidence. Destination columns compare the selected target implementation. SDD columns show whether missing or changed behavior is covered or explicitly deferred. Collapsed flow banners show audited completion as fully closed child rows divided by all child rows.</t>
   </si>
   <si>
-    <t>OVERALL DELIVERY PROGRESS  0.0%  (0 / 193 scenarios)</t>
+    <t>OVERALL DELIVERY PROGRESS  0.0%  (0 / 202 scenarios)</t>
   </si>
   <si>
     <t>Green</t>
@@ -202,16 +202,16 @@
     <t>class com.technoetic.xplanner.security.module.LoginSupportImpl#populateSubjectPrincipalFromDatabase (string "authentication.module.message.userNotFound"); class XPlannerLoginModule#isPasswordMatched (string "authentication.module.message.passwordNotSet"); ResourceBundle.properties same keys.</t>
   </si>
   <si>
-    <t>Submitting the login form with an empty user ID or password does not authenticate.</t>
-  </si>
-  <si>
-    <t>Avoids pointless authentication attempts.</t>
-  </si>
-  <si>
-    <t>Login page is shown again (notAuthenticated).</t>
-  </si>
-  <si>
-    <t>class AuthenticationAction#execute (StringUtils.isEmpty on "userId"/"password", forward "notAuthenticated"). Exact branch not decompiled.</t>
+    <t>A request to the login action without the submit field (for example a plain GET of /do/login) shows the login form; empty user ID or password values are not checked by the action and are passed to the login module, which rejects them.</t>
+  </si>
+  <si>
+    <t>The form is shown on first visit; blank credentials fail like wrong ones.</t>
+  </si>
+  <si>
+    <t>Login form (notAuthenticated) without an error on first visit; after submitting blank credentials: "Could not authenticate user." with a module message (for example "User has not been registered with XPlanner").</t>
+  </si>
+  <si>
+    <t>class AuthenticationAction#execute: the first branch tests StringUtils.isEmpty on the form field "action" (the submit button) and returns forward "notAuthenticated"; "userId" and "password" are then read and passed to Authenticator.authenticate without an emptiness check (bytecode listing, .migration-tmp/stage-01/tools/disasm.js); rejection messages per class LoginSupportImpl (authentication.module.message.userNotFound). Corrected in BA-001-04 (Source: stage-02-pass-002 F-005). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; authentication.module.message.userNotFound is defined only in the default, "--", de and ja bundles. Bundles without the key fall back to the default text (framework behavior, GAP-011).</t>
   </si>
   <si>
     <t>Remember me</t>
@@ -337,7 +337,7 @@
     <t>A sysadmin can do everything; an admin has editor and viewer rights plus admin*; an editor can create/edit/delete/integrate; a viewer can read.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/db-changelog.xml:363-386 (roles viewer lft1/rgt8, editor 2/7, admin 3/6, sysadmin 4/5) and :275-362 (permission rows); WAR:WEB-INF/classes/mappings/Metrics.xml queries "security.roles" and "security.role.permissions" (r1.left between r2.left and r2.right for positive permissions).</t>
+    <t>WAR:WEB-INF/classes/db-changelog.xml:363-386 (roles viewer lft1/rgt8, editor 2/7, admin 3/6, sysadmin 4/5) and :275-362 (permission rows); WAR:WEB-INF/classes/mappings/Metrics.xml queries "security.roles" and "security.role.permissions" (r1.left between r2.left and r2.right for positive permissions). Server-side enforcement (CHK-002, BA-001-04): the role model is evaluated on the server only on the paths in rows 28, 31, 160, 173, 210 and 222; everywhere else it only decides which links and fields the JSP pages show (rows 26, 29-30).</t>
   </si>
   <si>
     <t>Negative permissions apply to the exact role only: editors may not create projects, create people or delete iterations; admins may not create projects.</t>
@@ -346,10 +346,10 @@
     <t>Restricts structural changes to higher roles.</t>
   </si>
   <si>
-    <t>"Create project", "Add person" links and iteration delete buttons are hidden or refused for those roles.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/classes/db-changelog.xml permission ids 7, 8, 9, 19 (positive=false); WAR:WEB-INF/classes/mappings/Metrics.xml "security.role.permissions" (positive=0 and r1.id = r2.id). Evaluation order in class com.technoetic.xplanner.security.auth.AuthorizerImpl not decompiled.</t>
+    <t>"Create project" and "Add person" links and iteration delete buttons are hidden for those roles. Nothing refuses a direct request (rows 29-30).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/classes/db-changelog.xml permission ids 7, 8, 9, 19 (positive=false); WAR:WEB-INF/classes/mappings/Metrics.xml "security.role.permissions" (positive=0 and r1.id = r2.id). Evaluation order in class com.technoetic.xplanner.security.auth.AuthorizerImpl not decompiled. Server-side enforcement (CHK-002, BA-001-04): these restrictions only hide links and buttons; the create and delete handlers perform no server-side permission check (rows 29-30). Corrected in BA-001-04 (Source: stage-02-pass-002 F-007).</t>
   </si>
   <si>
     <t>A role assigned for project 0 applies to all projects (the seeded sysadmin is assigned this way).</t>
@@ -361,7 +361,7 @@
     <t>Seeded sysadmin sees and administers every project.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/db-changelog.xml:407-411 (person_role role 5, person 1, project 0); Metrics.xml "security.roles" (:includeWildcardProject = 1 and pr.id.projectId = 0).</t>
+    <t>WAR:WEB-INF/classes/db-changelog.xml:407-411 (person_role role 5, person 1, project 0); Metrics.xml "security.roles" (:includeWildcardProject = 1 and pr.id.projectId = 0). Server-side enforcement (CHK-002, BA-001-04): as for the role model, only the server-side paths in rows 28, 31, 160, 173, 210 and 222 evaluate it; project 0 is also the scope of the system-administrator rule in rows 31 and 34.</t>
   </si>
   <si>
     <t>Permission-driven UI actions</t>
@@ -376,7 +376,7 @@
     <t>Icons/links appear or disappear by permission (for example project delete requires sysadmin.delete, project edit admin.edit).</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.domain.DomainMetaDataRepository#init (action definitions with permissions "admin.edit", "sysadmin.delete", "edit", "delete"); WAR:WEB-INF/xplanner.tld (isUserAuthorized -&gt; com.technoetic.xplanner.tags.IsUserAuthorizedTag); e.g. WAR:WEB-INF/jsp/view/projects.jsp:82-100. Corrected in BA-001-03 (stage-02-pass-001 F-001): the gating is in JSP tags only.</t>
+    <t>class com.technoetic.xplanner.domain.DomainMetaDataRepository#init (action definitions with permissions "admin.edit", "sysadmin.delete", "edit", "delete"); WAR:WEB-INF/xplanner.tld (isUserAuthorized -&gt; com.technoetic.xplanner.tags.IsUserAuthorizedTag); e.g. WAR:WEB-INF/jsp/view/projects.jsp:82-100. Corrected in BA-001-03 (stage-02-pass-001 F-001): the gating is in JSP tags only. Server-side enforcement (CHK-002, BA-001-04): display-level only; the handlers behind these links perform no server-side permission check (rows 29-30), except the person-editor role rules (row 31).</t>
   </si>
   <si>
     <t>The projects list shows only projects the user may read.</t>
@@ -388,7 +388,7 @@
     <t>Projects without read permission are not listed.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/projects.jsp:32-48 (CollectionUtils.filter with SystemAuthorizer.hasPermission(..., "read")).</t>
+    <t>WAR:WEB-INF/jsp/view/projects.jsp:32-48 (CollectionUtils.filter with SystemAuthorizer.hasPermission(..., "read")). Server-side enforcement (CHK-002, BA-001-04): this filters the list rendered on the server, but the project pages themselves have no read check (row 29).</t>
   </si>
   <si>
     <t>Only views handled by DispatchForward with authorization required check permission (the flag defaults to true and is switched off for projects, people, settings, dashboard, twiki format and not-authorized): without a projectId parameter, or without read permission on system.project, they forward to security/notAuthorized, whose JSP is absent.</t>
@@ -427,16 +427,16 @@
     <t>.migration-tmp/stage-01/out/authtrace.json: 80 web action beans, 7 WAP actions, 43 SOAP operations, 4 REST methods, the iCal servlet and 3 Spring MVC handlers traced. For web actions, authorization calls are reachable only from DispatchForward, EditPersonAction (role changes), ViewAggregateTimesheetAction (result filter), InvalidateCacheAction (cache reset) and, not as a gate, inside e-mail recipient or metrics lookups (EditTaskAction, IntegrationAction, CommandExecutorAction, ViewIterationMetricsAction). Tracer limits: control flow and framework callbacks are not followed.</t>
   </si>
   <si>
-    <t>Server-side role changes in the person editor are applied only for projects on which the current user holds admin.edit.role; system-administrator promotion is offered only to sysadmin.promote holders.</t>
-  </si>
-  <si>
-    <t>The one web edit path with a real server-side permission check.</t>
-  </si>
-  <si>
-    <t>Role changes for other projects are ignored.</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.actions.EditPersonHelper#modifyRoles and #isCurrentUserAdminOfProject (Authorizer.hasPermission); class com.technoetic.xplanner.forms.PersonEditorForm calls the authorizer; path EditPersonAction#beforeObjectCommit in out/authtrace.json. The rest of the person edit (name, e-mail, password, hidden) is not permission-checked on the server.</t>
+    <t>Server-side role changes in the person editor are applied only for projects on which the current user holds admin.edit.role; in addition, when the current user holds admin.edit.role on project 0, every save of the person editor first removes the person's sysadmin role and re-adds it only if the form carries systemAdmin=true.</t>
+  </si>
+  <si>
+    <t>The one web edit path with a real server-side permission check; it also carries the system-administrator grant and revoke rule (row 34).</t>
+  </si>
+  <si>
+    <t>Role changes for other projects are ignored; the sysadmin role is revoked or granted by the project-0 rule (runtime unverified).</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.actions.EditPersonHelper#modifyRoles: for each submitted project role, #isCurrentUserAdminOfProject(projectId, user) (Authorizer.hasPermission with "system.project", "admin.edit.role") gates #setRoleOnProject; then #isCurrentUserAdminOfProject(0, user) gates RoleAssociationRepository.deleteForPersonOnProject("sysadmin", person, 0), followed by #setSysadmin only when the systemAdmin flag is true (bytecode listing); caller EditPersonAction#beforeObjectCommit passes PersonEditorForm#isSystemAdmin. class PersonEditorForm uses the authorizer only to preselect displayed roles (#getRoles, #isRoleSelected), not as a gate. The rest of the person edit (name, e-mail, password, hidden) is not permission-checked on the server. Corrected in BA-001-04 (Source: stage-02-pass-002 F-007). Server-side enforcement (CHK-002, BA-001-04): this row records the server-side check itself (Authorizer.hasPermission reached from EditPersonAction#beforeObjectCommit, .migration-tmp/stage-01/out/authtrace.json).</t>
   </si>
   <si>
     <t>URL role constraints in security.xml, mobile-security.xml and soap-security.xml are parsed but never evaluated; the security filters only check the bypass list and that the user is authenticated.</t>
@@ -463,19 +463,19 @@
     <t>Per-project radio buttons in the person editor; saved roles change what the person can see and do.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (isUserAuthorizedForAny projects permissions admin.edit.role; radio options none/viewer/editor/admin); WAR:WEB-INF/classes/spring-beans.xml:193-203 (editPersonHelper with invalidateCacheAfterPermissionChangedAdvisor on modifyRoles). Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
-  </si>
-  <si>
-    <t>Only a user with sysadmin.promote can grant or revoke system administrator status.</t>
-  </si>
-  <si>
-    <t>System administration is reserved to sysadmins.</t>
-  </si>
-  <si>
-    <t>Checkbox "System administrator" visible only to sysadmins.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (isUserAuthorized resourceType="system" permission="sysadmin.promote", input systemAdmin).</t>
+    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (isUserAuthorizedForAny projects permissions admin.edit.role; radio options none/viewer/editor/admin); WAR:WEB-INF/classes/spring-beans.xml:193-203 (editPersonHelper with invalidateCacheAfterPermissionChangedAdvisor on modifyRoles). Server-side enforcement (CHK-002, BA-001-04): enforced on the server per project by EditPersonHelper#isCurrentUserAdminOfProject (row 31); the editor page itself is reachable by any signed-in user (row 29). Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+  </si>
+  <si>
+    <t>The "System administrator" checkbox is shown only to sysadmin.promote holders, but on the server the sysadmin role is governed by admin.edit.role on project 0: when a user holding it saves any person editor, the person's sysadmin role is removed and re-added only if systemAdmin=true is posted.</t>
+  </si>
+  <si>
+    <t>System-administrator status can be granted by a direct request and is silently revoked when a project-0 administrator without the checkbox saves the person. Observed behavior and risk only (Q3 deferred; not permission to carry it into the new application).</t>
+  </si>
+  <si>
+    <t>Checkbox visible only to sysadmins; saving the person editor as a project-0 administrator without the checkbox revokes the person's system-administrator role; posting systemAdmin=true grants it (runtime unverified).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp:144-151 (isUserAuthorized resourceType="system" permission="sysadmin.promote", input systemAdmin); class EditPersonHelper#modifyRoles, #isCurrentUserAdminOfProject, #setSysadmin (bytecode listing: deleteForPersonOnProject("sysadmin", personId, 0) then setSysadmin when the flag is true); class EditPersonAction#beforeObjectCommit (PersonEditorForm#isSystemAdmin). Who holds admin.edit.role on project 0 follows the role model (rows 23-25; sysadmin via "%", admin via "admin%" when assigned on project 0), Inferred. Corrected in BA-001-04 (Source: stage-02-pass-002 F-007). Server-side enforcement (CHK-002, BA-001-04): sysadmin.promote is display-level only; the server-side check that governs the sysadmin role is admin.edit.role on project 0 (row 31).</t>
   </si>
   <si>
     <t>Edit project roles (project role editor)</t>
@@ -490,7 +490,7 @@
     <t>Form posted to /do/edit/roles; the role-saving code is expected never to run, so submitted roles are not saved (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:409-411; WAR:WEB-INF/action-servlet.xml:400-404 (EditRoleAction); WAR:WEB-INF/jsp/edit/editRoles.jsp; class com.technoetic.xplanner.actions.EditRoleAction (strings "admin.edit.role", HQL on PersonRole). No live link to this page was found (mechanical link scan .migration-tmp/stage-01/out/linkgraph.txt); reachable only by URL. BA-001-03 impact sweep: EditRoleAction#beforeObjectCommit(Object, Session, ActionMapping, ActionForm, HttpServletRequest, HttpServletResponse) overrides no superclass hook (AbstractAction#beforeObjectCommit takes Identifiable, ActionMapping, ActionForm, request, response) and has no caller, so its role update and its admin.edit.role check are unreachable; an orphan-hook scan over all action classes found only this method.</t>
+    <t>WAR:WEB-INF/struts-config.xml:409-411; WAR:WEB-INF/action-servlet.xml:400-404 (EditRoleAction); WAR:WEB-INF/jsp/edit/editRoles.jsp; class com.technoetic.xplanner.actions.EditRoleAction (strings "admin.edit.role", HQL on PersonRole). No live link to this page was found (mechanical link scan .migration-tmp/stage-01/out/linkgraph.txt); reachable only by URL. BA-001-03 impact sweep: EditRoleAction#beforeObjectCommit(Object, Session, ActionMapping, ActionForm, HttpServletRequest, HttpServletResponse) overrides no superclass hook (AbstractAction#beforeObjectCommit takes Identifiable, ActionMapping, ActionForm, request, response) and has no caller, so its role update and its admin.edit.role check are unreachable; an orphan-hook scan over all action classes found only this method. Server-side enforcement (CHK-002, BA-001-04): no server-side check is reached, because the only check sits in the unreachable EditRoleAction#beforeObjectCommit (above); the page is reachable by any signed-in user.</t>
   </si>
   <si>
     <t>UF-003</t>
@@ -523,7 +523,7 @@
     <t>Admins see hidden people; others do not.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/people.jsp (isUserAuthorized permission="admin.hide" resourceType="system.person"; useBeans where hidden = false).</t>
+    <t>WAR:WEB-INF/jsp/view/people.jsp (isUserAuthorized permission="admin.hide" resourceType="system.person"; useBeans where hidden = false). Server-side enforcement (CHK-002, BA-001-04): the filter is applied while the server renders people.jsp; /do/view/people is a DispatchForward with authorization switched off (row 28), and the page of a hidden person remains reachable by oid (ViewPersonAction has no permission check, row 29).</t>
   </si>
   <si>
     <t>With a projectId parameter the list is restricted to people with a role on that project and titled with the project name.</t>
@@ -562,7 +562,7 @@
     <t>Clock and edit icons per active task when the user may edit it.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/personTaskTableFragment.jsp (isUserAuthorized task edit; links /do/edit/time and /do/edit/task).</t>
+    <t>WAR:WEB-INF/jsp/view/personTaskTableFragment.jsp (isUserAuthorized task edit; links /do/edit/time and /do/edit/task). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); UpdateTimeAction or EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>The edit link on a person page is shown only to that person or to someone with admin.edit on system.person for some project.</t>
@@ -574,7 +574,7 @@
     <t>Edit link visible accordingly; links to people list, timesheet and exports.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/person.jsp (remoteUserId == person.getId() || hasPermissionForSomeProject(..., "admin.edit")).</t>
+    <t>WAR:WEB-INF/jsp/view/person.jsp (remoteUserId == person.getId() || hasPermissionForSomeProject(..., "admin.edit")). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction (except the role rules in row 31) performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>Create person</t>
@@ -589,7 +589,7 @@
     <t>Person saved; user returned to the people list (returnto).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/people.jsp (link /do/edit/person under create.person); WAR:WEB-INF/struts-config.xml:321-326; WAR:WEB-INF/jsp/edit/editPerson.jsp; class com.technoetic.xplanner.actions.EditPersonAction.</t>
+    <t>WAR:WEB-INF/jsp/view/people.jsp (link /do/edit/person under create.person); WAR:WEB-INF/struts-config.xml:321-326; WAR:WEB-INF/jsp/edit/editPerson.jsp; class com.technoetic.xplanner.actions.EditPersonAction. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>Name, user ID, e-mail and initials are mandatory; password and confirmation must match.</t>
@@ -628,7 +628,7 @@
     <t>Changes saved; returnto page shown.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (form /do/edit/person, Update button); WAR:WEB-INF/security.xml:15 (/do/edit/person in viewing constraint).</t>
+    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (form /do/edit/person, Update button); WAR:WEB-INF/security.xml:15 (/do/edit/person in viewing constraint). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction (except the role rules in row 31) performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>The password fields are shown only when the active login module can change passwords; a new password is stored as a salted digest.</t>
@@ -652,22 +652,22 @@
     <t>Hidden select Yes/No; hidden people disappear from normal lists.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (isUserAuthorized person hide; select hidden).</t>
+    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (isUserAuthorized person hide; select hidden). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>Delete person</t>
   </si>
   <si>
-    <t>A person can be deleted through /do/delete/person.</t>
+    <t>A person can be deleted through /do/delete/person; nothing cascades. If the person is a story customer or a notification receiver, the database foreign keys are expected to reject the delete; task acceptor, story tracker, time-entry person and person-role references are plain columns and are left dangling.</t>
   </si>
   <si>
     <t>Removes a person record.</t>
   </si>
   <si>
-    <t>Person removed; returnto or projects page shown.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/struts-config.xml:348; WAR:WEB-INF/action-servlet.xml:370-374 (DeleteObjectAction type Person). The person action metadata defines only "edit" (DomainMetaDataRepository#init) and no live link to /do/delete/person was found (linkgraph.txt).</t>
+    <t>Person removed, or a database error when foreign keys refer to the person (runtime unverified).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/struts-config.xml:348; WAR:WEB-INF/action-servlet.xml:370-374 (DeleteObjectAction type Person). The person action metadata defines only "edit" (DomainMetaDataRepository#init) and no live link to /do/delete/person was found (linkgraph.txt). BA-001-04 cascade sweep: net.sf.xplanner.domain.Person has no relationship annotations; WAR:WEB-INF/classes/db-changelog.xml:260 (notification_receivers.person_id -&gt; person) and :262 (story.customer_id -&gt; person) are the only foreign keys to person. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>Import people from a file</t>
@@ -682,7 +682,7 @@
     <t>Results table with line number, assigned ID, login ID, name and status "Success".</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/people.jsp (link /do/import/people); WAR:WEB-INF/struts-config.xml:329-330; WAR:WEB-INF/jsp/edit/importPeople.jsp; class com.technoetic.xplanner.actions.ImportPeopleAction (BufferedReader.readLine, String.split ",", PersonDao.save); ResourceBundle.properties people.import.editor.importFileFormat.</t>
+    <t>WAR:WEB-INF/jsp/view/people.jsp (link /do/import/people); WAR:WEB-INF/struts-config.xml:329-330; WAR:WEB-INF/jsp/edit/importPeople.jsp; class com.technoetic.xplanner.actions.ImportPeopleAction (BufferedReader.readLine, String.split ",", PersonDao.save); ResourceBundle.properties people.import.editor.importFileFormat. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); ImportPeopleAction (its AuthorizationException handler is unreachable because nothing on its path raises one) performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>Malformed lines, empty user IDs and existing user IDs are reported per line and not imported.</t>
@@ -784,7 +784,7 @@
     <t>Page headed "Settings" with a table; the add/edit editor JSP is missing.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:405,419-421; WAR:WEB-INF/jsp/view/settings.jsp (prints ${settings} raw; reuses projects.title); input WEB-INF/jsp/edit/editSetting.jsp ABSENT from WAR (GAP-003); db-changelog.xml changeSet 2-1 (setting, object_type). No live link to /do/view/settings found.</t>
+    <t>WAR:WEB-INF/struts-config.xml:405,419-421; WAR:WEB-INF/jsp/view/settings.jsp (prints ${settings} raw; reuses projects.title); input WEB-INF/jsp/edit/editSetting.jsp ABSENT from WAR (GAP-003); db-changelog.xml changeSet 2-1 (setting, object_type). No live link to /do/view/settings found. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditObjectAction for Setting performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>Generic Spring MVC handlers exist for /setting/{objectType}/list and /setting/{objectType}/edit/{objectId}.</t>
@@ -811,7 +811,7 @@
     <t>Plain confirmation "cache cleared" / "hibernate cache cleared".</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:233 (test-struts-config.xml loaded); WAR:WEB-INF/test-struts-config.xml:21-23; WAR:WEB-INF/test-action-servlet.xml:22-36; WAR:WEB-INF/security.xml:5 (bypass /do/invalidateHibernateCache); input JSP WEB-INF/jsp/admin/invalidateCache.jsp ABSENT.</t>
+    <t>WAR:WEB-INF/web.xml:233 (test-struts-config.xml loaded); WAR:WEB-INF/test-struts-config.xml:21-23; WAR:WEB-INF/test-action-servlet.xml:22-36; WAR:WEB-INF/security.xml:5 (bypass /do/invalidateHibernateCache); input JSP WEB-INF/jsp/admin/invalidateCache.jsp ABSENT. Server-side enforcement (CHK-002, BA-001-04): neither action checks a permission; InvalidateCacheAction obtains the authorizer only to reset its cache.</t>
   </si>
   <si>
     <t>Test-support URLs can execute data sampling, the missing-time-entry notifier, shift the application clock (dayOffset) and set a property value.</t>
@@ -964,16 +964,16 @@
     <t>WAR:WEB-INF/struts-config.xml:179; WAR:WEB-INF/action-servlet.xml:29-31 (DispatchForward, authorizationRequired=false); WAR:WEB-INF/jsp/view/projects.jsp:32-167 (useBeans order "is_hidden,name asc"; iterations where "? between startDate and endDate").</t>
   </si>
   <si>
-    <t>Users who may hide projects see an extra "hidden" column with yes/no; hidden projects are styled differently.</t>
+    <t>Users who may hide projects see an extra "hidden" column with yes/no; hidden projects are sorted after visible ones but are not styled differently.</t>
   </si>
   <si>
     <t>Admins can spot retired projects.</t>
   </si>
   <si>
-    <t>Hidden column visible only with hide permission.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/projects.jsp:137-142 (isUserAuthorizedForAny permissions="hide"); HiddenRowDecorator :65-74.</t>
+    <t>Hidden column visible only with hide permission; hidden projects listed last.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/projects.jsp:137-142 (isUserAuthorizedForAny permissions="hide") and :33 (order "is_hidden,name asc"). The class HiddenRowDecorator declared at :65-75 is never passed to the table: the writableTable at :82-84 has no rowDecorator attribute, and the name occurs only at :66 (CHK-003). Corrected in BA-001-04 (Source: stage-02-pass-002 F-006). Server-side enforcement (CHK-002, BA-001-04): the column is display-level only; hiding a project goes through EditProjectAction, which performs no server-side permission check (rows 29-30).</t>
   </si>
   <si>
     <t>When no readable project exists the page shows a "no projects" message.</t>
@@ -1000,7 +1000,7 @@
     <t>Project saved; user returned to the projects list.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/projects.jsp:153-158 (link /do/edit/project under create.project); WAR:WEB-INF/struts-config.xml:195; WAR:WEB-INF/action-servlet.xml:72-76 (EditProjectAction); WAR:WEB-INF/jsp/edit/editProject.jsp:42-112.</t>
+    <t>WAR:WEB-INF/jsp/view/projects.jsp:153-158 (link /do/edit/project under create.project); WAR:WEB-INF/struts-config.xml:195; WAR:WEB-INF/action-servlet.xml:72-76 (EditProjectAction); WAR:WEB-INF/jsp/edit/editProject.jsp:42-112. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditProjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>A project without a name is rejected.</t>
@@ -1039,22 +1039,22 @@
     <t>Editor titled "Edit project: &lt;name&gt;" with Update/Reset; changes saved.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:28-34,76-80,104-106; class DomainMetaDataRepository#init (project edit -&gt; /do/edit/project, permission admin.edit).</t>
+    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:28-34,76-80,104-106; class DomainMetaDataRepository#init (project edit -&gt; /do/edit/project, permission admin.edit). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditProjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>Delete project</t>
   </si>
   <si>
-    <t>A sysadmin can delete a project after a confirmation prompt.</t>
+    <t>A sysadmin can delete a project after a confirmation prompt; the delete cascades through the mappings to the project's iterations (including the backlog iteration), their stories, the stories' tasks and the tasks' time entries. Notes attached to any of these objects, their attachment files, history rows and person-role rows are not deleted.</t>
   </si>
   <si>
     <t>Remove obsolete projects.</t>
   </si>
   <si>
-    <t>Browser confirm "Do you want to delete project '&lt;name&gt;'?"; project removed; projects list shown.</t>
-  </si>
-  <si>
-    <t>class DomainMetaDataRepository#init (delete -&gt; /do/delete/project, permission sysadmin.delete, onclick action.delete.confirmation); WAR:WEB-INF/struts-config.xml:197; WAR:WEB-INF/action-servlet.xml:78-82 (DeleteObjectAction).</t>
+    <t>Browser confirm "Do you want to delete project '&lt;name&gt;'?"; the project and its iterations, stories, tasks and time entries removed; orphan notes remain (runtime unverified).</t>
+  </si>
+  <si>
+    <t>class DomainMetaDataRepository#init (delete -&gt; /do/delete/project, permission sysadmin.delete, onclick action.delete.confirmation); WAR:WEB-INF/struts-config.xml:197; WAR:WEB-INF/action-servlet.xml:78-82 (DeleteObjectAction#doExecute: CommonDao.delete). Cascades (CHK-003): net.sf.xplanner.domain.Project#getIterations @OneToMany(cascade=ALL), #getBacklog @OneToOne(cascade=REMOVE), Iteration#getUserStories, UserStory#getTasks, Task#getTimeEntries @OneToMany(cascade=REMOVE); The notification-receiver links (Project#getNotificationReceivers @ManyToMany, join table notification_receivers) and the project attributes (@ElementCollection, table attribute) are removed with the project row. Note refers to objects by attachedToId without a mapping; NoteHelper#deleteNotesFor is called from HibernateObjectRepository#delete, which the web delete path (DeleteObjectAction#doExecute -&gt; CommonDao.delete) does not reach. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002).</t>
   </si>
   <si>
     <t>View project</t>
@@ -1093,7 +1093,7 @@
     <t>Person selected and "Add" pressed; the person appears in the receivers list.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:115-158 (select personToAddId, action addTimeNotification); class EditProjectAction#doExecute (forward /do/edit/project/notification); WAR:WEB-INF/struts-config.xml:368-372; class com.technoetic.xplanner.actions.UpdateTimeNotificationReceivers#doAction; db-changelog.xml table notification_receivers.</t>
+    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:115-158 (select personToAddId, action addTimeNotification); class EditProjectAction#doExecute (forward /do/edit/project/notification); WAR:WEB-INF/struts-config.xml:368-372; class com.technoetic.xplanner.actions.UpdateTimeNotificationReceivers#doAction; db-changelog.xml table notification_receivers. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); UpdateTimeNotificationReceivers performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>A receiver can be removed with the delete icon.</t>
@@ -1126,19 +1126,19 @@
     <t>Iteration saved under the project; user returned.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/project.jsp:87-90 (link /do/edit/iteration); WAR:WEB-INF/struts-config.xml:241-243; WAR:WEB-INF/action-servlet.xml:177-181 (EditIterationAction); WAR:WEB-INF/jsp/edit/editIteration.jsp; class EditIterationAction#beforeObjectCommit (strings "Create", Project).</t>
-  </si>
-  <si>
-    <t>Missing name or unparsable dates are rejected.</t>
-  </si>
-  <si>
-    <t>Iterations need a name and valid dates.</t>
-  </si>
-  <si>
-    <t>Messages "Missing iteration name.", "Start date is invalid.", "End date is invalid."</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.forms.IterationEditorForm#validate (strings iteration.editor.missing_name, bad_start_date, bad_end_date).</t>
+    <t>WAR:WEB-INF/jsp/view/project.jsp:87-90 (link /do/edit/iteration); WAR:WEB-INF/struts-config.xml:241-243; WAR:WEB-INF/action-servlet.xml:177-181 (EditIterationAction); WAR:WEB-INF/jsp/edit/editIteration.jsp; class EditIterationAction#beforeObjectCommit (strings "Create", Project). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+  </si>
+  <si>
+    <t>Missing name, unparsable dates, or an end date that does not follow the start date are rejected.</t>
+  </si>
+  <si>
+    <t>Iterations need a name and a valid positive date interval.</t>
+  </si>
+  <si>
+    <t>Messages "Missing iteration name.", "Start date is invalid.", "End date is invalid.", "Iteration must be a positive time interval."</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.IterationEditorForm#validate (strings iteration.editor.missing_name, bad_start_date, bad_end_date) and #requirePositiveInterval (iteration.editor.nonpositive_interval); WAR:WEB-INF/classes/ResourceBundle.properties:265. Corrected in BA-001-04 (Source: stage-02-pass-002 F-001). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; iteration.editor.nonpositive_interval: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 66-68).</t>
   </si>
   <si>
     <t>Edit iteration</t>
@@ -1153,22 +1153,22 @@
     <t>Editor with Update/Reset; changes saved.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editIteration.jsp (logic:present oid: status display, daysWorked input); class DomainMetaDataRepository#init (iteration edit, permission edit).</t>
+    <t>WAR:WEB-INF/jsp/edit/editIteration.jsp (logic:present oid: status display, daysWorked input); class DomainMetaDataRepository#init (iteration edit, permission edit). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>Delete iteration</t>
   </si>
   <si>
-    <t>A user with delete permission on the iteration (not editors, per seeded permissions) can delete it after confirmation.</t>
+    <t>An iteration can be deleted after confirmation; the delete link is shown to users with delete permission on the iteration (not editors, per seeded permissions), and the delete cascades to the iteration's stories, their tasks and the tasks' time entries. Attached notes and history rows are not deleted.</t>
   </si>
   <si>
     <t>Remove mistaken iterations.</t>
   </si>
   <si>
-    <t>Confirm prompt; iteration removed.</t>
-  </si>
-  <si>
-    <t>class DomainMetaDataRepository#init (iteration delete, onclick action.delete.confirmation); WAR:WEB-INF/struts-config.xml:257; WAR:WEB-INF/action-servlet.xml:196-200; db-changelog.xml permission id 19 (editor, delete, system.project.iteration, positive=false).</t>
+    <t>Confirm prompt; iteration, stories, tasks and time entries removed (runtime unverified).</t>
+  </si>
+  <si>
+    <t>class DomainMetaDataRepository#init (iteration delete, onclick action.delete.confirmation); WAR:WEB-INF/struts-config.xml:257; WAR:WEB-INF/action-servlet.xml:196-200; db-changelog.xml permission id 19 (editor, delete, system.project.iteration, positive=false). Cascades: Iteration#getUserStories, UserStory#getTasks, Task#getTimeEntries @OneToMany(cascade=REMOVE). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002, F-007).</t>
   </si>
   <si>
     <t>View iteration stories</t>
@@ -1219,7 +1219,7 @@
     <t>After "save order" the page reloads with stories in the new order.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/iteration.jsp:33-36,79-89,160-162 (form /do/edit/reorderstories, orderNo inputs); WAR:WEB-INF/struts-config.xml:357-362; class com.technoetic.xplanner.actions.ReorderStoriesAction.</t>
+    <t>WAR:WEB-INF/jsp/view/iteration.jsp:33-36,79-89,160-162 (form /do/edit/reorderstories, orderNo inputs); WAR:WEB-INF/struts-config.xml:357-362; class com.technoetic.xplanner.actions.ReorderStoriesAction. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); ReorderStoriesAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>A non-numeric order number is rejected.</t>
@@ -1246,22 +1246,22 @@
     <t>Move page with target iteration select; selected stories moved; redirect to /do/view/iteration?oid=&lt;source&gt;.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/iteration.jsp:38-40,60-64 (selected[] checkboxes, submitMoveMultiple); WAR:WEB-INF/struts-config.xml:364-366; WAR:WEB-INF/jsp/edit/moveStories.jsp; class com.technoetic.xplanner.actions.MoveStoriesAction (string "/do/view/iteration?oid=").</t>
+    <t>WAR:WEB-INF/jsp/view/iteration.jsp:38-40,60-64 (selected[] checkboxes, submitMoveMultiple); WAR:WEB-INF/struts-config.xml:364-366; WAR:WEB-INF/jsp/edit/moveStories.jsp; class com.technoetic.xplanner.actions.MoveStoriesAction (string "/do/view/iteration?oid="). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); MoveStoriesAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>Start iteration</t>
   </si>
   <si>
-    <t>An editor can start an iteration; the confirmation page explains that starting baselines current task estimates.</t>
+    <t>An editor can start an iteration; the confirmation page asks "Do you want to start the iteration?" (the explanation that starting baselines current task estimates is shown only when arriving from time entry, row 97).</t>
   </si>
   <si>
     <t>Freeze the plan for velocity measurement.</t>
   </si>
   <si>
-    <t>Page "Start Iteration: &lt;name&gt;" with OK/Cancel; iteration becomes active; data sample taken.</t>
-  </si>
-  <si>
-    <t>class DomainMetaDataRepository#init (start -&gt; start/iteration, permission edit); WAR:WEB-INF/struts-config.xml:245-248; WAR:WEB-INF/jsp/edit/editIterationStatus.jsp; class StartIterationAction#beforeObjectCommit ("started"); references DataSampler (class StartIterationAction).</t>
+    <t>Page "Start Iteration: &lt;name&gt;" with "Do you want to start the iteration?" and OK/Cancel; iteration becomes active; opening data samples taken.</t>
+  </si>
+  <si>
+    <t>class DomainMetaDataRepository#init (start -&gt; start/iteration, permission edit); WAR:WEB-INF/struts-config.xml:245-248; WAR:WEB-INF/jsp/edit/editIterationStatus.jsp:43-47 (message_1 only when UpdateTimeAction.isFromUpdateTime) and :58-60 (message_4); WAR:WEB-INF/classes/ResourceBundle.properties:272,275; class StartIterationAction#beforeObjectCommit ("started", DataSampler.generateOpeningDataSamples). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); StartIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-005). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; iteration.status.editor.message_4 is defined only in the default and "--" bundles. Bundles without the key fall back to the default text (framework behavior, GAP-011).</t>
   </si>
   <si>
     <t>If other iterations are still started, the page proposes closing them (checked by default).</t>
@@ -1300,7 +1300,7 @@
     <t>Iteration set inactive; data sample taken; redirect to the continue-unfinished-stories page.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (close -&gt; close/iteration); WAR:WEB-INF/struts-config.xml:251-255 (forward onclose -&gt; /do/continue/unfinished/stories); class CloseIterationAction ("closed", "onclose").</t>
+    <t>class DomainMetaDataRepository#init (close -&gt; close/iteration); WAR:WEB-INF/struts-config.xml:251-255 (forward onclose -&gt; /do/continue/unfinished/stories); class CloseIterationAction ("closed", "onclose"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); CloseIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>On the continue page the user selects a future iteration and confirms; unfinished stories are continued there.</t>
@@ -1477,7 +1477,7 @@
     <t>Result "Imported &lt;n&gt; stories"; stories created.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (importStories -&gt; import/stories); WAR:WEB-INF/struts-config.xml:332-346; WAR:WEB-INF/action-servlet.xml:361-368 (ImportStoriesAction, SpreadsheetStoryImporter); WAR:WEB-INF/jsp/import/stories.jsp; xplanner.properties:277-284 (default headers). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>class DomainMetaDataRepository#init (importStories -&gt; import/stories); WAR:WEB-INF/struts-config.xml:332-346; WAR:WEB-INF/action-servlet.xml:361-368 (ImportStoriesAction, SpreadsheetStoryImporter); WAR:WEB-INF/jsp/import/stories.jsp; xplanner.properties:277-284 (default headers). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); ImportStoriesAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
   </si>
   <si>
     <t>Missing required inputs are rejected before import.</t>
@@ -1501,7 +1501,7 @@
     <t>Messages "Could not find worksheet named ...", "Could not find a column with ... as the header...", "Some stories did not have ... specified.", "...appears to be corrupt."</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:334-345 (exception mappings); classes WrongImportFileSpreadsheetImporterException, MissingFieldSpreadsheetImporterException, MissingColumnHeaderSpreadsheetImporterException exist; com.technoetic.xplanner.importer.MissingWorksheetException is ABSENT from the WAR (worksheet-not-found mapping cannot match).</t>
+    <t>class com.technoetic.xplanner.actions.ImportStoriesAction#execute: exception handlers (bytecode exception table) catch importer.WrongImportFileSpreadsheetImporterException, MissingFieldSpreadsheetImporterException, MissingColumnHeaderSpreadsheetImporterException and importer.spreadsheet.MissingWorksheetException and save import.status.corrupted_file, missing_required_field, wrong_header and worksheet_not_found. The Struts mapping for the non-existent com.technoetic.xplanner.importer.MissingWorksheetException (WAR:WEB-INF/struts-config.xml:343-345) is therefore redundant, not a defect of the behavior. Corrected in BA-001-04 (Source: stage-02-pass-002 F-008).</t>
   </si>
   <si>
     <t>Optionally only incomplete stories are imported (skip rows whose status equals the completed status, default "C").</t>
@@ -1516,6 +1516,18 @@
     <t>WAR:WEB-INF/jsp/import/stories.jsp (onlyIncomplete, completedStatus); xplanner.properties:284 (import.spreadsheet.completedStoryStatus=C); class SpreadsheetStoryImporter. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
   </si>
   <si>
+    <t>After an import the worksheet name, column headers, only-incomplete choice and completed status are saved in browser cookies, and the next import form is pre-filled from those cookies before the property defaults.</t>
+  </si>
+  <si>
+    <t>The import settings are remembered per browser.</t>
+  </si>
+  <si>
+    <t>Import form pre-filled with the last used settings.</t>
+  </si>
+  <si>
+    <t>class ImportStoriesAction#setCookies (cookie names import.spreadsheet.worksheet.name, .story.title.column.header, .iteration.end.date.column.header, .story.estimate.column.header, .story.priority.column.header, .story.status.column.header, .onlyIncomplete, .completedStoryStatus), called from EditObjectAction#doExecute after #saveForm; #populateForm with #getValueFromCookieOrProperties (defaults WAR:WEB-INF/classes/xplanner.properties:278-284; provenance of these default values as in row 111, GAP-005 P-03). Source: stage-02-pass-002 F-008.</t>
+  </si>
+  <si>
     <t>UF-007</t>
   </si>
   <si>
@@ -1534,7 +1546,7 @@
     <t>Story saved in the iteration; user returned to the iteration page.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (createStory -&gt; edit/userstory); WAR:WEB-INF/struts-config.xml:269-271; WAR:WEB-INF/action-servlet.xml:220-224 (EditStoryAction); WAR:WEB-INF/jsp/edit/editStory.jsp; classes com.technoetic.xplanner.domain.StoryStatus, StoryDisposition (enumeration strings).</t>
+    <t>class DomainMetaDataRepository#init (createStory -&gt; edit/userstory); WAR:WEB-INF/struts-config.xml:269-271; WAR:WEB-INF/action-servlet.xml:220-224 (EditStoryAction); WAR:WEB-INF/jsp/edit/editStory.jsp; classes com.technoetic.xplanner.domain.StoryStatus, StoryDisposition (enumeration strings). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>A new story defaults to priority 4.</t>
@@ -1573,22 +1585,22 @@
     <t>Editor titled for the story with Update/Reset; changes saved.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (story edit -&gt; /do/edit/userstory, permission edit); WAR:WEB-INF/jsp/edit/editStory.jsp.</t>
+    <t>class DomainMetaDataRepository#init (story edit -&gt; /do/edit/userstory, permission edit); WAR:WEB-INF/jsp/edit/editStory.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>Delete user story</t>
   </si>
   <si>
-    <t>A user with delete permission can delete a story after confirmation.</t>
+    <t>A story can be deleted after confirmation; the delete link is shown to users with delete permission, and the delete cascades to the story's tasks and their time entries. Attached notes and history rows are not deleted.</t>
   </si>
   <si>
     <t>Remove obsolete stories.</t>
   </si>
   <si>
-    <t>Confirm prompt; story removed.</t>
-  </si>
-  <si>
-    <t>class DomainMetaDataRepository#init (story delete -&gt; /do/delete/userstory, action.delete.confirmation); WAR:WEB-INF/struts-config.xml:285; WAR:WEB-INF/action-servlet.xml:256-260.</t>
+    <t>Confirm prompt; story, tasks and time entries removed (runtime unverified).</t>
+  </si>
+  <si>
+    <t>class DomainMetaDataRepository#init (story delete -&gt; /do/delete/userstory, action.delete.confirmation); WAR:WEB-INF/struts-config.xml:285; WAR:WEB-INF/action-servlet.xml:256-260. Cascades: UserStory#getTasks, Task#getTimeEntries @OneToMany(cascade=REMOVE). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002).</t>
   </si>
   <si>
     <t>View user story</t>
@@ -1627,7 +1639,7 @@
     <t>Move/Continue page with target iteration; story moved.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (movecontinue -&gt; /do/move/continue/userstory); WAR:WEB-INF/struts-config.xml:273-275; WAR:WEB-INF/jsp/edit/moveContinueStory.jsp; class MoveContinueStoryAction#saveForm ("Move").</t>
+    <t>class DomainMetaDataRepository#init (movecontinue -&gt; /do/move/continue/userstory); WAR:WEB-INF/struts-config.xml:273-275; WAR:WEB-INF/jsp/edit/moveContinueStory.jsp; class MoveContinueStoryAction#saveForm ("Move"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); MoveContinueStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>Continue creates a continuation of the story in the target iteration for the unfinished work, with cross-references in the descriptions.</t>
@@ -1672,19 +1684,19 @@
     <t>Task saved; user returned to the story.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/userstory.jsp (link /do/edit/task, story.link.create_task); WAR:WEB-INF/struts-config.xml:291; WAR:WEB-INF/action-servlet.xml:268-272 (EditTaskAction); WAR:WEB-INF/jsp/edit/editTask.jsp.</t>
-  </si>
-  <si>
-    <t>The task type is stored as the displayed (localized) label, e.g. "Feature", "Defect", "Overhead"; the German bundle uses different labels for some types.</t>
-  </si>
-  <si>
-    <t>Explains why type values depend on the UI language used when the task was saved.</t>
-  </si>
-  <si>
-    <t>Type select options carry label text as their values.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/edit/editTask.jsp (html:option value=messages.getMessage("task.type.feature") ... "task.type.overhead"); WAR:WEB-INF/classes/ResourceBundle.properties task.type.* vs ResourceBundle_de.properties (Fehler, Rückstand); class iCalServlet#generateTaskData filters task.type &lt;&gt; label of task.type.overhead.</t>
+    <t>WAR:WEB-INF/jsp/view/userstory.jsp (link /do/edit/task, story.link.create_task); WAR:WEB-INF/struts-config.xml:291; WAR:WEB-INF/action-servlet.xml:268-272 (EditTaskAction); WAR:WEB-INF/jsp/edit/editTask.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+  </si>
+  <si>
+    <t>The task type is stored as a message label, not a code: the type options carry label text as their values, resolved without the user's locale, so the stored value follows the server default locale. The labels differ between bundles.</t>
+  </si>
+  <si>
+    <t>Explains why stored type values are language text and differ between installations with a different server locale.</t>
+  </si>
+  <si>
+    <t>Type select shows the user's language; the stored value is the server-default-locale label (runtime unverified).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/edit/editTask.jsp:52-69 (html:option value=messages.getMessage("task.type.feature") ... "task.type.overhead", no locale argument); class net.sf.xplanner.struts.XPlannerMessageResources#getMessage delegates to the Spring MessageSource (null locale falls back to the JVM default, framework behavior, GAP-011). Per bundle (CHK-004, .migration-tmp/stage-01/out/task-type-labels.json): the default and "--" bundles use Feature, Defect, Debt, FTest, ATest, Overhead; da, de, es, fr, it, ja and ru differ from the default for at least one type; pt_br matches except that it has no overhead key; da, es, fr and pt_br define no task.type.overhead (fallback to the default). Corrected in BA-001-04 (Source: stage-02-pass-002 F-009).</t>
   </si>
   <si>
     <t>The default disposition of a new task depends on the story/iteration state.</t>
@@ -1735,7 +1747,7 @@
     <t>Task editor with Update/Reset; changes saved.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (task edit -&gt; /do/edit/task); WAR:WEB-INF/jsp/edit/editTask.jsp.</t>
+    <t>class DomainMetaDataRepository#init (task edit -&gt; /do/edit/task); WAR:WEB-INF/jsp/edit/editTask.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>Complete or reopen task</t>
@@ -1750,7 +1762,7 @@
     <t>"Complete" button; task becomes completed; page reloads.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/task.jsp:86-95 (form /do/edit/task, action Update, merge true, completed true).</t>
+    <t>WAR:WEB-INF/jsp/view/task.jsp:86-95 (form /do/edit/task, action Update, merge true, completed true). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>A completed task can be reopened.</t>
@@ -1762,22 +1774,22 @@
     <t>"Reopen" button; task becomes open again.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/task.jsp:75-84 (completed false).</t>
+    <t>WAR:WEB-INF/jsp/view/task.jsp:75-84 (completed false). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>Delete task</t>
   </si>
   <si>
-    <t>A user with delete permission can delete a task after confirmation.</t>
+    <t>A task can be deleted after confirmation; the delete link is shown to users with delete permission, and the delete cascades to the task's time entries. Attached notes and history rows are not deleted.</t>
   </si>
   <si>
     <t>Remove obsolete tasks.</t>
   </si>
   <si>
-    <t>Confirm prompt; task removed.</t>
-  </si>
-  <si>
-    <t>class DomainMetaDataRepository#init (task delete -&gt; /do/delete/task, action.delete.confirmation); WAR:WEB-INF/struts-config.xml:304; WAR:WEB-INF/action-servlet.xml:300-304.</t>
+    <t>Confirm prompt; task and its time entries removed (runtime unverified).</t>
+  </si>
+  <si>
+    <t>class DomainMetaDataRepository#init (task delete -&gt; /do/delete/task, action.delete.confirmation); WAR:WEB-INF/struts-config.xml:304; WAR:WEB-INF/action-servlet.xml:300-304. Cascade: Task#getTimeEntries @OneToMany(cascade=REMOVE). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002).</t>
   </si>
   <si>
     <t>View task</t>
@@ -1807,7 +1819,7 @@
     <t>Move/Continue page with target story; history records "moved".</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (task movecontinue -&gt; /do/move/continue/task); WAR:WEB-INF/struts-config.xml:293-295; WAR:WEB-INF/jsp/edit/moveContinueTask.jsp; class MoveContinueTaskAction#saveForm ("Move", "task.moved.from.to", "moved out", "moved in").</t>
+    <t>class DomainMetaDataRepository#init (task movecontinue -&gt; /do/move/continue/task); WAR:WEB-INF/struts-config.xml:293-295; WAR:WEB-INF/jsp/edit/moveContinueTask.jsp; class MoveContinueTaskAction#saveForm ("Move", "task.moved.from.to", "moved out", "moved in"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); MoveContinueTaskAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>Continue copies the unfinished task into the target story with cross-referenced descriptions.</t>
@@ -1849,7 +1861,7 @@
     <t>Time grid with an empty new row; "Insert Time" fills current time; Update saves; redirect to the task page.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (edittime -&gt; /do/edit/time); WAR:WEB-INF/struts-config.xml:350-355; WAR:WEB-INF/action-servlet.xml:376-378 (UpdateTimeAction); WAR:WEB-INF/jsp/edit/editTimeEntries.jsp; WAR:editTimeEntries.js; WAR:time.js.</t>
+    <t>class DomainMetaDataRepository#init (edittime -&gt; /do/edit/time); WAR:WEB-INF/struts-config.xml:350-355; WAR:WEB-INF/action-servlet.xml:376-378 (UpdateTimeAction); WAR:WEB-INF/jsp/edit/editTimeEntries.jsp; WAR:editTimeEntries.js; WAR:time.js. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); UpdateTimeAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>Existing entries can be edited or marked for deletion in the same grid.</t>
@@ -1876,13 +1888,109 @@
     <t>WAR:editTimeEntries.js:9-19,65-67 (remainingHours recalculation); class UpdateTimeAction#doUpdateTimeAction (TimeEditorForm.getRemainingHours, Task.setEstimatedHours).</t>
   </si>
   <si>
-    <t>Unparsable date/time input is rejected on the time editor.</t>
-  </si>
-  <si>
-    <t>Time editor redisplayed with an error (forward "error").</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/struts-config.xml:353-354 (error -&gt; editTimeEntries.jsp); class UpdateTimeAction (getDateTimeFormat format.datetime, getDateFormat format.date).</t>
+    <t>Unparsable date/time or number input in a time entry row is rejected.</t>
+  </si>
+  <si>
+    <t>Time editor redisplayed with "Can't parse the supplied date/time value." or "Can't parse the supplied number." (forward "error").</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.unparsable_time, edittime.error.unparsable_number; WAR:WEB-INF/classes/ResourceBundle.properties:675-676; WAR:WEB-INF/struts-config.xml:353-354 (error -&gt; editTimeEntries.jsp). Corrected in BA-001-04 (Source: stage-02-pass-002 F-001; the validator is the form, not UpdateTimeAction). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.unparsable_time: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). edittime.error.unparsable_number is missing in es and fr. Bundles without the key fall back to the default text (framework behavior, GAP-011). The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 66-68).</t>
+  </si>
+  <si>
+    <t>A time entry row with an end time but no start time, or a start time but no end time, is rejected.</t>
+  </si>
+  <si>
+    <t>Intervals must be complete.</t>
+  </si>
+  <si>
+    <t>Message "Missing start or end time."</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.missing_time; WAR:WEB-INF/classes/ResourceBundle.properties:677. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.missing_time: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru).</t>
+  </si>
+  <si>
+    <t>A time entry row without any person is rejected.</t>
+  </si>
+  <si>
+    <t>Time must be attributed to someone.</t>
+  </si>
+  <si>
+    <t>Message "No person is specified in a time entry."</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.missing_person; ResourceBundle.properties:678. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.missing_person: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru).</t>
+  </si>
+  <si>
+    <t>A time entry row naming the same person as both pair members is rejected.</t>
+  </si>
+  <si>
+    <t>Pairing needs two different people.</t>
+  </si>
+  <si>
+    <t>Message "Must specify different people for time entry."</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.same_people; ResourceBundle.properties:681. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.same_people: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru).</t>
+  </si>
+  <si>
+    <t>A time entry row whose end is not after its start is rejected.</t>
+  </si>
+  <si>
+    <t>Negative or empty intervals are invalid.</t>
+  </si>
+  <si>
+    <t>Message "Negative or zero-length intervals are not allowed."</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.negative_interval; ResourceBundle.properties:679. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.negative_interval: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru).</t>
+  </si>
+  <si>
+    <t>Time entry rows whose intervals overlap are rejected.</t>
+  </si>
+  <si>
+    <t>Prevents double-counted time.</t>
+  </si>
+  <si>
+    <t>Message "Overlapping intervals are not allowed."</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.overlapping_interval; ResourceBundle.properties:680. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.overlapping_interval: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru).</t>
+  </si>
+  <si>
+    <t>A time entry row with both a start/end interval and a duration is rejected.</t>
+  </si>
+  <si>
+    <t>Time is entered either as an interval or as a duration.</t>
+  </si>
+  <si>
+    <t>Message "Cannot specify both an interval and duration."</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.both_interval_and_duration; ResourceBundle.properties:682. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.both_interval_and_duration is missing in es. Bundles without the key fall back to the default text (framework behavior, GAP-011).</t>
+  </si>
+  <si>
+    <t>A time entry row without a report date is rejected.</t>
+  </si>
+  <si>
+    <t>Every entry needs the day it is reported for.</t>
+  </si>
+  <si>
+    <t>Message "Missing reported date."</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.missing_report_date; ResourceBundle.properties:683. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.missing_report_date is defined only in the default, "--", de, it, ja and ru bundles. Bundles without the key fall back to the default text (framework behavior, GAP-011).</t>
+  </si>
+  <si>
+    <t>A time entry description longer than the allowed maximum is rejected.</t>
+  </si>
+  <si>
+    <t>Keeps descriptions within the stored length.</t>
+  </si>
+  <si>
+    <t>Message "The time entry description is too long."</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.long_description; ResourceBundle.properties:684; the description input carries maxlength TimeEditorForm.MAX_DESCRIPTION_LENGTH (WAR:WEB-INF/jsp/edit/editTimeEntries.jsp). Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.long_description: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru).</t>
   </si>
   <si>
     <t>Re-estimate task (legacy page)</t>
@@ -1921,7 +2029,7 @@
     <t>Message "Can't parse the supplied date value."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.PersonTimesheetForm#validate (timesheet.error.unparsable_date).</t>
+    <t>class com.technoetic.xplanner.forms.PersonTimesheetForm#validate (timesheet.error.unparsable_date). Locale variants (CHK-004, BA-001-04): The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 66-68).</t>
   </si>
   <si>
     <t>The personal timesheet applies no permission filter: any signed-in user can open any person's timesheet by its oid.</t>
@@ -1951,7 +2059,7 @@
     <t>WAR:WEB-INF/jsp/view/projects.jsp:164 (link /do/view/aggregateTimesheet); WAR:WEB-INF/struts-config.xml:380-384; class ViewAggregateTimesheetAction (HQL people.hidden = false order by name); WAR:WEB-INF/jsp/view/aggregateTimesheet.jsp.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.AggregateTimesheetForm#validate (timesheet.error.unparsable_date).</t>
+    <t>class com.technoetic.xplanner.forms.AggregateTimesheetForm#validate (timesheet.error.unparsable_date). Locale variants (CHK-004, BA-001-04): The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 66-68).</t>
   </si>
   <si>
     <t>The aggregate timesheet includes only hours on projects the viewing user may read.</t>
@@ -1984,7 +2092,7 @@
     <t>Note editor (multipart form); after save the note appears in the Notes section of the object page.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/layout/viewLayout.jsp:114-116 (include view/notes.jsp in tiles:view pages); WAR:WEB-INF/jsp/view/notes.jsp:20-23 (isNoteEditor = hasPermission(..., "note", 0, "edit")) and link /do/edit/note?attachedToId=; WAR:WEB-INF/struts-config.xml:306-307; WAR:WEB-INF/action-servlet.xml:306-313 (EditNoteAction, virtualFileSystem); WAR:WEB-INF/jsp/edit/editNote.jsp.</t>
+    <t>WAR:WEB-INF/jsp/layout/viewLayout.jsp:114-116 (include view/notes.jsp in tiles:view pages); WAR:WEB-INF/jsp/view/notes.jsp:20-23 (isNoteEditor = hasPermission(..., "note", 0, "edit")) and link /do/edit/note?attachedToId=; WAR:WEB-INF/struts-config.xml:306-307; WAR:WEB-INF/action-servlet.xml:306-313 (EditNoteAction, virtualFileSystem); WAR:WEB-INF/jsp/edit/editNote.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>A note without subject, author or body is rejected.</t>
@@ -1999,16 +2107,16 @@
     <t>class com.technoetic.xplanner.forms.NoteEditorForm#validate (note.editor.missing_subject, missing_author, missing_body).</t>
   </si>
   <si>
-    <t>Each note with an attachment shows the attachment name and a download counter.</t>
-  </si>
-  <si>
-    <t>Shows how often a shared file was retrieved.</t>
-  </si>
-  <si>
-    <t>"Attachment" link and "attachment count" value on the note.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/notes.jsp:80-91 (link /do/download/attachment, notes.label.attachment.count, note.getAttachmentCount()).</t>
+    <t>Each note with an attachment shows the attachment name and a "References:" count, which is the number of notes that point to the same file.</t>
+  </si>
+  <si>
+    <t>Shows how many notes share one attached file.</t>
+  </si>
+  <si>
+    <t>"Attachment" link and "References: &lt;n&gt;" on the note.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/notes.jsp:80-92 (link /do/download/attachment, notes.label.attachment.count, note.getAttachmentCount()); class net.sf.xplanner.domain.Note#getAttachmentCount runs "select note from Note note where note.file.id=" + file id and returns the list size (bytecode listing); label WAR:WEB-INF/classes/ResourceBundle.properties:545 ("References:"); DownloadAttachmentAction counts nothing. Label per bundle (CHK-004): "References:" in the default, "--" and ja bundles, "Referenzen:" in de; the other bundles have no key and fall back to the default. Corrected in BA-001-04 (Source: stage-02-pass-002 F-004).</t>
   </si>
   <si>
     <t>An uploaded attachment is stored in the application virtual file system under /attachments/project/&lt;projectId&gt;; the file bytes are kept in the database as a BLOB (table xfile, column data), and directories are rows of table xdir.</t>
@@ -2035,7 +2143,7 @@
     <t>Note editor pre-filled; changes saved.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/notes.jsp (isUserAuthorized note edit; link /do/edit/note).</t>
+    <t>WAR:WEB-INF/jsp/view/notes.jsp (isUserAuthorized note edit; link /do/edit/note). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>An authorized user can delete a note after confirming "Do you want to delete note &lt;subject&gt;".</t>
@@ -2044,10 +2152,10 @@
     <t>Remove obsolete notes.</t>
   </si>
   <si>
-    <t>Confirm prompt; note removed.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/notes.jsp (link /do/delete/note with confirm); WAR:WEB-INF/struts-config.xml:309; class com.technoetic.xplanner.actions.DeleteNoteAction.</t>
+    <t>Confirm prompt; note removed; its attachment file removed too unless another note references it.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/notes.jsp (link /do/delete/note with confirm); WAR:WEB-INF/struts-config.xml:309; class com.technoetic.xplanner.actions.DeleteNoteAction#doExecute calls NoteHelper#deleteNote, which deletes the attached file only when no other note references it (query "select note from Note note where note.file.id= ?", size check), then the note (bytecode listing; BA-001-04 cascade sweep). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
   </si>
   <si>
     <t>Download attachment</t>
@@ -2077,7 +2185,7 @@
     <t>Directory listing with folder/file icons, "Create Directory" and "Upload" forms.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:401-403; WAR:WEB-INF/action-servlet.xml:396 (FileManagerAction); WAR:WEB-INF/jsp/view/directory.jsp; class FileManagerAction#doExecute (actions list, upload, download, delete, mkdir, rmdir). Only self-links from directory.jsp were found (linkgraph.txt); entry is by URL.</t>
+    <t>WAR:WEB-INF/struts-config.xml:401-403; WAR:WEB-INF/action-servlet.xml:396 (FileManagerAction); WAR:WEB-INF/jsp/view/directory.jsp; class FileManagerAction#doExecute (actions list, upload, download, delete, mkdir, rmdir). Only self-links from directory.jsp were found (linkgraph.txt); entry is by URL. Delete cascade sweep (BA-001-04): class com.technoetic.xplanner.file.FileSystemImpl#deleteFile and #deleteDirectory run an HQL delete by id without cascading; net.sf.xplanner.domain.Directory maps files and subdirectories without cascade. The foreign keys WAR:WEB-INF/classes/db-changelog.xml:259 (note.attachment_id -&gt; xfile), :266 (xdir.parent_id -&gt; xdir) and :267 (xfile.dir_id -&gt; xdir) are expected to make the database reject deleting a file that a note references or a directory that is not empty (runtime unverified).</t>
   </si>
   <si>
     <t>UF-011</t>
@@ -2278,16 +2386,16 @@
     <t>Share on social networks</t>
   </si>
   <si>
-    <t>View pages show Twitter and Facebook share links and a Facebook "like" widget loaded from facebook.net.</t>
+    <t>View pages show a Twitter status link and a Facebook feed-dialog share link with the object name; the LinkedIn link and the Facebook "like" widget are inside an HTML comment and not rendered.</t>
   </si>
   <si>
     <t>Social promotion of work items.</t>
   </si>
   <si>
-    <t>Share icons open external sites with the object name.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/layout/viewLayout.jsp:73-95 (twitter.com/home?status=..., facebook.com/dialog/feed, connect.facebook.net script).</t>
+    <t>Twitter and Facebook share icons open the external sites; no like widget, no LinkedIn link.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/layout/viewLayout.jsp:73-88 (twitter.com/home?status=..., facebook.com/dialog/feed with app_id and page URL) and :92-95 (HTML comment "&lt;!-- a class=\"in\" ... &lt;/span --&gt;" enclosing the LinkedIn link, the connect.facebook.net script and fb:like); the same comment in WAR:WEB-INF/jsp/layout/viewLayoutNew.jsp:114-117. Corrected in BA-001-04 (Source: stage-02-pass-002 F-003).</t>
   </si>
   <si>
     <t>Features (story features)</t>
@@ -2323,7 +2431,7 @@
     <t>Integration page with Start/Finished/Cancel buttons and a join form.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:388-394; WAR:WEB-INF/action-servlet.xml:390-392; WAR:WEB-INF/jsp/view/integrations.jsp; class com.technoetic.xplanner.actions.IntegrationAction (action.join, action.start, action.finish, action.cancel, action.leave). The used class com.technoetic.xplanner.domain.Integration has no @Entity and mappings/Integration.xml is not loaded; no live link to /do/view/integrations found. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the "not mapped" conclusion rests on spring-beans.xml:80 (rewritten entry) and is corroborated independently by the compiled class com.technoetic.xplanner.db.hibernate.HibernateHelper, whose mapped-class list also omits this class.</t>
+    <t>WAR:WEB-INF/struts-config.xml:388-394; WAR:WEB-INF/action-servlet.xml:390-392; WAR:WEB-INF/jsp/view/integrations.jsp; class com.technoetic.xplanner.actions.IntegrationAction (action.join, action.start, action.finish, action.cancel, action.leave). The used class com.technoetic.xplanner.domain.Integration has no @Entity and mappings/Integration.xml is not loaded; no live link to /do/view/integrations found. Server-side enforcement (CHK-002, BA-001-04): the view (DispatchForward) requires a projectId and system.project read (row 28); the join/start/finish/cancel/leave requests (IntegrationAction) perform no server-side permission check that gates the change (the only authorization call on the path is the recipient lookup inside the e-mail notifier), and the "integrate" condition only hides the buttons. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the "not mapped" conclusion rests on spring-beans.xml:80 (rewritten entry) and is corroborated independently by the compiled class com.technoetic.xplanner.db.hibernate.HibernateHelper, whose mapped-class list also omits this class.</t>
   </si>
   <si>
     <t>Joining without selecting a person or starting while another integration is active shows an error.</t>
@@ -2635,7 +2743,7 @@
     <t>Operations addX/update/removeX, setAttribute, deleteAttribute.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.soap.XPlanner (addProject ... removePerson, update(*Data), setAttribute, deleteAttribute; #saveHistory, #hasPermission).</t>
+    <t>class com.technoetic.xplanner.soap.XPlanner (addProject ... removePerson, update(*Data), setAttribute, deleteAttribute; #saveHistory, #hasPermission). Server-side enforcement (CHK-002, BA-001-04): enforced on the server by XPlanner#hasPermission for the object operations; the attribute operations have no check (row 210). Delete cascade sweep (BA-001-04): XPlanner#removeObject calls Session.delete, so the mapping cascades of the web deletes apply (rows 79, 88, 121, 136) and notes attached to the removed object are not deleted (NoteHelper#deleteNotesFor is not reached).</t>
   </si>
   <si>
     <t>UF-016</t>
@@ -2716,7 +2824,7 @@
     <t>text/calendar-like response (Content-type application/x-msoutlook) with VTODO and VEVENT entries.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:251-254,308-311 (iCalServlet /ical/*), :173-176 (BasicSecurityFilter /ical/*); class com.technoetic.xplanner.ical.iCalServlet#doGet, #generateTaskData, #generateTimeEntryData (HQL and VCALENDAR strings).</t>
+    <t>WAR:WEB-INF/web.xml:251-254,308-311 (iCalServlet /ical/*), :173-176 (BasicSecurityFilter /ical/*); class com.technoetic.xplanner.ical.iCalServlet#doGet, #generateTaskData, #generateTimeEntryData (HQL and VCALENDAR strings). Locale dependence (CHK-004, BA-001-04): the "non-overhead" filter compares the stored type with task.type.overhead from java.util.ResourceBundle.getBundle("ResourceBundle"), i.e. the JVM default locale (class iCalServlet#generateTaskData); overhead tasks saved under a different label are included (row 129).</t>
   </si>
   <si>
     <t>Requests without a file name or without the .ics suffix are rejected.</t>
@@ -3288,7 +3396,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N217"/>
+  <dimension ref="A1:N226"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="1" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="10.625" customWidth="1"/>
@@ -4244,7 +4352,7 @@
         <v>152</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="H34" s="23" t="s">
         <v>153</v>
@@ -6512,7 +6620,7 @@
         <v>494</v>
       </c>
       <c r="G113" s="23" t="s">
-        <v>99</v>
+        <v>37</v>
       </c>
       <c r="H113" s="23" t="s">
         <v>495</v>
@@ -6552,65 +6660,65 @@
       <c r="M114" s="23"/>
       <c r="N114" s="23"/>
     </row>
-    <row r="115" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A115" s="20" t="s">
+    <row r="115" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A115" s="21"/>
+      <c r="B115" s="21"/>
+      <c r="C115" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D115" s="23" t="s">
         <v>500</v>
       </c>
-      <c r="B115" s="20" t="s">
+      <c r="E115" s="23" t="s">
         <v>501</v>
       </c>
-      <c r="C115" s="20" t="s">
+      <c r="F115" s="23" t="s">
+        <v>502</v>
+      </c>
+      <c r="G115" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H115" s="23" t="s">
+        <v>503</v>
+      </c>
+      <c r="I115" s="23"/>
+      <c r="J115" s="23"/>
+      <c r="K115" s="23"/>
+      <c r="L115" s="23"/>
+      <c r="M115" s="23"/>
+      <c r="N115" s="23"/>
+    </row>
+    <row r="116" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A116" s="20" t="s">
+        <v>504</v>
+      </c>
+      <c r="B116" s="20" t="s">
+        <v>505</v>
+      </c>
+      <c r="C116" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="D115" s="20" t="s">
+      <c r="D116" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="E115" s="20"/>
-      <c r="F115" s="20"/>
-      <c r="G115" s="20"/>
-      <c r="H115" s="20"/>
-      <c r="I115" s="20"/>
-      <c r="J115" s="20"/>
-      <c r="K115" s="20"/>
-      <c r="L115" s="20"/>
-      <c r="M115" s="20"/>
-      <c r="N115" s="20"/>
-    </row>
-    <row r="116" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A116" s="21"/>
-      <c r="B116" s="22" t="s">
-        <v>502</v>
-      </c>
-      <c r="C116" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D116" s="23" t="s">
-        <v>503</v>
-      </c>
-      <c r="E116" s="23" t="s">
-        <v>504</v>
-      </c>
-      <c r="F116" s="23" t="s">
-        <v>505</v>
-      </c>
-      <c r="G116" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H116" s="23" t="s">
-        <v>506</v>
-      </c>
-      <c r="I116" s="23"/>
-      <c r="J116" s="23"/>
-      <c r="K116" s="23"/>
-      <c r="L116" s="23"/>
-      <c r="M116" s="23"/>
-      <c r="N116" s="23"/>
+      <c r="E116" s="20"/>
+      <c r="F116" s="20"/>
+      <c r="G116" s="20"/>
+      <c r="H116" s="20"/>
+      <c r="I116" s="20"/>
+      <c r="J116" s="20"/>
+      <c r="K116" s="20"/>
+      <c r="L116" s="20"/>
+      <c r="M116" s="20"/>
+      <c r="N116" s="20"/>
     </row>
     <row r="117" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A117" s="21"/>
-      <c r="B117" s="21"/>
+      <c r="B117" s="22" t="s">
+        <v>506</v>
+      </c>
       <c r="C117" s="21" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D117" s="23" t="s">
         <v>507</v>
@@ -6622,7 +6730,7 @@
         <v>509</v>
       </c>
       <c r="G117" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H117" s="23" t="s">
         <v>510</v>
@@ -6650,7 +6758,7 @@
         <v>513</v>
       </c>
       <c r="G118" s="23" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="H118" s="23" t="s">
         <v>514</v>
@@ -6664,26 +6772,24 @@
     </row>
     <row r="119" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A119" s="21"/>
-      <c r="B119" s="22" t="s">
+      <c r="B119" s="21"/>
+      <c r="C119" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D119" s="23" t="s">
         <v>515</v>
       </c>
-      <c r="C119" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D119" s="23" t="s">
+      <c r="E119" s="23" t="s">
         <v>516</v>
       </c>
-      <c r="E119" s="23" t="s">
+      <c r="F119" s="23" t="s">
         <v>517</v>
       </c>
-      <c r="F119" s="23" t="s">
+      <c r="G119" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H119" s="23" t="s">
         <v>518</v>
-      </c>
-      <c r="G119" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H119" s="23" t="s">
-        <v>519</v>
       </c>
       <c r="I119" s="23"/>
       <c r="J119" s="23"/>
@@ -6695,25 +6801,25 @@
     <row r="120" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A120" s="21"/>
       <c r="B120" s="22" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C120" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D120" s="23" t="s">
+        <v>520</v>
+      </c>
+      <c r="E120" s="23" t="s">
         <v>521</v>
       </c>
-      <c r="E120" s="23" t="s">
+      <c r="F120" s="23" t="s">
         <v>522</v>
       </c>
-      <c r="F120" s="23" t="s">
+      <c r="G120" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H120" s="23" t="s">
         <v>523</v>
-      </c>
-      <c r="G120" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H120" s="23" t="s">
-        <v>524</v>
       </c>
       <c r="I120" s="23"/>
       <c r="J120" s="23"/>
@@ -6725,25 +6831,25 @@
     <row r="121" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A121" s="21"/>
       <c r="B121" s="22" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="C121" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D121" s="23" t="s">
+        <v>525</v>
+      </c>
+      <c r="E121" s="23" t="s">
         <v>526</v>
       </c>
-      <c r="E121" s="23" t="s">
+      <c r="F121" s="23" t="s">
         <v>527</v>
       </c>
-      <c r="F121" s="23" t="s">
+      <c r="G121" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H121" s="23" t="s">
         <v>528</v>
-      </c>
-      <c r="G121" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H121" s="23" t="s">
-        <v>529</v>
       </c>
       <c r="I121" s="23"/>
       <c r="J121" s="23"/>
@@ -6754,24 +6860,26 @@
     </row>
     <row r="122" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A122" s="21"/>
-      <c r="B122" s="21"/>
+      <c r="B122" s="22" t="s">
+        <v>529</v>
+      </c>
       <c r="C122" s="21" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D122" s="23" t="s">
         <v>530</v>
       </c>
       <c r="E122" s="23" t="s">
-        <v>321</v>
+        <v>531</v>
       </c>
       <c r="F122" s="23" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="G122" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H122" s="23" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="I122" s="23"/>
       <c r="J122" s="23"/>
@@ -6782,26 +6890,24 @@
     </row>
     <row r="123" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A123" s="21"/>
-      <c r="B123" s="22" t="s">
-        <v>533</v>
-      </c>
+      <c r="B123" s="21"/>
       <c r="C123" s="21" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D123" s="23" t="s">
         <v>534</v>
       </c>
       <c r="E123" s="23" t="s">
+        <v>321</v>
+      </c>
+      <c r="F123" s="23" t="s">
         <v>535</v>
       </c>
-      <c r="F123" s="23" t="s">
+      <c r="G123" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H123" s="23" t="s">
         <v>536</v>
-      </c>
-      <c r="G123" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H123" s="23" t="s">
-        <v>537</v>
       </c>
       <c r="I123" s="23"/>
       <c r="J123" s="23"/>
@@ -6812,9 +6918,11 @@
     </row>
     <row r="124" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A124" s="21"/>
-      <c r="B124" s="21"/>
+      <c r="B124" s="22" t="s">
+        <v>537</v>
+      </c>
       <c r="C124" s="21" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D124" s="23" t="s">
         <v>538</v>
@@ -6826,7 +6934,7 @@
         <v>540</v>
       </c>
       <c r="G124" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H124" s="23" t="s">
         <v>541</v>
@@ -6854,7 +6962,7 @@
         <v>544</v>
       </c>
       <c r="G125" s="23" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="H125" s="23" t="s">
         <v>545</v>
@@ -6866,65 +6974,65 @@
       <c r="M125" s="23"/>
       <c r="N125" s="23"/>
     </row>
-    <row r="126" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A126" s="20" t="s">
+    <row r="126" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A126" s="21"/>
+      <c r="B126" s="21"/>
+      <c r="C126" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D126" s="23" t="s">
         <v>546</v>
       </c>
-      <c r="B126" s="20" t="s">
+      <c r="E126" s="23" t="s">
         <v>547</v>
       </c>
-      <c r="C126" s="20" t="s">
+      <c r="F126" s="23" t="s">
+        <v>548</v>
+      </c>
+      <c r="G126" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H126" s="23" t="s">
+        <v>549</v>
+      </c>
+      <c r="I126" s="23"/>
+      <c r="J126" s="23"/>
+      <c r="K126" s="23"/>
+      <c r="L126" s="23"/>
+      <c r="M126" s="23"/>
+      <c r="N126" s="23"/>
+    </row>
+    <row r="127" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A127" s="20" t="s">
+        <v>550</v>
+      </c>
+      <c r="B127" s="20" t="s">
+        <v>551</v>
+      </c>
+      <c r="C127" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="D126" s="20" t="s">
+      <c r="D127" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="E126" s="20"/>
-      <c r="F126" s="20"/>
-      <c r="G126" s="20"/>
-      <c r="H126" s="20"/>
-      <c r="I126" s="20"/>
-      <c r="J126" s="20"/>
-      <c r="K126" s="20"/>
-      <c r="L126" s="20"/>
-      <c r="M126" s="20"/>
-      <c r="N126" s="20"/>
-    </row>
-    <row r="127" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A127" s="21"/>
-      <c r="B127" s="22" t="s">
-        <v>548</v>
-      </c>
-      <c r="C127" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D127" s="23" t="s">
-        <v>549</v>
-      </c>
-      <c r="E127" s="23" t="s">
-        <v>550</v>
-      </c>
-      <c r="F127" s="23" t="s">
-        <v>551</v>
-      </c>
-      <c r="G127" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H127" s="23" t="s">
-        <v>552</v>
-      </c>
-      <c r="I127" s="23"/>
-      <c r="J127" s="23"/>
-      <c r="K127" s="23"/>
-      <c r="L127" s="23"/>
-      <c r="M127" s="23"/>
-      <c r="N127" s="23"/>
+      <c r="E127" s="20"/>
+      <c r="F127" s="20"/>
+      <c r="G127" s="20"/>
+      <c r="H127" s="20"/>
+      <c r="I127" s="20"/>
+      <c r="J127" s="20"/>
+      <c r="K127" s="20"/>
+      <c r="L127" s="20"/>
+      <c r="M127" s="20"/>
+      <c r="N127" s="20"/>
     </row>
     <row r="128" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A128" s="21"/>
-      <c r="B128" s="21"/>
+      <c r="B128" s="22" t="s">
+        <v>552</v>
+      </c>
       <c r="C128" s="21" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D128" s="23" t="s">
         <v>553</v>
@@ -6986,16 +7094,16 @@
         <v>561</v>
       </c>
       <c r="E130" s="23" t="s">
-        <v>512</v>
+        <v>562</v>
       </c>
       <c r="F130" s="23" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="G130" s="23" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="H130" s="23" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="I130" s="23"/>
       <c r="J130" s="23"/>
@@ -7006,26 +7114,24 @@
     </row>
     <row r="131" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A131" s="21"/>
-      <c r="B131" s="22" t="s">
-        <v>564</v>
-      </c>
+      <c r="B131" s="21"/>
       <c r="C131" s="21" t="s">
-        <v>90</v>
+        <v>39</v>
       </c>
       <c r="D131" s="23" t="s">
         <v>565</v>
       </c>
       <c r="E131" s="23" t="s">
+        <v>516</v>
+      </c>
+      <c r="F131" s="23" t="s">
         <v>566</v>
       </c>
-      <c r="F131" s="23" t="s">
+      <c r="G131" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H131" s="23" t="s">
         <v>567</v>
-      </c>
-      <c r="G131" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H131" s="23" t="s">
-        <v>568</v>
       </c>
       <c r="I131" s="23"/>
       <c r="J131" s="23"/>
@@ -7037,25 +7143,25 @@
     <row r="132" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A132" s="21"/>
       <c r="B132" s="22" t="s">
+        <v>568</v>
+      </c>
+      <c r="C132" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="D132" s="23" t="s">
         <v>569</v>
       </c>
-      <c r="C132" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D132" s="23" t="s">
+      <c r="E132" s="23" t="s">
         <v>570</v>
       </c>
-      <c r="E132" s="23" t="s">
+      <c r="F132" s="23" t="s">
         <v>571</v>
       </c>
-      <c r="F132" s="23" t="s">
+      <c r="G132" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H132" s="23" t="s">
         <v>572</v>
-      </c>
-      <c r="G132" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H132" s="23" t="s">
-        <v>573</v>
       </c>
       <c r="I132" s="23"/>
       <c r="J132" s="23"/>
@@ -7067,25 +7173,25 @@
     <row r="133" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A133" s="21"/>
       <c r="B133" s="22" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C133" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D133" s="23" t="s">
+        <v>574</v>
+      </c>
+      <c r="E133" s="23" t="s">
         <v>575</v>
       </c>
-      <c r="E133" s="23" t="s">
+      <c r="F133" s="23" t="s">
         <v>576</v>
       </c>
-      <c r="F133" s="23" t="s">
+      <c r="G133" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H133" s="23" t="s">
         <v>577</v>
-      </c>
-      <c r="G133" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H133" s="23" t="s">
-        <v>578</v>
       </c>
       <c r="I133" s="23"/>
       <c r="J133" s="23"/>
@@ -7096,9 +7202,11 @@
     </row>
     <row r="134" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A134" s="21"/>
-      <c r="B134" s="21"/>
+      <c r="B134" s="22" t="s">
+        <v>578</v>
+      </c>
       <c r="C134" s="21" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D134" s="23" t="s">
         <v>579</v>
@@ -7124,26 +7232,24 @@
     </row>
     <row r="135" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A135" s="21"/>
-      <c r="B135" s="22" t="s">
+      <c r="B135" s="21"/>
+      <c r="C135" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D135" s="23" t="s">
         <v>583</v>
       </c>
-      <c r="C135" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D135" s="23" t="s">
+      <c r="E135" s="23" t="s">
         <v>584</v>
       </c>
-      <c r="E135" s="23" t="s">
+      <c r="F135" s="23" t="s">
         <v>585</v>
       </c>
-      <c r="F135" s="23" t="s">
+      <c r="G135" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H135" s="23" t="s">
         <v>586</v>
-      </c>
-      <c r="G135" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H135" s="23" t="s">
-        <v>587</v>
       </c>
       <c r="I135" s="23"/>
       <c r="J135" s="23"/>
@@ -7155,25 +7261,25 @@
     <row r="136" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A136" s="21"/>
       <c r="B136" s="22" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="C136" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D136" s="23" t="s">
+        <v>588</v>
+      </c>
+      <c r="E136" s="23" t="s">
         <v>589</v>
       </c>
-      <c r="E136" s="23" t="s">
+      <c r="F136" s="23" t="s">
         <v>590</v>
       </c>
-      <c r="F136" s="23" t="s">
+      <c r="G136" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H136" s="23" t="s">
         <v>591</v>
-      </c>
-      <c r="G136" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H136" s="23" t="s">
-        <v>592</v>
       </c>
       <c r="I136" s="23"/>
       <c r="J136" s="23"/>
@@ -7185,25 +7291,25 @@
     <row r="137" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A137" s="21"/>
       <c r="B137" s="22" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C137" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D137" s="23" t="s">
+        <v>593</v>
+      </c>
+      <c r="E137" s="23" t="s">
         <v>594</v>
       </c>
-      <c r="E137" s="23" t="s">
+      <c r="F137" s="23" t="s">
         <v>595</v>
       </c>
-      <c r="F137" s="23" t="s">
+      <c r="G137" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H137" s="23" t="s">
         <v>596</v>
-      </c>
-      <c r="G137" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H137" s="23" t="s">
-        <v>597</v>
       </c>
       <c r="I137" s="23"/>
       <c r="J137" s="23"/>
@@ -7214,9 +7320,11 @@
     </row>
     <row r="138" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A138" s="21"/>
-      <c r="B138" s="21"/>
+      <c r="B138" s="22" t="s">
+        <v>597</v>
+      </c>
       <c r="C138" s="21" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D138" s="23" t="s">
         <v>598</v>
@@ -7228,7 +7336,7 @@
         <v>600</v>
       </c>
       <c r="G138" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H138" s="23" t="s">
         <v>601</v>
@@ -7250,16 +7358,16 @@
         <v>602</v>
       </c>
       <c r="E139" s="23" t="s">
-        <v>543</v>
+        <v>603</v>
       </c>
       <c r="F139" s="23" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="G139" s="23" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="H139" s="23" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="I139" s="23"/>
       <c r="J139" s="23"/>
@@ -7268,65 +7376,65 @@
       <c r="M139" s="23"/>
       <c r="N139" s="23"/>
     </row>
-    <row r="140" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A140" s="20" t="s">
-        <v>605</v>
-      </c>
-      <c r="B140" s="20" t="s">
+    <row r="140" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A140" s="21"/>
+      <c r="B140" s="21"/>
+      <c r="C140" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D140" s="23" t="s">
         <v>606</v>
       </c>
-      <c r="C140" s="20" t="s">
+      <c r="E140" s="23" t="s">
+        <v>547</v>
+      </c>
+      <c r="F140" s="23" t="s">
+        <v>607</v>
+      </c>
+      <c r="G140" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H140" s="23" t="s">
+        <v>608</v>
+      </c>
+      <c r="I140" s="23"/>
+      <c r="J140" s="23"/>
+      <c r="K140" s="23"/>
+      <c r="L140" s="23"/>
+      <c r="M140" s="23"/>
+      <c r="N140" s="23"/>
+    </row>
+    <row r="141" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A141" s="20" t="s">
+        <v>609</v>
+      </c>
+      <c r="B141" s="20" t="s">
+        <v>610</v>
+      </c>
+      <c r="C141" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="D140" s="20" t="s">
+      <c r="D141" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="E140" s="20"/>
-      <c r="F140" s="20"/>
-      <c r="G140" s="20"/>
-      <c r="H140" s="20"/>
-      <c r="I140" s="20"/>
-      <c r="J140" s="20"/>
-      <c r="K140" s="20"/>
-      <c r="L140" s="20"/>
-      <c r="M140" s="20"/>
-      <c r="N140" s="20"/>
-    </row>
-    <row r="141" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A141" s="21"/>
-      <c r="B141" s="22" t="s">
-        <v>607</v>
-      </c>
-      <c r="C141" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D141" s="23" t="s">
-        <v>608</v>
-      </c>
-      <c r="E141" s="23" t="s">
-        <v>609</v>
-      </c>
-      <c r="F141" s="23" t="s">
-        <v>610</v>
-      </c>
-      <c r="G141" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H141" s="23" t="s">
-        <v>611</v>
-      </c>
-      <c r="I141" s="23"/>
-      <c r="J141" s="23"/>
-      <c r="K141" s="23"/>
-      <c r="L141" s="23"/>
-      <c r="M141" s="23"/>
-      <c r="N141" s="23"/>
+      <c r="E141" s="20"/>
+      <c r="F141" s="20"/>
+      <c r="G141" s="20"/>
+      <c r="H141" s="20"/>
+      <c r="I141" s="20"/>
+      <c r="J141" s="20"/>
+      <c r="K141" s="20"/>
+      <c r="L141" s="20"/>
+      <c r="M141" s="20"/>
+      <c r="N141" s="20"/>
     </row>
     <row r="142" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A142" s="21"/>
-      <c r="B142" s="21"/>
+      <c r="B142" s="22" t="s">
+        <v>611</v>
+      </c>
       <c r="C142" s="21" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D142" s="23" t="s">
         <v>612</v>
@@ -7366,7 +7474,7 @@
         <v>618</v>
       </c>
       <c r="G143" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H143" s="23" t="s">
         <v>619</v>
@@ -7388,16 +7496,16 @@
         <v>620</v>
       </c>
       <c r="E144" s="23" t="s">
-        <v>512</v>
+        <v>621</v>
       </c>
       <c r="F144" s="23" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G144" s="23" t="s">
         <v>47</v>
       </c>
       <c r="H144" s="23" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="I144" s="23"/>
       <c r="J144" s="23"/>
@@ -7408,9 +7516,7 @@
     </row>
     <row r="145" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A145" s="21"/>
-      <c r="B145" s="22" t="s">
-        <v>623</v>
-      </c>
+      <c r="B145" s="21"/>
       <c r="C145" s="21" t="s">
         <v>39</v>
       </c>
@@ -7418,16 +7524,16 @@
         <v>624</v>
       </c>
       <c r="E145" s="23" t="s">
+        <v>516</v>
+      </c>
+      <c r="F145" s="23" t="s">
         <v>625</v>
       </c>
-      <c r="F145" s="23" t="s">
+      <c r="G145" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H145" s="23" t="s">
         <v>626</v>
-      </c>
-      <c r="G145" s="23" t="s">
-        <v>99</v>
-      </c>
-      <c r="H145" s="23" t="s">
-        <v>627</v>
       </c>
       <c r="I145" s="23"/>
       <c r="J145" s="23"/>
@@ -7438,26 +7544,24 @@
     </row>
     <row r="146" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A146" s="21"/>
-      <c r="B146" s="22" t="s">
+      <c r="B146" s="21"/>
+      <c r="C146" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D146" s="23" t="s">
+        <v>627</v>
+      </c>
+      <c r="E146" s="23" t="s">
         <v>628</v>
       </c>
-      <c r="C146" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D146" s="23" t="s">
+      <c r="F146" s="23" t="s">
         <v>629</v>
       </c>
-      <c r="E146" s="23" t="s">
+      <c r="G146" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H146" s="23" t="s">
         <v>630</v>
-      </c>
-      <c r="F146" s="23" t="s">
-        <v>631</v>
-      </c>
-      <c r="G146" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H146" s="23" t="s">
-        <v>632</v>
       </c>
       <c r="I146" s="23"/>
       <c r="J146" s="23"/>
@@ -7473,19 +7577,19 @@
         <v>39</v>
       </c>
       <c r="D147" s="23" t="s">
+        <v>631</v>
+      </c>
+      <c r="E147" s="23" t="s">
+        <v>632</v>
+      </c>
+      <c r="F147" s="23" t="s">
         <v>633</v>
       </c>
-      <c r="E147" s="23" t="s">
-        <v>512</v>
-      </c>
-      <c r="F147" s="23" t="s">
+      <c r="G147" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H147" s="23" t="s">
         <v>634</v>
-      </c>
-      <c r="G147" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H147" s="23" t="s">
-        <v>635</v>
       </c>
       <c r="I147" s="23"/>
       <c r="J147" s="23"/>
@@ -7501,19 +7605,19 @@
         <v>39</v>
       </c>
       <c r="D148" s="23" t="s">
+        <v>635</v>
+      </c>
+      <c r="E148" s="23" t="s">
         <v>636</v>
       </c>
-      <c r="E148" s="23" t="s">
+      <c r="F148" s="23" t="s">
         <v>637</v>
-      </c>
-      <c r="F148" s="23" t="s">
-        <v>638</v>
       </c>
       <c r="G148" s="23" t="s">
         <v>47</v>
       </c>
       <c r="H148" s="23" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="I148" s="23"/>
       <c r="J148" s="23"/>
@@ -7524,26 +7628,24 @@
     </row>
     <row r="149" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A149" s="21"/>
-      <c r="B149" s="22" t="s">
+      <c r="B149" s="21"/>
+      <c r="C149" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D149" s="23" t="s">
+        <v>639</v>
+      </c>
+      <c r="E149" s="23" t="s">
         <v>640</v>
       </c>
-      <c r="C149" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D149" s="23" t="s">
+      <c r="F149" s="23" t="s">
         <v>641</v>
       </c>
-      <c r="E149" s="23" t="s">
+      <c r="G149" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H149" s="23" t="s">
         <v>642</v>
-      </c>
-      <c r="F149" s="23" t="s">
-        <v>643</v>
-      </c>
-      <c r="G149" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H149" s="23" t="s">
-        <v>644</v>
       </c>
       <c r="I149" s="23"/>
       <c r="J149" s="23"/>
@@ -7559,19 +7661,19 @@
         <v>39</v>
       </c>
       <c r="D150" s="23" t="s">
-        <v>633</v>
+        <v>643</v>
       </c>
       <c r="E150" s="23" t="s">
-        <v>512</v>
+        <v>644</v>
       </c>
       <c r="F150" s="23" t="s">
-        <v>634</v>
+        <v>645</v>
       </c>
       <c r="G150" s="23" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="H150" s="23" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="I150" s="23"/>
       <c r="J150" s="23"/>
@@ -7587,19 +7689,19 @@
         <v>39</v>
       </c>
       <c r="D151" s="23" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="E151" s="23" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="F151" s="23" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="G151" s="23" t="s">
         <v>47</v>
       </c>
       <c r="H151" s="23" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="I151" s="23"/>
       <c r="J151" s="23"/>
@@ -7608,52 +7710,54 @@
       <c r="M151" s="23"/>
       <c r="N151" s="23"/>
     </row>
-    <row r="152" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A152" s="20" t="s">
-        <v>650</v>
-      </c>
-      <c r="B152" s="20" t="s">
+    <row r="152" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A152" s="21"/>
+      <c r="B152" s="21"/>
+      <c r="C152" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D152" s="23" t="s">
         <v>651</v>
       </c>
-      <c r="C152" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="D152" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="E152" s="20"/>
-      <c r="F152" s="20"/>
-      <c r="G152" s="20"/>
-      <c r="H152" s="20"/>
-      <c r="I152" s="20"/>
-      <c r="J152" s="20"/>
-      <c r="K152" s="20"/>
-      <c r="L152" s="20"/>
-      <c r="M152" s="20"/>
-      <c r="N152" s="20"/>
+      <c r="E152" s="23" t="s">
+        <v>652</v>
+      </c>
+      <c r="F152" s="23" t="s">
+        <v>653</v>
+      </c>
+      <c r="G152" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H152" s="23" t="s">
+        <v>654</v>
+      </c>
+      <c r="I152" s="23"/>
+      <c r="J152" s="23"/>
+      <c r="K152" s="23"/>
+      <c r="L152" s="23"/>
+      <c r="M152" s="23"/>
+      <c r="N152" s="23"/>
     </row>
     <row r="153" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A153" s="21"/>
-      <c r="B153" s="22" t="s">
-        <v>652</v>
-      </c>
+      <c r="B153" s="21"/>
       <c r="C153" s="21" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D153" s="23" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="E153" s="23" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="F153" s="23" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="G153" s="23" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="H153" s="23" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="I153" s="23"/>
       <c r="J153" s="23"/>
@@ -7664,24 +7768,26 @@
     </row>
     <row r="154" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A154" s="21"/>
-      <c r="B154" s="21"/>
+      <c r="B154" s="22" t="s">
+        <v>659</v>
+      </c>
       <c r="C154" s="21" t="s">
         <v>39</v>
       </c>
       <c r="D154" s="23" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
       <c r="E154" s="23" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
       <c r="F154" s="23" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
       <c r="G154" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H154" s="23" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="I154" s="23"/>
       <c r="J154" s="23"/>
@@ -7692,24 +7798,26 @@
     </row>
     <row r="155" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A155" s="21"/>
-      <c r="B155" s="21"/>
+      <c r="B155" s="22" t="s">
+        <v>664</v>
+      </c>
       <c r="C155" s="21" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D155" s="23" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="E155" s="23" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="F155" s="23" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
       <c r="G155" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H155" s="23" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="I155" s="23"/>
       <c r="J155" s="23"/>
@@ -7725,19 +7833,19 @@
         <v>39</v>
       </c>
       <c r="D156" s="23" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="E156" s="23" t="s">
-        <v>666</v>
+        <v>516</v>
       </c>
       <c r="F156" s="23" t="s">
-        <v>667</v>
+        <v>670</v>
       </c>
       <c r="G156" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H156" s="23" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="I156" s="23"/>
       <c r="J156" s="23"/>
@@ -7748,26 +7856,24 @@
     </row>
     <row r="157" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A157" s="21"/>
-      <c r="B157" s="22" t="s">
-        <v>669</v>
-      </c>
+      <c r="B157" s="21"/>
       <c r="C157" s="21" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D157" s="23" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="E157" s="23" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="F157" s="23" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="G157" s="23" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="H157" s="23" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="I157" s="23"/>
       <c r="J157" s="23"/>
@@ -7778,24 +7884,26 @@
     </row>
     <row r="158" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A158" s="21"/>
-      <c r="B158" s="21"/>
+      <c r="B158" s="22" t="s">
+        <v>676</v>
+      </c>
       <c r="C158" s="21" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D158" s="23" t="s">
-        <v>674</v>
+        <v>677</v>
       </c>
       <c r="E158" s="23" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
       <c r="F158" s="23" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="G158" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H158" s="23" t="s">
-        <v>677</v>
+        <v>680</v>
       </c>
       <c r="I158" s="23"/>
       <c r="J158" s="23"/>
@@ -7806,26 +7914,24 @@
     </row>
     <row r="159" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A159" s="21"/>
-      <c r="B159" s="22" t="s">
-        <v>678</v>
-      </c>
+      <c r="B159" s="21"/>
       <c r="C159" s="21" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D159" s="23" t="s">
-        <v>679</v>
+        <v>669</v>
       </c>
       <c r="E159" s="23" t="s">
-        <v>680</v>
+        <v>516</v>
       </c>
       <c r="F159" s="23" t="s">
+        <v>670</v>
+      </c>
+      <c r="G159" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H159" s="23" t="s">
         <v>681</v>
-      </c>
-      <c r="G159" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H159" s="23" t="s">
-        <v>682</v>
       </c>
       <c r="I159" s="23"/>
       <c r="J159" s="23"/>
@@ -7836,26 +7942,24 @@
     </row>
     <row r="160" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A160" s="21"/>
-      <c r="B160" s="22" t="s">
+      <c r="B160" s="21"/>
+      <c r="C160" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D160" s="23" t="s">
+        <v>682</v>
+      </c>
+      <c r="E160" s="23" t="s">
         <v>683</v>
       </c>
-      <c r="C160" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="D160" s="23" t="s">
+      <c r="F160" s="23" t="s">
         <v>684</v>
       </c>
-      <c r="E160" s="23" t="s">
+      <c r="G160" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H160" s="23" t="s">
         <v>685</v>
-      </c>
-      <c r="F160" s="23" t="s">
-        <v>686</v>
-      </c>
-      <c r="G160" s="23" t="s">
-        <v>99</v>
-      </c>
-      <c r="H160" s="23" t="s">
-        <v>687</v>
       </c>
       <c r="I160" s="23"/>
       <c r="J160" s="23"/>
@@ -7866,10 +7970,10 @@
     </row>
     <row r="161" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A161" s="20" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="B161" s="20" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="C161" s="20" t="s">
         <v>30</v>
@@ -7891,25 +7995,25 @@
     <row r="162" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A162" s="21"/>
       <c r="B162" s="22" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="C162" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D162" s="23" t="s">
+        <v>689</v>
+      </c>
+      <c r="E162" s="23" t="s">
+        <v>690</v>
+      </c>
+      <c r="F162" s="23" t="s">
         <v>691</v>
       </c>
-      <c r="E162" s="23" t="s">
+      <c r="G162" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H162" s="23" t="s">
         <v>692</v>
-      </c>
-      <c r="F162" s="23" t="s">
-        <v>693</v>
-      </c>
-      <c r="G162" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H162" s="23" t="s">
-        <v>694</v>
       </c>
       <c r="I162" s="23"/>
       <c r="J162" s="23"/>
@@ -7925,19 +8029,19 @@
         <v>39</v>
       </c>
       <c r="D163" s="23" t="s">
+        <v>693</v>
+      </c>
+      <c r="E163" s="23" t="s">
+        <v>694</v>
+      </c>
+      <c r="F163" s="23" t="s">
         <v>695</v>
       </c>
-      <c r="E163" s="23" t="s">
+      <c r="G163" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H163" s="23" t="s">
         <v>696</v>
-      </c>
-      <c r="F163" s="23" t="s">
-        <v>697</v>
-      </c>
-      <c r="G163" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H163" s="23" t="s">
-        <v>698</v>
       </c>
       <c r="I163" s="23"/>
       <c r="J163" s="23"/>
@@ -7953,19 +8057,19 @@
         <v>39</v>
       </c>
       <c r="D164" s="23" t="s">
+        <v>697</v>
+      </c>
+      <c r="E164" s="23" t="s">
+        <v>698</v>
+      </c>
+      <c r="F164" s="23" t="s">
         <v>699</v>
       </c>
-      <c r="E164" s="23" t="s">
+      <c r="G164" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H164" s="23" t="s">
         <v>700</v>
-      </c>
-      <c r="F164" s="23" t="s">
-        <v>701</v>
-      </c>
-      <c r="G164" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H164" s="23" t="s">
-        <v>702</v>
       </c>
       <c r="I164" s="23"/>
       <c r="J164" s="23"/>
@@ -7981,19 +8085,19 @@
         <v>39</v>
       </c>
       <c r="D165" s="23" t="s">
+        <v>701</v>
+      </c>
+      <c r="E165" s="23" t="s">
+        <v>702</v>
+      </c>
+      <c r="F165" s="23" t="s">
         <v>703</v>
       </c>
-      <c r="E165" s="23" t="s">
+      <c r="G165" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H165" s="23" t="s">
         <v>704</v>
-      </c>
-      <c r="F165" s="23" t="s">
-        <v>705</v>
-      </c>
-      <c r="G165" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H165" s="23" t="s">
-        <v>706</v>
       </c>
       <c r="I165" s="23"/>
       <c r="J165" s="23"/>
@@ -8005,25 +8109,25 @@
     <row r="166" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A166" s="21"/>
       <c r="B166" s="22" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="C166" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D166" s="23" t="s">
+        <v>706</v>
+      </c>
+      <c r="E166" s="23" t="s">
+        <v>707</v>
+      </c>
+      <c r="F166" s="23" t="s">
         <v>708</v>
       </c>
-      <c r="E166" s="23" t="s">
+      <c r="G166" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H166" s="23" t="s">
         <v>709</v>
-      </c>
-      <c r="F166" s="23" t="s">
-        <v>710</v>
-      </c>
-      <c r="G166" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H166" s="23" t="s">
-        <v>711</v>
       </c>
       <c r="I166" s="23"/>
       <c r="J166" s="23"/>
@@ -8039,19 +8143,19 @@
         <v>39</v>
       </c>
       <c r="D167" s="23" t="s">
+        <v>710</v>
+      </c>
+      <c r="E167" s="23" t="s">
+        <v>711</v>
+      </c>
+      <c r="F167" s="23" t="s">
         <v>712</v>
       </c>
-      <c r="E167" s="23" t="s">
+      <c r="G167" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H167" s="23" t="s">
         <v>713</v>
-      </c>
-      <c r="F167" s="23" t="s">
-        <v>714</v>
-      </c>
-      <c r="G167" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H167" s="23" t="s">
-        <v>715</v>
       </c>
       <c r="I167" s="23"/>
       <c r="J167" s="23"/>
@@ -8062,24 +8166,26 @@
     </row>
     <row r="168" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A168" s="21"/>
-      <c r="B168" s="21"/>
+      <c r="B168" s="22" t="s">
+        <v>714</v>
+      </c>
       <c r="C168" s="21" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D168" s="23" t="s">
+        <v>715</v>
+      </c>
+      <c r="E168" s="23" t="s">
         <v>716</v>
       </c>
-      <c r="E168" s="23" t="s">
+      <c r="F168" s="23" t="s">
         <v>717</v>
       </c>
-      <c r="F168" s="23" t="s">
+      <c r="G168" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H168" s="23" t="s">
         <v>718</v>
-      </c>
-      <c r="G168" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H168" s="23" t="s">
-        <v>719</v>
       </c>
       <c r="I168" s="23"/>
       <c r="J168" s="23"/>
@@ -8091,25 +8197,25 @@
     <row r="169" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A169" s="21"/>
       <c r="B169" s="22" t="s">
+        <v>719</v>
+      </c>
+      <c r="C169" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D169" s="23" t="s">
         <v>720</v>
       </c>
-      <c r="C169" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D169" s="23" t="s">
+      <c r="E169" s="23" t="s">
         <v>721</v>
       </c>
-      <c r="E169" s="23" t="s">
+      <c r="F169" s="23" t="s">
         <v>722</v>
       </c>
-      <c r="F169" s="23" t="s">
+      <c r="G169" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="H169" s="23" t="s">
         <v>723</v>
-      </c>
-      <c r="G169" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H169" s="23" t="s">
-        <v>724</v>
       </c>
       <c r="I169" s="23"/>
       <c r="J169" s="23"/>
@@ -8118,56 +8224,52 @@
       <c r="M169" s="23"/>
       <c r="N169" s="23"/>
     </row>
-    <row r="170" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A170" s="21"/>
-      <c r="B170" s="22" t="s">
+    <row r="170" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A170" s="20" t="s">
+        <v>724</v>
+      </c>
+      <c r="B170" s="20" t="s">
         <v>725</v>
       </c>
-      <c r="C170" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D170" s="23" t="s">
-        <v>726</v>
-      </c>
-      <c r="E170" s="23" t="s">
-        <v>727</v>
-      </c>
-      <c r="F170" s="23" t="s">
-        <v>728</v>
-      </c>
-      <c r="G170" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H170" s="23" t="s">
-        <v>729</v>
-      </c>
-      <c r="I170" s="23"/>
-      <c r="J170" s="23"/>
-      <c r="K170" s="23"/>
-      <c r="L170" s="23"/>
-      <c r="M170" s="23"/>
-      <c r="N170" s="23"/>
+      <c r="C170" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="D170" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="E170" s="20"/>
+      <c r="F170" s="20"/>
+      <c r="G170" s="20"/>
+      <c r="H170" s="20"/>
+      <c r="I170" s="20"/>
+      <c r="J170" s="20"/>
+      <c r="K170" s="20"/>
+      <c r="L170" s="20"/>
+      <c r="M170" s="20"/>
+      <c r="N170" s="20"/>
     </row>
     <row r="171" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A171" s="21"/>
-      <c r="B171" s="21"/>
+      <c r="B171" s="22" t="s">
+        <v>726</v>
+      </c>
       <c r="C171" s="21" t="s">
-        <v>90</v>
+        <v>33</v>
       </c>
       <c r="D171" s="23" t="s">
+        <v>727</v>
+      </c>
+      <c r="E171" s="23" t="s">
+        <v>728</v>
+      </c>
+      <c r="F171" s="23" t="s">
+        <v>729</v>
+      </c>
+      <c r="G171" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H171" s="23" t="s">
         <v>730</v>
-      </c>
-      <c r="E171" s="23" t="s">
-        <v>731</v>
-      </c>
-      <c r="F171" s="23" t="s">
-        <v>732</v>
-      </c>
-      <c r="G171" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H171" s="23" t="s">
-        <v>733</v>
       </c>
       <c r="I171" s="23"/>
       <c r="J171" s="23"/>
@@ -8178,26 +8280,24 @@
     </row>
     <row r="172" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A172" s="21"/>
-      <c r="B172" s="22" t="s">
+      <c r="B172" s="21"/>
+      <c r="C172" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D172" s="23" t="s">
+        <v>731</v>
+      </c>
+      <c r="E172" s="23" t="s">
+        <v>732</v>
+      </c>
+      <c r="F172" s="23" t="s">
+        <v>733</v>
+      </c>
+      <c r="G172" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H172" s="23" t="s">
         <v>734</v>
-      </c>
-      <c r="C172" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D172" s="23" t="s">
-        <v>735</v>
-      </c>
-      <c r="E172" s="23" t="s">
-        <v>736</v>
-      </c>
-      <c r="F172" s="23" t="s">
-        <v>737</v>
-      </c>
-      <c r="G172" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H172" s="23" t="s">
-        <v>738</v>
       </c>
       <c r="I172" s="23"/>
       <c r="J172" s="23"/>
@@ -8208,26 +8308,24 @@
     </row>
     <row r="173" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A173" s="21"/>
-      <c r="B173" s="22" t="s">
-        <v>739</v>
-      </c>
+      <c r="B173" s="21"/>
       <c r="C173" s="21" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D173" s="23" t="s">
-        <v>740</v>
+        <v>735</v>
       </c>
       <c r="E173" s="23" t="s">
-        <v>741</v>
+        <v>736</v>
       </c>
       <c r="F173" s="23" t="s">
-        <v>742</v>
+        <v>737</v>
       </c>
       <c r="G173" s="23" t="s">
         <v>47</v>
       </c>
       <c r="H173" s="23" t="s">
-        <v>743</v>
+        <v>738</v>
       </c>
       <c r="I173" s="23"/>
       <c r="J173" s="23"/>
@@ -8243,19 +8341,19 @@
         <v>39</v>
       </c>
       <c r="D174" s="23" t="s">
-        <v>744</v>
+        <v>739</v>
       </c>
       <c r="E174" s="23" t="s">
-        <v>745</v>
+        <v>740</v>
       </c>
       <c r="F174" s="23" t="s">
-        <v>746</v>
+        <v>741</v>
       </c>
       <c r="G174" s="23" t="s">
-        <v>99</v>
+        <v>47</v>
       </c>
       <c r="H174" s="23" t="s">
-        <v>747</v>
+        <v>742</v>
       </c>
       <c r="I174" s="23"/>
       <c r="J174" s="23"/>
@@ -8267,25 +8365,25 @@
     <row r="175" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A175" s="21"/>
       <c r="B175" s="22" t="s">
-        <v>748</v>
+        <v>743</v>
       </c>
       <c r="C175" s="21" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D175" s="23" t="s">
-        <v>749</v>
+        <v>744</v>
       </c>
       <c r="E175" s="23" t="s">
-        <v>750</v>
+        <v>745</v>
       </c>
       <c r="F175" s="23" t="s">
-        <v>751</v>
+        <v>746</v>
       </c>
       <c r="G175" s="23" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="H175" s="23" t="s">
-        <v>752</v>
+        <v>747</v>
       </c>
       <c r="I175" s="23"/>
       <c r="J175" s="23"/>
@@ -8296,26 +8394,24 @@
     </row>
     <row r="176" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A176" s="21"/>
-      <c r="B176" s="22" t="s">
-        <v>753</v>
-      </c>
+      <c r="B176" s="21"/>
       <c r="C176" s="21" t="s">
         <v>39</v>
       </c>
       <c r="D176" s="23" t="s">
-        <v>754</v>
+        <v>748</v>
       </c>
       <c r="E176" s="23" t="s">
-        <v>755</v>
+        <v>749</v>
       </c>
       <c r="F176" s="23" t="s">
-        <v>756</v>
+        <v>750</v>
       </c>
       <c r="G176" s="23" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="H176" s="23" t="s">
-        <v>757</v>
+        <v>751</v>
       </c>
       <c r="I176" s="23"/>
       <c r="J176" s="23"/>
@@ -8326,26 +8422,24 @@
     </row>
     <row r="177" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A177" s="21"/>
-      <c r="B177" s="22" t="s">
-        <v>758</v>
-      </c>
+      <c r="B177" s="21"/>
       <c r="C177" s="21" t="s">
         <v>39</v>
       </c>
       <c r="D177" s="23" t="s">
-        <v>759</v>
+        <v>752</v>
       </c>
       <c r="E177" s="23" t="s">
-        <v>760</v>
+        <v>753</v>
       </c>
       <c r="F177" s="23" t="s">
-        <v>761</v>
+        <v>754</v>
       </c>
       <c r="G177" s="23" t="s">
-        <v>99</v>
+        <v>47</v>
       </c>
       <c r="H177" s="23" t="s">
-        <v>762</v>
+        <v>755</v>
       </c>
       <c r="I177" s="23"/>
       <c r="J177" s="23"/>
@@ -8354,52 +8448,58 @@
       <c r="M177" s="23"/>
       <c r="N177" s="23"/>
     </row>
-    <row r="178" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A178" s="20" t="s">
-        <v>763</v>
-      </c>
-      <c r="B178" s="20" t="s">
-        <v>764</v>
-      </c>
-      <c r="C178" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="D178" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="E178" s="20"/>
-      <c r="F178" s="20"/>
-      <c r="G178" s="20"/>
-      <c r="H178" s="20"/>
-      <c r="I178" s="20"/>
-      <c r="J178" s="20"/>
-      <c r="K178" s="20"/>
-      <c r="L178" s="20"/>
-      <c r="M178" s="20"/>
-      <c r="N178" s="20"/>
+    <row r="178" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A178" s="21"/>
+      <c r="B178" s="22" t="s">
+        <v>756</v>
+      </c>
+      <c r="C178" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="D178" s="23" t="s">
+        <v>757</v>
+      </c>
+      <c r="E178" s="23" t="s">
+        <v>758</v>
+      </c>
+      <c r="F178" s="23" t="s">
+        <v>759</v>
+      </c>
+      <c r="G178" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H178" s="23" t="s">
+        <v>760</v>
+      </c>
+      <c r="I178" s="23"/>
+      <c r="J178" s="23"/>
+      <c r="K178" s="23"/>
+      <c r="L178" s="23"/>
+      <c r="M178" s="23"/>
+      <c r="N178" s="23"/>
     </row>
     <row r="179" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A179" s="21"/>
       <c r="B179" s="22" t="s">
+        <v>761</v>
+      </c>
+      <c r="C179" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="D179" s="23" t="s">
+        <v>762</v>
+      </c>
+      <c r="E179" s="23" t="s">
+        <v>763</v>
+      </c>
+      <c r="F179" s="23" t="s">
+        <v>764</v>
+      </c>
+      <c r="G179" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H179" s="23" t="s">
         <v>765</v>
-      </c>
-      <c r="C179" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="D179" s="23" t="s">
-        <v>766</v>
-      </c>
-      <c r="E179" s="23" t="s">
-        <v>767</v>
-      </c>
-      <c r="F179" s="23" t="s">
-        <v>768</v>
-      </c>
-      <c r="G179" s="23" t="s">
-        <v>99</v>
-      </c>
-      <c r="H179" s="23" t="s">
-        <v>769</v>
       </c>
       <c r="I179" s="23"/>
       <c r="J179" s="23"/>
@@ -8412,22 +8512,22 @@
       <c r="A180" s="21"/>
       <c r="B180" s="21"/>
       <c r="C180" s="21" t="s">
-        <v>39</v>
+        <v>90</v>
       </c>
       <c r="D180" s="23" t="s">
-        <v>770</v>
+        <v>766</v>
       </c>
       <c r="E180" s="23" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="F180" s="23" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="G180" s="23" t="s">
         <v>47</v>
       </c>
       <c r="H180" s="23" t="s">
-        <v>773</v>
+        <v>769</v>
       </c>
       <c r="I180" s="23"/>
       <c r="J180" s="23"/>
@@ -8438,24 +8538,26 @@
     </row>
     <row r="181" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A181" s="21"/>
-      <c r="B181" s="21"/>
+      <c r="B181" s="22" t="s">
+        <v>770</v>
+      </c>
       <c r="C181" s="21" t="s">
-        <v>90</v>
+        <v>33</v>
       </c>
       <c r="D181" s="23" t="s">
+        <v>771</v>
+      </c>
+      <c r="E181" s="23" t="s">
+        <v>772</v>
+      </c>
+      <c r="F181" s="23" t="s">
+        <v>773</v>
+      </c>
+      <c r="G181" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H181" s="23" t="s">
         <v>774</v>
-      </c>
-      <c r="E181" s="23" t="s">
-        <v>775</v>
-      </c>
-      <c r="F181" s="23" t="s">
-        <v>776</v>
-      </c>
-      <c r="G181" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H181" s="23" t="s">
-        <v>777</v>
       </c>
       <c r="I181" s="23"/>
       <c r="J181" s="23"/>
@@ -8464,52 +8566,56 @@
       <c r="M181" s="23"/>
       <c r="N181" s="23"/>
     </row>
-    <row r="182" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A182" s="20" t="s">
+    <row r="182" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A182" s="21"/>
+      <c r="B182" s="22" t="s">
+        <v>775</v>
+      </c>
+      <c r="C182" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="D182" s="23" t="s">
+        <v>776</v>
+      </c>
+      <c r="E182" s="23" t="s">
+        <v>777</v>
+      </c>
+      <c r="F182" s="23" t="s">
         <v>778</v>
       </c>
-      <c r="B182" s="20" t="s">
+      <c r="G182" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H182" s="23" t="s">
         <v>779</v>
       </c>
-      <c r="C182" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="D182" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="E182" s="20"/>
-      <c r="F182" s="20"/>
-      <c r="G182" s="20"/>
-      <c r="H182" s="20"/>
-      <c r="I182" s="20"/>
-      <c r="J182" s="20"/>
-      <c r="K182" s="20"/>
-      <c r="L182" s="20"/>
-      <c r="M182" s="20"/>
-      <c r="N182" s="20"/>
+      <c r="I182" s="23"/>
+      <c r="J182" s="23"/>
+      <c r="K182" s="23"/>
+      <c r="L182" s="23"/>
+      <c r="M182" s="23"/>
+      <c r="N182" s="23"/>
     </row>
     <row r="183" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A183" s="21"/>
-      <c r="B183" s="22" t="s">
+      <c r="B183" s="21"/>
+      <c r="C183" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D183" s="23" t="s">
         <v>780</v>
       </c>
-      <c r="C183" s="21" t="s">
-        <v>90</v>
-      </c>
-      <c r="D183" s="23" t="s">
+      <c r="E183" s="23" t="s">
         <v>781</v>
       </c>
-      <c r="E183" s="23" t="s">
+      <c r="F183" s="23" t="s">
         <v>782</v>
       </c>
-      <c r="F183" s="23" t="s">
+      <c r="G183" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="H183" s="23" t="s">
         <v>783</v>
-      </c>
-      <c r="G183" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H183" s="23" t="s">
-        <v>784</v>
       </c>
       <c r="I183" s="23"/>
       <c r="J183" s="23"/>
@@ -8520,9 +8626,11 @@
     </row>
     <row r="184" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A184" s="21"/>
-      <c r="B184" s="21"/>
+      <c r="B184" s="22" t="s">
+        <v>784</v>
+      </c>
       <c r="C184" s="21" t="s">
-        <v>90</v>
+        <v>39</v>
       </c>
       <c r="D184" s="23" t="s">
         <v>785</v>
@@ -8534,7 +8642,7 @@
         <v>787</v>
       </c>
       <c r="G184" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H184" s="23" t="s">
         <v>788</v>
@@ -8548,24 +8656,26 @@
     </row>
     <row r="185" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A185" s="21"/>
-      <c r="B185" s="21"/>
+      <c r="B185" s="22" t="s">
+        <v>789</v>
+      </c>
       <c r="C185" s="21" t="s">
-        <v>90</v>
+        <v>39</v>
       </c>
       <c r="D185" s="23" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="E185" s="23" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="F185" s="23" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="G185" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H185" s="23" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="I185" s="23"/>
       <c r="J185" s="23"/>
@@ -8576,24 +8686,26 @@
     </row>
     <row r="186" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A186" s="21"/>
-      <c r="B186" s="21"/>
+      <c r="B186" s="22" t="s">
+        <v>794</v>
+      </c>
       <c r="C186" s="21" t="s">
-        <v>90</v>
+        <v>39</v>
       </c>
       <c r="D186" s="23" t="s">
-        <v>793</v>
+        <v>795</v>
       </c>
       <c r="E186" s="23" t="s">
-        <v>794</v>
+        <v>796</v>
       </c>
       <c r="F186" s="23" t="s">
-        <v>795</v>
+        <v>797</v>
       </c>
       <c r="G186" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H186" s="23" t="s">
-        <v>796</v>
+        <v>798</v>
       </c>
       <c r="I186" s="23"/>
       <c r="J186" s="23"/>
@@ -8602,41 +8714,37 @@
       <c r="M186" s="23"/>
       <c r="N186" s="23"/>
     </row>
-    <row r="187" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A187" s="21"/>
-      <c r="B187" s="22" t="s">
-        <v>797</v>
-      </c>
-      <c r="C187" s="21" t="s">
-        <v>90</v>
-      </c>
-      <c r="D187" s="23" t="s">
-        <v>798</v>
-      </c>
-      <c r="E187" s="23" t="s">
+    <row r="187" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A187" s="20" t="s">
         <v>799</v>
       </c>
-      <c r="F187" s="23" t="s">
+      <c r="B187" s="20" t="s">
         <v>800</v>
       </c>
-      <c r="G187" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H187" s="23" t="s">
-        <v>801</v>
-      </c>
-      <c r="I187" s="23"/>
-      <c r="J187" s="23"/>
-      <c r="K187" s="23"/>
-      <c r="L187" s="23"/>
-      <c r="M187" s="23"/>
-      <c r="N187" s="23"/>
+      <c r="C187" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="D187" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="E187" s="20"/>
+      <c r="F187" s="20"/>
+      <c r="G187" s="20"/>
+      <c r="H187" s="20"/>
+      <c r="I187" s="20"/>
+      <c r="J187" s="20"/>
+      <c r="K187" s="20"/>
+      <c r="L187" s="20"/>
+      <c r="M187" s="20"/>
+      <c r="N187" s="20"/>
     </row>
     <row r="188" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A188" s="21"/>
-      <c r="B188" s="21"/>
+      <c r="B188" s="22" t="s">
+        <v>801</v>
+      </c>
       <c r="C188" s="21" t="s">
-        <v>90</v>
+        <v>39</v>
       </c>
       <c r="D188" s="23" t="s">
         <v>802</v>
@@ -8648,7 +8756,7 @@
         <v>804</v>
       </c>
       <c r="G188" s="23" t="s">
-        <v>47</v>
+        <v>99</v>
       </c>
       <c r="H188" s="23" t="s">
         <v>805</v>
@@ -8662,26 +8770,24 @@
     </row>
     <row r="189" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A189" s="21"/>
-      <c r="B189" s="22" t="s">
+      <c r="B189" s="21"/>
+      <c r="C189" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D189" s="23" t="s">
         <v>806</v>
       </c>
-      <c r="C189" s="21" t="s">
-        <v>90</v>
-      </c>
-      <c r="D189" s="23" t="s">
+      <c r="E189" s="23" t="s">
         <v>807</v>
       </c>
-      <c r="E189" s="23" t="s">
+      <c r="F189" s="23" t="s">
         <v>808</v>
-      </c>
-      <c r="F189" s="23" t="s">
-        <v>809</v>
       </c>
       <c r="G189" s="23" t="s">
         <v>47</v>
       </c>
       <c r="H189" s="23" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="I189" s="23"/>
       <c r="J189" s="23"/>
@@ -8690,82 +8796,80 @@
       <c r="M189" s="23"/>
       <c r="N189" s="23"/>
     </row>
-    <row r="190" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A190" s="20" t="s">
+    <row r="190" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A190" s="21"/>
+      <c r="B190" s="21"/>
+      <c r="C190" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="D190" s="23" t="s">
+        <v>810</v>
+      </c>
+      <c r="E190" s="23" t="s">
         <v>811</v>
       </c>
-      <c r="B190" s="20" t="s">
+      <c r="F190" s="23" t="s">
         <v>812</v>
       </c>
-      <c r="C190" s="20" t="s">
+      <c r="G190" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H190" s="23" t="s">
+        <v>813</v>
+      </c>
+      <c r="I190" s="23"/>
+      <c r="J190" s="23"/>
+      <c r="K190" s="23"/>
+      <c r="L190" s="23"/>
+      <c r="M190" s="23"/>
+      <c r="N190" s="23"/>
+    </row>
+    <row r="191" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A191" s="20" t="s">
+        <v>814</v>
+      </c>
+      <c r="B191" s="20" t="s">
+        <v>815</v>
+      </c>
+      <c r="C191" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="D190" s="20" t="s">
+      <c r="D191" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="E190" s="20"/>
-      <c r="F190" s="20"/>
-      <c r="G190" s="20"/>
-      <c r="H190" s="20"/>
-      <c r="I190" s="20"/>
-      <c r="J190" s="20"/>
-      <c r="K190" s="20"/>
-      <c r="L190" s="20"/>
-      <c r="M190" s="20"/>
-      <c r="N190" s="20"/>
-    </row>
-    <row r="191" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A191" s="21"/>
-      <c r="B191" s="22" t="s">
-        <v>813</v>
-      </c>
-      <c r="C191" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D191" s="23" t="s">
-        <v>814</v>
-      </c>
-      <c r="E191" s="23" t="s">
-        <v>815</v>
-      </c>
-      <c r="F191" s="23" t="s">
-        <v>816</v>
-      </c>
-      <c r="G191" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H191" s="23" t="s">
-        <v>817</v>
-      </c>
-      <c r="I191" s="23"/>
-      <c r="J191" s="23"/>
-      <c r="K191" s="23"/>
-      <c r="L191" s="23"/>
-      <c r="M191" s="23"/>
-      <c r="N191" s="23"/>
+      <c r="E191" s="20"/>
+      <c r="F191" s="20"/>
+      <c r="G191" s="20"/>
+      <c r="H191" s="20"/>
+      <c r="I191" s="20"/>
+      <c r="J191" s="20"/>
+      <c r="K191" s="20"/>
+      <c r="L191" s="20"/>
+      <c r="M191" s="20"/>
+      <c r="N191" s="20"/>
     </row>
     <row r="192" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A192" s="21"/>
       <c r="B192" s="22" t="s">
+        <v>816</v>
+      </c>
+      <c r="C192" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="D192" s="23" t="s">
+        <v>817</v>
+      </c>
+      <c r="E192" s="23" t="s">
         <v>818</v>
       </c>
-      <c r="C192" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D192" s="23" t="s">
+      <c r="F192" s="23" t="s">
         <v>819</v>
       </c>
-      <c r="E192" s="23" t="s">
+      <c r="G192" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H192" s="23" t="s">
         <v>820</v>
-      </c>
-      <c r="F192" s="23" t="s">
-        <v>821</v>
-      </c>
-      <c r="G192" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H192" s="23" t="s">
-        <v>822</v>
       </c>
       <c r="I192" s="23"/>
       <c r="J192" s="23"/>
@@ -8776,26 +8880,24 @@
     </row>
     <row r="193" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A193" s="21"/>
-      <c r="B193" s="22" t="s">
+      <c r="B193" s="21"/>
+      <c r="C193" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="D193" s="23" t="s">
+        <v>821</v>
+      </c>
+      <c r="E193" s="23" t="s">
+        <v>822</v>
+      </c>
+      <c r="F193" s="23" t="s">
         <v>823</v>
       </c>
-      <c r="C193" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D193" s="23" t="s">
+      <c r="G193" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H193" s="23" t="s">
         <v>824</v>
-      </c>
-      <c r="E193" s="23" t="s">
-        <v>825</v>
-      </c>
-      <c r="F193" s="23" t="s">
-        <v>826</v>
-      </c>
-      <c r="G193" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H193" s="23" t="s">
-        <v>827</v>
       </c>
       <c r="I193" s="23"/>
       <c r="J193" s="23"/>
@@ -8808,22 +8910,22 @@
       <c r="A194" s="21"/>
       <c r="B194" s="21"/>
       <c r="C194" s="21" t="s">
-        <v>39</v>
+        <v>90</v>
       </c>
       <c r="D194" s="23" t="s">
+        <v>825</v>
+      </c>
+      <c r="E194" s="23" t="s">
+        <v>826</v>
+      </c>
+      <c r="F194" s="23" t="s">
+        <v>827</v>
+      </c>
+      <c r="G194" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H194" s="23" t="s">
         <v>828</v>
-      </c>
-      <c r="E194" s="23" t="s">
-        <v>829</v>
-      </c>
-      <c r="F194" s="23" t="s">
-        <v>830</v>
-      </c>
-      <c r="G194" s="23" t="s">
-        <v>99</v>
-      </c>
-      <c r="H194" s="23" t="s">
-        <v>831</v>
       </c>
       <c r="I194" s="23"/>
       <c r="J194" s="23"/>
@@ -8834,26 +8936,24 @@
     </row>
     <row r="195" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A195" s="21"/>
-      <c r="B195" s="22" t="s">
+      <c r="B195" s="21"/>
+      <c r="C195" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="D195" s="23" t="s">
+        <v>829</v>
+      </c>
+      <c r="E195" s="23" t="s">
+        <v>830</v>
+      </c>
+      <c r="F195" s="23" t="s">
+        <v>831</v>
+      </c>
+      <c r="G195" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H195" s="23" t="s">
         <v>832</v>
-      </c>
-      <c r="C195" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D195" s="23" t="s">
-        <v>833</v>
-      </c>
-      <c r="E195" s="23" t="s">
-        <v>834</v>
-      </c>
-      <c r="F195" s="23" t="s">
-        <v>835</v>
-      </c>
-      <c r="G195" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H195" s="23" t="s">
-        <v>836</v>
       </c>
       <c r="I195" s="23"/>
       <c r="J195" s="23"/>
@@ -8864,24 +8964,26 @@
     </row>
     <row r="196" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A196" s="21"/>
-      <c r="B196" s="21"/>
+      <c r="B196" s="22" t="s">
+        <v>833</v>
+      </c>
       <c r="C196" s="21" t="s">
-        <v>39</v>
+        <v>90</v>
       </c>
       <c r="D196" s="23" t="s">
+        <v>834</v>
+      </c>
+      <c r="E196" s="23" t="s">
+        <v>835</v>
+      </c>
+      <c r="F196" s="23" t="s">
+        <v>836</v>
+      </c>
+      <c r="G196" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H196" s="23" t="s">
         <v>837</v>
-      </c>
-      <c r="E196" s="23" t="s">
-        <v>838</v>
-      </c>
-      <c r="F196" s="23" t="s">
-        <v>830</v>
-      </c>
-      <c r="G196" s="23" t="s">
-        <v>99</v>
-      </c>
-      <c r="H196" s="23" t="s">
-        <v>839</v>
       </c>
       <c r="I196" s="23"/>
       <c r="J196" s="23"/>
@@ -8890,29 +8992,33 @@
       <c r="M196" s="23"/>
       <c r="N196" s="23"/>
     </row>
-    <row r="197" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A197" s="20" t="s">
+    <row r="197" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A197" s="21"/>
+      <c r="B197" s="21"/>
+      <c r="C197" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="D197" s="23" t="s">
+        <v>838</v>
+      </c>
+      <c r="E197" s="23" t="s">
+        <v>839</v>
+      </c>
+      <c r="F197" s="23" t="s">
         <v>840</v>
       </c>
-      <c r="B197" s="20" t="s">
+      <c r="G197" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H197" s="23" t="s">
         <v>841</v>
       </c>
-      <c r="C197" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="D197" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="E197" s="20"/>
-      <c r="F197" s="20"/>
-      <c r="G197" s="20"/>
-      <c r="H197" s="20"/>
-      <c r="I197" s="20"/>
-      <c r="J197" s="20"/>
-      <c r="K197" s="20"/>
-      <c r="L197" s="20"/>
-      <c r="M197" s="20"/>
-      <c r="N197" s="20"/>
+      <c r="I197" s="23"/>
+      <c r="J197" s="23"/>
+      <c r="K197" s="23"/>
+      <c r="L197" s="23"/>
+      <c r="M197" s="23"/>
+      <c r="N197" s="23"/>
     </row>
     <row r="198" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A198" s="21"/>
@@ -8920,7 +9026,7 @@
         <v>842</v>
       </c>
       <c r="C198" s="21" t="s">
-        <v>33</v>
+        <v>90</v>
       </c>
       <c r="D198" s="23" t="s">
         <v>843</v>
@@ -8932,7 +9038,7 @@
         <v>845</v>
       </c>
       <c r="G198" s="23" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="H198" s="23" t="s">
         <v>846</v>
@@ -8944,54 +9050,52 @@
       <c r="M198" s="23"/>
       <c r="N198" s="23"/>
     </row>
-    <row r="199" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A199" s="21"/>
-      <c r="B199" s="21"/>
-      <c r="C199" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="D199" s="23" t="s">
+    <row r="199" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A199" s="20" t="s">
         <v>847</v>
       </c>
-      <c r="E199" s="23" t="s">
+      <c r="B199" s="20" t="s">
         <v>848</v>
       </c>
-      <c r="F199" s="23" t="s">
-        <v>849</v>
-      </c>
-      <c r="G199" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H199" s="23" t="s">
-        <v>850</v>
-      </c>
-      <c r="I199" s="23"/>
-      <c r="J199" s="23"/>
-      <c r="K199" s="23"/>
-      <c r="L199" s="23"/>
-      <c r="M199" s="23"/>
-      <c r="N199" s="23"/>
+      <c r="C199" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="D199" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="E199" s="20"/>
+      <c r="F199" s="20"/>
+      <c r="G199" s="20"/>
+      <c r="H199" s="20"/>
+      <c r="I199" s="20"/>
+      <c r="J199" s="20"/>
+      <c r="K199" s="20"/>
+      <c r="L199" s="20"/>
+      <c r="M199" s="20"/>
+      <c r="N199" s="20"/>
     </row>
     <row r="200" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A200" s="21"/>
-      <c r="B200" s="21"/>
+      <c r="B200" s="22" t="s">
+        <v>849</v>
+      </c>
       <c r="C200" s="21" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D200" s="23" t="s">
+        <v>850</v>
+      </c>
+      <c r="E200" s="23" t="s">
         <v>851</v>
       </c>
-      <c r="E200" s="23" t="s">
+      <c r="F200" s="23" t="s">
         <v>852</v>
       </c>
-      <c r="F200" s="23" t="s">
+      <c r="G200" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H200" s="23" t="s">
         <v>853</v>
-      </c>
-      <c r="G200" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H200" s="23" t="s">
-        <v>854</v>
       </c>
       <c r="I200" s="23"/>
       <c r="J200" s="23"/>
@@ -9002,9 +9106,11 @@
     </row>
     <row r="201" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A201" s="21"/>
-      <c r="B201" s="21"/>
+      <c r="B201" s="22" t="s">
+        <v>854</v>
+      </c>
       <c r="C201" s="21" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D201" s="23" t="s">
         <v>855</v>
@@ -9016,7 +9122,7 @@
         <v>857</v>
       </c>
       <c r="G201" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H201" s="23" t="s">
         <v>858</v>
@@ -9030,21 +9136,23 @@
     </row>
     <row r="202" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A202" s="21"/>
-      <c r="B202" s="21"/>
+      <c r="B202" s="22" t="s">
+        <v>859</v>
+      </c>
       <c r="C202" s="21" t="s">
-        <v>90</v>
+        <v>33</v>
       </c>
       <c r="D202" s="23" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="E202" s="23" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="F202" s="23" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="G202" s="23" t="s">
-        <v>862</v>
+        <v>37</v>
       </c>
       <c r="H202" s="23" t="s">
         <v>863</v>
@@ -9058,26 +9166,24 @@
     </row>
     <row r="203" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A203" s="21"/>
-      <c r="B203" s="22" t="s">
+      <c r="B203" s="21"/>
+      <c r="C203" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D203" s="23" t="s">
         <v>864</v>
       </c>
-      <c r="C203" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D203" s="23" t="s">
+      <c r="E203" s="23" t="s">
         <v>865</v>
       </c>
-      <c r="E203" s="23" t="s">
+      <c r="F203" s="23" t="s">
         <v>866</v>
       </c>
-      <c r="F203" s="23" t="s">
+      <c r="G203" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="H203" s="23" t="s">
         <v>867</v>
-      </c>
-      <c r="G203" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H203" s="23" t="s">
-        <v>868</v>
       </c>
       <c r="I203" s="23"/>
       <c r="J203" s="23"/>
@@ -9089,25 +9195,25 @@
     <row r="204" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A204" s="21"/>
       <c r="B204" s="22" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="C204" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D204" s="23" t="s">
+        <v>869</v>
+      </c>
+      <c r="E204" s="23" t="s">
         <v>870</v>
       </c>
-      <c r="E204" s="23" t="s">
+      <c r="F204" s="23" t="s">
         <v>871</v>
       </c>
-      <c r="F204" s="23" t="s">
+      <c r="G204" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H204" s="23" t="s">
         <v>872</v>
-      </c>
-      <c r="G204" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H204" s="23" t="s">
-        <v>873</v>
       </c>
       <c r="I204" s="23"/>
       <c r="J204" s="23"/>
@@ -9116,80 +9222,80 @@
       <c r="M204" s="23"/>
       <c r="N204" s="23"/>
     </row>
-    <row r="205" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A205" s="20" t="s">
+    <row r="205" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A205" s="21"/>
+      <c r="B205" s="21"/>
+      <c r="C205" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D205" s="23" t="s">
+        <v>873</v>
+      </c>
+      <c r="E205" s="23" t="s">
         <v>874</v>
       </c>
-      <c r="B205" s="20" t="s">
+      <c r="F205" s="23" t="s">
+        <v>866</v>
+      </c>
+      <c r="G205" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="H205" s="23" t="s">
         <v>875</v>
       </c>
-      <c r="C205" s="20" t="s">
+      <c r="I205" s="23"/>
+      <c r="J205" s="23"/>
+      <c r="K205" s="23"/>
+      <c r="L205" s="23"/>
+      <c r="M205" s="23"/>
+      <c r="N205" s="23"/>
+    </row>
+    <row r="206" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A206" s="20" t="s">
+        <v>876</v>
+      </c>
+      <c r="B206" s="20" t="s">
+        <v>877</v>
+      </c>
+      <c r="C206" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="D205" s="20" t="s">
+      <c r="D206" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="E205" s="20"/>
-      <c r="F205" s="20"/>
-      <c r="G205" s="20"/>
-      <c r="H205" s="20"/>
-      <c r="I205" s="20"/>
-      <c r="J205" s="20"/>
-      <c r="K205" s="20"/>
-      <c r="L205" s="20"/>
-      <c r="M205" s="20"/>
-      <c r="N205" s="20"/>
-    </row>
-    <row r="206" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A206" s="21"/>
-      <c r="B206" s="22" t="s">
-        <v>876</v>
-      </c>
-      <c r="C206" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D206" s="23" t="s">
-        <v>877</v>
-      </c>
-      <c r="E206" s="23" t="s">
-        <v>878</v>
-      </c>
-      <c r="F206" s="23" t="s">
-        <v>879</v>
-      </c>
-      <c r="G206" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H206" s="23" t="s">
-        <v>880</v>
-      </c>
-      <c r="I206" s="23"/>
-      <c r="J206" s="23"/>
-      <c r="K206" s="23"/>
-      <c r="L206" s="23"/>
-      <c r="M206" s="23"/>
-      <c r="N206" s="23"/>
+      <c r="E206" s="20"/>
+      <c r="F206" s="20"/>
+      <c r="G206" s="20"/>
+      <c r="H206" s="20"/>
+      <c r="I206" s="20"/>
+      <c r="J206" s="20"/>
+      <c r="K206" s="20"/>
+      <c r="L206" s="20"/>
+      <c r="M206" s="20"/>
+      <c r="N206" s="20"/>
     </row>
     <row r="207" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A207" s="21"/>
-      <c r="B207" s="21"/>
+      <c r="B207" s="22" t="s">
+        <v>878</v>
+      </c>
       <c r="C207" s="21" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D207" s="23" t="s">
+        <v>879</v>
+      </c>
+      <c r="E207" s="23" t="s">
+        <v>880</v>
+      </c>
+      <c r="F207" s="23" t="s">
         <v>881</v>
       </c>
-      <c r="E207" s="23" t="s">
+      <c r="G207" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H207" s="23" t="s">
         <v>882</v>
-      </c>
-      <c r="F207" s="23" t="s">
-        <v>883</v>
-      </c>
-      <c r="G207" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H207" s="23" t="s">
-        <v>884</v>
       </c>
       <c r="I207" s="23"/>
       <c r="J207" s="23"/>
@@ -9205,19 +9311,19 @@
         <v>39</v>
       </c>
       <c r="D208" s="23" t="s">
+        <v>883</v>
+      </c>
+      <c r="E208" s="23" t="s">
+        <v>884</v>
+      </c>
+      <c r="F208" s="23" t="s">
         <v>885</v>
-      </c>
-      <c r="E208" s="23" t="s">
-        <v>886</v>
-      </c>
-      <c r="F208" s="23" t="s">
-        <v>887</v>
       </c>
       <c r="G208" s="23" t="s">
         <v>47</v>
       </c>
       <c r="H208" s="23" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
       <c r="I208" s="23"/>
       <c r="J208" s="23"/>
@@ -9228,26 +9334,24 @@
     </row>
     <row r="209" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A209" s="21"/>
-      <c r="B209" s="22" t="s">
+      <c r="B209" s="21"/>
+      <c r="C209" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D209" s="23" t="s">
+        <v>887</v>
+      </c>
+      <c r="E209" s="23" t="s">
+        <v>888</v>
+      </c>
+      <c r="F209" s="23" t="s">
         <v>889</v>
       </c>
-      <c r="C209" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D209" s="23" t="s">
+      <c r="G209" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H209" s="23" t="s">
         <v>890</v>
-      </c>
-      <c r="E209" s="23" t="s">
-        <v>891</v>
-      </c>
-      <c r="F209" s="23" t="s">
-        <v>892</v>
-      </c>
-      <c r="G209" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H209" s="23" t="s">
-        <v>893</v>
       </c>
       <c r="I209" s="23"/>
       <c r="J209" s="23"/>
@@ -9256,52 +9360,54 @@
       <c r="M209" s="23"/>
       <c r="N209" s="23"/>
     </row>
-    <row r="210" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A210" s="20" t="s">
+    <row r="210" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A210" s="21"/>
+      <c r="B210" s="21"/>
+      <c r="C210" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D210" s="23" t="s">
+        <v>891</v>
+      </c>
+      <c r="E210" s="23" t="s">
+        <v>892</v>
+      </c>
+      <c r="F210" s="23" t="s">
+        <v>893</v>
+      </c>
+      <c r="G210" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H210" s="23" t="s">
         <v>894</v>
       </c>
-      <c r="B210" s="20" t="s">
-        <v>895</v>
-      </c>
-      <c r="C210" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="D210" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="E210" s="20"/>
-      <c r="F210" s="20"/>
-      <c r="G210" s="20"/>
-      <c r="H210" s="20"/>
-      <c r="I210" s="20"/>
-      <c r="J210" s="20"/>
-      <c r="K210" s="20"/>
-      <c r="L210" s="20"/>
-      <c r="M210" s="20"/>
-      <c r="N210" s="20"/>
+      <c r="I210" s="23"/>
+      <c r="J210" s="23"/>
+      <c r="K210" s="23"/>
+      <c r="L210" s="23"/>
+      <c r="M210" s="23"/>
+      <c r="N210" s="23"/>
     </row>
     <row r="211" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A211" s="21"/>
-      <c r="B211" s="22" t="s">
+      <c r="B211" s="21"/>
+      <c r="C211" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="D211" s="23" t="s">
+        <v>895</v>
+      </c>
+      <c r="E211" s="23" t="s">
         <v>896</v>
       </c>
-      <c r="C211" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D211" s="23" t="s">
+      <c r="F211" s="23" t="s">
         <v>897</v>
       </c>
-      <c r="E211" s="23" t="s">
+      <c r="G211" s="23" t="s">
         <v>898</v>
       </c>
-      <c r="F211" s="23" t="s">
+      <c r="H211" s="23" t="s">
         <v>899</v>
-      </c>
-      <c r="G211" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="H211" s="23" t="s">
-        <v>900</v>
       </c>
       <c r="I211" s="23"/>
       <c r="J211" s="23"/>
@@ -9312,9 +9418,11 @@
     </row>
     <row r="212" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A212" s="21"/>
-      <c r="B212" s="21"/>
+      <c r="B212" s="22" t="s">
+        <v>900</v>
+      </c>
       <c r="C212" s="21" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D212" s="23" t="s">
         <v>901</v>
@@ -9340,24 +9448,26 @@
     </row>
     <row r="213" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A213" s="21"/>
-      <c r="B213" s="21"/>
+      <c r="B213" s="22" t="s">
+        <v>905</v>
+      </c>
       <c r="C213" s="21" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D213" s="23" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="E213" s="23" t="s">
-        <v>906</v>
+        <v>907</v>
       </c>
       <c r="F213" s="23" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="G213" s="23" t="s">
         <v>47</v>
       </c>
       <c r="H213" s="23" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="I213" s="23"/>
       <c r="J213" s="23"/>
@@ -9368,10 +9478,10 @@
     </row>
     <row r="214" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A214" s="20" t="s">
-        <v>909</v>
+        <v>910</v>
       </c>
       <c r="B214" s="20" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="C214" s="20" t="s">
         <v>30</v>
@@ -9393,25 +9503,25 @@
     <row r="215" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A215" s="21"/>
       <c r="B215" s="22" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="C215" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D215" s="23" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="E215" s="23" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="F215" s="23" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="G215" s="23" t="s">
-        <v>99</v>
+        <v>37</v>
       </c>
       <c r="H215" s="23" t="s">
-        <v>915</v>
+        <v>916</v>
       </c>
       <c r="I215" s="23"/>
       <c r="J215" s="23"/>
@@ -9427,19 +9537,19 @@
         <v>39</v>
       </c>
       <c r="D216" s="23" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="E216" s="23" t="s">
-        <v>917</v>
+        <v>918</v>
       </c>
       <c r="F216" s="23" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
       <c r="G216" s="23" t="s">
         <v>47</v>
       </c>
       <c r="H216" s="23" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="I216" s="23"/>
       <c r="J216" s="23"/>
@@ -9455,19 +9565,19 @@
         <v>39</v>
       </c>
       <c r="D217" s="23" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
       <c r="E217" s="23" t="s">
-        <v>921</v>
+        <v>922</v>
       </c>
       <c r="F217" s="23" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="G217" s="23" t="s">
         <v>47</v>
       </c>
       <c r="H217" s="23" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
       <c r="I217" s="23"/>
       <c r="J217" s="23"/>
@@ -9475,6 +9585,256 @@
       <c r="L217" s="23"/>
       <c r="M217" s="23"/>
       <c r="N217" s="23"/>
+    </row>
+    <row r="218" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A218" s="21"/>
+      <c r="B218" s="22" t="s">
+        <v>925</v>
+      </c>
+      <c r="C218" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="D218" s="23" t="s">
+        <v>926</v>
+      </c>
+      <c r="E218" s="23" t="s">
+        <v>927</v>
+      </c>
+      <c r="F218" s="23" t="s">
+        <v>928</v>
+      </c>
+      <c r="G218" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H218" s="23" t="s">
+        <v>929</v>
+      </c>
+      <c r="I218" s="23"/>
+      <c r="J218" s="23"/>
+      <c r="K218" s="23"/>
+      <c r="L218" s="23"/>
+      <c r="M218" s="23"/>
+      <c r="N218" s="23"/>
+    </row>
+    <row r="219" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A219" s="20" t="s">
+        <v>930</v>
+      </c>
+      <c r="B219" s="20" t="s">
+        <v>931</v>
+      </c>
+      <c r="C219" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="D219" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="E219" s="20"/>
+      <c r="F219" s="20"/>
+      <c r="G219" s="20"/>
+      <c r="H219" s="20"/>
+      <c r="I219" s="20"/>
+      <c r="J219" s="20"/>
+      <c r="K219" s="20"/>
+      <c r="L219" s="20"/>
+      <c r="M219" s="20"/>
+      <c r="N219" s="20"/>
+    </row>
+    <row r="220" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A220" s="21"/>
+      <c r="B220" s="22" t="s">
+        <v>932</v>
+      </c>
+      <c r="C220" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="D220" s="23" t="s">
+        <v>933</v>
+      </c>
+      <c r="E220" s="23" t="s">
+        <v>934</v>
+      </c>
+      <c r="F220" s="23" t="s">
+        <v>935</v>
+      </c>
+      <c r="G220" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H220" s="23" t="s">
+        <v>936</v>
+      </c>
+      <c r="I220" s="23"/>
+      <c r="J220" s="23"/>
+      <c r="K220" s="23"/>
+      <c r="L220" s="23"/>
+      <c r="M220" s="23"/>
+      <c r="N220" s="23"/>
+    </row>
+    <row r="221" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A221" s="21"/>
+      <c r="B221" s="21"/>
+      <c r="C221" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D221" s="23" t="s">
+        <v>937</v>
+      </c>
+      <c r="E221" s="23" t="s">
+        <v>938</v>
+      </c>
+      <c r="F221" s="23" t="s">
+        <v>939</v>
+      </c>
+      <c r="G221" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H221" s="23" t="s">
+        <v>940</v>
+      </c>
+      <c r="I221" s="23"/>
+      <c r="J221" s="23"/>
+      <c r="K221" s="23"/>
+      <c r="L221" s="23"/>
+      <c r="M221" s="23"/>
+      <c r="N221" s="23"/>
+    </row>
+    <row r="222" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A222" s="21"/>
+      <c r="B222" s="21"/>
+      <c r="C222" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D222" s="23" t="s">
+        <v>941</v>
+      </c>
+      <c r="E222" s="23" t="s">
+        <v>942</v>
+      </c>
+      <c r="F222" s="23" t="s">
+        <v>943</v>
+      </c>
+      <c r="G222" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H222" s="23" t="s">
+        <v>944</v>
+      </c>
+      <c r="I222" s="23"/>
+      <c r="J222" s="23"/>
+      <c r="K222" s="23"/>
+      <c r="L222" s="23"/>
+      <c r="M222" s="23"/>
+      <c r="N222" s="23"/>
+    </row>
+    <row r="223" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A223" s="20" t="s">
+        <v>945</v>
+      </c>
+      <c r="B223" s="20" t="s">
+        <v>946</v>
+      </c>
+      <c r="C223" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="D223" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="E223" s="20"/>
+      <c r="F223" s="20"/>
+      <c r="G223" s="20"/>
+      <c r="H223" s="20"/>
+      <c r="I223" s="20"/>
+      <c r="J223" s="20"/>
+      <c r="K223" s="20"/>
+      <c r="L223" s="20"/>
+      <c r="M223" s="20"/>
+      <c r="N223" s="20"/>
+    </row>
+    <row r="224" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A224" s="21"/>
+      <c r="B224" s="22" t="s">
+        <v>947</v>
+      </c>
+      <c r="C224" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="D224" s="23" t="s">
+        <v>948</v>
+      </c>
+      <c r="E224" s="23" t="s">
+        <v>949</v>
+      </c>
+      <c r="F224" s="23" t="s">
+        <v>950</v>
+      </c>
+      <c r="G224" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="H224" s="23" t="s">
+        <v>951</v>
+      </c>
+      <c r="I224" s="23"/>
+      <c r="J224" s="23"/>
+      <c r="K224" s="23"/>
+      <c r="L224" s="23"/>
+      <c r="M224" s="23"/>
+      <c r="N224" s="23"/>
+    </row>
+    <row r="225" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A225" s="21"/>
+      <c r="B225" s="21"/>
+      <c r="C225" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D225" s="23" t="s">
+        <v>952</v>
+      </c>
+      <c r="E225" s="23" t="s">
+        <v>953</v>
+      </c>
+      <c r="F225" s="23" t="s">
+        <v>954</v>
+      </c>
+      <c r="G225" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H225" s="23" t="s">
+        <v>955</v>
+      </c>
+      <c r="I225" s="23"/>
+      <c r="J225" s="23"/>
+      <c r="K225" s="23"/>
+      <c r="L225" s="23"/>
+      <c r="M225" s="23"/>
+      <c r="N225" s="23"/>
+    </row>
+    <row r="226" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A226" s="21"/>
+      <c r="B226" s="21"/>
+      <c r="C226" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D226" s="23" t="s">
+        <v>956</v>
+      </c>
+      <c r="E226" s="23" t="s">
+        <v>957</v>
+      </c>
+      <c r="F226" s="23" t="s">
+        <v>958</v>
+      </c>
+      <c r="G226" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H226" s="23" t="s">
+        <v>959</v>
+      </c>
+      <c r="I226" s="23"/>
+      <c r="J226" s="23"/>
+      <c r="K226" s="23"/>
+      <c r="L226" s="23"/>
+      <c r="M226" s="23"/>
+      <c r="N226" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>

<commit_message>
Stage 1 re-entry: correct F-001..F-004 from Stage 2 pass 006
BA-001-08 impact-scoped correction within the PM boundary in
analysis/stages/stage-01/stage-02-pass-006-dispositions.md: request
binding (merge=true), unvalidated returnto redirects and view names,
person content of XML/MPX/MSPDI exports, and configuration-key figures
(114 entries, 106 distinct). Related-occurrence checks (d)-(g) run;
26 rows changed, none added, no status changes. PM admitted reviewer
proposals P-1/P-2 as refinements of CHK-012 and CHK-007.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -490,7 +490,7 @@
     <t>Form posted to /do/edit/roles; the role-saving code is expected never to run, so submitted roles are not saved (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:409-411; WAR:WEB-INF/action-servlet.xml:400-404 (EditRoleAction); WAR:WEB-INF/jsp/edit/editRoles.jsp; class com.technoetic.xplanner.actions.EditRoleAction (strings "admin.edit.role", HQL on PersonRole). No live link to this page was found (mechanical link scan .migration-tmp/stage-01/out/linkgraph.txt); reachable only by URL. BA-001-03 impact sweep: EditRoleAction#beforeObjectCommit(Object, Session, ActionMapping, ActionForm, HttpServletRequest, HttpServletResponse) overrides no superclass hook (AbstractAction#beforeObjectCommit takes Identifiable, ActionMapping, ActionForm, request, response) and has no caller, so its role update and its admin.edit.role check are unreachable; an orphan-hook scan over all action classes found only this method. Server-side enforcement (CHK-002, BA-001-04): no server-side check is reached, because the only check sits in the unreachable EditRoleAction#beforeObjectCommit (above); the page is reachable by any signed-in user. Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editRoles.jsp writes the raw request parameters oid (55), returnto (56) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt.</t>
+    <t>WAR:WEB-INF/struts-config.xml:409-411; WAR:WEB-INF/action-servlet.xml:400-404 (EditRoleAction); WAR:WEB-INF/jsp/edit/editRoles.jsp; class com.technoetic.xplanner.actions.EditRoleAction (strings "admin.edit.role", HQL on PersonRole). No live link to this page was found (mechanical link scan .migration-tmp/stage-01/out/linkgraph.txt); reachable only by URL. BA-001-03 impact sweep: EditRoleAction#beforeObjectCommit(Object, Session, ActionMapping, ActionForm, HttpServletRequest, HttpServletResponse) overrides no superclass hook (AbstractAction#beforeObjectCommit takes Identifiable, ActionMapping, ActionForm, request, response) and has no caller, so its role update and its admin.edit.role check are unreachable; an orphan-hook scan over all action classes found only this method. Server-side enforcement (CHK-002, BA-001-04): no server-side check is reached, because the only check sits in the unreachable EditRoleAction#beforeObjectCommit (above); the page is reachable by any signed-in user. Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editRoles.jsp writes the raw request parameters oid (55), returnto (56) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): /do/edit/roles runs EditObjectAction#doExecute with type net.sf.xplanner.domain.Project (WAR:WEB-INF/action-servlet.xml:400-404), so a direct request with merge=true binds the request parameters onto the loaded project as in row 78 (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
   </si>
   <si>
     <t>UF-003</t>
@@ -589,7 +589,7 @@
     <t>Person saved; user returned to the people list (returnto).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/people.jsp (link /do/edit/person under create.person); WAR:WEB-INF/struts-config.xml:321-326; WAR:WEB-INF/jsp/edit/editPerson.jsp; class com.technoetic.xplanner.actions.EditPersonAction. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editPerson.jsp writes the raw request parameters oid (39), returnto (43) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt.</t>
+    <t>WAR:WEB-INF/jsp/view/people.jsp (link /do/edit/person under create.person); WAR:WEB-INF/struts-config.xml:321-326; WAR:WEB-INF/jsp/edit/editPerson.jsp; class com.technoetic.xplanner.actions.EditPersonAction. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editPerson.jsp writes the raw request parameters oid (39), returnto (43) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/person that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Person object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). The settable properties include ones the person editor does not show, for example the stored password digest (Person#setPassword) and the hidden flag; EditPersonAction#beforeObjectCommit still reads the new-password and role fields from the form. No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
   </si>
   <si>
     <t>Name, user ID, e-mail and initials are mandatory; password and confirmation must match.</t>
@@ -628,7 +628,7 @@
     <t>Changes saved; returnto page shown.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (form /do/edit/person, Update button); WAR:WEB-INF/security.xml:15 (/do/edit/person in viewing constraint). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction (except the role rules in row 31) performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (form /do/edit/person, Update button); WAR:WEB-INF/security.xml:15 (/do/edit/person in viewing constraint). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction (except the role rules in row 31) performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 43 applies to every /do/edit/person request (Inferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002): the unvalidated returnto redirect of row 43 applies (Q3 facts).</t>
   </si>
   <si>
     <t>The password fields are shown only when the active login module can change passwords; a new password is stored as a salted digest.</t>
@@ -781,7 +781,7 @@
     <t>Texts change to the selected language; user returned to returnto or projects.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:158; WAR:WEB-INF/action-servlet.xml:6; class com.technoetic.xplanner.actions.ChangeLocaleAction (strings "language", "org.apache.struts.action.LOCALE"); WAR:WEB-INF/classes/ResourceBundle*.properties (10 files). No live link to /do/changeLocale was found (linkgraph.txt).</t>
+    <t>WAR:WEB-INF/struts-config.xml:158; WAR:WEB-INF/action-servlet.xml:6; class com.technoetic.xplanner.actions.ChangeLocaleAction (strings "language", "org.apache.struts.action.LOCALE"); WAR:WEB-INF/classes/ResourceBundle*.properties (10 files). No live link to /do/changeLocale was found (linkgraph.txt). Redirect target (BA-001-08, pass-006 F-002, check (e)): ChangeLocaleAction#execute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only an empty value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
   </si>
   <si>
     <t>Settings pages (work in progress)</t>
@@ -796,7 +796,7 @@
     <t>Page headed "Settings" with a table; the add/edit editor JSP is missing.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:405,419-421; WAR:WEB-INF/jsp/view/settings.jsp (prints ${settings} raw; reuses projects.title); input WEB-INF/jsp/edit/editSetting.jsp ABSENT from WAR (GAP-003); db-changelog.xml changeSet 2-1 (setting, object_type). No live link to /do/view/settings found. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditObjectAction for Setting performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>WAR:WEB-INF/struts-config.xml:405,419-421; WAR:WEB-INF/jsp/view/settings.jsp (prints ${settings} raw; reuses projects.title); input WEB-INF/jsp/edit/editSetting.jsp ABSENT from WAR (GAP-003); db-changelog.xml changeSet 2-1 (setting, object_type). No live link to /do/view/settings found. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditObjectAction for Setting performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/setting that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Setting object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
   </si>
   <si>
     <t>Generic Spring MVC handlers exist for /setting/{objectType}/list and /setting/{objectType}/edit/{objectId}.</t>
@@ -805,10 +805,10 @@
     <t>Experimental generic object pages.</t>
   </si>
   <si>
-    <t>Unknown view output.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/web.xml:264-272,313-316 (SpringServlet on /setting/*); class net.sf.xplanner.web.CommonObjectHandler (@RequestMapping "/{objectType}/list", "/{objectType}/edit/{objectId}"). Views not determinable statically.</t>
+    <t>The handlers print the objectType path value to standard output and return it as the view name; the view resolver turns it into /WEB-INF/jsp/&lt;objectType&gt;.jsp, where no JSP exists, so no usable page is expected (runtime unverified).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/web.xml:264-272,313-316 (SpringServlet on /setting/*); class net.sf.xplanner.web.CommonObjectHandler (@RequestMapping "/{objectType}/list", "/{objectType}/edit/{objectId}"). View selection (BA-001-08, pass-006 F-002, check (e)): CommonObjectHandler#list and #edit call PrintStream.println and return the {objectType} path variable as the view name; InternalResourceViewResolver adds the prefix /WEB-INF/jsp/ and the suffix .jsp (WAR:WEB-INF/classes/spring-web.xml:26-30; the Tiles view resolver at :31-35 is commented out). No JSP file lies directly in WEB-INF/jsp (0 files; the pages sit in 7 subdirectories), and a single path segment cannot name a subdirectory, so the path value selects no existing page (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
   </si>
   <si>
     <t>Administrative and test actions</t>
@@ -835,7 +835,7 @@
     <t>Action executes and redirects to returnto or projects.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/test-struts-config.xml:13-19; WAR:WEB-INF/test-action-servlet.xml:4-20 (CommandExecutorAction with txDataSamplingCommand / missingTimeEntryNotifier, PutTheClockForwardAction, EditPropertiesAction); class PutTheClockForwardAction (string "dayOffset"); class EditPropertiesAction ("propertyName", "propertyValue").</t>
+    <t>WAR:WEB-INF/test-struts-config.xml:13-19; WAR:WEB-INF/test-action-servlet.xml:4-20 (CommandExecutorAction with txDataSamplingCommand / missingTimeEntryNotifier, PutTheClockForwardAction, EditPropertiesAction); class PutTheClockForwardAction (string "dayOffset"); class EditPropertiesAction ("propertyName", "propertyValue"). Redirect target (BA-001-08, pass-006 F-002, check (e)): CommandExecutorAction#execute, PutTheClockForwardAction#execute and EditPropertiesAction#execute each redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
   </si>
   <si>
     <t>Tiles definitions can be reloaded via /do/admin/reload-tiles.</t>
@@ -1036,7 +1036,7 @@
     <t>Project saved; user returned to the projects list.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/projects.jsp:153-158 (link /do/edit/project under create.project); WAR:WEB-INF/struts-config.xml:195; WAR:WEB-INF/action-servlet.xml:72-76 (EditProjectAction); WAR:WEB-INF/jsp/edit/editProject.jsp:42-112. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditProjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editProject.jsp writes the raw request parameters oid (48), returnto (52) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt.</t>
+    <t>WAR:WEB-INF/jsp/view/projects.jsp:153-158 (link /do/edit/project under create.project); WAR:WEB-INF/struts-config.xml:195; WAR:WEB-INF/action-servlet.xml:72-76 (EditProjectAction); WAR:WEB-INF/jsp/edit/editProject.jsp:42-112. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditProjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editProject.jsp writes the raw request parameters oid (48), returnto (52) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/project that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Project object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). EditProjectAction#saveForm calls the same #populateObject. No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute (reached from EditProjectAction#doExecute) redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
   </si>
   <si>
     <t>A project without a name is rejected.</t>
@@ -1075,7 +1075,7 @@
     <t>Editor titled "Edit project: &lt;name&gt;" with Update/Reset; changes saved.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:28-34,76-80,104-106; class DomainMetaDataRepository#init (project edit -&gt; /do/edit/project, permission admin.edit). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditProjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:28-34,76-80,104-106; class DomainMetaDataRepository#init (project edit -&gt; /do/edit/project, permission admin.edit). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditProjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 78 applies to every /do/edit/project request, and also to /do/edit/roles, whose action type is Project (row 35) (Inferred; Q3 facts).</t>
   </si>
   <si>
     <t>Delete project</t>
@@ -1162,7 +1162,7 @@
     <t>Iteration saved under the project; user returned.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/project.jsp:87-90 (link /do/edit/iteration); WAR:WEB-INF/struts-config.xml:241-243; WAR:WEB-INF/action-servlet.xml:177-181 (EditIterationAction); WAR:WEB-INF/jsp/edit/editIteration.jsp; class EditIterationAction#beforeObjectCommit (strings "Create", Project). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editIteration.jsp writes the raw request parameters oid (31), returnto (34), fkey (36,37) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt.</t>
+    <t>WAR:WEB-INF/jsp/view/project.jsp:87-90 (link /do/edit/iteration); WAR:WEB-INF/struts-config.xml:241-243; WAR:WEB-INF/action-servlet.xml:177-181 (EditIterationAction); WAR:WEB-INF/jsp/edit/editIteration.jsp; class EditIterationAction#beforeObjectCommit (strings "Create", Project). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editIteration.jsp writes the raw request parameters oid (31), returnto (34), fkey (36,37) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/iteration that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Iteration object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
   </si>
   <si>
     <t>Missing name, unparsable dates, or an end date that does not follow the start date are rejected.</t>
@@ -1189,7 +1189,7 @@
     <t>Editor with Update/Reset; changes saved.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editIteration.jsp (logic:present oid: status display, daysWorked input); class DomainMetaDataRepository#init (iteration edit, permission edit). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>WAR:WEB-INF/jsp/edit/editIteration.jsp (logic:present oid: status display, daysWorked input); class DomainMetaDataRepository#init (iteration edit, permission edit). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 88 applies to every /do/edit/iteration request (Inferred; Q3 facts).</t>
   </si>
   <si>
     <t>Delete iteration</t>
@@ -1336,7 +1336,7 @@
     <t>Iteration set inactive; data sample taken; redirect to the continue-unfinished-stories page.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (close -&gt; close/iteration); WAR:WEB-INF/struts-config.xml:251-255 (forward onclose -&gt; /do/continue/unfinished/stories); class CloseIterationAction ("closed", "onclose"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); CloseIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>class DomainMetaDataRepository#init (close -&gt; close/iteration); WAR:WEB-INF/struts-config.xml:251-255 (forward onclose -&gt; /do/continue/unfinished/stories); class CloseIterationAction ("closed", "onclose"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); CloseIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Redirect target (BA-001-08, pass-006 F-002, check (e)): CloseIterationAction#doExecute redirects to the fixed onclose forward (/do/continue/unfinished/stories) and appends "?iterationId=", the iteration id, "&amp;" and the returnto request value unencoded to it, followed by "?oid=" and "&amp;fkey=" parts (bytecode listing), so the host of this redirect is fixed; the continue step (ContinueUnfinishedStoriesAction#doExecute) then redirects to its own returnto parameter unchanged (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
   </si>
   <si>
     <t>On the continue page the user selects a future iteration and confirms; unfinished stories are continued there.</t>
@@ -1594,7 +1594,7 @@
     <t>Story saved in the iteration; user returned to the iteration page.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (createStory -&gt; edit/userstory); WAR:WEB-INF/struts-config.xml:269-271; WAR:WEB-INF/action-servlet.xml:220-224 (EditStoryAction); WAR:WEB-INF/jsp/edit/editStory.jsp; classes com.technoetic.xplanner.domain.StoryStatus, StoryDisposition (enumeration strings). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editStory.jsp writes the raw request parameters oid (37), fkey (41,44), returnto (43) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt.</t>
+    <t>class DomainMetaDataRepository#init (createStory -&gt; edit/userstory); WAR:WEB-INF/struts-config.xml:269-271; WAR:WEB-INF/action-servlet.xml:220-224 (EditStoryAction); WAR:WEB-INF/jsp/edit/editStory.jsp; classes com.technoetic.xplanner.domain.StoryStatus, StoryDisposition (enumeration strings). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editStory.jsp writes the raw request parameters oid (37), fkey (41,44), returnto (43) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/userstory that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new UserStory object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). With merge=true the story validator also skips its name, estimate and priority checks (row 124). No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
   </si>
   <si>
     <t>A new story defaults to priority 4.</t>
@@ -1621,16 +1621,16 @@
     <t>class com.technoetic.xplanner.forms.UserStoryEditorForm#validate (story.editor.missing_name, negative_estimated_hours, invalid_priority).</t>
   </si>
   <si>
-    <t>A story editor request that carries merge=true skips the name, estimate and priority checks and is rejected only when the target iteration equals the current one; no page of the WAR posts merge=true to the story editor, so this applies to direct requests.</t>
+    <t>A story editor request that carries merge=true skips the name, estimate and priority checks, is rejected only when the target iteration equals the current one, and otherwise binds its request parameters directly onto the story; no page of the WAR posts merge=true to the story editor, so this applies to direct requests.</t>
   </si>
   <si>
     <t>Documents the second validation branch of the story editor.</t>
   </si>
   <si>
-    <t>Message "Cannot move or continue story in same iteration." for merge=true with the same iteration; otherwise no validation message (runtime unverified).</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.forms.UserStoryEditorForm#validate (bytecode listing: #isMerge false -&gt; story.editor.missing_name, negative_estimated_hours, #validateIsNumber invalid_priority; #isMerge true -&gt; story.editor.same_iteration when targetIterationId equals iterationId). The hidden merge field occurs only in moveContinueStory.jsp, moveContinueTask.jsp, continueUnfinishedStories.jsp and task.jsp, none of which posts to /do/edit/userstory (WAR:WEB-INF/jsp/edit/moveContinueStory.jsp:20,24). CHK-005 (BA-001-05). Source: stage-02-pass-003 F-003.</t>
+    <t>Message "Cannot move or continue story in same iteration." for merge=true with the same iteration; otherwise no validation message, and the story properties named by request parameters are set without the form copy (runtime unverified).</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.UserStoryEditorForm#validate (bytecode listing: #isMerge false -&gt; story.editor.missing_name, negative_estimated_hours, #validateIsNumber invalid_priority; #isMerge true -&gt; story.editor.same_iteration when targetIterationId equals iterationId). The hidden merge field occurs only in moveContinueStory.jsp, moveContinueTask.jsp, continueUnfinishedStories.jsp and task.jsp, none of which posts to /do/edit/userstory (WAR:WEB-INF/jsp/edit/moveContinueStory.jsp:20,24). CHK-005 (BA-001-05). Source: stage-02-pass-003 F-003. Request binding (BA-001-08, pass-006 F-001): with merge=true, EditObjectAction#populateObject calls org.apache.struts.util.RequestUtils.populate onto the story instead of copying the form and resolving its many-to-one references (bytecode listing), so any writable story property named by a parameter is set, including properties the editor does not show; together with the skipped checks, unvalidated values reach the saved story (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
   </si>
   <si>
     <t>Edit user story</t>
@@ -1645,7 +1645,7 @@
     <t>Editor titled for the story with Update/Reset; changes saved.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (story edit -&gt; /do/edit/userstory, permission edit); WAR:WEB-INF/jsp/edit/editStory.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>class DomainMetaDataRepository#init (story edit -&gt; /do/edit/userstory, permission edit); WAR:WEB-INF/jsp/edit/editStory.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 121 applies to every /do/edit/userstory request (Inferred; Q3 facts).</t>
   </si>
   <si>
     <t>Delete user story</t>
@@ -1699,7 +1699,7 @@
     <t>Move/Continue page with target iteration; story moved.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (movecontinue -&gt; /do/move/continue/userstory); WAR:WEB-INF/struts-config.xml:273-275; WAR:WEB-INF/jsp/edit/moveContinueStory.jsp; class MoveContinueStoryAction#saveForm ("Move"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); MoveContinueStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/moveContinueStory.jsp writes the raw request parameters fkey (25) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt.</t>
+    <t>class DomainMetaDataRepository#init (movecontinue -&gt; /do/move/continue/userstory); WAR:WEB-INF/struts-config.xml:273-275; WAR:WEB-INF/jsp/edit/moveContinueStory.jsp; class MoveContinueStoryAction#saveForm ("Move"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); MoveContinueStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/moveContinueStory.jsp writes the raw request parameters fkey (25) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001): the Move/Continue page posts merge=true together with oid, iterationId, fkey, action and returnto (WAR:WEB-INF/jsp/edit/moveContinueStory.jsp:20-28); MoveContinueStoryAction#saveForm calls EditObjectAction#populateObject, which binds every request parameter onto the story with org.apache.struts.util.RequestUtils.populate before the move (bytecode listing; Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect (F-002): MoveContinueStoryAction#doExecute then redirects to the returnto request value unchanged (Q3 facts).</t>
   </si>
   <si>
     <t>Continue creates a continuation of the story in the target iteration for the unfinished work, with cross-references in the descriptions.</t>
@@ -1756,7 +1756,7 @@
     <t>Task saved; user returned to the story.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/userstory.jsp (link /do/edit/task, story.link.create_task); WAR:WEB-INF/struts-config.xml:291; WAR:WEB-INF/action-servlet.xml:268-272 (EditTaskAction); WAR:WEB-INF/jsp/edit/editTask.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editTask.jsp writes the raw request parameters oid (31), returnto (34), fkey (36,37) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt.</t>
+    <t>WAR:WEB-INF/jsp/view/userstory.jsp (link /do/edit/task, story.link.create_task); WAR:WEB-INF/struts-config.xml:291; WAR:WEB-INF/action-servlet.xml:268-272 (EditTaskAction); WAR:WEB-INF/jsp/edit/editTask.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editTask.jsp writes the raw request parameters oid (31), returnto (34), fkey (36,37) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/task that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Task object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). EditTaskAction#populateObject calls the parent method. With merge=true the task validator skips its name and estimate checks (row 137). The complete and reopen buttons of the task page post merge=true (rows 140-141); any other parameter added to such a request is bound as well (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute (reached from EditTaskAction#doExecute) redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
   </si>
   <si>
     <t>The task type is stored as a message label, not a code: the type options carry label text as their values, resolved without the user's locale, so the stored value follows the server default locale. The labels differ between bundles.</t>
@@ -1789,7 +1789,7 @@
     <t>Messages "Missing task name.", "Please provide an estimate greater than or equal to zero.", "Created date is invalid."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TaskEditorForm#validate (task.editor.missing_name, negative_estimated_hours, bad_created_date). Merge branch (CHK-005, BA-001-05): TaskEditorForm#validate checks the created date first and skips the name and estimate checks when merge=true, which the complete and reopen buttons post (WAR:WEB-INF/jsp/view/task.jsp:76-79,87-90).</t>
+    <t>class com.technoetic.xplanner.forms.TaskEditorForm#validate (task.editor.missing_name, negative_estimated_hours, bad_created_date). Merge branch (CHK-005, BA-001-05): TaskEditorForm#validate checks the created date first and skips the name and estimate checks when merge=true, which the complete and reopen buttons post (WAR:WEB-INF/jsp/view/task.jsp:76-79,87-90). Request binding (BA-001-08, pass-006 F-001): the same merge=true requests are bound onto the task by EditObjectAction#populateObject with org.apache.struts.util.RequestUtils.populate instead of the form copy (EditTaskAction#populateObject calls the parent), so the skipped name and estimate checks leave any task property named by a parameter unvalidated (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
   </si>
   <si>
     <t>Task e-mail notification</t>
@@ -1819,7 +1819,7 @@
     <t>Task editor with Update/Reset; changes saved.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (task edit -&gt; /do/edit/task); WAR:WEB-INF/jsp/edit/editTask.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>class DomainMetaDataRepository#init (task edit -&gt; /do/edit/task); WAR:WEB-INF/jsp/edit/editTask.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 134 applies to every /do/edit/task request (Inferred; Q3 facts).</t>
   </si>
   <si>
     <t>Complete or reopen task</t>
@@ -1834,7 +1834,7 @@
     <t>"Complete" button; task becomes completed; page reloads.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/task.jsp:86-95 (form /do/edit/task, action Update, merge true, completed true). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>WAR:WEB-INF/jsp/view/task.jsp:86-95 (form /do/edit/task, action Update, merge true, completed true). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Mechanism (BA-001-08, pass-006 F-001): the completion takes effect through the merge=true binding, not through the task form: EditObjectAction#populateObject calls org.apache.struts.util.RequestUtils.populate, which sets Task#setCompleted from the posted completed=true (WAR:WEB-INF/jsp/view/task.jsp:87-94); any further parameter added to the request is bound onto the task as well (Inferred; Q3 facts). After the save, EditObjectAction#doExecute redirects to the posted returnto value (F-002).</t>
   </si>
   <si>
     <t>A completed task can be reopened.</t>
@@ -1846,7 +1846,7 @@
     <t>"Reopen" button; task becomes open again.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/task.jsp:75-84 (completed false). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>WAR:WEB-INF/jsp/view/task.jsp:75-84 (completed false). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Mechanism (BA-001-08, pass-006 F-001): the reopen form posts merge=true and completed=false (WAR:WEB-INF/jsp/view/task.jsp:76-83), so the change is made by the same RequestUtils.populate binding as in row 140 (Inferred; Q3 facts).</t>
   </si>
   <si>
     <t>Delete task</t>
@@ -1945,7 +1945,7 @@
     <t>Time grid with an empty new row; "Insert Time" fills current time; Update saves; redirect to the task page.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (edittime -&gt; /do/edit/time); WAR:WEB-INF/struts-config.xml:350-355; WAR:WEB-INF/action-servlet.xml:376-378 (UpdateTimeAction); WAR:WEB-INF/jsp/edit/editTimeEntries.jsp; WAR:editTimeEntries.js; WAR:time.js. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); UpdateTimeAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editTimeEntries.jsp writes the raw request parameters oid (59), returnto (61), fkey (63,64) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt.</t>
+    <t>class DomainMetaDataRepository#init (edittime -&gt; /do/edit/time); WAR:WEB-INF/struts-config.xml:350-355; WAR:WEB-INF/action-servlet.xml:376-378 (UpdateTimeAction); WAR:WEB-INF/jsp/edit/editTimeEntries.jsp; WAR:editTimeEntries.js; WAR:time.js. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); UpdateTimeAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editTimeEntries.jsp writes the raw request parameters oid (59), returnto (61), fkey (63,64) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Redirect target (BA-001-08, pass-006 F-002, check (e)): UpdateTimeAction#doUpdateTimeAction (and #doUpdateEstimateAction for the estimate action) redirects to the returnto value posted by the time editor, unchanged (new ActionForward(returnto, true)); there is no fallback for a missing value, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
   </si>
   <si>
     <t>Existing entries can be edited or marked for deletion in the same grid.</t>
@@ -2176,7 +2176,7 @@
     <t>Note editor (multipart form); after save the note appears in the Notes section of the object page.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/layout/viewLayout.jsp:114-116 (include view/notes.jsp in tiles:view pages); WAR:WEB-INF/jsp/view/notes.jsp:20-23 (isNoteEditor = hasPermission(..., "note", 0, "edit")) and link /do/edit/note?attachedToId=; WAR:WEB-INF/struts-config.xml:306-307; WAR:WEB-INF/action-servlet.xml:306-313 (EditNoteAction, virtualFileSystem); WAR:WEB-INF/jsp/edit/editNote.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request-value flow (BA-001-07, mechanism (b)): the note list included in these pages reads the oid request parameter (WAR:WEB-INF/jsp/view/notes.jsp:13, bean:parameter) and concatenates it into the useBeans where clause "attachedToId=" + oid (:14-15), which UseBeansTag#doEndTag appends into the HQL text; this is the same pattern as the time-log query of WAR:WEB-INF/jsp/view/task.jsp:101-103 (Q3 facts). Exploitability is not established (static only; observed risk only, Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editNote.jsp writes the raw request parameters oid (31), returnto (35,106), projectId (37), attachedToId (39), formFileName (82) [parameter (lines); line 106 passes returnto as the page attribute of html:link] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt.</t>
+    <t>WAR:WEB-INF/jsp/layout/viewLayout.jsp:114-116 (include view/notes.jsp in tiles:view pages); WAR:WEB-INF/jsp/view/notes.jsp:20-23 (isNoteEditor = hasPermission(..., "note", 0, "edit")) and link /do/edit/note?attachedToId=; WAR:WEB-INF/struts-config.xml:306-307; WAR:WEB-INF/action-servlet.xml:306-313 (EditNoteAction, virtualFileSystem); WAR:WEB-INF/jsp/edit/editNote.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request-value flow (BA-001-07, mechanism (b)): the note list included in these pages reads the oid request parameter (WAR:WEB-INF/jsp/view/notes.jsp:13, bean:parameter) and concatenates it into the useBeans where clause "attachedToId=" + oid (:14-15), which UseBeansTag#doEndTag appends into the HQL text; this is the same pattern as the time-log query of WAR:WEB-INF/jsp/view/task.jsp:101-103 (Q3 facts). Exploitability is not established (static only; observed risk only, Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editNote.jsp writes the raw request parameters oid (31), returnto (35,106), projectId (37), attachedToId (39), formFileName (82) [parameter (lines); line 106 passes returnto as the page attribute of html:link] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/note that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Note object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). EditNoteAction#populateObject calls the parent method before it stores the attachment. No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
   </si>
   <si>
     <t>A note without subject, author or body is rejected.</t>
@@ -2227,7 +2227,7 @@
     <t>Note editor pre-filled; changes saved.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/notes.jsp (isUserAuthorized note edit; link /do/edit/note). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>WAR:WEB-INF/jsp/view/notes.jsp (isUserAuthorized note edit; link /do/edit/note). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 169 applies to every /do/edit/note request (Inferred; Q3 facts).</t>
   </si>
   <si>
     <t>An authorized user can delete a note after confirming "Do you want to delete note &lt;subject&gt;".</t>
@@ -2686,7 +2686,7 @@
     <t>Download export.xml (text/xml), export.mpx (application/mpx) or export.xml (application/mspdi).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:189-193; WAR:WEB-INF/action-servlet.xml:45-70; classes com.technoetic.xplanner.export.XmlExporter, MpxExporter, MspdiExporter (Content-type and filename strings); WAR:WEB-INF/lib/mpxj-3.0.1.jar.</t>
+    <t>WAR:WEB-INF/struts-config.xml:189-193; WAR:WEB-INF/action-servlet.xml:45-70; classes com.technoetic.xplanner.export.XmlExporter, MpxExporter, MspdiExporter (Content-type and filename strings); WAR:WEB-INF/lib/mpxj-3.0.1.jar. Content (BA-001-08, pass-006 F-003, check (f)): besides the selected project, all three formats contain every person of the system. XmlExporter#export runs the unconditional query "from person in class net.sf.xplanner.domain.Person" and writes the result as the people of the document (XmlExporter$XPlannerData#setPeople); XmlExporter#configureBindings hides the person password and lastUpdateTime, so the other readable person properties (for example id, name, user ID, e-mail, phone, initials, hidden flag and description) are expected in the file (Betwixt, exact set Inferred). MpxExporter#export and MspdiExporter#export load all persons into MpxExporter$ResourceRegistry, which adds each one as a resource with its name only (Person#getName). The export actions have no server-side permission check (rows 29-30). Inferred; observed fact for Stage 9, Q3 deferred.</t>
   </si>
   <si>
     <t>Export iteration</t>
@@ -2701,7 +2701,7 @@
     <t>Downloads export.xml, export.mpx, export.xml, export.pdf.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:231-237; WAR:WEB-INF/action-servlet.xml:132-166; class com.technoetic.xplanner.export.PdfExporter ("application/pdf", "export.pdf"); WAR:WEB-INF/lib/itext-1.01.jar.</t>
+    <t>WAR:WEB-INF/struts-config.xml:231-237; WAR:WEB-INF/action-servlet.xml:132-166; class com.technoetic.xplanner.export.PdfExporter ("application/pdf", "export.pdf"); WAR:WEB-INF/lib/itext-1.01.jar. Content (BA-001-08, pass-006 F-003, check (f)): the XML, MPX and MSPDI files contain every person of the system, as in row 209 (the same exporter beans, WAR:WEB-INF/action-servlet.xml:132-166). The PDF listing (PdfExporter) shows only the names of the customers and acceptors of the exported stories and tasks (Person#getName), no person list (Inferred).</t>
   </si>
   <si>
     <t>An iteration JasperReports PDF (jrpdf) report is offered but its report template is missing from the WAR.</t>

</xml_diff>

<commit_message>
Stage 1 re-entry: correct F-001..F-003 from Stage 2 pass 007
BA-001-09 impact-scoped correction within the PM boundary in
analysis/stages/stage-01/stage-02-pass-007-dispositions.md: Spring
redirect:/forward: view-name resolution and the Tiles definition case
for returnto (F-001), the returnto script sink on the start/close
iteration page (F-002, rows 98 and 101), and the public-page key figure
of 45 with per-bundle notes (F-003). Directly related checks (h)-(j)
run; 5 rows changed, none added, no status changes. PM admitted
reviewer proposals P-1/P-2 as refinements of CHK-012 and CHK-007.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -130,7 +130,7 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>WAR: = paths inside legacy/xplanner-plus.war. WAR:WEB-INF/struts-config.xml:164-167 (/login, forwards notAuthenticated -&gt; WEB-INF/jsp/security/login.jsp, authenticated -&gt; /do/view/projects redirect); WAR:WEB-INF/action-servlet.xml:10 (AuthenticationAction); WAR:WEB-INF/jsp/security/login.jsp:16-33; class com.technoetic.xplanner.actions.AuthenticationAction#execute (calls Authenticator.authenticate, forward "authenticated"). Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; login.label and login.remember are defined in the default, "--", de, it, ja and ru bundles; login.label.user_id and login.label.password in all bundles except fr; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9).</t>
+    <t>WAR: = paths inside legacy/xplanner-plus.war. WAR:WEB-INF/struts-config.xml:164-167 (/login, forwards notAuthenticated -&gt; WEB-INF/jsp/security/login.jsp, authenticated -&gt; /do/view/projects redirect); WAR:WEB-INF/action-servlet.xml:10 (AuthenticationAction); WAR:WEB-INF/jsp/security/login.jsp:16-33; class com.technoetic.xplanner.actions.AuthenticationAction#execute (calls Authenticator.authenticate, forward "authenticated"). Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; login.label and login.remember are defined in the default, "--", de, it, ja and ru bundles; login.label.user_id and login.label.password in all bundles except fr; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Page-text keys (BA-001-09, pass-007 F-003, check (j)): the login page also renders login.title, given as titleKey (WAR:WEB-INF/jsp/security/login.jsp:14; defined in all bundles except fr). Through the tiles:default layout that xplanner:content inserts (class ContentTag#doStartTag; WAR:WEB-INF/tiles-definitions.xml:5-10) it also renders the footer keys app.label.version (all 10 bundles) and footer.message (only the default, "--" and de bundles; WAR:WEB-INF/jsp/common/footer.jsp:25,38) and the breadcrumb link text navigation.top (all 10 bundles; WAR:WEB-INF/jsp/layout/defaultLayout.jsp:44, WAR:WEB-INF/tags/breadcrumb.tag:10, class net.sf.xplanner.tags.NavigationBarTag#render). Bundles without a key fall back to the default text (framework behavior, GAP-011). None of these texts is credential-like (.migration-tmp/stage-01/out/public-keys-09.txt).</t>
   </si>
   <si>
     <t>Alternative path</t>
@@ -754,7 +754,7 @@
     <t>Error page with message, support links (support.issue.url), "Cause" and "Stack Trace" boxes.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:16-29 (error-page JspException, ServletException, Throwable -&gt; unexpectedError.jsp); WAR:WEB-INF/jsp/common/unexpectedError.jsp; xplanner.properties:289-309 (error.filingInfo). Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; error.unknownError and error.moreInfo are defined only in the default and "--" bundles; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Request echo (BA-001-07, mechanism (b)): unexpectedError.jsp is the container error page for every JspException, ServletException and Throwable (WAR:WEB-INF/web.xml:16-29). It prints the first lines of the exception message unescaped with &lt;%= message %&gt; (unexpectedError.jsp:66) and lists the referer, URL, query string, every request parameter (including any password field of the failing request) and every request attribute (:100-121; values HTML-encoded by BoxedListTag). Observed risk only (Q3 deferred). Source: stage-02-pass-005 F-003. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/web.xml:16-29 (error-page JspException, ServletException, Throwable -&gt; unexpectedError.jsp); WAR:WEB-INF/jsp/common/unexpectedError.jsp; xplanner.properties:289-309 (error.filingInfo). Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; error.unknownError and error.moreInfo are defined only in the default and "--" bundles; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Request echo (BA-001-07, mechanism (b)): unexpectedError.jsp is the container error page for every JspException, ServletException and Throwable (WAR:WEB-INF/web.xml:16-29). It prints the first lines of the exception message unescaped with &lt;%= message %&gt; (unexpectedError.jsp:66) and lists the referer, URL, query string, every request parameter (including any password field of the failing request) and every request attribute (:100-121; values HTML-encoded by BoxedListTag). Observed risk only (Q3 deferred). Source: stage-02-pass-005 F-003. Page-text keys (BA-001-09, pass-007 F-003, check (j)): the page title comes from a scriptlet-selected key (WAR:WEB-INF/jsp/common/unexpectedError.jsp:19,27,47): error.title, defined in all bundles except de and es, and, when the same page serves the system information page (row 55), system.info.title, defined only in the default and "--" bundles. The tiles:default layout adds the footer keys app.label.version (all 10 bundles) and footer.message (only the default, "--" and de bundles; WAR:WEB-INF/jsp/common/footer.jsp:25,38) and the breadcrumb link text navigation.top (all 10 bundles; WAR:WEB-INF/tags/breadcrumb.tag:10). Bundles without a key fall back to the default text (framework behavior, GAP-011). None of these texts is credential-like (.migration-tmp/stage-01/out/public-keys-09.txt). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
   </si>
   <si>
     <t>Requesting a non-existent object shows "Object &lt;id&gt; not found".</t>
@@ -805,10 +805,10 @@
     <t>Experimental generic object pages.</t>
   </si>
   <si>
-    <t>The handlers print the objectType path value to standard output and return it as the view name; the view resolver turns it into /WEB-INF/jsp/&lt;objectType&gt;.jsp, where no JSP exists, so no usable page is expected (runtime unverified).</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/web.xml:264-272,313-316 (SpringServlet on /setting/*); class net.sf.xplanner.web.CommonObjectHandler (@RequestMapping "/{objectType}/list", "/{objectType}/edit/{objectId}"). View selection (BA-001-08, pass-006 F-002, check (e)): CommonObjectHandler#list and #edit call PrintStream.println and return the {objectType} path variable as the view name; InternalResourceViewResolver adds the prefix /WEB-INF/jsp/ and the suffix .jsp (WAR:WEB-INF/classes/spring-web.xml:26-30; the Tiles view resolver at :31-35 is commented out). No JSP file lies directly in WEB-INF/jsp (0 files; the pages sit in 7 subdirectories), and a single path segment cannot name a subdirectory, so the path value selects no existing page (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
+    <t>The handlers print the objectType path value to standard output and return it as the view name. A plain value becomes /WEB-INF/jsp/&lt;objectType&gt;.jsp, where no JSP exists, so no usable page is expected; a value that starts with redirect: sends the browser to the rest of the value, and one that starts with forward: forwards inside the application (runtime unverified).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/web.xml:264-272,313-316 (SpringServlet on /setting/*); class net.sf.xplanner.web.CommonObjectHandler (@RequestMapping "/{objectType}/list", "/{objectType}/edit/{objectId}"). View selection (BA-001-08, pass-006 F-002, check (e)): CommonObjectHandler#list and #edit call PrintStream.println and return the {objectType} path variable as the view name; InternalResourceViewResolver adds the prefix /WEB-INF/jsp/ and the suffix .jsp (WAR:WEB-INF/classes/spring-web.xml:26-30; the Tiles view resolver at :31-35 is commented out). No JSP file lies directly in WEB-INF/jsp (0 files; the pages sit in 7 subdirectories), and a single path segment cannot name a subdirectory, so a value without a view prefix selects no existing page. Framework resolution (BA-001-09, pass-007 F-001, check (h)): InternalResourceViewResolver extends UrlBasedViewResolver, whose #createView in the bundled WAR:WEB-INF/lib/spring-webmvc-3.0.5.RELEASE.jar (bytecode listing) checks the view name before prefix and suffix are applied: a name that starts with "redirect:" becomes a RedirectView of the rest of the name (RedirectView#renderMergedOutputModel adds the context path only to a target that starts with "/", then HttpServletResponse#sendRedirect; spring-web.xml sets no redirect options, so the defaults apply), and a name that starts with "forward:" becomes an InternalResourceView forward of the rest. /setting/* is mapped to the Spring servlet and to WebSecurityFilter (WAR:WEB-INF/web.xml:164-167,313-316), so a signed-in user who follows /setting/redirect:&lt;target&gt;/list is redirected to &lt;target&gt;, and after a login the saved URL returns the user to it. One path segment cannot carry "/", but a scheme-qualified target whose scheme differs from the page is expected to be resolved by browsers as another host (Inferred; the container's handling of encoded slashes and the browser behavior are unverified; observed risk only, Q3 deferred; Q3 facts).</t>
   </si>
   <si>
     <t>Administrative and test actions</t>
@@ -1297,7 +1297,7 @@
     <t>Page "Start Iteration: &lt;name&gt;" with "Do you want to start the iteration?" and OK/Cancel; iteration becomes active; opening data samples taken.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (start -&gt; start/iteration, permission edit); WAR:WEB-INF/struts-config.xml:245-248; WAR:WEB-INF/jsp/edit/editIterationStatus.jsp:43-47 (message_1 only when UpdateTimeAction.isFromUpdateTime) and :58-60 (message_4); WAR:WEB-INF/classes/ResourceBundle.properties:272,275; class StartIterationAction#beforeObjectCommit ("started", DataSampler.generateOpeningDataSamples). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); StartIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-005). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; iteration.status.editor.message_4 is defined only in the default and "--" bundles. Bundles without the key fall back to the default text (framework behavior, GAP-011). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editIterationStatus.jsp writes the raw request parameters fkey (34), returnto (35) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt.</t>
+    <t>class DomainMetaDataRepository#init (start -&gt; start/iteration, permission edit); WAR:WEB-INF/struts-config.xml:245-248; WAR:WEB-INF/jsp/edit/editIterationStatus.jsp:43-47 (message_1 only when UpdateTimeAction.isFromUpdateTime) and :58-60 (message_4); WAR:WEB-INF/classes/ResourceBundle.properties:272,275; class StartIterationAction#beforeObjectCommit ("started", DataSampler.generateOpeningDataSamples). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); StartIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-005). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; iteration.status.editor.message_4 is defined only in the default and "--" bundles. Bundles without the key fall back to the default text (framework behavior, GAP-011). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editIterationStatus.jsp writes the raw request parameters fkey (34), returnto (35) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Script context (BA-001-09, pass-007 F-002, check (i)): the page binds returnto from the request (WAR:WEB-INF/jsp/edit/editIterationStatus.jsp:32, bean:parameter) and writes it unescaped after the context path into the JavaScript string of the Cancel button's onclick handler (document.location='&lt;context path&gt;&lt;returnto&gt;', :70). A crafted value can end the string and add script, and it chooses where Cancel leads on the same host. The page is the input and forward of /do/start/iteration and /do/close/iteration (WAR:WEB-INF/struts-config.xml:119-120,245,251) (Inferred; observed risk only, Q3 deferred; Q3 facts). Inventory: .migration-tmp/stage-01/out/script-sinks-09.txt.</t>
   </si>
   <si>
     <t>If other iterations are still started, the page proposes closing them (checked by default).</t>
@@ -1336,7 +1336,7 @@
     <t>Iteration set inactive; data sample taken; redirect to the continue-unfinished-stories page.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (close -&gt; close/iteration); WAR:WEB-INF/struts-config.xml:251-255 (forward onclose -&gt; /do/continue/unfinished/stories); class CloseIterationAction ("closed", "onclose"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); CloseIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Redirect target (BA-001-08, pass-006 F-002, check (e)): CloseIterationAction#doExecute redirects to the fixed onclose forward (/do/continue/unfinished/stories) and appends "?iterationId=", the iteration id, "&amp;" and the returnto request value unencoded to it, followed by "?oid=" and "&amp;fkey=" parts (bytecode listing), so the host of this redirect is fixed; the continue step (ContinueUnfinishedStoriesAction#doExecute) then redirects to its own returnto parameter unchanged (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
+    <t>class DomainMetaDataRepository#init (close -&gt; close/iteration); WAR:WEB-INF/struts-config.xml:251-255 (forward onclose -&gt; /do/continue/unfinished/stories); class CloseIterationAction ("closed", "onclose"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); CloseIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Redirect target (BA-001-08, pass-006 F-002, check (e)): CloseIterationAction#doExecute redirects to the fixed onclose forward (/do/continue/unfinished/stories) and appends "?iterationId=", the iteration id, "&amp;" and the returnto request value unencoded to it, followed by "?oid=" and "&amp;fkey=" parts (bytecode listing), so the host of this redirect is fixed; the continue step (ContinueUnfinishedStoriesAction#doExecute) then redirects to its own returnto parameter unchanged (Inferred; observed risk only, Q3 deferred; Q3 facts). Script context (BA-001-09, pass-007 F-002): the close confirmation uses the same page, WAR:WEB-INF/jsp/edit/editIterationStatus.jsp (WAR:WEB-INF/struts-config.xml:120,251), whose Cancel button writes the returnto request value unescaped into its onclick script (:70; row 98; Q3 facts).</t>
   </si>
   <si>
     <t>On the continue page the user selects a future iteration and confirms; unfinished stories are continued there.</t>

</xml_diff>

<commit_message>
Stage 1 remediation: correct pass-008 observations F-001..F-003
Owner-approved bounded Stage 1 return after the invalid Stage 2
correction-validation attempt 008 (transition owner_approval with the
exact pass-008 scope; report 008 in gate_evidence). BA-001-10 verified
each lead from the WAR: the shared Tiles factory yields 5 definition
names (F-001, plus single-argument forwards and request-keyed caches),
the public-page breadcrumb loads a request-named object without sign-in
(F-002), and the BA-001-09 figures are recounted with stated rules
(F-003). Unescaped stored-value EL output is recorded as a bounded fact
without an inventory. 3 rows changed, none added. PM admitted P-1..P-3
as refinements of CHK-003, CHK-011 and CHK-007. Pass 008 stays invalid.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -130,7 +130,7 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>WAR: = paths inside legacy/xplanner-plus.war. WAR:WEB-INF/struts-config.xml:164-167 (/login, forwards notAuthenticated -&gt; WEB-INF/jsp/security/login.jsp, authenticated -&gt; /do/view/projects redirect); WAR:WEB-INF/action-servlet.xml:10 (AuthenticationAction); WAR:WEB-INF/jsp/security/login.jsp:16-33; class com.technoetic.xplanner.actions.AuthenticationAction#execute (calls Authenticator.authenticate, forward "authenticated"). Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; login.label and login.remember are defined in the default, "--", de, it, ja and ru bundles; login.label.user_id and login.label.password in all bundles except fr; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Page-text keys (BA-001-09, pass-007 F-003, check (j)): the login page also renders login.title, given as titleKey (WAR:WEB-INF/jsp/security/login.jsp:14; defined in all bundles except fr). Through the tiles:default layout that xplanner:content inserts (class ContentTag#doStartTag; WAR:WEB-INF/tiles-definitions.xml:5-10) it also renders the footer keys app.label.version (all 10 bundles) and footer.message (only the default, "--" and de bundles; WAR:WEB-INF/jsp/common/footer.jsp:25,38) and the breadcrumb link text navigation.top (all 10 bundles; WAR:WEB-INF/jsp/layout/defaultLayout.jsp:44, WAR:WEB-INF/tags/breadcrumb.tag:10, class net.sf.xplanner.tags.NavigationBarTag#render). Bundles without a key fall back to the default text (framework behavior, GAP-011). None of these texts is credential-like (.migration-tmp/stage-01/out/public-keys-09.txt).</t>
+    <t>WAR: = paths inside legacy/xplanner-plus.war. WAR:WEB-INF/struts-config.xml:164-167 (/login, forwards notAuthenticated -&gt; WEB-INF/jsp/security/login.jsp, authenticated -&gt; /do/view/projects redirect); WAR:WEB-INF/action-servlet.xml:10 (AuthenticationAction); WAR:WEB-INF/jsp/security/login.jsp:16-33; class com.technoetic.xplanner.actions.AuthenticationAction#execute (calls Authenticator.authenticate, forward "authenticated"). Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; login.label and login.remember are defined in the default, "--", de, it, ja and ru bundles; login.label.user_id and login.label.password in all bundles except fr; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Page-text keys (BA-001-09, pass-007 F-003, check (j)): the login page also renders login.title, given as titleKey (WAR:WEB-INF/jsp/security/login.jsp:14; defined in all bundles except fr). Through the tiles:default layout that xplanner:content inserts (class ContentTag#doStartTag; WAR:WEB-INF/tiles-definitions.xml:5-10) it also renders the footer keys app.label.version (all 10 bundles) and footer.message (only the default, "--" and de bundles; WAR:WEB-INF/jsp/common/footer.jsp:25,38) and the breadcrumb link text navigation.top (all 10 bundles; WAR:WEB-INF/jsp/layout/defaultLayout.jsp:44, WAR:WEB-INF/tags/breadcrumb.tag:10, class net.sf.xplanner.tags.NavigationBarTag#render). Bundles without a key fall back to the default text (framework behavior, GAP-011). None of these texts is credential-like (.migration-tmp/stage-01/out/public-keys-09.txt). Breadcrumb lookup (BA-001-10, pass-008 F-002 lead, check (l)): on this page the layout breadcrumb (WAR:WEB-INF/jsp/layout/defaultLayout.jsp:44, WAR:WEB-INF/tags/breadcrumb.tag:10) reads the request parameter oid, or else fkey, and loads that object without a sign-in or permission check (class net.sf.xplanner.tags.NavigationBarTag#doEndTag, #setObject(int): the type attribute arrives as an empty string, so IdSearchHelper#search runs Session#get over Project, Iteration, UserStory, Task, Person and Note). #render then adds links whose texts are the names of the object's project, iteration, story, task or feature, and breadcrumb.tag:15,18 prints them with unescaped EL. /do/login is in the security bypass list (WAR:WEB-INF/security.xml:3), so /do/login?oid=&lt;id&gt; is expected to show those names, including any markup stored in them, to a visitor who has not signed in (Inferred; the EL coercion and runtime are unverified; row 185; GAP-007; observed risk only, Q3 deferred). Page-text scope (BA-001-10): the 45 keys are the keys named by the page and layout chain; after a failed login the page also shows messages queued in code (WAR:WEB-INF/jsp/security/login.jsp:50-59): login.failed and 9 authentication.module.message.* keys named in the class bytecode, of which rows 12-13 describe the ones the XPlanner login module produces.</t>
   </si>
   <si>
     <t>Alternative path</t>
@@ -754,7 +754,7 @@
     <t>Error page with message, support links (support.issue.url), "Cause" and "Stack Trace" boxes.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:16-29 (error-page JspException, ServletException, Throwable -&gt; unexpectedError.jsp); WAR:WEB-INF/jsp/common/unexpectedError.jsp; xplanner.properties:289-309 (error.filingInfo). Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; error.unknownError and error.moreInfo are defined only in the default and "--" bundles; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Request echo (BA-001-07, mechanism (b)): unexpectedError.jsp is the container error page for every JspException, ServletException and Throwable (WAR:WEB-INF/web.xml:16-29). It prints the first lines of the exception message unescaped with &lt;%= message %&gt; (unexpectedError.jsp:66) and lists the referer, URL, query string, every request parameter (including any password field of the failing request) and every request attribute (:100-121; values HTML-encoded by BoxedListTag). Observed risk only (Q3 deferred). Source: stage-02-pass-005 F-003. Page-text keys (BA-001-09, pass-007 F-003, check (j)): the page title comes from a scriptlet-selected key (WAR:WEB-INF/jsp/common/unexpectedError.jsp:19,27,47): error.title, defined in all bundles except de and es, and, when the same page serves the system information page (row 55), system.info.title, defined only in the default and "--" bundles. The tiles:default layout adds the footer keys app.label.version (all 10 bundles) and footer.message (only the default, "--" and de bundles; WAR:WEB-INF/jsp/common/footer.jsp:25,38) and the breadcrumb link text navigation.top (all 10 bundles; WAR:WEB-INF/tags/breadcrumb.tag:10). Bundles without a key fall back to the default text (framework behavior, GAP-011). None of these texts is credential-like (.migration-tmp/stage-01/out/public-keys-09.txt). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/web.xml:16-29 (error-page JspException, ServletException, Throwable -&gt; unexpectedError.jsp); WAR:WEB-INF/jsp/common/unexpectedError.jsp; xplanner.properties:289-309 (error.filingInfo). Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; error.unknownError and error.moreInfo are defined only in the default and "--" bundles; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Request echo (BA-001-07, mechanism (b)): unexpectedError.jsp is the container error page for every JspException, ServletException and Throwable (WAR:WEB-INF/web.xml:16-29). It prints the first lines of the exception message unescaped with &lt;%= message %&gt; (unexpectedError.jsp:66) and lists the referer, URL, query string, every request parameter (including any password field of the failing request) and every request attribute (:100-121; values HTML-encoded by BoxedListTag). Observed risk only (Q3 deferred). Source: stage-02-pass-005 F-003. Page-text keys (BA-001-09, pass-007 F-003, check (j)): the page title comes from a scriptlet-selected key (WAR:WEB-INF/jsp/common/unexpectedError.jsp:19,27,47): error.title, defined in all bundles except de and es, and, when the same page serves the system information page (row 55), system.info.title, defined only in the default and "--" bundles. The tiles:default layout adds the footer keys app.label.version (all 10 bundles) and footer.message (only the default, "--" and de bundles; WAR:WEB-INF/jsp/common/footer.jsp:25,38) and the breadcrumb link text navigation.top (all 10 bundles; WAR:WEB-INF/tags/breadcrumb.tag:10). Bundles without a key fall back to the default text (framework behavior, GAP-011). None of these texts is credential-like (.migration-tmp/stage-01/out/public-keys-09.txt). Breadcrumb lookup (BA-001-10, pass-008 F-002 lead, check (l)): the error page uses the same tiles:default layout, and the layout breadcrumb (WAR:WEB-INF/jsp/layout/defaultLayout.jsp:44, WAR:WEB-INF/tags/breadcrumb.tag:10) reads the request parameter oid, or else fkey, and loads that object without a sign-in or permission check (class net.sf.xplanner.tags.NavigationBarTag#doEndTag, #setObject(int): the type attribute arrives as an empty string, so IdSearchHelper#search runs Session#get over Project, Iteration, UserStory, Task, Person and Note). #render then adds links whose texts are the names of the object's project, iteration, story, task or feature, and breadcrumb.tag:15,18 prints them with unescaped EL. The error page renders for every failing request, including one without a session, so the names of the object named by the failing request's oid or fkey are expected to be shown there too (Inferred; row 185; GAP-007; observed risk only, Q3 deferred). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
   </si>
   <si>
     <t>Requesting a non-existent object shows "Object &lt;id&gt; not found".</t>
@@ -2380,7 +2380,7 @@
     <t>Breadcrumb links above the page content.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/tags/breadcrumb.tag; class net.sf.xplanner.tags.NavigationBarTag#render (strings "navigation.top", project, iteration, userstory, task, feature); layouts viewLayout.jsp:59, defaultLayout.jsp:44, defaultEditLayout.jsp:55.</t>
+    <t>WAR:WEB-INF/tags/breadcrumb.tag; class net.sf.xplanner.tags.NavigationBarTag#render (strings "navigation.top", project, iteration, userstory, task, feature); layouts viewLayout.jsp:59, defaultLayout.jsp:44, defaultEditLayout.jsp:55. Request-driven lookup (BA-001-10, pass-008 F-002 lead, check (l)): NavigationBarTag#doEndTag reads the request parameter oid, or else fkey. Because breadcrumb.tag passes type="${objectType}", which is an empty string when the attribute is unset, #setObject(int) looks the id up with IdSearchHelper#search (Session#get over Project, Iteration, UserStory, Task, Person and Note; WAR:WEB-INF/classes/spring-dao.xml:61) and applies no permission check. The link texts are the stored names of the hierarchy and are printed with unescaped EL (WAR:WEB-INF/tags/breadcrumb.tag:15,18). On signed-in pages this adds no exposure beyond the missing read checks (rows 29-30); on the public login and error pages it runs before sign-in (rows 8, 56; Inferred; GAP-007; Q3 facts).</t>
   </si>
   <si>
     <t>Object and project history</t>

</xml_diff>

<commit_message>
Stage 1 source reconciliation: 210 rows against upstream source and WAR
BA-001-11 reconciled every existing parity-map row against the
A4-admitted XPlanner+ SVN r426 source and the authoritative baseline
WAR: 167 confirmed, 21 correction needed, 21 runtime-only, 1 still
unsupported. 58 rows move Inferred -> Yes on method-level evidence not
contradicted by bytecode or WAR configuration (111/77/21/1 ->
169/19/21/1); 23 requirement/expected cells in 19 rows corrected;
every row keeps its old evidence as prefix plus a reconciliation note.
Carried pass-009 F-001/F-002 resolved statically; F-003 stays an
accepted residual. 27 rows keep runtime questions for Stage 3. Records
the owner's direct confirmation of the relayed source-intake decision.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -130,7 +130,7 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>WAR: = paths inside legacy/xplanner-plus.war. WAR:WEB-INF/struts-config.xml:164-167 (/login, forwards notAuthenticated -&gt; WEB-INF/jsp/security/login.jsp, authenticated -&gt; /do/view/projects redirect); WAR:WEB-INF/action-servlet.xml:10 (AuthenticationAction); WAR:WEB-INF/jsp/security/login.jsp:16-33; class com.technoetic.xplanner.actions.AuthenticationAction#execute (calls Authenticator.authenticate, forward "authenticated"). Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; login.label and login.remember are defined in the default, "--", de, it, ja and ru bundles; login.label.user_id and login.label.password in all bundles except fr; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Page-text keys (BA-001-09, pass-007 F-003, check (j)): the login page also renders login.title, given as titleKey (WAR:WEB-INF/jsp/security/login.jsp:14; defined in all bundles except fr). Through the tiles:default layout that xplanner:content inserts (class ContentTag#doStartTag; WAR:WEB-INF/tiles-definitions.xml:5-10) it also renders the footer keys app.label.version (all 10 bundles) and footer.message (only the default, "--" and de bundles; WAR:WEB-INF/jsp/common/footer.jsp:25,38) and the breadcrumb link text navigation.top (all 10 bundles; WAR:WEB-INF/jsp/layout/defaultLayout.jsp:44, WAR:WEB-INF/tags/breadcrumb.tag:10, class net.sf.xplanner.tags.NavigationBarTag#render). Bundles without a key fall back to the default text (framework behavior, GAP-011). None of these texts is credential-like (.migration-tmp/stage-01/out/public-keys-09.txt). Breadcrumb lookup (BA-001-10, pass-008 F-002 lead, check (l)): on this page the layout breadcrumb (WAR:WEB-INF/jsp/layout/defaultLayout.jsp:44, WAR:WEB-INF/tags/breadcrumb.tag:10) reads the request parameter oid, or else fkey, and loads that object without a sign-in or permission check (class net.sf.xplanner.tags.NavigationBarTag#doEndTag, #setObject(int): the type attribute arrives as an empty string, so IdSearchHelper#search runs Session#get over Project, Iteration, UserStory, Task, Person and Note). #render then adds links whose texts are the names of the object's project, iteration, story, task or feature, and breadcrumb.tag:15,18 prints them with unescaped EL. /do/login is in the security bypass list (WAR:WEB-INF/security.xml:3), so /do/login?oid=&lt;id&gt; is expected to show those names, including any markup stored in them, to a visitor who has not signed in (Inferred; the EL coercion and runtime are unverified; row 185; GAP-007; observed risk only, Q3 deferred). Page-text scope (BA-001-10): the 45 keys are the keys named by the page and layout chain; after a failed login the page also shows messages queued in code (WAR:WEB-INF/jsp/security/login.jsp:50-59): login.failed and 9 authentication.module.message.* keys named in the class bytecode, of which rows 12-13 describe the ones the XPlanner login module produces.</t>
+    <t>WAR: = paths inside legacy/xplanner-plus.war. WAR:WEB-INF/struts-config.xml:164-167 (/login, forwards notAuthenticated -&gt; WEB-INF/jsp/security/login.jsp, authenticated -&gt; /do/view/projects redirect); WAR:WEB-INF/action-servlet.xml:10 (AuthenticationAction); WAR:WEB-INF/jsp/security/login.jsp:16-33; class com.technoetic.xplanner.actions.AuthenticationAction#execute (calls Authenticator.authenticate, forward "authenticated"). Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; login.label and login.remember are defined in the default, "--", de, it, ja and ru bundles; login.label.user_id and login.label.password in all bundles except fr; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Page-text keys (BA-001-09, pass-007 F-003, check (j)): the login page also renders login.title, given as titleKey (WAR:WEB-INF/jsp/security/login.jsp:14; defined in all bundles except fr). Through the tiles:default layout that xplanner:content inserts (class ContentTag#doStartTag; WAR:WEB-INF/tiles-definitions.xml:5-10) it also renders the footer keys app.label.version (all 10 bundles) and footer.message (only the default, "--" and de bundles; WAR:WEB-INF/jsp/common/footer.jsp:25,38) and the breadcrumb link text navigation.top (all 10 bundles; WAR:WEB-INF/jsp/layout/defaultLayout.jsp:44, WAR:WEB-INF/tags/breadcrumb.tag:10, class net.sf.xplanner.tags.NavigationBarTag#render). Bundles without a key fall back to the default text (framework behavior, GAP-011). None of these texts is credential-like (.migration-tmp/stage-01/out/public-keys-09.txt). Breadcrumb lookup (BA-001-10, pass-008 F-002 lead, check (l)): on this page the layout breadcrumb (WAR:WEB-INF/jsp/layout/defaultLayout.jsp:44, WAR:WEB-INF/tags/breadcrumb.tag:10) reads the request parameter oid, or else fkey, and loads that object without a sign-in or permission check (class net.sf.xplanner.tags.NavigationBarTag#doEndTag, #setObject(int): the type attribute arrives as an empty string, so IdSearchHelper#search runs Session#get over Project, Iteration, UserStory, Task, Person and Note). #render then adds links whose texts are the names of the object's project, iteration, story, task or feature, and breadcrumb.tag:15,18 prints them with unescaped EL. /do/login is in the security bypass list (WAR:WEB-INF/security.xml:3), so /do/login?oid=&lt;id&gt; is expected to show those names, including any markup stored in them, to a visitor who has not signed in (Inferred; the EL coercion and runtime are unverified; row 185; GAP-007; observed risk only, Q3 deferred). Page-text scope (BA-001-10): the 45 keys are the keys named by the page and layout chain; after a failed login the page also shows messages queued in code (WAR:WEB-INF/jsp/security/login.jsp:50-59): login.failed and 9 authentication.module.message.* keys named in the class bytecode, of which rows 12-13 describe the ones the XPlanner login module produces. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/AuthenticationAction.java AuthenticationAction#execute (withheld file, cited by path only). WAR: classes byte-identical to the v1.1a4 release. After a successful authentication without a saved URL the action returns the authenticated forward.</t>
   </si>
   <si>
     <t>Alternative path</t>
@@ -145,7 +145,7 @@
     <t>Help text "login.instructions" with a link; the effective override file sets the URL to the XPlanner+ documentation site. With the default bundle, and with every bundle that has no own key, the text ends with the default administrator login pair (value not reproduced, CHK-009).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/security/login.jsp:34-39 (XPlannerProperties.getProperty("login.instructions.url")); WAR:WEB-INF/classes/xplanner-custom.properties:49 (login.instructions.url set) overriding WAR:WEB-INF/classes/xplanner.properties:311 (empty); override order per class com.technoetic.xplanner.XPlannerProperties$PropertyInitializer (strings "xplanner.properties", "xplanner.overrides", "xplanner-custom.properties"). Credential disclosure (BA-001-06): WAR:WEB-INF/jsp/security/login.jsp:34-39 renders bean:message login.instructions with arg0 = login.instructions.url when that URL is not empty; WAR:WEB-INF/classes/ResourceBundle.properties:784 ends with a sentence naming the default login name and password. Checked in memory without writing the value: the name equals the userId seeded at WAR:WEB-INF/classes/db-changelog.xml:403, and MD5(salt, password) matches the seeded digest at :404 (layout Base64 of a 12-byte salt followed by the digest, class XPlannerLoginModule#isPasswordMatched, #digestPassword). Locale variants (CHK-004, BA-001-06): login.instructions is defined only in the default bundle (:784, with the credential sentence), ResourceBundle--.properties:780 and ResourceBundle_de.properties:753 (both without it); da, es, fr, it, ja, pt_br and ru have no key and are expected to fall back to the default text (framework behavior, GAP-011). Whether earlier installations still accepted this pair is not established. Corrected in BA-001-06 (Source: stage-02-pass-004 F-001). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-04: the cited value is read from xplanner-custom.properties (rewritten entry, known patch target); upstream value not determinable.</t>
+    <t>WAR:WEB-INF/jsp/security/login.jsp:34-39 (XPlannerProperties.getProperty("login.instructions.url")); WAR:WEB-INF/classes/xplanner-custom.properties:49 (login.instructions.url set) overriding WAR:WEB-INF/classes/xplanner.properties:311 (empty); override order per class com.technoetic.xplanner.XPlannerProperties$PropertyInitializer (strings "xplanner.properties", "xplanner.overrides", "xplanner-custom.properties"). Credential disclosure (BA-001-06): WAR:WEB-INF/jsp/security/login.jsp:34-39 renders bean:message login.instructions with arg0 = login.instructions.url when that URL is not empty; WAR:WEB-INF/classes/ResourceBundle.properties:784 ends with a sentence naming the default login name and password. Checked in memory without writing the value: the name equals the userId seeded at WAR:WEB-INF/classes/db-changelog.xml:403, and MD5(salt, password) matches the seeded digest at :404 (layout Base64 of a 12-byte salt followed by the digest, class XPlannerLoginModule#isPasswordMatched, #digestPassword). Locale variants (CHK-004, BA-001-06): login.instructions is defined only in the default bundle (:784, with the credential sentence), ResourceBundle--.properties:780 and ResourceBundle_de.properties:753 (both without it); da, es, fr, it, ja, pt_br and ru have no key and are expected to fall back to the default text (framework behavior, GAP-011). Whether earlier installations still accepted this pair is not established. Corrected in BA-001-06 (Source: stage-02-pass-004 F-001). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/XPlannerProperties.java XPlannerProperties; SRC:src/com/technoetic/xplanner/security/module/XPlannerLoginModule.java XPlannerLoginModule#isPasswordMatched (withheld file, cited by path only). WAR: classes byte-identical to the v1.1a4 release; values from the patched WAR xplanner.properties, xplanner-custom.properties (WAR governs); the WAR db-changelog.xml differs from the SVN copy, which is withheld (WAR governs). The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-04: the cited value is read from xplanner-custom.properties (rewritten entry, known patch target); upstream value not determinable.</t>
   </si>
   <si>
     <t>After login the user is returned to the protected page they originally requested, when one was saved.</t>
@@ -154,25 +154,25 @@
     <t>Deep links (for example from an e-mail) keep working after the login detour.</t>
   </si>
   <si>
-    <t>Browser lands on the originally requested GET URL instead of the projects list.</t>
+    <t>Browser lands on the originally requested GET URL instead of the projects list; a URL that had no query string is saved and restored with the suffix "?null".</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.security.filter.FormSecurityFilter#onAuthenticationFailure (checks "GET", calls SecurityHelper.saveUrl, sendRedirect); class com.technoetic.xplanner.actions.AuthenticationAction#execute (calls SecurityHelper.getSavedUrl, new ActionForward(url, redirect)). Control flow not decompiled. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/filter/FormSecurityFilter.java FormSecurityFilter#onAuthenticationFailure; SRC:src/com/technoetic/xplanner/actions/AuthenticationAction.java AuthenticationAction#execute (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/SecurityHelper.java SecurityHelper#saveUrl, #getSavedUrl. WAR: classes byte-identical to the v1.1a4 release. The filter saves the request URL for GET requests only and redirects to the login page; after a successful login the action redirects to the saved URL when one is present. The saveUrl bytecode listing appends "?" and the query string unconditionally, as the source does, so a URL without a query string is saved with the suffix "?null".</t>
+  </si>
+  <si>
+    <t>The configured login module (XPlanner database module) validates the password against a salted MD5 digest stored for the person; the userIdCaseSensitive option is read by no live code, so whether the user ID must match in letter case is decided by the database comparison.</t>
+  </si>
+  <si>
+    <t>Explains which credential store is authoritative in the shipped configuration.</t>
+  </si>
+  <si>
+    <t>Only a matching password authenticates; whether a user ID in different letter case matches depends on the database comparison (runtime unverified).</t>
   </si>
   <si>
     <t>Inferred</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.security.filter.FormSecurityFilter#onAuthenticationFailure (checks "GET", calls SecurityHelper.saveUrl, sendRedirect); class com.technoetic.xplanner.actions.AuthenticationAction#execute (calls SecurityHelper.getSavedUrl, new ActionForward(url, redirect)). Control flow not decompiled.</t>
-  </si>
-  <si>
-    <t>The configured login module (XPlanner database module) validates the password against a salted MD5 digest stored for the person; user IDs are case sensitive.</t>
-  </si>
-  <si>
-    <t>Explains which credential store is authoritative in the shipped configuration.</t>
-  </si>
-  <si>
-    <t>Only a matching user ID (exact case) and password authenticate.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/classes/xplanner.properties:162-164 (login[0] = XPlannerLoginModule, userIdCaseSensitive=true); class com.technoetic.xplanner.security.module.XPlannerLoginModule#isPasswordMatched/#digestPassword (strings "MD5", Base64.decode); class com.technoetic.xplanner.security.module.LoginSupportImpl#getPerson (HQL "from person ... where userid = ?"). Query form (BA-001-05): LoginSupportImpl#getPerson queries "from person in class net.sf.xplanner.domain.Person where userid = ?" with the unqualified name userid, while Person maps userId (column userId). Whether the name is passed to SQL unchanged, and matched case-insensitively by the database, is framework and database behavior (GAP-011, P-01). Sweep of pass-003 F-001. Digest layout (BA-001-06): #isPasswordMatched Base64-decodes the stored value, takes the first 12 bytes as salt and compares MD5 over salt then the UTF-8 password with the rest (bytecode listing). Source: stage-02-pass-004 F-001. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/classes/xplanner.properties:162-164 (login[0] = XPlannerLoginModule, userIdCaseSensitive=true); class com.technoetic.xplanner.security.module.XPlannerLoginModule#isPasswordMatched/#digestPassword (strings "MD5", Base64.decode); class com.technoetic.xplanner.security.module.LoginSupportImpl#getPerson (HQL "from person ... where userid = ?"). Query form (BA-001-05): LoginSupportImpl#getPerson queries "from person in class net.sf.xplanner.domain.Person where userid = ?" with the unqualified name userid, while Person maps userId (column userId). Whether the name is passed to SQL unchanged, and matched case-insensitively by the database, is framework and database behavior (GAP-011, P-01). Sweep of pass-003 F-001. Digest layout (BA-001-06): #isPasswordMatched Base64-decodes the stored value, takes the first 12 bytes as salt and compares MD5 over salt then the UTF-8 password with the rest (bytecode listing). Source: stage-02-pass-004 F-001. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/security/module/XPlannerLoginModule.java XPlannerLoginModule#authenticate, #isPasswordMatched, #digestPassword (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/module/LoginSupportImpl.java LoginSupportImpl#getPerson; SRC:src/com/technoetic/xplanner/security/SecurityHelper.java SecurityHelper#isAuthenticationCaseSensitive; SRC:src/com/technoetic/xplanner/domain/repository/PersonHibernateObjectRepository.java PersonHibernateObjectRepository#hasSameUserId. WAR: classes byte-identical to the v1.1a4 release; login-module keys from the patched WAR xplanner.properties (WAR governs). The salted digest check is confirmed (12-byte salt, digest over salt and password, byte comparison). The case-sensitivity claim is not: the userIdCaseSensitive option is read only by SecurityHelper#isAuthenticationCaseSensitive, whose only use is commented out in PersonHibernateObjectRepository#hasSameUserId (the bytecode has no caller either); the login query compares the user ID with an HQL equality, so case matching is decided by the database comparison. Live question: Does a login with the seeded user ID in different letter case succeed against the MySQL database? Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
   </si>
   <si>
     <t>Login rejected</t>
@@ -187,7 +187,7 @@
     <t>Login page redisplayed with "Could not authenticate user." plus a module message such as "Wrong userid or password".</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/security/login.jsp:50-59 (GLOBAL_MESSAGE and moduleMessages); class AuthenticationAction#execute (strings "login.failed", "moduleMessages", forward "notAuthenticated"); WAR:WEB-INF/classes/ResourceBundle.properties keys login.failed, authentication.module.message.authenticationFailed. Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; login.failed is defined in all bundles except fr; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9).</t>
+    <t>WAR:WEB-INF/jsp/security/login.jsp:50-59 (GLOBAL_MESSAGE and moduleMessages); class AuthenticationAction#execute (strings "login.failed", "moduleMessages", forward "notAuthenticated"); WAR:WEB-INF/classes/ResourceBundle.properties keys login.failed, authentication.module.message.authenticationFailed. Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; login.failed is defined in all bundles except fr; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/AuthenticationAction.java AuthenticationAction#execute (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/LoginContext.java LoginContext#authenticate. WAR: classes byte-identical to the v1.1a4 release. A failed authentication adds the global login-failed message and one message per module, and returns the login page.</t>
   </si>
   <si>
     <t>An unknown user ID or a person without a password produces a specific module message.</t>
@@ -199,7 +199,7 @@
     <t>Messages "User has not been registered with XPlanner..." or "Password has not been set...".</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.security.module.LoginSupportImpl#populateSubjectPrincipalFromDatabase (string "authentication.module.message.userNotFound"); class XPlannerLoginModule#isPasswordMatched (string "authentication.module.message.passwordNotSet"); ResourceBundle.properties same keys. Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; authentication.module.message.userNotFound and passwordNotSet are defined only in the default, "--", de and ja bundles; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9).</t>
+    <t>class com.technoetic.xplanner.security.module.LoginSupportImpl#populateSubjectPrincipalFromDatabase (string "authentication.module.message.userNotFound"); class XPlannerLoginModule#isPasswordMatched (string "authentication.module.message.passwordNotSet"); ResourceBundle.properties same keys. Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; authentication.module.message.userNotFound and passwordNotSet are defined only in the default, "--", de and ja bundles; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/module/LoginSupportImpl.java LoginSupportImpl#populateSubjectPrincipalFromDatabase; SRC:src/com/technoetic/xplanner/security/module/XPlannerLoginModule.java XPlannerLoginModule#isPasswordMatched (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/LoginContext.java LoginContext#authenticate. WAR: classes byte-identical to the v1.1a4 release. A missing person raises the user-not-found key and a null stored password raises the password-not-set key; LoginContext#authenticate collects each module's message key per module name, and the action shows them as module messages.</t>
   </si>
   <si>
     <t>A request to the login action without the submit field (for example a plain GET of /do/login) shows the login form; empty user ID or password values are not checked by the action and are passed to the login module, which rejects them.</t>
@@ -211,7 +211,7 @@
     <t>Login form (notAuthenticated) without an error on first visit; after submitting blank credentials: "Could not authenticate user." with a module message (for example "User has not been registered with XPlanner").</t>
   </si>
   <si>
-    <t>class AuthenticationAction#execute: the first branch tests StringUtils.isEmpty on the form field "action" (the submit button) and returns forward "notAuthenticated"; "userId" and "password" are then read and passed to Authenticator.authenticate without an emptiness check (bytecode listing, .migration-tmp/stage-01/tools/disasm.js); rejection messages per class LoginSupportImpl (authentication.module.message.userNotFound). Corrected in BA-001-04 (Source: stage-02-pass-002 F-005). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; authentication.module.message.userNotFound is defined only in the default, "--", de and ja bundles. Bundles without the key fall back to the default text (framework behavior, GAP-011).</t>
+    <t>class AuthenticationAction#execute: the first branch tests StringUtils.isEmpty on the form field "action" (the submit button) and returns forward "notAuthenticated"; "userId" and "password" are then read and passed to Authenticator.authenticate without an emptiness check (bytecode listing, .migration-tmp/stage-01/tools/disasm.js); rejection messages per class LoginSupportImpl (authentication.module.message.userNotFound). Corrected in BA-001-04 (Source: stage-02-pass-002 F-005). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; authentication.module.message.userNotFound is defined only in the default, "--", de and ja bundles. Bundles without the key fall back to the default text (framework behavior, GAP-011). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/AuthenticationAction.java AuthenticationAction#execute (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/AuthenticatorImpl.java AuthenticatorImpl#authenticate; SRC:src/com/technoetic/xplanner/security/module/LoginSupportImpl.java LoginSupportImpl#getPerson, #populateSubjectPrincipalFromDatabase. WAR: classes byte-identical to the v1.1a4 release. The action returns the not-authenticated forward when the submit field is empty and otherwise passes user ID and password unchecked to the authenticator; an empty user ID finds no person (as long as no person has an empty user ID) and raises the user-not-found message.</t>
   </si>
   <si>
     <t>Remember me</t>
@@ -226,7 +226,7 @@
     <t>Cookies "userid" and "password" are set (Base64-encoded values).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/security/login.jsp:29 (checkbox remember, value Y, checked by default); class AuthenticationAction#execute (strings "remember", "Y", CredentialCookie.set); class com.technoetic.xplanner.security.CredentialCookie#set (cookie names "userid", "password", Base64.encode). Cookie lifetime and flags (BA-001-07, mechanism (b)): CredentialCookie#set writes the user id and the Base64 of the clear password through CookieSupport#createCookie, which sets max-age 2147483647 seconds (about 68 years), sets neither Secure nor a path, and cannot set HttpOnly under the Servlet 2.4 API (bytecode listings). Observed risk only (Q3 deferred). Source: stage-02-pass-005 F-003.</t>
+    <t>WAR:WEB-INF/jsp/security/login.jsp:29 (checkbox remember, value Y, checked by default); class AuthenticationAction#execute (strings "remember", "Y", CredentialCookie.set); class com.technoetic.xplanner.security.CredentialCookie#set (cookie names "userid", "password", Base64.encode). Cookie lifetime and flags (BA-001-07, mechanism (b)): CredentialCookie#set writes the user id and the Base64 of the clear password through CookieSupport#createCookie, which sets max-age 2147483647 seconds (about 68 years), sets neither Secure nor a path, and cannot set HttpOnly under the Servlet 2.4 API (bytecode listings). Observed risk only (Q3 deferred). Source: stage-02-pass-005 F-003. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/security/CredentialCookie.java CredentialCookie#set (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/util/CookieSupport.java CookieSupport#createCookie. WAR: classes byte-identical to the v1.1a4 release. The user ID and the Base64-encoded password are stored in two cookies with max-age Integer.MAX_VALUE, no Secure flag and no path.</t>
   </si>
   <si>
     <t>A request without a session but with the credential cookies is authenticated automatically.</t>
@@ -238,7 +238,7 @@
     <t>Protected page opens without the login form; a failed cookie login falls back to the login redirect.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.security.filter.FormSecurityFilter#isAuthenticated (CredentialCookie.isPresent/getUserId/getPassword, Authenticator.authenticate, log "cookie-based authentication failed"); #onAuthenticationFailure (CredentialCookie.remove).</t>
+    <t>class com.technoetic.xplanner.security.filter.FormSecurityFilter#isAuthenticated (CredentialCookie.isPresent/getUserId/getPassword, Authenticator.authenticate, log "cookie-based authentication failed"); #onAuthenticationFailure (CredentialCookie.remove). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/filter/FormSecurityFilter.java FormSecurityFilter#isAuthenticated, #onAuthenticationFailure; SRC:src/com/technoetic/xplanner/security/filter/AbstractSecurityFilter.java AbstractSecurityFilter#doFilter. WAR: classes byte-identical to the v1.1a4 release. Without a subject in the session the filter authenticates with the cookie values; a failure is logged and leads to onAuthenticationFailure, which removes the cookies, saves the URL for GET requests and redirects to the login page.</t>
   </si>
   <si>
     <t>Access protected pages without a session</t>
@@ -253,7 +253,7 @@
     <t>Unauthenticated request is redirected to the login page.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:85-96,160-167 (WebSecurityFilter on /do/* and /setting/*, authenticatorUrl /do/login); WAR:WEB-INF/security.xml:2-6 (bypass /do/login, /do/notAuthorized, /do/invalidateHibernateCache); class com.technoetic.xplanner.security.config.SecurityConfiguration#isSecureRequest (uses only securityBypass).</t>
+    <t>WAR:WEB-INF/web.xml:85-96,160-167 (WebSecurityFilter on /do/* and /setting/*, authenticatorUrl /do/login); WAR:WEB-INF/security.xml:2-6 (bypass /do/login, /do/notAuthorized, /do/invalidateHibernateCache); class com.technoetic.xplanner.security.config.SecurityConfiguration#isSecureRequest (uses only securityBypass). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/security/filter/AbstractSecurityFilter.java AbstractSecurityFilter#doFilter; SRC:src/com/technoetic/xplanner/security/config/SecurityConfiguration.java SecurityConfiguration#isSecureRequest; SRC:src/com/technoetic/xplanner/security/filter/FormSecurityFilter.java FormSecurityFilter#onAuthenticationFailure. WAR: security.xml and web.xml identical to the SVN webapp copies. Every request not on the bypass list must be authenticated; otherwise the filter redirects to its login URL.</t>
   </si>
   <si>
     <t>The root URL routes the user: with exactly one visible project that has a current iteration it redirects to that iteration, otherwise to the projects list.</t>
@@ -265,7 +265,7 @@
     <t>Browser is redirected to /do/view/iteration?oid=&lt;current&gt; or /do/view/projects.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:321-323 (welcome-file index.jsp); WAR:index.jsp:7-31 (useBeans Project where hidden = false; redirects). Access condition (BA-001-06): index.jsp is not covered by any security filter mapping (WAR:WEB-INF/web.xml:155-176 map the filters to /do/mobile/*, /do/*, /setting/*, /soap/* and /ical/*; welcome file at :321-323); the /index.jsp entry in WAR:WEB-INF/security.xml:16 is never evaluated (row 32). Without a session the page runs the hidden = false project query and, when exactly one visible project with a current iteration exists, redirects to /do/view/iteration?oid=&lt;id&gt;, which reveals that id before login; the target page then requires login. Observed risk only (Q3 deferred). Mechanical list: .migration-tmp/stage-01/out/unauth-06.txt. Source: stage-02-pass-004 F-005.</t>
+    <t>WAR:WEB-INF/web.xml:321-323 (welcome-file index.jsp); WAR:index.jsp:7-31 (useBeans Project where hidden = false; redirects). Access condition (BA-001-06): index.jsp is not covered by any security filter mapping (WAR:WEB-INF/web.xml:155-176 map the filters to /do/mobile/*, /do/*, /setting/*, /soap/* and /ical/*; welcome file at :321-323); the /index.jsp entry in WAR:WEB-INF/security.xml:16 is never evaluated (row 32). Without a session the page runs the hidden = false project query and, when exactly one visible project with a current iteration exists, redirects to /do/view/iteration?oid=&lt;id&gt;, which reveals that id before login; the target page then requires login. Observed risk only (Q3 deferred). Mechanical list: .migration-tmp/stage-01/out/unauth-06.txt. Source: stage-02-pass-004 F-005. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Log out</t>
@@ -280,7 +280,7 @@
     <t>Session is invalidated, remember-me cookies are removed and the login page is shown.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:21 (link /do/logout); WAR:WEB-INF/struts-config.xml:171; WAR:WEB-INF/action-servlet.xml:16; class com.technoetic.xplanner.actions.LogoutAction#execute (Authenticator.logout, CredentialCookie.remove, forward "security/login"); class XPlannerLoginModule#logout (HttpSession.invalidate).</t>
+    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:21 (link /do/logout); WAR:WEB-INF/struts-config.xml:171; WAR:WEB-INF/action-servlet.xml:16; class com.technoetic.xplanner.actions.LogoutAction#execute (Authenticator.logout, CredentialCookie.remove, forward "security/login"); class XPlannerLoginModule#logout (HttpSession.invalidate). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/LogoutAction.java LogoutAction#execute. WAR: classes byte-identical to the v1.1a4 release. Logout calls the authenticator, removes the credential cookies and forwards to the login page.</t>
   </si>
   <si>
     <t>Session expiry</t>
@@ -298,7 +298,7 @@
     <t>Next request after 30 idle minutes is treated as unauthenticated (unless the remember-me cookies re-authenticate).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:318-320 (session-timeout 30); cookie re-login per class FormSecurityFilter#isAuthenticated.</t>
+    <t>WAR:WEB-INF/web.xml:318-320 (session-timeout 30); cookie re-login per class FormSecurityFilter#isAuthenticated. Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/security/filter/FormSecurityFilter.java FormSecurityFilter#isAuthenticated. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
   </si>
   <si>
     <t>Alternative login modules (LDAP/JNDI, NTLM, JAAS)</t>
@@ -316,7 +316,7 @@
     <t>Partial</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/xplanner.properties:167-190 (login[1] JNDI and login[2] NTLM commented out); WAR:WEB-INF/classes/spring-security.xml:38-43 (JaasLoginModuleAdapterFactory, NtlmLoginModule, JNDILoginModule, JNDIAuthenticatorImpl beans); classes com.technoetic.xplanner.security.module.jndi.JNDILoginModule, .ntlm.NtlmLoginModule, com.sabre.security.jndi.*. Not active in the shipped file. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/classes/xplanner.properties:167-190 (login[1] JNDI and login[2] NTLM commented out); WAR:WEB-INF/classes/spring-security.xml:38-43 (JaasLoginModuleAdapterFactory, NtlmLoginModule, JNDILoginModule, JNDIAuthenticatorImpl beans); classes com.technoetic.xplanner.security.module.jndi.JNDILoginModule, .ntlm.NtlmLoginModule, com.sabre.security.jndi.*. Not active in the shipped file. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/security/module/LoginModuleLoader.java LoginModuleLoader#loadLoginModules; SRC:src/com/technoetic/xplanner/security/module/jndi/JNDILoginModule.java JNDILoginModule; SRC:src/com/sabre/security/jndi/JNDIAuthenticatorImpl.java (withheld file, cited by path only). WAR: classes byte-identical to the v1.1a4 release; login modules from the patched WAR xplanner.properties (WAR governs). The loader builds modules only from the login[n] keys present, and the WAR file defines login[0] only. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
   </si>
   <si>
     <t>UF-002</t>
@@ -337,7 +337,7 @@
     <t>A sysadmin can do everything; an admin has editor and viewer rights plus admin*; an editor can create/edit/delete/integrate; a viewer can read.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/db-changelog.xml:363-386 (roles viewer lft1/rgt8, editor 2/7, admin 3/6, sysadmin 4/5) and :275-362 (permission rows); WAR:WEB-INF/classes/mappings/Metrics.xml queries "security.roles" and "security.role.permissions" (r1.left between r2.left and r2.right for positive permissions). Server-side enforcement (CHK-002, BA-001-04): the role model is evaluated on the server only on the paths in rows 28, 31, 167, 180, 218 and 230; everywhere else it only decides which links and fields the JSP pages show (rows 26, 29-30).</t>
+    <t>WAR:WEB-INF/classes/db-changelog.xml:363-386 (roles viewer lft1/rgt8, editor 2/7, admin 3/6, sysadmin 4/5) and :275-362 (permission rows); WAR:WEB-INF/classes/mappings/Metrics.xml queries "security.roles" and "security.role.permissions" (r1.left between r2.left and r2.right for positive permissions). Server-side enforcement (CHK-002, BA-001-04): the role model is evaluated on the server only on the paths in rows 28, 31, 167, 180, 218 and 230; everywhere else it only decides which links and fields the JSP pages show (rows 26, 29-30). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/auth/AuthorizerImpl.java AuthorizerImpl#hasPermission, #permissionMatches, #isMatching; SRC:src/com/technoetic/xplanner/security/auth/PrincipalSpecificPermissionHelper.java PrincipalSpecificPermissionHelper#getPermissionsForPrincipal. WAR: classes byte-identical to the v1.1a4 release; seed data in db-changelog.xml (WAR entry; the SVN copy differs and is withheld; WAR governs). Permissions are loaded per principal and project and matched with trailing-% prefix patterns; the nested role ranges come from the WAR seed data and the named queries of Metrics.xml, so the hierarchy holds for the seeded data.</t>
   </si>
   <si>
     <t>Negative permissions apply to the exact role only: editors may not create projects, create people or delete iterations; admins may not create projects.</t>
@@ -349,7 +349,7 @@
     <t>"Create project" and "Add person" links and iteration delete buttons are hidden for those roles. Nothing refuses a direct request (rows 29-30).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/db-changelog.xml permission ids 7, 8, 9, 19 (positive=false); WAR:WEB-INF/classes/mappings/Metrics.xml "security.role.permissions" (positive=0 and r1.id = r2.id). Evaluation order in class com.technoetic.xplanner.security.auth.AuthorizerImpl not decompiled. Server-side enforcement (CHK-002, BA-001-04): these restrictions only hide links and buttons; the create and delete handlers perform no server-side permission check (rows 29-30). Corrected in BA-001-04 (Source: stage-02-pass-002 F-007).</t>
+    <t>WAR:WEB-INF/classes/db-changelog.xml permission ids 7, 8, 9, 19 (positive=false); WAR:WEB-INF/classes/mappings/Metrics.xml "security.role.permissions" (positive=0 and r1.id = r2.id). Evaluation order in class com.technoetic.xplanner.security.auth.AuthorizerImpl not decompiled. Server-side enforcement (CHK-002, BA-001-04): these restrictions only hide links and buttons; the create and delete handlers perform no server-side permission check (rows 29-30). Corrected in BA-001-04 (Source: stage-02-pass-002 F-007). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/auth/AuthorizerImpl.java AuthorizerImpl#permissionMatches. WAR: classes byte-identical to the v1.1a4 release; seed data in the WAR db-changelog.xml. The evaluation order is now visible: within one project list a matching negative permission defeats any matching positive one (positive and not negative); the exact-role scope of negative permissions comes from the Metrics.xml query.</t>
   </si>
   <si>
     <t>A role assigned for project 0 applies to all projects (the seeded sysadmin is assigned this way).</t>
@@ -361,7 +361,7 @@
     <t>Seeded sysadmin sees and administers every project.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/db-changelog.xml:407-411 (person_role role 5, person 1, project 0); Metrics.xml "security.roles" (:includeWildcardProject = 1 and pr.id.projectId = 0). Server-side enforcement (CHK-002, BA-001-04): as for the role model, only the server-side paths in rows 28, 31, 167, 180, 218 and 230 evaluate it; project 0 is also the scope of the system-administrator rule in rows 31 and 34.</t>
+    <t>WAR:WEB-INF/classes/db-changelog.xml:407-411 (person_role role 5, person 1, project 0); Metrics.xml "security.roles" (:includeWildcardProject = 1 and pr.id.projectId = 0). Server-side enforcement (CHK-002, BA-001-04): as for the role model, only the server-side paths in rows 28, 31, 167, 180, 218 and 230 evaluate it; project 0 is also the scope of the system-administrator rule in rows 31 and 34. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/auth/AuthorizerImpl.java AuthorizerImpl#hasPermission (ANY_PROJECT = 0). WAR: classes byte-identical to the v1.1a4 release; seed data in the WAR db-changelog.xml. HasPermission grants when the permissions of the requested project or those of project 0 match, so a role on project 0 applies to every project.</t>
   </si>
   <si>
     <t>Permission-driven UI actions</t>
@@ -376,7 +376,7 @@
     <t>Icons/links appear or disappear by permission (for example project delete requires sysadmin.delete, project edit admin.edit).</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.domain.DomainMetaDataRepository#init (action definitions with permissions "admin.edit", "sysadmin.delete", "edit", "delete"); WAR:WEB-INF/xplanner.tld (isUserAuthorized -&gt; com.technoetic.xplanner.tags.IsUserAuthorizedTag); e.g. WAR:WEB-INF/jsp/view/projects.jsp:82-100. Corrected in BA-001-03 (stage-02-pass-001 F-001): the gating is in JSP tags only. Server-side enforcement (CHK-002, BA-001-04): display-level only; the handlers behind these links perform no server-side permission check (rows 29-30), except the person-editor role rules (row 31).</t>
+    <t>class com.technoetic.xplanner.domain.DomainMetaDataRepository#init (action definitions with permissions "admin.edit", "sysadmin.delete", "edit", "delete"); WAR:WEB-INF/xplanner.tld (isUserAuthorized -&gt; com.technoetic.xplanner.tags.IsUserAuthorizedTag); e.g. WAR:WEB-INF/jsp/view/projects.jsp:82-100. Corrected in BA-001-03 (stage-02-pass-001 F-001): the gating is in JSP tags only. Server-side enforcement (CHK-002, BA-001-04): display-level only; the handlers behind these links perform no server-side permission check (rows 29-30), except the person-editor role rules (row 31). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init; SRC:src/com/technoetic/xplanner/tags/IsUserAuthorizedTag.java IsUserAuthorizedTag. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
   </si>
   <si>
     <t>The projects list shows only projects the user may read.</t>
@@ -388,7 +388,7 @@
     <t>Projects without read permission are not listed.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/projects.jsp:32-48 (CollectionUtils.filter with SystemAuthorizer.hasPermission(..., "read")). Server-side enforcement (CHK-002, BA-001-04): this filters the list rendered on the server, but the project pages themselves have no read check (row 29).</t>
+    <t>WAR:WEB-INF/jsp/view/projects.jsp:32-48 (CollectionUtils.filter with SystemAuthorizer.hasPermission(..., "read")). Server-side enforcement (CHK-002, BA-001-04): this filters the list rendered on the server, but the project pages themselves have no read check (row 29). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Only views handled by DispatchForward with authorization required check permission (the flag defaults to true and is switched off for projects, people, settings, dashboard, twiki format and not-authorized): without a projectId parameter, or without read permission on system.project, they forward to security/notAuthorized, whose JSP is absent.</t>
@@ -400,7 +400,7 @@
     <t>For /do/view/integrations and the WAP views: not-authorized forward (expected error, page missing). The global AuthorizationException mapping to generalError.jsp (security.notauthorized) is reachable only through the secure repository adapter, which no working web path uses.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.actions.DispatchForward: #isSecure uses a "@secure" forward if present, otherwise field isAuthorizationRequired; #&lt;init&gt; sets isAuthorizationRequired true; #execute reads projectId and calls Authorizer.hasPermission(..., "system.project", ..., "read"), else forward "security/notAuthorized" (bytecode listing by .migration-tmp/stage-01/tools/disasm.js); no "@secure" forward in any descriptor; WAR:WEB-INF/action-servlet.xml:12-14,25-31,327-331,390,412-418; WAR:WEB-INF/struts-config.xml:139 (notAuthorized.jsp ABSENT, GAP-003) and :87-89; RepositorySecurityAdapter#checkAuthorization is the only constructor call of AuthorizationException. Corrected in BA-001-03 (F-001; narrows the reviewer statement that DispatchForward never checks).</t>
+    <t>class com.technoetic.xplanner.actions.DispatchForward: #isSecure uses a "@secure" forward if present, otherwise field isAuthorizationRequired; #&lt;init&gt; sets isAuthorizationRequired true; #execute reads projectId and calls Authorizer.hasPermission(..., "system.project", ..., "read"), else forward "security/notAuthorized" (bytecode listing by .migration-tmp/stage-01/tools/disasm.js); no "@secure" forward in any descriptor; WAR:WEB-INF/action-servlet.xml:12-14,25-31,327-331,390,412-418; WAR:WEB-INF/struts-config.xml:139 (notAuthorized.jsp ABSENT, GAP-003) and :87-89; RepositorySecurityAdapter#checkAuthorization is the only constructor call of AuthorizationException. Corrected in BA-001-03 (F-001; narrows the reviewer statement that DispatchForward never checks). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DispatchForward.java DispatchForward#execute, #isSecure. WAR: classes byte-identical to the v1.1a4 release. The view checks a "@secure" forward first and otherwise the authorization flag, then requires a projectId and system.project read, as recorded; the not-authorized JSP stays absent from the WAR.</t>
   </si>
   <si>
     <t>Server-side permission enforcement</t>
@@ -415,7 +415,7 @@
     <t>Direct requests succeed for any signed-in user (runtime unverified).</t>
   </si>
   <si>
-    <t>Static call graph from each entry point to authorization calls (.migration-tmp/stage-01/tools/authtrace.js, out/authtrace.json): no Authorizer, SystemAuthorizer or RepositorySecurityAdapter call is reachable from ViewObjectAction#doExecute, EditObjectAction#updateObject/#createObject or DeleteObjectAction#doExecute, which call CommonDao.getById/save/delete and EventManager.publish*; beans WAR:WEB-INF/action-servlet.xml:33-43,72-82,84-130,196-212,214-224,256-272,300-304,352-356,370-374,420-424. Inferred from bytecode; Stage 3 confirmation needed. Source: stage-02-pass-001 F-001.</t>
+    <t>Static call graph from each entry point to authorization calls (.migration-tmp/stage-01/tools/authtrace.js, out/authtrace.json): no Authorizer, SystemAuthorizer or RepositorySecurityAdapter call is reachable from ViewObjectAction#doExecute, EditObjectAction#updateObject/#createObject or DeleteObjectAction#doExecute, which call CommonDao.getById/save/delete and EventManager.publish*; beans WAR:WEB-INF/action-servlet.xml:33-43,72-82,84-130,196-212,214-224,256-272,300-304,352-356,370-374,420-424. Inferred from bytecode; Stage 3 confirmation needed. Source: stage-02-pass-001 F-001. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/AbstractAction.java AbstractAction#execute; SRC:src/com/technoetic/xplanner/actions/ViewObjectAction.java ViewObjectAction#doExecute, #isSecure; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#doExecute, #updateObject, #createObject; SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. None of these methods calls an authorizer; AbstractAction#execute only wraps doExecute and the hooks in a transaction. ViewObjectAction's authorizationRequired flag only decides whether the object is loaded into the domain context, it gates nothing.</t>
   </si>
   <si>
     <t>The other web actions likewise have no server-side permission check: export, import of people and stories, move/continue of stories and tasks, multi-move, reorder, time entry, notes and attachment download, file manager, integration queue, iteration start/close and continue, notification receivers, project role editor, personal timesheet, ID search, the "me" page and the test/admin utilities.</t>
@@ -424,7 +424,7 @@
     <t>Same enforcement gap across all action types (impact sweep of F-001). Observed behavior and risk only (Q3 deferred).</t>
   </si>
   <si>
-    <t>.migration-tmp/stage-01/out/authtrace.json: 80 web action beans, 7 WAP actions, 43 SOAP operations, 4 REST methods, the iCal servlet and 3 Spring MVC handlers traced. For web actions, authorization calls are reachable only from DispatchForward, EditPersonAction (role changes), ViewAggregateTimesheetAction (result filter), InvalidateCacheAction (cache reset) and, not as a gate, inside e-mail recipient or metrics lookups (EditTaskAction, IntegrationAction, CommandExecutorAction, ViewIterationMetricsAction). Tracer limits: control flow and framework callbacks are not followed.</t>
+    <t>.migration-tmp/stage-01/out/authtrace.json: 80 web action beans, 7 WAP actions, 43 SOAP operations, 4 REST methods, the iCal servlet and 3 Spring MVC handlers traced. For web actions, authorization calls are reachable only from DispatchForward, EditPersonAction (role changes), ViewAggregateTimesheetAction (result filter), InvalidateCacheAction (cache reset) and, not as a gate, inside e-mail recipient or metrics lookups (EditTaskAction, IntegrationAction, CommandExecutorAction, ViewIterationMetricsAction). Tracer limits: control flow and framework callbacks are not followed. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ (package search: only DispatchForward, EditPersonHelper, EditRoleAction, SearchResultAuthorizationPredicate and admin/InvalidateCacheAction refer to the authorizer). WAR: classes byte-identical to the v1.1a4 release. The package search agrees with the bytecode trace; the status stays Inferred because not every listed action was read at method level.</t>
   </si>
   <si>
     <t>Server-side role changes in the person editor are applied only for projects on which the current user holds admin.edit.role; in addition, when the current user holds admin.edit.role on project 0, every save of the person editor first removes the person's sysadmin role and re-adds it only if the form carries systemAdmin=true.</t>
@@ -436,7 +436,7 @@
     <t>Role changes for other projects are ignored; the sysadmin role is revoked or granted by the project-0 rule (runtime unverified).</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.actions.EditPersonHelper#modifyRoles: for each submitted project role, #isCurrentUserAdminOfProject(projectId, user) (Authorizer.hasPermission with "system.project", "admin.edit.role") gates #setRoleOnProject; then #isCurrentUserAdminOfProject(0, user) gates RoleAssociationRepository.deleteForPersonOnProject("sysadmin", person, 0), followed by #setSysadmin only when the systemAdmin flag is true (bytecode listing); caller EditPersonAction#beforeObjectCommit passes PersonEditorForm#isSystemAdmin. class PersonEditorForm uses the authorizer only to preselect displayed roles (#getRoles, #isRoleSelected), not as a gate. The rest of the person edit (name, e-mail, password, hidden) is not permission-checked on the server. Corrected in BA-001-04 (Source: stage-02-pass-002 F-007). Server-side enforcement (CHK-002, BA-001-04): this row records the server-side check itself (Authorizer.hasPermission reached from EditPersonAction#beforeObjectCommit, .migration-tmp/stage-01/out/authtrace.json).</t>
+    <t>class com.technoetic.xplanner.actions.EditPersonHelper#modifyRoles: for each submitted project role, #isCurrentUserAdminOfProject(projectId, user) (Authorizer.hasPermission with "system.project", "admin.edit.role") gates #setRoleOnProject; then #isCurrentUserAdminOfProject(0, user) gates RoleAssociationRepository.deleteForPersonOnProject("sysadmin", person, 0), followed by #setSysadmin only when the systemAdmin flag is true (bytecode listing); caller EditPersonAction#beforeObjectCommit passes PersonEditorForm#isSystemAdmin. class PersonEditorForm uses the authorizer only to preselect displayed roles (#getRoles, #isRoleSelected), not as a gate. The rest of the person edit (name, e-mail, password, hidden) is not permission-checked on the server. Corrected in BA-001-04 (Source: stage-02-pass-002 F-007). Server-side enforcement (CHK-002, BA-001-04): this row records the server-side check itself (Authorizer.hasPermission reached from EditPersonAction#beforeObjectCommit, .migration-tmp/stage-01/out/authtrace.json). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/EditPersonHelper.java EditPersonHelper#modifyRoles, #isCurrentUserAdminOfProject, #setSysadmin; SRC:src/com/technoetic/xplanner/actions/EditPersonAction.java EditPersonAction#beforeObjectCommit. WAR: classes byte-identical to the v1.1a4 release. ModifyRoles applies each submitted project role only when the current user is admin of that project, then, for a project-0 admin, deletes the person's sysadmin role on project 0 and re-adds it only when the flag is set; the order matches the bytecode listing.</t>
   </si>
   <si>
     <t>URL role constraints in security.xml, mobile-security.xml and soap-security.xml are parsed but never evaluated; the security filters only check the bypass list and that the user is authenticated.</t>
@@ -448,7 +448,7 @@
     <t>Any authenticated user passes the filters for every constrained URL.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.security.config.SecurityConfiguration#isAuthorized has no caller in any class (positive control: #isSecureRequest is called by AbstractSecurityFilter#isSecureRequest); AbstractSecurityFilter#doFilter calls only isSecureRequest, isAuthenticated and onAuthenticationFailure; WAR:WEB-INF/security.xml:9-39, WAR:WEB-INF/mobile-security.xml:6-16, WAR:WEB-INF/soap-security.xml:2-34. Source: stage-02-pass-001 F-001 and F-004.</t>
+    <t>class com.technoetic.xplanner.security.config.SecurityConfiguration#isAuthorized has no caller in any class (positive control: #isSecureRequest is called by AbstractSecurityFilter#isSecureRequest); AbstractSecurityFilter#doFilter calls only isSecureRequest, isAuthenticated and onAuthenticationFailure; WAR:WEB-INF/security.xml:9-39, WAR:WEB-INF/mobile-security.xml:6-16, WAR:WEB-INF/soap-security.xml:2-34. Source: stage-02-pass-001 F-001 and F-004. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/filter/AbstractSecurityFilter.java AbstractSecurityFilter#doFilter, #isSecureRequest; SRC:src/com/technoetic/xplanner/security/config/SecurityConfiguration.java SecurityConfiguration#isAuthorized (no caller in the source tree). WAR: classes byte-identical to the v1.1a4 release. DoFilter only checks the bypass list and authentication; no source file calls SecurityConfiguration#isAuthorized.</t>
   </si>
   <si>
     <t>Assign project roles to a person</t>
@@ -463,7 +463,7 @@
     <t>Per-project radio buttons in the person editor; saved roles change what the person can see and do.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (isUserAuthorizedForAny projects permissions admin.edit.role; radio options none/viewer/editor/admin); WAR:WEB-INF/classes/spring-beans.xml:193-203 (editPersonHelper with invalidateCacheAfterPermissionChangedAdvisor on modifyRoles). Server-side enforcement (CHK-002, BA-001-04): enforced on the server per project by EditPersonHelper#isCurrentUserAdminOfProject (row 31); the editor page itself is reachable by any signed-in user (row 29). Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (isUserAuthorizedForAny projects permissions admin.edit.role; radio options none/viewer/editor/admin); WAR:WEB-INF/classes/spring-beans.xml:193-203 (editPersonHelper with invalidateCacheAfterPermissionChangedAdvisor on modifyRoles). Server-side enforcement (CHK-002, BA-001-04): enforced on the server per project by EditPersonHelper#isCurrentUserAdminOfProject (row 31); the editor page itself is reachable by any signed-in user (row 29). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/EditPersonHelper.java EditPersonHelper#modifyRoles, #isCurrentUserAdminOfProject. WAR: classes byte-identical to the v1.1a4 release. Each project role is set only when the current user is admin of that project. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
   </si>
   <si>
     <t>The "System administrator" checkbox is shown only to sysadmin.promote holders, but on the server the sysadmin role is governed by admin.edit.role on project 0: when a user holding it saves any person editor, the person's sysadmin role is removed and re-added only if systemAdmin=true is posted.</t>
@@ -475,7 +475,7 @@
     <t>Checkbox visible only to sysadmins; saving the person editor as a project-0 administrator without the checkbox revokes the person's system-administrator role; posting systemAdmin=true grants it (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp:144-151 (isUserAuthorized resourceType="system" permission="sysadmin.promote", input systemAdmin); class EditPersonHelper#modifyRoles, #isCurrentUserAdminOfProject, #setSysadmin (bytecode listing: deleteForPersonOnProject("sysadmin", personId, 0) then setSysadmin when the flag is true); class EditPersonAction#beforeObjectCommit (PersonEditorForm#isSystemAdmin). Who holds admin.edit.role on project 0 follows the role model (rows 23-25; sysadmin via "%", admin via "admin%" when assigned on project 0), Inferred. Corrected in BA-001-04 (Source: stage-02-pass-002 F-007). Server-side enforcement (CHK-002, BA-001-04): sysadmin.promote is display-level only; the server-side check that governs the sysadmin role is admin.edit.role on project 0 (row 31).</t>
+    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp:144-151 (isUserAuthorized resourceType="system" permission="sysadmin.promote", input systemAdmin); class EditPersonHelper#modifyRoles, #isCurrentUserAdminOfProject, #setSysadmin (bytecode listing: deleteForPersonOnProject("sysadmin", personId, 0) then setSysadmin when the flag is true); class EditPersonAction#beforeObjectCommit (PersonEditorForm#isSystemAdmin). Who holds admin.edit.role on project 0 follows the role model (rows 23-25; sysadmin via "%", admin via "admin%" when assigned on project 0), Inferred. Corrected in BA-001-04 (Source: stage-02-pass-002 F-007). Server-side enforcement (CHK-002, BA-001-04): sysadmin.promote is display-level only; the server-side check that governs the sysadmin role is admin.edit.role on project 0 (row 31). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/EditPersonHelper.java EditPersonHelper#modifyRoles, #setSysadmin; SRC:src/com/technoetic/xplanner/actions/EditPersonAction.java EditPersonAction#beforeObjectCommit. WAR: classes byte-identical to the v1.1a4 release. As row 31: the checkbox is display-level (editPerson.jsp), and the server applies the project-0 admin.edit.role rule.</t>
   </si>
   <si>
     <t>Edit project roles (project role editor)</t>
@@ -490,7 +490,7 @@
     <t>Form posted to /do/edit/roles; the role-saving code is expected never to run, so submitted roles are not saved (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:409-411; WAR:WEB-INF/action-servlet.xml:400-404 (EditRoleAction); WAR:WEB-INF/jsp/edit/editRoles.jsp; class com.technoetic.xplanner.actions.EditRoleAction (strings "admin.edit.role", HQL on PersonRole). No live link to this page was found (mechanical link scan .migration-tmp/stage-01/out/linkgraph.txt); reachable only by URL. BA-001-03 impact sweep: EditRoleAction#beforeObjectCommit(Object, Session, ActionMapping, ActionForm, HttpServletRequest, HttpServletResponse) overrides no superclass hook (AbstractAction#beforeObjectCommit takes Identifiable, ActionMapping, ActionForm, request, response) and has no caller, so its role update and its admin.edit.role check are unreachable; an orphan-hook scan over all action classes found only this method. Server-side enforcement (CHK-002, BA-001-04): no server-side check is reached, because the only check sits in the unreachable EditRoleAction#beforeObjectCommit (above); the page is reachable by any signed-in user. Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editRoles.jsp writes the raw request parameters oid (55), returnto (56) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): /do/edit/roles runs EditObjectAction#doExecute with type net.sf.xplanner.domain.Project (WAR:WEB-INF/action-servlet.xml:400-404), so a direct request with merge=true binds the request parameters onto the loaded project as in row 78 (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
+    <t>WAR:WEB-INF/struts-config.xml:409-411; WAR:WEB-INF/action-servlet.xml:400-404 (EditRoleAction); WAR:WEB-INF/jsp/edit/editRoles.jsp; class com.technoetic.xplanner.actions.EditRoleAction (strings "admin.edit.role", HQL on PersonRole). No live link to this page was found (mechanical link scan .migration-tmp/stage-01/out/linkgraph.txt); reachable only by URL. BA-001-03 impact sweep: EditRoleAction#beforeObjectCommit(Object, Session, ActionMapping, ActionForm, HttpServletRequest, HttpServletResponse) overrides no superclass hook (AbstractAction#beforeObjectCommit takes Identifiable, ActionMapping, ActionForm, request, response) and has no caller, so its role update and its admin.edit.role check are unreachable; an orphan-hook scan over all action classes found only this method. Server-side enforcement (CHK-002, BA-001-04): no server-side check is reached, because the only check sits in the unreachable EditRoleAction#beforeObjectCommit (above); the page is reachable by any signed-in user. Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editRoles.jsp writes the raw request parameters oid (55), returnto (56) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): /do/edit/roles runs EditObjectAction#doExecute with type net.sf.xplanner.domain.Project (WAR:WEB-INF/action-servlet.xml:400-404), so a direct request with merge=true binds the request parameters onto the loaded project as in row 78 (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/EditRoleAction.java EditRoleAction#beforeObjectCommit; SRC:src/com/technoetic/xplanner/actions/AbstractAction.java AbstractAction#execute. WAR: classes byte-identical to the v1.1a4 release. The role-saving method takes an extra Session parameter, so it does not override the hook that AbstractAction#execute calls, and nothing else calls it.</t>
   </si>
   <si>
     <t>UF-003</t>
@@ -511,7 +511,7 @@
     <t>Table of people with mailto links; default sort by name.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:313; WAR:WEB-INF/jsp/view/people.jsp (writableTable peopleToShow, columns userId/name/initials/phone/email); linked from projects.jsp:161 and project.jsp:96.</t>
+    <t>WAR:WEB-INF/struts-config.xml:313; WAR:WEB-INF/jsp/view/people.jsp (writableTable peopleToShow, columns userId/name/initials/phone/email); linked from projects.jsp:161 and project.jsp:96. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Hidden people are listed only for users with admin.hide on system.person; others see only visible people.</t>
@@ -523,7 +523,7 @@
     <t>Admins see hidden people; others do not.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/people.jsp (isUserAuthorized permission="admin.hide" resourceType="system.person"; useBeans where hidden = false). Server-side enforcement (CHK-002, BA-001-04): the filter is applied while the server renders people.jsp; /do/view/people is a DispatchForward with authorization switched off (row 28), and the page of a hidden person remains reachable by oid (ViewPersonAction has no permission check, row 29).</t>
+    <t>WAR:WEB-INF/jsp/view/people.jsp (isUserAuthorized permission="admin.hide" resourceType="system.person"; useBeans where hidden = false). Server-side enforcement (CHK-002, BA-001-04): the filter is applied while the server renders people.jsp; /do/view/people is a DispatchForward with authorization switched off (row 28), and the page of a hidden person remains reachable by oid (ViewPersonAction has no permission check, row 29). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>With a projectId parameter the list is restricted to people with a role on that project and titled with the project name.</t>
@@ -535,7 +535,7 @@
     <t>Title "People in project &lt;name&gt;"; only project members listed.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/people.jsp (bean:parameter projectId; PermissionHelper.getPeopleWithProjectRole; message people.project.title).</t>
+    <t>WAR:WEB-INF/jsp/view/people.jsp (bean:parameter projectId; PermissionHelper.getPeopleWithProjectRole; message people.project.title). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>View person page</t>
@@ -550,7 +550,7 @@
     <t>Sections with tables per category or "none" messages; links to iteration, story and task.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:317-319; WAR:WEB-INF/action-servlet.xml:342-350 (ViewPersonAction, authorizationRequired=false); WAR:WEB-INF/jsp/view/person.jsp with WAR:WEB-INF/jsp/view/personTaskTableFragment.jsp and WAR:WEB-INF/jsp/view/personStoryTableFragment.jsp; class com.technoetic.xplanner.actions.ViewPersonAction (strings currentActiveTasksForPerson ... storiesForTracker).</t>
+    <t>WAR:WEB-INF/struts-config.xml:317-319; WAR:WEB-INF/action-servlet.xml:342-350 (ViewPersonAction, authorizationRequired=false); WAR:WEB-INF/jsp/view/person.jsp with WAR:WEB-INF/jsp/view/personTaskTableFragment.jsp and WAR:WEB-INF/jsp/view/personStoryTableFragment.jsp; class com.technoetic.xplanner.actions.ViewPersonAction (strings currentActiveTasksForPerson ... storiesForTracker). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ViewPersonAction.java ViewPersonAction#doExecute. WAR: classes byte-identical to the v1.1a4 release; SOURCE MISMATCH: the WAR bytecode of ViewPersonAction differs from the r426 source (WAR governs). The bytecode sets the recorded six attributes plus "person", loading the tasks through TaskDao#getCurrentTasksForPerson and TaskRepository and the stories through UserStoryDao; the r426 source uses a StoryRepository and declares setStoryRepository and setTaskRepository instead of setTaskDao and setUserStoryDao. This is the only class whose method names differ between source and bytecode.</t>
   </si>
   <si>
     <t>From a task row on the person page an authorized user can jump to time entry or task edit.</t>
@@ -562,7 +562,7 @@
     <t>Clock and edit icons per active task when the user may edit it.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/personTaskTableFragment.jsp (isUserAuthorized task edit; links /do/edit/time and /do/edit/task). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); UpdateTimeAction or EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>WAR:WEB-INF/jsp/view/personTaskTableFragment.jsp (isUserAuthorized task edit; links /do/edit/time and /do/edit/task). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); UpdateTimeAction or EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>The edit link on a person page is shown only to that person or to someone with admin.edit on system.person for some project.</t>
@@ -574,7 +574,7 @@
     <t>Edit link visible accordingly; links to people list, timesheet and exports.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/person.jsp (remoteUserId == person.getId() || hasPermissionForSomeProject(..., "admin.edit")). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction (except the role rules in row 31) performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>WAR:WEB-INF/jsp/view/person.jsp (remoteUserId == person.getId() || hasPermissionForSomeProject(..., "admin.edit")). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction (except the role rules in row 31) performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Create person</t>
@@ -589,7 +589,7 @@
     <t>Person saved; user returned to the people list (returnto).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/people.jsp (link /do/edit/person under create.person); WAR:WEB-INF/struts-config.xml:321-326; WAR:WEB-INF/jsp/edit/editPerson.jsp; class com.technoetic.xplanner.actions.EditPersonAction. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editPerson.jsp writes the raw request parameters oid (39), returnto (43) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/person that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Person object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). The settable properties include ones the person editor does not show, for example the stored password digest (Person#setPassword) and the hidden flag; EditPersonAction#beforeObjectCommit still reads the new-password and role fields from the form. No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
+    <t>WAR:WEB-INF/jsp/view/people.jsp (link /do/edit/person under create.person); WAR:WEB-INF/struts-config.xml:321-326; WAR:WEB-INF/jsp/edit/editPerson.jsp; class com.technoetic.xplanner.actions.EditPersonAction. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editPerson.jsp writes the raw request parameters oid (39), returnto (43) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/person that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Person object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). The settable properties include ones the person editor does not show, for example the stored password digest (Person#setPassword) and the hidden flag; EditPersonAction#beforeObjectCommit still reads the new-password and role fields from the form. No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/net/sf/xplanner/domain/Person.java Person#setPassword (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/actions/EditPersonAction.java EditPersonAction#beforeObjectCommit; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject, #doExecute. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
   </si>
   <si>
     <t>Name, user ID, e-mail and initials are mandatory; password and confirmation must match.</t>
@@ -601,7 +601,7 @@
     <t>Messages "Missing name.", "Missing user Id.", "Missing email.", "Missing initials.", "Passwords do not match".</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.PersonEditorForm#validate (strings person.editor.missing_name, missing_user_id, missing_email, missing_initials, password_mismatch); ResourceBundle.properties same keys.</t>
+    <t>class com.technoetic.xplanner.forms.PersonEditorForm#validate (strings person.editor.missing_name, missing_user_id, missing_email, missing_initials, password_mismatch); ResourceBundle.properties same keys. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/PersonEditorForm.java PersonEditorForm#validate (withheld file, cited by path only). WAR: classes byte-identical to the v1.1a4 release. Name, user ID, e-mail and initials are required; the confirmation is compared only when a new password is given.</t>
   </si>
   <si>
     <t>A duplicate user ID is rejected on the editor.</t>
@@ -613,7 +613,7 @@
     <t>Editor redisplayed with "User Id exists."</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:323-325 (DuplicateUserIdException -&gt; editPerson.jsp, key person.editor.userid_exist); db-changelog.xml:252 (unique index userId).</t>
+    <t>WAR:WEB-INF/struts-config.xml:323-325 (DuplicateUserIdException -&gt; editPerson.jsp, key person.editor.userid_exist); db-changelog.xml:252 (unique index userId). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); the WAR db-changelog.xml differs from the SVN copy, which is withheld (WAR governs). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Edit person and password</t>
@@ -628,7 +628,7 @@
     <t>Changes saved; returnto page shown.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (form /do/edit/person, Update button); WAR:WEB-INF/security.xml:15 (/do/edit/person in viewing constraint). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction (except the role rules in row 31) performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 43 applies to every /do/edit/person request (Inferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002): the unvalidated returnto redirect of row 43 applies (Q3 facts).</t>
+    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (form /do/edit/person, Update button); WAR:WEB-INF/security.xml:15 (/do/edit/person in viewing constraint). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction (except the role rules in row 31) performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 43 applies to every /do/edit/person request (Inferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002): the unvalidated returnto redirect of row 43 applies (Q3 facts). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>The password fields are shown only when the active login module can change passwords; a new password is stored as a salted digest.</t>
@@ -640,7 +640,7 @@
     <t>New password / confirm fields; saved password replaces the old one.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp:78-79 (AuthenticatorImpl.getLoginModule(request).isCapableOfChangingPasswords()); class XPlannerLoginModule#changePassword/#encodePassword (SecureRandom salt, MD5, Base64). Provenance (fixed baseline, see reconnaissance GAP-005): P-02: spring-beans.xml:65-68 sets defaultAutoCommit=false with a comment describing a MySQL fix for the login module's changePassword commit; this setting is treated as patch-introduced.</t>
+    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp:78-79 (AuthenticatorImpl.getLoginModule(request).isCapableOfChangingPasswords()); class XPlannerLoginModule#changePassword/#encodePassword (SecureRandom salt, MD5, Base64). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/module/XPlannerLoginModule.java XPlannerLoginModule#isCapableOfChangingPasswords, #changePassword, #encodePassword (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/AuthenticatorImpl.java AuthenticatorImpl#getLoginModule. WAR: classes byte-identical to the v1.1a4 release. The XPlanner module declares that it can change passwords, and changePassword stores a newly salted digest of the new password and commits it. Provenance (fixed baseline, see reconnaissance GAP-005): P-02: spring-beans.xml:65-68 sets defaultAutoCommit=false with a comment describing a MySQL fix for the login module's changePassword commit; this setting is treated as patch-introduced.</t>
   </si>
   <si>
     <t>Users with hide permission can mark a person hidden.</t>
@@ -652,7 +652,7 @@
     <t>Hidden select Yes/No; hidden people disappear from normal lists.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (isUserAuthorized person hide; select hidden). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (isUserAuthorized person hide; select hidden). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Delete person</t>
@@ -667,7 +667,7 @@
     <t>Person removed, or a database error when foreign keys refer to the person (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:348; WAR:WEB-INF/action-servlet.xml:370-374 (DeleteObjectAction type Person). The person action metadata defines only "edit" (DomainMetaDataRepository#init) and no live link to /do/delete/person was found (linkgraph.txt). BA-001-04 cascade sweep: net.sf.xplanner.domain.Person has no relationship annotations; WAR:WEB-INF/classes/db-changelog.xml:260 (notification_receivers.person_id -&gt; person) and :262 (story.customer_id -&gt; person) are the only foreign keys to person. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>WAR:WEB-INF/struts-config.xml:348; WAR:WEB-INF/action-servlet.xml:370-374 (DeleteObjectAction type Person). The person action metadata defines only "edit" (DomainMetaDataRepository#init) and no live link to /do/delete/person was found (linkgraph.txt). BA-001-04 cascade sweep: net.sf.xplanner.domain.Person has no relationship annotations; WAR:WEB-INF/classes/db-changelog.xml:260 (notification_receivers.person_id -&gt; person) and :262 (story.customer_id -&gt; person) are the only foreign keys to person. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute; SRC:src/net/sf/xplanner/domain/Person.java (withheld file, cited by path only: no relationship or cascade annotation). WAR: classes byte-identical to the v1.1a4 release. The delete publishes a delete event and deletes the object; the outcome with referencing rows depends on the database foreign keys. Live question: Deleting a person who is a story customer: is the delete rejected by the database, and do task, time-entry and role rows keep the dangling id?</t>
   </si>
   <si>
     <t>Import people from a file</t>
@@ -682,7 +682,7 @@
     <t>Upload form and per-line checks work, but saving the first valid line is expected to fail with a null reference, because the person DAO is never injected; no results table with "Success" is expected (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/people.jsp (link /do/import/people); WAR:WEB-INF/struts-config.xml:329-330; WAR:WEB-INF/jsp/edit/importPeople.jsp; class com.technoetic.xplanner.actions.ImportPeopleAction (BufferedReader.readLine, String.split ",", PersonDao.save); ResourceBundle.properties people.import.editor.importFileFormat. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); ImportPeopleAction (its AuthorizationException handler is unreachable because nothing on its path raises one) performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Wiring (BA-001-07, mechanism (a)): WAR:WEB-INF/action-servlet.xml:2 sets default-autowire="byName"; the bean /import/people (:359) has no properties; ImportPeopleAction#setPersonDao carries no annotation, and no Spring file defines a bean named personDao (WAR:WEB-INF/classes/spring-dao.xml:17-57 define commonDao, taskDao, userStoryDao, projectDao, viewDao, dataSampleDao, settingDao, objectTypeDao and attributeDao; PersonDaoImpl has no stereotype and no component scan covers net.sf.xplanner.dao). ImportPeopleAction$1#run calls personDao.save for each accepted line inside the transaction template; the handlers of #execute catch DuplicateUserIdException, the local import exception and AuthorizationException only (exception table), so the null reference is expected to propagate to the error page. Sweep: .migration-tmp/stage-01/out/wiring-07.txt, wiring-impact-07.txt. Corrected in BA-001-07 (Source: stage-02-pass-005 F-001). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/importPeople.jsp writes the raw request parameters returnto (34,78), formFileName (39) [parameter (lines); line 78 passes returnto as the page attribute of html:link] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt.</t>
+    <t>WAR:WEB-INF/jsp/view/people.jsp (link /do/import/people); WAR:WEB-INF/struts-config.xml:329-330; WAR:WEB-INF/jsp/edit/importPeople.jsp; class com.technoetic.xplanner.actions.ImportPeopleAction (BufferedReader.readLine, String.split ",", PersonDao.save); ResourceBundle.properties people.import.editor.importFileFormat. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); ImportPeopleAction (its AuthorizationException handler is unreachable because nothing on its path raises one) performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Wiring (BA-001-07, mechanism (a)): WAR:WEB-INF/action-servlet.xml:2 sets default-autowire="byName"; the bean /import/people (:359) has no properties; ImportPeopleAction#setPersonDao carries no annotation, and no Spring file defines a bean named personDao (WAR:WEB-INF/classes/spring-dao.xml:17-57 define commonDao, taskDao, userStoryDao, projectDao, viewDao, dataSampleDao, settingDao, objectTypeDao and attributeDao; PersonDaoImpl has no stereotype and no component scan covers net.sf.xplanner.dao). ImportPeopleAction$1#run calls personDao.save for each accepted line inside the transaction template; the handlers of #execute catch DuplicateUserIdException, the local import exception and AuthorizationException only (exception table), so the null reference is expected to propagate to the error page. Sweep: .migration-tmp/stage-01/out/wiring-07.txt, wiring-impact-07.txt. Corrected in BA-001-07 (Source: stage-02-pass-005 F-001). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/importPeople.jsp writes the raw request parameters returnto (34,78), formFileName (39) [parameter (lines); line 78 passes returnto as the page attribute of html:link] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/ImportPeopleAction.java ImportPeopleAction#execute, #setPersonDao. WAR: classes byte-identical to the v1.1a4 release. The setter has no annotation and no bean named personDao exists, as recorded; the null-reference outcome is a runtime effect. Live question: Does uploading a file with one valid line fail on save?</t>
   </si>
   <si>
     <t>Malformed lines and empty user IDs are reported per line before any save; the "User already exists" outcome can only come from the save, which is expected to fail first (row 50).</t>
@@ -694,7 +694,7 @@
     <t>Statuses "Entry is not formated properly" and "User id can not be empty" for the lines checked before the save; "User already exists" is not expected (runtime unverified).</t>
   </si>
   <si>
-    <t>class ImportPeopleAction (strings people.import.status.wrong_entry_format, empty_userId, userId_exists); ResourceBundle.properties same keys. Wiring (BA-001-07): the wrong_entry_format and empty_userId checks run in ImportPeopleAction#execute before ImportPeopleAction$1#run; userId_exists comes from DuplicateUserIdException, which only PersonDao.save raises (row 50). Source: stage-02-pass-005 F-001.</t>
+    <t>class ImportPeopleAction (strings people.import.status.wrong_entry_format, empty_userId, userId_exists); ResourceBundle.properties same keys. Wiring (BA-001-07): the wrong_entry_format and empty_userId checks run in ImportPeopleAction#execute before ImportPeopleAction$1#run; userId_exists comes from DuplicateUserIdException, which only PersonDao.save raises (row 50). Source: stage-02-pass-005 F-001. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ImportPeopleAction.java ImportPeopleAction#execute. WAR: classes byte-identical to the v1.1a4 release. The format and empty-id checks run per line before the save; the duplicate outcome needs the save.</t>
   </si>
   <si>
     <t>Submitting the people import without a file is rejected before any line is read.</t>
@@ -706,7 +706,7 @@
     <t>Import page redisplayed with "Please select a file to import."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.ImportPeopleForm extends ImportForm without its own validate; ImportForm#validate raises import.status.no_import_file when the form is submitted without a file (bytecode constants); form bean import/people (WAR:WEB-INF/struts-config.xml:48-49) on the mapping /import/people (:329-330). Message at WAR:WEB-INF/classes/ResourceBundle.properties:39. CHK-005 (BA-001-05). Source: stage-02-pass-003 F-003.</t>
+    <t>class com.technoetic.xplanner.forms.ImportPeopleForm extends ImportForm without its own validate; ImportForm#validate raises import.status.no_import_file when the form is submitted without a file (bytecode constants); form bean import/people (WAR:WEB-INF/struts-config.xml:48-49) on the mapping /import/people (:329-330). Message at WAR:WEB-INF/classes/ResourceBundle.properties:39. CHK-005 (BA-001-05). Source: stage-02-pass-003 F-003. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/ImportForm.java ImportForm#validate. WAR: classes byte-identical to the v1.1a4 release. A submitted form without a file name raises the no-import-file key.</t>
   </si>
   <si>
     <t>The import page offers a template download link.</t>
@@ -718,7 +718,7 @@
     <t>Link to files/peopleImportTemplate.xls (an Excel file, although the importer reads comma-separated text).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/importPeople.jsp (link to people.import.download.template.file.name); WAR:files/peopleImportTemplate.xls; ResourceBundle.properties:574. Format mismatch between .xls template and line/comma parser is recorded as an unresolved question.</t>
+    <t>WAR:WEB-INF/jsp/edit/importPeople.jsp (link to people.import.download.template.file.name); WAR:files/peopleImportTemplate.xls; ResourceBundle.properties:574. Format mismatch between .xls template and line/comma parser is recorded as an unresolved question. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ImportPeopleAction.java ImportPeopleAction#execute (reads text lines). WAR: importPeople.jsp and files/peopleImportTemplate.xls identical to the SVN webapp copies. The link points to an Excel file while the importer reads comma-separated text lines.</t>
   </si>
   <si>
     <t>UF-004</t>
@@ -739,7 +739,7 @@
     <t>Page titled system info with version 1.1a4, build date/revision, dialect, driver, DB URL/user (password masked), servlet version, memory.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/common/footer.jsp:38 (link appUrl + /do/systemInfo); WAR:WEB-INF/struts-config.xml:160-162 (forward to unexpectedError.jsp); class com.technoetic.xplanner.actions.SystemInfoAction (attribute isSystemInfo); class com.technoetic.xplanner.SystemInfo#getDatabaseInfo (strings "Database User Password", "******"). Request echo (BA-001-07, mechanism (b)): /do/systemInfo forwards to WAR:WEB-INF/jsp/common/unexpectedError.jsp (WAR:WEB-INF/struts-config.xml:160-161), which also lists the request information of the current request: referer, URL, URI, query string, all request parameters and all request attributes (unexpectedError.jsp:100-121). Values in those lists are HTML-encoded by BoxedListTag (StringUtilities#htmlEncode in #getStringValue and #renderRow). Source: stage-02-pass-005 F-003. Provenance (fixed baseline, see reconnaissance GAP-005): P-01: database engine, dialect, driver, URL and credential values come from the rewritten entries xplanner.properties / xplanner-custom.properties that carry the known MySQL patch; the upstream values cannot be separated.</t>
+    <t>WAR:WEB-INF/jsp/common/footer.jsp:38 (link appUrl + /do/systemInfo); WAR:WEB-INF/struts-config.xml:160-162 (forward to unexpectedError.jsp); class com.technoetic.xplanner.actions.SystemInfoAction (attribute isSystemInfo); class com.technoetic.xplanner.SystemInfo#getDatabaseInfo (strings "Database User Password", "******"). Request echo (BA-001-07, mechanism (b)): /do/systemInfo forwards to WAR:WEB-INF/jsp/common/unexpectedError.jsp (WAR:WEB-INF/struts-config.xml:160-161), which also lists the request information of the current request: referer, URL, URI, query string, all request parameters and all request attributes (unexpectedError.jsp:100-121). Values in those lists are HTML-encoded by BoxedListTag (StringUtilities#htmlEncode in #getStringValue and #renderRow). Source: stage-02-pass-005 F-003. Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/actions/SystemInfoAction.java SystemInfoAction; SRC:src/com/technoetic/xplanner/SystemInfo.java SystemInfo#getDatabaseInfo (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/util/StringUtilities.java StringUtilities#htmlEncode. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Provenance (fixed baseline, see reconnaissance GAP-005): P-01: database engine, dialect, driver, URL and credential values come from the rewritten entries xplanner.properties / xplanner-custom.properties that carry the known MySQL patch; the upstream values cannot be separated.</t>
   </si>
   <si>
     <t>Error pages</t>
@@ -754,7 +754,7 @@
     <t>Error page with message, support links (support.issue.url), "Cause" and "Stack Trace" boxes.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:16-29 (error-page JspException, ServletException, Throwable -&gt; unexpectedError.jsp); WAR:WEB-INF/jsp/common/unexpectedError.jsp; xplanner.properties:289-309 (error.filingInfo). Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; error.unknownError and error.moreInfo are defined only in the default and "--" bundles; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Request echo (BA-001-07, mechanism (b)): unexpectedError.jsp is the container error page for every JspException, ServletException and Throwable (WAR:WEB-INF/web.xml:16-29). It prints the first lines of the exception message unescaped with &lt;%= message %&gt; (unexpectedError.jsp:66) and lists the referer, URL, query string, every request parameter (including any password field of the failing request) and every request attribute (:100-121; values HTML-encoded by BoxedListTag). Observed risk only (Q3 deferred). Source: stage-02-pass-005 F-003. Page-text keys (BA-001-09, pass-007 F-003, check (j)): the page title comes from a scriptlet-selected key (WAR:WEB-INF/jsp/common/unexpectedError.jsp:19,27,47): error.title, defined in all bundles except de and es, and, when the same page serves the system information page (row 55), system.info.title, defined only in the default and "--" bundles. The tiles:default layout adds the footer keys app.label.version (all 10 bundles) and footer.message (only the default, "--" and de bundles; WAR:WEB-INF/jsp/common/footer.jsp:25,38) and the breadcrumb link text navigation.top (all 10 bundles; WAR:WEB-INF/tags/breadcrumb.tag:10). Bundles without a key fall back to the default text (framework behavior, GAP-011). None of these texts is credential-like (.migration-tmp/stage-01/out/public-keys-09.txt). Breadcrumb lookup (BA-001-10, pass-008 F-002 lead, check (l)): the error page uses the same tiles:default layout, and the layout breadcrumb (WAR:WEB-INF/jsp/layout/defaultLayout.jsp:44, WAR:WEB-INF/tags/breadcrumb.tag:10) reads the request parameter oid, or else fkey, and loads that object without a sign-in or permission check (class net.sf.xplanner.tags.NavigationBarTag#doEndTag, #setObject(int): the type attribute arrives as an empty string, so IdSearchHelper#search runs Session#get over Project, Iteration, UserStory, Task, Person and Note). #render then adds links whose texts are the names of the object's project, iteration, story, task or feature, and breadcrumb.tag:15,18 prints them with unescaped EL. The error page renders for every failing request, including one without a session, so the names of the object named by the failing request's oid or fkey are expected to be shown there too (Inferred; row 185; GAP-007; observed risk only, Q3 deferred). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/web.xml:16-29 (error-page JspException, ServletException, Throwable -&gt; unexpectedError.jsp); WAR:WEB-INF/jsp/common/unexpectedError.jsp; xplanner.properties:289-309 (error.filingInfo). Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; error.unknownError and error.moreInfo are defined only in the default and "--" bundles; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Request echo (BA-001-07, mechanism (b)): unexpectedError.jsp is the container error page for every JspException, ServletException and Throwable (WAR:WEB-INF/web.xml:16-29). It prints the first lines of the exception message unescaped with &lt;%= message %&gt; (unexpectedError.jsp:66) and lists the referer, URL, query string, every request parameter (including any password field of the failing request) and every request attribute (:100-121; values HTML-encoded by BoxedListTag). Observed risk only (Q3 deferred). Source: stage-02-pass-005 F-003. Page-text keys (BA-001-09, pass-007 F-003, check (j)): the page title comes from a scriptlet-selected key (WAR:WEB-INF/jsp/common/unexpectedError.jsp:19,27,47): error.title, defined in all bundles except de and es, and, when the same page serves the system information page (row 55), system.info.title, defined only in the default and "--" bundles. The tiles:default layout adds the footer keys app.label.version (all 10 bundles) and footer.message (only the default, "--" and de bundles; WAR:WEB-INF/jsp/common/footer.jsp:25,38) and the breadcrumb link text navigation.top (all 10 bundles; WAR:WEB-INF/tags/breadcrumb.tag:10). Bundles without a key fall back to the default text (framework behavior, GAP-011). None of these texts is credential-like (.migration-tmp/stage-01/out/public-keys-09.txt). Breadcrumb lookup (BA-001-10, pass-008 F-002 lead, check (l)): the error page uses the same tiles:default layout, and the layout breadcrumb (WAR:WEB-INF/jsp/layout/defaultLayout.jsp:44, WAR:WEB-INF/tags/breadcrumb.tag:10) reads the request parameter oid, or else fkey, and loads that object without a sign-in or permission check (class net.sf.xplanner.tags.NavigationBarTag#doEndTag, #setObject(int): the type attribute arrives as an empty string, so IdSearchHelper#search runs Session#get over Project, Iteration, UserStory, Task, Person and Note). #render then adds links whose texts are the names of the object's project, iteration, story, task or feature, and breadcrumb.tag:15,18 prints them with unescaped EL. The error page renders for every failing request, including one without a session, so the names of the object named by the failing request's oid or fkey are expected to be shown there too (Inferred; row 185; GAP-007; observed risk only, Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/net/sf/xplanner/tags/NavigationBarTag.java NavigationBarTag#doEndTag; SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search. WAR: classes byte-identical to the v1.1a4 release; values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
   </si>
   <si>
     <t>Requesting a non-existent object shows "Object &lt;id&gt; not found".</t>
@@ -766,7 +766,7 @@
     <t>General error page with object-not-found message.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:82-86 (ObjectNotFoundException, UnresolvableObjectException -&gt; generalError.jsp); WAR:WEB-INF/jsp/common/generalError.jsp. Request-value flow (BA-001-07, mechanism (b)): for ObjectNotFoundException, WAR:WEB-INF/jsp/common/generalError.jsp:26 passes request.getParameter("oid") as arg0 of bean:message, which does not escape its arguments, so the raw parameter is written into the page (Inferred; observed risk only, Q3 deferred).</t>
+    <t>WAR:WEB-INF/struts-config.xml:82-86 (ObjectNotFoundException, UnresolvableObjectException -&gt; generalError.jsp); WAR:WEB-INF/jsp/common/generalError.jsp. Request-value flow (BA-001-07, mechanism (b)): for ObjectNotFoundException, WAR:WEB-INF/jsp/common/generalError.jsp:26 passes request.getParameter("oid") as arg0 of bean:message, which does not escape its arguments, so the raw parameter is written into the page (Inferred; observed risk only, Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Change display language</t>
@@ -781,7 +781,7 @@
     <t>Texts change to the selected language; user returned to returnto or projects.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:158; WAR:WEB-INF/action-servlet.xml:6; class com.technoetic.xplanner.actions.ChangeLocaleAction (strings "language", "org.apache.struts.action.LOCALE"); WAR:WEB-INF/classes/ResourceBundle*.properties (10 files). No live link to /do/changeLocale was found (linkgraph.txt). Redirect target (BA-001-08, pass-006 F-002, check (e)): ChangeLocaleAction#execute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only an empty value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
+    <t>WAR:WEB-INF/struts-config.xml:158; WAR:WEB-INF/action-servlet.xml:6; class com.technoetic.xplanner.actions.ChangeLocaleAction (strings "language", "org.apache.struts.action.LOCALE"); WAR:WEB-INF/classes/ResourceBundle*.properties (10 files). No live link to /do/changeLocale was found (linkgraph.txt). Redirect target (BA-001-08, pass-006 F-002, check (e)): ChangeLocaleAction#execute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only an empty value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ChangeLocaleAction.java ChangeLocaleAction#execute. WAR: classes byte-identical to the v1.1a4 release. The action stores new Locale(language) in the session (the default locale when empty) and redirects to returnto or the projects list.</t>
   </si>
   <si>
     <t>Settings pages (work in progress)</t>
@@ -796,7 +796,7 @@
     <t>Page headed "Settings" with a table; the add/edit editor JSP is missing.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:405,419-421; WAR:WEB-INF/jsp/view/settings.jsp (prints ${settings} raw; reuses projects.title); input WEB-INF/jsp/edit/editSetting.jsp ABSENT from WAR (GAP-003); db-changelog.xml changeSet 2-1 (setting, object_type). No live link to /do/view/settings found. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditObjectAction for Setting performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/setting that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Setting object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
+    <t>WAR:WEB-INF/struts-config.xml:405,419-421; WAR:WEB-INF/jsp/view/settings.jsp (prints ${settings} raw; reuses projects.title); input WEB-INF/jsp/edit/editSetting.jsp ABSENT from WAR (GAP-003); db-changelog.xml changeSet 2-1 (setting, object_type). No live link to /do/view/settings found. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditObjectAction for Setting performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/setting that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Setting object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#doExecute, #populateObject. WAR: classes byte-identical to the v1.1a4 release. The list action and the generic editor exist; the editor JSP is absent from the WAR (GAP-003).</t>
   </si>
   <si>
     <t>Generic Spring MVC handlers exist for /setting/{objectType}/list and /setting/{objectType}/edit/{objectId}.</t>
@@ -808,7 +808,7 @@
     <t>The handlers print the objectType path value to standard output and return it as the view name. A plain value becomes /WEB-INF/jsp/&lt;objectType&gt;.jsp, where no JSP exists, so no usable page is expected; a value that starts with redirect: sends the browser to the rest of the value, and one that starts with forward: forwards inside the application (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:264-272,313-316 (SpringServlet on /setting/*); class net.sf.xplanner.web.CommonObjectHandler (@RequestMapping "/{objectType}/list", "/{objectType}/edit/{objectId}"). View selection (BA-001-08, pass-006 F-002, check (e)): CommonObjectHandler#list and #edit call PrintStream.println and return the {objectType} path variable as the view name; InternalResourceViewResolver adds the prefix /WEB-INF/jsp/ and the suffix .jsp (WAR:WEB-INF/classes/spring-web.xml:26-30; the Tiles view resolver at :31-35 is commented out). No JSP file lies directly in WEB-INF/jsp (0 files; the pages sit in 7 subdirectories), and a single path segment cannot name a subdirectory, so a value without a view prefix selects no existing page. Framework resolution (BA-001-09, pass-007 F-001, check (h)): InternalResourceViewResolver extends UrlBasedViewResolver, whose #createView in the bundled WAR:WEB-INF/lib/spring-webmvc-3.0.5.RELEASE.jar (bytecode listing) checks the view name before prefix and suffix are applied: a name that starts with "redirect:" becomes a RedirectView of the rest of the name (RedirectView#renderMergedOutputModel adds the context path only to a target that starts with "/", then HttpServletResponse#sendRedirect; spring-web.xml sets no redirect options, so the defaults apply), and a name that starts with "forward:" becomes an InternalResourceView forward of the rest. /setting/* is mapped to the Spring servlet and to WebSecurityFilter (WAR:WEB-INF/web.xml:164-167,313-316), so a signed-in user who follows /setting/redirect:&lt;target&gt;/list is redirected to &lt;target&gt;, and after a login the saved URL returns the user to it. One path segment cannot carry "/", but a scheme-qualified target whose scheme differs from the page is expected to be resolved by browsers as another host (Inferred; the container's handling of encoded slashes and the browser behavior are unverified; observed risk only, Q3 deferred; Q3 facts).</t>
+    <t>WAR:WEB-INF/web.xml:264-272,313-316 (SpringServlet on /setting/*); class net.sf.xplanner.web.CommonObjectHandler (@RequestMapping "/{objectType}/list", "/{objectType}/edit/{objectId}"). View selection (BA-001-08, pass-006 F-002, check (e)): CommonObjectHandler#list and #edit call PrintStream.println and return the {objectType} path variable as the view name; InternalResourceViewResolver adds the prefix /WEB-INF/jsp/ and the suffix .jsp (WAR:WEB-INF/classes/spring-web.xml:26-30; the Tiles view resolver at :31-35 is commented out). No JSP file lies directly in WEB-INF/jsp (0 files; the pages sit in 7 subdirectories), and a single path segment cannot name a subdirectory, so a value without a view prefix selects no existing page. Framework resolution (BA-001-09, pass-007 F-001, check (h)): InternalResourceViewResolver extends UrlBasedViewResolver, whose #createView in the bundled WAR:WEB-INF/lib/spring-webmvc-3.0.5.RELEASE.jar (bytecode listing) checks the view name before prefix and suffix are applied: a name that starts with "redirect:" becomes a RedirectView of the rest of the name (RedirectView#renderMergedOutputModel adds the context path only to a target that starts with "/", then HttpServletResponse#sendRedirect; spring-web.xml sets no redirect options, so the defaults apply), and a name that starts with "forward:" becomes an InternalResourceView forward of the rest. /setting/* is mapped to the Spring servlet and to WebSecurityFilter (WAR:WEB-INF/web.xml:164-167,313-316), so a signed-in user who follows /setting/redirect:&lt;target&gt;/list is redirected to &lt;target&gt;, and after a login the saved URL returns the user to it. One path segment cannot carry "/", but a scheme-qualified target whose scheme differs from the page is expected to be resolved by browsers as another host (Inferred; the container's handling of encoded slashes and the browser behavior are unverified; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/net/sf/xplanner/web/CommonObjectHandler.java CommonObjectHandler#list, #edit. WAR: classes byte-identical to the v1.1a4 release. Both handlers print the path value and return it as the view name, as recorded; the outcome is framework and browser behavior. Live question: What do /setting/&lt;value&gt;/list, /setting/redirect:&lt;target&gt;/list and /setting/forward:&lt;path&gt;/list return for a signed-in user?</t>
   </si>
   <si>
     <t>Administrative and test actions</t>
@@ -820,10 +820,10 @@
     <t>Operator maintenance.</t>
   </si>
   <si>
-    <t>Plain confirmation "cache cleared" / "hibernate cache cleared".</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/web.xml:233 (test-struts-config.xml loaded); WAR:WEB-INF/test-struts-config.xml:21-23; WAR:WEB-INF/test-action-servlet.xml:22-36; WAR:WEB-INF/security.xml:5 (bypass /do/invalidateHibernateCache); input JSP WEB-INF/jsp/admin/invalidateCache.jsp ABSENT. Server-side enforcement (CHK-002, BA-001-04): neither action checks a permission; InvalidateCacheAction obtains the authorizer only to reset its cache.</t>
+    <t>The permission cache is cleared, or the Hibernate query cache is evicted; the actions return no forward, so the response has no page, and "cache cleared" / "hibernate cache cleared" are only log messages.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/web.xml:233 (test-struts-config.xml loaded); WAR:WEB-INF/test-struts-config.xml:21-23; WAR:WEB-INF/test-action-servlet.xml:22-36; WAR:WEB-INF/security.xml:5 (bypass /do/invalidateHibernateCache); input JSP WEB-INF/jsp/admin/invalidateCache.jsp ABSENT. Server-side enforcement (CHK-002, BA-001-04): neither action checks a permission; InvalidateCacheAction obtains the authorizer only to reset its cache. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/admin/InvalidateCacheAction.java InvalidateCacheAction#execute; SRC:src/com/technoetic/xplanner/actions/admin/InvalidateHibernateCacheAction.java InvalidateHibernateCacheAction#execute. WAR: classes byte-identical to the v1.1a4 release. Both actions write "cache cleared" / "hibernate cache cleared" only to the log and return no forward (bytecode listing: aconst_null, areturn), so no confirmation page is sent; the Hibernate action evicts only the query cache (SessionFactory#evictQueries).</t>
   </si>
   <si>
     <t>Test-support URLs can execute data sampling, the missing-time-entry notifier, shift the application clock (dayOffset) and set a property value.</t>
@@ -835,7 +835,7 @@
     <t>Action executes and redirects to returnto or projects.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/test-struts-config.xml:13-19; WAR:WEB-INF/test-action-servlet.xml:4-20 (CommandExecutorAction with txDataSamplingCommand / missingTimeEntryNotifier, PutTheClockForwardAction, EditPropertiesAction); class PutTheClockForwardAction (string "dayOffset"); class EditPropertiesAction ("propertyName", "propertyValue"). Redirect target (BA-001-08, pass-006 F-002, check (e)): CommandExecutorAction#execute, PutTheClockForwardAction#execute and EditPropertiesAction#execute each redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
+    <t>WAR:WEB-INF/test-struts-config.xml:13-19; WAR:WEB-INF/test-action-servlet.xml:4-20 (CommandExecutorAction with txDataSamplingCommand / missingTimeEntryNotifier, PutTheClockForwardAction, EditPropertiesAction); class PutTheClockForwardAction (string "dayOffset"); class EditPropertiesAction ("propertyName", "propertyValue"). Redirect target (BA-001-08, pass-006 F-002, check (e)): CommandExecutorAction#execute, PutTheClockForwardAction#execute and EditPropertiesAction#execute each redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/CommandExecutorAction.java CommandExecutorAction#execute; SRC:src/com/technoetic/xplanner/actions/PutTheClockForwardAction.java PutTheClockForwardAction#execute; SRC:src/com/technoetic/xplanner/actions/EditPropertiesAction.java EditPropertiesAction#execute. WAR: classes byte-identical to the v1.1a4 release. The command runs, the clock moves by a positive dayOffset (any other value resets it), the property is set when a name and a value are given, and each action redirects to returnto or to the projects list.</t>
   </si>
   <si>
     <t>Tiles definitions can be reloaded via /do/admin/reload-tiles.</t>
@@ -847,7 +847,7 @@
     <t>Struts tiles reload response.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:407; WAR:WEB-INF/action-servlet.xml:398 (org.apache.struts.tiles.actions.ReloadDefinitionsAction).</t>
+    <t>WAR:WEB-INF/struts-config.xml:407; WAR:WEB-INF/action-servlet.xml:398 (org.apache.struts.tiles.actions.ReloadDefinitionsAction). Source reconciliation (BA-001-11, A4): still unsupported. none: framework class, no source in the SVN tree (GAP-011). WAR: library class org.apache.struts.tiles.actions.ReloadDefinitionsAction in struts-1.2.9.jar (no source). The behavior lies in a bundled library whose source is not available. Live question: What does /do/admin/reload-tiles return, and does it reload the shared Tiles factory?</t>
   </si>
   <si>
     <t>Startup schema creation and seed data</t>
@@ -862,7 +862,7 @@
     <t>Empty database gets tables and one system administrator person on project 0. Its factory default login pair is the one the login page advertises (row 9); the value is not reproduced here (CHK-009).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/spring-beans.xml:71-81 (SpringLiquibase changeLog classpath:db-changelog.xml, contexts test, production; sessionFactory depends-on liquibase); WAR:WEB-INF/classes/db-changelog.xml changeSets 1-1..2-5. Loading (BA-001-05): the liquibase bean is instantiated by both Spring contexts (row 65), so the change log is expected to run twice at startup; the second run is expected to find every change set already applied (Inferred). Source: stage-02-pass-003 F-002. Seed account (BA-001-06): WAR:WEB-INF/classes/db-changelog.xml:403-404 (userId and password digest of the seeded person). The earlier wording "credentials documented only in legacy/README.md, not evidence" was wrong: the WAR itself states the pair on the login page (row 9). Corrected in BA-001-06 (Source: stage-02-pass-004 F-001). Provenance (fixed baseline, see reconnaissance GAP-005): P-01: database engine, dialect, driver, URL and credential values come from the rewritten entries xplanner.properties / xplanner-custom.properties that carry the known MySQL patch; the upstream values cannot be separated. P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>WAR:WEB-INF/classes/spring-beans.xml:71-81 (SpringLiquibase changeLog classpath:db-changelog.xml, contexts test, production; sessionFactory depends-on liquibase); WAR:WEB-INF/classes/db-changelog.xml changeSets 1-1..2-5. Loading (BA-001-05): the liquibase bean is instantiated by both Spring contexts (row 65), so the change log is expected to run twice at startup; the second run is expected to find every change set already applied (Inferred). Source: stage-02-pass-003 F-002. Seed account (BA-001-06): WAR:WEB-INF/classes/db-changelog.xml:403-404 (userId and password digest of the seeded person). The earlier wording "credentials documented only in legacy/README.md, not evidence" was wrong: the WAR itself states the pair on the login page (row 9). Corrected in BA-001-06 (Source: stage-02-pass-004 F-001). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR spring-beans.xml (WAR governs); the WAR db-changelog.xml differs from the SVN copy, which is withheld (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-01: database engine, dialect, driver, URL and credential values come from the rewritten entries xplanner.properties / xplanner-custom.properties that carry the known MySQL patch; the upstream values cannot be separated. P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
   </si>
   <si>
     <t>spring-beans.xml (with its imports spring-caching.xml, spring-dao.xml and spring-security.xml) is loaded by two Spring contexts: the root context of the ContextLoaderListener and the Struts ContextLoaderPlugIn context, which also loads action-servlet.xml and test-action-servlet.xml. Every singleton is expected to exist twice: Liquibase runs a second time at startup, a second scheduler registers the daily reminder job again, and a second connection pool and session factory are created; the Struts action beans are wired from the plug-in context.</t>
@@ -874,7 +874,7 @@
     <t>Two initialisations of every spring-beans.xml bean at startup; the reminder job expected to run twice at 00:05 (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:32-38 (contextConfigLocation classpath:spring-beans.xml) and :194-196 (org.springframework.web.context.ContextLoaderListener); WAR:WEB-INF/struts-config.xml:438-441 (org.springframework.web.struts.ContextLoaderPlugIn, contextConfigLocation /WEB-INF/action-servlet.xml,/WEB-INF/classes/spring-beans.xml,/WEB-INF/test-action-servlet.xml), started with the Struts servlet (WAR:WEB-INF/web.xml:227-249, load-on-startup 2 at :248); WAR:WEB-INF/classes/spring-beans.xml:60 (dataSource), :71-81 (liquibase, sessionFactory), :362-367 (task:scheduler, task:scheduled missingTimeEntryNotifier); WAR:WEB-INF/classes/spring-security.xml:49-50 (authorizerInitializer, init-method, lazy-init false). Loader sweep (.migration-tmp/stage-01/out/loaders-05.txt): a third loader, class com.technoetic.xplanner.util.MainBeanFactory#createDefaultFactory ("/spring-beans.xml", XmlBeanFactory), has no caller (out/orphans.txt). The effect of a child context redefining parent beans is framework behavior (GAP-011). Provenance: spring-beans.xml is a rewritten entry (GAP-005 P-05); struts-config.xml and web.xml show no rewrite sign (P-06). Source: stage-02-pass-003 F-002.</t>
+    <t>WAR:WEB-INF/web.xml:32-38 (contextConfigLocation classpath:spring-beans.xml) and :194-196 (org.springframework.web.context.ContextLoaderListener); WAR:WEB-INF/struts-config.xml:438-441 (org.springframework.web.struts.ContextLoaderPlugIn, contextConfigLocation /WEB-INF/action-servlet.xml,/WEB-INF/classes/spring-beans.xml,/WEB-INF/test-action-servlet.xml), started with the Struts servlet (WAR:WEB-INF/web.xml:227-249, load-on-startup 2 at :248); WAR:WEB-INF/classes/spring-beans.xml:60 (dataSource), :71-81 (liquibase, sessionFactory), :362-367 (task:scheduler, task:scheduled missingTimeEntryNotifier); WAR:WEB-INF/classes/spring-security.xml:49-50 (authorizerInitializer, init-method, lazy-init false). Loader sweep (.migration-tmp/stage-01/out/loaders-05.txt): a third loader, class com.technoetic.xplanner.util.MainBeanFactory#createDefaultFactory ("/spring-beans.xml", XmlBeanFactory), has no caller (out/orphans.txt). The effect of a child context redefining parent beans is framework behavior (GAP-011). Provenance: spring-beans.xml is a rewritten entry (GAP-005 P-05); struts-config.xml and web.xml show no rewrite sign (P-06). Source: stage-02-pass-003 F-002. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/util/MainBeanFactory.java MainBeanFactory#createDefaultFactory (three classes import MainBeanFactory but none uses it; no other class references it in the bytecode). WAR: classes byte-identical to the v1.1a4 release; patched spring-beans.xml (WAR governs; the SVN copy is withheld). The double loading is a Spring and container effect; the source only confirms that the third loader has no caller. Live question: At startup, do the log and the database show two Liquibase runs, two schedulers and a doubled reminder job?</t>
   </si>
   <si>
     <t>An in-process HSQLDB server is started only when xplanner.migration.databasetype is hsqldb (the shipped value is mysql).</t>
@@ -886,7 +886,7 @@
     <t>No HSQLDB server with the shipped properties.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:190-192 (HsqldbServerContextListener); class com.technoetic.xplanner.filters.HsqldbServerContextListener (strings "xplanner.migration.databasetype", "hsqldb"); WAR:WEB-INF/classes/xplanner.properties:16 (databasetype=mysql). Provenance (fixed baseline, see reconnaissance GAP-005): P-01: database engine, dialect, driver, URL and credential values come from the rewritten entries xplanner.properties / xplanner-custom.properties that carry the known MySQL patch; the upstream values cannot be separated.</t>
+    <t>WAR:WEB-INF/web.xml:190-192 (HsqldbServerContextListener); class com.technoetic.xplanner.filters.HsqldbServerContextListener (strings "xplanner.migration.databasetype", "hsqldb"); WAR:WEB-INF/classes/xplanner.properties:16 (databasetype=mysql). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/filters/HsqldbServerContextListener.java HsqldbServerContextListener#contextInitialized. WAR: classes byte-identical to the v1.1a4 release; databasetype from the patched WAR xplanner.properties (WAR governs). The listener starts HsqlServer only when xplanner.migration.databasetype equals hsqldb (ignoring case) and otherwise only logs; the WAR value is mysql. Provenance (fixed baseline, see reconnaissance GAP-005): P-01: database engine, dialect, driver, URL and credential values come from the rewritten entries xplanner.properties / xplanner-custom.properties that carry the known MySQL patch; the upstream values cannot be separated.</t>
   </si>
   <si>
     <t>Configuration layering and request encoding</t>
@@ -901,7 +901,7 @@
     <t>Effective values such as the MySQL connection, application URL http://localhost:8080/xplanner and login instructions URL come from xplanner-custom.properties.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.XPlannerProperties$PropertyInitializer (strings "xplanner.properties", "xplanner.overrides", "xplanner-custom.properties", "error during custom property loading"); WAR:WEB-INF/classes/xplanner-custom.properties:19-30,49; WAR:WEB-INF/classes/spring-beans.xml:18-32 (properties bean feeds PropertyPlaceholderConfigurer). Provenance (fixed baseline, see reconnaissance GAP-005): P-01: database engine, dialect, driver, URL and credential values come from the rewritten entries xplanner.properties / xplanner-custom.properties that carry the known MySQL patch; the upstream values cannot be separated. P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-04: the cited value is read from xplanner-custom.properties (rewritten entry, known patch target); upstream value not determinable. P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>class com.technoetic.xplanner.XPlannerProperties$PropertyInitializer (strings "xplanner.properties", "xplanner.overrides", "xplanner-custom.properties", "error during custom property loading"); WAR:WEB-INF/classes/xplanner-custom.properties:19-30,49; WAR:WEB-INF/classes/spring-beans.xml:18-32 (properties bean feeds PropertyPlaceholderConfigurer). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/XPlannerProperties.java XPlannerProperties$PropertyInitializer#loadProperties, #setCustomPropertyOverrides. WAR: classes byte-identical to the v1.1a4 release; both property files are patched WAR entries (WAR governs). Xplanner.properties is loaded from the class path, then every key of the file named by the xplanner.overrides system property (default xplanner-custom.properties) replaces it; no other file name is loaded. Provenance (fixed baseline, see reconnaissance GAP-005): P-01: database engine, dialect, driver, URL and credential values come from the rewritten entries xplanner.properties / xplanner-custom.properties that carry the known MySQL patch; the upstream values cannot be separated. P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-04: the cited value is read from xplanner-custom.properties (rewritten entry, known patch target); upstream value not determinable. P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
   </si>
   <si>
     <t>The hibernate.* settings of the property files other than the four connection values (dialect, show_sql, second-level and query cache, query substitutions) and the hibernate.dbcp.* pool settings are not passed to the web application's session factory or connection pool, so they are expected to have no effect there: the dialect is resolved by Hibernate itself, no second-level or query cache is configured, and the pool uses its defaults.</t>
@@ -913,10 +913,10 @@
     <t>Pool connects with the configured driver, URL and account; Hibernate settings from the property files do not appear in the web session factory (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/spring-beans.xml:60-69 (dataSource receives only ${hibernate.connection.driver_class}, url, username and password plus defaultAutoCommit) and :77-81 (sessionFactory AnnotationSessionFactoryBean with dataSource, packagesToScan and mappingLocations only; no hibernateProperties); no hibernate.properties or hibernate.cfg.xml in the WAR or at any JAR root (search; positive control ehcache-failsafe.xml in ehcache-1.2.3.jar). Consumers by name (.migration-tmp/stage-01/out/config-consumers-06.txt): hibernate.dialect only SystemInfo#getDatabaseInfo (display) and class com.technoetic.xplanner.db.hibernate.HibernateHelper#initializeConfiguration (Configuration.addProperties, a separate factory built only by #initializeHibernate, whose only outside caller is TomcatUserImporter#main); hibernate.show_sql only HsqlServer#isTraceOn; hibernate.query.substitutions only UseBeansTag#initializeQueryTranslations (the tag applies it to its own queries); hibernate.cache.* and hibernate.dbcp.* have no consumer. Keys: WAR:WEB-INF/classes/xplanner.properties:10,57-58,202-203,207-218; WAR:WEB-INF/classes/xplanner-custom.properties:15,19. Which dialect Hibernate picks and pool defaults are framework behavior (GAP-011). Provenance: all three files are rewritten entries (GAP-005 P-01, P-03, P-05). Source: stage-02-pass-004 F-003.</t>
-  </si>
-  <si>
-    <t>In the default, alternate (--), Danish, German, Japanese and Russian bundles, dates are displayed and entered as yyyy-MM-dd and date-times as yyyy-MM-dd HH:mm.</t>
+    <t>WAR:WEB-INF/classes/spring-beans.xml:60-69 (dataSource receives only ${hibernate.connection.driver_class}, url, username and password plus defaultAutoCommit) and :77-81 (sessionFactory AnnotationSessionFactoryBean with dataSource, packagesToScan and mappingLocations only; no hibernateProperties); no hibernate.properties or hibernate.cfg.xml in the WAR or at any JAR root (search; positive control ehcache-failsafe.xml in ehcache-1.2.3.jar). Consumers by name (.migration-tmp/stage-01/out/config-consumers-06.txt): hibernate.dialect only SystemInfo#getDatabaseInfo (display) and class com.technoetic.xplanner.db.hibernate.HibernateHelper#initializeConfiguration (Configuration.addProperties, a separate factory built only by #initializeHibernate, whose only outside caller is TomcatUserImporter#main); hibernate.show_sql only HsqlServer#isTraceOn; hibernate.query.substitutions only UseBeansTag#initializeQueryTranslations (the tag applies it to its own queries); hibernate.cache.* and hibernate.dbcp.* have no consumer. Keys: WAR:WEB-INF/classes/xplanner.properties:10,57-58,202-203,207-218; WAR:WEB-INF/classes/xplanner-custom.properties:15,19. Which dialect Hibernate picks and pool defaults are framework behavior (GAP-011). Provenance: all three files are rewritten entries (GAP-005 P-01, P-03, P-05). Source: stage-02-pass-004 F-003. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/db/hibernate/HibernateHelper.java HibernateHelper#initializeConfiguration. WAR: classes byte-identical to the v1.1a4 release; patched spring-beans.xml (WAR governs; the SVN copy is withheld). The source confirms that the property-file settings reach only the separate HibernateHelper configuration; which defaults the web session factory and pool then use is framework behavior. Live question: Does the running web application show no second-level or query cache and the default pool limits?</t>
+  </si>
+  <si>
+    <t>In the default, alternate (--), Danish, German, Japanese and Russian bundles, dates are displayed and entered as yyyy-MM-dd and date-times as yyyy-MM-dd HH:mm; the history view is an exception (row 186).</t>
   </si>
   <si>
     <t>Date formats follow the UI locale bundle.</t>
@@ -925,10 +925,10 @@
     <t>Date fields and calendar pickers use yyyy-MM-dd for these locales.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/ResourceBundle.properties:8-9, ResourceBundle--.properties:5-6, ResourceBundle_da.properties:7-8, ResourceBundle_de.properties:8-9, ResourceBundle_ja.properties:12,14, ResourceBundle_ru.properties:9-10 (format.date, format.datetime); consumers editIteration.jsp, timesheet.jsp, editTimeEntries.jsp, UpdateTimeAction (format.date / format.datetime keys). Corrected in BA-001-03 (F-003): all 10 bundles compared.</t>
-  </si>
-  <si>
-    <t>In the Spanish, French, Italian and Brazilian Portuguese bundles, dates use dd-MM-yyyy; the Spanish date-time pattern is dd-MM-yyyy HH:MM, which uses the month letters in the minutes position.</t>
+    <t>WAR:WEB-INF/classes/ResourceBundle.properties:8-9, ResourceBundle--.properties:5-6, ResourceBundle_da.properties:7-8, ResourceBundle_de.properties:8-9, ResourceBundle_ja.properties:12,14, ResourceBundle_ru.properties:9-10 (format.date, format.datetime); consumers editIteration.jsp, timesheet.jsp, editTimeEntries.jsp, UpdateTimeAction (format.date / format.datetime keys). Corrected in BA-001-03 (F-003): all 10 bundles compared. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag. WAR: the WAR bundles govern (the WAR copies of the da, es, fr, it and pt_br bundles differ from the SVN copies). The bundle patterns are confirmed for the format.date and format.datetime consumers, but not for every date display: the history view (history.jsp:61,106) uses xplanner:formatDate without a pattern, so FormatDateTag falls back to its built-in pattern "EEE MMM dd k:mm:ss z" (bytecode listing agrees). Resolves carried pass-009 F-002 statically; the observed format stays a live check. Live question: Which date format does the history view show after a fresh start for two sessions with different Accept-Language values?</t>
+  </si>
+  <si>
+    <t>In the Spanish, French, Italian and Brazilian Portuguese bundles, dates use dd-MM-yyyy; the Spanish date-time pattern is dd-MM-yyyy HH:MM, which uses the month letters in the minutes position; the history view is an exception (row 186).</t>
   </si>
   <si>
     <t>Locale-dependent date entry and display; the Spanish pattern prints the month where minutes are expected.</t>
@@ -937,7 +937,7 @@
     <t>dd-MM-yyyy dates for these locales; Spanish date-times show the month number in place of minutes (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/ResourceBundle_es.properties:7-8, ResourceBundle_fr.properties:5-6, ResourceBundle_it.properties:11-12, ResourceBundle_pt_br.properties:8-9. Source: stage-02-pass-001 F-003.</t>
+    <t>WAR:WEB-INF/classes/ResourceBundle_es.properties:7-8, ResourceBundle_fr.properties:5-6, ResourceBundle_it.properties:11-12, ResourceBundle_pt_br.properties:8-9. Source: stage-02-pass-001 F-003. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag. WAR: the WAR bundles govern (the WAR copies of the es, fr, it and pt_br bundles differ from the SVN copies). As row 69: the history view does not use these patterns. Resolves carried pass-009 F-002 statically.</t>
   </si>
   <si>
     <t>The jQuery date picker attached to date fields always inserts yyyy-MM-dd, while the iteration editor calendar button and date parsing use the locale pattern; with a dd-MM-yyyy locale a date picked this way is expected to be rejected as invalid.</t>
@@ -949,7 +949,7 @@
     <t>Possible "Start date is invalid." after using the jQuery picker in es/fr/it/pt_br (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:js/global.js:39 (.dateField datepicker dateFormat yy-mm-dd); WAR:WEB-INF/jsp/edit/editIteration.jsp:54,57 (class dateField plus showCalendar with format.date); class IterationEditorForm#validate (iteration.editor.bad_start_date). Source: stage-02-pass-001 F-003.</t>
+    <t>WAR:js/global.js:39 (.dateField datepicker dateFormat yy-mm-dd); WAR:WEB-INF/jsp/edit/editIteration.jsp:54,57 (class dateField plus showCalendar with format.date); class IterationEditorForm#validate (iteration.editor.bad_start_date). Source: stage-02-pass-001 F-003. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release; js/global.js and editIteration.jsp identical to the SVN webapp copies. The picker format and the locale pattern are as recorded; whether a picked date is rejected is browser and locale behavior. Live question: In an es, fr, it or pt_br session, is a date picked with the jQuery picker rejected as "Start date is invalid."?</t>
   </si>
   <si>
     <t>Request parameters under /do/* are decoded as UTF-8.</t>
@@ -961,7 +961,7 @@
     <t>Non-ASCII input round-trips in forms.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:121-128,178-181 (RequestCharacterEncodingFilter, requestCharacterEncoding UTF-8, /do/*).</t>
+    <t>WAR:WEB-INF/web.xml:121-128,178-181 (RequestCharacterEncodingFilter, requestCharacterEncoding UTF-8, /do/*). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/filters/RequestCharacterEncodingFilter.java RequestCharacterEncodingFilter#doFilter. WAR: classes byte-identical to the v1.1a4 release. The filter sets the configured request encoding before the chain.</t>
   </si>
   <si>
     <t>Activity logging</t>
@@ -976,7 +976,7 @@
     <t>Log lines START/END with duration in xplanner-plus-activity.log, which is written into the web application root, a publicly served location with no security filter; the container is expected to serve it to anyone (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:54-57,130-133 (ActivityLogFilter on /do/*); WAR:WEB-INF/classes/log4j-war.xml:44-55 (ACTIVITY_FILE ${xplanner-plus.root}/xplanner-plus-activity.log); class com.technoetic.xplanner.filters.ActivityLogFilter#doFilter. Public location (BA-001-06): the ACTIVITY_FILE appender writes ${xplanner-plus.root}/xplanner-plus-activity.log (WAR:WEB-INF/classes/log4j-war.xml:44-58, used by the ActivityLogFilter category at :54-58); webAppRootKey sets xplanner-plus.root to the web application root (WAR:WEB-INF/web.xml:45-52). class ActivityLogFilterHelper reads getUserId, getRemoteAddr, getRequestURI and getQueryString. No security filter covers the web root (web.xml:155-176). Static serving of web-root files is container behavior (GAP-011). A 2011 copy of this file also ships in the WAR (GAP-013). Observed risk only (Q3 deferred). Source: stage-02-pass-004 F-005.</t>
+    <t>WAR:WEB-INF/web.xml:54-57,130-133 (ActivityLogFilter on /do/*); WAR:WEB-INF/classes/log4j-war.xml:44-55 (ACTIVITY_FILE ${xplanner-plus.root}/xplanner-plus-activity.log); class com.technoetic.xplanner.filters.ActivityLogFilter#doFilter. Public location (BA-001-06): the ACTIVITY_FILE appender writes ${xplanner-plus.root}/xplanner-plus-activity.log (WAR:WEB-INF/classes/log4j-war.xml:44-58, used by the ActivityLogFilter category at :54-58); webAppRootKey sets xplanner-plus.root to the web application root (WAR:WEB-INF/web.xml:45-52). class ActivityLogFilterHelper reads getUserId, getRemoteAddr, getRequestURI and getQueryString. No security filter covers the web root (web.xml:155-176). Static serving of web-root files is container behavior (GAP-011). A 2011 copy of this file also ships in the WAR (GAP-013). Observed risk only (Q3 deferred). Source: stage-02-pass-004 F-005. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/filters/ActivityLogFilter.java ActivityLogFilter#doFilter. WAR: classes byte-identical to the v1.1a4 release. A start and an end record are logged around every filtered request.</t>
   </si>
   <si>
     <t>UF-005</t>
@@ -997,7 +997,7 @@
     <t>Table of projects with links to project and current iteration; "people" and "aggregate timesheet" links.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:179; WAR:WEB-INF/action-servlet.xml:29-31 (DispatchForward, authorizationRequired=false); WAR:WEB-INF/jsp/view/projects.jsp:32-167 (useBeans order "is_hidden,name asc"; iterations where "? between startDate and endDate").</t>
+    <t>WAR:WEB-INF/struts-config.xml:179; WAR:WEB-INF/action-servlet.xml:29-31 (DispatchForward, authorizationRequired=false); WAR:WEB-INF/jsp/view/projects.jsp:32-167 (useBeans order "is_hidden,name asc"; iterations where "? between startDate and endDate"). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Users who may hide projects see an extra "hidden" column with yes/no; hidden projects are sorted after visible ones but are not styled differently.</t>
@@ -1009,7 +1009,7 @@
     <t>Hidden column visible only with hide permission; hidden projects listed last.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/projects.jsp:137-142 (isUserAuthorizedForAny permissions="hide") and :33 (order "is_hidden,name asc"). The class HiddenRowDecorator declared at :65-75 is never passed to the table: the writableTable at :82-84 has no rowDecorator attribute, and the name occurs only at :66 (CHK-003). Corrected in BA-001-04 (Source: stage-02-pass-002 F-006). Server-side enforcement (CHK-002, BA-001-04): the column is display-level only; hiding a project goes through EditProjectAction, which performs no server-side permission check (rows 29-30).</t>
+    <t>WAR:WEB-INF/jsp/view/projects.jsp:137-142 (isUserAuthorizedForAny permissions="hide") and :33 (order "is_hidden,name asc"). The class HiddenRowDecorator declared at :65-75 is never passed to the table: the writableTable at :82-84 has no rowDecorator attribute, and the name occurs only at :66 (CHK-003). Corrected in BA-001-04 (Source: stage-02-pass-002 F-006). Server-side enforcement (CHK-002, BA-001-04): the column is display-level only; hiding a project goes through EditProjectAction, which performs no server-side permission check (rows 29-30). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>When no readable project exists the page shows a "no projects" message.</t>
@@ -1021,7 +1021,7 @@
     <t>Message projects.none.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/projects.jsp:147-150.</t>
+    <t>WAR:WEB-INF/jsp/view/projects.jsp:147-150. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Create project</t>
@@ -1036,7 +1036,7 @@
     <t>Project saved; user returned to the projects list.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/projects.jsp:153-158 (link /do/edit/project under create.project); WAR:WEB-INF/struts-config.xml:195; WAR:WEB-INF/action-servlet.xml:72-76 (EditProjectAction); WAR:WEB-INF/jsp/edit/editProject.jsp:42-112. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditProjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editProject.jsp writes the raw request parameters oid (48), returnto (52) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/project that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Project object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). EditProjectAction#saveForm calls the same #populateObject. No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute (reached from EditProjectAction#doExecute) redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
+    <t>WAR:WEB-INF/jsp/view/projects.jsp:153-158 (link /do/edit/project under create.project); WAR:WEB-INF/struts-config.xml:195; WAR:WEB-INF/action-servlet.xml:72-76 (EditProjectAction); WAR:WEB-INF/jsp/edit/editProject.jsp:42-112. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditProjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editProject.jsp writes the raw request parameters oid (48), returnto (52) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/project that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Project object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). EditProjectAction#saveForm calls the same #populateObject. No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute (reached from EditProjectAction#doExecute) redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/actions/EditProjectAction.java EditProjectAction#saveForm, #doExecute; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject, #doExecute. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
   </si>
   <si>
     <t>A project without a name is rejected.</t>
@@ -1048,10 +1048,10 @@
     <t>Editor redisplayed with "Missing project name."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.ProjectEditorForm#validate (string project.editor.missing_name).</t>
-  </si>
-  <si>
-    <t>Project options (wiki URL, send missing-time notification, escape brackets) are stored as per-project attributes.</t>
+    <t>class com.technoetic.xplanner.forms.ProjectEditorForm#validate (string project.editor.missing_name). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/ProjectEditorForm.java ProjectEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release. The name is required on submit, except for the add and delete receiver actions.</t>
+  </si>
+  <si>
+    <t>Project options (wiki URL, send missing-time notification, escape brackets) are stored as per-project attributes when they differ from the global defaults in the property files (or the project already has the attribute); a value equal to the default is not stored.</t>
   </si>
   <si>
     <t>Per-project behaviour switches.</t>
@@ -1060,7 +1060,7 @@
     <t>Options persist and are re-shown when editing.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.actions.EditProjectAction#saveForm/#saveOrUpdateAttribute (strings "twiki.scheme.wiki", "xplanner.project.send.notification", "xplanner.escape.brackets"); db-changelog.xml table attribute.</t>
+    <t>class com.technoetic.xplanner.actions.EditProjectAction#saveForm/#saveOrUpdateAttribute (strings "twiki.scheme.wiki", "xplanner.project.send.notification", "xplanner.escape.brackets"); db-changelog.xml table attribute. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/EditProjectAction.java EditProjectAction#saveForm, #saveOrUpdateAttribute. WAR: classes byte-identical to the v1.1a4 release. An option is written as a project attribute only when the project already has that attribute, or when the new value is not empty and differs from the global default in the property files (or there is no default); a value equal to the default is not stored and the default keeps applying. The branches match the bytecode listing.</t>
   </si>
   <si>
     <t>Edit project</t>
@@ -1075,7 +1075,7 @@
     <t>Editor titled "Edit project: &lt;name&gt;" with Update/Reset; changes saved.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:28-34,76-80,104-106; class DomainMetaDataRepository#init (project edit -&gt; /do/edit/project, permission admin.edit). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditProjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 78 applies to every /do/edit/project request, and also to /do/edit/roles, whose action type is Project (row 35) (Inferred; Q3 facts).</t>
+    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:28-34,76-80,104-106; class DomainMetaDataRepository#init (project edit -&gt; /do/edit/project, permission admin.edit). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditProjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 78 applies to every /do/edit/project request, and also to /do/edit/roles, whose action type is Project (row 35) (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
   </si>
   <si>
     <t>Delete project</t>
@@ -1090,7 +1090,7 @@
     <t>Browser confirm "Do you want to delete project '&lt;name&gt;'?"; the project and its iterations, stories, tasks and time entries removed; orphan notes remain (runtime unverified).</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (delete -&gt; /do/delete/project, permission sysadmin.delete, onclick action.delete.confirmation); WAR:WEB-INF/struts-config.xml:197; WAR:WEB-INF/action-servlet.xml:78-82 (DeleteObjectAction#doExecute: CommonDao.delete). Cascades (CHK-003): net.sf.xplanner.domain.Project#getIterations @OneToMany(cascade=ALL), #getBacklog @OneToOne(cascade=REMOVE), Iteration#getUserStories, UserStory#getTasks, Task#getTimeEntries @OneToMany(cascade=REMOVE); The notification-receiver links (Project#getNotificationReceivers @ManyToMany, join table notification_receivers) and the project attributes (@ElementCollection, table attribute) are removed with the project row. Note refers to objects by attachedToId without a mapping; NoteHelper#deleteNotesFor is called from HibernateObjectRepository#delete, which the web delete path (DeleteObjectAction#doExecute -&gt; CommonDao.delete) does not reach. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002).</t>
+    <t>class DomainMetaDataRepository#init (delete -&gt; /do/delete/project, permission sysadmin.delete, onclick action.delete.confirmation); WAR:WEB-INF/struts-config.xml:197; WAR:WEB-INF/action-servlet.xml:78-82 (DeleteObjectAction#doExecute: CommonDao.delete). Cascades (CHK-003): net.sf.xplanner.domain.Project#getIterations @OneToMany(cascade=ALL), #getBacklog @OneToOne(cascade=REMOVE), Iteration#getUserStories, UserStory#getTasks, Task#getTimeEntries @OneToMany(cascade=REMOVE); The notification-receiver links (Project#getNotificationReceivers @ManyToMany, join table notification_receivers) and the project attributes (@ElementCollection, table attribute) are removed with the project row. Note refers to objects by attachedToId without a mapping; NoteHelper#deleteNotesFor is called from HibernateObjectRepository#delete, which the web delete path (DeleteObjectAction#doExecute -&gt; CommonDao.delete) does not reach. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute; SRC:src/net/sf/xplanner/domain/Project.java Project#getIterations; SRC:src/net/sf/xplanner/domain/Iteration.java Iteration#getUserStories; SRC:src/net/sf/xplanner/domain/UserStory.java UserStory#getTasks; SRC:src/net/sf/xplanner/domain/Task.java Task#getTimeEntries. WAR: classes byte-identical to the v1.1a4 release. The cascade annotations of the source match the recorded ones (ALL on project iterations, REMOVE on stories, tasks and time entries).</t>
   </si>
   <si>
     <t>View project</t>
@@ -1105,7 +1105,7 @@
     <t>Iteration table with edit/delete icons by permission; "create iteration", "people", export and history links.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:181-183; WAR:WEB-INF/action-servlet.xml:33-37; WAR:WEB-INF/jsp/view/project.jsp:41-70 (writableTable pagesize 10, defaultsort 5 descending) and :87-105 (links /do/edit/iteration, /do/view/people, exportLinks.jsp, /do/view/history).</t>
+    <t>WAR:WEB-INF/struts-config.xml:181-183; WAR:WEB-INF/action-servlet.xml:33-37; WAR:WEB-INF/jsp/view/project.jsp:41-70 (writableTable pagesize 10, defaultsort 5 descending) and :87-105 (links /do/edit/iteration, /do/view/people, exportLinks.jsp, /do/view/history). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>A project without iterations shows a "no iterations" message.</t>
@@ -1114,7 +1114,7 @@
     <t>Message iterations.none.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/project.jsp:73-75 (logic:equal name="iterationCount" value="0"); no iterationCount bean is defined on the page, so the message display is unverified.</t>
+    <t>WAR:WEB-INF/jsp/view/project.jsp:73-75 (logic:equal name="iterationCount" value="0"); no iterationCount bean is defined on the page, so the message display is unverified. Source reconciliation (BA-001-11, A4): runtime-only. none: no Java class or other JSP of the source tree sets iterationCount. WAR: project.jsp identical to the SVN webapp copy. The source confirms that nothing defines the bean the page compares; what Struts logic:equal then does is framework behavior. Live question: What does the project page show for a project without iterations?</t>
   </si>
   <si>
     <t>Missing time entry notification receivers</t>
@@ -1129,7 +1129,7 @@
     <t>Person selected and "Add" pressed; the person appears in the receivers list.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:115-158 (select personToAddId, action addTimeNotification); class EditProjectAction#doExecute (forward /do/edit/project/notification); WAR:WEB-INF/struts-config.xml:368-372; class com.technoetic.xplanner.actions.UpdateTimeNotificationReceivers#doAction; db-changelog.xml table notification_receivers. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); UpdateTimeNotificationReceivers performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:115-158 (select personToAddId, action addTimeNotification); class EditProjectAction#doExecute (forward /do/edit/project/notification); WAR:WEB-INF/struts-config.xml:368-372; class com.technoetic.xplanner.actions.UpdateTimeNotificationReceivers#doAction; db-changelog.xml table notification_receivers. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); UpdateTimeNotificationReceivers performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/UpdateTimeNotificationReceivers.java UpdateTimeNotificationReceivers#doAction. WAR: classes byte-identical to the v1.1a4 release. The add action appends the selected person to the project's receivers.</t>
   </si>
   <si>
     <t>A receiver can be removed with the delete icon.</t>
@@ -1141,7 +1141,7 @@
     <t>Person disappears from the receivers list.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:20-25,146 (deleteNotifiedPerson, action delTimeNotification); class UpdateTimeNotificationReceivers (string "delTimeNotification").</t>
+    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:20-25,146 (deleteNotifiedPerson, action delTimeNotification); class UpdateTimeNotificationReceivers (string "delTimeNotification"). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/UpdateTimeNotificationReceivers.java UpdateTimeNotificationReceivers#doAction. WAR: classes byte-identical to the v1.1a4 release. The delete action removes the selected person from the receivers.</t>
   </si>
   <si>
     <t>UF-006</t>
@@ -1162,7 +1162,7 @@
     <t>Iteration saved under the project; user returned.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/project.jsp:87-90 (link /do/edit/iteration); WAR:WEB-INF/struts-config.xml:241-243; WAR:WEB-INF/action-servlet.xml:177-181 (EditIterationAction); WAR:WEB-INF/jsp/edit/editIteration.jsp; class EditIterationAction#beforeObjectCommit (strings "Create", Project). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editIteration.jsp writes the raw request parameters oid (31), returnto (34), fkey (36,37) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/iteration that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Iteration object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
+    <t>WAR:WEB-INF/jsp/view/project.jsp:87-90 (link /do/edit/iteration); WAR:WEB-INF/struts-config.xml:241-243; WAR:WEB-INF/action-servlet.xml:177-181 (EditIterationAction); WAR:WEB-INF/jsp/edit/editIteration.jsp; class EditIterationAction#beforeObjectCommit (strings "Create", Project). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editIteration.jsp writes the raw request parameters oid (31), returnto (34), fkey (36,37) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/iteration that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Iteration object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/EditIterationAction.java EditIterationAction#beforeObjectCommit. WAR: classes byte-identical to the v1.1a4 release. A created iteration gets its project, the inactive status and zero days worked.</t>
   </si>
   <si>
     <t>Missing name, unparsable dates, or an end date that does not follow the start date are rejected.</t>
@@ -1174,7 +1174,7 @@
     <t>Messages "Missing iteration name.", "Start date is invalid.", "End date is invalid.", "Iteration must be a positive time interval."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.IterationEditorForm#validate (strings iteration.editor.missing_name, bad_start_date, bad_end_date) and #requirePositiveInterval (iteration.editor.nonpositive_interval); WAR:WEB-INF/classes/ResourceBundle.properties:265. Corrected in BA-001-04 (Source: stage-02-pass-002 F-001). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; iteration.editor.nonpositive_interval: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71).</t>
+    <t>class com.technoetic.xplanner.forms.IterationEditorForm#validate (strings iteration.editor.missing_name, bad_start_date, bad_end_date) and #requirePositiveInterval (iteration.editor.nonpositive_interval); WAR:WEB-INF/classes/ResourceBundle.properties:265. Corrected in BA-001-04 (Source: stage-02-pass-002 F-001). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; iteration.editor.nonpositive_interval: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release. Name and both dates are required and the interval must be positive.</t>
   </si>
   <si>
     <t>Edit iteration</t>
@@ -1189,7 +1189,7 @@
     <t>Editor with Update/Reset; changes saved.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editIteration.jsp (logic:present oid: status display, daysWorked input); class DomainMetaDataRepository#init (iteration edit, permission edit). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 88 applies to every /do/edit/iteration request (Inferred; Q3 facts).</t>
+    <t>WAR:WEB-INF/jsp/edit/editIteration.jsp (logic:present oid: status display, daysWorked input); class DomainMetaDataRepository#init (iteration edit, permission edit). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 88 applies to every /do/edit/iteration request (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
   </si>
   <si>
     <t>Delete iteration</t>
@@ -1204,7 +1204,7 @@
     <t>Confirm prompt; iteration, stories, tasks and time entries removed (runtime unverified).</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (iteration delete, onclick action.delete.confirmation); WAR:WEB-INF/struts-config.xml:257; WAR:WEB-INF/action-servlet.xml:196-200; db-changelog.xml permission id 19 (editor, delete, system.project.iteration, positive=false). Cascades: Iteration#getUserStories, UserStory#getTasks, Task#getTimeEntries @OneToMany(cascade=REMOVE). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002, F-007).</t>
+    <t>class DomainMetaDataRepository#init (iteration delete, onclick action.delete.confirmation); WAR:WEB-INF/struts-config.xml:257; WAR:WEB-INF/action-servlet.xml:196-200; db-changelog.xml permission id 19 (editor, delete, system.project.iteration, positive=false). Cascades: Iteration#getUserStories, UserStory#getTasks, Task#getTimeEntries @OneToMany(cascade=REMOVE). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002, F-007). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute; SRC:src/net/sf/xplanner/domain/Iteration.java Iteration#getUserStories. WAR: classes byte-identical to the v1.1a4 release. The cascades match the source annotations.</t>
   </si>
   <si>
     <t>View iteration stories</t>
@@ -1219,7 +1219,7 @@
     <t>Story table with per-story action icons by permission; zero values highlighted.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:203-205; WAR:WEB-INF/jsp/view/iteration.jsp:20-176; WAR:WEB-INF/jsp/layout/iterationTileParams.jsp:15-41; WAR:WEB-INF/jsp/view/iteration/progress.jsp.</t>
+    <t>WAR:WEB-INF/struts-config.xml:203-205; WAR:WEB-INF/jsp/view/iteration.jsp:20-176; WAR:WEB-INF/jsp/layout/iterationTileParams.jsp:15-41; WAR:WEB-INF/jsp/view/iteration/progress.jsp. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>An iteration without stories shows a "no stories" message.</t>
@@ -1228,7 +1228,7 @@
     <t>Message stories.none.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/iteration.jsp:166-168.</t>
+    <t>WAR:WEB-INF/jsp/view/iteration.jsp:166-168. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>The progress bar is rendered as HTML by default (xplanner.progressbar.impl=html); the actual-hours column is hidden when the image implementation is configured.</t>
@@ -1240,7 +1240,7 @@
     <t>HTML progress bars and actual hours column in the shipped configuration.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/xplanner.properties:133; WAR:WEB-INF/jsp/view/iteration.jsp:115-121. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/classes/xplanner.properties:133; WAR:WEB-INF/jsp/view/iteration.jsp:115-121. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
   </si>
   <si>
     <t>Reorder stories</t>
@@ -1255,7 +1255,7 @@
     <t>After "save order" the page reloads with stories in the new order.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/iteration.jsp:33-36,79-89,160-162 (form /do/edit/reorderstories, orderNo inputs); WAR:WEB-INF/struts-config.xml:357-362; class com.technoetic.xplanner.actions.ReorderStoriesAction. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); ReorderStoriesAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>WAR:WEB-INF/jsp/view/iteration.jsp:33-36,79-89,160-162 (form /do/edit/reorderstories, orderNo inputs); WAR:WEB-INF/struts-config.xml:357-362; class com.technoetic.xplanner.actions.ReorderStoriesAction. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); ReorderStoriesAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed at class level. SRC:src/com/technoetic/xplanner/actions/ReorderStoriesAction.java ReorderStoriesAction. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes exist and nothing read contradicts the claim.</t>
   </si>
   <si>
     <t>A non-numeric order number is rejected.</t>
@@ -1267,7 +1267,7 @@
     <t>Message "Invalid order number &lt;n&gt; entered" on the iteration page.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.ReorderStoriesForm#validate (string story.editor.invalid.order.number); struts-config.xml:360 (error -&gt; iteration.jsp).</t>
+    <t>class com.technoetic.xplanner.forms.ReorderStoriesForm#validate (string story.editor.invalid.order.number); struts-config.xml:360 (error -&gt; iteration.jsp). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/ReorderStoriesForm.java ReorderStoriesForm#validate. WAR: classes byte-identical to the v1.1a4 release. Each order value must parse as a number.</t>
   </si>
   <si>
     <t>Move multiple stories</t>
@@ -1282,22 +1282,22 @@
     <t>Move page with target iteration select; selected stories moved; redirect to /do/view/iteration?oid=&lt;source&gt;.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/iteration.jsp:38-40,60-64 (selected[] checkboxes, submitMoveMultiple); WAR:WEB-INF/struts-config.xml:364-366; WAR:WEB-INF/jsp/edit/moveStories.jsp; class com.technoetic.xplanner.actions.MoveStoriesAction (string "/do/view/iteration?oid="). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); MoveStoriesAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>WAR:WEB-INF/jsp/view/iteration.jsp:38-40,60-64 (selected[] checkboxes, submitMoveMultiple); WAR:WEB-INF/struts-config.xml:364-366; WAR:WEB-INF/jsp/edit/moveStories.jsp; class com.technoetic.xplanner.actions.MoveStoriesAction (string "/do/view/iteration?oid="). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); MoveStoriesAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/MoveStoriesAction.java MoveStoriesAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. Each selected story is moved, both iterations are reordered and the browser is redirected to the source iteration.</t>
   </si>
   <si>
     <t>Start iteration</t>
   </si>
   <si>
-    <t>An editor can start an iteration; the confirmation page asks "Do you want to start the iteration?" (the explanation that starting baselines current task estimates is shown only when arriving from time entry, row 100).</t>
+    <t>An editor can start an iteration; a confirmation page asking "Do you want to start the iteration?" appears only when another iteration of the project is active (row 99) or when arriving from time entry, otherwise the iteration is started at once (the explanation that starting baselines current task estimates is shown only when arriving from time entry, row 100).</t>
   </si>
   <si>
     <t>Freeze the plan for velocity measurement.</t>
   </si>
   <si>
-    <t>Page "Start Iteration: &lt;name&gt;" with "Do you want to start the iteration?" and OK/Cancel; iteration becomes active; opening data samples taken.</t>
-  </si>
-  <si>
-    <t>class DomainMetaDataRepository#init (start -&gt; start/iteration, permission edit); WAR:WEB-INF/struts-config.xml:245-248; WAR:WEB-INF/jsp/edit/editIterationStatus.jsp:43-47 (message_1 only when UpdateTimeAction.isFromUpdateTime) and :58-60 (message_4); WAR:WEB-INF/classes/ResourceBundle.properties:272,275; class StartIterationAction#beforeObjectCommit ("started", DataSampler.generateOpeningDataSamples). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); StartIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-005). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; iteration.status.editor.message_4 is defined only in the default and "--" bundles. Bundles without the key fall back to the default text (framework behavior, GAP-011). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editIterationStatus.jsp writes the raw request parameters fkey (34), returnto (35) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Script context (BA-001-09, pass-007 F-002, check (i)): the page binds returnto from the request (WAR:WEB-INF/jsp/edit/editIterationStatus.jsp:32, bean:parameter) and writes it unescaped after the context path into the JavaScript string of the Cancel button's onclick handler (document.location='&lt;context path&gt;&lt;returnto&gt;', :70). A crafted value can end the string and add script, and it chooses where Cancel leads on the same host. The page is the input and forward of /do/start/iteration and /do/close/iteration (WAR:WEB-INF/struts-config.xml:119-120,245,251) (Inferred; observed risk only, Q3 deferred; Q3 facts). Inventory: .migration-tmp/stage-01/out/script-sinks-09.txt.</t>
+    <t>Iteration becomes active and opening data samples are taken; the page "Start Iteration: &lt;name&gt;" with "Do you want to start the iteration?" and OK/Cancel appears only in the two cases above.</t>
+  </si>
+  <si>
+    <t>class DomainMetaDataRepository#init (start -&gt; start/iteration, permission edit); WAR:WEB-INF/struts-config.xml:245-248; WAR:WEB-INF/jsp/edit/editIterationStatus.jsp:43-47 (message_1 only when UpdateTimeAction.isFromUpdateTime) and :58-60 (message_4); WAR:WEB-INF/classes/ResourceBundle.properties:272,275; class StartIterationAction#beforeObjectCommit ("started", DataSampler.generateOpeningDataSamples). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); StartIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-005). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; iteration.status.editor.message_4 is defined only in the default and "--" bundles. Bundles without the key fall back to the default text (framework behavior, GAP-011). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editIterationStatus.jsp writes the raw request parameters fkey (34), returnto (35) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Script context (BA-001-09, pass-007 F-002, check (i)): the page binds returnto from the request (WAR:WEB-INF/jsp/edit/editIterationStatus.jsp:32, bean:parameter) and writes it unescaped after the context path into the JavaScript string of the Cancel button's onclick handler (document.location='&lt;context path&gt;&lt;returnto&gt;', :70). A crafted value can end the string and add script, and it chooses where Cancel leads on the same host. The page is the input and forward of /do/start/iteration and /do/close/iteration (WAR:WEB-INF/struts-config.xml:119-120,245,251) (Inferred; observed risk only, Q3 deferred; Q3 facts). Inventory: .migration-tmp/stage-01/out/script-sinks-09.txt. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/actions/StartIterationAction.java StartIterationAction#doExecute, #beforeObjectCommit; SRC:src/net/sf/xplanner/domain/Iteration.java Iteration#close, #start. WAR: classes byte-identical to the v1.1a4 release. The confirmation page is shown only when another iteration of the project is active (row 99) or when the request comes from time entry (row 100); otherwise the first request starts the iteration at once and redirects to returnto or the projects list. The action first calls Iteration#close (status inactive) and the hook then calls Iteration#start, so the iteration ends active (bytecode listing: Iteration.close at offsets 173 and 285).</t>
   </si>
   <si>
     <t>If other iterations are still started, the page proposes closing them (checked by default).</t>
@@ -1309,7 +1309,7 @@
     <t>Message "...{n} started iteration(s) need(s) to be closed." with "Close started iterations?" checkbox.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editIterationStatus.jsp (startedIterationsNr, closeIterations checkbox); ResourceBundle.properties iteration.status.editor.message_2/3; class StartIterationAction ("startedIterationsNr").</t>
+    <t>WAR:WEB-INF/jsp/edit/editIterationStatus.jsp (startedIterationsNr, closeIterations checkbox); ResourceBundle.properties iteration.status.editor.message_2/3; class StartIterationAction ("startedIterationsNr"). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/StartIterationAction.java StartIterationAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. With started iterations in the project the action counts them and shows the start page; a confirmed start with the checkbox closes them.</t>
   </si>
   <si>
     <t>Entering time on a task of a not-yet-started iteration first asks to start the iteration and then continues to the time entry.</t>
@@ -1321,7 +1321,7 @@
     <t>Start page with message "The iteration has not been started yet"; after OK the saved time form is processed.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.actions.UpdateTimeAction#isIterationStarted/#doExecute (strings "/do/start/iteration", "from_edit/time", "UpdateTimeAction.savedForm"); WAR:WEB-INF/struts-config.xml:247 (forward edit/time); editIterationStatus.jsp (UpdateTimeAction.isFromUpdateTime).</t>
+    <t>class com.technoetic.xplanner.actions.UpdateTimeAction#isIterationStarted/#doExecute (strings "/do/start/iteration", "from_edit/time", "UpdateTimeAction.savedForm"); WAR:WEB-INF/struts-config.xml:247 (forward edit/time); editIterationStatus.jsp (UpdateTimeAction.isFromUpdateTime). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#doExecute, #isIterationStarted; SRC:src/com/technoetic/xplanner/actions/StartIterationAction.java StartIterationAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. A submitted time form for a task of an inactive iteration is saved in the session and forwarded to /do/start/iteration; after the confirmation the start action forwards to the time editor in wizard mode.</t>
   </si>
   <si>
     <t>Close iteration and continue unfinished stories</t>
@@ -1336,7 +1336,7 @@
     <t>Iteration set inactive; data sample taken; redirect to the continue-unfinished-stories page.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (close -&gt; close/iteration); WAR:WEB-INF/struts-config.xml:251-255 (forward onclose -&gt; /do/continue/unfinished/stories); class CloseIterationAction ("closed", "onclose"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); CloseIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Redirect target (BA-001-08, pass-006 F-002, check (e)): CloseIterationAction#doExecute redirects to the fixed onclose forward (/do/continue/unfinished/stories) and appends "?iterationId=", the iteration id, "&amp;" and the returnto request value unencoded to it, followed by "?oid=" and "&amp;fkey=" parts (bytecode listing), so the host of this redirect is fixed; the continue step (ContinueUnfinishedStoriesAction#doExecute) then redirects to its own returnto parameter unchanged (Inferred; observed risk only, Q3 deferred; Q3 facts). Script context (BA-001-09, pass-007 F-002): the close confirmation uses the same page, WAR:WEB-INF/jsp/edit/editIterationStatus.jsp (WAR:WEB-INF/struts-config.xml:120,251), whose Cancel button writes the returnto request value unescaped into its onclick script (:70; row 98; Q3 facts).</t>
+    <t>class DomainMetaDataRepository#init (close -&gt; close/iteration); WAR:WEB-INF/struts-config.xml:251-255 (forward onclose -&gt; /do/continue/unfinished/stories); class CloseIterationAction ("closed", "onclose"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); CloseIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Redirect target (BA-001-08, pass-006 F-002, check (e)): CloseIterationAction#doExecute redirects to the fixed onclose forward (/do/continue/unfinished/stories) and appends "?iterationId=", the iteration id, "&amp;" and the returnto request value unencoded to it, followed by "?oid=" and "&amp;fkey=" parts (bytecode listing), so the host of this redirect is fixed; the continue step (ContinueUnfinishedStoriesAction#doExecute) then redirects to its own returnto parameter unchanged (Inferred; observed risk only, Q3 deferred; Q3 facts). Script context (BA-001-09, pass-007 F-002): the close confirmation uses the same page, WAR:WEB-INF/jsp/edit/editIterationStatus.jsp (WAR:WEB-INF/struts-config.xml:120,251), whose Cancel button writes the returnto request value unescaped into its onclick script (:70; row 98; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/CloseIterationAction.java CloseIterationAction#doExecute, #beforeObjectCommit. WAR: classes byte-identical to the v1.1a4 release. An active iteration is set inactive (closing samples in the hook) and the browser goes to the continue page.</t>
   </si>
   <si>
     <t>On the continue page the user selects a future iteration and confirms; unfinished stories are continued there.</t>
@@ -1348,7 +1348,7 @@
     <t>Target select with OK/Cancel; continued stories appear in the target iteration.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:277-279; WAR:WEB-INF/jsp/edit/continueUnfinishedStories.jsp; class ContinueUnfinishedStoriesAction#continueIteration. Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/continueUnfinishedStories.jsp writes the raw request parameters fkey (32) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt.</t>
+    <t>WAR:WEB-INF/struts-config.xml:277-279; WAR:WEB-INF/jsp/edit/continueUnfinishedStories.jsp; class ContinueUnfinishedStoriesAction#continueIteration. Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/continueUnfinishedStories.jsp writes the raw request parameters fkey (32) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ContinueUnfinishedStoriesAction.java ContinueUnfinishedStoriesAction#continueIteration. WAR: classes byte-identical to the v1.1a4 release. With a target iteration the unfinished stories are continued there.</t>
   </si>
   <si>
     <t>If no future iteration exists, the page says so.</t>
@@ -1360,7 +1360,7 @@
     <t>Message "No Future Iteration Available."</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/continueUnfinishedStories.jsp (iterationLoader.getIterationOptions(...).size() == 0; key iteration.status.editor.no_future_iteration).</t>
+    <t>WAR:WEB-INF/jsp/edit/continueUnfinishedStories.jsp (iterationLoader.getIterationOptions(...).size() == 0; key iteration.status.editor.no_future_iteration). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Choosing the same iteration is rejected.</t>
@@ -1372,7 +1372,7 @@
     <t>Message "You cannot continue in the same iteration. Please choose a different one."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.ContinueUnfinishedStoriesForm#validate (string iteration.status.editor.continue_in_same_iteration).</t>
+    <t>class com.technoetic.xplanner.forms.ContinueUnfinishedStoriesForm#validate (string iteration.status.editor.continue_in_same_iteration). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/ContinueUnfinishedStoriesForm.java ContinueUnfinishedStoriesForm#validate. WAR: classes byte-identical to the v1.1a4 release. The same iteration is rejected on OK.</t>
   </si>
   <si>
     <t>Tabbed iteration view</t>
@@ -1387,7 +1387,7 @@
     <t>Request expected to fail (missing JSP).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:199-201 (forward display -&gt; /WEB-INF/jsp/view/iterationTabs.jsp, ABSENT); WAR:WEB-INF/action-servlet.xml:84-88 (ViewObjectAction type Iteration); no live link found (linkgraph.txt).</t>
+    <t>WAR:WEB-INF/struts-config.xml:199-201 (forward display -&gt; /WEB-INF/jsp/view/iterationTabs.jsp, ABSENT); WAR:WEB-INF/action-servlet.xml:84-88 (ViewObjectAction type Iteration); no live link found (linkgraph.txt). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ViewObjectAction.java ViewObjectAction#doExecute. WAR: classes byte-identical to the v1.1a4 release; iterationTabs.jsp absent from both the WAR and the SVN webapp. The action forwards to the display path, whose JSP is missing.</t>
   </si>
   <si>
     <t>View all tasks of an iteration</t>
@@ -1402,7 +1402,7 @@
     <t>Grouped sortable task table with legend (started, completed, unassigned, unestimated).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:211-213; WAR:WEB-INF/jsp/view/iterationTasks.jsp; links from WAR:WEB-INF/jsp/view/iteration/links.jsp:29 and globalLinks.jsp:22.</t>
+    <t>WAR:WEB-INF/struts-config.xml:211-213; WAR:WEB-INF/jsp/view/iterationTasks.jsp; links from WAR:WEB-INF/jsp/view/iteration/links.jsp:29 and globalLinks.jsp:22. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Iteration metrics</t>
@@ -1417,7 +1417,7 @@
     <t>Page layout with developer table, paired/unpaired bars and legend; in this baseline the figures are expected to be empty or zero.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:219-221; WAR:WEB-INF/action-servlet.xml:114-118 (ViewIterationMetricsAction); WAR:WEB-INF/jsp/view/iterationMetrics.jsp:19-90; mappings/Metrics.xml query iterationHoursWorkedQuery. BA-001-03 impact sweep: ViewIterationMetricsAction#doExecute passes #getRepository(mapping, request) to IterationMetrics#setIterationRepository, and #getRepository returns null (bytecode listing: aconst_null, areturn); IterationMetrics#calculateDeveloperMetrics first calls #getIterationObject, which calls load on that repository, so the developer calculation is expected to fail with a null reference that IterationMetrics#analyze catches and logs; the page then shows zero totals and empty developer tables (runtime unverified).</t>
+    <t>WAR:WEB-INF/struts-config.xml:219-221; WAR:WEB-INF/action-servlet.xml:114-118 (ViewIterationMetricsAction); WAR:WEB-INF/jsp/view/iterationMetrics.jsp:19-90; mappings/Metrics.xml query iterationHoursWorkedQuery. BA-001-03 impact sweep: ViewIterationMetricsAction#doExecute passes #getRepository(mapping, request) to IterationMetrics#setIterationRepository, and #getRepository returns null (bytecode listing: aconst_null, areturn); IterationMetrics#calculateDeveloperMetrics first calls #getIterationObject, which calls load on that repository, so the developer calculation is expected to fail with a null reference that IterationMetrics#analyze catches and logs; the page then shows zero totals and empty developer tables (runtime unverified). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/ViewIterationMetricsAction.java ViewIterationMetricsAction#getRepository; SRC:src/com/technoetic/xplanner/metrics/IterationMetrics.java IterationMetrics#analyze, #calculateDeveloperMetrics. WAR: classes byte-identical to the v1.1a4 release. GetRepository returns null in the source as in the bytecode (the repository lookup is commented out); the page result is a runtime effect. Live question: Does the iteration metrics page show zero totals and empty developer tables?</t>
   </si>
   <si>
     <t>A second table shows per developer accepted hours (story and task), own worked hours, remaining hours and a worked-of-accepted bar.</t>
@@ -1429,7 +1429,7 @@
     <t>Accepted-hours table with bars; expected empty in this baseline for the same reason.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/iterationMetrics.jsp:96-175. BA-001-03 impact sweep: ViewIterationMetricsAction#doExecute passes #getRepository(mapping, request) to IterationMetrics#setIterationRepository, and #getRepository returns null (bytecode listing: aconst_null, areturn); IterationMetrics#calculateDeveloperMetrics first calls #getIterationObject, which calls load on that repository, so the developer calculation is expected to fail with a null reference that IterationMetrics#analyze catches and logs; the page then shows zero totals and empty developer tables (runtime unverified).</t>
+    <t>WAR:WEB-INF/jsp/view/iterationMetrics.jsp:96-175. BA-001-03 impact sweep: ViewIterationMetricsAction#doExecute passes #getRepository(mapping, request) to IterationMetrics#setIterationRepository, and #getRepository returns null (bytecode listing: aconst_null, areturn); IterationMetrics#calculateDeveloperMetrics first calls #getIterationObject, which calls load on that repository, so the developer calculation is expected to fail with a null reference that IterationMetrics#analyze catches and logs; the page then shows zero totals and empty developer tables (runtime unverified). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/ViewIterationMetricsAction.java ViewIterationMetricsAction#getRepository. WAR: classes byte-identical to the v1.1a4 release. Same cause as row 107. Live question: Is the accepted-hours table empty?</t>
   </si>
   <si>
     <t>Iteration statistics charts</t>
@@ -1444,7 +1444,7 @@
     <t>Cewolf-rendered 3D pie charts and the progress and burn-down line chart images.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/iteration/globalLinks.jsp:33-37; WAR:WEB-INF/struts-config.xml:223-225; WAR:WEB-INF/action-servlet.xml:120-124; WAR:WEB-INF/classes/xplanner.properties:66-73,197; WAR:WEB-INF/jsp/view/iterationStatistics.jsp:46-230 (cewolf charts); WAR:WEB-INF/web.xml:211-225,293-296 (CewolfServlet /cewolf/*). Chart sweep (BA-001-05): live charts in WAR:WEB-INF/jsp/view/iterationStatistics.jsp: taskTypeChart, taskDispositionChart, taskTypeEstimatedHoursChart, taskDispositionEstimatedHoursChart, taskTypeActualHoursChart, taskDispositionActualHoursChart (pie3d, lines 46-112); velocityChart (:123-153, flag xplanner.effort.chart.velocity), velocityChart2 progress chart (:155-191, flag xplanner.effort.chart.progress), burnDownChart (:193-228, flag xplanner.effort.chart.burndown); flags at WAR:WEB-INF/classes/xplanner.properties:66-68 (burndown and progress displayed, velocity notDisplayed). Corrected in BA-001-05 (Source: stage-02-pass-003 F-004). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/jsp/view/iteration/globalLinks.jsp:33-37; WAR:WEB-INF/struts-config.xml:223-225; WAR:WEB-INF/action-servlet.xml:120-124; WAR:WEB-INF/classes/xplanner.properties:66-73,197; WAR:WEB-INF/jsp/view/iterationStatistics.jsp:46-230 (cewolf charts); WAR:WEB-INF/web.xml:211-225,293-296 (CewolfServlet /cewolf/*). Chart sweep (BA-001-05): live charts in WAR:WEB-INF/jsp/view/iterationStatistics.jsp: taskTypeChart, taskDispositionChart, taskTypeEstimatedHoursChart, taskDispositionEstimatedHoursChart, taskTypeActualHoursChart, taskDispositionActualHoursChart (pie3d, lines 46-112); velocityChart (:123-153, flag xplanner.effort.chart.velocity), velocityChart2 progress chart (:155-191, flag xplanner.effort.chart.progress), burnDownChart (:193-228, flag xplanner.effort.chart.burndown); flags at WAR:WEB-INF/classes/xplanner.properties:66-68 (burndown and progress displayed, velocity notDisplayed). Corrected in BA-001-05 (Source: stage-02-pass-003 F-004). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
   </si>
   <si>
     <t>A progress line chart plots the iteration's estimated and actual hours from the stored data samples; it is shown while xplanner.effort.chart.progress is "displayed", which is the shipped value.</t>
@@ -1456,7 +1456,7 @@
     <t>Line chart "velocityChart2" with the aspects estimatedHours and actualHours; weekends included per xplanner.effort.chart.include.weekends.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/iterationStatistics.jsp:155-191 (propertyEqual key xplanner.effort.chart.progress value displayed; jsp:useBean velocityData2 class com.technoetic.xplanner.charts.DataSampleData, aspects estimatedHours,actualHours at :163-165; cewolf:chart velocityChart2 type line); WAR:WEB-INF/classes/xplanner.properties:67 (xplanner.effort.chart.progress=displayed), :73 (include.weekends=true). Data comes from the data samples (row 112). Provenance: property value from a rewritten entry (GAP-005 P-03). Source: stage-02-pass-003 F-004.</t>
+    <t>WAR:WEB-INF/jsp/view/iterationStatistics.jsp:155-191 (propertyEqual key xplanner.effort.chart.progress value displayed; jsp:useBean velocityData2 class com.technoetic.xplanner.charts.DataSampleData, aspects estimatedHours,actualHours at :163-165; cewolf:chart velocityChart2 type line); WAR:WEB-INF/classes/xplanner.properties:67 (xplanner.effort.chart.progress=displayed), :73 (include.weekends=true). Data comes from the data samples (row 112). Provenance: property value from a rewritten entry (GAP-005 P-03). Source: stage-02-pass-003 F-004. Source reconciliation (BA-001-11, A4): confirmed at class level. SRC:src/com/technoetic/xplanner/charts/DataSampleData.java DataSampleData. WAR: classes byte-identical to the v1.1a4 release; values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes exist and nothing read contradicts the claim.</t>
   </si>
   <si>
     <t>Velocity charts appear only if xplanner.effort.chart.velocity is "displayed" (shipped: notDisplayed); weekends are included in charts (include.weekends=true).</t>
@@ -1468,7 +1468,7 @@
     <t>No velocity chart in the shipped configuration.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/xplanner.properties:66-73; WAR:WEB-INF/jsp/view/iterationStatistics.jsp:123-153 (propertyEqual xplanner.effort.chart.velocity, velocityChart). Citation range narrowed in BA-001-05 (was 122-196, which also spanned the progress and burn-down blocks). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/classes/xplanner.properties:66-73; WAR:WEB-INF/jsp/view/iterationStatistics.jsp:123-153 (propertyEqual xplanner.effort.chart.velocity, velocityChart). Citation range narrowed in BA-001-05 (was 122-196, which also spanned the progress and burn-down blocks). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
   </si>
   <si>
     <t>The burn-down and progress charts depend on stored data samples; samples are written at iteration start/close and by the manual sampling action, while the nightly Quartz sampling trigger is not scheduled.</t>
@@ -1480,7 +1480,7 @@
     <t>Burn-down and progress charts may be sparse between start and close.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/spring-beans.xml:343-383 (datasamplingJob, datasamplingTrigger) and :385-402 (SchedulerFactoryBean commented out); references from classes StartIterationAction and CloseIterationAction to DataSampler; test-action-servlet.xml:4-7. Both charts use class com.technoetic.xplanner.charts.DataSampleData (WAR:WEB-INF/jsp/view/iterationStatistics.jsp:163-165 aspects estimatedHours,actualHours; :202-205 aspect remainingHours). Corrected in BA-001-05 (Source: stage-02-pass-003 F-004). Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>WAR:WEB-INF/classes/spring-beans.xml:343-383 (datasamplingJob, datasamplingTrigger) and :385-402 (SchedulerFactoryBean commented out); references from classes StartIterationAction and CloseIterationAction to DataSampler; test-action-servlet.xml:4-7. Both charts use class com.technoetic.xplanner.charts.DataSampleData (WAR:WEB-INF/jsp/view/iterationStatistics.jsp:163-165 aspects estimatedHours,actualHours; :202-205 aspect remainingHours). Corrected in BA-001-05 (Source: stage-02-pass-003 F-004). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/StartIterationAction.java StartIterationAction#beforeObjectCommit; SRC:src/com/technoetic/xplanner/actions/CloseIterationAction.java CloseIterationAction#beforeObjectCommit, #closeIteration. WAR: classes byte-identical to the v1.1a4 release; patched spring-beans.xml with the Quartz scheduler commented out (WAR governs). Opening samples are generated when an iteration starts and closing samples when an active iteration is closed; nothing else schedules sampling in the WAR configuration. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
   </si>
   <si>
     <t>Iteration accuracy</t>
@@ -1495,7 +1495,7 @@
     <t>Two summary tables with tooltips and a per-story table.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:227-229; WAR:WEB-INF/jsp/view/iterationAccuracy.jsp:21-186.</t>
+    <t>WAR:WEB-INF/struts-config.xml:227-229; WAR:WEB-INF/jsp/view/iterationAccuracy.jsp:21-186. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Iteration task board (dashboard)</t>
@@ -1510,7 +1510,7 @@
     <t>Story rows with task cards in three columns; cards can be dragged, but the drag only moves page elements and saves nothing.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/iteration/globalLinks.jsp:14-18 (xplanner:link to /do/view/dashboard with paramId iterationId, only if iteration.active); class com.technoetic.xplanner.tags.LinkTag#addNavigationParameters puts fkey = the tag attribute fkey when set, otherwise the current request's oid, and adds returnto and projectId when enabled (bytecode listing), so on /do/view/iteration*?oid=&lt;id&gt; the link carries fkey=&lt;id&gt;; WAR:WEB-INF/struts-config.xml:386; WAR:WEB-INF/jsp/view/dashboard.jsp:101-103 (column titles not started, in progress, done) and :131-132 ($.getJSON rest/view/iteration/${param.fkey}/userstories, row 223); no update call in dashboard.jsp. Corrected in BA-001-06 (Source: stage-02-pass-004 F-002): the earlier "parameter mismatch" did not account for the fkey parameter that the link tag adds. Request-value flow (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/view/dashboard.jsp:132 writes ${param.fkey} into a JavaScript string with EL (enabled under the Servlet 2.4 descriptor) without escaping, so the request value is reflected into the script (Inferred; observed risk only, Q3 deferred). Source: stage-02-pass-005 F-003.</t>
+    <t>WAR:WEB-INF/jsp/view/iteration/globalLinks.jsp:14-18 (xplanner:link to /do/view/dashboard with paramId iterationId, only if iteration.active); class com.technoetic.xplanner.tags.LinkTag#addNavigationParameters puts fkey = the tag attribute fkey when set, otherwise the current request's oid, and adds returnto and projectId when enabled (bytecode listing), so on /do/view/iteration*?oid=&lt;id&gt; the link carries fkey=&lt;id&gt;; WAR:WEB-INF/struts-config.xml:386; WAR:WEB-INF/jsp/view/dashboard.jsp:101-103 (column titles not started, in progress, done) and :131-132 ($.getJSON rest/view/iteration/${param.fkey}/userstories, row 223); no update call in dashboard.jsp. Corrected in BA-001-06 (Source: stage-02-pass-004 F-002): the earlier "parameter mismatch" did not account for the fkey parameter that the link tag adds. Request-value flow (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/view/dashboard.jsp:132 writes ${param.fkey} into a JavaScript string with EL (enabled under the Servlet 2.4 descriptor) without escaping, so the request value is reflected into the script (Inferred; observed risk only, Q3 deferred). Source: stage-02-pass-005 F-003. Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/tags/LinkTag.java LinkTag#addNavigationParameters. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
   </si>
   <si>
     <t>Import stories from a spreadsheet</t>
@@ -1525,7 +1525,7 @@
     <t>Result "Imported &lt;n&gt; stories"; stories created.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (importStories -&gt; import/stories); WAR:WEB-INF/struts-config.xml:332-346; WAR:WEB-INF/action-servlet.xml:361-368 (ImportStoriesAction, SpreadsheetStoryImporter); WAR:WEB-INF/jsp/import/stories.jsp; xplanner.properties:277-284 (default headers). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); ImportStoriesAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/import/stories.jsp writes the raw request parameters returnto (32), oid (36) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>class DomainMetaDataRepository#init (importStories -&gt; import/stories); WAR:WEB-INF/struts-config.xml:332-346; WAR:WEB-INF/action-servlet.xml:361-368 (ImportStoriesAction, SpreadsheetStoryImporter); WAR:WEB-INF/jsp/import/stories.jsp; xplanner.properties:277-284 (default headers). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); ImportStoriesAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/import/stories.jsp writes the raw request parameters returnto (32), oid (36) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init. WAR: classes byte-identical to the v1.1a4 release; values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
   </si>
   <si>
     <t>Missing required inputs are rejected before import.</t>
@@ -1537,7 +1537,7 @@
     <t>Messages for missing worksheet name, title, end date or priority header, completed status, or file.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.ImportStoriesForm#validate and ImportForm#validate (import.status.worksheet_name, no_title_column, no_end_date_column, no_priority_column, no_completed_story_status, no_import_file).</t>
+    <t>class com.technoetic.xplanner.forms.ImportStoriesForm#validate and ImportForm#validate (import.status.worksheet_name, no_title_column, no_end_date_column, no_priority_column, no_completed_story_status, no_import_file). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/ImportStoriesForm.java ImportStoriesForm#validate, #isNotEmpty; SRC:src/com/technoetic/xplanner/forms/ImportForm.java ImportForm#validate. WAR: classes byte-identical to the v1.1a4 release. Worksheet name, title, end-date and priority columns and (with the option) the completed status are required; the helper named isNotEmpty returns StringUtils.isEmpty, so the checks are correct despite the name (bytecode listing agrees).</t>
   </si>
   <si>
     <t>Import errors for a missing worksheet, missing header, missing required field or corrupt file are shown on the import page.</t>
@@ -1549,10 +1549,10 @@
     <t>Messages "Could not find worksheet named ...", "Could not find a column with ... as the header...", "Some stories did not have ... specified.", "...appears to be corrupt."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.actions.ImportStoriesAction#execute: exception handlers (bytecode exception table) catch importer.WrongImportFileSpreadsheetImporterException, MissingFieldSpreadsheetImporterException, MissingColumnHeaderSpreadsheetImporterException and importer.spreadsheet.MissingWorksheetException and save import.status.corrupted_file, missing_required_field, wrong_header and worksheet_not_found. The Struts mapping for the non-existent com.technoetic.xplanner.importer.MissingWorksheetException (WAR:WEB-INF/struts-config.xml:343-345) is therefore redundant, not a defect of the behavior. Corrected in BA-001-04 (Source: stage-02-pass-002 F-008).</t>
-  </si>
-  <si>
-    <t>Optionally only incomplete stories are imported (skip rows whose status equals the completed status, default "C").</t>
+    <t>class com.technoetic.xplanner.actions.ImportStoriesAction#execute: exception handlers (bytecode exception table) catch importer.WrongImportFileSpreadsheetImporterException, MissingFieldSpreadsheetImporterException, MissingColumnHeaderSpreadsheetImporterException and importer.spreadsheet.MissingWorksheetException and save import.status.corrupted_file, missing_required_field, wrong_header and worksheet_not_found. The Struts mapping for the non-existent com.technoetic.xplanner.importer.MissingWorksheetException (WAR:WEB-INF/struts-config.xml:343-345) is therefore redundant, not a defect of the behavior. Corrected in BA-001-04 (Source: stage-02-pass-002 F-008). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ImportStoriesAction.java ImportStoriesAction#execute. WAR: classes byte-identical to the v1.1a4 release. The four importer exceptions become global errors on the import page.</t>
+  </si>
+  <si>
+    <t>Optionally only incomplete stories are imported: rows whose status is "C" (ignoring case) are skipped; the completed-status field must be filled in but does not change this value.</t>
   </si>
   <si>
     <t>Avoid importing finished work.</t>
@@ -1561,7 +1561,7 @@
     <t>Completed rows skipped when the checkbox is set.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/import/stories.jsp (onlyIncomplete, completedStatus); xplanner.properties:284 (import.spreadsheet.completedStoryStatus=C); class SpreadsheetStoryImporter. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/jsp/import/stories.jsp (onlyIncomplete, completedStatus); xplanner.properties:284 (import.spreadsheet.completedStoryStatus=C); class SpreadsheetStoryImporter. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/importer/SpreadsheetStoryImporter.java SpreadsheetStoryImporter#importStories; SRC:src/com/technoetic/xplanner/forms/ImportStoriesForm.java ImportStoriesForm#validate; SRC:src/com/technoetic/xplanner/actions/ImportStoriesAction.java ImportStoriesAction#setCookies. WAR: classes byte-identical to the v1.1a4 release. With the option set, the importer skips rows whose status equals "C" ignoring case; this value is hard-coded (bytecode listing: ldc "C", equalsIgnoreCase). The completed-status field is only required by the form validation and kept in a cookie; it does not change the filter. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
   </si>
   <si>
     <t>After an import the worksheet name, column headers, only-incomplete choice and completed status are saved in browser cookies, and the next import form is pre-filled from those cookies before the property defaults.</t>
@@ -1573,7 +1573,7 @@
     <t>Import form pre-filled with the last used settings.</t>
   </si>
   <si>
-    <t>class ImportStoriesAction#setCookies (cookie names import.spreadsheet.worksheet.name, .story.title.column.header, .iteration.end.date.column.header, .story.estimate.column.header, .story.priority.column.header, .story.status.column.header, .onlyIncomplete, .completedStoryStatus), called from EditObjectAction#doExecute after #saveForm; #populateForm with #getValueFromCookieOrProperties (defaults WAR:WEB-INF/classes/xplanner.properties:278-284; provenance of these default values as in row 115, GAP-005 P-03). Source: stage-02-pass-002 F-008. Cookie lifetime and flags (BA-001-07, mechanism (b)): ImportStoriesAction#addCookie uses the same CookieSupport#createCookie (max-age 2147483647 seconds, no Secure flag, no path).</t>
+    <t>class ImportStoriesAction#setCookies (cookie names import.spreadsheet.worksheet.name, .story.title.column.header, .iteration.end.date.column.header, .story.estimate.column.header, .story.priority.column.header, .story.status.column.header, .onlyIncomplete, .completedStoryStatus), called from EditObjectAction#doExecute after #saveForm; #populateForm with #getValueFromCookieOrProperties (defaults WAR:WEB-INF/classes/xplanner.properties:278-284; provenance of these default values as in row 115, GAP-005 P-03). Source: stage-02-pass-002 F-008. Cookie lifetime and flags (BA-001-07, mechanism (b)): ImportStoriesAction#addCookie uses the same CookieSupport#createCookie (max-age 2147483647 seconds, no Secure flag, no path). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/ImportStoriesAction.java ImportStoriesAction#setCookies, #addCookie, #populateForm, #getValueFromCookieOrProperties; SRC:src/com/technoetic/xplanner/util/CookieSupport.java CookieSupport#createCookie. WAR: classes byte-identical to the v1.1a4 release. The eight settings are written as cookies after an import and read back, before the property defaults, when the form is shown.</t>
   </si>
   <si>
     <t>UF-007</t>
@@ -1594,7 +1594,7 @@
     <t>Story saved in the iteration; user returned to the iteration page.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (createStory -&gt; edit/userstory); WAR:WEB-INF/struts-config.xml:269-271; WAR:WEB-INF/action-servlet.xml:220-224 (EditStoryAction); WAR:WEB-INF/jsp/edit/editStory.jsp; classes com.technoetic.xplanner.domain.StoryStatus, StoryDisposition (enumeration strings). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editStory.jsp writes the raw request parameters oid (37), fkey (41,44), returnto (43) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/userstory that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new UserStory object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). With merge=true the story validator also skips its name, estimate and priority checks (row 124). No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
+    <t>class DomainMetaDataRepository#init (createStory -&gt; edit/userstory); WAR:WEB-INF/struts-config.xml:269-271; WAR:WEB-INF/action-servlet.xml:220-224 (EditStoryAction); WAR:WEB-INF/jsp/edit/editStory.jsp; classes com.technoetic.xplanner.domain.StoryStatus, StoryDisposition (enumeration strings). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editStory.jsp writes the raw request parameters oid (37), fkey (41,44), returnto (43) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/userstory that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new UserStory object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). With merge=true the story validator also skips its name, estimate and priority checks (row 124). No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init; SRC:src/com/technoetic/xplanner/domain/StoryStatus.java StoryStatus; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject, #doExecute. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
   </si>
   <si>
     <t>A new story defaults to priority 4.</t>
@@ -1606,7 +1606,7 @@
     <t>Priority field pre-filled with 4.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/xplanner.properties:150 (xplanner.story.defaultpriority=4); class UserStoryEditorForm (DEFAULT_PRIORITY_KEY, string "xplanner.story.defaultpriority"). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/classes/xplanner.properties:150 (xplanner.story.defaultpriority=4); class UserStoryEditorForm (DEFAULT_PRIORITY_KEY, string "xplanner.story.defaultpriority"). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/UserStoryEditorForm.java UserStoryEditorForm#reset, #resetPriority. WAR: classes byte-identical to the v1.1a4 release; default priority from the patched WAR xplanner.properties (WAR governs). Reset sets the priority from xplanner.story.defaultpriority, or from the class default when the key is missing. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
   </si>
   <si>
     <t>A missing name, a negative estimate or a non-numeric priority is rejected.</t>
@@ -1618,7 +1618,7 @@
     <t>Messages "Missing story name.", "Please provide an estimate greater than or equal to zero.", "Please provide a numeric priority."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.UserStoryEditorForm#validate (story.editor.missing_name, negative_estimated_hours, invalid_priority).</t>
+    <t>class com.technoetic.xplanner.forms.UserStoryEditorForm#validate (story.editor.missing_name, negative_estimated_hours, invalid_priority). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/UserStoryEditorForm.java UserStoryEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release. Without merge the name, a non-negative estimate and a numeric priority are required.</t>
   </si>
   <si>
     <t>A story editor request that carries merge=true skips the name, estimate and priority checks, is rejected only when the target iteration equals the current one, and otherwise binds its request parameters directly onto the story; no page of the WAR posts merge=true to the story editor, so this applies to direct requests.</t>
@@ -1630,7 +1630,7 @@
     <t>Message "Cannot move or continue story in same iteration." for merge=true with the same iteration; otherwise no validation message, and the story properties named by request parameters are set without the form copy (runtime unverified).</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.UserStoryEditorForm#validate (bytecode listing: #isMerge false -&gt; story.editor.missing_name, negative_estimated_hours, #validateIsNumber invalid_priority; #isMerge true -&gt; story.editor.same_iteration when targetIterationId equals iterationId). The hidden merge field occurs only in moveContinueStory.jsp, moveContinueTask.jsp, continueUnfinishedStories.jsp and task.jsp, none of which posts to /do/edit/userstory (WAR:WEB-INF/jsp/edit/moveContinueStory.jsp:20,24). CHK-005 (BA-001-05). Source: stage-02-pass-003 F-003. Request binding (BA-001-08, pass-006 F-001): with merge=true, EditObjectAction#populateObject calls org.apache.struts.util.RequestUtils.populate onto the story instead of copying the form and resolving its many-to-one references (bytecode listing), so any writable story property named by a parameter is set, including properties the editor does not show; together with the skipped checks, unvalidated values reach the saved story (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
+    <t>class com.technoetic.xplanner.forms.UserStoryEditorForm#validate (bytecode listing: #isMerge false -&gt; story.editor.missing_name, negative_estimated_hours, #validateIsNumber invalid_priority; #isMerge true -&gt; story.editor.same_iteration when targetIterationId equals iterationId). The hidden merge field occurs only in moveContinueStory.jsp, moveContinueTask.jsp, continueUnfinishedStories.jsp and task.jsp, none of which posts to /do/edit/userstory (WAR:WEB-INF/jsp/edit/moveContinueStory.jsp:20,24). CHK-005 (BA-001-05). Source: stage-02-pass-003 F-003. Request binding (BA-001-08, pass-006 F-001): with merge=true, EditObjectAction#populateObject calls org.apache.struts.util.RequestUtils.populate onto the story instead of copying the form and resolving its many-to-one references (bytecode listing), so any writable story property named by a parameter is set, including properties the editor does not show; together with the skipped checks, unvalidated values reach the saved story (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/forms/UserStoryEditorForm.java UserStoryEditorForm#validate; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject. WAR: classes byte-identical to the v1.1a4 release. The two validation branches are confirmed; which properties the binding sets is commons-beanutils behavior (GAP-011). Live question: Does a direct story-editor request with merge=true and an extra property parameter change that property?</t>
   </si>
   <si>
     <t>Edit user story</t>
@@ -1645,7 +1645,7 @@
     <t>Editor titled for the story with Update/Reset; changes saved.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (story edit -&gt; /do/edit/userstory, permission edit); WAR:WEB-INF/jsp/edit/editStory.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 121 applies to every /do/edit/userstory request (Inferred; Q3 facts).</t>
+    <t>class DomainMetaDataRepository#init (story edit -&gt; /do/edit/userstory, permission edit); WAR:WEB-INF/jsp/edit/editStory.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 121 applies to every /do/edit/userstory request (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
   </si>
   <si>
     <t>Delete user story</t>
@@ -1660,7 +1660,7 @@
     <t>Confirm prompt; story, tasks and time entries removed (runtime unverified).</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (story delete -&gt; /do/delete/userstory, action.delete.confirmation); WAR:WEB-INF/struts-config.xml:285; WAR:WEB-INF/action-servlet.xml:256-260. Cascades: UserStory#getTasks, Task#getTimeEntries @OneToMany(cascade=REMOVE). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002).</t>
+    <t>class DomainMetaDataRepository#init (story delete -&gt; /do/delete/userstory, action.delete.confirmation); WAR:WEB-INF/struts-config.xml:285; WAR:WEB-INF/action-servlet.xml:256-260. Cascades: UserStory#getTasks, Task#getTimeEntries @OneToMany(cascade=REMOVE). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute; SRC:src/net/sf/xplanner/domain/UserStory.java UserStory#getTasks. WAR: classes byte-identical to the v1.1a4 release. The cascades match the source annotations.</t>
   </si>
   <si>
     <t>View user story</t>
@@ -1675,7 +1675,7 @@
     <t>Story summary card and task table with action icons; "create task", export and history links.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:265-267; WAR:WEB-INF/jsp/view/userstory.jsp.</t>
+    <t>WAR:WEB-INF/struts-config.xml:265-267; WAR:WEB-INF/jsp/view/userstory.jsp. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>A story without tasks shows a "no tasks" message.</t>
@@ -1684,7 +1684,7 @@
     <t>Message story.no_tasks.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/userstory.jsp (story.no_tasks).</t>
+    <t>WAR:WEB-INF/jsp/view/userstory.jsp (story.no_tasks). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Move or continue a story</t>
@@ -1699,7 +1699,7 @@
     <t>Move/Continue page with target iteration; story moved.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (movecontinue -&gt; /do/move/continue/userstory); WAR:WEB-INF/struts-config.xml:273-275; WAR:WEB-INF/jsp/edit/moveContinueStory.jsp; class MoveContinueStoryAction#saveForm ("Move"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); MoveContinueStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/moveContinueStory.jsp writes the raw request parameters fkey (25) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001): the Move/Continue page posts merge=true together with oid, iterationId, fkey, action and returnto (WAR:WEB-INF/jsp/edit/moveContinueStory.jsp:20-28); MoveContinueStoryAction#saveForm calls EditObjectAction#populateObject, which binds every request parameter onto the story with org.apache.struts.util.RequestUtils.populate before the move (bytecode listing; Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect (F-002): MoveContinueStoryAction#doExecute then redirects to the returnto request value unchanged (Q3 facts).</t>
+    <t>class DomainMetaDataRepository#init (movecontinue -&gt; /do/move/continue/userstory); WAR:WEB-INF/struts-config.xml:273-275; WAR:WEB-INF/jsp/edit/moveContinueStory.jsp; class MoveContinueStoryAction#saveForm ("Move"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); MoveContinueStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/moveContinueStory.jsp writes the raw request parameters fkey (25) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001): the Move/Continue page posts merge=true together with oid, iterationId, fkey, action and returnto (WAR:WEB-INF/jsp/edit/moveContinueStory.jsp:20-28); MoveContinueStoryAction#saveForm calls EditObjectAction#populateObject, which binds every request parameter onto the story with org.apache.struts.util.RequestUtils.populate before the move (bytecode listing; Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect (F-002): MoveContinueStoryAction#doExecute then redirects to the returnto request value unchanged (Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init; SRC:src/com/technoetic/xplanner/actions/MoveContinueStoryAction.java MoveContinueStoryAction#saveForm, #doExecute; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
   </si>
   <si>
     <t>Continue creates a continuation of the story in the target iteration for the unfinished work, with cross-references in the descriptions.</t>
@@ -1711,7 +1711,7 @@
     <t>New continued story in target; descriptions reference the origin/continuation.</t>
   </si>
   <si>
-    <t>class MoveContinueStoryAction#saveForm ("Continue"); classes com.technoetic.xplanner.actions.StoryContinuer, TaskContinuer (strings continue.description.from/to); ResourceBundle.properties task.continued.to/from.</t>
+    <t>class MoveContinueStoryAction#saveForm ("Continue"); classes com.technoetic.xplanner.actions.StoryContinuer, TaskContinuer (strings continue.description.from/to); ResourceBundle.properties task.continued.to/from. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/Continuer.java Continuer#continueObject, #updateDescriptionAndHistory; SRC:src/com/technoetic/xplanner/actions/StoryContinuer.java StoryContinuer#doContinueObject. WAR: classes byte-identical to the v1.1a4 release. The continuation gets the remaining task-based hours, a disposition from the target iteration state and continuations of the unfinished tasks; both descriptions and the history receive the cross-references.</t>
   </si>
   <si>
     <t>Moving or continuing into the same iteration is rejected.</t>
@@ -1723,7 +1723,7 @@
     <t>Message "Cannot move or continue story in same iteration."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.MoveContinueStoryForm#validate (story.editor.same_iteration). The check runs on the merge branch of MoveContinueStoryForm#validate, which is the branch the move/continue page posts (row 132 covers the other branch). BA-001-05.</t>
+    <t>class com.technoetic.xplanner.forms.MoveContinueStoryForm#validate (story.editor.same_iteration). The check runs on the merge branch of MoveContinueStoryForm#validate, which is the branch the move/continue page posts (row 132 covers the other branch). BA-001-05. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/MoveContinueStoryForm.java MoveContinueStoryForm#validate. WAR: classes byte-identical to the v1.1a4 release. With merge the target iteration must differ.</t>
   </si>
   <si>
     <t>A move/continue story request without merge=true and without a name is rejected; the move/continue page always posts merge=true, so this applies to direct requests.</t>
@@ -1735,7 +1735,7 @@
     <t>Message "Missing story name." (runtime unverified).</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.MoveContinueStoryForm#validate (bytecode listing: #isMerge false -&gt; story.editor.missing_name; #isMerge true -&gt; story.editor.same_iteration); WAR:WEB-INF/jsp/edit/moveContinueStory.jsp:20,24 (form to /do/move/continue/userstory with hidden merge=true). CHK-005 (BA-001-05). Source: stage-02-pass-003 F-003.</t>
+    <t>class com.technoetic.xplanner.forms.MoveContinueStoryForm#validate (bytecode listing: #isMerge false -&gt; story.editor.missing_name; #isMerge true -&gt; story.editor.same_iteration); WAR:WEB-INF/jsp/edit/moveContinueStory.jsp:20,24 (form to /do/move/continue/userstory with hidden merge=true). CHK-005 (BA-001-05). Source: stage-02-pass-003 F-003. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/MoveContinueStoryForm.java MoveContinueStoryForm#validate. WAR: classes byte-identical to the v1.1a4 release. Without merge the name is required; with merge only the target iteration is checked.</t>
   </si>
   <si>
     <t>UF-008</t>
@@ -1756,7 +1756,7 @@
     <t>Task saved; user returned to the story.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/userstory.jsp (link /do/edit/task, story.link.create_task); WAR:WEB-INF/struts-config.xml:291; WAR:WEB-INF/action-servlet.xml:268-272 (EditTaskAction); WAR:WEB-INF/jsp/edit/editTask.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editTask.jsp writes the raw request parameters oid (31), returnto (34), fkey (36,37) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/task that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Task object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). EditTaskAction#populateObject calls the parent method. With merge=true the task validator skips its name and estimate checks (row 137). The complete and reopen buttons of the task page post merge=true (rows 140-141); any other parameter added to such a request is bound as well (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute (reached from EditTaskAction#doExecute) redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
+    <t>WAR:WEB-INF/jsp/view/userstory.jsp (link /do/edit/task, story.link.create_task); WAR:WEB-INF/struts-config.xml:291; WAR:WEB-INF/action-servlet.xml:268-272 (EditTaskAction); WAR:WEB-INF/jsp/edit/editTask.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editTask.jsp writes the raw request parameters oid (31), returnto (34), fkey (36,37) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/task that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Task object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). EditTaskAction#populateObject calls the parent method. With merge=true the task validator skips its name and estimate checks (row 137). The complete and reopen buttons of the task page post merge=true (rows 140-141); any other parameter added to such a request is bound as well (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute (reached from EditTaskAction#doExecute) redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/actions/EditTaskAction.java EditTaskAction#populateObject, #doExecute; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject, #doExecute. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
   </si>
   <si>
     <t>The task type is stored as a message label, not a code: the type options carry label text as their values, resolved without the user's locale, so the stored value follows the server default locale. The labels differ between bundles.</t>
@@ -1768,10 +1768,10 @@
     <t>Type select shows the user's language; the stored value is the server-default-locale label (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editTask.jsp:52-69 (html:option value=messages.getMessage("task.type.feature") ... "task.type.overhead", no locale argument); class net.sf.xplanner.struts.XPlannerMessageResources#getMessage delegates to the Spring MessageSource (null locale falls back to the JVM default, framework behavior, GAP-011). Per bundle (CHK-004, .migration-tmp/stage-01/out/task-type-labels.json): the default and "--" bundles use Feature, Defect, Debt, FTest, ATest, Overhead; da, de, es, fr, it, ja and ru differ from the default for at least one type; pt_br matches except that it has no overhead key; da, es, fr and pt_br define no task.type.overhead (fallback to the default). Corrected in BA-001-04 (Source: stage-02-pass-002 F-009).</t>
-  </si>
-  <si>
-    <t>The default disposition of a new task depends on the story/iteration state.</t>
+    <t>WAR:WEB-INF/jsp/edit/editTask.jsp:52-69 (html:option value=messages.getMessage("task.type.feature") ... "task.type.overhead", no locale argument); class net.sf.xplanner.struts.XPlannerMessageResources#getMessage delegates to the Spring MessageSource (null locale falls back to the JVM default, framework behavior, GAP-011). Per bundle (CHK-004, .migration-tmp/stage-01/out/task-type-labels.json): the default and "--" bundles use Feature, Defect, Debt, FTest, ATest, Overhead; da, de, es, fr, it, ja and ru differ from the default for at least one type; pt_br matches except that it has no overhead key; da, es, fr and pt_br define no task.type.overhead (fallback to the default). Corrected in BA-001-04 (Source: stage-02-pass-002 F-009). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/net/sf/xplanner/struts/XPlannerMessageResources.java XPlannerMessageResources#getMessage. WAR: classes byte-identical to the v1.1a4 release; editTask.jsp identical to the SVN webapp copy. The page asks for the label without a locale; the stored value then follows the Spring message source and the JVM default locale (framework behavior). Live question: Which type value is stored for a task created in a de session on a server whose default locale is English?</t>
+  </si>
+  <si>
+    <t>The default disposition of a new task is "discovered" when its story is started or its iteration is active, and "planned" otherwise.</t>
   </si>
   <si>
     <t>Distinguishes planned from added/discovered work.</t>
@@ -1780,7 +1780,7 @@
     <t>Disposition pre-selected.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.actions.EditTaskAction#setTaskDisposition/#getTaskDisposition (UserStory, Iteration). Rule not decompiled.</t>
+    <t>class com.technoetic.xplanner.actions.EditTaskAction#setTaskDisposition/#getTaskDisposition (UserStory, Iteration). Rule not decompiled. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/EditTaskAction.java EditTaskAction#setTaskDisposition, #getTaskDisposition; SRC:src/net/sf/xplanner/domain/Iteration.java Iteration#getNewTaskDisposition. WAR: classes byte-identical to the v1.1a4 release. The rule is now visible: for a new task (no oid, form not submitted) the disposition is "discovered" when the story is started or the iteration is active, otherwise "planned".</t>
   </si>
   <si>
     <t>A missing name, a negative estimate or an invalid created date is rejected.</t>
@@ -1789,7 +1789,7 @@
     <t>Messages "Missing task name.", "Please provide an estimate greater than or equal to zero.", "Created date is invalid."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TaskEditorForm#validate (task.editor.missing_name, negative_estimated_hours, bad_created_date). Merge branch (CHK-005, BA-001-05): TaskEditorForm#validate checks the created date first and skips the name and estimate checks when merge=true, which the complete and reopen buttons post (WAR:WEB-INF/jsp/view/task.jsp:76-79,87-90). Request binding (BA-001-08, pass-006 F-001): the same merge=true requests are bound onto the task by EditObjectAction#populateObject with org.apache.struts.util.RequestUtils.populate instead of the form copy (EditTaskAction#populateObject calls the parent), so the skipped name and estimate checks leave any task property named by a parameter unvalidated (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
+    <t>class com.technoetic.xplanner.forms.TaskEditorForm#validate (task.editor.missing_name, negative_estimated_hours, bad_created_date). Merge branch (CHK-005, BA-001-05): TaskEditorForm#validate checks the created date first and skips the name and estimate checks when merge=true, which the complete and reopen buttons post (WAR:WEB-INF/jsp/view/task.jsp:76-79,87-90). Request binding (BA-001-08, pass-006 F-001): the same merge=true requests are bound onto the task by EditObjectAction#populateObject with org.apache.struts.util.RequestUtils.populate instead of the form copy (EditTaskAction#populateObject calls the parent), so the skipped name and estimate checks leave any task property named by a parameter unvalidated (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/TaskEditorForm.java TaskEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release. A given created date must parse; without merge the name and a non-negative estimate are required.</t>
   </si>
   <si>
     <t>Task e-mail notification</t>
@@ -1801,10 +1801,10 @@
     <t>Keeps assignees informed.</t>
   </si>
   <si>
-    <t>E-mail "Task was created." or "Task was updated." with task, assignee and old assignee details.</t>
-  </si>
-  <si>
-    <t>class EditTaskAction#sendNotification (templates com/technoetic/xplanner/mail/velocity/email_notification_task_created.vm and ..._updated.vm; EmailNotificationSupport.compileEmail/sendNotifications); WAR:WEB-INF/classes/EmailResourceBundle.properties task.created.*, task.updated.*; recipients not determinable statically.</t>
+    <t>E-mail "Task was created." or "Task was updated." to the editor and, when the task has an acceptor, to the acceptor, with task and assignee details; the old-assignee value is taken from the new acceptor, so after a reassignment it shows the new assignee (runtime unverified).</t>
+  </si>
+  <si>
+    <t>class EditTaskAction#sendNotification (templates com/technoetic/xplanner/mail/velocity/email_notification_task_created.vm and ..._updated.vm; EmailNotificationSupport.compileEmail/sendNotifications); WAR:WEB-INF/classes/EmailResourceBundle.properties task.created.*, task.updated.*; recipients not determinable statically. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/actions/EditTaskAction.java EditTaskAction#sendNotification; SRC:src/com/technoetic/xplanner/mail/EmailNotificationSupport.java EmailNotificationSupport#compileEmail. WAR: classes byte-identical to the v1.1a4 release. The recipients are determinable: mail is compiled only after a redirecting save by a signed-in user, for the editor and, when the task has an acceptor, for the acceptor. The "old assignee" is always derived from the new acceptor id (bytecode listing agrees), so it names the new assignee whenever one is set. Delivery depends on SMTP. Live question: Are the created and updated mails delivered to the editor and the acceptor, and which old assignee does an updated mail show after a reassignment?</t>
   </si>
   <si>
     <t>Edit task</t>
@@ -1819,7 +1819,7 @@
     <t>Task editor with Update/Reset; changes saved.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (task edit -&gt; /do/edit/task); WAR:WEB-INF/jsp/edit/editTask.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 134 applies to every /do/edit/task request (Inferred; Q3 facts).</t>
+    <t>class DomainMetaDataRepository#init (task edit -&gt; /do/edit/task); WAR:WEB-INF/jsp/edit/editTask.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 134 applies to every /do/edit/task request (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
   </si>
   <si>
     <t>Complete or reopen task</t>
@@ -1834,7 +1834,7 @@
     <t>"Complete" button; task becomes completed; page reloads.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/task.jsp:86-95 (form /do/edit/task, action Update, merge true, completed true). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Mechanism (BA-001-08, pass-006 F-001): the completion takes effect through the merge=true binding, not through the task form: EditObjectAction#populateObject calls org.apache.struts.util.RequestUtils.populate, which sets Task#setCompleted from the posted completed=true (WAR:WEB-INF/jsp/view/task.jsp:87-94); any further parameter added to the request is bound onto the task as well (Inferred; Q3 facts). After the save, EditObjectAction#doExecute redirects to the posted returnto value (F-002).</t>
+    <t>WAR:WEB-INF/jsp/view/task.jsp:86-95 (form /do/edit/task, action Update, merge true, completed true). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Mechanism (BA-001-08, pass-006 F-001): the completion takes effect through the merge=true binding, not through the task form: EditObjectAction#populateObject calls org.apache.struts.util.RequestUtils.populate, which sets Task#setCompleted from the posted completed=true (WAR:WEB-INF/jsp/view/task.jsp:87-94); any further parameter added to the request is bound onto the task as well (Inferred; Q3 facts). After the save, EditObjectAction#doExecute redirects to the posted returnto value (F-002). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject, #doExecute; SRC:src/net/sf/xplanner/domain/Task.java Task#setCompleted. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
   </si>
   <si>
     <t>A completed task can be reopened.</t>
@@ -1846,7 +1846,7 @@
     <t>"Reopen" button; task becomes open again.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/task.jsp:75-84 (completed false). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Mechanism (BA-001-08, pass-006 F-001): the reopen form posts merge=true and completed=false (WAR:WEB-INF/jsp/view/task.jsp:76-83), so the change is made by the same RequestUtils.populate binding as in row 140 (Inferred; Q3 facts).</t>
+    <t>WAR:WEB-INF/jsp/view/task.jsp:75-84 (completed false). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Mechanism (BA-001-08, pass-006 F-001): the reopen form posts merge=true and completed=false (WAR:WEB-INF/jsp/view/task.jsp:76-83), so the change is made by the same RequestUtils.populate binding as in row 140 (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Delete task</t>
@@ -1861,7 +1861,7 @@
     <t>Confirm prompt; task and its time entries removed (runtime unverified).</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (task delete -&gt; /do/delete/task, action.delete.confirmation); WAR:WEB-INF/struts-config.xml:304; WAR:WEB-INF/action-servlet.xml:300-304. Cascade: Task#getTimeEntries @OneToMany(cascade=REMOVE). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002).</t>
+    <t>class DomainMetaDataRepository#init (task delete -&gt; /do/delete/task, action.delete.confirmation); WAR:WEB-INF/struts-config.xml:304; WAR:WEB-INF/action-servlet.xml:300-304. Cascade: Task#getTimeEntries @OneToMany(cascade=REMOVE). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute; SRC:src/net/sf/xplanner/domain/Task.java Task#getTimeEntries. WAR: classes byte-identical to the v1.1a4 release. The cascade matches the source annotation.</t>
   </si>
   <si>
     <t>View task</t>
@@ -1876,7 +1876,7 @@
     <t>Task card and time-log table; action links (edit, delete, move/continue, time) by permission; export and history links.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:287-289; WAR:WEB-INF/jsp/view/task.jsp.</t>
+    <t>WAR:WEB-INF/struts-config.xml:287-289; WAR:WEB-INF/jsp/view/task.jsp. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Move or continue a task</t>
@@ -1891,7 +1891,7 @@
     <t>Move/Continue page with target story; history records "moved".</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (task movecontinue -&gt; /do/move/continue/task); WAR:WEB-INF/struts-config.xml:293-295; WAR:WEB-INF/jsp/edit/moveContinueTask.jsp; class MoveContinueTaskAction#saveForm ("Move", "task.moved.from.to", "moved out", "moved in"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); MoveContinueTaskAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/moveContinueTask.jsp writes the raw request parameters fkey (25) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt.</t>
+    <t>class DomainMetaDataRepository#init (task movecontinue -&gt; /do/move/continue/task); WAR:WEB-INF/struts-config.xml:293-295; WAR:WEB-INF/jsp/edit/moveContinueTask.jsp; class MoveContinueTaskAction#saveForm ("Move", "task.moved.from.to", "moved out", "moved in"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); MoveContinueTaskAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/moveContinueTask.jsp writes the raw request parameters fkey (25) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init; SRC:src/com/technoetic/xplanner/actions/MoveContinueTaskAction.java MoveContinueTaskAction#saveForm. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
   </si>
   <si>
     <t>Continue copies the unfinished task into the target story with cross-referenced descriptions.</t>
@@ -1903,7 +1903,7 @@
     <t>New task "Continued from task:&lt;id&gt;".</t>
   </si>
   <si>
-    <t>class MoveContinueTaskAction#saveForm ("Continue"); class TaskContinuer; ResourceBundle.properties task.continued.to/from.</t>
+    <t>class MoveContinueTaskAction#saveForm ("Continue"); class TaskContinuer; ResourceBundle.properties task.continued.to/from. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/TaskContinuer.java TaskContinuer#doContinueObject; SRC:src/com/technoetic/xplanner/actions/Continuer.java Continuer#continueObject, #updateDescriptionAndHistory. WAR: classes byte-identical to the v1.1a4 release. The continued task gets the remaining hours as its estimate, no acceptor and no time entries, and the original task is postponed; descriptions and history receive the cross-references.</t>
   </si>
   <si>
     <t>Moving or continuing into the same story is rejected.</t>
@@ -1912,7 +1912,7 @@
     <t>Validation message task.editor.same_story.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.MoveContinueTaskForm#validate (merge branch: task.editor.same_story; the non-merge branch task.editor.missing_name is row 147). Wording corrected in BA-001-05 (Source: stage-02-pass-003 F-003).</t>
+    <t>class com.technoetic.xplanner.forms.MoveContinueTaskForm#validate (merge branch: task.editor.same_story; the non-merge branch task.editor.missing_name is row 147). Wording corrected in BA-001-05 (Source: stage-02-pass-003 F-003). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/MoveContinueTaskForm.java MoveContinueTaskForm#validate. WAR: classes byte-identical to the v1.1a4 release. With merge the target story must differ.</t>
   </si>
   <si>
     <t>A move/continue task request without merge=true and without a name is rejected; the move/continue page always posts merge=true, so this applies to direct requests.</t>
@@ -1924,7 +1924,7 @@
     <t>Message "Missing task name." (runtime unverified).</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.MoveContinueTaskForm#validate (bytecode listing: #isMerge false -&gt; task.editor.missing_name; #isMerge true -&gt; task.editor.same_story); WAR:WEB-INF/jsp/edit/moveContinueTask.jsp:21,24 (form to /do/move/continue/task with hidden merge=true). CHK-005 (BA-001-05), wording point of pass-003 F-003.</t>
+    <t>class com.technoetic.xplanner.forms.MoveContinueTaskForm#validate (bytecode listing: #isMerge false -&gt; task.editor.missing_name; #isMerge true -&gt; task.editor.same_story); WAR:WEB-INF/jsp/edit/moveContinueTask.jsp:21,24 (form to /do/move/continue/task with hidden merge=true). CHK-005 (BA-001-05), wording point of pass-003 F-003. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/MoveContinueTaskForm.java MoveContinueTaskForm#validate. WAR: classes byte-identical to the v1.1a4 release. Without merge the name is required; with merge only the target story is checked.</t>
   </si>
   <si>
     <t>UF-009</t>
@@ -1945,7 +1945,7 @@
     <t>Time grid with an empty new row; "Insert Time" fills current time; Update saves; redirect to the task page.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (edittime -&gt; /do/edit/time); WAR:WEB-INF/struts-config.xml:350-355; WAR:WEB-INF/action-servlet.xml:376-378 (UpdateTimeAction); WAR:WEB-INF/jsp/edit/editTimeEntries.jsp; WAR:editTimeEntries.js; WAR:time.js. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); UpdateTimeAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editTimeEntries.jsp writes the raw request parameters oid (59), returnto (61), fkey (63,64) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Redirect target (BA-001-08, pass-006 F-002, check (e)): UpdateTimeAction#doUpdateTimeAction (and #doUpdateEstimateAction for the estimate action) redirects to the returnto value posted by the time editor, unchanged (new ActionForward(returnto, true)); there is no fallback for a missing value, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
+    <t>class DomainMetaDataRepository#init (edittime -&gt; /do/edit/time); WAR:WEB-INF/struts-config.xml:350-355; WAR:WEB-INF/action-servlet.xml:376-378 (UpdateTimeAction); WAR:WEB-INF/jsp/edit/editTimeEntries.jsp; WAR:editTimeEntries.js; WAR:time.js. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); UpdateTimeAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editTimeEntries.jsp writes the raw request parameters oid (59), returnto (61), fkey (63,64) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Redirect target (BA-001-08, pass-006 F-002, check (e)): UpdateTimeAction#doUpdateTimeAction (and #doUpdateEstimateAction for the estimate action) redirects to the returnto value posted by the time editor, unchanged (new ActionForward(returnto, true)); there is no fallback for a missing value, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#doUpdateTimeAction. WAR: classes byte-identical to the v1.1a4 release. New rows with a start time or a duration are saved, existing rows are edited or deleted, and the browser is redirected to returnto.</t>
   </si>
   <si>
     <t>Existing entries can be edited or marked for deletion in the same grid.</t>
@@ -1957,7 +1957,7 @@
     <t>Delete checkbox per row; changes saved on Update.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editTimeEntries.jsp (deleted[row] checkbox).</t>
+    <t>WAR:WEB-INF/jsp/edit/editTimeEntries.jsp (deleted[row] checkbox). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>The remaining-hours field recalculates as durations change and updates the task estimate on save.</t>
@@ -1969,7 +1969,7 @@
     <t>Remaining hours shown (red when negative); task estimate updated.</t>
   </si>
   <si>
-    <t>WAR:editTimeEntries.js:9-19,65-67 (remainingHours recalculation); class UpdateTimeAction#doUpdateTimeAction (TimeEditorForm.getRemainingHours, Task.setEstimatedHours).</t>
+    <t>WAR:editTimeEntries.js:9-19,65-67 (remainingHours recalculation); class UpdateTimeAction#doUpdateTimeAction (TimeEditorForm.getRemainingHours, Task.setEstimatedHours). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#doUpdateTimeAction. WAR: classes byte-identical to the v1.1a4 release; editTimeEntries.js identical to the SVN webapp copy. On save, when the remaining hours are given and not negative, the task estimate becomes the effort of the form's entries plus the remaining hours.</t>
   </si>
   <si>
     <t>Unparsable date/time or number input in a time entry row is rejected.</t>
@@ -1978,10 +1978,10 @@
     <t>Time editor redisplayed with "Can't parse the supplied date/time value." or "Can't parse the supplied number." (forward "error").</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.unparsable_time, edittime.error.unparsable_number; WAR:WEB-INF/classes/ResourceBundle.properties:675-676; WAR:WEB-INF/struts-config.xml:353-354 (error -&gt; editTimeEntries.jsp). Corrected in BA-001-04 (Source: stage-02-pass-002 F-001; the validator is the form, not UpdateTimeAction). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.unparsable_time: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). edittime.error.unparsable_number is missing in es and fr. Bundles without the key fall back to the default text (framework behavior, GAP-011). The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71).</t>
-  </si>
-  <si>
-    <t>A time entry row with an end time but no start time, or a start time but no end time, is rejected.</t>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.unparsable_time, edittime.error.unparsable_number; WAR:WEB-INF/classes/ResourceBundle.properties:675-676; WAR:WEB-INF/struts-config.xml:353-354 (error -&gt; editTimeEntries.jsp). Corrected in BA-001-04 (Source: stage-02-pass-002 F-001; the validator is the form, not UpdateTimeAction). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.unparsable_time: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). edittime.error.unparsable_number is missing in es and fr. Bundles without the key fall back to the default text (framework behavior, GAP-011). The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#valideRow. WAR: classes byte-identical to the v1.1a4 release. Start, end and report date are converted with the unparsable-time key and the duration with the unparsable-number key, as recorded.</t>
+  </si>
+  <si>
+    <t>A time entry row other than the last one that lacks a start or an end time and has no duration is rejected, as is any row with an end time and a duration but no start time; in the last row a start time alone is accepted.</t>
   </si>
   <si>
     <t>Intervals must be complete.</t>
@@ -1990,7 +1990,7 @@
     <t>Message "Missing start or end time."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.missing_time; WAR:WEB-INF/classes/ResourceBundle.properties:677. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.missing_time: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru).</t>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.missing_time; WAR:WEB-INF/classes/ResourceBundle.properties:677. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.missing_time: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. The missing-time check (#1) applies to every row except the last one: a row that lacks a start or an end time and has no duration is rejected; a row with an end time, no start time and a duration is also rejected (#6). In the last row a start time without end time or duration is not rejected and is saved as an entry without end time (UpdateTimeAction#doUpdateTimeAction saves a new row when it has a start time or a duration).</t>
   </si>
   <si>
     <t>A time entry row without any person is rejected.</t>
@@ -2002,10 +2002,10 @@
     <t>Message "No person is specified in a time entry."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.missing_person; ResourceBundle.properties:678. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.missing_person: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru).</t>
-  </si>
-  <si>
-    <t>A time entry row naming the same person as both pair members is rejected.</t>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.missing_person; ResourceBundle.properties:678. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.missing_person: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. A row that has an id, a start or end time, or a positive duration, but neither person, is rejected with the missing-person key.</t>
+  </si>
+  <si>
+    <t>A time entry row with a start time that names the same person as both pair members is rejected; a duration-only row is not checked.</t>
   </si>
   <si>
     <t>Pairing needs two different people.</t>
@@ -2014,7 +2014,7 @@
     <t>Message "Must specify different people for time entry."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.same_people; ResourceBundle.properties:681. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.same_people: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru).</t>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.same_people; ResourceBundle.properties:681. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.same_people: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. The same-people check runs only when a person is present and the row has a start time: a duration-only row with the same person twice is not rejected.</t>
   </si>
   <si>
     <t>A time entry row whose end is not after its start is rejected.</t>
@@ -2026,7 +2026,7 @@
     <t>Message "Negative or zero-length intervals are not allowed."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.negative_interval; ResourceBundle.properties:679. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.negative_interval: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru).</t>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.negative_interval; ResourceBundle.properties:679. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.negative_interval: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. When start and end are both present and the end is not after the start, the negative-interval key is raised.</t>
   </si>
   <si>
     <t>Time entry rows whose intervals overlap are rejected.</t>
@@ -2038,10 +2038,10 @@
     <t>Message "Overlapping intervals are not allowed."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.overlapping_interval; ResourceBundle.properties:680. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.overlapping_interval: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru).</t>
-  </si>
-  <si>
-    <t>A time entry row with both a start/end interval and a duration is rejected.</t>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.overlapping_interval; ResourceBundle.properties:680. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.overlapping_interval: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow; SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#isOverlapping. WAR: classes byte-identical to the v1.1a4 release. Rows whose interval does not end before its start are compared with the earlier rows of the same form; an overlap raises the overlapping-interval key.</t>
+  </si>
+  <si>
+    <t>The last (new) time entry row is rejected when it has both a start/end interval and a duration; the other rows are not checked for this.</t>
   </si>
   <si>
     <t>Time is entered either as an interval or as a duration.</t>
@@ -2050,7 +2050,7 @@
     <t>Message "Cannot specify both an interval and duration."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.both_interval_and_duration; ResourceBundle.properties:682. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.both_interval_and_duration is missing in es. Bundles without the key fall back to the default text (framework behavior, GAP-011).</t>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.both_interval_and_duration; ResourceBundle.properties:682. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.both_interval_and_duration is missing in es. Bundles without the key fall back to the default text (framework behavior, GAP-011). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. The interval-and-duration check (#7) applies only to the last row; in other rows a start time, an end time and a duration together are accepted.</t>
   </si>
   <si>
     <t>A time entry row without a report date is rejected.</t>
@@ -2062,7 +2062,7 @@
     <t>Message "Missing reported date."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.missing_report_date; ResourceBundle.properties:683. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.missing_report_date is defined only in the default, "--", de, it, ja and ru bundles. Bundles without the key fall back to the default text (framework behavior, GAP-011).</t>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.missing_report_date; ResourceBundle.properties:683. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.missing_report_date is defined only in the default, "--", de, it, ja and ru bundles. Bundles without the key fall back to the default text (framework behavior, GAP-011). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. Every row except an empty last row and a deleted row needs a report date.</t>
   </si>
   <si>
     <t>A time entry description longer than the allowed maximum is rejected.</t>
@@ -2074,7 +2074,7 @@
     <t>Message "The time entry description is too long."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.long_description; ResourceBundle.properties:684; the description input carries maxlength TimeEditorForm.MAX_DESCRIPTION_LENGTH (WAR:WEB-INF/jsp/edit/editTimeEntries.jsp). Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.long_description: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru).</t>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.long_description; ResourceBundle.properties:684; the description input carries maxlength TimeEditorForm.MAX_DESCRIPTION_LENGTH (WAR:WEB-INF/jsp/edit/editTimeEntries.jsp). Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.long_description: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. A description longer than MAX_DESCRIPTION_LENGTH raises the long-description key.</t>
   </si>
   <si>
     <t>Re-estimate task (legacy page)</t>
@@ -2089,7 +2089,7 @@
     <t>Page reachable only by URL; the mapped action class is a plain Struts Action.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:130,301-302 (global forward edit/task/estimate; action /edit/task/estimate); WAR:WEB-INF/action-servlet.xml:298 (org.apache.struts.action.Action); WAR:WEB-INF/jsp/edit/editTaskEstimate.jsp (UPDATE_ESTIMATE); class UpdateTimeAction#doUpdateEstimateAction ("reestimated", "Estimate changed from "). No class references the forward (grep over class dumps). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editTaskEstimate.jsp writes the raw request parameters fkey (43), returnto (45), oid (48) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt.</t>
+    <t>WAR:WEB-INF/struts-config.xml:130,301-302 (global forward edit/task/estimate; action /edit/task/estimate); WAR:WEB-INF/action-servlet.xml:298 (org.apache.struts.action.Action); WAR:WEB-INF/jsp/edit/editTaskEstimate.jsp (UPDATE_ESTIMATE); class UpdateTimeAction#doUpdateEstimateAction ("reestimated", "Estimate changed from "). No class references the forward (grep over class dumps). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editTaskEstimate.jsp writes the raw request parameters fkey (43), returnto (45), oid (48) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#doUpdateEstimateAction. WAR: classes byte-identical to the v1.1a4 release. The estimate update and its history text exist, but the page's action mapping uses a plain Struts Action.</t>
   </si>
   <si>
     <t>Personal timesheet</t>
@@ -2104,7 +2104,7 @@
     <t>Summary table with total, daily table, and pie charts by project, iteration and story.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/person.jsp (link /do/view/timesheet); WAR:WEB-INF/struts-config.xml:374-378; class ViewTimesheetAction; WAR:calendar/calendar-i18n.jsp, WAR:calendar/calendar.js (date picker); WAR:WEB-INF/jsp/view/timesheet.jsp (cewolf charts personTimesheetProjectChart, ...IterationChart, ...StoryChart).</t>
+    <t>WAR:WEB-INF/jsp/view/person.jsp (link /do/view/timesheet); WAR:WEB-INF/struts-config.xml:374-378; class ViewTimesheetAction; WAR:calendar/calendar-i18n.jsp, WAR:calendar/calendar.js (date picker); WAR:WEB-INF/jsp/view/timesheet.jsp (cewolf charts personTimesheetProjectChart, ...IterationChart, ...StoryChart). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ViewTimesheetAction.java ViewTimesheetAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. The timesheet of the posted person and period is queried and shown.</t>
   </si>
   <si>
     <t>An unparsable period date is rejected.</t>
@@ -2113,7 +2113,7 @@
     <t>Message "Can't parse the supplied date value."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.PersonTimesheetForm#validate (timesheet.error.unparsable_date). Locale variants (CHK-004, BA-001-04): The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71).</t>
+    <t>class com.technoetic.xplanner.forms.PersonTimesheetForm#validate (timesheet.error.unparsable_date). Locale variants (CHK-004, BA-001-04): The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/PersonTimesheetForm.java PersonTimesheetForm#validate. WAR: classes byte-identical to the v1.1a4 release. An unparsable start or end date raises the unparsable-date key; the pattern comes from format.date in the request (Accept-Language) locale.</t>
   </si>
   <si>
     <t>The personal timesheet applies no permission filter: any signed-in user can open any person's timesheet by its oid.</t>
@@ -2125,7 +2125,7 @@
     <t>Timesheet of the requested person is shown to any signed-in user (runtime unverified).</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.actions.ViewTimesheetAction: no authorization call reachable (.migration-tmp/stage-01/out/authtrace.json); the "timesheet" link on WAR:WEB-INF/jsp/view/person.jsp is not permission-gated. BA-001-03 impact sweep of F-007.</t>
+    <t>class com.technoetic.xplanner.actions.ViewTimesheetAction: no authorization call reachable (.migration-tmp/stage-01/out/authtrace.json); the "timesheet" link on WAR:WEB-INF/jsp/view/person.jsp is not permission-gated. BA-001-03 impact sweep of F-007. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/ViewTimesheetAction.java ViewTimesheetAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. The action queries the timesheet of the posted person id with no authorizer call.</t>
   </si>
   <si>
     <t>Aggregate timesheet</t>
@@ -2140,10 +2140,10 @@
     <t>Multi-select of people, date range, summary tables and three pie charts.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/projects.jsp:164 (link /do/view/aggregateTimesheet); WAR:WEB-INF/struts-config.xml:380-384; class ViewAggregateTimesheetAction (HQL people.hidden = false order by name); WAR:WEB-INF/jsp/view/aggregateTimesheet.jsp. Request-value flow (BA-001-07, mechanism (b)): the posted selectedPeople values (AggregateTimesheetForm#setSelectedPeople, String[]) are passed to AggregateTimesheetQuery#setPersonIds; #getTimesheet appends each element unchanged into "AND person.id IN (...)", substitutes it for the placeholder "AND 1=1" with String#replaceAll and runs Session.iterate with only the two dates bound (bytecode listing). The query text is kept in a static field that each call re-initialises, so concurrent requests may share it (Inferred). AggregateTimesheetForm#validate checks only the dates. Mapping WAR:WEB-INF/struts-config.xml:380-384, any signed-in user. Exploitability is not established (static only). Observed risk only (Q3 deferred). Source: stage-02-pass-005 F-002.</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.forms.AggregateTimesheetForm#validate (timesheet.error.unparsable_date). Locale variants (CHK-004, BA-001-04): The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71).</t>
+    <t>WAR:WEB-INF/jsp/view/projects.jsp:164 (link /do/view/aggregateTimesheet); WAR:WEB-INF/struts-config.xml:380-384; class ViewAggregateTimesheetAction (HQL people.hidden = false order by name); WAR:WEB-INF/jsp/view/aggregateTimesheet.jsp. Request-value flow (BA-001-07, mechanism (b)): the posted selectedPeople values (AggregateTimesheetForm#setSelectedPeople, String[]) are passed to AggregateTimesheetQuery#setPersonIds; #getTimesheet appends each element unchanged into "AND person.id IN (...)", substitutes it for the placeholder "AND 1=1" with String#replaceAll and runs Session.iterate with only the two dates bound (bytecode listing). The query text is kept in a static field that each call re-initialises, so concurrent requests may share it (Inferred). AggregateTimesheetForm#validate checks only the dates. Mapping WAR:WEB-INF/struts-config.xml:380-384, any signed-in user. Exploitability is not established (static only). Observed risk only (Q3 deferred). Source: stage-02-pass-005 F-002. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/db/AggregateTimesheetQuery.java AggregateTimesheetQuery#getTimesheet. WAR: classes byte-identical to the v1.1a4 release. The query groups hours by project, iteration and story for the selected people and period.</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.AggregateTimesheetForm#validate (timesheet.error.unparsable_date). Locale variants (CHK-004, BA-001-04): The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/AggregateTimesheetForm.java AggregateTimesheetForm#validate. WAR: classes byte-identical to the v1.1a4 release. An unparsable date raises the unparsable-date key.</t>
   </si>
   <si>
     <t>The aggregate timesheet includes only hours on projects the viewing user may read.</t>
@@ -2155,7 +2155,7 @@
     <t>Rows and charts cover readable projects only.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.db.AggregateTimesheetQuery#getTimesheet (SystemAuthorizer.get, Authorizer.hasPermission with "system.project" and "read"); path ViewAggregateTimesheetAction#doExecute in .migration-tmp/stage-01/out/authtrace.json. Source: stage-02-pass-001 F-007.</t>
+    <t>class com.technoetic.xplanner.db.AggregateTimesheetQuery#getTimesheet (SystemAuthorizer.get, Authorizer.hasPermission with "system.project" and "read"); path ViewAggregateTimesheetAction#doExecute in .migration-tmp/stage-01/out/authtrace.json. Source: stage-02-pass-001 F-007. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/db/AggregateTimesheetQuery.java AggregateTimesheetQuery#getTimesheet. WAR: classes byte-identical to the v1.1a4 release. Each result row is added only when the viewing user has read permission on its project.</t>
   </si>
   <si>
     <t>UF-010</t>
@@ -2176,10 +2176,10 @@
     <t>Note editor (multipart form); after save the note appears in the Notes section of the object page.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/layout/viewLayout.jsp:114-116 (include view/notes.jsp in tiles:view pages); WAR:WEB-INF/jsp/view/notes.jsp:20-23 (isNoteEditor = hasPermission(..., "note", 0, "edit")) and link /do/edit/note?attachedToId=; WAR:WEB-INF/struts-config.xml:306-307; WAR:WEB-INF/action-servlet.xml:306-313 (EditNoteAction, virtualFileSystem); WAR:WEB-INF/jsp/edit/editNote.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request-value flow (BA-001-07, mechanism (b)): the note list included in these pages reads the oid request parameter (WAR:WEB-INF/jsp/view/notes.jsp:13, bean:parameter) and concatenates it into the useBeans where clause "attachedToId=" + oid (:14-15), which UseBeansTag#doEndTag appends into the HQL text; this is the same pattern as the time-log query of WAR:WEB-INF/jsp/view/task.jsp:101-103 (Q3 facts). Exploitability is not established (static only; observed risk only, Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editNote.jsp writes the raw request parameters oid (31), returnto (35,106), projectId (37), attachedToId (39), formFileName (82) [parameter (lines); line 106 passes returnto as the page attribute of html:link] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/note that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Note object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). EditNoteAction#populateObject calls the parent method before it stores the attachment. No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts).</t>
-  </si>
-  <si>
-    <t>A note without subject, author or body is rejected.</t>
+    <t>WAR:WEB-INF/jsp/layout/viewLayout.jsp:114-116 (include view/notes.jsp in tiles:view pages); WAR:WEB-INF/jsp/view/notes.jsp:20-23 (isNoteEditor = hasPermission(..., "note", 0, "edit")) and link /do/edit/note?attachedToId=; WAR:WEB-INF/struts-config.xml:306-307; WAR:WEB-INF/action-servlet.xml:306-313 (EditNoteAction, virtualFileSystem); WAR:WEB-INF/jsp/edit/editNote.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request-value flow (BA-001-07, mechanism (b)): the note list included in these pages reads the oid request parameter (WAR:WEB-INF/jsp/view/notes.jsp:13, bean:parameter) and concatenates it into the useBeans where clause "attachedToId=" + oid (:14-15), which UseBeansTag#doEndTag appends into the HQL text; this is the same pattern as the time-log query of WAR:WEB-INF/jsp/view/task.jsp:101-103 (Q3 facts). Exploitability is not established (static only; observed risk only, Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editNote.jsp writes the raw request parameters oid (31), returnto (35,106), projectId (37), attachedToId (39), formFileName (82) [parameter (lines); line 106 passes returnto as the page attribute of html:link] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/note that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Note object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). EditNoteAction#populateObject calls the parent method before it stores the attachment. No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/actions/EditNoteAction.java EditNoteAction#populateObject; SRC:src/com/technoetic/xplanner/tags/db/UseBeansTag.java UseBeansTag#doEndTag; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
+  </si>
+  <si>
+    <t>A note without subject or author is rejected; a note without body is rejected only when no file is attached.</t>
   </si>
   <si>
     <t>Notes must be meaningful and attributed.</t>
@@ -2188,7 +2188,7 @@
     <t>Messages "Missing subject.", "Missing author.", "Missing body."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.NoteEditorForm#validate (note.editor.missing_subject, missing_author, missing_body).</t>
+    <t>class com.technoetic.xplanner.forms.NoteEditorForm#validate (note.editor.missing_subject, missing_author, missing_body). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/forms/NoteEditorForm.java NoteEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release. Subject and author are always required, but the body only when no file is attached.</t>
   </si>
   <si>
     <t>Each note with an attachment shows the attachment name and a "References:" count, which is the number of notes that point to the same file.</t>
@@ -2200,7 +2200,7 @@
     <t>"Attachment" link and "References: &lt;n&gt;" on the note.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/notes.jsp:80-92 (link /do/download/attachment, notes.label.attachment.count, note.getAttachmentCount()); class net.sf.xplanner.domain.Note#getAttachmentCount runs "select note from Note note where note.file.id=" + file id and returns the list size (bytecode listing); label WAR:WEB-INF/classes/ResourceBundle.properties:545 ("References:"); DownloadAttachmentAction counts nothing. Label per bundle (CHK-004): "References:" in the default, "--" and ja bundles, "Referenzen:" in de; the other bundles have no key and fall back to the default. Corrected in BA-001-04 (Source: stage-02-pass-002 F-004).</t>
+    <t>WAR:WEB-INF/jsp/view/notes.jsp:80-92 (link /do/download/attachment, notes.label.attachment.count, note.getAttachmentCount()); class net.sf.xplanner.domain.Note#getAttachmentCount runs "select note from Note note where note.file.id=" + file id and returns the list size (bytecode listing); label WAR:WEB-INF/classes/ResourceBundle.properties:545 ("References:"); DownloadAttachmentAction counts nothing. Label per bundle (CHK-004): "References:" in the default, "--" and ja bundles, "Referenzen:" in de; the other bundles have no key and fall back to the default. Corrected in BA-001-04 (Source: stage-02-pass-002 F-004). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/net/sf/xplanner/domain/Note.java Note#getAttachmentCount. WAR: classes byte-identical to the v1.1a4 release. The count is the number of notes whose file id equals this note's file id.</t>
   </si>
   <si>
     <t>An uploaded attachment is stored in the application virtual file system under /attachments/project/&lt;projectId&gt;; the file bytes are kept in the database as a BLOB (table xfile, column data), and directories are rows of table xdir.</t>
@@ -2212,7 +2212,7 @@
     <t>Attachment readable via the download link; the first attachment of a project also creates the root directory and the /attachments/project/&lt;projectId&gt; directory rows (runtime unverified).</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.actions.EditNoteAction#populateObject (strings "/attachments/project/", "Saving note: filename="; calls FileSystem.getDirectory, FileSystem.createFile, Note.setFile); class com.technoetic.xplanner.file.FileSystemImpl#createFile (Hibernate.createBlob, File.setData); class net.sf.xplanner.domain.File field data (@Lob, @Column(name="data", length=1000000000)); WAR:WEB-INF/classes/spring-beans.xml:263 (virtualFileSystem FileSystemImpl); WAR:WEB-INF/classes/db-changelog.xml:234 (xfile.data LONGBLOB). Corrected in BA-001-03 (stage-02-pass-001 F-008). Directory creation on first use (BA-001-07, mechanism (c)): EditNoteAction#populateObject calls FileSystem#getDirectory("/attachments/project/&lt;id&gt;"); FileSystemImpl#getDirectory(String) calls #getRootDirectory, which saves, flushes and refreshes a new root Directory when none exists, and calls #createDirectory for each missing path segment (bytecode listings). The file system is wired into /edit/note explicitly (WAR:WEB-INF/action-servlet.xml:306-309). Source: stage-02-pass-005 F-005. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>class com.technoetic.xplanner.actions.EditNoteAction#populateObject (strings "/attachments/project/", "Saving note: filename="; calls FileSystem.getDirectory, FileSystem.createFile, Note.setFile); class com.technoetic.xplanner.file.FileSystemImpl#createFile (Hibernate.createBlob, File.setData); class net.sf.xplanner.domain.File field data (@Lob, @Column(name="data", length=1000000000)); WAR:WEB-INF/classes/spring-beans.xml:263 (virtualFileSystem FileSystemImpl); WAR:WEB-INF/classes/db-changelog.xml:234 (xfile.data LONGBLOB). Corrected in BA-001-03 (stage-02-pass-001 F-008). Directory creation on first use (BA-001-07, mechanism (c)): EditNoteAction#populateObject calls FileSystem#getDirectory("/attachments/project/&lt;id&gt;"); FileSystemImpl#getDirectory(String) calls #getRootDirectory, which saves, flushes and refreshes a new root Directory when none exists, and calls #createDirectory for each missing path segment (bytecode listings). The file system is wired into /edit/note explicitly (WAR:WEB-INF/action-servlet.xml:306-309). Source: stage-02-pass-005 F-005. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/EditNoteAction.java EditNoteAction#populateObject; SRC:src/com/technoetic/xplanner/file/FileSystemImpl.java FileSystemImpl#createFile. WAR: classes byte-identical to the v1.1a4 release. The file bytes are stored as a BLOB in a File row of the directory /attachments/project/&lt;projectId&gt; (the projectId request parameter, 0 when missing). Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
   </si>
   <si>
     <t>Edit and delete note</t>
@@ -2227,7 +2227,7 @@
     <t>Note editor pre-filled; changes saved.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/notes.jsp (isUserAuthorized note edit; link /do/edit/note). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 169 applies to every /do/edit/note request (Inferred; Q3 facts).</t>
+    <t>WAR:WEB-INF/jsp/view/notes.jsp (isUserAuthorized note edit; link /do/edit/note). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 169 applies to every /do/edit/note request (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>An authorized user can delete a note after confirming "Do you want to delete note &lt;subject&gt;".</t>
@@ -2239,7 +2239,7 @@
     <t>Confirm prompt; note removed; its attachment file removed too unless another note references it.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/notes.jsp (link /do/delete/note with confirm); WAR:WEB-INF/struts-config.xml:309; class com.technoetic.xplanner.actions.DeleteNoteAction#doExecute calls NoteHelper#deleteNote, which deletes the attached file only when no other note references it (query "select note from Note note where note.file.id= ?", size check), then the note (bytecode listing; BA-001-04 cascade sweep). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred).</t>
+    <t>WAR:WEB-INF/jsp/view/notes.jsp (link /do/delete/note with confirm); WAR:WEB-INF/struts-config.xml:309; class com.technoetic.xplanner.actions.DeleteNoteAction#doExecute calls NoteHelper#deleteNote, which deletes the attached file only when no other note references it (query "select note from Note note where note.file.id= ?", size check), then the note (bytecode listing; BA-001-04 cascade sweep). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/db/NoteHelper.java NoteHelper#deleteNote. WAR: classes byte-identical to the v1.1a4 release. The note is deleted, and its file only when no other note refers to it.</t>
   </si>
   <si>
     <t>Download attachment</t>
@@ -2254,7 +2254,7 @@
     <t>File streamed with Content-disposition filename.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/notes.jsp (link /do/download/attachment?oid=); WAR:WEB-INF/struts-config.xml:311; class com.technoetic.xplanner.actions.DownloadAttachmentAction (strings "Content-disposition", "note;filename=").</t>
+    <t>WAR:WEB-INF/jsp/view/notes.jsp (link /do/download/attachment?oid=); WAR:WEB-INF/struts-config.xml:311; class com.technoetic.xplanner.actions.DownloadAttachmentAction (strings "Content-disposition", "note;filename="). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DownloadAttachmentAction.java DownloadAttachmentAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. The file of the note is written to the response with its content type and name.</t>
   </si>
   <si>
     <t>File manager (directories)</t>
@@ -2269,7 +2269,7 @@
     <t>Pages reachable by URL only; every file-manager operation, including the default listing, is expected to fail with a null reference because the file system is never injected into the action (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:401-403; WAR:WEB-INF/action-servlet.xml:396 (FileManagerAction); WAR:WEB-INF/jsp/view/directory.jsp; class FileManagerAction#doExecute (actions list, upload, download, delete, mkdir, rmdir). Only self-links from directory.jsp were found (linkgraph.txt); entry is by URL. Delete cascade sweep (BA-001-04): class com.technoetic.xplanner.file.FileSystemImpl#deleteFile and #deleteDirectory run an HQL delete by id without cascading; net.sf.xplanner.domain.Directory maps files and subdirectories without cascade. The foreign keys WAR:WEB-INF/classes/db-changelog.xml:259 (note.attachment_id -&gt; xfile), :266 (xdir.parent_id -&gt; xdir) and :267 (xfile.dir_id -&gt; xdir) are expected to make the database reject deleting a file that a note references or a directory that is not empty (runtime unverified). Wiring and read-path writes (BA-001-07, mechanisms (a) and (c)): the bean /view/directory (WAR:WEB-INF/action-servlet.xml:396) has no properties; FileManagerAction#setFileSystem would need a bean named fileSystem, but the file system bean is named virtualFileSystem (WAR:WEB-INF/classes/spring-beans.xml:263; provenance P-05) and is wired explicitly only into /edit/note (action-servlet.xml:306-309). FileManagerAction#doExecute reads the field for every action (list, upload, download, delete, mkdir, rmdir), so the first call is expected to fail. The write-on-read of FileSystemImpl#getRootDirectory (it saves, flushes and refreshes a new root Directory when none exists) is therefore not expected to be reached from GET /do/view/directory. Corrected in BA-001-07 (Source: stage-02-pass-005 F-005, narrowed).</t>
+    <t>WAR:WEB-INF/struts-config.xml:401-403; WAR:WEB-INF/action-servlet.xml:396 (FileManagerAction); WAR:WEB-INF/jsp/view/directory.jsp; class FileManagerAction#doExecute (actions list, upload, download, delete, mkdir, rmdir). Only self-links from directory.jsp were found (linkgraph.txt); entry is by URL. Delete cascade sweep (BA-001-04): class com.technoetic.xplanner.file.FileSystemImpl#deleteFile and #deleteDirectory run an HQL delete by id without cascading; net.sf.xplanner.domain.Directory maps files and subdirectories without cascade. The foreign keys WAR:WEB-INF/classes/db-changelog.xml:259 (note.attachment_id -&gt; xfile), :266 (xdir.parent_id -&gt; xdir) and :267 (xfile.dir_id -&gt; xdir) are expected to make the database reject deleting a file that a note references or a directory that is not empty (runtime unverified). Wiring and read-path writes (BA-001-07, mechanisms (a) and (c)): the bean /view/directory (WAR:WEB-INF/action-servlet.xml:396) has no properties; FileManagerAction#setFileSystem would need a bean named fileSystem, but the file system bean is named virtualFileSystem (WAR:WEB-INF/classes/spring-beans.xml:263; provenance P-05) and is wired explicitly only into /edit/note (action-servlet.xml:306-309). FileManagerAction#doExecute reads the field for every action (list, upload, download, delete, mkdir, rmdir), so the first call is expected to fail. The write-on-read of FileSystemImpl#getRootDirectory (it saves, flushes and refreshes a new root Directory when none exists) is therefore not expected to be reached from GET /do/view/directory. Corrected in BA-001-07 (Source: stage-02-pass-005 F-005, narrowed). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/FileManagerAction.java FileManagerAction#doExecute, #setFileSystem. WAR: classes byte-identical to the v1.1a4 release. The setter has no annotation and no bean named fileSystem exists; the null-reference outcome is a runtime effect. Live question: Does /do/view/directory fail on the default listing?</t>
   </si>
   <si>
     <t>UF-011</t>
@@ -2290,7 +2290,7 @@
     <t>Results page "Search results - &lt;text&gt;" with type, ID, title (links to object or to the object a note is attached to) and match.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:22-35 (form /do/search/content, searchedContent, restrictToProjectId); WAR:WEB-INF/struts-config.xml:415-417; class ContentSearchAction (search.content.globalScopeEnable); WAR:WEB-INF/classes/xplanner.properties:287; WAR:WEB-INF/classes/spring-beans.xml:210-226; WAR:WEB-INF/jsp/view/searchResults.jsp. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:22-35 (form /do/search/content, searchedContent, restrictToProjectId); WAR:WEB-INF/struts-config.xml:415-417; class ContentSearchAction (search.content.globalScopeEnable); WAR:WEB-INF/classes/xplanner.properties:287; WAR:WEB-INF/classes/spring-beans.xml:210-226; WAR:WEB-INF/jsp/view/searchResults.jsp. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute. WAR: classes byte-identical to the v1.1a4 release; search.content.globalScopeEnable=true in the WAR xplanner.properties. With the global scope the whole database is searched; a numeric search text also adds the object with that id first (row 180). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
   </si>
   <si>
     <t>A search without results shows an empty-results message.</t>
@@ -2302,10 +2302,10 @@
     <t>Message empty.search.results.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/searchResults.jsp (empty.search.results).</t>
-  </si>
-  <si>
-    <t>Search results are filtered to objects the searching user may read; matches in unreadable projects are dropped.</t>
+    <t>WAR:WEB-INF/jsp/view/searchResults.jsp (empty.search.results). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+  </si>
+  <si>
+    <t>Text matches are filtered to objects the searching user may read; a numeric search text also puts the object with that id at the top of the results, without a read check.</t>
   </si>
   <si>
     <t>Search does not reveal items outside the user's permissions.</t>
@@ -2314,7 +2314,7 @@
     <t>Only readable matches are listed.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.db.ContentSearchHelper#search calls #excludeResultsBasedOnUserPermissions, which filters with #getAuthorizationPredicate -&gt; class com.technoetic.xplanner.actions.SearchResultAuthorizationPredicate#evaluate/#isResultReadableByUser (SystemAuthorizer.get, Authorizer.hasPermission, string "read"). Source: stage-02-pass-001 F-007.</t>
+    <t>class com.technoetic.xplanner.db.ContentSearchHelper#search calls #excludeResultsBasedOnUserPermissions, which filters with #getAuthorizationPredicate -&gt; class com.technoetic.xplanner.actions.SearchResultAuthorizationPredicate#evaluate/#isResultReadableByUser (SystemAuthorizer.get, Authorizer.hasPermission, string "read"). Source: stage-02-pass-001 F-007. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/db/ContentSearchHelper.java ContentSearchHelper#search, #excludeResultsBasedOnUserPermissions; SRC:src/com/technoetic/xplanner/actions/SearchResultAuthorizationPredicate.java SearchResultAuthorizationPredicate#isResultReadableByUser; SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute; SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search. WAR: classes byte-identical to the v1.1a4 release; search.content.globalScopeEnable=true in the WAR xplanner.properties. Text matches are filtered by read permission. After the filter, when the search text is a number and the scope is global (the WAR value), ContentSearchAction adds the object with that id at the top of the results without a permission check (bytecode listing agrees).</t>
   </si>
   <si>
     <t>Submitting an empty search yields an error.</t>
@@ -2323,25 +2323,25 @@
     <t>Guides the user to enter text.</t>
   </si>
   <si>
-    <t>Error "missing content" style message.</t>
-  </si>
-  <si>
-    <t>class ContentSearchAction#produceException (strings "missing content", "contentsearch.invalid_id").</t>
+    <t>General error page "Invalid content specified for search.: missing content" (text in the Accept-Language locale; bundles without contentsearch.invalid_id fall back to the default text).</t>
+  </si>
+  <si>
+    <t>class ContentSearchAction#produceException (strings "missing content", "contentsearch.invalid_id"). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute, #produceException. WAR: classes byte-identical to the v1.1a4 release. An empty search text forwards to the general error page with the message of contentsearch.invalid_id followed by ": missing content", resolved in the request (Accept-Language) locale; the key is missing in da, es, fr, it, pt_br and ru.</t>
   </si>
   <si>
     <t>Jump to object by ID</t>
   </si>
   <si>
-    <t>Searching by numeric ID opens the matching project, iteration, story, task or note directly.</t>
+    <t>Searching by a numeric ID in the header search lists the matching project, iteration, story, task, person or note first among the results; the direct jump (/do/search/id) is reachable by URL only.</t>
   </si>
   <si>
     <t>Direct navigation by ID ("search by word or ID").</t>
   </si>
   <si>
-    <t>Browser redirected to /do/view/&lt;type&gt;?oid=&lt;id&gt;.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:46 (tooltip "search by word or ID"); class ContentSearchAction (setIdSearchHelper); class IdSearchAction (strings "/do/view/", "?oid="); WAR:WEB-INF/struts-config.xml:141,413 (search/id).</t>
+    <t>Search results headed by the object with that id; a request to /do/search/id?searchedId=&lt;id&gt; redirects to /do/view/&lt;type&gt;?oid=&lt;id&gt;.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:46 (tooltip "search by word or ID"); class ContentSearchAction (setIdSearchHelper); class IdSearchAction (strings "/do/view/", "?oid="); WAR:WEB-INF/struts-config.xml:141,413 (search/id). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute; SRC:src/com/technoetic/xplanner/actions/IdSearchAction.java IdSearchAction#doExecute. WAR: classes byte-identical to the v1.1a4 release; baseHeader.jsp of the WAR (differs from the SVN copy; WAR governs). The header search box posts to /do/search/content: a numeric text lists the object with that id first among the search results, without a redirect. The redirecting ID search (/do/search/id, IdSearchAction) is linked from no page of the WAR.</t>
   </si>
   <si>
     <t>A missing, malformed or unknown ID shows an error.</t>
@@ -2353,7 +2353,7 @@
     <t>Messages idsearch.error.missingId, badId, idNotFound.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.actions.IdSearchAction#doExecute (idsearch.error.missingId, idsearch.error.badId, idsearch.error.idNotFound).</t>
+    <t>class com.technoetic.xplanner.actions.IdSearchAction#doExecute (idsearch.error.missingId, idsearch.error.badId, idsearch.error.idNotFound). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/IdSearchAction.java IdSearchAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. An empty, non-numeric or unknown id returns the general error forward with the three keys; they exist only in the default and "--" bundles.</t>
   </si>
   <si>
     <t>Jumping by ID applies no read-permission check, unlike text search; the target view page does not check either.</t>
@@ -2365,7 +2365,7 @@
     <t>Any existing object ID opens its page for any signed-in user (runtime unverified).</t>
   </si>
   <si>
-    <t>classes IdSearchAction and ViewObjectAction: no authorization call reachable (.migration-tmp/stage-01/out/authtrace.json). BA-001-03 impact sweep of F-001 and F-007.</t>
+    <t>classes IdSearchAction and ViewObjectAction: no authorization call reachable (.migration-tmp/stage-01/out/authtrace.json). BA-001-03 impact sweep of F-001 and F-007. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/IdSearchAction.java IdSearchAction#doExecute; SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search; SRC:src/com/technoetic/xplanner/actions/ViewObjectAction.java ViewObjectAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. Neither the ID search nor the view action calls an authorizer.</t>
   </si>
   <si>
     <t>Breadcrumb navigation</t>
@@ -2380,7 +2380,7 @@
     <t>Breadcrumb links above the page content.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/tags/breadcrumb.tag; class net.sf.xplanner.tags.NavigationBarTag#render (strings "navigation.top", project, iteration, userstory, task, feature); layouts viewLayout.jsp:59, defaultLayout.jsp:44, defaultEditLayout.jsp:55. Request-driven lookup (BA-001-10, pass-008 F-002 lead, check (l)): NavigationBarTag#doEndTag reads the request parameter oid, or else fkey. Because breadcrumb.tag passes type="${objectType}", which is an empty string when the attribute is unset, #setObject(int) looks the id up with IdSearchHelper#search (Session#get over Project, Iteration, UserStory, Task, Person and Note; WAR:WEB-INF/classes/spring-dao.xml:61) and applies no permission check. The link texts are the stored names of the hierarchy and are printed with unescaped EL (WAR:WEB-INF/tags/breadcrumb.tag:15,18). On signed-in pages this adds no exposure beyond the missing read checks (rows 29-30); on the public login and error pages it runs before sign-in (rows 8, 56; Inferred; GAP-007; Q3 facts).</t>
+    <t>WAR:WEB-INF/tags/breadcrumb.tag; class net.sf.xplanner.tags.NavigationBarTag#render (strings "navigation.top", project, iteration, userstory, task, feature); layouts viewLayout.jsp:59, defaultLayout.jsp:44, defaultEditLayout.jsp:55. Request-driven lookup (BA-001-10, pass-008 F-002 lead, check (l)): NavigationBarTag#doEndTag reads the request parameter oid, or else fkey. Because breadcrumb.tag passes type="${objectType}", which is an empty string when the attribute is unset, #setObject(int) looks the id up with IdSearchHelper#search (Session#get over Project, Iteration, UserStory, Task, Person and Note; WAR:WEB-INF/classes/spring-dao.xml:61) and applies no permission check. The link texts are the stored names of the hierarchy and are printed with unescaped EL (WAR:WEB-INF/tags/breadcrumb.tag:15,18). On signed-in pages this adds no exposure beyond the missing read checks (rows 29-30); on the public login and error pages it runs before sign-in (rows 8, 56; Inferred; GAP-007; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/net/sf/xplanner/tags/NavigationBarTag.java NavigationBarTag#render, #doEndTag; SRC:src/com/technoetic/xplanner/tags/NavigationBarTag.java NavigationBarTag#doEndTag; SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
   </si>
   <si>
     <t>Object and project history</t>
@@ -2392,10 +2392,10 @@
     <t>Audit trail of recorded changes.</t>
   </si>
   <si>
-    <t>Sortable history table; the container view adds object type and name links.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/project.jsp:99-104, iteration/globalLinks.jsp:41-45, userstory.jsp, task.jsp (links /do/view/history, container flag for projects); WAR:WEB-INF/struts-config.xml:396-398; WAR:WEB-INF/jsp/view/history.jsp:30-32 (HistorySupport#getEvents) and :71-73 (#getContainerEvents); class com.technoetic.xplanner.history.HistorySupport#getContainerEvents (strings "created", "deleted"); WAR:WEB-INF/classes/spring-dao.xml:63-65 (historySupport); db-changelog.xml table history. Corrected in BA-001-03 (stage-02-pass-001 F-002).</t>
+    <t>Sortable history table; the container view adds object type and name links. The "when" dates use the built-in pattern "EEE MMM dd k:mm:ss z" in the Accept-Language locale of the first request after start-up, for every later user (Inferred).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/project.jsp:99-104, iteration/globalLinks.jsp:41-45, userstory.jsp, task.jsp (links /do/view/history, container flag for projects); WAR:WEB-INF/struts-config.xml:396-398; WAR:WEB-INF/jsp/view/history.jsp:30-32 (HistorySupport#getEvents) and :71-73 (#getContainerEvents); class com.technoetic.xplanner.history.HistorySupport#getContainerEvents (strings "created", "deleted"); WAR:WEB-INF/classes/spring-dao.xml:63-65 (historySupport); db-changelog.xml table history. Corrected in BA-001-03 (stage-02-pass-001 F-002). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/history/HistorySupport.java HistorySupport#getEvents, #getContainerEvents; SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag. WAR: classes byte-identical to the v1.1a4 release; history.jsp of the WAR (differs from the SVN copy, which calls HistorySupport statically; the WAR page calls the historySupport bean; WAR governs). The "when" column (history.jsp:61,106) uses xplanner:formatDate without format or formatKey: FormatDateTag uses its built-in pattern "EEE MMM dd k:mm:ss z" and keeps one SimpleDateFormat per pattern in a static, unsynchronized map, created with request.getLocale() (Accept-Language) of the first request after start-up, so later users see day and month names in that first locale (bytecode listing agrees). Resolves carried pass-009 F-002 statically (Inferred for the runtime effect). Live question: After a fresh start, which language do the history dates show for a second session with a different Accept-Language?</t>
   </si>
   <si>
     <t>History is written only by these entry points: web iteration start and close, story move/continue (including multi-move and continue unfinished stories), task move/continue and task re-estimate; and every SOAP add, update and remove ("created", "updated", "deleted"). Web create, edit and delete of projects, iterations, stories, tasks, notes, people and settings write no history.</t>
@@ -2407,7 +2407,7 @@
     <t>No history entry after a web edit or delete (runtime unverified).</t>
   </si>
   <si>
-    <t>Callers of com.technoetic.xplanner.history.HistorySupport#saveEvent reachable per entry point in .migration-tmp/stage-01/out/authtrace.json: StartIterationAction, CloseIterationAction, MoveContinueStoryAction, MoveStoriesAction and ContinueUnfinishedStoriesAction (via MoveContinueStory and Continuer), MoveContinueTaskAction, UpdateTimeAction#doUpdateEstimateAction ("reestimated"), SOAP XPlanner#addObject/#updateObject/#removeObject (#saveHistory; strings "created", "updated", "deleted"); none from EditObjectAction or DeleteObjectAction, which only publish events that no registered listener receives. Source: stage-02-pass-001 F-002.</t>
+    <t>Callers of com.technoetic.xplanner.history.HistorySupport#saveEvent reachable per entry point in .migration-tmp/stage-01/out/authtrace.json: StartIterationAction, CloseIterationAction, MoveContinueStoryAction, MoveStoriesAction and ContinueUnfinishedStoriesAction (via MoveContinueStory and Continuer), MoveContinueTaskAction, UpdateTimeAction#doUpdateEstimateAction ("reestimated"), SOAP XPlanner#addObject/#updateObject/#removeObject (#saveHistory; strings "created", "updated", "deleted"); none from EditObjectAction or DeleteObjectAction, which only publish events that no registered listener receives. Source: stage-02-pass-001 F-002. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/history/HistorySupport.java HistorySupport#saveEvent (callers: StartIterationAction, CloseIterationAction, Continuer, MoveContinueStory, MoveContinueTaskAction, UpdateTimeAction, soap/XPlanner); SRC:src/net/sf/xplanner/events/EventManager.java EventManager (publishes Spring application events); SRC:src/net/sf/xplanner/email/EmailPerChangeListener.java (the only ApplicationListener; no bean). WAR: classes byte-identical to the v1.1a4 release. The source callers of saveEvent are exactly the recorded entry points; the generic web edit and delete only publish events, and no listener bean receives them.</t>
   </si>
   <si>
     <t>My status page</t>
@@ -2422,7 +2422,7 @@
     <t>Page /setting/me/status/&lt;personId&gt; with the same sections as the person page.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:17 (link ${appUrl}/setting/me/status/${person.id}); class net.sf.xplanner.web.MePage (@RequestMapping "/me/status/{id}", view "view/meStatus"); WAR:WEB-INF/jsp/view/meStatus.jsp; WAR:WEB-INF/classes/spring-web.xml. The link base appUrl comes from xplanner.application.url (class net.sf.xplanner.context.ContextLoaderListener; effective value http://localhost:8080/xplanner in xplanner-custom.properties:30), so the link target depends on that configured URL. Provenance (fixed baseline, see reconnaissance GAP-005): P-04: the cited value is read from xplanner-custom.properties (rewritten entry, known patch target); upstream value not determinable.</t>
+    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:17 (link ${appUrl}/setting/me/status/${person.id}); class net.sf.xplanner.web.MePage (@RequestMapping "/me/status/{id}", view "view/meStatus"); WAR:WEB-INF/jsp/view/meStatus.jsp; WAR:WEB-INF/classes/spring-web.xml. The link base appUrl comes from xplanner.application.url (class net.sf.xplanner.context.ContextLoaderListener; effective value http://localhost:8080/xplanner in xplanner-custom.properties:30), so the link target depends on that configured URL. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/net/sf/xplanner/web/MePage.java MePage. WAR: classes byte-identical to the v1.1a4 release; baseHeader.jsp of the WAR links through xplanner:link with the application URL (the SVN copy uses html:link; WAR governs). The controller is component-scanned with its DAO and repository fields autowired. Provenance (fixed baseline, see reconnaissance GAP-005): P-04: the cited value is read from xplanner-custom.properties (rewritten entry, known patch target); upstream value not determinable.</t>
   </si>
   <si>
     <t>Wiki-style formatting of descriptions</t>
@@ -2437,7 +2437,7 @@
     <t>Formatted HTML with links; bracket escaping can be enabled per project.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/xplanner.tld (twiki -&gt; com.technoetic.xplanner.tags.TwikiTag); WAR:WEB-INF/classes/xplanner.properties:92-127 (twiki.scheme.*, GenericWikiAdapter); package com.technoetic.xplanner.wiki (11 classes). Server-side request (BA-001-06): TwikiTag builds com.technoetic.xplanner.wiki.TwikiFormat, which instantiates the adapter class named by twiki.wikiadapter (WAR:WEB-INF/classes/xplanner.properties:113, GenericWikiAdapter) and calls ExternalWikiAdapter#formatWikiWord for each WikiWord; GenericWikiAdapter#formatWikiWord calls #isTopicExisting, which opens new URL(topic.url.existing with the word).openStream() (:114, http://localhost:9090/vqw/...) and reads it; no connect or read timeout is set. Existing topics are cached; an IOException returns false, so the word is rendered as a new-topic link and is requested again on the next rendering (bytecode listing with exception table). Rendering a description with a WikiWord is therefore expected to make an outbound HTTP request and to wait for it (runtime unverified). Provenance of the URL: GAP-005 P-03. Source: stage-02-pass-004 F-006. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/xplanner.tld (twiki -&gt; com.technoetic.xplanner.tags.TwikiTag); WAR:WEB-INF/classes/xplanner.properties:92-127 (twiki.scheme.*, GenericWikiAdapter); package com.technoetic.xplanner.wiki (11 classes). Server-side request (BA-001-06): TwikiTag builds com.technoetic.xplanner.wiki.TwikiFormat, which instantiates the adapter class named by twiki.wikiadapter (WAR:WEB-INF/classes/xplanner.properties:113, GenericWikiAdapter) and calls ExternalWikiAdapter#formatWikiWord for each WikiWord; GenericWikiAdapter#formatWikiWord calls #isTopicExisting, which opens new URL(topic.url.existing with the word).openStream() (:114, http://localhost:9090/vqw/...) and reads it; no connect or read timeout is set. Existing topics are cached; an IOException returns false, so the word is rendered as a new-topic link and is requested again on the next rendering (bytecode listing with exception table). Rendering a description with a WikiWord is therefore expected to make an outbound HTTP request and to wait for it (runtime unverified). Provenance of the URL: GAP-005 P-03. Source: stage-02-pass-004 F-006. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/tags/TwikiTag.java TwikiTag; SRC:src/com/technoetic/xplanner/wiki/TwikiFormat.java TwikiFormat#format; SRC:src/com/technoetic/xplanner/wiki/GenericWikiAdapter.java GenericWikiAdapter#formatWikiWord. WAR: classes byte-identical to the v1.1a4 release; wiki settings from the patched WAR xplanner.properties. The rendering path is as recorded; the result of the many format rules and of the external wiki lookup is not established without rendering. Live question: How are a description with TWiki markup, a WikiWord and an object link (story:&lt;id&gt;) rendered? Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
   </si>
   <si>
     <t>Editors show a formatting-help link to a TWiki formatting reference page.</t>
@@ -2449,7 +2449,7 @@
     <t>Help page describing the markup.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/common/formattingHelpLink.jsp (hard-coded /xplanner/do/view/twikiformat, which does not match the WAR context path /xplanner-plus in META-INF/context.xml); WAR:WEB-INF/struts-config.xml:177; WAR:WEB-INF/jsp/view/twikiformat.jsp.</t>
+    <t>WAR:WEB-INF/jsp/common/formattingHelpLink.jsp (hard-coded /xplanner/do/view/twikiformat, which does not match the WAR context path /xplanner-plus in META-INF/context.xml); WAR:WEB-INF/struts-config.xml:177; WAR:WEB-INF/jsp/view/twikiformat.jsp. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: JSP and descriptor fact. WAR: formattingHelpLink.jsp and META-INF/context.xml identical to the SVN webapp copies. The link hard-codes /xplanner while the context path is /xplanner-plus.</t>
   </si>
   <si>
     <t>Switch page width</t>
@@ -2464,7 +2464,7 @@
     <t>Page toggles between normal and wide layout; preference persists across pages via browser localStorage.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/common/footer.jsp:11-14 (page_footer, wider.png, label); WAR:js/global.js:1-10 (click on .page_footer toggles class wide, localStorage.widescreen); included by layouts defaultLayout.jsp:41 and defaultEditLayout.jsp:52.</t>
+    <t>WAR:WEB-INF/jsp/common/footer.jsp:11-14 (page_footer, wider.png, label); WAR:js/global.js:1-10 (click on .page_footer toggles class wide, localStorage.widescreen); included by layouts defaultLayout.jsp:41 and defaultEditLayout.jsp:52. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Any page built with the xplanner:content tag is rendered with the print layout (no header, no footer) when the request carries a print parameter, for example ?print=true; no page links to this mode, so it is reachable by URL only.</t>
@@ -2476,7 +2476,7 @@
     <t>Page body without the header and footer tiles.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.tags.ContentTag#doStartTag calls PrintLinkTag#isInPrintMode, which returns true when ServletRequest.getParameter("print") is not null, and then inserts the Tiles definition "tiles:print" (bytecode listings); WAR:WEB-INF/tiles-definitions.xml:23-28 (tiles:print extends tiles:view with displayMode print and empty header and footer). xplanner:content has 43 live opening tags in 43 JSPs (comment-blanked count); the printLink tag (WAR:WEB-INF/xplanner.tld:707-708) is used by no JSP. Request-parameter sweep of all tag classes (.migration-tmp/stage-01/out/render-side-effects-06.txt): print is the only parameter that switches the layout. Source: stage-02-pass-004 F-004. Related switch (BA-001-07, mechanism (b)): the Spring MVC Tiles definition viewLayout (WAR:WEB-INF/tiles-pages.xml:6) uses WAR:WEB-INF/jsp/layout/viewLayoutNew.jsp, which compares ${param.mode} with print (:15) and then omits the sections guarded by isScreenMode (:47, :84, :93); the value is compared only, not written.</t>
+    <t>class com.technoetic.xplanner.tags.ContentTag#doStartTag calls PrintLinkTag#isInPrintMode, which returns true when ServletRequest.getParameter("print") is not null, and then inserts the Tiles definition "tiles:print" (bytecode listings); WAR:WEB-INF/tiles-definitions.xml:23-28 (tiles:print extends tiles:view with displayMode print and empty header and footer). xplanner:content has 43 live opening tags in 43 JSPs (comment-blanked count); the printLink tag (WAR:WEB-INF/xplanner.tld:707-708) is used by no JSP. Request-parameter sweep of all tag classes (.migration-tmp/stage-01/out/render-side-effects-06.txt): print is the only parameter that switches the layout. Source: stage-02-pass-004 F-004. Related switch (BA-001-07, mechanism (b)): the Spring MVC Tiles definition viewLayout (WAR:WEB-INF/tiles-pages.xml:6) uses WAR:WEB-INF/jsp/layout/viewLayoutNew.jsp, which compares ${param.mode} with print (:15) and then omits the sections guarded by isScreenMode (:47, :84, :93); the value is compared only, not written. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/tags/ContentTag.java ContentTag#doStartTag; SRC:src/com/technoetic/xplanner/tags/PrintLinkTag.java PrintLinkTag#isInPrintMode. WAR: classes byte-identical to the v1.1a4 release. Any non-null print parameter selects tiles:print; otherwise a missing definition becomes tiles:default and a caller-given one is kept.</t>
   </si>
   <si>
     <t>Share on social networks</t>
@@ -2491,7 +2491,7 @@
     <t>Twitter and Facebook share icons open the external sites; no like widget, no LinkedIn link.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/layout/viewLayout.jsp:73-88 (twitter.com/home?status=..., facebook.com/dialog/feed with app_id and page URL) and :92-95 (HTML comment "&lt;!-- a class=\"in\" ... &lt;/span --&gt;" enclosing the LinkedIn link, the connect.facebook.net script and fb:like); the same comment in WAR:WEB-INF/jsp/layout/viewLayoutNew.jsp:114-117. Corrected in BA-001-04 (Source: stage-02-pass-002 F-003).</t>
+    <t>WAR:WEB-INF/jsp/layout/viewLayout.jsp:73-88 (twitter.com/home?status=..., facebook.com/dialog/feed with app_id and page URL) and :92-95 (HTML comment "&lt;!-- a class=\"in\" ... &lt;/span --&gt;" enclosing the LinkedIn link, the connect.facebook.net script and fb:like); the same comment in WAR:WEB-INF/jsp/layout/viewLayoutNew.jsp:114-117. Corrected in BA-001-04 (Source: stage-02-pass-002 F-003). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Features (story features)</t>
@@ -2506,7 +2506,7 @@
     <t>Pages reachable only by URL; runtime behaviour expected to fail.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:185-187,207-209,215-217,259-263; WAR:WEB-INF/action-servlet.xml:96-100,202-212 (type net.sf.xplanner.domain.Feature - class ABSENT from WAR); class com.technoetic.xplanner.domain.Feature has no @Entity; WAR:WEB-INF/classes/mappings/Feature.xml not loaded (spring-beans.xml:80 loads only Metrics.xml); iteration/links.jsp:32-35 commented; pages WAR:WEB-INF/jsp/view/projectFeatures.jsp, WAR:WEB-INF/jsp/view/iterationFeatures.jsp, WAR:WEB-INF/jsp/view/feature.jsp (uses com.technoetic.xplanner.domain.Feature), WAR:WEB-INF/jsp/edit/editFeature.jsp; class FeatureEditorForm#validate (feature.editor.missing_name). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editFeature.jsp writes the raw request parameters oid (29), returnto (32), fkey (34,35) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the "not mapped" conclusion rests on spring-beans.xml:80 (rewritten entry) and is corroborated independently by the compiled class com.technoetic.xplanner.db.hibernate.HibernateHelper, whose mapped-class list also omits this class.</t>
+    <t>WAR:WEB-INF/struts-config.xml:185-187,207-209,215-217,259-263; WAR:WEB-INF/action-servlet.xml:96-100,202-212 (type net.sf.xplanner.domain.Feature - class ABSENT from WAR); class com.technoetic.xplanner.domain.Feature has no @Entity; WAR:WEB-INF/classes/mappings/Feature.xml not loaded (spring-beans.xml:80 loads only Metrics.xml); iteration/links.jsp:32-35 commented; pages WAR:WEB-INF/jsp/view/projectFeatures.jsp, WAR:WEB-INF/jsp/view/iterationFeatures.jsp, WAR:WEB-INF/jsp/view/feature.jsp (uses com.technoetic.xplanner.domain.Feature), WAR:WEB-INF/jsp/edit/editFeature.jsp; class FeatureEditorForm#validate (feature.editor.missing_name). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editFeature.jsp writes the raw request parameters oid (29), returnto (32), fkey (34,35) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/domain/Feature.java Feature (no @Entity); SRC:src/com/technoetic/xplanner/forms/FeatureEditorForm.java FeatureEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release; net.sf.xplanner.domain.Feature absent from both the WAR and the SVN source. The type named by the action beans does not exist in the source either, and the old Feature class is not mapped. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the "not mapped" conclusion rests on spring-beans.xml:80 (rewritten entry) and is corroborated independently by the compiled class com.technoetic.xplanner.db.hibernate.HibernateHelper, whose mapped-class list also omits this class.</t>
   </si>
   <si>
     <t>UF-012</t>
@@ -2527,7 +2527,7 @@
     <t>Integration page with Start/Finished/Cancel buttons and a join form.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:388-394; WAR:WEB-INF/action-servlet.xml:390-392; WAR:WEB-INF/jsp/view/integrations.jsp; class com.technoetic.xplanner.actions.IntegrationAction (action.join, action.start, action.finish, action.cancel, action.leave). The used class com.technoetic.xplanner.domain.Integration has no @Entity and mappings/Integration.xml is not loaded; no live link to /do/view/integrations found. Server-side enforcement (CHK-002, BA-001-04): the view (DispatchForward) requires a projectId and system.project read (row 28); the join/start/finish/cancel/leave requests (IntegrationAction) perform no server-side permission check that gates the change (the only authorization call on the path is the recipient lookup inside the e-mail notifier), and the "integrate" condition only hides the buttons. Query property paths (BA-001-05): IntegrationAction#getIntegrationsInState and the three useBeans tags of WAR:WEB-INF/jsp/view/integrations.jsp (lines 23, 29, 155) query com.technoetic.xplanner.domain.Integration, which is not a mapped entity (GAP-004). Sweep of pass-003 F-001. Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/view/integrations.jsp writes the raw request parameters projectId (36) [parameter (lines); lines 26, 32 and 160 bind it as a query parameter] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the "not mapped" conclusion rests on spring-beans.xml:80 (rewritten entry) and is corroborated independently by the compiled class com.technoetic.xplanner.db.hibernate.HibernateHelper, whose mapped-class list also omits this class.</t>
+    <t>WAR:WEB-INF/struts-config.xml:388-394; WAR:WEB-INF/action-servlet.xml:390-392; WAR:WEB-INF/jsp/view/integrations.jsp; class com.technoetic.xplanner.actions.IntegrationAction (action.join, action.start, action.finish, action.cancel, action.leave). The used class com.technoetic.xplanner.domain.Integration has no @Entity and mappings/Integration.xml is not loaded; no live link to /do/view/integrations found. Server-side enforcement (CHK-002, BA-001-04): the view (DispatchForward) requires a projectId and system.project read (row 28); the join/start/finish/cancel/leave requests (IntegrationAction) perform no server-side permission check that gates the change (the only authorization call on the path is the recipient lookup inside the e-mail notifier), and the "integrate" condition only hides the buttons. Query property paths (BA-001-05): IntegrationAction#getIntegrationsInState and the three useBeans tags of WAR:WEB-INF/jsp/view/integrations.jsp (lines 23, 29, 155) query com.technoetic.xplanner.domain.Integration, which is not a mapped entity (GAP-004). Sweep of pass-003 F-001. Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/view/integrations.jsp writes the raw request parameters projectId (36) [parameter (lines); lines 26, 32 and 160 bind it as a query parameter] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/domain/Integration.java Integration (no @Entity); SRC:src/com/technoetic/xplanner/actions/IntegrationAction.java IntegrationAction#onJoinRequest, #onStartRequest. WAR: classes byte-identical to the v1.1a4 release; src/mappings/Integration.xml exists in the source but is not loaded by the WAR spring-beans.xml. The page and actions exist; the entity is neither annotated nor mapped by a loaded file. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the "not mapped" conclusion rests on spring-beans.xml:80 (rewritten entry) and is corroborated independently by the compiled class com.technoetic.xplanner.db.hibernate.HibernateHelper, whose mapped-class list also omits this class.</t>
   </si>
   <si>
     <t>Joining without selecting a person or starting while another integration is active shows an error.</t>
@@ -2539,7 +2539,7 @@
     <t>Messages integrations.error.noperson / integrations.error.alreadyactive.</t>
   </si>
   <si>
-    <t>class IntegrationAction#onJoinRequest ("integrations.error.noperson"), #onStartRequest ("integrations.error.alreadyactive").</t>
+    <t>class IntegrationAction#onJoinRequest ("integrations.error.noperson"), #onStartRequest ("integrations.error.alreadyactive"). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/IntegrationAction.java IntegrationAction#onJoinRequest, #onStartRequest. WAR: classes byte-identical to the v1.1a4 release. A join without a person (empty or "0") and a start while an integration is active return the error forward with the two keys.</t>
   </si>
   <si>
     <t>Integration events notify listeners; the configured listener sends e-mail (suppressed with a nonotify parameter).</t>
@@ -2551,7 +2551,7 @@
     <t>E-mail on integration events.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/xplanner.properties:86-87 (xplanner.integration.listeners=IntegrationEmailNotifier); class IntegrationAction#init/#fireIntegrationEvent/#isNotificationEnabled ("nonotify"). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/classes/xplanner.properties:86-87 (xplanner.integration.listeners=IntegrationEmailNotifier); class IntegrationAction#init/#fireIntegrationEvent/#isNotificationEnabled ("nonotify"). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/IntegrationAction.java IntegrationAction#init, #fireIntegrationEvent, #isNotificationEnabled; SRC:src/com/technoetic/xplanner/actions/IntegrationEmailNotifier.java IntegrationEmailNotifier. WAR: classes byte-identical to the v1.1a4 release; listener list from the patched WAR xplanner.properties. The listeners named in the property are instantiated with Class.forName (not by Spring) and receive every event; the e-mail itself depends on SMTP. Live question: Is an e-mail sent when an integration is joined and started, and suppressed with nonotify? Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
   </si>
   <si>
     <t>UF-013</t>
@@ -2572,7 +2572,7 @@
     <t>E-mail "XPlanner time entry reminder." listing tasks.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/spring-beans.xml:362-367 (task:scheduled missingTimeEntryNotifier execute cron "0 5 0 * * *"); class com.technoetic.xplanner.mail.MissingTimeEntryNotifier#execute/#sendMissingTimeEntryReminderToAcceptors; ResourceBundle.properties job.emailnotifier.subjectForAcceptors; mappings/Metrics.xml TimeEntryEmailNotificationToAcceptors. Loading (BA-001-05): the task:scheduled registration sits in spring-beans.xml, which both Spring contexts load (row 65), so two schedulers are expected to run the job, and each acceptor is expected to receive the reminder twice (Inferred, runtime unverified). Source: stage-02-pass-003 F-002. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>WAR:WEB-INF/classes/spring-beans.xml:362-367 (task:scheduled missingTimeEntryNotifier execute cron "0 5 0 * * *"); class com.technoetic.xplanner.mail.MissingTimeEntryNotifier#execute/#sendMissingTimeEntryReminderToAcceptors; ResourceBundle.properties job.emailnotifier.subjectForAcceptors; mappings/Metrics.xml TimeEntryEmailNotificationToAcceptors. Loading (BA-001-05): the task:scheduled registration sits in spring-beans.xml, which both Spring contexts load (row 65), so two schedulers are expected to run the job, and each acceptor is expected to receive the reminder twice (Inferred, runtime unverified). Source: stage-02-pass-003 F-002. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/mail/MissingTimeEntryNotifier.java MissingTimeEntryNotifier#execute, #sendMissingTimeEntryReminderToAcceptors. WAR: classes byte-identical to the v1.1a4 release; patched spring-beans.xml (WAR governs). The cut-off is hard-coded to the previous midnight; the schedule, the double registration and the delivery are runtime effects. Live question: At 00:05, are reminders sent, and are they sent twice? Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
   </si>
   <si>
     <t>The same job e-mails project notification receivers listing people who may have forgotten to enter time the previous working day.</t>
@@ -2584,7 +2584,7 @@
     <t>E-mail "XPlanner project time entry status."</t>
   </si>
   <si>
-    <t>class MissingTimeEntryNotifier#sendMissingTimeEntryReportToLeads; ResourceBundle.properties job.emailnotifier.subjectForProjectLeeds, bodyheaderForProjectLeeds; mappings/Metrics.xml TimeEntryEmailNotificationToProjectSpecificLeads; project option sendemail (editProject.jsp). Loading (BA-001-05): because the job is registered in both Spring contexts (row 65), receivers are expected to get the report twice (Inferred, runtime unverified). Source: stage-02-pass-003 F-002.</t>
+    <t>class MissingTimeEntryNotifier#sendMissingTimeEntryReportToLeads; ResourceBundle.properties job.emailnotifier.subjectForProjectLeeds, bodyheaderForProjectLeeds; mappings/Metrics.xml TimeEntryEmailNotificationToProjectSpecificLeads; project option sendemail (editProject.jsp). Loading (BA-001-05): because the job is registered in both Spring contexts (row 65), receivers are expected to get the report twice (Inferred, runtime unverified). Source: stage-02-pass-003 F-002. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/mail/MissingTimeEntryNotifier.java MissingTimeEntryNotifier#execute, #sendMissingTimeEntryReportToLeads. WAR: classes byte-identical to the v1.1a4 release; patched spring-beans.xml (WAR governs). The same run sends the report to the leads; the delivery is a runtime effect. Live question: Do the notification receivers of a project with the option on receive the report, and twice?</t>
   </si>
   <si>
     <t>Before each notification e-mail is composed, the application fetches the stylesheet xplanner.application.url + "/css/email.css" over HTTP and embeds it in the message.</t>
@@ -2596,7 +2596,7 @@
     <t>Styled e-mail when the URL is reachable; otherwise the style is expected to be missing or the e-mail to fail (runtime unverified).</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.mail.EmailFormatterImpl#formatEmailEntry (strings "xplanner.application.url", "/css/email.css", "style"; calls com.technoetic.xplanner.util.HttpClient#getPage); caller EmailNotificationSupport; WAR:css/email.css; WAR:WEB-INF/classes/xplanner-custom.properties:30. Source: stage-02-pass-001 F-006.</t>
+    <t>class com.technoetic.xplanner.mail.EmailFormatterImpl#formatEmailEntry (strings "xplanner.application.url", "/css/email.css", "style"; calls com.technoetic.xplanner.util.HttpClient#getPage); caller EmailNotificationSupport; WAR:css/email.css; WAR:WEB-INF/classes/xplanner-custom.properties:30. Source: stage-02-pass-001 F-006. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/mail/EmailFormatterImpl.java EmailFormatterImpl#formatEmailEntry (both variants). WAR: classes byte-identical to the v1.1a4 release; application URL from the patched WAR xplanner-custom.properties. Both variants fetch the stylesheet from the application URL before merging the template; the effect of an unreachable URL depends on HttpClient and the network. Live question: With the application URL unreachable from the server, is a notification sent without style, delayed or not sent?</t>
   </si>
   <si>
     <t>Mail is sent through the configured SMTP server (localhost:25, from xplanner@xplannerplus.org in the shipped properties).</t>
@@ -2608,7 +2608,7 @@
     <t>No e-mail without a reachable SMTP server.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/xplanner.properties:78-80; WAR:WEB-INF/classes/xplanner-custom.properties:30-34; package com.technoetic.xplanner.mail (EmailMessageImpl, SmtpAuthenticator). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-04: the cited value is read from xplanner-custom.properties (rewritten entry, known patch target); upstream value not determinable.</t>
+    <t>WAR:WEB-INF/classes/xplanner.properties:78-80; WAR:WEB-INF/classes/xplanner-custom.properties:30-34; package com.technoetic.xplanner.mail (EmailMessageImpl, SmtpAuthenticator). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR xplanner.properties, xplanner-custom.properties (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-04: the cited value is read from xplanner-custom.properties (rewritten entry, known patch target); upstream value not determinable.</t>
   </si>
   <si>
     <t>Data sampling for burn-down</t>
@@ -2623,7 +2623,7 @@
     <t>No nightly samples in the shipped configuration.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/spring-beans.xml:343-360 (datasamplingJob), :369-383 (trigger "0 55 23 ? 1-12 *"), :385-402 (SchedulerFactoryBean commented out); class com.technoetic.xplanner.charts.DataSamplingJob; WAR:WEB-INF/test-action-servlet.xml:4-7. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>WAR:WEB-INF/classes/spring-beans.xml:343-360 (datasamplingJob), :369-383 (trigger "0 55 23 ? 1-12 *"), :385-402 (SchedulerFactoryBean commented out); class com.technoetic.xplanner.charts.DataSamplingJob; WAR:WEB-INF/test-action-servlet.xml:4-7. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/charts/DataSamplingJob.java DataSamplingJob. WAR: patched spring-beans.xml with the scheduler factory commented out (WAR governs). The job class exists, but the WAR configuration registers no scheduler for its trigger. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
   </si>
   <si>
     <t>If iteration.automatically.extend.endDate were true, sampling would extend the end date of unclosed iterations (shipped: false).</t>
@@ -2635,7 +2635,7 @@
     <t>No automatic extension with shipped properties.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/xplanner.properties:314; class com.technoetic.xplanner.charts.DataSamplerImpl ("iteration.automatically.extend.endDate", "Extend iteration end day to "). Wiring (BA-001-07, mechanism (a)): DataSamplerImpl#extendIterationEndDateIfNeeded uses the hibernateOperations property only when the flag is true; the bean dataSampler (WAR:WEB-INF/classes/spring-beans.xml:303, autowire byName) finds no bean named hibernateOperations, so enabling the flag is expected to fail with a null reference (Inferred). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/classes/xplanner.properties:314; class com.technoetic.xplanner.charts.DataSamplerImpl ("iteration.automatically.extend.endDate", "Extend iteration end day to "). Wiring (BA-001-07, mechanism (a)): DataSamplerImpl#extendIterationEndDateIfNeeded uses the hibernateOperations property only when the flag is true; the bean dataSampler (WAR:WEB-INF/classes/spring-beans.xml:303, autowire byName) finds no bean named hibernateOperations, so enabling the flag is expected to fail with a null reference (Inferred). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/charts/DataSamplerImpl.java DataSamplerImpl#extendIterationEndDateIfNeeded. WAR: classes byte-identical to the v1.1a4 release; flag false in the patched WAR xplanner.properties. The end date is extended only when the flag is true and the iteration is active with a past end date; with the shipped value nothing is extended. The expected failure with the flag enabled stays Inferred (wiring). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
   </si>
   <si>
     <t>Per-change e-mail listener</t>
@@ -2650,7 +2650,7 @@
     <t>No e-mail per object change.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/spring-beans.xml:404-406 (eventBus EventManager); class net.sf.xplanner.email.EmailPerChangeListener (no annotation, no bean definition in any Spring XML - grep of WAR XML for EmailPerChangeListener returned no match while the same grep found eventBus). Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>WAR:WEB-INF/classes/spring-beans.xml:404-406 (eventBus EventManager); class net.sf.xplanner.email.EmailPerChangeListener (no annotation, no bean definition in any Spring XML - grep of WAR XML for EmailPerChangeListener returned no match while the same grep found eventBus). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/net/sf/xplanner/email/EmailPerChangeListener.java EmailPerChangeListener (implements ApplicationListener, no annotation); SRC:src/net/sf/xplanner/events/EventManager.java EventManager. WAR: classes byte-identical to the v1.1a4 release; component scans only net.sf.xplanner.rest (spring-beans.xml:50) and net.sf.xplanner.web (spring-web.xml:12). Events are published as Spring application events; the listener is neither annotated nor defined as a bean, and no scan covers its package. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
   </si>
   <si>
     <t>UF-014</t>
@@ -2671,7 +2671,7 @@
     <t>Overlib pop-up with format links such as XML, MPX, MSPDI, PDF, Report.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/exportLinks.jsp:16-40 (formats filtered by findActionConfig("/export/"+name+"/"+format)); WAR:WEB-INF/classes/xplanner.properties:145 (xml,mpx,mspdi,pdf,jrpdf). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/jsp/view/exportLinks.jsp:16-40 (formats filtered by findActionConfig("/export/"+name+"/"+format)); WAR:WEB-INF/classes/xplanner.properties:145 (xml,mpx,mspdi,pdf,jrpdf). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
   </si>
   <si>
     <t>Export project</t>
@@ -2686,7 +2686,7 @@
     <t>Download export.xml (text/xml), export.mpx (application/mpx) or export.xml (application/mspdi).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:189-193; WAR:WEB-INF/action-servlet.xml:45-70; classes com.technoetic.xplanner.export.XmlExporter, MpxExporter, MspdiExporter (Content-type and filename strings); WAR:WEB-INF/lib/mpxj-3.0.1.jar. Content (BA-001-08, pass-006 F-003, check (f)): besides the selected project, all three formats contain every person of the system. XmlExporter#export runs the unconditional query "from person in class net.sf.xplanner.domain.Person" and writes the result as the people of the document (XmlExporter$XPlannerData#setPeople); XmlExporter#configureBindings hides the person password and lastUpdateTime, so the other readable person properties (for example id, name, user ID, e-mail, phone, initials, hidden flag and description) are expected in the file (Betwixt, exact set Inferred). MpxExporter#export and MspdiExporter#export load all persons into MpxExporter$ResourceRegistry, which adds each one as a resource with its name only (Person#getName). The export actions have no server-side permission check (rows 29-30). Inferred; observed fact for Stage 9, Q3 deferred.</t>
+    <t>WAR:WEB-INF/struts-config.xml:189-193; WAR:WEB-INF/action-servlet.xml:45-70; classes com.technoetic.xplanner.export.XmlExporter, MpxExporter, MspdiExporter (Content-type and filename strings); WAR:WEB-INF/lib/mpxj-3.0.1.jar. Content (BA-001-08, pass-006 F-003, check (f)): besides the selected project, all three formats contain every person of the system. XmlExporter#export runs the unconditional query "from person in class net.sf.xplanner.domain.Person" and writes the result as the people of the document (XmlExporter$XPlannerData#setPeople); XmlExporter#configureBindings hides the person password and lastUpdateTime, so the other readable person properties (for example id, name, user ID, e-mail, phone, initials, hidden flag and description) are expected in the file (Betwixt, exact set Inferred). MpxExporter#export and MspdiExporter#export load all persons into MpxExporter$ResourceRegistry, which adds each one as a resource with its name only (Person#getName). The export actions have no server-side permission check (rows 29-30). Inferred; observed fact for Stage 9, Q3 deferred. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/export/XmlExporter.java XmlExporter#export; SRC:src/com/technoetic/xplanner/export/MpxExporter.java MpxExporter#export. WAR: classes byte-identical to the v1.1a4 release. Both exporters load all persons (the XML file as people, MPX and MSPDI as resources), as recorded.</t>
   </si>
   <si>
     <t>Export iteration</t>
@@ -2701,7 +2701,7 @@
     <t>Downloads export.xml, export.mpx, export.xml, export.pdf.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:231-237; WAR:WEB-INF/action-servlet.xml:132-166; class com.technoetic.xplanner.export.PdfExporter ("application/pdf", "export.pdf"); WAR:WEB-INF/lib/itext-1.01.jar. Content (BA-001-08, pass-006 F-003, check (f)): the XML, MPX and MSPDI files contain every person of the system, as in row 209 (the same exporter beans, WAR:WEB-INF/action-servlet.xml:132-166). The PDF listing (PdfExporter) shows only the names of the customers and acceptors of the exported stories and tasks (Person#getName), no person list (Inferred).</t>
+    <t>WAR:WEB-INF/struts-config.xml:231-237; WAR:WEB-INF/action-servlet.xml:132-166; class com.technoetic.xplanner.export.PdfExporter ("application/pdf", "export.pdf"); WAR:WEB-INF/lib/itext-1.01.jar. Content (BA-001-08, pass-006 F-003, check (f)): the XML, MPX and MSPDI files contain every person of the system, as in row 209 (the same exporter beans, WAR:WEB-INF/action-servlet.xml:132-166). The PDF listing (PdfExporter) shows only the names of the customers and acceptors of the exported stories and tasks (Person#getName), no person list (Inferred). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/export/XmlExporter.java XmlExporter#export; SRC:src/com/technoetic/xplanner/export/PdfExporter.java PdfExporter. WAR: classes byte-identical to the v1.1a4 release. As row 209 for XML, MPX and MSPDI; the PDF exporter lists the iteration's stories and tasks.</t>
   </si>
   <si>
     <t>An iteration JasperReports PDF (jrpdf) report is offered but its report template is missing from the WAR.</t>
@@ -2713,7 +2713,7 @@
     <t>report.pdf expected; generation expected to fail.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:239; WAR:WEB-INF/action-servlet.xml:168-175 (reportExporter); class com.technoetic.xplanner.export.PdfReportExporter (template com/technoetic/xplanner/export/reports/JRIteration.jrxml) - no *.jrxml or *.jasper in the WAR or its JARs (search also matched JRXml* classes, proving the pattern works). Query property paths (BA-001-05): class PdfReportExporter$PersonDataSource and $UserStoryDataSource also query "task.story", which Task does not map, so the person and story reports would fail even with templates present. Sweep of pass-003 F-001.</t>
+    <t>WAR:WEB-INF/struts-config.xml:239; WAR:WEB-INF/action-servlet.xml:168-175 (reportExporter); class com.technoetic.xplanner.export.PdfReportExporter (template com/technoetic/xplanner/export/reports/JRIteration.jrxml) - no *.jrxml or *.jasper in the WAR or its JARs (search also matched JRXml* classes, proving the pattern works). Query property paths (BA-001-05): class PdfReportExporter$PersonDataSource and $UserStoryDataSource also query "task.story", which Task does not map, so the person and story reports would fail even with templates present. Sweep of pass-003 F-001. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/export/PdfReportExporter.java PdfReportExporter (loads the templates with getResourceAsStream); SRC:src/com/technoetic/xplanner/export/reports/JRIteration.jrxml. WAR: classes byte-identical to the v1.1a4 release; the four report templates exist in the SVN source (src/com/technoetic/xplanner/export/reports/JR*.jrxml) but not in the WAR (WAR governs). The template is missing from the delivered package only: the release build did not include the SVN templates. For the WAR the generation is still expected to fail.</t>
   </si>
   <si>
     <t>Export story, task and person</t>
@@ -2728,7 +2728,7 @@
     <t>export.pdf download.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:281,297; WAR:WEB-INF/action-servlet.xml:238-245,280-287 (pdfExporter).</t>
+    <t>WAR:WEB-INF/struts-config.xml:281,297; WAR:WEB-INF/action-servlet.xml:238-245,280-287 (pdfExporter). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>Story, task and person JasperReports reports (jrpdf) are offered but their templates are missing.</t>
@@ -2737,7 +2737,7 @@
     <t>Formatted reports.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:283,299,315; WAR:WEB-INF/action-servlet.xml:247-254,289-296,333-340; class PdfReportExporter (JRStory.jrxml, JRTask.jrxml, JRPerson.jrxml absent). Query property paths (BA-001-05): the story and person report data sources (PdfReportExporter$UserStoryDataSource "task.story = ?", $PersonDataSource "task.story = story.id") use a property that Task does not map. Sweep of pass-003 F-001.</t>
+    <t>WAR:WEB-INF/struts-config.xml:283,299,315; WAR:WEB-INF/action-servlet.xml:247-254,289-296,333-340; class PdfReportExporter (JRStory.jrxml, JRTask.jrxml, JRPerson.jrxml absent). Query property paths (BA-001-05): the story and person report data sources (PdfReportExporter$UserStoryDataSource "task.story = ?", $PersonDataSource "task.story = story.id") use a property that Task does not map. Sweep of pass-003 F-001. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/export/PdfReportExporter.java PdfReportExporter; SRC:src/com/technoetic/xplanner/export/reports/JRStory.jrxml, JRTask.jrxml, JRPerson.jrxml. WAR: classes byte-identical to the v1.1a4 release; JRStory, JRTask and JRPerson.jrxml exist in the SVN source but not in the WAR (WAR governs). As row 211: the templates exist in the source tree but were not packaged; the task.story query defect remains.</t>
   </si>
   <si>
     <t>UF-015</t>
@@ -2758,7 +2758,7 @@
     <t>SOAP responses with ProjectData, IterationData, UserStoryData, TaskData, TimeEntryData, NoteData, PersonData beans; 401 challenge "Basic realm=XPlanner" without credentials.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:206-209,298-306 (AxisServlet /servlet/AxisServlet and /soap/*), :111-119,168-171 (BasicSecurityFilter on /soap/*); WAR:WEB-INF/server-config.wsdd:25-28,44-51 (service XPlanner, class com.technoetic.xplanner.soap.XPlanner, 8 bean mappings); class BasicSecurityFilter#challenge ("WWW-Authenticate", "Basic realm=\"XPlanner\"").</t>
+    <t>WAR:WEB-INF/web.xml:206-209,298-306 (AxisServlet /servlet/AxisServlet and /soap/*), :111-119,168-171 (BasicSecurityFilter on /soap/*); WAR:WEB-INF/server-config.wsdd:25-28,44-51 (service XPlanner, class com.technoetic.xplanner.soap.XPlanner, 8 bean mappings); class BasicSecurityFilter#challenge ("WWW-Authenticate", "Basic realm=\"XPlanner\""). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/security/filter/BasicSecurityFilter.java BasicSecurityFilter#onAuthenticationFailure, #challenge. WAR: classes byte-identical to the v1.1a4 release. An unauthenticated SOAP request is answered with a Basic challenge.</t>
   </si>
   <si>
     <t>The same Axis servlet is also mapped at /servlet/AxisServlet, where no Basic security filter is applied.</t>
@@ -2770,7 +2770,7 @@
     <t>SOAP reachable without the filter at the alternate path (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:298-301 (servlet-mapping /servlet/AxisServlet) versus filter mappings :168-176 (/soap/*, /ical/* only).</t>
+    <t>WAR:WEB-INF/web.xml:298-301 (servlet-mapping /servlet/AxisServlet) versus filter mappings :168-176 (/soap/*, /ical/* only). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact); status Inferred -&gt; Yes. none: descriptor fact, no Java involved. WAR: web.xml identical to the SVN webapp copy. The servlet mapping /servlet/AxisServlet has no security filter mapping.</t>
   </si>
   <si>
     <t>An Axis "Version" service reports the Axis version.</t>
@@ -2782,7 +2782,7 @@
     <t>getVersion response.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/server-config.wsdd:29-32.</t>
+    <t>WAR:WEB-INF/server-config.wsdd:29-32. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
     <t>SOAP operations check the caller's permission on each object (read for get operations, create/edit/delete for changes); the five attribute operations (setAttribute, getAttribute, deleteAttribute, getAttributes, getAttributesWithPrefix) have no permission check.</t>
@@ -2794,7 +2794,7 @@
     <t>Messages such as "no permission to update object"; lists contain only accessible objects; attribute calls succeed for any authenticated caller (runtime unverified).</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.soap.XPlanner#hasPermission via #getObject, #getObjects/#selectAccessibleObjects, #addObject, #updateObject, #removeObject (strings "no permission to create object", "no permission to update object", "no permission to delete object"); no authorization call reachable from the attribute operations (.migration-tmp/stage-01/out/authtrace.json). BA-001-03 impact sweep of F-001.</t>
+    <t>class com.technoetic.xplanner.soap.XPlanner#hasPermission via #getObject, #getObjects/#selectAccessibleObjects, #addObject, #updateObject, #removeObject (strings "no permission to create object", "no permission to update object", "no permission to delete object"); no authorization call reachable from the attribute operations (.migration-tmp/stage-01/out/authtrace.json). BA-001-03 impact sweep of F-001. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/soap/XPlanner.java XPlanner#hasPermission, #setAttribute, #getAttribute, #deleteAttribute, #getAttributes, #getAttributesWithPrefix. WAR: classes byte-identical to the v1.1a4 release. Object operations call hasPermission; the attribute operations delegate straight to the attribute repository.</t>
   </si>
   <si>
     <t>A JAX-WS endpoint net.sf.xplanner.soap.XPlanner is declared but not active (servlet commented out, class absent).</t>
@@ -2809,7 +2809,7 @@
     <t>No</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/sun-jaxws.xml:3; WAR:WEB-INF/web.xml:183-185,273-282 (WSServlet commented); class net.sf.xplanner.soap.XPlanner ABSENT.</t>
+    <t>WAR:WEB-INF/sun-jaxws.xml:3; WAR:WEB-INF/web.xml:183-185,273-282 (WSServlet commented); class net.sf.xplanner.soap.XPlanner ABSENT. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: net.sf.xplanner.soap.XPlanner is absent from the SVN source as from the WAR. WAR: sun-jaxws.xml identical to the SVN webapp copy. The declared endpoint class exists nowhere.</t>
   </si>
   <si>
     <t>SOAP read operations</t>
@@ -2824,7 +2824,7 @@
     <t>Operations getProjects, getProject, getIterations, getIteration, getUserStories, getUserStory, getTasks, getTask, getCurrentTasksForPerson, getPlannedTasksForPerson, getTimeEntries, getTimeEntry, getNote, getNotesForObject, getPerson, getPeople, getAttribute, getAttributes, getAttributesWithPrefix; getCurrentIteration expected to return a SOAP fault (runtime unverified).</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.soap.XPlanner public methods (43 public operations enumerated in .migration-tmp/stage-01/out/enumeration.json); #selectAccessibleObjects/#hasPermission (permission filtering). Query property paths (BA-001-05): XPlanner#getCurrentIteration passes "object.startDate &lt;= ? and object.endDate &gt;= ? and object.projectId = ?" to #getObjects, which builds "from net.sf.xplanner.domain.Iteration where " + condition without declaring an alias; Iteration maps project (@ManyToOne) but no projectId. #getObjects logs "error loading objects" and rethrows. #getNotesForObject uses "attachedTo_Id = &lt;id&gt;", an unqualified column name (Note maps attachedToId, column attachedTo_id) whose treatment is framework behavior (GAP-011, Stage 3). Source: stage-02-pass-003 F-001.</t>
+    <t>class com.technoetic.xplanner.soap.XPlanner public methods (43 public operations enumerated in .migration-tmp/stage-01/out/enumeration.json); #selectAccessibleObjects/#hasPermission (permission filtering). Query property paths (BA-001-05): XPlanner#getCurrentIteration passes "object.startDate &lt;= ? and object.endDate &gt;= ? and object.projectId = ?" to #getObjects, which builds "from net.sf.xplanner.domain.Iteration where " + condition without declaring an alias; Iteration maps project (@ManyToOne) but no projectId. #getObjects logs "error loading objects" and rethrows. #getNotesForObject uses "attachedTo_Id = &lt;id&gt;", an unqualified column name (Note maps attachedToId, column attachedTo_id) whose treatment is framework behavior (GAP-011, Stage 3). Source: stage-02-pass-003 F-001. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/soap/XPlanner.java XPlanner#getCurrentIteration, #getObjects. WAR: classes byte-identical to the v1.1a4 release. The source confirms the condition text; how Hibernate treats it is framework behavior. Live question: Does getCurrentIteration return a SOAP fault, and does getNotesForObject return the notes of an object?</t>
   </si>
   <si>
     <t>SOAP write operations</t>
@@ -2839,7 +2839,7 @@
     <t>Operations addX/update/removeX, setAttribute, deleteAttribute.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.soap.XPlanner (addProject ... removePerson, update(*Data), setAttribute, deleteAttribute; #saveHistory, #hasPermission). Server-side enforcement (CHK-002, BA-001-04): enforced on the server by XPlanner#hasPermission for the object operations; the attribute operations have no check (row 218). Delete cascade sweep (BA-001-04): XPlanner#removeObject calls Session.delete, so the mapping cascades of the web deletes apply (rows 82, 91, 126, 142) and notes attached to the removed object are not deleted (NoteHelper#deleteNotesFor is not reached). Query property paths (BA-001-05): deleteAttribute calls AttributeRepositoryImpl#delete with "from a in net.sf.xplanner.domain.Attribute where a.targetId = ? and a.name = ?"; Attribute keeps targetId and name in its embedded id (#getAttributeId, @EmbeddedId; #getName is @Transient), so a.targetId and a.name are not mapped paths and deleteAttribute is expected to fail. setAttribute and getAttributes use unqualified targetId and name (framework behavior, GAP-011). Sweep of pass-003 F-001.</t>
+    <t>class com.technoetic.xplanner.soap.XPlanner (addProject ... removePerson, update(*Data), setAttribute, deleteAttribute; #saveHistory, #hasPermission). Server-side enforcement (CHK-002, BA-001-04): enforced on the server by XPlanner#hasPermission for the object operations; the attribute operations have no check (row 218). Delete cascade sweep (BA-001-04): XPlanner#removeObject calls Session.delete, so the mapping cascades of the web deletes apply (rows 82, 91, 126, 142) and notes attached to the removed object are not deleted (NoteHelper#deleteNotesFor is not reached). Query property paths (BA-001-05): deleteAttribute calls AttributeRepositoryImpl#delete with "from a in net.sf.xplanner.domain.Attribute where a.targetId = ? and a.name = ?"; Attribute keeps targetId and name in its embedded id (#getAttributeId, @EmbeddedId; #getName is @Transient), so a.targetId and a.name are not mapped paths and deleteAttribute is expected to fail. setAttribute and getAttributes use unqualified targetId and name (framework behavior, GAP-011). Sweep of pass-003 F-001. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/soap/XPlanner.java XPlanner#addObject, #updateObject, #removeObject, #saveHistory; SRC:src/com/technoetic/xplanner/domain/repository/AttributeRepositoryImpl.java AttributeRepositoryImpl#delete. WAR: classes byte-identical to the v1.1a4 release. Permission checks and history on the object operations are confirmed; the delete cascades and the deleteAttribute query depend on Hibernate. Live question: Does SOAP removeProject leave the project notes, and does deleteAttribute fail?</t>
   </si>
   <si>
     <t>UF-016</t>
@@ -2860,7 +2860,7 @@
     <t>XML/JSON payloads (ProjectView, UserStoryView[]).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:256-263,288-291 (Jersey SpringServlet /rest/*, POJOMappingFeature); class net.sf.xplanner.rest.ViewService (@Path "/view", "/project/{projectId}", "/iteration/{iterationId}/userstories", @Produces application/xml, application/json); WAR:WEB-INF/classes/spring-beans.xml:50 (component-scan net.sf.xplanner.rest). Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>WAR:WEB-INF/web.xml:256-263,288-291 (Jersey SpringServlet /rest/*, POJOMappingFeature); class net.sf.xplanner.rest.ViewService (@Path "/view", "/project/{projectId}", "/iteration/{iterationId}/userstories", @Produces application/xml, application/json); WAR:WEB-INF/classes/spring-beans.xml:50 (component-scan net.sf.xplanner.rest). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/net/sf/xplanner/rest/ViewService.java ViewService#getProject, #getUserStories. WAR: classes byte-identical to the v1.1a4 release. The two GET resources return the project view and the story views as XML or JSON. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
   </si>
   <si>
     <t>GET /rest/view returns a plain-text response.</t>
@@ -2872,7 +2872,7 @@
     <t>text/plain body.</t>
   </si>
   <si>
-    <t>class ViewService#getIt (@GET, @Produces text/plain).</t>
+    <t>class ViewService#getIt (@GET, @Produces text/plain). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/net/sf/xplanner/rest/ViewService.java ViewService#getIt. WAR: classes byte-identical to the v1.1a4 release. GET /rest/view returns a constant text/plain string.</t>
   </si>
   <si>
     <t>No security filter is mapped to /rest/*.</t>
@@ -2884,7 +2884,7 @@
     <t>Endpoints reachable without authentication (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:130-181 (no filter-mapping for /rest/*). BA-001-03 impact sweep of F-001: ViewService, UpdateService, ViewManager and UpdateManager reach no authorization call either (.migration-tmp/stage-01/out/authtrace.json).</t>
+    <t>WAR:WEB-INF/web.xml:130-181 (no filter-mapping for /rest/*). BA-001-03 impact sweep of F-001: ViewService, UpdateService, ViewManager and UpdateManager reach no authorization call either (.migration-tmp/stage-01/out/authtrace.json). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/net/sf/xplanner/rest/ViewService.java ViewService; SRC:src/net/sf/xplanner/rest/UpdateService.java UpdateService; SRC:src/net/sf/xplanner/rest/ViewManager.java ViewManager; SRC:src/net/sf/xplanner/rest/UpdateManager.java UpdateManager. WAR: web.xml identical to the SVN webapp copy. No filter mapping covers /rest/* and none of the REST classes calls an authorizer.</t>
   </si>
   <si>
     <t>REST task status update</t>
@@ -2899,7 +2899,7 @@
     <t>Result "Task updated", "Task not found", "Task status not changed" or "Moving Task to not started not implemented".</t>
   </si>
   <si>
-    <t>class net.sf.xplanner.rest.UpdateService (@Path "/update", @POST "/task/{taskId}/status", @FormParam status, originalEstimate); class net.sf.xplanner.rest.UpdateManager#updateTaskStatus (result strings); class net.sf.xplanner.domain.enums.TaskStatus.</t>
+    <t>class net.sf.xplanner.rest.UpdateService (@Path "/update", @POST "/task/{taskId}/status", @FormParam status, originalEstimate); class net.sf.xplanner.rest.UpdateManager#updateTaskStatus (result strings); class net.sf.xplanner.domain.enums.TaskStatus. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/net/sf/xplanner/rest/UpdateService.java UpdateService#post; SRC:src/net/sf/xplanner/rest/UpdateManager.java UpdateManager#updateTaskStatus. WAR: classes byte-identical to the v1.1a4 release. The four results are returned as recorded: not found, unchanged status, not-started not implemented, otherwise started (with the original estimate) or completed and saved.</t>
   </si>
   <si>
     <t>UF-017</t>
@@ -2920,7 +2920,7 @@
     <t>Expected: the first query fails, "ical error" is logged and the servlet answers with sendError and the exception message; no VCALENDAR body (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:251-254,308-311 (iCalServlet /ical/*), :173-176 (BasicSecurityFilter /ical/*); class com.technoetic.xplanner.ical.iCalServlet#doGet, #generateTaskData, #generateTimeEntryData (HQL and VCALENDAR strings). Locale dependence (CHK-004, BA-001-04): the "non-overhead" filter compares the stored type with task.type.overhead from java.util.ResourceBundle.getBundle("ResourceBundle"), i.e. the JVM default locale (class iCalServlet#generateTaskData); overhead tasks saved under a different label are included (row 135). Query property paths (BA-001-05): class iCalServlet#generateTimeEntryData (called first, before #generateTaskData) and #generateTaskData pass HQL containing "task.story = story.id" to Session.find; net.sf.xplanner.domain.Task maps the story only as userStory (#getUserStory, @ManyToOne @JoinColumn story_id) and has no story property; mappings/Task.xml is not loaded (WAR:WEB-INF/classes/spring-beans.xml:77-81). The exception propagates to #doGet, whose handler logs "ical error" and calls HttpServletResponse.sendError (bytecode listing with exception table). The query failure itself is framework behavior (Hibernate rejects an unresolvable property path; GAP-011). Corrected in BA-001-05 (Source: stage-02-pass-003 F-001).</t>
+    <t>WAR:WEB-INF/web.xml:251-254,308-311 (iCalServlet /ical/*), :173-176 (BasicSecurityFilter /ical/*); class com.technoetic.xplanner.ical.iCalServlet#doGet, #generateTaskData, #generateTimeEntryData (HQL and VCALENDAR strings). Locale dependence (CHK-004, BA-001-04): the "non-overhead" filter compares the stored type with task.type.overhead from java.util.ResourceBundle.getBundle("ResourceBundle"), i.e. the JVM default locale (class iCalServlet#generateTaskData); overhead tasks saved under a different label are included (row 135). Query property paths (BA-001-05): class iCalServlet#generateTimeEntryData (called first, before #generateTaskData) and #generateTaskData pass HQL containing "task.story = story.id" to Session.find; net.sf.xplanner.domain.Task maps the story only as userStory (#getUserStory, @ManyToOne @JoinColumn story_id) and has no story property; mappings/Task.xml is not loaded (WAR:WEB-INF/classes/spring-beans.xml:77-81). The exception propagates to #doGet, whose handler logs "ical error" and calls HttpServletResponse.sendError (bytecode listing with exception table). The query failure itself is framework behavior (Hibernate rejects an unresolvable property path; GAP-011). Corrected in BA-001-05 (Source: stage-02-pass-003 F-001). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/ical/iCalServlet.java iCalServlet#doGet, #generateTimeEntryData, #generateTaskData. WAR: classes byte-identical to the v1.1a4 release. The queries use task.story as recorded; whether Hibernate rejects them is framework behavior. Live question: Does GET /ical/&lt;own userId&gt;.ics return an error instead of a calendar?</t>
   </si>
   <si>
     <t>Requests without a file name or without the .ics suffix are rejected.</t>
@@ -2932,7 +2932,7 @@
     <t>Messages "No iCal file requested." / "No .ics suffix for requested iCal file."</t>
   </si>
   <si>
-    <t>class iCalServlet#doGet (strings "No iCal file requested.", "No .ics suffix for requested iCal file.").</t>
+    <t>class iCalServlet#doGet (strings "No iCal file requested.", "No .ics suffix for requested iCal file."). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/ical/iCalServlet.java iCalServlet#doGet. WAR: classes byte-identical to the v1.1a4 release. A missing file name and a missing .ics suffix return HTTP 400 with the two messages.</t>
   </si>
   <si>
     <t>Requesting another person's calendar requires admin.edit on system.person.</t>
@@ -2944,7 +2944,7 @@
     <t>Message "No authorization for accessing calendar for &lt;user&gt;".</t>
   </si>
   <si>
-    <t>class iCalServlet#doGet (strings "system.person", "admin.edit", "No authorization for accessing calendar for ").</t>
+    <t>class iCalServlet#doGet (strings "system.person", "admin.edit", "No authorization for accessing calendar for "). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/ical/iCalServlet.java iCalServlet#doGet. WAR: classes byte-identical to the v1.1a4 release. For another user's calendar the servlet requires admin.edit on system.person for some project (checked against the caller's own person id) and otherwise returns HTTP 403 with the message.</t>
   </si>
   <si>
     <t>UF-018</t>
@@ -2965,19 +2965,19 @@
     <t>WML cards with links to the underlying objects (hard-coded /xplanner path). Submitting the WAP login is expected to fail with a null reference, and a view request that carries a projectId is expected to fail the same way, because these actions are created by Struts without Spring injection (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/mobile-struts-config.xml:20-49 (7 actions); WAR:WEB-INF/jsp/wap/login.jsp, projects.jsp, project.jsp, iteration.jsp, story.jsp, task.jsp, person.jsp; WAR:WEB-INF/web.xml:98-109,155-158 (MobileSecurityFilter /do/mobile/*); WAR:WEB-INF/mobile-security.xml. All WML links hard-code /xplanner/do/mobile/..., which does not match the WAR context path /xplanner-plus. Wiring (BA-001-07, mechanism (a)): the seven mappings of WAR:WEB-INF/mobile-struts-config.xml:20-49 have no bean in action-servlet.xml; the Spring request processor falls back to the Struts-created instance (framework behavior, GAP-011), which receives no injection. AuthenticationAction#execute uses the authenticator field, set only by #setAuthenticator; DispatchForward#execute uses the authorizer field, set only by #setAuthorizer (sweep .migration-tmp/stage-01/out/wiring-07.txt, wiring-impact-07.txt). Corrected in BA-001-07 (Source: stage-02-pass-005 F-004).</t>
-  </si>
-  <si>
-    <t>The general web security filter also covers /do/mobile/* and does not bypass /do/mobile/login, so an unauthenticated mobile login may be redirected to the HTML login.</t>
+    <t>WAR:WEB-INF/mobile-struts-config.xml:20-49 (7 actions); WAR:WEB-INF/jsp/wap/login.jsp, projects.jsp, project.jsp, iteration.jsp, story.jsp, task.jsp, person.jsp; WAR:WEB-INF/web.xml:98-109,155-158 (MobileSecurityFilter /do/mobile/*); WAR:WEB-INF/mobile-security.xml. All WML links hard-code /xplanner/do/mobile/..., which does not match the WAR context path /xplanner-plus. Wiring (BA-001-07, mechanism (a)): the seven mappings of WAR:WEB-INF/mobile-struts-config.xml:20-49 have no bean in action-servlet.xml; the Spring request processor falls back to the Struts-created instance (framework behavior, GAP-011), which receives no injection. AuthenticationAction#execute uses the authenticator field, set only by #setAuthenticator; DispatchForward#execute uses the authorizer field, set only by #setAuthorizer (sweep .migration-tmp/stage-01/out/wiring-07.txt, wiring-impact-07.txt). Corrected in BA-001-07 (Source: stage-02-pass-005 F-004). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/AuthenticationAction.java AuthenticationAction#execute (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/actions/DispatchForward.java DispatchForward#execute. WAR: classes byte-identical to the v1.1a4 release; WAP JSPs identical to the SVN webapp copies. Both actions depend on injected fields that the Struts-created instances do not receive; the outcome is a runtime effect. Live question: Does a WAP login submission fail with an error page?</t>
+  </si>
+  <si>
+    <t>The general web security filter also covers /do/mobile/* and does not bypass /do/mobile/login, so an unauthenticated mobile login request is redirected to the HTML login.</t>
   </si>
   <si>
     <t>Records a filter conflict affecting mobile login.</t>
   </si>
   <si>
-    <t>Possible redirect to /do/login (runtime unverified).</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/web.xml:155-163 (MobileSecurityFilter /do/mobile/* then WebSecurityFilter /do/*); WAR:WEB-INF/security.xml:2-6 (no /do/mobile/login bypass); class SecurityConfiguration#isSecureRequest. The viewer/editor/admin roles listed in WAR:WEB-INF/mobile-security.xml:11-15 are never evaluated (SecurityConfiguration#isAuthorized has no caller; stage-02-pass-001 F-004).</t>
+    <t>Redirect to /do/login before the mobile login is reached.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/web.xml:155-163 (MobileSecurityFilter /do/mobile/* then WebSecurityFilter /do/*); WAR:WEB-INF/security.xml:2-6 (no /do/mobile/login bypass); class SecurityConfiguration#isSecureRequest. The viewer/editor/admin roles listed in WAR:WEB-INF/mobile-security.xml:11-15 are never evaluated (SecurityConfiguration#isAuthorized has no caller; stage-02-pass-001 F-004). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/filter/AbstractSecurityFilter.java AbstractSecurityFilter#doFilter; SRC:src/com/technoetic/xplanner/security/config/SecurityConfiguration.java SecurityConfiguration#isSecureRequest; SRC:src/com/technoetic/xplanner/security/filter/FormSecurityFilter.java FormSecurityFilter#onAuthenticationFailure. WAR: web.xml, security.xml and mobile-security.xml identical to the SVN webapp copies. Both filters are FormSecurityFilter instances; a request is secure unless it matches the filter's own bypass list. The mobile filter bypasses /do/mobile/login, but the web filter on /do/* uses security.xml, which does not, so an unauthenticated mobile login request is redirected to /do/login.</t>
   </si>
   <si>
     <t>The WAP view actions are DispatchForward actions with authorization required (the default); the WML links pass only oid, so without a projectId parameter each view is expected to forward to the not-authorized page (absent) instead of the WML card.</t>
@@ -2989,7 +2989,7 @@
     <t>Not-authorized forward instead of the project, iteration, story, task or person card (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/mobile-struts-config.xml:27-49 (type DispatchForward, no Spring bean and no authorizationRequired override); class DispatchForward#&lt;init&gt; (isAuthorizationRequired true) and #execute ("no project identifier supplied for secure access", forward "security/notAuthorized"); WAR:WEB-INF/jsp/wap/projects.jsp, project.jsp (links with oid only). Depends on Spring DelegatingTilesRequestProcessor falling back to the mapping type when no bean exists (framework behavior, GAP-011). BA-001-03 impact sweep of F-001. Null dependency (BA-001-07): because the Struts-created DispatchForward has no authorizer, a request that does carry a non-zero projectId is expected to fail with a null reference in #execute at Authorizer.hasPermission; without projectId the not-authorized forward described here remains the outcome. Source: stage-02-pass-005 F-004.</t>
+    <t>WAR:WEB-INF/mobile-struts-config.xml:27-49 (type DispatchForward, no Spring bean and no authorizationRequired override); class DispatchForward#&lt;init&gt; (isAuthorizationRequired true) and #execute ("no project identifier supplied for secure access", forward "security/notAuthorized"); WAR:WEB-INF/jsp/wap/projects.jsp, project.jsp (links with oid only). Depends on Spring DelegatingTilesRequestProcessor falling back to the mapping type when no bean exists (framework behavior, GAP-011). BA-001-03 impact sweep of F-001. Null dependency (BA-001-07): because the Struts-created DispatchForward has no authorizer, a request that does carry a non-zero projectId is expected to fail with a null reference in #execute at Authorizer.hasPermission; without projectId the not-authorized forward described here remains the outcome. Source: stage-02-pass-005 F-004. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/DispatchForward.java DispatchForward#execute, #isSecure. WAR: classes byte-identical to the v1.1a4 release. The authorization-required default and the missing projectId branch are confirmed; the fallback to the mapping type without a bean is framework behavior. Live question: Which page does /do/mobile/view/project?oid=&lt;id&gt; show after a mobile login?</t>
   </si>
 </sst>
 </file>
@@ -3760,10 +3760,10 @@
         <v>46</v>
       </c>
       <c r="G10" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H10" s="23" t="s">
         <v>47</v>
-      </c>
-      <c r="H10" s="23" t="s">
-        <v>48</v>
       </c>
       <c r="I10" s="23"/>
       <c r="J10" s="23"/>
@@ -3779,16 +3779,16 @@
         <v>39</v>
       </c>
       <c r="D11" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="E11" s="23" t="s">
+      <c r="F11" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="F11" s="23" t="s">
+      <c r="G11" s="23" t="s">
         <v>51</v>
-      </c>
-      <c r="G11" s="23" t="s">
-        <v>47</v>
       </c>
       <c r="H11" s="23" t="s">
         <v>52</v>
@@ -3846,7 +3846,7 @@
         <v>60</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H13" s="23" t="s">
         <v>61</v>
@@ -3874,7 +3874,7 @@
         <v>64</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H14" s="23" t="s">
         <v>65</v>
@@ -3932,7 +3932,7 @@
         <v>73</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H16" s="23" t="s">
         <v>74</v>
@@ -4134,7 +4134,7 @@
         <v>106</v>
       </c>
       <c r="G23" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H23" s="23" t="s">
         <v>107</v>
@@ -4162,7 +4162,7 @@
         <v>110</v>
       </c>
       <c r="G24" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H24" s="23" t="s">
         <v>111</v>
@@ -4190,7 +4190,7 @@
         <v>114</v>
       </c>
       <c r="G25" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H25" s="23" t="s">
         <v>115</v>
@@ -4306,7 +4306,7 @@
         <v>132</v>
       </c>
       <c r="G29" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H29" s="23" t="s">
         <v>133</v>
@@ -4334,7 +4334,7 @@
         <v>132</v>
       </c>
       <c r="G30" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H30" s="23" t="s">
         <v>136</v>
@@ -4362,7 +4362,7 @@
         <v>139</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H31" s="23" t="s">
         <v>140</v>
@@ -4390,7 +4390,7 @@
         <v>143</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H32" s="23" t="s">
         <v>144</v>
@@ -4448,7 +4448,7 @@
         <v>152</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H34" s="23" t="s">
         <v>153</v>
@@ -4818,7 +4818,7 @@
         <v>207</v>
       </c>
       <c r="G47" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H47" s="23" t="s">
         <v>208</v>
@@ -4876,7 +4876,7 @@
         <v>216</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H49" s="23" t="s">
         <v>217</v>
@@ -5190,7 +5190,7 @@
         <v>263</v>
       </c>
       <c r="G60" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H60" s="23" t="s">
         <v>264</v>
@@ -5220,7 +5220,7 @@
         <v>268</v>
       </c>
       <c r="G61" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H61" s="23" t="s">
         <v>269</v>
@@ -5248,7 +5248,7 @@
         <v>272</v>
       </c>
       <c r="G62" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H62" s="23" t="s">
         <v>273</v>
@@ -5276,7 +5276,7 @@
         <v>276</v>
       </c>
       <c r="G63" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H63" s="23" t="s">
         <v>277</v>
@@ -5334,7 +5334,7 @@
         <v>285</v>
       </c>
       <c r="G65" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H65" s="23" t="s">
         <v>286</v>
@@ -5362,7 +5362,7 @@
         <v>289</v>
       </c>
       <c r="G66" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H66" s="23" t="s">
         <v>290</v>
@@ -5392,7 +5392,7 @@
         <v>294</v>
       </c>
       <c r="G67" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H67" s="23" t="s">
         <v>295</v>
@@ -5420,7 +5420,7 @@
         <v>298</v>
       </c>
       <c r="G68" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H68" s="23" t="s">
         <v>299</v>
@@ -5504,7 +5504,7 @@
         <v>310</v>
       </c>
       <c r="G71" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H71" s="23" t="s">
         <v>311</v>
@@ -5758,7 +5758,7 @@
         <v>347</v>
       </c>
       <c r="G80" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H80" s="23" t="s">
         <v>348</v>
@@ -6336,7 +6336,7 @@
         <v>434</v>
       </c>
       <c r="G100" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H100" s="23" t="s">
         <v>435</v>
@@ -6682,7 +6682,7 @@
         <v>487</v>
       </c>
       <c r="G112" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H112" s="23" t="s">
         <v>488</v>
@@ -6856,7 +6856,7 @@
         <v>514</v>
       </c>
       <c r="G118" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H118" s="23" t="s">
         <v>515</v>
@@ -6884,7 +6884,7 @@
         <v>518</v>
       </c>
       <c r="G119" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H119" s="23" t="s">
         <v>519</v>
@@ -6966,7 +6966,7 @@
         <v>529</v>
       </c>
       <c r="G122" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H122" s="23" t="s">
         <v>530</v>
@@ -7022,7 +7022,7 @@
         <v>537</v>
       </c>
       <c r="G124" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H124" s="23" t="s">
         <v>538</v>
@@ -7198,7 +7198,7 @@
         <v>564</v>
       </c>
       <c r="G130" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H130" s="23" t="s">
         <v>565</v>
@@ -7254,7 +7254,7 @@
         <v>572</v>
       </c>
       <c r="G132" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H132" s="23" t="s">
         <v>573</v>
@@ -7336,7 +7336,7 @@
         <v>583</v>
       </c>
       <c r="G135" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H135" s="23" t="s">
         <v>584</v>
@@ -7364,7 +7364,7 @@
         <v>587</v>
       </c>
       <c r="G136" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H136" s="23" t="s">
         <v>588</v>
@@ -7422,7 +7422,7 @@
         <v>595</v>
       </c>
       <c r="G138" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H138" s="23" t="s">
         <v>596</v>
@@ -7628,7 +7628,7 @@
         <v>628</v>
       </c>
       <c r="G145" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H145" s="23" t="s">
         <v>629</v>
@@ -7684,7 +7684,7 @@
         <v>635</v>
       </c>
       <c r="G147" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H147" s="23" t="s">
         <v>636</v>
@@ -7794,7 +7794,7 @@
         <v>650</v>
       </c>
       <c r="G151" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H151" s="23" t="s">
         <v>651</v>
@@ -7822,7 +7822,7 @@
         <v>653</v>
       </c>
       <c r="G152" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H152" s="23" t="s">
         <v>654</v>
@@ -7850,7 +7850,7 @@
         <v>657</v>
       </c>
       <c r="G153" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H153" s="23" t="s">
         <v>658</v>
@@ -7878,7 +7878,7 @@
         <v>661</v>
       </c>
       <c r="G154" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H154" s="23" t="s">
         <v>662</v>
@@ -7906,7 +7906,7 @@
         <v>665</v>
       </c>
       <c r="G155" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H155" s="23" t="s">
         <v>666</v>
@@ -7934,7 +7934,7 @@
         <v>669</v>
       </c>
       <c r="G156" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H156" s="23" t="s">
         <v>670</v>
@@ -7962,7 +7962,7 @@
         <v>673</v>
       </c>
       <c r="G157" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H157" s="23" t="s">
         <v>674</v>
@@ -7990,7 +7990,7 @@
         <v>677</v>
       </c>
       <c r="G158" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H158" s="23" t="s">
         <v>678</v>
@@ -8018,7 +8018,7 @@
         <v>681</v>
       </c>
       <c r="G159" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H159" s="23" t="s">
         <v>682</v>
@@ -8046,7 +8046,7 @@
         <v>685</v>
       </c>
       <c r="G160" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H160" s="23" t="s">
         <v>686</v>
@@ -8162,7 +8162,7 @@
         <v>702</v>
       </c>
       <c r="G164" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H164" s="23" t="s">
         <v>703</v>
@@ -8248,7 +8248,7 @@
         <v>712</v>
       </c>
       <c r="G167" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H167" s="23" t="s">
         <v>713</v>
@@ -8614,7 +8614,7 @@
         <v>765</v>
       </c>
       <c r="G180" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H180" s="23" t="s">
         <v>766</v>
@@ -8642,7 +8642,7 @@
         <v>769</v>
       </c>
       <c r="G181" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H181" s="23" t="s">
         <v>770</v>
@@ -8672,7 +8672,7 @@
         <v>774</v>
       </c>
       <c r="G182" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H182" s="23" t="s">
         <v>775</v>
@@ -8700,7 +8700,7 @@
         <v>778</v>
       </c>
       <c r="G183" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H183" s="23" t="s">
         <v>779</v>
@@ -8728,7 +8728,7 @@
         <v>782</v>
       </c>
       <c r="G184" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H184" s="23" t="s">
         <v>783</v>
@@ -8816,7 +8816,7 @@
         <v>796</v>
       </c>
       <c r="G187" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H187" s="23" t="s">
         <v>797</v>
@@ -8876,7 +8876,7 @@
         <v>806</v>
       </c>
       <c r="G189" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H189" s="23" t="s">
         <v>807</v>
@@ -8962,7 +8962,7 @@
         <v>819</v>
       </c>
       <c r="G192" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H192" s="23" t="s">
         <v>820</v>
@@ -9104,7 +9104,7 @@
         <v>840</v>
       </c>
       <c r="G197" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H197" s="23" t="s">
         <v>841</v>
@@ -9132,7 +9132,7 @@
         <v>844</v>
       </c>
       <c r="G198" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H198" s="23" t="s">
         <v>845</v>
@@ -9186,7 +9186,7 @@
         <v>851</v>
       </c>
       <c r="G200" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H200" s="23" t="s">
         <v>852</v>
@@ -9214,7 +9214,7 @@
         <v>855</v>
       </c>
       <c r="G201" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H201" s="23" t="s">
         <v>856</v>
@@ -9242,7 +9242,7 @@
         <v>859</v>
       </c>
       <c r="G202" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H202" s="23" t="s">
         <v>860</v>
@@ -9300,7 +9300,7 @@
         <v>868</v>
       </c>
       <c r="G204" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H204" s="23" t="s">
         <v>869</v>
@@ -9328,7 +9328,7 @@
         <v>872</v>
       </c>
       <c r="G205" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H205" s="23" t="s">
         <v>873</v>
@@ -9358,7 +9358,7 @@
         <v>877</v>
       </c>
       <c r="G206" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H206" s="23" t="s">
         <v>878</v>
@@ -9640,7 +9640,7 @@
         <v>917</v>
       </c>
       <c r="G216" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H216" s="23" t="s">
         <v>918</v>
@@ -9696,7 +9696,7 @@
         <v>925</v>
       </c>
       <c r="G218" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H218" s="23" t="s">
         <v>926</v>
@@ -9754,7 +9754,7 @@
         <v>935</v>
       </c>
       <c r="G220" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H220" s="23" t="s">
         <v>936</v>
@@ -9784,7 +9784,7 @@
         <v>940</v>
       </c>
       <c r="G221" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H221" s="23" t="s">
         <v>941</v>
@@ -9866,7 +9866,7 @@
         <v>951</v>
       </c>
       <c r="G224" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H224" s="23" t="s">
         <v>952</v>
@@ -9894,7 +9894,7 @@
         <v>955</v>
       </c>
       <c r="G225" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H225" s="23" t="s">
         <v>956</v>
@@ -9924,7 +9924,7 @@
         <v>960</v>
       </c>
       <c r="G226" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H226" s="23" t="s">
         <v>961</v>
@@ -10006,7 +10006,7 @@
         <v>971</v>
       </c>
       <c r="G229" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H229" s="23" t="s">
         <v>972</v>
@@ -10034,7 +10034,7 @@
         <v>975</v>
       </c>
       <c r="G230" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H230" s="23" t="s">
         <v>976</v>
@@ -10116,7 +10116,7 @@
         <v>986</v>
       </c>
       <c r="G233" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H233" s="23" t="s">
         <v>987</v>
@@ -10144,7 +10144,7 @@
         <v>990</v>
       </c>
       <c r="G234" s="23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H234" s="23" t="s">
         <v>991</v>

</xml_diff>

<commit_message>
Stage 1 re-entry: correct pass-010 F-001..F-005 and pass-009 F-003
BA-001-12 bounded correction (operator Codex under the owner's
operational mandate; no new personal owner approval claimed):
correspondence claims narrowed to what is proven, with stated counting
rules and all three known divergent classes; note ids resolve to the
parent (rows 178-184); static editor date converters in the server
default locale and a first-request number parser (rows 69-71, 89, 186;
runtime Inferred); row 216 back to Inferred; the BA-001-11 record
inaccuracy recorded without rewriting it; the script-context counting
rule made reproducible (103/78). 10 rows changed; statuses
169/19/21/1 -> 168/20/21/1. WAR unchanged and authoritative.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -916,40 +916,40 @@
     <t>WAR:WEB-INF/classes/spring-beans.xml:60-69 (dataSource receives only ${hibernate.connection.driver_class}, url, username and password plus defaultAutoCommit) and :77-81 (sessionFactory AnnotationSessionFactoryBean with dataSource, packagesToScan and mappingLocations only; no hibernateProperties); no hibernate.properties or hibernate.cfg.xml in the WAR or at any JAR root (search; positive control ehcache-failsafe.xml in ehcache-1.2.3.jar). Consumers by name (.migration-tmp/stage-01/out/config-consumers-06.txt): hibernate.dialect only SystemInfo#getDatabaseInfo (display) and class com.technoetic.xplanner.db.hibernate.HibernateHelper#initializeConfiguration (Configuration.addProperties, a separate factory built only by #initializeHibernate, whose only outside caller is TomcatUserImporter#main); hibernate.show_sql only HsqlServer#isTraceOn; hibernate.query.substitutions only UseBeansTag#initializeQueryTranslations (the tag applies it to its own queries); hibernate.cache.* and hibernate.dbcp.* have no consumer. Keys: WAR:WEB-INF/classes/xplanner.properties:10,57-58,202-203,207-218; WAR:WEB-INF/classes/xplanner-custom.properties:15,19. Which dialect Hibernate picks and pool defaults are framework behavior (GAP-011). Provenance: all three files are rewritten entries (GAP-005 P-01, P-03, P-05). Source: stage-02-pass-004 F-003. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/db/hibernate/HibernateHelper.java HibernateHelper#initializeConfiguration. WAR: classes byte-identical to the v1.1a4 release; patched spring-beans.xml (WAR governs; the SVN copy is withheld). The source confirms that the property-file settings reach only the separate HibernateHelper configuration; which defaults the web session factory and pool then use is framework behavior. Live question: Does the running web application show no second-level or query cache and the default pool limits?</t>
   </si>
   <si>
-    <t>In the default, alternate (--), Danish, German, Japanese and Russian bundles, dates are displayed and entered as yyyy-MM-dd and date-times as yyyy-MM-dd HH:mm; the history view is an exception (row 186).</t>
+    <t>In the default, alternate (--), Danish, German, Japanese and Russian bundles, format.date is yyyy-MM-dd and format.datetime is yyyy-MM-dd HH:mm; they apply to the consumers that take the pattern from the session locale (the formatKey date displays, the calendar buttons and the saving of time entries). Exceptions: the history view (row 186), and the editor form converters, which validate and show dates with the patterns of the server default locale for every user (row 89).</t>
   </si>
   <si>
     <t>Date formats follow the UI locale bundle.</t>
   </si>
   <si>
-    <t>Date fields and calendar pickers use yyyy-MM-dd for these locales.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/classes/ResourceBundle.properties:8-9, ResourceBundle--.properties:5-6, ResourceBundle_da.properties:7-8, ResourceBundle_de.properties:8-9, ResourceBundle_ja.properties:12,14, ResourceBundle_ru.properties:9-10 (format.date, format.datetime); consumers editIteration.jsp, timesheet.jsp, editTimeEntries.jsp, UpdateTimeAction (format.date / format.datetime keys). Corrected in BA-001-03 (F-003): all 10 bundles compared. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag. WAR: the WAR bundles govern (the WAR copies of the da, es, fr, it and pt_br bundles differ from the SVN copies). The bundle patterns are confirmed for the format.date and format.datetime consumers, but not for every date display: the history view (history.jsp:61,106) uses xplanner:formatDate without a pattern, so FormatDateTag falls back to its built-in pattern "EEE MMM dd k:mm:ss z" (bytecode listing agrees). Resolves carried pass-009 F-002 statically; the observed format stays a live check. Live question: Which date format does the history view show after a fresh start for two sessions with different Accept-Language values?</t>
-  </si>
-  <si>
-    <t>In the Spanish, French, Italian and Brazilian Portuguese bundles, dates use dd-MM-yyyy; the Spanish date-time pattern is dd-MM-yyyy HH:MM, which uses the month letters in the minutes position; the history view is an exception (row 186).</t>
+    <t>Date displays with formatKey, the calendar buttons and saved time entries use yyyy-MM-dd in these session locales; editor validation and the iteration editor date fields use the server default locale's pattern (Inferred for the runtime effect).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/classes/ResourceBundle.properties:8-9, ResourceBundle--.properties:5-6, ResourceBundle_da.properties:7-8, ResourceBundle_de.properties:8-9, ResourceBundle_ja.properties:12,14, ResourceBundle_ru.properties:9-10 (format.date, format.datetime); consumers editIteration.jsp, timesheet.jsp, editTimeEntries.jsp, UpdateTimeAction (format.date / format.datetime keys). Corrected in BA-001-03 (F-003): all 10 bundles compared. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag. WAR: the WAR bundles govern (the WAR copies of the da, es, fr, it and pt_br bundles differ from the SVN copies). The bundle patterns are confirmed for the format.date and format.datetime consumers, but not for every date display: the history view (history.jsp:61,106) uses xplanner:formatDate without a pattern, so FormatDateTag falls back to its built-in pattern "EEE MMM dd k:mm:ss z" (bytecode listing agrees). Resolves carried pass-009 F-002 statically; the observed format stays a live check. Live question: Which date format does the history view show after a fresh start for two sessions with different Accept-Language values? Correction (BA-001-12, pass-010 F-003): narrowed to the session-locale consumers. The editor form converters are static: SRC:src/com/technoetic/xplanner/forms/AbstractEditorForm.java AbstractEditorForm#initConverters, #getResources, #convertToDate, #convertToDateTime fills dateConverter and dateTimeConverter once from format.date and format.datetime of the server default locale's bundle (Struts MessageResources#getMessage(String) passes no locale, so the default locale taken from Locale.getDefault() when the resources were constructed applies (struts-1.2.9.jar listing), and XPlannerMessageResources#getMessage hands that locale to the Spring message source; SRC:src/net/sf/xplanner/struts/XPlannerMessageResources.java XPlannerMessageResources#getMessage), and decimalConverter with SRC:src/com/technoetic/xplanner/format/DecimalFormat.java DecimalFormat#DecimalFormat, whose parser uses the Accept-Language locale of the first request that calls initConverters (IterationEditorForm#validate, TimeEditorForm#validate or IdSearchAction#doExecute). SRC:src/com/technoetic/xplanner/forms/TaskEditorForm.java TaskEditorForm#validate keeps its own static date converter built the same way. Consumers: SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate, #toString, #reset (start and end dates are shown and parsed with the static converter; reset clears it and the next initConverters call rebuilds it from the same server-default pattern), SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#valideRow (dates, date-times and durations), TaskEditorForm#validate (created date). Session-locale consumers: SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#getDateFormat, #getDateTimeFormat (saving time entries), the calendar buttons (WAR:WEB-INF/jsp/edit/editIteration.jsp:52-57) and the formatKey displays of FormatDateTag. Bytecode listings agree. The runtime effect is Inferred.</t>
+  </si>
+  <si>
+    <t>In the Spanish, French, Italian and Brazilian Portuguese bundles, format.date is dd-MM-yyyy; the Spanish format.datetime is dd-MM-yyyy HH:MM, which uses the month letters in the minutes position. They apply to the session-locale consumers (row 69); the history view (row 186) and the editor form converters (row 89) are exceptions.</t>
   </si>
   <si>
     <t>Locale-dependent date entry and display; the Spanish pattern prints the month where minutes are expected.</t>
   </si>
   <si>
-    <t>dd-MM-yyyy dates for these locales; Spanish date-times show the month number in place of minutes (runtime unverified).</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/classes/ResourceBundle_es.properties:7-8, ResourceBundle_fr.properties:5-6, ResourceBundle_it.properties:11-12, ResourceBundle_pt_br.properties:8-9. Source: stage-02-pass-001 F-003. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag. WAR: the WAR bundles govern (the WAR copies of the es, fr, it and pt_br bundles differ from the SVN copies). As row 69: the history view does not use these patterns. Resolves carried pass-009 F-002 statically.</t>
-  </si>
-  <si>
-    <t>The jQuery date picker attached to date fields always inserts yyyy-MM-dd, while the iteration editor calendar button and date parsing use the locale pattern; with a dd-MM-yyyy locale a date picked this way is expected to be rejected as invalid.</t>
+    <t>dd-MM-yyyy dates on the session-locale consumers for these locales; Spanish date-times show the month number in place of minutes (runtime unverified).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/classes/ResourceBundle_es.properties:7-8, ResourceBundle_fr.properties:5-6, ResourceBundle_it.properties:11-12, ResourceBundle_pt_br.properties:8-9. Source: stage-02-pass-001 F-003. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag. WAR: the WAR bundles govern (the WAR copies of the es, fr, it and pt_br bundles differ from the SVN copies). As row 69: the history view does not use these patterns. Resolves carried pass-009 F-002 statically. Correction (BA-001-12, pass-010 F-003): narrowed as row 69: the editor form converters use the server default locale's patterns, not these bundles, unless that is the server default locale.</t>
+  </si>
+  <si>
+    <t>The jQuery date picker attached to date fields always inserts yyyy-MM-dd, and the iteration editor calendar button inserts the session bundle's format.date, while the iteration editor parses both with the static converter built from the server default locale's format.date. Whether a picked date is accepted therefore depends on the server default locale, not the session locale; the converter is lenient, so a date in the other order is read as a different date rather than rejected (Inferred).</t>
   </si>
   <si>
     <t>Conflict between two date pickers for non-ISO locales.</t>
   </si>
   <si>
-    <t>Possible "Start date is invalid." after using the jQuery picker in es/fr/it/pt_br (runtime unverified).</t>
-  </si>
-  <si>
-    <t>WAR:js/global.js:39 (.dateField datepicker dateFormat yy-mm-dd); WAR:WEB-INF/jsp/edit/editIteration.jsp:54,57 (class dateField plus showCalendar with format.date); class IterationEditorForm#validate (iteration.editor.bad_start_date). Source: stage-02-pass-001 F-003. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release; js/global.js and editIteration.jsp identical to the SVN webapp copies. The picker format and the locale pattern are as recorded; whether a picked date is rejected is browser and locale behavior. Live question: In an es, fr, it or pt_br session, is a date picked with the jQuery picker rejected as "Start date is invalid."?</t>
+    <t>On a server whose default locale bundle uses yyyy-MM-dd, a date from the jQuery picker parses in every session, and a dd-MM-yyyy date from the calendar button of an es, fr, it or pt_br session is read with the server pattern as a different date; on a server with a dd-MM-yyyy default the reverse applies (runtime unverified).</t>
+  </si>
+  <si>
+    <t>WAR:js/global.js:39 (.dateField datepicker dateFormat yy-mm-dd); WAR:WEB-INF/jsp/edit/editIteration.jsp:54,57 (class dateField plus showCalendar with format.date); class IterationEditorForm#validate (iteration.editor.bad_start_date). Source: stage-02-pass-001 F-003. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release; js/global.js and editIteration.jsp identical to the SVN webapp copies. The picker format and the locale pattern are as recorded; whether a picked date is rejected is browser and locale behavior. Live question: In an es, fr, it or pt_br session, is a date picked with the jQuery picker rejected as "Start date is invalid."? Correction (BA-001-12, pass-010 F-003): the BA-001-11 note ("the locale pattern [is] as recorded") and its live question are superseded. The editor form converters are static: SRC:src/com/technoetic/xplanner/forms/AbstractEditorForm.java AbstractEditorForm#initConverters, #getResources, #convertToDate, #convertToDateTime fills dateConverter and dateTimeConverter once from format.date and format.datetime of the server default locale's bundle (Struts MessageResources#getMessage(String) passes no locale, so the default locale taken from Locale.getDefault() when the resources were constructed applies (struts-1.2.9.jar listing), and XPlannerMessageResources#getMessage hands that locale to the Spring message source; SRC:src/net/sf/xplanner/struts/XPlannerMessageResources.java XPlannerMessageResources#getMessage), and decimalConverter with SRC:src/com/technoetic/xplanner/format/DecimalFormat.java DecimalFormat#DecimalFormat, whose parser uses the Accept-Language locale of the first request that calls initConverters (IterationEditorForm#validate, TimeEditorForm#validate or IdSearchAction#doExecute). SRC:src/com/technoetic/xplanner/forms/TaskEditorForm.java TaskEditorForm#validate keeps its own static date converter built the same way. Consumers: SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate, #toString, #reset (start and end dates are shown and parsed with the static converter; reset clears it and the next initConverters call rebuilds it from the same server-default pattern), SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#valideRow (dates, date-times and durations), TaskEditorForm#validate (created date). Session-locale consumers: SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#getDateFormat, #getDateTimeFormat (saving time entries), the calendar buttons (WAR:WEB-INF/jsp/edit/editIteration.jsp:52-57) and the formatKey displays of FormatDateTag. Bytecode listings agree. The runtime effect is Inferred. New live question: on a server with a known default locale, which start date does the iteration editor store for a date from the jQuery picker and for one from the calendar button in an es session?</t>
   </si>
   <si>
     <t>Request parameters under /do/* are decoded as UTF-8.</t>
@@ -1174,7 +1174,7 @@
     <t>Messages "Missing iteration name.", "Start date is invalid.", "End date is invalid.", "Iteration must be a positive time interval."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.IterationEditorForm#validate (strings iteration.editor.missing_name, bad_start_date, bad_end_date) and #requirePositiveInterval (iteration.editor.nonpositive_interval); WAR:WEB-INF/classes/ResourceBundle.properties:265. Corrected in BA-001-04 (Source: stage-02-pass-002 F-001). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; iteration.editor.nonpositive_interval: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release. Name and both dates are required and the interval must be positive.</t>
+    <t>class com.technoetic.xplanner.forms.IterationEditorForm#validate (strings iteration.editor.missing_name, bad_start_date, bad_end_date) and #requirePositiveInterval (iteration.editor.nonpositive_interval); WAR:WEB-INF/classes/ResourceBundle.properties:265. Corrected in BA-001-04 (Source: stage-02-pass-002 F-001). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; iteration.editor.nonpositive_interval: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release. Name and both dates are required and the interval must be positive. Correction (BA-001-12, pass-010 F-003): the accepted date and date-time patterns are those of the server default locale's bundle, not of the active (session) bundle as stated above: IterationEditorForm#validate parses with the static converters. The editor form converters are static: SRC:src/com/technoetic/xplanner/forms/AbstractEditorForm.java AbstractEditorForm#initConverters, #getResources, #convertToDate, #convertToDateTime fills dateConverter and dateTimeConverter once from format.date and format.datetime of the server default locale's bundle (Struts MessageResources#getMessage(String) passes no locale, so the default locale taken from Locale.getDefault() when the resources were constructed applies (struts-1.2.9.jar listing), and XPlannerMessageResources#getMessage hands that locale to the Spring message source; SRC:src/net/sf/xplanner/struts/XPlannerMessageResources.java XPlannerMessageResources#getMessage), and decimalConverter with SRC:src/com/technoetic/xplanner/format/DecimalFormat.java DecimalFormat#DecimalFormat, whose parser uses the Accept-Language locale of the first request that calls initConverters (IterationEditorForm#validate, TimeEditorForm#validate or IdSearchAction#doExecute). SRC:src/com/technoetic/xplanner/forms/TaskEditorForm.java TaskEditorForm#validate keeps its own static date converter built the same way. Consumers: SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate, #toString, #reset (start and end dates are shown and parsed with the static converter; reset clears it and the next initConverters call rebuilds it from the same server-default pattern), SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#valideRow (dates, date-times and durations), TaskEditorForm#validate (created date). Session-locale consumers: SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#getDateFormat, #getDateTimeFormat (saving time entries), the calendar buttons (WAR:WEB-INF/jsp/edit/editIteration.jsp:52-57) and the formatKey displays of FormatDateTag. Bytecode listings agree. The runtime effect is Inferred.</t>
   </si>
   <si>
     <t>Edit iteration</t>
@@ -2290,7 +2290,7 @@
     <t>Results page "Search results - &lt;text&gt;" with type, ID, title (links to object or to the object a note is attached to) and match.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:22-35 (form /do/search/content, searchedContent, restrictToProjectId); WAR:WEB-INF/struts-config.xml:415-417; class ContentSearchAction (search.content.globalScopeEnable); WAR:WEB-INF/classes/xplanner.properties:287; WAR:WEB-INF/classes/spring-beans.xml:210-226; WAR:WEB-INF/jsp/view/searchResults.jsp. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute. WAR: classes byte-identical to the v1.1a4 release; search.content.globalScopeEnable=true in the WAR xplanner.properties. With the global scope the whole database is searched; a numeric search text also adds the object with that id first (row 180). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:22-35 (form /do/search/content, searchedContent, restrictToProjectId); WAR:WEB-INF/struts-config.xml:415-417; class ContentSearchAction (search.content.globalScopeEnable); WAR:WEB-INF/classes/xplanner.properties:287; WAR:WEB-INF/classes/spring-beans.xml:210-226; WAR:WEB-INF/jsp/view/searchResults.jsp. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute. WAR: classes byte-identical to the v1.1a4 release; search.content.globalScopeEnable=true in the WAR xplanner.properties. With the global scope the whole database is searched; a numeric search text also adds the object with that id first (row 180). Correction (BA-001-12, pass-010 F-002): the object added first for a numeric text is the one found by SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search; IdSearchHelper#search tries Project, Iteration, UserStory, Task, Person and Note in that order and, when the object is a Note, returns Note#getParent instead: the object whose id is the note's attached-to id, looked up the same way (a failed lookup gives null). For a note's id the parent object is added, not the note (SRC:src/net/sf/xplanner/domain/Note.java Note#getParent; SRC:src/com/technoetic/xplanner/tags/DomainContext.java DomainContext#getNoteTarget; SRC:src/com/technoetic/xplanner/db/OLDIdSearchHelper.java OLDIdSearchHelper#search; bytecode listings agree: instanceof Note, getParent; the thread session is bound by SRC:src/com/technoetic/xplanner/db/hibernate/HibernateSessionFilter.java HibernateSessionFilter#doFilter before the filter chain, mapped at /* (WAR:WEB-INF/web.xml:147-152)). See row 180. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
   </si>
   <si>
     <t>A search without results shows an empty-results message.</t>
@@ -2305,7 +2305,7 @@
     <t>WAR:WEB-INF/jsp/view/searchResults.jsp (empty.search.results). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
   </si>
   <si>
-    <t>Text matches are filtered to objects the searching user may read; a numeric search text also puts the object with that id at the top of the results, without a read check.</t>
+    <t>Text matches are filtered to objects the searching user may read; a numeric search text also puts the object with that id at the top of the results (for the id of a note, the note's parent object), without a read check.</t>
   </si>
   <si>
     <t>Search does not reveal items outside the user's permissions.</t>
@@ -2314,7 +2314,7 @@
     <t>Only readable matches are listed.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.db.ContentSearchHelper#search calls #excludeResultsBasedOnUserPermissions, which filters with #getAuthorizationPredicate -&gt; class com.technoetic.xplanner.actions.SearchResultAuthorizationPredicate#evaluate/#isResultReadableByUser (SystemAuthorizer.get, Authorizer.hasPermission, string "read"). Source: stage-02-pass-001 F-007. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/db/ContentSearchHelper.java ContentSearchHelper#search, #excludeResultsBasedOnUserPermissions; SRC:src/com/technoetic/xplanner/actions/SearchResultAuthorizationPredicate.java SearchResultAuthorizationPredicate#isResultReadableByUser; SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute; SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search. WAR: classes byte-identical to the v1.1a4 release; search.content.globalScopeEnable=true in the WAR xplanner.properties. Text matches are filtered by read permission. After the filter, when the search text is a number and the scope is global (the WAR value), ContentSearchAction adds the object with that id at the top of the results without a permission check (bytecode listing agrees).</t>
+    <t>class com.technoetic.xplanner.db.ContentSearchHelper#search calls #excludeResultsBasedOnUserPermissions, which filters with #getAuthorizationPredicate -&gt; class com.technoetic.xplanner.actions.SearchResultAuthorizationPredicate#evaluate/#isResultReadableByUser (SystemAuthorizer.get, Authorizer.hasPermission, string "read"). Source: stage-02-pass-001 F-007. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/db/ContentSearchHelper.java ContentSearchHelper#search, #excludeResultsBasedOnUserPermissions; SRC:src/com/technoetic/xplanner/actions/SearchResultAuthorizationPredicate.java SearchResultAuthorizationPredicate#isResultReadableByUser; SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute; SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search. WAR: classes byte-identical to the v1.1a4 release; search.content.globalScopeEnable=true in the WAR xplanner.properties. Text matches are filtered by read permission. After the filter, when the search text is a number and the scope is global (the WAR value), ContentSearchAction adds the object with that id at the top of the results without a permission check (bytecode listing agrees). Correction (BA-001-12, pass-010 F-002): method-level reading of the corrected claim: SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search; SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute (adds the returned object at position 0 when it is Nameable, with no authorizer call); SRC:src/net/sf/xplanner/domain/Note.java Note#getParent; SRC:src/com/technoetic/xplanner/tags/DomainContext.java DomainContext#getNoteTarget; SRC:src/com/technoetic/xplanner/db/OLDIdSearchHelper.java OLDIdSearchHelper#search. IdSearchHelper#search tries Project, Iteration, UserStory, Task, Person and Note in that order and, when the object is a Note, returns Note#getParent instead: the object whose id is the note's attached-to id, looked up the same way (a failed lookup gives null). Bytecode listings agree; the thread session is bound by SRC:src/com/technoetic/xplanner/db/hibernate/HibernateSessionFilter.java HibernateSessionFilter#doFilter before the filter chain, mapped at /* (WAR:WEB-INF/web.xml:147-152). Status stays Yes on this reading.</t>
   </si>
   <si>
     <t>Submitting an empty search yields an error.</t>
@@ -2332,16 +2332,16 @@
     <t>Jump to object by ID</t>
   </si>
   <si>
-    <t>Searching by a numeric ID in the header search lists the matching project, iteration, story, task, person or note first among the results; the direct jump (/do/search/id) is reachable by URL only.</t>
+    <t>Searching by a numeric ID in the header search lists the matching project, iteration, story, task or person first among the results, and for the id of a note the note's parent object; the direct jump (/do/search/id) is reachable by URL only.</t>
   </si>
   <si>
     <t>Direct navigation by ID ("search by word or ID").</t>
   </si>
   <si>
-    <t>Search results headed by the object with that id; a request to /do/search/id?searchedId=&lt;id&gt; redirects to /do/view/&lt;type&gt;?oid=&lt;id&gt;.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:46 (tooltip "search by word or ID"); class ContentSearchAction (setIdSearchHelper); class IdSearchAction (strings "/do/view/", "?oid="); WAR:WEB-INF/struts-config.xml:141,413 (search/id). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute; SRC:src/com/technoetic/xplanner/actions/IdSearchAction.java IdSearchAction#doExecute. WAR: classes byte-identical to the v1.1a4 release; baseHeader.jsp of the WAR (differs from the SVN copy; WAR governs). The header search box posts to /do/search/content: a numeric text lists the object with that id first among the search results, without a redirect. The redirecting ID search (/do/search/id, IdSearchAction) is linked from no page of the WAR.</t>
+    <t>Search results headed by the object with that id (for a note's id, the note's parent); a request to /do/search/id?searchedId=&lt;id&gt; redirects to /do/view/&lt;type&gt;?oid=&lt;id&gt; of the found object, which for a note's id are the parent's type and id.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:46 (tooltip "search by word or ID"); class ContentSearchAction (setIdSearchHelper); class IdSearchAction (strings "/do/view/", "?oid="); WAR:WEB-INF/struts-config.xml:141,413 (search/id). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute; SRC:src/com/technoetic/xplanner/actions/IdSearchAction.java IdSearchAction#doExecute. WAR: classes byte-identical to the v1.1a4 release; baseHeader.jsp of the WAR (differs from the SVN copy; WAR governs). The header search box posts to /do/search/content: a numeric text lists the object with that id first among the search results, without a redirect. The redirecting ID search (/do/search/id, IdSearchAction) is linked from no page of the WAR. Correction (BA-001-12, pass-010 F-002): method-level reading of the corrected claim: SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search; SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute; SRC:src/com/technoetic/xplanner/actions/IdSearchAction.java IdSearchAction#doExecute (builds the redirect from the class of the returned object through DomainMetaDataRepository#classToTypeName and from its getId); SRC:src/net/sf/xplanner/domain/Note.java Note#getParent; SRC:src/com/technoetic/xplanner/tags/DomainContext.java DomainContext#getNoteTarget; SRC:src/com/technoetic/xplanner/db/OLDIdSearchHelper.java OLDIdSearchHelper#search. IdSearchHelper#search tries Project, Iteration, UserStory, Task, Person and Note in that order and, when the object is a Note, returns Note#getParent instead: the object whose id is the note's attached-to id, looked up the same way (a failed lookup gives null). Bytecode listings agree; the thread session is bound by SRC:src/com/technoetic/xplanner/db/hibernate/HibernateSessionFilter.java HibernateSessionFilter#doFilter before the filter chain, mapped at /* (WAR:WEB-INF/web.xml:147-152). Status stays Yes on this reading.</t>
   </si>
   <si>
     <t>A missing, malformed or unknown ID shows an error.</t>
@@ -2362,10 +2362,10 @@
     <t>Differs from the filtered text search. Observed behavior and risk only (Q3 deferred).</t>
   </si>
   <si>
-    <t>Any existing object ID opens its page for any signed-in user (runtime unverified).</t>
-  </si>
-  <si>
-    <t>classes IdSearchAction and ViewObjectAction: no authorization call reachable (.migration-tmp/stage-01/out/authtrace.json). BA-001-03 impact sweep of F-001 and F-007. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/IdSearchAction.java IdSearchAction#doExecute; SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search; SRC:src/com/technoetic/xplanner/actions/ViewObjectAction.java ViewObjectAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. Neither the ID search nor the view action calls an authorizer.</t>
+    <t>Any existing object ID opens the page of that object, or for a note's ID the page of the note's parent, for any signed-in user (runtime unverified).</t>
+  </si>
+  <si>
+    <t>classes IdSearchAction and ViewObjectAction: no authorization call reachable (.migration-tmp/stage-01/out/authtrace.json). BA-001-03 impact sweep of F-001 and F-007. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/IdSearchAction.java IdSearchAction#doExecute; SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search; SRC:src/com/technoetic/xplanner/actions/ViewObjectAction.java ViewObjectAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. Neither the ID search nor the view action calls an authorizer. Correction (BA-001-12, pass-010 F-002): the page opened is that of the object returned by SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search; for a note's id this is the note's parent (SRC:src/net/sf/xplanner/domain/Note.java Note#getParent; SRC:src/com/technoetic/xplanner/tags/DomainContext.java DomainContext#getNoteTarget; SRC:src/com/technoetic/xplanner/db/OLDIdSearchHelper.java OLDIdSearchHelper#search). The missing read check is unchanged.</t>
   </si>
   <si>
     <t>Breadcrumb navigation</t>
@@ -2392,10 +2392,10 @@
     <t>Audit trail of recorded changes.</t>
   </si>
   <si>
-    <t>Sortable history table; the container view adds object type and name links. The "when" dates use the built-in pattern "EEE MMM dd k:mm:ss z" in the Accept-Language locale of the first request after start-up, for every later user (Inferred).</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/project.jsp:99-104, iteration/globalLinks.jsp:41-45, userstory.jsp, task.jsp (links /do/view/history, container flag for projects); WAR:WEB-INF/struts-config.xml:396-398; WAR:WEB-INF/jsp/view/history.jsp:30-32 (HistorySupport#getEvents) and :71-73 (#getContainerEvents); class com.technoetic.xplanner.history.HistorySupport#getContainerEvents (strings "created", "deleted"); WAR:WEB-INF/classes/spring-dao.xml:63-65 (historySupport); db-changelog.xml table history. Corrected in BA-001-03 (stage-02-pass-001 F-002). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/history/HistorySupport.java HistorySupport#getEvents, #getContainerEvents; SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag. WAR: classes byte-identical to the v1.1a4 release; history.jsp of the WAR (differs from the SVN copy, which calls HistorySupport statically; the WAR page calls the historySupport bean; WAR governs). The "when" column (history.jsp:61,106) uses xplanner:formatDate without format or formatKey: FormatDateTag uses its built-in pattern "EEE MMM dd k:mm:ss z" and keeps one SimpleDateFormat per pattern in a static, unsynchronized map, created with request.getLocale() (Accept-Language) of the first request after start-up, so later users see day and month names in that first locale (bytecode listing agrees). Resolves carried pass-009 F-002 statically (Inferred for the runtime effect). Live question: After a fresh start, which language do the history dates show for a second session with a different Accept-Language?</t>
+    <t>Sortable history table; the container view adds object type and name links. The "when" dates use the built-in pattern "EEE MMM dd k:mm:ss z" in the Accept-Language locale of the first request after start-up that renders a history date, for every later user (Inferred).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/project.jsp:99-104, iteration/globalLinks.jsp:41-45, userstory.jsp, task.jsp (links /do/view/history, container flag for projects); WAR:WEB-INF/struts-config.xml:396-398; WAR:WEB-INF/jsp/view/history.jsp:30-32 (HistorySupport#getEvents) and :71-73 (#getContainerEvents); class com.technoetic.xplanner.history.HistorySupport#getContainerEvents (strings "created", "deleted"); WAR:WEB-INF/classes/spring-dao.xml:63-65 (historySupport); db-changelog.xml table history. Corrected in BA-001-03 (stage-02-pass-001 F-002). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/history/HistorySupport.java HistorySupport#getEvents, #getContainerEvents; SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag. WAR: classes byte-identical to the v1.1a4 release; history.jsp of the WAR (differs from the SVN copy, which calls HistorySupport statically; the WAR page calls the historySupport bean; WAR governs). The "when" column (history.jsp:61,106) uses xplanner:formatDate without format or formatKey: FormatDateTag uses its built-in pattern "EEE MMM dd k:mm:ss z" and keeps one SimpleDateFormat per pattern in a static, unsynchronized map, created with request.getLocale() (Accept-Language) of the first request after start-up, so later users see day and month names in that first locale (bytecode listing agrees). Resolves carried pass-009 F-002 statically (Inferred for the runtime effect). Live question: After a fresh start, which language do the history dates show for a second session with a different Accept-Language? Correction (BA-001-12, pass-010 F-003): the formatter for the built-in pattern is created by the first request that renders a history date (the only formatDate uses without format or formatKey are WAR:WEB-INF/jsp/view/history.jsp:61,106), not by the first request after start-up. SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag.</t>
   </si>
   <si>
     <t>History is written only by these entry points: web iteration start and close, story move/continue (including multi-move and continue unfinished stories), task move/continue and task re-estimate; and every SOAP add, update and remove ("created", "updated", "deleted"). Web create, edit and delete of projects, iterations, stories, tasks, notes, people and settings write no history.</t>
@@ -2770,7 +2770,7 @@
     <t>SOAP reachable without the filter at the alternate path (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:298-301 (servlet-mapping /servlet/AxisServlet) versus filter mappings :168-176 (/soap/*, /ical/* only). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact); status Inferred -&gt; Yes. none: descriptor fact, no Java involved. WAR: web.xml identical to the SVN webapp copy. The servlet mapping /servlet/AxisServlet has no security filter mapping.</t>
+    <t>WAR:WEB-INF/web.xml:298-301 (servlet-mapping /servlet/AxisServlet) versus filter mappings :168-176 (/soap/*, /ical/* only). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact); status Inferred -&gt; Yes. none: descriptor fact, no Java involved. WAR: web.xml identical to the SVN webapp copy. The servlet mapping /servlet/AxisServlet has no security filter mapping. Correction (BA-001-12, pass-010 F-004): the BA-001-11 change to Yes had no evidence that was new since the Inferred status. Its only basis is the descriptor fact already cited (WAR:WEB-INF/web.xml:168-176,299-302); no method-level reading of the Axis servlet or of its handler chain was made, and no rule permits a descriptor-only status change. Status returned Yes -&gt; Inferred; the descriptor fact stands.</t>
   </si>
   <si>
     <t>An Axis "Version" service reports the Axis version.</t>
@@ -9640,7 +9640,7 @@
         <v>917</v>
       </c>
       <c r="G216" s="23" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="H216" s="23" t="s">
         <v>918</v>

</xml_diff>

<commit_message>
Stage 1 correction BA-001-13 from Stage 3 walkthrough W001
Apply the bounded 88-item map-correction list of the live walkthrough W001 to
the parity map and the reconnaissance (81 applied, 7 in part, 0 rejected;
no new research). Column G: 37 status changes on live evidence (27 Yes and
5 Inferred to Partial where the claim fails live; 5 Inferred to Yes where the
whole claim was observed); statuses 146 Yes, 10 Inferred, 53 Partial, 1 No.
Every business row's notes now carry its W001 live verdict and check IDs.
PM formatting-only link fix in its own assignment section after authoring.
Next: one fresh independent Stage 2 correction-validation.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1451" uniqueCount="992">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1451" uniqueCount="993">
   <si>
     <t>Legacy Project - User Flows from Golden Code</t>
   </si>
@@ -124,13 +124,13 @@
     <t>Only registered people may use the planning tool; signing in establishes their identity for authorization and time tracking.</t>
   </si>
   <si>
-    <t>Login form (User ID, Password, Remember me, Log In button); after success the browser is redirected to /do/view/projects.</t>
+    <t>Login form (User ID, Password, "Remember me?" checkbox, Login button); after success the browser is redirected to /do/view/projects.</t>
   </si>
   <si>
     <t>Yes</t>
   </si>
   <si>
-    <t>WAR: = paths inside legacy/xplanner-plus.war. WAR:WEB-INF/struts-config.xml:164-167 (/login, forwards notAuthenticated -&gt; WEB-INF/jsp/security/login.jsp, authenticated -&gt; /do/view/projects redirect); WAR:WEB-INF/action-servlet.xml:10 (AuthenticationAction); WAR:WEB-INF/jsp/security/login.jsp:16-33; class com.technoetic.xplanner.actions.AuthenticationAction#execute (calls Authenticator.authenticate, forward "authenticated"). Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; login.label and login.remember are defined in the default, "--", de, it, ja and ru bundles; login.label.user_id and login.label.password in all bundles except fr; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Page-text keys (BA-001-09, pass-007 F-003, check (j)): the login page also renders login.title, given as titleKey (WAR:WEB-INF/jsp/security/login.jsp:14; defined in all bundles except fr). Through the tiles:default layout that xplanner:content inserts (class ContentTag#doStartTag; WAR:WEB-INF/tiles-definitions.xml:5-10) it also renders the footer keys app.label.version (all 10 bundles) and footer.message (only the default, "--" and de bundles; WAR:WEB-INF/jsp/common/footer.jsp:25,38) and the breadcrumb link text navigation.top (all 10 bundles; WAR:WEB-INF/jsp/layout/defaultLayout.jsp:44, WAR:WEB-INF/tags/breadcrumb.tag:10, class net.sf.xplanner.tags.NavigationBarTag#render). Bundles without a key fall back to the default text (framework behavior, GAP-011). None of these texts is credential-like (.migration-tmp/stage-01/out/public-keys-09.txt). Breadcrumb lookup (BA-001-10, pass-008 F-002 lead, check (l)): on this page the layout breadcrumb (WAR:WEB-INF/jsp/layout/defaultLayout.jsp:44, WAR:WEB-INF/tags/breadcrumb.tag:10) reads the request parameter oid, or else fkey, and loads that object without a sign-in or permission check (class net.sf.xplanner.tags.NavigationBarTag#doEndTag, #setObject(int): the type attribute arrives as an empty string, so IdSearchHelper#search runs Session#get over Project, Iteration, UserStory, Task, Person and Note). #render then adds links whose texts are the names of the object's project, iteration, story, task or feature, and breadcrumb.tag:15,18 prints them with unescaped EL. /do/login is in the security bypass list (WAR:WEB-INF/security.xml:3), so /do/login?oid=&lt;id&gt; is expected to show those names, including any markup stored in them, to a visitor who has not signed in (Inferred; the EL coercion and runtime are unverified; row 185; GAP-007; observed risk only, Q3 deferred). Page-text scope (BA-001-10): the 45 keys are the keys named by the page and layout chain; after a failed login the page also shows messages queued in code (WAR:WEB-INF/jsp/security/login.jsp:50-59): login.failed and 9 authentication.module.message.* keys named in the class bytecode, of which rows 12-13 describe the ones the XPlanner login module produces. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/AuthenticationAction.java AuthenticationAction#execute (withheld file, cited by path only). WAR: classes byte-identical to the v1.1a4 release. After a successful authentication without a saved URL the action returns the authenticated forward.</t>
+    <t>WAR: = paths inside legacy/xplanner-plus.war. WAR:WEB-INF/struts-config.xml:164-167 (/login, forwards notAuthenticated -&gt; WEB-INF/jsp/security/login.jsp, authenticated -&gt; /do/view/projects redirect); WAR:WEB-INF/action-servlet.xml:10 (AuthenticationAction); WAR:WEB-INF/jsp/security/login.jsp:16-33; class com.technoetic.xplanner.actions.AuthenticationAction#execute (calls Authenticator.authenticate, forward "authenticated"). Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; login.label and login.remember are defined in the default, "--", de, it, ja and ru bundles; login.label.user_id and login.label.password in all bundles except fr; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Page-text keys (BA-001-09, pass-007 F-003, check (j)): the login page also renders login.title, given as titleKey (WAR:WEB-INF/jsp/security/login.jsp:14; defined in all bundles except fr). Through the tiles:default layout that xplanner:content inserts (class ContentTag#doStartTag; WAR:WEB-INF/tiles-definitions.xml:5-10) it also renders the footer keys app.label.version (all 10 bundles) and footer.message (only the default, "--" and de bundles; WAR:WEB-INF/jsp/common/footer.jsp:25,38) and the breadcrumb link text navigation.top (all 10 bundles; WAR:WEB-INF/jsp/layout/defaultLayout.jsp:44, WAR:WEB-INF/tags/breadcrumb.tag:10, class net.sf.xplanner.tags.NavigationBarTag#render). Bundles without a key fall back to the default text (framework behavior, GAP-011). None of these texts is credential-like (.migration-tmp/stage-01/out/public-keys-09.txt). Breadcrumb lookup (BA-001-10, pass-008 F-002 lead, check (l)): on this page the layout breadcrumb (WAR:WEB-INF/jsp/layout/defaultLayout.jsp:44, WAR:WEB-INF/tags/breadcrumb.tag:10) reads the request parameter oid, or else fkey, and loads that object without a sign-in or permission check (class net.sf.xplanner.tags.NavigationBarTag#doEndTag, #setObject(int): the type attribute arrives as an empty string, so IdSearchHelper#search runs Session#get over Project, Iteration, UserStory, Task, Person and Note). #render then adds links whose texts are the names of the object's project, iteration, story, task or feature, and breadcrumb.tag:15,18 prints them with unescaped EL. /do/login is in the security bypass list (WAR:WEB-INF/security.xml:3), so /do/login?oid=&lt;id&gt; is expected to show those names, including any markup stored in them, to a visitor who has not signed in (Inferred; the EL coercion and runtime are unverified; row 185; GAP-007; observed risk only, Q3 deferred). Page-text scope (BA-001-10): the 45 keys are the keys named by the page and layout chain; after a failed login the page also shows messages queued in code (WAR:WEB-INF/jsp/security/login.jsp:50-59): login.failed and 9 authentication.module.message.* keys named in the class bytecode, of which rows 12-13 describe the ones the XPlanner login module produces. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/AuthenticationAction.java AuthenticationAction#execute (withheld file, cited by path only). WAR: classes byte-identical to the v1.1a4 release. After a successful authentication without a saved URL the action returns the authenticated forward. Stage 3 W001 (BA-001-13, MC-A-02, W001-F-02): without a session, GET /do/login?oid=220 (project S3 Shared) answered HTTP 200 and the page did not contain the name "S3 Shared" (L-C-001; PM presence flag only). The expected name exposure was not observed for a project object. Other object types, the fkey variant and stored markup were not requested, so the lookup claim above stays Inferred for them. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-009, setup-C-010, setup-C-011, setup-C-012, setup-C-013, A-C-001, A-C-002, L-C-001).</t>
   </si>
   <si>
     <t>Alternative path</t>
@@ -145,7 +145,7 @@
     <t>Help text "login.instructions" with a link; the effective override file sets the URL to the XPlanner+ documentation site. With the default bundle, and with every bundle that has no own key, the text ends with the default administrator login pair (value not reproduced, CHK-009).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/security/login.jsp:34-39 (XPlannerProperties.getProperty("login.instructions.url")); WAR:WEB-INF/classes/xplanner-custom.properties:49 (login.instructions.url set) overriding WAR:WEB-INF/classes/xplanner.properties:311 (empty); override order per class com.technoetic.xplanner.XPlannerProperties$PropertyInitializer (strings "xplanner.properties", "xplanner.overrides", "xplanner-custom.properties"). Credential disclosure (BA-001-06): WAR:WEB-INF/jsp/security/login.jsp:34-39 renders bean:message login.instructions with arg0 = login.instructions.url when that URL is not empty; WAR:WEB-INF/classes/ResourceBundle.properties:784 ends with a sentence naming the default login name and password. Checked in memory without writing the value: the name equals the userId seeded at WAR:WEB-INF/classes/db-changelog.xml:403, and MD5(salt, password) matches the seeded digest at :404 (layout Base64 of a 12-byte salt followed by the digest, class XPlannerLoginModule#isPasswordMatched, #digestPassword). Locale variants (CHK-004, BA-001-06): login.instructions is defined only in the default bundle (:784, with the credential sentence), ResourceBundle--.properties:780 and ResourceBundle_de.properties:753 (both without it); da, es, fr, it, ja, pt_br and ru have no key and are expected to fall back to the default text (framework behavior, GAP-011). Whether earlier installations still accepted this pair is not established. Corrected in BA-001-06 (Source: stage-02-pass-004 F-001). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/XPlannerProperties.java XPlannerProperties; SRC:src/com/technoetic/xplanner/security/module/XPlannerLoginModule.java XPlannerLoginModule#isPasswordMatched (withheld file, cited by path only). WAR: classes byte-identical to the v1.1a4 release; values from the patched WAR xplanner.properties, xplanner-custom.properties (WAR governs); the WAR db-changelog.xml differs from the SVN copy, which is withheld (WAR governs). The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-04: the cited value is read from xplanner-custom.properties (rewritten entry, known patch target); upstream value not determinable.</t>
+    <t>WAR:WEB-INF/jsp/security/login.jsp:34-39 (XPlannerProperties.getProperty("login.instructions.url")); WAR:WEB-INF/classes/xplanner-custom.properties:49 (login.instructions.url set) overriding WAR:WEB-INF/classes/xplanner.properties:311 (empty); override order per class com.technoetic.xplanner.XPlannerProperties$PropertyInitializer (strings "xplanner.properties", "xplanner.overrides", "xplanner-custom.properties"). Credential disclosure (BA-001-06): WAR:WEB-INF/jsp/security/login.jsp:34-39 renders bean:message login.instructions with arg0 = login.instructions.url when that URL is not empty; WAR:WEB-INF/classes/ResourceBundle.properties:784 ends with a sentence naming the default login name and password. Checked in memory without writing the value: the name equals the userId seeded at WAR:WEB-INF/classes/db-changelog.xml:403, and MD5(salt, password) matches the seeded digest at :404 (layout Base64 of a 12-byte salt followed by the digest, class XPlannerLoginModule#isPasswordMatched, #digestPassword). Locale variants (CHK-004, BA-001-06): login.instructions is defined only in the default bundle (:784, with the credential sentence), ResourceBundle--.properties:780 and ResourceBundle_de.properties:753 (both without it); da, es, fr, it, ja, pt_br and ru have no key and are expected to fall back to the default text (framework behavior, GAP-011). Whether earlier installations still accepted this pair is not established. Corrected in BA-001-06 (Source: stage-02-pass-004 F-001). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/XPlannerProperties.java XPlannerProperties; SRC:src/com/technoetic/xplanner/security/module/XPlannerLoginModule.java XPlannerLoginModule#isPasswordMatched (withheld file, cited by path only). WAR: classes byte-identical to the v1.1a4 release; values from the patched WAR xplanner.properties, xplanner-custom.properties (WAR governs); the WAR db-changelog.xml differs from the SVN copy, which is withheld (WAR governs). The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-04: the cited value is read from xplanner-custom.properties (rewritten entry, known patch target); upstream value not determinable. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-003, A-C-004, L-C-002).</t>
   </si>
   <si>
     <t>After login the user is returned to the protected page they originally requested, when one was saved.</t>
@@ -157,7 +157,7 @@
     <t>Browser lands on the originally requested GET URL instead of the projects list; a URL that had no query string is saved and restored with the suffix "?null".</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.security.filter.FormSecurityFilter#onAuthenticationFailure (checks "GET", calls SecurityHelper.saveUrl, sendRedirect); class com.technoetic.xplanner.actions.AuthenticationAction#execute (calls SecurityHelper.getSavedUrl, new ActionForward(url, redirect)). Control flow not decompiled. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/filter/FormSecurityFilter.java FormSecurityFilter#onAuthenticationFailure; SRC:src/com/technoetic/xplanner/actions/AuthenticationAction.java AuthenticationAction#execute (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/SecurityHelper.java SecurityHelper#saveUrl, #getSavedUrl. WAR: classes byte-identical to the v1.1a4 release. The filter saves the request URL for GET requests only and redirects to the login page; after a successful login the action redirects to the saved URL when one is present. The saveUrl bytecode listing appends "?" and the query string unconditionally, as the source does, so a URL without a query string is saved with the suffix "?null".</t>
+    <t>class com.technoetic.xplanner.security.filter.FormSecurityFilter#onAuthenticationFailure (checks "GET", calls SecurityHelper.saveUrl, sendRedirect); class com.technoetic.xplanner.actions.AuthenticationAction#execute (calls SecurityHelper.getSavedUrl, new ActionForward(url, redirect)). Control flow not decompiled. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/filter/FormSecurityFilter.java FormSecurityFilter#onAuthenticationFailure; SRC:src/com/technoetic/xplanner/actions/AuthenticationAction.java AuthenticationAction#execute (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/SecurityHelper.java SecurityHelper#saveUrl, #getSavedUrl. WAR: classes byte-identical to the v1.1a4 release. The filter saves the request URL for GET requests only and redirects to the login page; after a successful login the action redirects to the saved URL when one is present. The saveUrl bytecode listing appends "?" and the query string unconditionally, as the source does, so a URL without a query string is saved with the suffix "?null". Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-005, A-C-006).</t>
   </si>
   <si>
     <t>The configured login module (XPlanner database module) validates the password against a salted MD5 digest stored for the person; the userIdCaseSensitive option is read by no live code, so whether the user ID must match in letter case is decided by the database comparison.</t>
@@ -172,7 +172,7 @@
     <t>Inferred</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/xplanner.properties:162-164 (login[0] = XPlannerLoginModule, userIdCaseSensitive=true); class com.technoetic.xplanner.security.module.XPlannerLoginModule#isPasswordMatched/#digestPassword (strings "MD5", Base64.decode); class com.technoetic.xplanner.security.module.LoginSupportImpl#getPerson (HQL "from person ... where userid = ?"). Query form (BA-001-05): LoginSupportImpl#getPerson queries "from person in class net.sf.xplanner.domain.Person where userid = ?" with the unqualified name userid, while Person maps userId (column userId). Whether the name is passed to SQL unchanged, and matched case-insensitively by the database, is framework and database behavior (GAP-011, P-01). Sweep of pass-003 F-001. Digest layout (BA-001-06): #isPasswordMatched Base64-decodes the stored value, takes the first 12 bytes as salt and compares MD5 over salt then the UTF-8 password with the rest (bytecode listing). Source: stage-02-pass-004 F-001. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/security/module/XPlannerLoginModule.java XPlannerLoginModule#authenticate, #isPasswordMatched, #digestPassword (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/module/LoginSupportImpl.java LoginSupportImpl#getPerson; SRC:src/com/technoetic/xplanner/security/SecurityHelper.java SecurityHelper#isAuthenticationCaseSensitive; SRC:src/com/technoetic/xplanner/domain/repository/PersonHibernateObjectRepository.java PersonHibernateObjectRepository#hasSameUserId. WAR: classes byte-identical to the v1.1a4 release; login-module keys from the patched WAR xplanner.properties (WAR governs). The salted digest check is confirmed (12-byte salt, digest over salt and password, byte comparison). The case-sensitivity claim is not: the userIdCaseSensitive option is read only by SecurityHelper#isAuthenticationCaseSensitive, whose only use is commented out in PersonHibernateObjectRepository#hasSameUserId (the bytecode has no caller either); the login query compares the user ID with an HQL equality, so case matching is decided by the database comparison. Live question: Does a login with the seeded user ID in different letter case succeed against the MySQL database? Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/classes/xplanner.properties:162-164 (login[0] = XPlannerLoginModule, userIdCaseSensitive=true); class com.technoetic.xplanner.security.module.XPlannerLoginModule#isPasswordMatched/#digestPassword (strings "MD5", Base64.decode); class com.technoetic.xplanner.security.module.LoginSupportImpl#getPerson (HQL "from person ... where userid = ?"). Query form (BA-001-05): LoginSupportImpl#getPerson queries "from person in class net.sf.xplanner.domain.Person where userid = ?" with the unqualified name userid, while Person maps userId (column userId). Whether the name is passed to SQL unchanged, and matched case-insensitively by the database, is framework and database behavior (GAP-011, P-01). Sweep of pass-003 F-001. Digest layout (BA-001-06): #isPasswordMatched Base64-decodes the stored value, takes the first 12 bytes as salt and compares MD5 over salt then the UTF-8 password with the rest (bytecode listing). Source: stage-02-pass-004 F-001. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/security/module/XPlannerLoginModule.java XPlannerLoginModule#authenticate, #isPasswordMatched, #digestPassword (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/module/LoginSupportImpl.java LoginSupportImpl#getPerson; SRC:src/com/technoetic/xplanner/security/SecurityHelper.java SecurityHelper#isAuthenticationCaseSensitive; SRC:src/com/technoetic/xplanner/domain/repository/PersonHibernateObjectRepository.java PersonHibernateObjectRepository#hasSameUserId. WAR: classes byte-identical to the v1.1a4 release; login-module keys from the patched WAR xplanner.properties (WAR governs). The salted digest check is confirmed (12-byte salt, digest over salt and password, byte comparison). The case-sensitivity claim is not: the userIdCaseSensitive option is read only by SecurityHelper#isAuthenticationCaseSensitive, whose only use is commented out in PersonHibernateObjectRepository#hasSameUserId (the bytecode has no caller either); the login query compares the user ID with an HQL equality, so case matching is decided by the database comparison. Live question: Does a login with the seeded user ID in different letter case succeed against the MySQL database? Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. Stage 3 W001 live answer (BA-001-13, MC-C-06): Yes: an upper-case user ID signed in (302 to the projects list); the header then shows the stored lower-case ID. Depends on the database comparison; observed on MySQL 5.7 (A-C-007). The status stays Inferred: the digest and option claims are static. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-007).</t>
   </si>
   <si>
     <t>Login rejected</t>
@@ -187,7 +187,7 @@
     <t>Login page redisplayed with "Could not authenticate user." plus a module message such as "Wrong userid or password".</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/security/login.jsp:50-59 (GLOBAL_MESSAGE and moduleMessages); class AuthenticationAction#execute (strings "login.failed", "moduleMessages", forward "notAuthenticated"); WAR:WEB-INF/classes/ResourceBundle.properties keys login.failed, authentication.module.message.authenticationFailed. Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; login.failed is defined in all bundles except fr; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/AuthenticationAction.java AuthenticationAction#execute (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/LoginContext.java LoginContext#authenticate. WAR: classes byte-identical to the v1.1a4 release. A failed authentication adds the global login-failed message and one message per module, and returns the login page.</t>
+    <t>WAR:WEB-INF/jsp/security/login.jsp:50-59 (GLOBAL_MESSAGE and moduleMessages); class AuthenticationAction#execute (strings "login.failed", "moduleMessages", forward "notAuthenticated"); WAR:WEB-INF/classes/ResourceBundle.properties keys login.failed, authentication.module.message.authenticationFailed. Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; login.failed is defined in all bundles except fr; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/AuthenticationAction.java AuthenticationAction#execute (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/LoginContext.java LoginContext#authenticate. WAR: classes byte-identical to the v1.1a4 release. A failed authentication adds the global login-failed message and one message per module, and returns the login page. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-008).</t>
   </si>
   <si>
     <t>An unknown user ID or a person without a password produces a specific module message.</t>
@@ -199,19 +199,19 @@
     <t>Messages "User has not been registered with XPlanner..." or "Password has not been set...".</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.security.module.LoginSupportImpl#populateSubjectPrincipalFromDatabase (string "authentication.module.message.userNotFound"); class XPlannerLoginModule#isPasswordMatched (string "authentication.module.message.passwordNotSet"); ResourceBundle.properties same keys. Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; authentication.module.message.userNotFound and passwordNotSet are defined only in the default, "--", de and ja bundles; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/module/LoginSupportImpl.java LoginSupportImpl#populateSubjectPrincipalFromDatabase; SRC:src/com/technoetic/xplanner/security/module/XPlannerLoginModule.java XPlannerLoginModule#isPasswordMatched (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/LoginContext.java LoginContext#authenticate. WAR: classes byte-identical to the v1.1a4 release. A missing person raises the user-not-found key and a null stored password raises the password-not-set key; LoginContext#authenticate collects each module's message key per module name, and the action shows them as module messages.</t>
-  </si>
-  <si>
-    <t>A request to the login action without the submit field (for example a plain GET of /do/login) shows the login form; empty user ID or password values are not checked by the action and are passed to the login module, which rejects them.</t>
+    <t>class com.technoetic.xplanner.security.module.LoginSupportImpl#populateSubjectPrincipalFromDatabase (string "authentication.module.message.userNotFound"); class XPlannerLoginModule#isPasswordMatched (string "authentication.module.message.passwordNotSet"); ResourceBundle.properties same keys. Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; authentication.module.message.userNotFound and passwordNotSet are defined only in the default, "--", de and ja bundles; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/module/LoginSupportImpl.java LoginSupportImpl#populateSubjectPrincipalFromDatabase; SRC:src/com/technoetic/xplanner/security/module/XPlannerLoginModule.java XPlannerLoginModule#isPasswordMatched (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/LoginContext.java LoginContext#authenticate. WAR: classes byte-identical to the v1.1a4 release. A missing person raises the user-not-found key and a null stored password raises the password-not-set key; LoginContext#authenticate collects each module's message key per module name, and the action shows them as module messages. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-009, A-C-010).</t>
+  </si>
+  <si>
+    <t>A request to the login action without the submit field (for example a plain GET of /do/login) shows the login form in a fresh session. After one failed sign-in that posted action=Login, a later login POST without the submit field in the same session authenticates the user (W001). Empty user ID or password values are not checked by the action and are passed to the login module, which rejects them.</t>
   </si>
   <si>
     <t>The form is shown on first visit; blank credentials fail like wrong ones.</t>
   </si>
   <si>
-    <t>Login form (notAuthenticated) without an error on first visit; after submitting blank credentials: "Could not authenticate user." with a module message (for example "User has not been registered with XPlanner").</t>
-  </si>
-  <si>
-    <t>class AuthenticationAction#execute: the first branch tests StringUtils.isEmpty on the form field "action" (the submit button) and returns forward "notAuthenticated"; "userId" and "password" are then read and passed to Authenticator.authenticate without an emptiness check (bytecode listing, .migration-tmp/stage-01/tools/disasm.js); rejection messages per class LoginSupportImpl (authentication.module.message.userNotFound). Corrected in BA-001-04 (Source: stage-02-pass-002 F-005). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; authentication.module.message.userNotFound is defined only in the default, "--", de and ja bundles. Bundles without the key fall back to the default text (framework behavior, GAP-011). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/AuthenticationAction.java AuthenticationAction#execute (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/AuthenticatorImpl.java AuthenticatorImpl#authenticate; SRC:src/com/technoetic/xplanner/security/module/LoginSupportImpl.java LoginSupportImpl#getPerson, #populateSubjectPrincipalFromDatabase. WAR: classes byte-identical to the v1.1a4 release. The action returns the not-authenticated forward when the submit field is empty and otherwise passes user ID and password unchecked to the authenticator; an empty user ID finds no person (as long as no person has an empty user ID) and raises the user-not-found message.</t>
+    <t>Login form (notAuthenticated) without an error on first visit; after submitting blank credentials: "Could not authenticate user." with a module message (for example "User has not been registered with XPlanner"). In a session that already posted action=Login once, a POST of user ID and password without the submit field signs the user in (302 to /do/view/projects) (W001).</t>
+  </si>
+  <si>
+    <t>class AuthenticationAction#execute: the first branch tests StringUtils.isEmpty on the form field "action" (the submit button) and returns forward "notAuthenticated"; "userId" and "password" are then read and passed to Authenticator.authenticate without an emptiness check (bytecode listing, .migration-tmp/stage-01/tools/disasm.js); rejection messages per class LoginSupportImpl (authentication.module.message.userNotFound). Corrected in BA-001-04 (Source: stage-02-pass-002 F-005). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; authentication.module.message.userNotFound is defined only in the default, "--", de and ja bundles. Bundles without the key fall back to the default text (framework behavior, GAP-011). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/AuthenticationAction.java AuthenticationAction#execute (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/AuthenticatorImpl.java AuthenticatorImpl#authenticate; SRC:src/com/technoetic/xplanner/security/module/LoginSupportImpl.java LoginSupportImpl#getPerson, #populateSubjectPrincipalFromDatabase. WAR: classes byte-identical to the v1.1a4 release. The action returns the not-authenticated forward when the submit field is empty and otherwise passes user ID and password unchecked to the authenticator; an empty user ID finds no person (as long as no person has an empty user ID) and raises the user-not-found message. Stage 3 W001 (BA-001-13, MC-B-01, W001-F-03): failed sign-in with action=Login, then a POST with the correct password and no action field in the same session: 302 to the projects list; in a fresh session the same POST only showed the form (A-C-013). Part A reads this as a session-scoped form value (interpretation). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks A-C-011, A-C-012, A-C-013).</t>
   </si>
   <si>
     <t>Remember me</t>
@@ -226,7 +226,7 @@
     <t>Cookies "userid" and "password" are set (Base64-encoded values).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/security/login.jsp:29 (checkbox remember, value Y, checked by default); class AuthenticationAction#execute (strings "remember", "Y", CredentialCookie.set); class com.technoetic.xplanner.security.CredentialCookie#set (cookie names "userid", "password", Base64.encode). Cookie lifetime and flags (BA-001-07, mechanism (b)): CredentialCookie#set writes the user id and the Base64 of the clear password through CookieSupport#createCookie, which sets max-age 2147483647 seconds (about 68 years), sets neither Secure nor a path, and cannot set HttpOnly under the Servlet 2.4 API (bytecode listings). Observed risk only (Q3 deferred). Source: stage-02-pass-005 F-003. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/security/CredentialCookie.java CredentialCookie#set (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/util/CookieSupport.java CookieSupport#createCookie. WAR: classes byte-identical to the v1.1a4 release. The user ID and the Base64-encoded password are stored in two cookies with max-age Integer.MAX_VALUE, no Secure flag and no path.</t>
+    <t>WAR:WEB-INF/jsp/security/login.jsp:29 (checkbox remember, value Y, checked by default); class AuthenticationAction#execute (strings "remember", "Y", CredentialCookie.set); class com.technoetic.xplanner.security.CredentialCookie#set (cookie names "userid", "password", Base64.encode). Cookie lifetime and flags (BA-001-07, mechanism (b)): CredentialCookie#set writes the user id and the Base64 of the clear password through CookieSupport#createCookie, which sets max-age 2147483647 seconds (about 68 years), sets neither Secure nor a path, and cannot set HttpOnly under the Servlet 2.4 API (bytecode listings). Observed risk only (Q3 deferred). Source: stage-02-pass-005 F-003. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/security/CredentialCookie.java CredentialCookie#set (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/util/CookieSupport.java CookieSupport#createCookie. WAR: classes byte-identical to the v1.1a4 release. The user ID and the Base64-encoded password are stored in two cookies with max-age Integer.MAX_VALUE, no Secure flag and no path. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-014).</t>
   </si>
   <si>
     <t>A request without a session but with the credential cookies is authenticated automatically.</t>
@@ -238,7 +238,7 @@
     <t>Protected page opens without the login form; a failed cookie login falls back to the login redirect.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.security.filter.FormSecurityFilter#isAuthenticated (CredentialCookie.isPresent/getUserId/getPassword, Authenticator.authenticate, log "cookie-based authentication failed"); #onAuthenticationFailure (CredentialCookie.remove). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/filter/FormSecurityFilter.java FormSecurityFilter#isAuthenticated, #onAuthenticationFailure; SRC:src/com/technoetic/xplanner/security/filter/AbstractSecurityFilter.java AbstractSecurityFilter#doFilter. WAR: classes byte-identical to the v1.1a4 release. Without a subject in the session the filter authenticates with the cookie values; a failure is logged and leads to onAuthenticationFailure, which removes the cookies, saves the URL for GET requests and redirects to the login page.</t>
+    <t>class com.technoetic.xplanner.security.filter.FormSecurityFilter#isAuthenticated (CredentialCookie.isPresent/getUserId/getPassword, Authenticator.authenticate, log "cookie-based authentication failed"); #onAuthenticationFailure (CredentialCookie.remove). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/filter/FormSecurityFilter.java FormSecurityFilter#isAuthenticated, #onAuthenticationFailure; SRC:src/com/technoetic/xplanner/security/filter/AbstractSecurityFilter.java AbstractSecurityFilter#doFilter. WAR: classes byte-identical to the v1.1a4 release. Without a subject in the session the filter authenticates with the cookie values; a failure is logged and leads to onAuthenticationFailure, which removes the cookies, saves the URL for GET requests and redirects to the login page. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-015, A-C-016).</t>
   </si>
   <si>
     <t>Access protected pages without a session</t>
@@ -253,7 +253,7 @@
     <t>Unauthenticated request is redirected to the login page.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:85-96,160-167 (WebSecurityFilter on /do/* and /setting/*, authenticatorUrl /do/login); WAR:WEB-INF/security.xml:2-6 (bypass /do/login, /do/notAuthorized, /do/invalidateHibernateCache); class com.technoetic.xplanner.security.config.SecurityConfiguration#isSecureRequest (uses only securityBypass). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/security/filter/AbstractSecurityFilter.java AbstractSecurityFilter#doFilter; SRC:src/com/technoetic/xplanner/security/config/SecurityConfiguration.java SecurityConfiguration#isSecureRequest; SRC:src/com/technoetic/xplanner/security/filter/FormSecurityFilter.java FormSecurityFilter#onAuthenticationFailure. WAR: security.xml and web.xml identical to the SVN webapp copies. Every request not on the bypass list must be authenticated; otherwise the filter redirects to its login URL.</t>
+    <t>WAR:WEB-INF/web.xml:85-96,160-167 (WebSecurityFilter on /do/* and /setting/*, authenticatorUrl /do/login); WAR:WEB-INF/security.xml:2-6 (bypass /do/login, /do/notAuthorized, /do/invalidateHibernateCache); class com.technoetic.xplanner.security.config.SecurityConfiguration#isSecureRequest (uses only securityBypass). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/security/filter/AbstractSecurityFilter.java AbstractSecurityFilter#doFilter; SRC:src/com/technoetic/xplanner/security/config/SecurityConfiguration.java SecurityConfiguration#isSecureRequest; SRC:src/com/technoetic/xplanner/security/filter/FormSecurityFilter.java FormSecurityFilter#onAuthenticationFailure. WAR: security.xml and web.xml identical to the SVN webapp copies. Every request not on the bypass list must be authenticated; otherwise the filter redirects to its login URL. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-018, A-C-017).</t>
   </si>
   <si>
     <t>The root URL routes the user: with exactly one visible project that has a current iteration it redirects to that iteration, otherwise to the projects list.</t>
@@ -262,10 +262,10 @@
     <t>Single-project teams land directly on their current work.</t>
   </si>
   <si>
-    <t>Browser is redirected to /do/view/iteration?oid=&lt;current&gt; or /do/view/projects.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/web.xml:321-323 (welcome-file index.jsp); WAR:index.jsp:7-31 (useBeans Project where hidden = false; redirects). Access condition (BA-001-06): index.jsp is not covered by any security filter mapping (WAR:WEB-INF/web.xml:155-176 map the filters to /do/mobile/*, /do/*, /setting/*, /soap/* and /ical/*; welcome file at :321-323); the /index.jsp entry in WAR:WEB-INF/security.xml:16 is never evaluated (row 32). Without a session the page runs the hidden = false project query and, when exactly one visible project with a current iteration exists, redirects to /do/view/iteration?oid=&lt;id&gt;, which reveals that id before login; the target page then requires login. Observed risk only (Q3 deferred). Mechanical list: .migration-tmp/stage-01/out/unauth-06.txt. Source: stage-02-pass-004 F-005. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>Browser is redirected to /do/view/iteration?oid=&lt;current&gt; or /do/view/projects. Live (W001): the redirect to the current iteration was observed only while exactly one project existed in the system; with five projects in the system and one readable project whose current iteration had started, the user landed on /do/view/projects.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/web.xml:321-323 (welcome-file index.jsp); WAR:index.jsp:7-31 (useBeans Project where hidden = false; redirects). Access condition (BA-001-06): index.jsp is not covered by any security filter mapping (WAR:WEB-INF/web.xml:155-176 map the filters to /do/mobile/*, /do/*, /setting/*, /soap/* and /ical/*; welcome file at :321-323); the /index.jsp entry in WAR:WEB-INF/security.xml:16 is never evaluated (row 32). Without a session the page runs the hidden = false project query and, when exactly one visible project with a current iteration exists, redirects to /do/view/iteration?oid=&lt;id&gt;, which reveals that id before login; the target page then requires login. Observed risk only (Q3 deferred). Mechanical list: .migration-tmp/stage-01/out/unauth-06.txt. Source: stage-02-pass-004 F-005. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Stage 3 W001 (BA-001-13, MC-A-03, W001-F-04): GET / as a person who can read only project 221 (current iteration started), with five projects in the system: 302 to /do/view/projects (A-C-018); the iteration redirect was seen while one project existed (setup-C-035). The result is consistent with a one-project count that is not limited to the projects the user may read; the rule was not re-read from source in BA-001-13 (no new research), so the meaning of "visible" in the requirement stays open. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-035, A-C-018, A-C-019, A-C-020).</t>
   </si>
   <si>
     <t>Log out</t>
@@ -280,7 +280,7 @@
     <t>Session is invalidated, remember-me cookies are removed and the login page is shown.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:21 (link /do/logout); WAR:WEB-INF/struts-config.xml:171; WAR:WEB-INF/action-servlet.xml:16; class com.technoetic.xplanner.actions.LogoutAction#execute (Authenticator.logout, CredentialCookie.remove, forward "security/login"); class XPlannerLoginModule#logout (HttpSession.invalidate). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/LogoutAction.java LogoutAction#execute. WAR: classes byte-identical to the v1.1a4 release. Logout calls the authenticator, removes the credential cookies and forwards to the login page.</t>
+    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:21 (link /do/logout); WAR:WEB-INF/struts-config.xml:171; WAR:WEB-INF/action-servlet.xml:16; class com.technoetic.xplanner.actions.LogoutAction#execute (Authenticator.logout, CredentialCookie.remove, forward "security/login"); class XPlannerLoginModule#logout (HttpSession.invalidate). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/LogoutAction.java LogoutAction#execute. WAR: classes byte-identical to the v1.1a4 release. Logout calls the authenticator, removes the credential cookies and forwards to the login page. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-014, setup-C-015, setup-C-016, setup-C-017, A-C-021).</t>
   </si>
   <si>
     <t>Session expiry</t>
@@ -298,7 +298,7 @@
     <t>Next request after 30 idle minutes is treated as unauthenticated (unless the remember-me cookies re-authenticate).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:318-320 (session-timeout 30); cookie re-login per class FormSecurityFilter#isAuthenticated. Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/security/filter/FormSecurityFilter.java FormSecurityFilter#isAuthenticated. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
+    <t>WAR:WEB-INF/web.xml:318-320 (session-timeout 30); cookie re-login per class FormSecurityFilter#isAuthenticated. Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/security/filter/FormSecurityFilter.java FormSecurityFilter#isAuthenticated. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-022).</t>
   </si>
   <si>
     <t>Alternative login modules (LDAP/JNDI, NTLM, JAAS)</t>
@@ -316,7 +316,7 @@
     <t>Partial</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/xplanner.properties:167-190 (login[1] JNDI and login[2] NTLM commented out); WAR:WEB-INF/classes/spring-security.xml:38-43 (JaasLoginModuleAdapterFactory, NtlmLoginModule, JNDILoginModule, JNDIAuthenticatorImpl beans); classes com.technoetic.xplanner.security.module.jndi.JNDILoginModule, .ntlm.NtlmLoginModule, com.sabre.security.jndi.*. Not active in the shipped file. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/security/module/LoginModuleLoader.java LoginModuleLoader#loadLoginModules; SRC:src/com/technoetic/xplanner/security/module/jndi/JNDILoginModule.java JNDILoginModule; SRC:src/com/sabre/security/jndi/JNDIAuthenticatorImpl.java (withheld file, cited by path only). WAR: classes byte-identical to the v1.1a4 release; login modules from the patched WAR xplanner.properties (WAR governs). The loader builds modules only from the login[n] keys present, and the WAR file defines login[0] only. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/classes/xplanner.properties:167-190 (login[1] JNDI and login[2] NTLM commented out); WAR:WEB-INF/classes/spring-security.xml:38-43 (JaasLoginModuleAdapterFactory, NtlmLoginModule, JNDILoginModule, JNDIAuthenticatorImpl beans); classes com.technoetic.xplanner.security.module.jndi.JNDILoginModule, .ntlm.NtlmLoginModule, com.sabre.security.jndi.*. Not active in the shipped file. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/security/module/LoginModuleLoader.java LoginModuleLoader#loadLoginModules; SRC:src/com/technoetic/xplanner/security/module/jndi/JNDILoginModule.java JNDILoginModule; SRC:src/com/sabre/security/jndi/JNDIAuthenticatorImpl.java (withheld file, cited by path only). WAR: classes byte-identical to the v1.1a4 release; login modules from the patched WAR xplanner.properties (WAR governs). The loader builds modules only from the login[n] keys present, and the WAR file defines login[0] only. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks A-C-023; open residual scope R-46 (e)).</t>
   </si>
   <si>
     <t>UF-002</t>
@@ -337,19 +337,19 @@
     <t>A sysadmin can do everything; an admin has editor and viewer rights plus admin*; an editor can create/edit/delete/integrate; a viewer can read.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/db-changelog.xml:363-386 (roles viewer lft1/rgt8, editor 2/7, admin 3/6, sysadmin 4/5) and :275-362 (permission rows); WAR:WEB-INF/classes/mappings/Metrics.xml queries "security.roles" and "security.role.permissions" (r1.left between r2.left and r2.right for positive permissions). Server-side enforcement (CHK-002, BA-001-04): the role model is evaluated on the server only on the paths in rows 28, 31, 167, 180, 218 and 230; everywhere else it only decides which links and fields the JSP pages show (rows 26, 29-30). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/auth/AuthorizerImpl.java AuthorizerImpl#hasPermission, #permissionMatches, #isMatching; SRC:src/com/technoetic/xplanner/security/auth/PrincipalSpecificPermissionHelper.java PrincipalSpecificPermissionHelper#getPermissionsForPrincipal. WAR: classes byte-identical to the v1.1a4 release; seed data in db-changelog.xml (WAR entry; the SVN copy differs and is withheld; WAR governs). Permissions are loaded per principal and project and matched with trailing-% prefix patterns; the nested role ranges come from the WAR seed data and the named queries of Metrics.xml, so the hierarchy holds for the seeded data.</t>
-  </si>
-  <si>
-    <t>Negative permissions apply to the exact role only: editors may not create projects, create people or delete iterations; admins may not create projects.</t>
+    <t>WAR:WEB-INF/classes/db-changelog.xml:363-386 (roles viewer lft1/rgt8, editor 2/7, admin 3/6, sysadmin 4/5) and :275-362 (permission rows); WAR:WEB-INF/classes/mappings/Metrics.xml queries "security.roles" and "security.role.permissions" (r1.left between r2.left and r2.right for positive permissions). Server-side enforcement (CHK-002, BA-001-04): the role model is evaluated on the server only on the paths in rows 28, 31, 167, 180, 218 and 230; everywhere else it only decides which links and fields the JSP pages show (rows 26, 29-30). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/auth/AuthorizerImpl.java AuthorizerImpl#hasPermission, #permissionMatches, #isMatching; SRC:src/com/technoetic/xplanner/security/auth/PrincipalSpecificPermissionHelper.java PrincipalSpecificPermissionHelper#getPermissionsForPrincipal. WAR: classes byte-identical to the v1.1a4 release; seed data in db-changelog.xml (WAR entry; the SVN copy differs and is withheld; WAR governs). Permissions are loaded per principal and project and matched with trailing-% prefix patterns; the nested role ranges come from the WAR seed data and the named queries of Metrics.xml, so the hierarchy holds for the seeded data. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-028, A-C-030, A-C-033).</t>
+  </si>
+  <si>
+    <t>Negative permissions apply to the exact role only: editors may not create projects, create people or delete iterations; admins may not create projects. On the people list the create-people restriction has no visible effect: the Add Person and Import People links are shown to every signed-in role (W001).</t>
   </si>
   <si>
     <t>Restricts structural changes to higher roles.</t>
   </si>
   <si>
-    <t>"Create project" and "Add person" links and iteration delete buttons are hidden for those roles. Nothing refuses a direct request (rows 29-30).</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/classes/db-changelog.xml permission ids 7, 8, 9, 19 (positive=false); WAR:WEB-INF/classes/mappings/Metrics.xml "security.role.permissions" (positive=0 and r1.id = r2.id). Evaluation order in class com.technoetic.xplanner.security.auth.AuthorizerImpl not decompiled. Server-side enforcement (CHK-002, BA-001-04): these restrictions only hide links and buttons; the create and delete handlers perform no server-side permission check (rows 29-30). Corrected in BA-001-04 (Source: stage-02-pass-002 F-007). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/auth/AuthorizerImpl.java AuthorizerImpl#permissionMatches. WAR: classes byte-identical to the v1.1a4 release; seed data in the WAR db-changelog.xml. The evaluation order is now visible: within one project list a matching negative permission defeats any matching positive one (positive and not negative); the exact-role scope of negative permissions comes from the Metrics.xml query.</t>
+    <t>"Create project" links and iteration delete buttons are hidden for those roles; the "Add Person" and "Import People" links of /do/view/people are shown to the viewer, editor, admin and system-administrator role accounts, and a viewer can create a person (W001). Nothing refuses a direct request (rows 29-30).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/classes/db-changelog.xml permission ids 7, 8, 9, 19 (positive=false); WAR:WEB-INF/classes/mappings/Metrics.xml "security.role.permissions" (positive=0 and r1.id = r2.id). Evaluation order in class com.technoetic.xplanner.security.auth.AuthorizerImpl not decompiled. Server-side enforcement (CHK-002, BA-001-04): these restrictions only hide links and buttons; the create and delete handlers perform no server-side permission check (rows 29-30). Corrected in BA-001-04 (Source: stage-02-pass-002 F-007). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/auth/AuthorizerImpl.java AuthorizerImpl#permissionMatches. WAR: classes byte-identical to the v1.1a4 release; seed data in the WAR db-changelog.xml. The evaluation order is now visible: within one project list a matching negative permission defeats any matching positive one (positive and not negative); the exact-role scope of negative permissions comes from the Metrics.xml query. Stage 3 W001 (BA-001-13, MC-A-04, W001-F-05): Add Project shown only to the system administrator (setup-C-020); iteration delete hidden from the editor (setup-C-024, A-C-024); Add Person and Import People shown to all four role accounts (setup-C-021); a viewer created a person through the offered form (A-C-025). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-020, setup-C-021, setup-C-024, A-C-024, A-C-025).</t>
   </si>
   <si>
     <t>A role assigned for project 0 applies to all projects (the seeded sysadmin is assigned this way).</t>
@@ -361,7 +361,7 @@
     <t>Seeded sysadmin sees and administers every project.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/db-changelog.xml:407-411 (person_role role 5, person 1, project 0); Metrics.xml "security.roles" (:includeWildcardProject = 1 and pr.id.projectId = 0). Server-side enforcement (CHK-002, BA-001-04): as for the role model, only the server-side paths in rows 28, 31, 167, 180, 218 and 230 evaluate it; project 0 is also the scope of the system-administrator rule in rows 31 and 34. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/auth/AuthorizerImpl.java AuthorizerImpl#hasPermission (ANY_PROJECT = 0). WAR: classes byte-identical to the v1.1a4 release; seed data in the WAR db-changelog.xml. HasPermission grants when the permissions of the requested project or those of project 0 match, so a role on project 0 applies to every project.</t>
+    <t>WAR:WEB-INF/classes/db-changelog.xml:407-411 (person_role role 5, person 1, project 0); Metrics.xml "security.roles" (:includeWildcardProject = 1 and pr.id.projectId = 0). Server-side enforcement (CHK-002, BA-001-04): as for the role model, only the server-side paths in rows 28, 31, 167, 180, 218 and 230 evaluate it; project 0 is also the scope of the system-administrator rule in rows 31 and 34. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/auth/AuthorizerImpl.java AuthorizerImpl#hasPermission (ANY_PROJECT = 0). WAR: classes byte-identical to the v1.1a4 release; seed data in the WAR db-changelog.xml. HasPermission grants when the permissions of the requested project or those of project 0 match, so a role on project 0 applies to every project. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-026, setup-C-062).</t>
   </si>
   <si>
     <t>Permission-driven UI actions</t>
@@ -376,7 +376,7 @@
     <t>Icons/links appear or disappear by permission (for example project delete requires sysadmin.delete, project edit admin.edit).</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.domain.DomainMetaDataRepository#init (action definitions with permissions "admin.edit", "sysadmin.delete", "edit", "delete"); WAR:WEB-INF/xplanner.tld (isUserAuthorized -&gt; com.technoetic.xplanner.tags.IsUserAuthorizedTag); e.g. WAR:WEB-INF/jsp/view/projects.jsp:82-100. Corrected in BA-001-03 (stage-02-pass-001 F-001): the gating is in JSP tags only. Server-side enforcement (CHK-002, BA-001-04): display-level only; the handlers behind these links perform no server-side permission check (rows 29-30), except the person-editor role rules (row 31). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init; SRC:src/com/technoetic/xplanner/tags/IsUserAuthorizedTag.java IsUserAuthorizedTag. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
+    <t>class com.technoetic.xplanner.domain.DomainMetaDataRepository#init (action definitions with permissions "admin.edit", "sysadmin.delete", "edit", "delete"); WAR:WEB-INF/xplanner.tld (isUserAuthorized -&gt; com.technoetic.xplanner.tags.IsUserAuthorizedTag); e.g. WAR:WEB-INF/jsp/view/projects.jsp:82-100. Corrected in BA-001-03 (stage-02-pass-001 F-001): the gating is in JSP tags only. Server-side enforcement (CHK-002, BA-001-04): display-level only; the handlers behind these links perform no server-side permission check (rows 29-30), except the person-editor role rules (row 31). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init; SRC:src/com/technoetic/xplanner/tags/IsUserAuthorizedTag.java IsUserAuthorizedTag. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-027, setup-C-063).</t>
   </si>
   <si>
     <t>The projects list shows only projects the user may read.</t>
@@ -388,7 +388,7 @@
     <t>Projects without read permission are not listed.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/projects.jsp:32-48 (CollectionUtils.filter with SystemAuthorizer.hasPermission(..., "read")). Server-side enforcement (CHK-002, BA-001-04): this filters the list rendered on the server, but the project pages themselves have no read check (row 29). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/jsp/view/projects.jsp:32-48 (CollectionUtils.filter with SystemAuthorizer.hasPermission(..., "read")). Server-side enforcement (CHK-002, BA-001-04): this filters the list rendered on the server, but the project pages themselves have no read check (row 29). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-026).</t>
   </si>
   <si>
     <t>Only views handled by DispatchForward with authorization required check permission (the flag defaults to true and is switched off for projects, people, settings, dashboard, twiki format and not-authorized): without a projectId parameter, or without read permission on system.project, they forward to security/notAuthorized, whose JSP is absent.</t>
@@ -400,7 +400,7 @@
     <t>For /do/view/integrations and the WAP views: not-authorized forward (expected error, page missing). The global AuthorizationException mapping to generalError.jsp (security.notauthorized) is reachable only through the secure repository adapter, which no working web path uses.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.actions.DispatchForward: #isSecure uses a "@secure" forward if present, otherwise field isAuthorizationRequired; #&lt;init&gt; sets isAuthorizationRequired true; #execute reads projectId and calls Authorizer.hasPermission(..., "system.project", ..., "read"), else forward "security/notAuthorized" (bytecode listing by .migration-tmp/stage-01/tools/disasm.js); no "@secure" forward in any descriptor; WAR:WEB-INF/action-servlet.xml:12-14,25-31,327-331,390,412-418; WAR:WEB-INF/struts-config.xml:139 (notAuthorized.jsp ABSENT, GAP-003) and :87-89; RepositorySecurityAdapter#checkAuthorization is the only constructor call of AuthorizationException. Corrected in BA-001-03 (F-001; narrows the reviewer statement that DispatchForward never checks). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DispatchForward.java DispatchForward#execute, #isSecure. WAR: classes byte-identical to the v1.1a4 release. The view checks a "@secure" forward first and otherwise the authorization flag, then requires a projectId and system.project read, as recorded; the not-authorized JSP stays absent from the WAR.</t>
+    <t>class com.technoetic.xplanner.actions.DispatchForward: #isSecure uses a "@secure" forward if present, otherwise field isAuthorizationRequired; #&lt;init&gt; sets isAuthorizationRequired true; #execute reads projectId and calls Authorizer.hasPermission(..., "system.project", ..., "read"), else forward "security/notAuthorized" (bytecode listing by .migration-tmp/stage-01/tools/disasm.js); no "@secure" forward in any descriptor; WAR:WEB-INF/action-servlet.xml:12-14,25-31,327-331,390,412-418; WAR:WEB-INF/struts-config.xml:139 (notAuthorized.jsp ABSENT, GAP-003) and :87-89; RepositorySecurityAdapter#checkAuthorization is the only constructor call of AuthorizationException. Corrected in BA-001-03 (F-001; narrows the reviewer statement that DispatchForward never checks). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DispatchForward.java DispatchForward#execute, #isSecure. WAR: classes byte-identical to the v1.1a4 release. The view checks a "@secure" forward first and otherwise the authorization flag, then requires a projectId and system.project read, as recorded; the not-authorized JSP stays absent from the WAR. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-027, A-C-028, A-C-029, D-C-072, D-C-073).</t>
   </si>
   <si>
     <t>Server-side permission enforcement</t>
@@ -415,7 +415,7 @@
     <t>Direct requests succeed for any signed-in user (runtime unverified).</t>
   </si>
   <si>
-    <t>Static call graph from each entry point to authorization calls (.migration-tmp/stage-01/tools/authtrace.js, out/authtrace.json): no Authorizer, SystemAuthorizer or RepositorySecurityAdapter call is reachable from ViewObjectAction#doExecute, EditObjectAction#updateObject/#createObject or DeleteObjectAction#doExecute, which call CommonDao.getById/save/delete and EventManager.publish*; beans WAR:WEB-INF/action-servlet.xml:33-43,72-82,84-130,196-212,214-224,256-272,300-304,352-356,370-374,420-424. Inferred from bytecode; Stage 3 confirmation needed. Source: stage-02-pass-001 F-001. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/AbstractAction.java AbstractAction#execute; SRC:src/com/technoetic/xplanner/actions/ViewObjectAction.java ViewObjectAction#doExecute, #isSecure; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#doExecute, #updateObject, #createObject; SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. None of these methods calls an authorizer; AbstractAction#execute only wraps doExecute and the hooks in a transaction. ViewObjectAction's authorizationRequired flag only decides whether the object is loaded into the domain context, it gates nothing.</t>
+    <t>Static call graph from each entry point to authorization calls (.migration-tmp/stage-01/tools/authtrace.js, out/authtrace.json): no Authorizer, SystemAuthorizer or RepositorySecurityAdapter call is reachable from ViewObjectAction#doExecute, EditObjectAction#updateObject/#createObject or DeleteObjectAction#doExecute, which call CommonDao.getById/save/delete and EventManager.publish*; beans WAR:WEB-INF/action-servlet.xml:33-43,72-82,84-130,196-212,214-224,256-272,300-304,352-356,370-374,420-424. Inferred from bytecode; Stage 3 confirmation needed. Source: stage-02-pass-001 F-001. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/AbstractAction.java AbstractAction#execute; SRC:src/com/technoetic/xplanner/actions/ViewObjectAction.java ViewObjectAction#doExecute, #isSecure; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#doExecute, #updateObject, #createObject; SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. None of these methods calls an authorizer; AbstractAction#execute only wraps doExecute and the hooks in a transaction. ViewObjectAction's authorizationRequired flag only decides whether the object is loaded into the domain context, it gates nothing. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-030, A-C-031, A-C-032).</t>
   </si>
   <si>
     <t>The other web actions likewise have no server-side permission check: export, import of people and stories, move/continue of stories and tasks, multi-move, reorder, time entry, notes and attachment download, file manager, integration queue, iteration start/close and continue, notification receivers, project role editor, personal timesheet, ID search, the "me" page and the test/admin utilities.</t>
@@ -424,7 +424,7 @@
     <t>Same enforcement gap across all action types (impact sweep of F-001). Observed behavior and risk only (Q3 deferred).</t>
   </si>
   <si>
-    <t>.migration-tmp/stage-01/out/authtrace.json: 80 web action beans, 7 WAP actions, 43 SOAP operations, 4 REST methods, the iCal servlet and 3 Spring MVC handlers traced. For web actions, authorization calls are reachable only from DispatchForward, EditPersonAction (role changes), ViewAggregateTimesheetAction (result filter), InvalidateCacheAction (cache reset) and, not as a gate, inside e-mail recipient or metrics lookups (EditTaskAction, IntegrationAction, CommandExecutorAction, ViewIterationMetricsAction). Tracer limits: control flow and framework callbacks are not followed. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ (package search: only DispatchForward, EditPersonHelper, EditRoleAction, SearchResultAuthorizationPredicate and admin/InvalidateCacheAction refer to the authorizer). WAR: classes byte-identical to the v1.1a4 release. The package search agrees with the bytecode trace; the status stays Inferred because not every listed action was read at method level.</t>
+    <t>.migration-tmp/stage-01/out/authtrace.json: 80 web action beans, 7 WAP actions, 43 SOAP operations, 4 REST methods, the iCal servlet and 3 Spring MVC handlers traced. For web actions, authorization calls are reachable only from DispatchForward, EditPersonAction (role changes), ViewAggregateTimesheetAction (result filter), InvalidateCacheAction (cache reset) and, not as a gate, inside e-mail recipient or metrics lookups (EditTaskAction, IntegrationAction, CommandExecutorAction, ViewIterationMetricsAction). Tracer limits: control flow and framework callbacks are not followed. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ (package search: only DispatchForward, EditPersonHelper, EditRoleAction, SearchResultAuthorizationPredicate and admin/InvalidateCacheAction refer to the authorizer). WAR: classes byte-identical to the v1.1a4 release. The package search agrees with the bytecode trace; the status stays Inferred because not every listed action was read at method level. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-033, A-C-070, B-C-018, B-C-020, B-C-034, B-C-037, B-C-077, C-C-008, C-C-024, C-C-029, C-C-051, D-C-023, E-C-009, E-C-020).</t>
   </si>
   <si>
     <t>Server-side role changes in the person editor are applied only for projects on which the current user holds admin.edit.role; in addition, when the current user holds admin.edit.role on project 0, every save of the person editor first removes the person's sysadmin role and re-adds it only if the form carries systemAdmin=true.</t>
@@ -436,7 +436,7 @@
     <t>Role changes for other projects are ignored; the sysadmin role is revoked or granted by the project-0 rule (runtime unverified).</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.actions.EditPersonHelper#modifyRoles: for each submitted project role, #isCurrentUserAdminOfProject(projectId, user) (Authorizer.hasPermission with "system.project", "admin.edit.role") gates #setRoleOnProject; then #isCurrentUserAdminOfProject(0, user) gates RoleAssociationRepository.deleteForPersonOnProject("sysadmin", person, 0), followed by #setSysadmin only when the systemAdmin flag is true (bytecode listing); caller EditPersonAction#beforeObjectCommit passes PersonEditorForm#isSystemAdmin. class PersonEditorForm uses the authorizer only to preselect displayed roles (#getRoles, #isRoleSelected), not as a gate. The rest of the person edit (name, e-mail, password, hidden) is not permission-checked on the server. Corrected in BA-001-04 (Source: stage-02-pass-002 F-007). Server-side enforcement (CHK-002, BA-001-04): this row records the server-side check itself (Authorizer.hasPermission reached from EditPersonAction#beforeObjectCommit, .migration-tmp/stage-01/out/authtrace.json). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/EditPersonHelper.java EditPersonHelper#modifyRoles, #isCurrentUserAdminOfProject, #setSysadmin; SRC:src/com/technoetic/xplanner/actions/EditPersonAction.java EditPersonAction#beforeObjectCommit. WAR: classes byte-identical to the v1.1a4 release. ModifyRoles applies each submitted project role only when the current user is admin of that project, then, for a project-0 admin, deletes the person's sysadmin role on project 0 and re-adds it only when the flag is set; the order matches the bytecode listing.</t>
+    <t>class com.technoetic.xplanner.actions.EditPersonHelper#modifyRoles: for each submitted project role, #isCurrentUserAdminOfProject(projectId, user) (Authorizer.hasPermission with "system.project", "admin.edit.role") gates #setRoleOnProject; then #isCurrentUserAdminOfProject(0, user) gates RoleAssociationRepository.deleteForPersonOnProject("sysadmin", person, 0), followed by #setSysadmin only when the systemAdmin flag is true (bytecode listing); caller EditPersonAction#beforeObjectCommit passes PersonEditorForm#isSystemAdmin. class PersonEditorForm uses the authorizer only to preselect displayed roles (#getRoles, #isRoleSelected), not as a gate. The rest of the person edit (name, e-mail, password, hidden) is not permission-checked on the server. Corrected in BA-001-04 (Source: stage-02-pass-002 F-007). Server-side enforcement (CHK-002, BA-001-04): this row records the server-side check itself (Authorizer.hasPermission reached from EditPersonAction#beforeObjectCommit, .migration-tmp/stage-01/out/authtrace.json). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/EditPersonHelper.java EditPersonHelper#modifyRoles, #isCurrentUserAdminOfProject, #setSysadmin; SRC:src/com/technoetic/xplanner/actions/EditPersonAction.java EditPersonAction#beforeObjectCommit. WAR: classes byte-identical to the v1.1a4 release. ModifyRoles applies each submitted project role only when the current user is admin of that project, then, for a project-0 admin, deletes the person's sysadmin role on project 0 and re-adds it only when the flag is set; the order matches the bytecode listing. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks A-C-034; open residual scope R-35 (e)).</t>
   </si>
   <si>
     <t>URL role constraints in security.xml, mobile-security.xml and soap-security.xml are parsed but never evaluated; the security filters only check the bypass list and that the user is authenticated.</t>
@@ -448,7 +448,7 @@
     <t>Any authenticated user passes the filters for every constrained URL.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.security.config.SecurityConfiguration#isAuthorized has no caller in any class (positive control: #isSecureRequest is called by AbstractSecurityFilter#isSecureRequest); AbstractSecurityFilter#doFilter calls only isSecureRequest, isAuthenticated and onAuthenticationFailure; WAR:WEB-INF/security.xml:9-39, WAR:WEB-INF/mobile-security.xml:6-16, WAR:WEB-INF/soap-security.xml:2-34. Source: stage-02-pass-001 F-001 and F-004. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/filter/AbstractSecurityFilter.java AbstractSecurityFilter#doFilter, #isSecureRequest; SRC:src/com/technoetic/xplanner/security/config/SecurityConfiguration.java SecurityConfiguration#isAuthorized (no caller in the source tree). WAR: classes byte-identical to the v1.1a4 release. DoFilter only checks the bypass list and authentication; no source file calls SecurityConfiguration#isAuthorized.</t>
+    <t>class com.technoetic.xplanner.security.config.SecurityConfiguration#isAuthorized has no caller in any class (positive control: #isSecureRequest is called by AbstractSecurityFilter#isSecureRequest); AbstractSecurityFilter#doFilter calls only isSecureRequest, isAuthenticated and onAuthenticationFailure; WAR:WEB-INF/security.xml:9-39, WAR:WEB-INF/mobile-security.xml:6-16, WAR:WEB-INF/soap-security.xml:2-34. Source: stage-02-pass-001 F-001 and F-004. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/filter/AbstractSecurityFilter.java AbstractSecurityFilter#doFilter, #isSecureRequest; SRC:src/com/technoetic/xplanner/security/config/SecurityConfiguration.java SecurityConfiguration#isAuthorized (no caller in the source tree). WAR: classes byte-identical to the v1.1a4 release. DoFilter only checks the bypass list and authentication; no source file calls SecurityConfiguration#isAuthorized. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks A-C-035; open residual scope R-41 (e)).</t>
   </si>
   <si>
     <t>Assign project roles to a person</t>
@@ -460,10 +460,10 @@
     <t>Project administrators manage team membership.</t>
   </si>
   <si>
-    <t>Per-project radio buttons in the person editor; saved roles change what the person can see and do.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (isUserAuthorizedForAny projects permissions admin.edit.role; radio options none/viewer/editor/admin); WAR:WEB-INF/classes/spring-beans.xml:193-203 (editPersonHelper with invalidateCacheAfterPermissionChangedAdvisor on modifyRoles). Server-side enforcement (CHK-002, BA-001-04): enforced on the server per project by EditPersonHelper#isCurrentUserAdminOfProject (row 31); the editor page itself is reachable by any signed-in user (row 29). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/EditPersonHelper.java EditPersonHelper#modifyRoles, #isCurrentUserAdminOfProject. WAR: classes byte-identical to the v1.1a4 release. Each project role is set only when the current user is admin of that project. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>Per-project role drop-down (None, Viewer, Editor, Admin) in the person editor; saved roles change what the person can see and do.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (isUserAuthorizedForAny projects permissions admin.edit.role; radio options none/viewer/editor/admin); WAR:WEB-INF/classes/spring-beans.xml:193-203 (editPersonHelper with invalidateCacheAfterPermissionChangedAdvisor on modifyRoles). Server-side enforcement (CHK-002, BA-001-04): enforced on the server per project by EditPersonHelper#isCurrentUserAdminOfProject (row 31); the editor page itself is reachable by any signed-in user (row 29). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/EditPersonHelper.java EditPersonHelper#modifyRoles, #isCurrentUserAdminOfProject. WAR: classes byte-identical to the v1.1a4 release. Each project role is set only when the current user is admin of that project. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream. Stage 3 W001 (BA-001-13, MC-A-05, W001-F-06): the person editor offers one select projectRole[i] with a hidden projectId[i] per project, options None, Viewer, Editor and Admin; saved viewer, editor and admin roles were shown again and changed the visible controls (setup-C-006). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-006, setup-C-061).</t>
   </si>
   <si>
     <t>The "System administrator" checkbox is shown only to sysadmin.promote holders, but on the server the sysadmin role is governed by admin.edit.role on project 0: when a user holding it saves any person editor, the person's sysadmin role is removed and re-added only if systemAdmin=true is posted.</t>
@@ -475,22 +475,22 @@
     <t>Checkbox visible only to sysadmins; saving the person editor as a project-0 administrator without the checkbox revokes the person's system-administrator role; posting systemAdmin=true grants it (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp:144-151 (isUserAuthorized resourceType="system" permission="sysadmin.promote", input systemAdmin); class EditPersonHelper#modifyRoles, #isCurrentUserAdminOfProject, #setSysadmin (bytecode listing: deleteForPersonOnProject("sysadmin", personId, 0) then setSysadmin when the flag is true); class EditPersonAction#beforeObjectCommit (PersonEditorForm#isSystemAdmin). Who holds admin.edit.role on project 0 follows the role model (rows 23-25; sysadmin via "%", admin via "admin%" when assigned on project 0), Inferred. Corrected in BA-001-04 (Source: stage-02-pass-002 F-007). Server-side enforcement (CHK-002, BA-001-04): sysadmin.promote is display-level only; the server-side check that governs the sysadmin role is admin.edit.role on project 0 (row 31). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/EditPersonHelper.java EditPersonHelper#modifyRoles, #setSysadmin; SRC:src/com/technoetic/xplanner/actions/EditPersonAction.java EditPersonAction#beforeObjectCommit. WAR: classes byte-identical to the v1.1a4 release. As row 31: the checkbox is display-level (editPerson.jsp), and the server applies the project-0 admin.edit.role rule.</t>
+    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp:144-151 (isUserAuthorized resourceType="system" permission="sysadmin.promote", input systemAdmin); class EditPersonHelper#modifyRoles, #isCurrentUserAdminOfProject, #setSysadmin (bytecode listing: deleteForPersonOnProject("sysadmin", personId, 0) then setSysadmin when the flag is true); class EditPersonAction#beforeObjectCommit (PersonEditorForm#isSystemAdmin). Who holds admin.edit.role on project 0 follows the role model (rows 23-25; sysadmin via "%", admin via "admin%" when assigned on project 0), Inferred. Corrected in BA-001-04 (Source: stage-02-pass-002 F-007). Server-side enforcement (CHK-002, BA-001-04): sysadmin.promote is display-level only; the server-side check that governs the sysadmin role is admin.edit.role on project 0 (row 31). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/EditPersonHelper.java EditPersonHelper#modifyRoles, #setSysadmin; SRC:src/com/technoetic/xplanner/actions/EditPersonAction.java EditPersonAction#beforeObjectCommit. WAR: classes byte-identical to the v1.1a4 release. As row 31: the checkbox is display-level (editPerson.jsp), and the server applies the project-0 admin.edit.role rule. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks setup-C-003, A-C-036, A-C-037, A-C-038, A-C-039, F-C-001; open residual scope R-34 (e)).</t>
   </si>
   <si>
     <t>Edit project roles (project role editor)</t>
   </si>
   <si>
-    <t>A project role editor lists people with viewer/editor/admin radio choices for one project.</t>
+    <t>A project role editor is meant to list people with viewer/editor/admin radio choices for one project. It is reachable by URL only (no link on the project page), and in this baseline it answered HTTP 500 without rendering a form for the parameter forms tried (W001).</t>
   </si>
   <si>
     <t>Bulk role maintenance per project.</t>
   </si>
   <si>
-    <t>Form posted to /do/edit/roles; the role-saving code is expected never to run, so submitted roles are not saved (runtime unverified).</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/struts-config.xml:409-411; WAR:WEB-INF/action-servlet.xml:400-404 (EditRoleAction); WAR:WEB-INF/jsp/edit/editRoles.jsp; class com.technoetic.xplanner.actions.EditRoleAction (strings "admin.edit.role", HQL on PersonRole). No live link to this page was found (mechanical link scan .migration-tmp/stage-01/out/linkgraph.txt); reachable only by URL. BA-001-03 impact sweep: EditRoleAction#beforeObjectCommit(Object, Session, ActionMapping, ActionForm, HttpServletRequest, HttpServletResponse) overrides no superclass hook (AbstractAction#beforeObjectCommit takes Identifiable, ActionMapping, ActionForm, request, response) and has no caller, so its role update and its admin.edit.role check are unreachable; an orphan-hook scan over all action classes found only this method. Server-side enforcement (CHK-002, BA-001-04): no server-side check is reached, because the only check sits in the unreachable EditRoleAction#beforeObjectCommit (above); the page is reachable by any signed-in user. Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editRoles.jsp writes the raw request parameters oid (55), returnto (56) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): /do/edit/roles runs EditObjectAction#doExecute with type net.sf.xplanner.domain.Project (WAR:WEB-INF/action-servlet.xml:400-404), so a direct request with merge=true binds the request parameters onto the loaded project as in row 78 (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/EditRoleAction.java EditRoleAction#beforeObjectCommit; SRC:src/com/technoetic/xplanner/actions/AbstractAction.java AbstractAction#execute. WAR: classes byte-identical to the v1.1a4 release. The role-saving method takes an extra Session parameter, so it does not override the hook that AbstractAction#execute calls, and nothing else calls it.</t>
+    <t>Opened by URL (/do/edit/roles with projectId and fkey, or with oid) the editor answers HTTP 500 (with oid: NullPointerException) and shows no form (W001), so the source-based expectation that submitted roles are not saved (the role-saving code never runs) cannot be reached.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/struts-config.xml:409-411; WAR:WEB-INF/action-servlet.xml:400-404 (EditRoleAction); WAR:WEB-INF/jsp/edit/editRoles.jsp; class com.technoetic.xplanner.actions.EditRoleAction (strings "admin.edit.role", HQL on PersonRole). No live link to this page was found (mechanical link scan .migration-tmp/stage-01/out/linkgraph.txt); reachable only by URL. BA-001-03 impact sweep: EditRoleAction#beforeObjectCommit(Object, Session, ActionMapping, ActionForm, HttpServletRequest, HttpServletResponse) overrides no superclass hook (AbstractAction#beforeObjectCommit takes Identifiable, ActionMapping, ActionForm, request, response) and has no caller, so its role update and its admin.edit.role check are unreachable; an orphan-hook scan over all action classes found only this method. Server-side enforcement (CHK-002, BA-001-04): no server-side check is reached, because the only check sits in the unreachable EditRoleAction#beforeObjectCommit (above); the page is reachable by any signed-in user. Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editRoles.jsp writes the raw request parameters oid (55), returnto (56) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): /do/edit/roles runs EditObjectAction#doExecute with type net.sf.xplanner.domain.Project (WAR:WEB-INF/action-servlet.xml:400-404), so a direct request with merge=true binds the request parameters onto the loaded project as in row 78 (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/EditRoleAction.java EditRoleAction#beforeObjectCommit; SRC:src/com/technoetic/xplanner/actions/AbstractAction.java AbstractAction#execute. WAR: classes byte-identical to the v1.1a4 release. The role-saving method takes an extra Session parameter, so it does not override the hook that AbstractAction#execute calls, and nothing else calls it. Stage 3 W001 (BA-001-13, MC-A-06, W001-F-07): A-C-040 (part A blocked, reclassified as an observed failure by the W001 lead). Other parameter forms were not tried, and the parameters the editor requires were not re-read from source (no new research). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks A-C-040).</t>
   </si>
   <si>
     <t>UF-003</t>
@@ -511,7 +511,7 @@
     <t>Table of people with mailto links; default sort by name.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:313; WAR:WEB-INF/jsp/view/people.jsp (writableTable peopleToShow, columns userId/name/initials/phone/email); linked from projects.jsp:161 and project.jsp:96. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/struts-config.xml:313; WAR:WEB-INF/jsp/view/people.jsp (writableTable peopleToShow, columns userId/name/initials/phone/email); linked from projects.jsp:161 and project.jsp:96. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks setup-C-004, F-C-015; open residual scope R-28 (d)).</t>
   </si>
   <si>
     <t>Hidden people are listed only for users with admin.hide on system.person; others see only visible people.</t>
@@ -520,10 +520,10 @@
     <t>Retired accounts stay out of normal views.</t>
   </si>
   <si>
-    <t>Admins see hidden people; others do not.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/people.jsp (isUserAuthorized permission="admin.hide" resourceType="system.person"; useBeans where hidden = false). Server-side enforcement (CHK-002, BA-001-04): the filter is applied while the server renders people.jsp; /do/view/people is a DispatchForward with authorization switched off (row 28), and the page of a hidden person remains reachable by oid (ViewPersonAction has no permission check, row 29). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>Admins see hidden people; others do not (source claim). Live (W001): a person whose hidden flag is stored is still listed on /do/view/people for the viewer, editor, admin and system-administrator role accounts and for an editor of project 221.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/people.jsp (isUserAuthorized permission="admin.hide" resourceType="system.person"; useBeans where hidden = false). Server-side enforcement (CHK-002, BA-001-04): the filter is applied while the server renders people.jsp; /do/view/people is a DispatchForward with authorization switched off (row 28), and the page of a hidden person remains reachable by oid (ViewPersonAction has no permission check, row 29). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Stage 3 W001 (BA-001-13, MC-A-07, W001-F-08): the hidden test person is listed for every account (A-C-042). The source claim is kept and contradicted live; the list filter was not re-read from source (no new research). Status Yes -&gt; Partial. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks A-C-041, A-C-042).</t>
   </si>
   <si>
     <t>With a projectId parameter the list is restricted to people with a role on that project and titled with the project name.</t>
@@ -532,25 +532,25 @@
     <t>Per-project team view.</t>
   </si>
   <si>
-    <t>Title "People in project &lt;name&gt;"; only project members listed.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/people.jsp (bean:parameter projectId; PermissionHelper.getPeopleWithProjectRole; message people.project.title). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>Heading "People on project: &lt;name&gt;" (HTML title "People"); the project members are listed, including the system administrators through their project-0 role.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/people.jsp (bean:parameter projectId; PermissionHelper.getPeopleWithProjectRole; message people.project.title). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Stage 3 W001 (BA-001-13, MC-A-08, W001-F-09): /do/view/people?projectId=220 shows the heading "People on project: S3 Shared" (key people.project.title) and lists the three project members plus the two system administrators, who hold only the project-0 role (setup-C-030). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-030).</t>
   </si>
   <si>
     <t>View person page</t>
   </si>
   <si>
-    <t>A person page shows the person's active, planned and completed tasks, stories as customer and as tracker, and future tasks.</t>
+    <t>A person page shows the person's active, planned and completed tasks, stories as customer and as tracker, and future tasks. Live (W001): the page answers HTTP 500 for a person who tracks a story and accepts a completed task with a time entry.</t>
   </si>
   <si>
     <t>Personal work overview.</t>
   </si>
   <si>
-    <t>Sections with tables per category or "none" messages; links to iteration, story and task.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/struts-config.xml:317-319; WAR:WEB-INF/action-servlet.xml:342-350 (ViewPersonAction, authorizationRequired=false); WAR:WEB-INF/jsp/view/person.jsp with WAR:WEB-INF/jsp/view/personTaskTableFragment.jsp and WAR:WEB-INF/jsp/view/personStoryTableFragment.jsp; class com.technoetic.xplanner.actions.ViewPersonAction (strings currentActiveTasksForPerson ... storiesForTracker). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ViewPersonAction.java ViewPersonAction#doExecute. WAR: classes byte-identical to the v1.1a4 release; SOURCE MISMATCH: the WAR bytecode of ViewPersonAction differs from the r426 source (WAR governs). The bytecode sets the recorded six attributes plus "person", loading the tasks through TaskDao#getCurrentTasksForPerson and TaskRepository and the stories through UserStoryDao; the r426 source uses a StoryRepository and declares setStoryRepository and setTaskRepository instead of setTaskDao and setUserStoryDao. This is the only class whose method names differ between source and bytecode.</t>
+    <t>Sections with tables per category or "none" messages; links to iteration, story and task. Alternative outcome (W001): for a person who tracks a story and accepts a completed task with a time entry the page answers HTTP 500 (ELException reading cachedActualHours, root LazyInitializationException for UserStory.tasks and Task.timeEntries: lazy loading outside the session); the page of a person without such work renders.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/struts-config.xml:317-319; WAR:WEB-INF/action-servlet.xml:342-350 (ViewPersonAction, authorizationRequired=false); WAR:WEB-INF/jsp/view/person.jsp with WAR:WEB-INF/jsp/view/personTaskTableFragment.jsp and WAR:WEB-INF/jsp/view/personStoryTableFragment.jsp; class com.technoetic.xplanner.actions.ViewPersonAction (strings currentActiveTasksForPerson ... storiesForTracker). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ViewPersonAction.java ViewPersonAction#doExecute. WAR: classes byte-identical to the v1.1a4 release; SOURCE MISMATCH: the WAR bytecode of ViewPersonAction differs from the r426 source (WAR governs). The bytecode sets the recorded six attributes plus "person", loading the tasks through TaskDao#getCurrentTasksForPerson and TaskRepository and the stories through UserStoryDao; the r426 source uses a StoryRepository and declares setStoryRepository and setTaskRepository instead of setTaskDao and setUserStoryDao. This is the only class whose method names differ between source and bytecode. Stage 3 W001 (BA-001-13, MC-A-09, W001-F-10): /do/view/person?oid=210 answered HTTP 500 three times (setup-C-032); the page of a person without such work renders (A-C-043). Status Yes -&gt; Partial. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-031, setup-C-032).</t>
   </si>
   <si>
     <t>From a task row on the person page an authorized user can jump to time entry or task edit.</t>
@@ -562,7 +562,7 @@
     <t>Clock and edit icons per active task when the user may edit it.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/personTaskTableFragment.jsp (isUserAuthorized task edit; links /do/edit/time and /do/edit/task). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); UpdateTimeAction or EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/jsp/view/personTaskTableFragment.jsp (isUserAuthorized task edit; links /do/edit/time and /do/edit/task). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); UpdateTimeAction or EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Stage 3 W001 (BA-001-13, MC-A-09): depends on row 40: the person page that carries these icons answered HTTP 500 for a person who tracks a story and accepts a completed task with a time entry (setup-C-032); the icons were observed on the page of a person without time entries (A-C-043). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-033, A-C-043).</t>
   </si>
   <si>
     <t>The edit link on a person page is shown only to that person or to someone with admin.edit on system.person for some project.</t>
@@ -574,7 +574,7 @@
     <t>Edit link visible accordingly; links to people list, timesheet and exports.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/person.jsp (remoteUserId == person.getId() || hasPermissionForSomeProject(..., "admin.edit")). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction (except the role rules in row 31) performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/jsp/view/person.jsp (remoteUserId == person.getId() || hasPermissionForSomeProject(..., "admin.edit")). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction (except the role rules in row 31) performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-029).</t>
   </si>
   <si>
     <t>Create person</t>
@@ -589,7 +589,7 @@
     <t>Person saved; user returned to the people list (returnto).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/people.jsp (link /do/edit/person under create.person); WAR:WEB-INF/struts-config.xml:321-326; WAR:WEB-INF/jsp/edit/editPerson.jsp; class com.technoetic.xplanner.actions.EditPersonAction. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editPerson.jsp writes the raw request parameters oid (39), returnto (43) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/person that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Person object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). The settable properties include ones the person editor does not show, for example the stored password digest (Person#setPassword) and the hidden flag; EditPersonAction#beforeObjectCommit still reads the new-password and role fields from the form. No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/net/sf/xplanner/domain/Person.java Person#setPassword (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/actions/EditPersonAction.java EditPersonAction#beforeObjectCommit; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject, #doExecute. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
+    <t>WAR:WEB-INF/jsp/view/people.jsp (link /do/edit/person under create.person); WAR:WEB-INF/struts-config.xml:321-326; WAR:WEB-INF/jsp/edit/editPerson.jsp; class com.technoetic.xplanner.actions.EditPersonAction. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editPerson.jsp writes the raw request parameters oid (39), returnto (43) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/person that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Person object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). The settable properties include ones the person editor does not show, for example the stored password digest (Person#setPassword) and the hidden flag; EditPersonAction#beforeObjectCommit still reads the new-password and role fields from the form. No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/net/sf/xplanner/domain/Person.java Person#setPassword (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/actions/EditPersonAction.java EditPersonAction#beforeObjectCommit; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject, #doExecute. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Stage 3 W001 (BA-001-13, MC-A-04, W001-F-05): the create.person condition does not hide the Add Person link (/do/edit/person) from viewers or editors live: it is shown to both (setup-C-022) and to the admin and system-administrator accounts (setup-C-021); a viewer can create a person (A-C-025, A-C-044). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-002, setup-C-022, A-C-025, A-C-044).</t>
   </si>
   <si>
     <t>Name, user ID, e-mail and initials are mandatory; password and confirmation must match.</t>
@@ -601,7 +601,7 @@
     <t>Messages "Missing name.", "Missing user Id.", "Missing email.", "Missing initials.", "Passwords do not match".</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.PersonEditorForm#validate (strings person.editor.missing_name, missing_user_id, missing_email, missing_initials, password_mismatch); ResourceBundle.properties same keys. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/PersonEditorForm.java PersonEditorForm#validate (withheld file, cited by path only). WAR: classes byte-identical to the v1.1a4 release. Name, user ID, e-mail and initials are required; the confirmation is compared only when a new password is given.</t>
+    <t>class com.technoetic.xplanner.forms.PersonEditorForm#validate (strings person.editor.missing_name, missing_user_id, missing_email, missing_initials, password_mismatch); ResourceBundle.properties same keys. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/PersonEditorForm.java PersonEditorForm#validate (withheld file, cited by path only). WAR: classes byte-identical to the v1.1a4 release. Name, user ID, e-mail and initials are required; the confirmation is compared only when a new password is given. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-045, A-C-046).</t>
   </si>
   <si>
     <t>A duplicate user ID is rejected on the editor.</t>
@@ -610,10 +610,10 @@
     <t>User IDs identify logins and must be unique.</t>
   </si>
   <si>
-    <t>Editor redisplayed with "User Id exists."</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/struts-config.xml:323-325 (DuplicateUserIdException -&gt; editPerson.jsp, key person.editor.userid_exist); db-changelog.xml:252 (unique index userId). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); the WAR db-changelog.xml differs from the SVN copy, which is withheld (WAR governs). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>HTTP 500 error page (database constraint violation); "User Id exists." is not shown and no duplicate is stored (W001; the outcome rests on a database constraint and may depend on this runtime (Tomcat 9 / JRE 8, MySQL 5.7)).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/struts-config.xml:323-325 (DuplicateUserIdException -&gt; editPerson.jsp, key person.editor.userid_exist); db-changelog.xml:252 (unique index userId). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); the WAR db-changelog.xml differs from the SVN copy, which is withheld (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Stage 3 W001 (BA-001-13, MC-A-10, W001-F-11): POST of the add-person form with an existing user ID, twice: HTTP 500 (ConstraintViolationException, BatchUpdateException), message not shown, no duplicate (A-C-047). The editor-message path above is not reached live. Status Yes -&gt; Partial. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks A-C-047).</t>
   </si>
   <si>
     <t>Edit person and password</t>
@@ -628,7 +628,7 @@
     <t>Changes saved; returnto page shown.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (form /do/edit/person, Update button); WAR:WEB-INF/security.xml:15 (/do/edit/person in viewing constraint). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction (except the role rules in row 31) performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 43 applies to every /do/edit/person request (Inferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002): the unvalidated returnto redirect of row 43 applies (Q3 facts). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (form /do/edit/person, Update button); WAR:WEB-INF/security.xml:15 (/do/edit/person in viewing constraint). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction (except the role rules in row 31) performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 43 applies to every /do/edit/person request (Inferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002): the unvalidated returnto redirect of row 43 applies (Q3 facts). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-007, A-C-048).</t>
   </si>
   <si>
     <t>The password fields are shown only when the active login module can change passwords; a new password is stored as a salted digest.</t>
@@ -640,7 +640,7 @@
     <t>New password / confirm fields; saved password replaces the old one.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp:78-79 (AuthenticatorImpl.getLoginModule(request).isCapableOfChangingPasswords()); class XPlannerLoginModule#changePassword/#encodePassword (SecureRandom salt, MD5, Base64). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/module/XPlannerLoginModule.java XPlannerLoginModule#isCapableOfChangingPasswords, #changePassword, #encodePassword (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/AuthenticatorImpl.java AuthenticatorImpl#getLoginModule. WAR: classes byte-identical to the v1.1a4 release. The XPlanner module declares that it can change passwords, and changePassword stores a newly salted digest of the new password and commits it. Provenance (fixed baseline, see reconnaissance GAP-005): P-02: spring-beans.xml:65-68 sets defaultAutoCommit=false with a comment describing a MySQL fix for the login module's changePassword commit; this setting is treated as patch-introduced.</t>
+    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp:78-79 (AuthenticatorImpl.getLoginModule(request).isCapableOfChangingPasswords()); class XPlannerLoginModule#changePassword/#encodePassword (SecureRandom salt, MD5, Base64). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/module/XPlannerLoginModule.java XPlannerLoginModule#isCapableOfChangingPasswords, #changePassword, #encodePassword (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/security/AuthenticatorImpl.java AuthenticatorImpl#getLoginModule. WAR: classes byte-identical to the v1.1a4 release. The XPlanner module declares that it can change passwords, and changePassword stores a newly salted digest of the new password and commits it. Provenance (fixed baseline, see reconnaissance GAP-005): P-02: spring-beans.xml:65-68 sets defaultAutoCommit=false with a comment describing a MySQL fix for the login module's changePassword commit; this setting is treated as patch-introduced. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks setup-C-008, A-C-049; open residual scope R-37 (e)).</t>
   </si>
   <si>
     <t>Users with hide permission can mark a person hidden.</t>
@@ -649,25 +649,25 @@
     <t>Retire accounts without deleting history.</t>
   </si>
   <si>
-    <t>Hidden select Yes/No; hidden people disappear from normal lists.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (isUserAuthorized person hide; select hidden). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>Hidden select Yes/No; the hidden flag is stored (the editor shows it set), but hidden people stay listed on /do/view/people for every observed role (W001).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/edit/editPerson.jsp (isUserAuthorized person hide; select hidden). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditPersonAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Stage 3 W001 (BA-001-13, MC-A-07, W001-F-08): the system administrator saved hidden=true (302, stored) and the person stayed listed for every account (A-C-050). Status Yes -&gt; Partial. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks A-C-050).</t>
   </si>
   <si>
     <t>Delete person</t>
   </si>
   <si>
-    <t>A person can be deleted through /do/delete/person; nothing cascades. If the person is a story customer or a notification receiver, the database foreign keys are expected to reject the delete; task acceptor, story tracker, time-entry person and person-role references are plain columns and are left dangling.</t>
+    <t>A person can be deleted through /do/delete/person, which no page links to (the people list and the person page offer no delete control; reachable by URL only, W001); nothing cascades. If the person is a story customer or a notification receiver, the database foreign keys are expected to reject the delete; task acceptor, story tracker, time-entry person and person-role references are plain columns and are left dangling. Live (W001): a person without references is removed; the delete of a story customer is rejected (HTTP 500, not removed); a task acceptor is removed, and the task page and its story page then answer HTTP 500.</t>
   </si>
   <si>
     <t>Removes a person record.</t>
   </si>
   <si>
-    <t>Person removed, or a database error when foreign keys refer to the person (runtime unverified).</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/struts-config.xml:348; WAR:WEB-INF/action-servlet.xml:370-374 (DeleteObjectAction type Person). The person action metadata defines only "edit" (DomainMetaDataRepository#init) and no live link to /do/delete/person was found (linkgraph.txt). BA-001-04 cascade sweep: net.sf.xplanner.domain.Person has no relationship annotations; WAR:WEB-INF/classes/db-changelog.xml:260 (notification_receivers.person_id -&gt; person) and :262 (story.customer_id -&gt; person) are the only foreign keys to person. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute; SRC:src/net/sf/xplanner/domain/Person.java (withheld file, cited by path only: no relationship or cascade annotation). WAR: classes byte-identical to the v1.1a4 release. The delete publishes a delete event and deletes the object; the outcome with referencing rows depends on the database foreign keys. Live question: Deleting a person who is a story customer: is the delete rejected by the database, and do task, time-entry and role rows keep the dangling id?</t>
+    <t>Person removed (302) when nothing refers to it; for a story customer HTTP 500 and the person is kept; for a task acceptor the person is removed, and pages that show the deleted acceptor (the task and its story) answer HTTP 500 (W001). The notification-receiver, tracker, time-entry and role cases were not observed live.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/struts-config.xml:348; WAR:WEB-INF/action-servlet.xml:370-374 (DeleteObjectAction type Person). The person action metadata defines only "edit" (DomainMetaDataRepository#init) and no live link to /do/delete/person was found (linkgraph.txt). BA-001-04 cascade sweep: net.sf.xplanner.domain.Person has no relationship annotations; WAR:WEB-INF/classes/db-changelog.xml:260 (notification_receivers.person_id -&gt; person) and :262 (story.customer_id -&gt; person) are the only foreign keys to person. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute; SRC:src/net/sf/xplanner/domain/Person.java (withheld file, cited by path only: no relationship or cascade annotation). WAR: classes byte-identical to the v1.1a4 release. The delete publishes a delete event and deletes the object; the outcome with referencing rows depends on the database foreign keys. Live question: Deleting a person who is a story customer: is the delete rejected by the database, and do task, time-entry and role rows keep the dangling id? Stage 3 W001 (BA-001-13, MC-B-02, W001-F-12): A-C-052 (story customer), A-C-053 (task acceptor), A-C-054 (no delete link on the people list or the person page). Status stays Inferred: the row-level status cannot be split per case, and the other reference cases were not observed. Stage 3 W001 live answer (BA-001-13, MC-C-07): The delete of a story customer is rejected (HTTP 500, not removed). A deleted task acceptor leaves a dangling reference: the task and story pages then answer HTTP 500. Time-entry and role rows were not inspected (database level) (A-C-052, A-C-053). The D/F correction is under W001-F-12. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks A-C-051, A-C-052, A-C-053, A-C-054).</t>
   </si>
   <si>
     <t>Import people from a file</t>
@@ -679,10 +679,10 @@
     <t>Bulk onboarding.</t>
   </si>
   <si>
-    <t>Upload form and per-line checks work, but saving the first valid line is expected to fail with a null reference, because the person DAO is never injected; no results table with "Success" is expected (runtime unverified).</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/people.jsp (link /do/import/people); WAR:WEB-INF/struts-config.xml:329-330; WAR:WEB-INF/jsp/edit/importPeople.jsp; class com.technoetic.xplanner.actions.ImportPeopleAction (BufferedReader.readLine, String.split ",", PersonDao.save); ResourceBundle.properties people.import.editor.importFileFormat. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); ImportPeopleAction (its AuthorizationException handler is unreachable because nothing on its path raises one) performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Wiring (BA-001-07, mechanism (a)): WAR:WEB-INF/action-servlet.xml:2 sets default-autowire="byName"; the bean /import/people (:359) has no properties; ImportPeopleAction#setPersonDao carries no annotation, and no Spring file defines a bean named personDao (WAR:WEB-INF/classes/spring-dao.xml:17-57 define commonDao, taskDao, userStoryDao, projectDao, viewDao, dataSampleDao, settingDao, objectTypeDao and attributeDao; PersonDaoImpl has no stereotype and no component scan covers net.sf.xplanner.dao). ImportPeopleAction$1#run calls personDao.save for each accepted line inside the transaction template; the handlers of #execute catch DuplicateUserIdException, the local import exception and AuthorizationException only (exception table), so the null reference is expected to propagate to the error page. Sweep: .migration-tmp/stage-01/out/wiring-07.txt, wiring-impact-07.txt. Corrected in BA-001-07 (Source: stage-02-pass-005 F-001). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/importPeople.jsp writes the raw request parameters returnto (34,78), formFileName (39) [parameter (lines); line 78 passes returnto as the page attribute of html:link] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/ImportPeopleAction.java ImportPeopleAction#execute, #setPersonDao. WAR: classes byte-identical to the v1.1a4 release. The setter has no annotation and no bean named personDao exists, as recorded; the null-reference outcome is a runtime effect. Live question: Does uploading a file with one valid line fail on save?</t>
+    <t>The import page and form work. Uploading a synthetic 3-line text file (a malformed line, an empty user ID and one valid line) ends in HTTP 500 (IndexOutOfBoundsException) before any per-line status is shown: no results table and no person created (W001; which line triggers the failure was not isolated). The source-based expectation that saving the first valid line fails with a null reference, because the person DAO is never injected, was not reached.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/people.jsp (link /do/import/people); WAR:WEB-INF/struts-config.xml:329-330; WAR:WEB-INF/jsp/edit/importPeople.jsp; class com.technoetic.xplanner.actions.ImportPeopleAction (BufferedReader.readLine, String.split ",", PersonDao.save); ResourceBundle.properties people.import.editor.importFileFormat. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); ImportPeopleAction (its AuthorizationException handler is unreachable because nothing on its path raises one) performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Wiring (BA-001-07, mechanism (a)): WAR:WEB-INF/action-servlet.xml:2 sets default-autowire="byName"; the bean /import/people (:359) has no properties; ImportPeopleAction#setPersonDao carries no annotation, and no Spring file defines a bean named personDao (WAR:WEB-INF/classes/spring-dao.xml:17-57 define commonDao, taskDao, userStoryDao, projectDao, viewDao, dataSampleDao, settingDao, objectTypeDao and attributeDao; PersonDaoImpl has no stereotype and no component scan covers net.sf.xplanner.dao). ImportPeopleAction$1#run calls personDao.save for each accepted line inside the transaction template; the handlers of #execute catch DuplicateUserIdException, the local import exception and AuthorizationException only (exception table), so the null reference is expected to propagate to the error page. Sweep: .migration-tmp/stage-01/out/wiring-07.txt, wiring-impact-07.txt. Corrected in BA-001-07 (Source: stage-02-pass-005 F-001). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/importPeople.jsp writes the raw request parameters returnto (34,78), formFileName (39) [parameter (lines); line 78 passes returnto as the page attribute of html:link] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/ImportPeopleAction.java ImportPeopleAction#execute, #setPersonDao. WAR: classes byte-identical to the v1.1a4 release. The setter has no annotation and no bean named personDao exists, as recorded; the null-reference outcome is a runtime effect. Live question: Does uploading a file with one valid line fail on save? Stage 3 W001 (BA-001-13, MC-A-04, W001-F-05): the create.person condition does not hide the Import People link (/do/import/people) from viewers or editors live (setup-C-023). Stage 3 W001 live answer (BA-001-13, MC-C-08): A 3-line file (malformed, empty user ID, one valid line) failed with HTTP 500 (IndexOutOfBoundsException) before any per-line status or save; a file with only one valid line was not tried (A-C-056). The D/F correction is under W001-F-13. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-023, A-C-055, A-C-056).</t>
   </si>
   <si>
     <t>Malformed lines and empty user IDs are reported per line before any save; the "User already exists" outcome can only come from the save, which is expected to fail first (row 50).</t>
@@ -691,10 +691,10 @@
     <t>Partial failures are visible.</t>
   </si>
   <si>
-    <t>Statuses "Entry is not formated properly" and "User id can not be empty" for the lines checked before the save; "User already exists" is not expected (runtime unverified).</t>
-  </si>
-  <si>
-    <t>class ImportPeopleAction (strings people.import.status.wrong_entry_format, empty_userId, userId_exists); ResourceBundle.properties same keys. Wiring (BA-001-07): the wrong_entry_format and empty_userId checks run in ImportPeopleAction#execute before ImportPeopleAction$1#run; userId_exists comes from DuplicateUserIdException, which only PersonDao.save raises (row 50). Source: stage-02-pass-005 F-001. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ImportPeopleAction.java ImportPeopleAction#execute. WAR: classes byte-identical to the v1.1a4 release. The format and empty-id checks run per line before the save; the duplicate outcome needs the save.</t>
+    <t>No per-line status is shown: the upload of the 3-line file ended in the HTTP 500 page before any status (W001), so "Entry is not formated properly" and "User id can not be empty" were not displayed; "User already exists" is not expected (row 50).</t>
+  </si>
+  <si>
+    <t>class ImportPeopleAction (strings people.import.status.wrong_entry_format, empty_userId, userId_exists); ResourceBundle.properties same keys. Wiring (BA-001-07): the wrong_entry_format and empty_userId checks run in ImportPeopleAction#execute before ImportPeopleAction$1#run; userId_exists comes from DuplicateUserIdException, which only PersonDao.save raises (row 50). Source: stage-02-pass-005 F-001. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ImportPeopleAction.java ImportPeopleAction#execute. WAR: classes byte-identical to the v1.1a4 release. The format and empty-id checks run per line before the save; the duplicate outcome needs the save. Stage 3 W001 (BA-001-13, MC-A-11, W001-F-13): the same upload as row 50 showed no per-line status (A-C-057). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks A-C-057).</t>
   </si>
   <si>
     <t>Submitting the people import without a file is rejected before any line is read.</t>
@@ -703,10 +703,10 @@
     <t>The import needs a file.</t>
   </si>
   <si>
-    <t>Import page redisplayed with "Please select a file to import."</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.forms.ImportPeopleForm extends ImportForm without its own validate; ImportForm#validate raises import.status.no_import_file when the form is submitted without a file (bytecode constants); form bean import/people (WAR:WEB-INF/struts-config.xml:48-49) on the mapping /import/people (:329-330). Message at WAR:WEB-INF/classes/ResourceBundle.properties:39. CHK-005 (BA-001-05). Source: stage-02-pass-003 F-003. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/ImportForm.java ImportForm#validate. WAR: classes byte-identical to the v1.1a4 release. A submitted form without a file name raises the no-import-file key.</t>
+    <t>HTTP 500 error page (AbstractMethodError); "Please select a file to import." is not shown (W001; lead interpretation: probably the bundled Struts 1.2 multipart wrapper on a Servlet 3+ container, so it may depend on this runtime (Tomcat 9)).</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.ImportPeopleForm extends ImportForm without its own validate; ImportForm#validate raises import.status.no_import_file when the form is submitted without a file (bytecode constants); form bean import/people (WAR:WEB-INF/struts-config.xml:48-49) on the mapping /import/people (:329-330). Message at WAR:WEB-INF/classes/ResourceBundle.properties:39. CHK-005 (BA-001-05). Source: stage-02-pass-003 F-003. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/ImportForm.java ImportForm#validate. WAR: classes byte-identical to the v1.1a4 release. A submitted form without a file name raises the no-import-file key. Stage 3 W001 (BA-001-13, MC-A-12, W001-F-14): submitting the import form without a file answered HTTP 500 (java.lang.AbstractMethodError) (A-C-058). Status Yes -&gt; Partial. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks A-C-058).</t>
   </si>
   <si>
     <t>The import page offers a template download link.</t>
@@ -718,7 +718,7 @@
     <t>Link to files/peopleImportTemplate.xls (an Excel file, although the importer reads comma-separated text).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/importPeople.jsp (link to people.import.download.template.file.name); WAR:files/peopleImportTemplate.xls; ResourceBundle.properties:574. Format mismatch between .xls template and line/comma parser is recorded as an unresolved question. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ImportPeopleAction.java ImportPeopleAction#execute (reads text lines). WAR: importPeople.jsp and files/peopleImportTemplate.xls identical to the SVN webapp copies. The link points to an Excel file while the importer reads comma-separated text lines.</t>
+    <t>WAR:WEB-INF/jsp/edit/importPeople.jsp (link to people.import.download.template.file.name); WAR:files/peopleImportTemplate.xls; ResourceBundle.properties:574. Format mismatch between .xls template and line/comma parser is recorded as an unresolved question. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ImportPeopleAction.java ImportPeopleAction#execute (reads text lines). WAR: importPeople.jsp and files/peopleImportTemplate.xls identical to the SVN webapp copies. The link points to an Excel file while the importer reads comma-separated text lines. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-059).</t>
   </si>
   <si>
     <t>UF-004</t>
@@ -739,7 +739,7 @@
     <t>Page titled system info with version 1.1a4, build date/revision, dialect, driver, DB URL/user (password masked), servlet version, memory.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/common/footer.jsp:38 (link appUrl + /do/systemInfo); WAR:WEB-INF/struts-config.xml:160-162 (forward to unexpectedError.jsp); class com.technoetic.xplanner.actions.SystemInfoAction (attribute isSystemInfo); class com.technoetic.xplanner.SystemInfo#getDatabaseInfo (strings "Database User Password", "******"). Request echo (BA-001-07, mechanism (b)): /do/systemInfo forwards to WAR:WEB-INF/jsp/common/unexpectedError.jsp (WAR:WEB-INF/struts-config.xml:160-161), which also lists the request information of the current request: referer, URL, URI, query string, all request parameters and all request attributes (unexpectedError.jsp:100-121). Values in those lists are HTML-encoded by BoxedListTag (StringUtilities#htmlEncode in #getStringValue and #renderRow). Source: stage-02-pass-005 F-003. Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/actions/SystemInfoAction.java SystemInfoAction; SRC:src/com/technoetic/xplanner/SystemInfo.java SystemInfo#getDatabaseInfo (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/util/StringUtilities.java StringUtilities#htmlEncode. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Provenance (fixed baseline, see reconnaissance GAP-005): P-01: database engine, dialect, driver, URL and credential values come from the rewritten entries xplanner.properties / xplanner-custom.properties that carry the known MySQL patch; the upstream values cannot be separated.</t>
+    <t>WAR:WEB-INF/jsp/common/footer.jsp:38 (link appUrl + /do/systemInfo); WAR:WEB-INF/struts-config.xml:160-162 (forward to unexpectedError.jsp); class com.technoetic.xplanner.actions.SystemInfoAction (attribute isSystemInfo); class com.technoetic.xplanner.SystemInfo#getDatabaseInfo (strings "Database User Password", "******"). Request echo (BA-001-07, mechanism (b)): /do/systemInfo forwards to WAR:WEB-INF/jsp/common/unexpectedError.jsp (WAR:WEB-INF/struts-config.xml:160-161), which also lists the request information of the current request: referer, URL, URI, query string, all request parameters and all request attributes (unexpectedError.jsp:100-121). Values in those lists are HTML-encoded by BoxedListTag (StringUtilities#htmlEncode in #getStringValue and #renderRow). Source: stage-02-pass-005 F-003. Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/actions/SystemInfoAction.java SystemInfoAction; SRC:src/com/technoetic/xplanner/SystemInfo.java SystemInfo#getDatabaseInfo (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/util/StringUtilities.java StringUtilities#htmlEncode. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Provenance (fixed baseline, see reconnaissance GAP-005): P-01: database engine, dialect, driver, URL and credential values come from the rewritten entries xplanner.properties / xplanner-custom.properties that carry the known MySQL patch; the upstream values cannot be separated. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-060).</t>
   </si>
   <si>
     <t>Error pages</t>
@@ -754,7 +754,7 @@
     <t>Error page with message, support links (support.issue.url), "Cause" and "Stack Trace" boxes.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:16-29 (error-page JspException, ServletException, Throwable -&gt; unexpectedError.jsp); WAR:WEB-INF/jsp/common/unexpectedError.jsp; xplanner.properties:289-309 (error.filingInfo). Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; error.unknownError and error.moreInfo are defined only in the default and "--" bundles; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Request echo (BA-001-07, mechanism (b)): unexpectedError.jsp is the container error page for every JspException, ServletException and Throwable (WAR:WEB-INF/web.xml:16-29). It prints the first lines of the exception message unescaped with &lt;%= message %&gt; (unexpectedError.jsp:66) and lists the referer, URL, query string, every request parameter (including any password field of the failing request) and every request attribute (:100-121; values HTML-encoded by BoxedListTag). Observed risk only (Q3 deferred). Source: stage-02-pass-005 F-003. Page-text keys (BA-001-09, pass-007 F-003, check (j)): the page title comes from a scriptlet-selected key (WAR:WEB-INF/jsp/common/unexpectedError.jsp:19,27,47): error.title, defined in all bundles except de and es, and, when the same page serves the system information page (row 55), system.info.title, defined only in the default and "--" bundles. The tiles:default layout adds the footer keys app.label.version (all 10 bundles) and footer.message (only the default, "--" and de bundles; WAR:WEB-INF/jsp/common/footer.jsp:25,38) and the breadcrumb link text navigation.top (all 10 bundles; WAR:WEB-INF/tags/breadcrumb.tag:10). Bundles without a key fall back to the default text (framework behavior, GAP-011). None of these texts is credential-like (.migration-tmp/stage-01/out/public-keys-09.txt). Breadcrumb lookup (BA-001-10, pass-008 F-002 lead, check (l)): the error page uses the same tiles:default layout, and the layout breadcrumb (WAR:WEB-INF/jsp/layout/defaultLayout.jsp:44, WAR:WEB-INF/tags/breadcrumb.tag:10) reads the request parameter oid, or else fkey, and loads that object without a sign-in or permission check (class net.sf.xplanner.tags.NavigationBarTag#doEndTag, #setObject(int): the type attribute arrives as an empty string, so IdSearchHelper#search runs Session#get over Project, Iteration, UserStory, Task, Person and Note). #render then adds links whose texts are the names of the object's project, iteration, story, task or feature, and breadcrumb.tag:15,18 prints them with unescaped EL. The error page renders for every failing request, including one without a session, so the names of the object named by the failing request's oid or fkey are expected to be shown there too (Inferred; row 185; GAP-007; observed risk only, Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/net/sf/xplanner/tags/NavigationBarTag.java NavigationBarTag#doEndTag; SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search. WAR: classes byte-identical to the v1.1a4 release; values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/web.xml:16-29 (error-page JspException, ServletException, Throwable -&gt; unexpectedError.jsp); WAR:WEB-INF/jsp/common/unexpectedError.jsp; xplanner.properties:289-309 (error.filingInfo). Locale variants, public page (CHK-004, BA-001-06): quoted texts are from the default bundle; error.unknownError and error.moreInfo are defined only in the default and "--" bundles; bundles without a key fall back to the default text (framework behavior, GAP-011). No credential-like text in any variant (.migration-tmp/stage-01/out/unauth-06.txt; the only such text is login.instructions, row 9). Request echo (BA-001-07, mechanism (b)): unexpectedError.jsp is the container error page for every JspException, ServletException and Throwable (WAR:WEB-INF/web.xml:16-29). It prints the first lines of the exception message unescaped with &lt;%= message %&gt; (unexpectedError.jsp:66) and lists the referer, URL, query string, every request parameter (including any password field of the failing request) and every request attribute (:100-121; values HTML-encoded by BoxedListTag). Observed risk only (Q3 deferred). Source: stage-02-pass-005 F-003. Page-text keys (BA-001-09, pass-007 F-003, check (j)): the page title comes from a scriptlet-selected key (WAR:WEB-INF/jsp/common/unexpectedError.jsp:19,27,47): error.title, defined in all bundles except de and es, and, when the same page serves the system information page (row 55), system.info.title, defined only in the default and "--" bundles. The tiles:default layout adds the footer keys app.label.version (all 10 bundles) and footer.message (only the default, "--" and de bundles; WAR:WEB-INF/jsp/common/footer.jsp:25,38) and the breadcrumb link text navigation.top (all 10 bundles; WAR:WEB-INF/tags/breadcrumb.tag:10). Bundles without a key fall back to the default text (framework behavior, GAP-011). None of these texts is credential-like (.migration-tmp/stage-01/out/public-keys-09.txt). Breadcrumb lookup (BA-001-10, pass-008 F-002 lead, check (l)): the error page uses the same tiles:default layout, and the layout breadcrumb (WAR:WEB-INF/jsp/layout/defaultLayout.jsp:44, WAR:WEB-INF/tags/breadcrumb.tag:10) reads the request parameter oid, or else fkey, and loads that object without a sign-in or permission check (class net.sf.xplanner.tags.NavigationBarTag#doEndTag, #setObject(int): the type attribute arrives as an empty string, so IdSearchHelper#search runs Session#get over Project, Iteration, UserStory, Task, Person and Note). #render then adds links whose texts are the names of the object's project, iteration, story, task or feature, and breadcrumb.tag:15,18 prints them with unescaped EL. The error page renders for every failing request, including one without a session, so the names of the object named by the failing request's oid or fkey are expected to be shown there too (Inferred; row 185; GAP-007; observed risk only, Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/net/sf/xplanner/tags/NavigationBarTag.java NavigationBarTag#doEndTag; SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search. WAR: classes byte-identical to the v1.1a4 release; values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-061).</t>
   </si>
   <si>
     <t>Requesting a non-existent object shows "Object &lt;id&gt; not found".</t>
@@ -763,10 +763,10 @@
     <t>Clear feedback for stale links.</t>
   </si>
   <si>
-    <t>General error page with object-not-found message.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/struts-config.xml:82-86 (ObjectNotFoundException, UnresolvableObjectException -&gt; generalError.jsp); WAR:WEB-INF/jsp/common/generalError.jsp. Request-value flow (BA-001-07, mechanism (b)): for ObjectNotFoundException, WAR:WEB-INF/jsp/common/generalError.jsp:26 passes request.getParameter("oid") as arg0 of bean:message, which does not escape its arguments, so the raw parameter is written into the page (Inferred; observed risk only, Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>HTTP 500 with the generic error page "An error has occurred.", without the object id or a not-found text (W001, GET /do/view/project?oid=999999).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/struts-config.xml:82-86 (ObjectNotFoundException, UnresolvableObjectException -&gt; generalError.jsp); WAR:WEB-INF/jsp/common/generalError.jsp. Request-value flow (BA-001-07, mechanism (b)): for ObjectNotFoundException, WAR:WEB-INF/jsp/common/generalError.jsp:26 passes request.getParameter("oid") as arg0 of bean:message, which does not escape its arguments, so the raw parameter is written into the page (Inferred; observed risk only, Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Stage 3 W001 (BA-001-13, MC-A-13, W001-F-15): GET /do/view/project?oid=999999, twice: HTTP 500 "An error has occurred.", no id, no not-found text, no Cause or Stack Trace section (A-C-062). The not-found message path of the requirement is not reached for a project id; which exception the view raises was not re-read from source (no new research). Status Yes -&gt; Partial. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks A-C-062).</t>
   </si>
   <si>
     <t>Change display language</t>
@@ -781,22 +781,22 @@
     <t>Texts change to the selected language; user returned to returnto or projects.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:158; WAR:WEB-INF/action-servlet.xml:6; class com.technoetic.xplanner.actions.ChangeLocaleAction (strings "language", "org.apache.struts.action.LOCALE"); WAR:WEB-INF/classes/ResourceBundle*.properties (10 files). No live link to /do/changeLocale was found (linkgraph.txt). Redirect target (BA-001-08, pass-006 F-002, check (e)): ChangeLocaleAction#execute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only an empty value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ChangeLocaleAction.java ChangeLocaleAction#execute. WAR: classes byte-identical to the v1.1a4 release. The action stores new Locale(language) in the session (the default locale when empty) and redirects to returnto or the projects list.</t>
+    <t>WAR:WEB-INF/struts-config.xml:158; WAR:WEB-INF/action-servlet.xml:6; class com.technoetic.xplanner.actions.ChangeLocaleAction (strings "language", "org.apache.struts.action.LOCALE"); WAR:WEB-INF/classes/ResourceBundle*.properties (10 files). No live link to /do/changeLocale was found (linkgraph.txt). Redirect target (BA-001-08, pass-006 F-002, check (e)): ChangeLocaleAction#execute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only an empty value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ChangeLocaleAction.java ChangeLocaleAction#execute. WAR: classes byte-identical to the v1.1a4 release. The action stores new Locale(language) in the session (the default locale when empty) and redirects to returnto or the projects list. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-063, A-C-064, L-C-003).</t>
   </si>
   <si>
     <t>Settings pages (work in progress)</t>
   </si>
   <si>
-    <t>A settings list shows Setting records and offers "add setting" to users with create.project.</t>
+    <t>A settings list shows Setting records and offers "Add Setting"; its source condition is create.project, but live the link is shown to the viewer as well as to the system administrator (W001).</t>
   </si>
   <si>
     <t>Intended central configuration.</t>
   </si>
   <si>
-    <t>Page headed "Settings" with a table; the add/edit editor JSP is missing.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/struts-config.xml:405,419-421; WAR:WEB-INF/jsp/view/settings.jsp (prints ${settings} raw; reuses projects.title); input WEB-INF/jsp/edit/editSetting.jsp ABSENT from WAR (GAP-003); db-changelog.xml changeSet 2-1 (setting, object_type). No live link to /do/view/settings found. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditObjectAction for Setting performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/setting that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Setting object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#doExecute, #populateObject. WAR: classes byte-identical to the v1.1a4 release. The list action and the generic editor exist; the editor JSP is absent from the WAR (GAP-003).</t>
+    <t>Page titled "XPlanner Projects" with the heading "Settings XPlanner Projects" and a table; "Add Setting" is shown to the viewer and to the system administrator (W001); the add/edit editor JSP is missing.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/struts-config.xml:405,419-421; WAR:WEB-INF/jsp/view/settings.jsp (prints ${settings} raw; reuses projects.title); input WEB-INF/jsp/edit/editSetting.jsp ABSENT from WAR (GAP-003); db-changelog.xml changeSet 2-1 (setting, object_type). No live link to /do/view/settings found. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditObjectAction for Setting performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/setting that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Setting object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#doExecute, #populateObject. WAR: classes byte-identical to the v1.1a4 release. The list action and the generic editor exist; the editor JSP is absent from the WAR (GAP-003). Stage 3 W001 (BA-001-13, MC-A-14, W001-F-16): GET /do/view/settings as viewer and as system administrator: both HTTP 200 with the title and heading above and "Add Setting" (A-C-065). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks A-C-065, A-C-066).</t>
   </si>
   <si>
     <t>Generic Spring MVC handlers exist for /setting/{objectType}/list and /setting/{objectType}/edit/{objectId}.</t>
@@ -808,7 +808,7 @@
     <t>The handlers print the objectType path value to standard output and return it as the view name. A plain value becomes /WEB-INF/jsp/&lt;objectType&gt;.jsp, where no JSP exists, so no usable page is expected; a value that starts with redirect: sends the browser to the rest of the value, and one that starts with forward: forwards inside the application (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:264-272,313-316 (SpringServlet on /setting/*); class net.sf.xplanner.web.CommonObjectHandler (@RequestMapping "/{objectType}/list", "/{objectType}/edit/{objectId}"). View selection (BA-001-08, pass-006 F-002, check (e)): CommonObjectHandler#list and #edit call PrintStream.println and return the {objectType} path variable as the view name; InternalResourceViewResolver adds the prefix /WEB-INF/jsp/ and the suffix .jsp (WAR:WEB-INF/classes/spring-web.xml:26-30; the Tiles view resolver at :31-35 is commented out). No JSP file lies directly in WEB-INF/jsp (0 files; the pages sit in 7 subdirectories), and a single path segment cannot name a subdirectory, so a value without a view prefix selects no existing page. Framework resolution (BA-001-09, pass-007 F-001, check (h)): InternalResourceViewResolver extends UrlBasedViewResolver, whose #createView in the bundled WAR:WEB-INF/lib/spring-webmvc-3.0.5.RELEASE.jar (bytecode listing) checks the view name before prefix and suffix are applied: a name that starts with "redirect:" becomes a RedirectView of the rest of the name (RedirectView#renderMergedOutputModel adds the context path only to a target that starts with "/", then HttpServletResponse#sendRedirect; spring-web.xml sets no redirect options, so the defaults apply), and a name that starts with "forward:" becomes an InternalResourceView forward of the rest. /setting/* is mapped to the Spring servlet and to WebSecurityFilter (WAR:WEB-INF/web.xml:164-167,313-316), so a signed-in user who follows /setting/redirect:&lt;target&gt;/list is redirected to &lt;target&gt;, and after a login the saved URL returns the user to it. One path segment cannot carry "/", but a scheme-qualified target whose scheme differs from the page is expected to be resolved by browsers as another host (Inferred; the container's handling of encoded slashes and the browser behavior are unverified; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/net/sf/xplanner/web/CommonObjectHandler.java CommonObjectHandler#list, #edit. WAR: classes byte-identical to the v1.1a4 release. Both handlers print the path value and return it as the view name, as recorded; the outcome is framework and browser behavior. Live question: What do /setting/&lt;value&gt;/list, /setting/redirect:&lt;target&gt;/list and /setting/forward:&lt;path&gt;/list return for a signed-in user?</t>
+    <t>WAR:WEB-INF/web.xml:264-272,313-316 (SpringServlet on /setting/*); class net.sf.xplanner.web.CommonObjectHandler (@RequestMapping "/{objectType}/list", "/{objectType}/edit/{objectId}"). View selection (BA-001-08, pass-006 F-002, check (e)): CommonObjectHandler#list and #edit call PrintStream.println and return the {objectType} path variable as the view name; InternalResourceViewResolver adds the prefix /WEB-INF/jsp/ and the suffix .jsp (WAR:WEB-INF/classes/spring-web.xml:26-30; the Tiles view resolver at :31-35 is commented out). No JSP file lies directly in WEB-INF/jsp (0 files; the pages sit in 7 subdirectories), and a single path segment cannot name a subdirectory, so a value without a view prefix selects no existing page. Framework resolution (BA-001-09, pass-007 F-001, check (h)): InternalResourceViewResolver extends UrlBasedViewResolver, whose #createView in the bundled WAR:WEB-INF/lib/spring-webmvc-3.0.5.RELEASE.jar (bytecode listing) checks the view name before prefix and suffix are applied: a name that starts with "redirect:" becomes a RedirectView of the rest of the name (RedirectView#renderMergedOutputModel adds the context path only to a target that starts with "/", then HttpServletResponse#sendRedirect; spring-web.xml sets no redirect options, so the defaults apply), and a name that starts with "forward:" becomes an InternalResourceView forward of the rest. /setting/* is mapped to the Spring servlet and to WebSecurityFilter (WAR:WEB-INF/web.xml:164-167,313-316), so a signed-in user who follows /setting/redirect:&lt;target&gt;/list is redirected to &lt;target&gt;, and after a login the saved URL returns the user to it. One path segment cannot carry "/", but a scheme-qualified target whose scheme differs from the page is expected to be resolved by browsers as another host (Inferred; the container's handling of encoded slashes and the browser behavior are unverified; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/net/sf/xplanner/web/CommonObjectHandler.java CommonObjectHandler#list, #edit. WAR: classes byte-identical to the v1.1a4 release. Both handlers print the path value and return it as the view name, as recorded; the outcome is framework and browser behavior. Live question: What do /setting/&lt;value&gt;/list, /setting/redirect:&lt;target&gt;/list and /setting/forward:&lt;path&gt;/list return for a signed-in user? Stage 3 W001 live answer (BA-001-13, MC-C-09): Plain value: 404. redirect: with a single-segment target: 302 with the rest of the value as Location; with a slash in the target: 404. forward: 404 for every value tried (A-C-067, A-C-068, L-C-004). The forward itself and the standard-output print are not observable. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks A-C-067, A-C-068, L-C-004; open residual scope R-42 (e)).</t>
   </si>
   <si>
     <t>Administrative and test actions</t>
@@ -823,7 +823,7 @@
     <t>The permission cache is cleared, or the Hibernate query cache is evicted; the actions return no forward, so the response has no page, and "cache cleared" / "hibernate cache cleared" are only log messages.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:233 (test-struts-config.xml loaded); WAR:WEB-INF/test-struts-config.xml:21-23; WAR:WEB-INF/test-action-servlet.xml:22-36; WAR:WEB-INF/security.xml:5 (bypass /do/invalidateHibernateCache); input JSP WEB-INF/jsp/admin/invalidateCache.jsp ABSENT. Server-side enforcement (CHK-002, BA-001-04): neither action checks a permission; InvalidateCacheAction obtains the authorizer only to reset its cache. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/admin/InvalidateCacheAction.java InvalidateCacheAction#execute; SRC:src/com/technoetic/xplanner/actions/admin/InvalidateHibernateCacheAction.java InvalidateHibernateCacheAction#execute. WAR: classes byte-identical to the v1.1a4 release. Both actions write "cache cleared" / "hibernate cache cleared" only to the log and return no forward (bytecode listing: aconst_null, areturn), so no confirmation page is sent; the Hibernate action evicts only the query cache (SessionFactory#evictQueries).</t>
+    <t>WAR:WEB-INF/web.xml:233 (test-struts-config.xml loaded); WAR:WEB-INF/test-struts-config.xml:21-23; WAR:WEB-INF/test-action-servlet.xml:22-36; WAR:WEB-INF/security.xml:5 (bypass /do/invalidateHibernateCache); input JSP WEB-INF/jsp/admin/invalidateCache.jsp ABSENT. Server-side enforcement (CHK-002, BA-001-04): neither action checks a permission; InvalidateCacheAction obtains the authorizer only to reset its cache. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/admin/InvalidateCacheAction.java InvalidateCacheAction#execute; SRC:src/com/technoetic/xplanner/actions/admin/InvalidateHibernateCacheAction.java InvalidateHibernateCacheAction#execute. WAR: classes byte-identical to the v1.1a4 release. Both actions write "cache cleared" / "hibernate cache cleared" only to the log and return no forward (bytecode listing: aconst_null, areturn), so no confirmation page is sent; the Hibernate action evicts only the query cache (SessionFactory#evictQueries). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks A-C-069, A-C-070; open residual scope R-43 (e), candidate outside the core (owner decision at Stage 4)).</t>
   </si>
   <si>
     <t>Test-support URLs can execute data sampling, the missing-time-entry notifier, shift the application clock (dayOffset) and set a property value.</t>
@@ -835,7 +835,7 @@
     <t>Action executes and redirects to returnto or projects.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/test-struts-config.xml:13-19; WAR:WEB-INF/test-action-servlet.xml:4-20 (CommandExecutorAction with txDataSamplingCommand / missingTimeEntryNotifier, PutTheClockForwardAction, EditPropertiesAction); class PutTheClockForwardAction (string "dayOffset"); class EditPropertiesAction ("propertyName", "propertyValue"). Redirect target (BA-001-08, pass-006 F-002, check (e)): CommandExecutorAction#execute, PutTheClockForwardAction#execute and EditPropertiesAction#execute each redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/CommandExecutorAction.java CommandExecutorAction#execute; SRC:src/com/technoetic/xplanner/actions/PutTheClockForwardAction.java PutTheClockForwardAction#execute; SRC:src/com/technoetic/xplanner/actions/EditPropertiesAction.java EditPropertiesAction#execute. WAR: classes byte-identical to the v1.1a4 release. The command runs, the clock moves by a positive dayOffset (any other value resets it), the property is set when a name and a value are given, and each action redirects to returnto or to the projects list.</t>
+    <t>WAR:WEB-INF/test-struts-config.xml:13-19; WAR:WEB-INF/test-action-servlet.xml:4-20 (CommandExecutorAction with txDataSamplingCommand / missingTimeEntryNotifier, PutTheClockForwardAction, EditPropertiesAction); class PutTheClockForwardAction (string "dayOffset"); class EditPropertiesAction ("propertyName", "propertyValue"). Redirect target (BA-001-08, pass-006 F-002, check (e)): CommandExecutorAction#execute, PutTheClockForwardAction#execute and EditPropertiesAction#execute each redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/CommandExecutorAction.java CommandExecutorAction#execute; SRC:src/com/technoetic/xplanner/actions/PutTheClockForwardAction.java PutTheClockForwardAction#execute; SRC:src/com/technoetic/xplanner/actions/EditPropertiesAction.java EditPropertiesAction#execute. WAR: classes byte-identical to the v1.1a4 release. The command runs, the clock moves by a positive dayOffset (any other value resets it), the property is set when a name and a value are given, and each action redirects to returnto or to the projects list. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks A-C-071, E-C-020, E-C-021, E-C-022, E-C-023, E-C-024, F-C-003, F-C-005, F-C-006; open residual scope R-29 (e), candidate outside the core (owner decision at Stage 4)).</t>
   </si>
   <si>
     <t>Tiles definitions can be reloaded via /do/admin/reload-tiles.</t>
@@ -847,7 +847,7 @@
     <t>Struts tiles reload response.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:407; WAR:WEB-INF/action-servlet.xml:398 (org.apache.struts.tiles.actions.ReloadDefinitionsAction). Source reconciliation (BA-001-11, A4): still unsupported. none: framework class, no source in the SVN tree (GAP-011). WAR: library class org.apache.struts.tiles.actions.ReloadDefinitionsAction in struts-1.2.9.jar (no source). The behavior lies in a bundled library whose source is not available. Live question: What does /do/admin/reload-tiles return, and does it reload the shared Tiles factory?</t>
+    <t>WAR:WEB-INF/struts-config.xml:407; WAR:WEB-INF/action-servlet.xml:398 (org.apache.struts.tiles.actions.ReloadDefinitionsAction). Source reconciliation (BA-001-11, A4): still unsupported. none: framework class, no source in the SVN tree (GAP-011). WAR: library class org.apache.struts.tiles.actions.ReloadDefinitionsAction in struts-1.2.9.jar (no source). The behavior lies in a bundled library whose source is not available. Live question: What does /do/admin/reload-tiles return, and does it reload the shared Tiles factory? Stage 3 W001 live answer (BA-001-13, MC-C-10): HTTP 200, text/plain, body "OK". Whether the shared factory is reloaded is not observable over HTTP (A-C-072). Candidate outside the core (owner decision at Stage 4), residual R-43. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks A-C-072; open residual scope R-43 (e), candidate outside the core (owner decision at Stage 4)).</t>
   </si>
   <si>
     <t>Startup schema creation and seed data</t>
@@ -862,7 +862,7 @@
     <t>Empty database gets tables and one system administrator person on project 0. Its factory default login pair is the one the login page advertises (row 9); the value is not reproduced here (CHK-009).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/spring-beans.xml:71-81 (SpringLiquibase changeLog classpath:db-changelog.xml, contexts test, production; sessionFactory depends-on liquibase); WAR:WEB-INF/classes/db-changelog.xml changeSets 1-1..2-5. Loading (BA-001-05): the liquibase bean is instantiated by both Spring contexts (row 65), so the change log is expected to run twice at startup; the second run is expected to find every change set already applied (Inferred). Source: stage-02-pass-003 F-002. Seed account (BA-001-06): WAR:WEB-INF/classes/db-changelog.xml:403-404 (userId and password digest of the seeded person). The earlier wording "credentials documented only in legacy/README.md, not evidence" was wrong: the WAR itself states the pair on the login page (row 9). Corrected in BA-001-06 (Source: stage-02-pass-004 F-001). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR spring-beans.xml (WAR governs); the WAR db-changelog.xml differs from the SVN copy, which is withheld (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-01: database engine, dialect, driver, URL and credential values come from the rewritten entries xplanner.properties / xplanner-custom.properties that carry the known MySQL patch; the upstream values cannot be separated. P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>WAR:WEB-INF/classes/spring-beans.xml:71-81 (SpringLiquibase changeLog classpath:db-changelog.xml, contexts test, production; sessionFactory depends-on liquibase); WAR:WEB-INF/classes/db-changelog.xml changeSets 1-1..2-5. Loading (BA-001-05): the liquibase bean is instantiated by both Spring contexts (row 65), so the change log is expected to run twice at startup; the second run is expected to find every change set already applied (Inferred). Source: stage-02-pass-003 F-002. Seed account (BA-001-06): WAR:WEB-INF/classes/db-changelog.xml:403-404 (userId and password digest of the seeded person). The earlier wording "credentials documented only in legacy/README.md, not evidence" was wrong: the WAR itself states the pair on the login page (row 9). Corrected in BA-001-06 (Source: stage-02-pass-004 F-001). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR spring-beans.xml (WAR governs); the WAR db-changelog.xml differs from the SVN copy, which is withheld (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-01: database engine, dialect, driver, URL and credential values come from the rewritten entries xplanner.properties / xplanner-custom.properties that carry the known MySQL patch; the upstream values cannot be separated. P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks A-C-073; open residual scope R-38 (e)).</t>
   </si>
   <si>
     <t>spring-beans.xml (with its imports spring-caching.xml, spring-dao.xml and spring-security.xml) is loaded by two Spring contexts: the root context of the ContextLoaderListener and the Struts ContextLoaderPlugIn context, which also loads action-servlet.xml and test-action-servlet.xml. Every singleton is expected to exist twice: Liquibase runs a second time at startup, a second scheduler registers the daily reminder job again, and a second connection pool and session factory are created; the Struts action beans are wired from the plug-in context.</t>
@@ -874,7 +874,7 @@
     <t>Two initialisations of every spring-beans.xml bean at startup; the reminder job expected to run twice at 00:05 (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:32-38 (contextConfigLocation classpath:spring-beans.xml) and :194-196 (org.springframework.web.context.ContextLoaderListener); WAR:WEB-INF/struts-config.xml:438-441 (org.springframework.web.struts.ContextLoaderPlugIn, contextConfigLocation /WEB-INF/action-servlet.xml,/WEB-INF/classes/spring-beans.xml,/WEB-INF/test-action-servlet.xml), started with the Struts servlet (WAR:WEB-INF/web.xml:227-249, load-on-startup 2 at :248); WAR:WEB-INF/classes/spring-beans.xml:60 (dataSource), :71-81 (liquibase, sessionFactory), :362-367 (task:scheduler, task:scheduled missingTimeEntryNotifier); WAR:WEB-INF/classes/spring-security.xml:49-50 (authorizerInitializer, init-method, lazy-init false). Loader sweep (.migration-tmp/stage-01/out/loaders-05.txt): a third loader, class com.technoetic.xplanner.util.MainBeanFactory#createDefaultFactory ("/spring-beans.xml", XmlBeanFactory), has no caller (out/orphans.txt). The effect of a child context redefining parent beans is framework behavior (GAP-011). Provenance: spring-beans.xml is a rewritten entry (GAP-005 P-05); struts-config.xml and web.xml show no rewrite sign (P-06). Source: stage-02-pass-003 F-002. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/util/MainBeanFactory.java MainBeanFactory#createDefaultFactory (three classes import MainBeanFactory but none uses it; no other class references it in the bytecode). WAR: classes byte-identical to the v1.1a4 release; patched spring-beans.xml (WAR governs; the SVN copy is withheld). The double loading is a Spring and container effect; the source only confirms that the third loader has no caller. Live question: At startup, do the log and the database show two Liquibase runs, two schedulers and a doubled reminder job?</t>
+    <t>WAR:WEB-INF/web.xml:32-38 (contextConfigLocation classpath:spring-beans.xml) and :194-196 (org.springframework.web.context.ContextLoaderListener); WAR:WEB-INF/struts-config.xml:438-441 (org.springframework.web.struts.ContextLoaderPlugIn, contextConfigLocation /WEB-INF/action-servlet.xml,/WEB-INF/classes/spring-beans.xml,/WEB-INF/test-action-servlet.xml), started with the Struts servlet (WAR:WEB-INF/web.xml:227-249, load-on-startup 2 at :248); WAR:WEB-INF/classes/spring-beans.xml:60 (dataSource), :71-81 (liquibase, sessionFactory), :362-367 (task:scheduler, task:scheduled missingTimeEntryNotifier); WAR:WEB-INF/classes/spring-security.xml:49-50 (authorizerInitializer, init-method, lazy-init false). Loader sweep (.migration-tmp/stage-01/out/loaders-05.txt): a third loader, class com.technoetic.xplanner.util.MainBeanFactory#createDefaultFactory ("/spring-beans.xml", XmlBeanFactory), has no caller (out/orphans.txt). The effect of a child context redefining parent beans is framework behavior (GAP-011). Provenance: spring-beans.xml is a rewritten entry (GAP-005 P-05); struts-config.xml and web.xml show no rewrite sign (P-06). Source: stage-02-pass-003 F-002. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/util/MainBeanFactory.java MainBeanFactory#createDefaultFactory (three classes import MainBeanFactory but none uses it; no other class references it in the bytecode). WAR: classes byte-identical to the v1.1a4 release; patched spring-beans.xml (WAR governs; the SVN copy is withheld). The double loading is a Spring and container effect; the source only confirms that the third loader has no caller. Live question: At startup, do the log and the database show two Liquibase runs, two schedulers and a doubled reminder job? Stage 3 W001 live answer (BA-001-13, MC-C-11): Two Liquibase runs (the second applies nothing) and two "scheduler" executors are in the startup log. At 00:05 the job made two send attempts per recipient, consistent with a doubled job; the two contexts cannot be told apart in the log, so the double run is inferred (A-C-074, L-C-005). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-074, L-C-005).</t>
   </si>
   <si>
     <t>An in-process HSQLDB server is started only when xplanner.migration.databasetype is hsqldb (the shipped value is mysql).</t>
@@ -886,7 +886,7 @@
     <t>No HSQLDB server with the shipped properties.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:190-192 (HsqldbServerContextListener); class com.technoetic.xplanner.filters.HsqldbServerContextListener (strings "xplanner.migration.databasetype", "hsqldb"); WAR:WEB-INF/classes/xplanner.properties:16 (databasetype=mysql). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/filters/HsqldbServerContextListener.java HsqldbServerContextListener#contextInitialized. WAR: classes byte-identical to the v1.1a4 release; databasetype from the patched WAR xplanner.properties (WAR governs). The listener starts HsqlServer only when xplanner.migration.databasetype equals hsqldb (ignoring case) and otherwise only logs; the WAR value is mysql. Provenance (fixed baseline, see reconnaissance GAP-005): P-01: database engine, dialect, driver, URL and credential values come from the rewritten entries xplanner.properties / xplanner-custom.properties that carry the known MySQL patch; the upstream values cannot be separated.</t>
+    <t>WAR:WEB-INF/web.xml:190-192 (HsqldbServerContextListener); class com.technoetic.xplanner.filters.HsqldbServerContextListener (strings "xplanner.migration.databasetype", "hsqldb"); WAR:WEB-INF/classes/xplanner.properties:16 (databasetype=mysql). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/filters/HsqldbServerContextListener.java HsqldbServerContextListener#contextInitialized. WAR: classes byte-identical to the v1.1a4 release; databasetype from the patched WAR xplanner.properties (WAR governs). The listener starts HsqlServer only when xplanner.migration.databasetype equals hsqldb (ignoring case) and otherwise only logs; the WAR value is mysql. Provenance (fixed baseline, see reconnaissance GAP-005): P-01: database engine, dialect, driver, URL and credential values come from the rewritten entries xplanner.properties / xplanner-custom.properties that carry the known MySQL patch; the upstream values cannot be separated. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks A-C-075; open residual scope R-44 (e)).</t>
   </si>
   <si>
     <t>Configuration layering and request encoding</t>
@@ -901,7 +901,7 @@
     <t>Effective values such as the MySQL connection, application URL http://localhost:8080/xplanner and login instructions URL come from xplanner-custom.properties.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.XPlannerProperties$PropertyInitializer (strings "xplanner.properties", "xplanner.overrides", "xplanner-custom.properties", "error during custom property loading"); WAR:WEB-INF/classes/xplanner-custom.properties:19-30,49; WAR:WEB-INF/classes/spring-beans.xml:18-32 (properties bean feeds PropertyPlaceholderConfigurer). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/XPlannerProperties.java XPlannerProperties$PropertyInitializer#loadProperties, #setCustomPropertyOverrides. WAR: classes byte-identical to the v1.1a4 release; both property files are patched WAR entries (WAR governs). Xplanner.properties is loaded from the class path, then every key of the file named by the xplanner.overrides system property (default xplanner-custom.properties) replaces it; no other file name is loaded. Provenance (fixed baseline, see reconnaissance GAP-005): P-01: database engine, dialect, driver, URL and credential values come from the rewritten entries xplanner.properties / xplanner-custom.properties that carry the known MySQL patch; the upstream values cannot be separated. P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-04: the cited value is read from xplanner-custom.properties (rewritten entry, known patch target); upstream value not determinable. P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>class com.technoetic.xplanner.XPlannerProperties$PropertyInitializer (strings "xplanner.properties", "xplanner.overrides", "xplanner-custom.properties", "error during custom property loading"); WAR:WEB-INF/classes/xplanner-custom.properties:19-30,49; WAR:WEB-INF/classes/spring-beans.xml:18-32 (properties bean feeds PropertyPlaceholderConfigurer). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/XPlannerProperties.java XPlannerProperties$PropertyInitializer#loadProperties, #setCustomPropertyOverrides. WAR: classes byte-identical to the v1.1a4 release; both property files are patched WAR entries (WAR governs). Xplanner.properties is loaded from the class path, then every key of the file named by the xplanner.overrides system property (default xplanner-custom.properties) replaces it; no other file name is loaded. Provenance (fixed baseline, see reconnaissance GAP-005): P-01: database engine, dialect, driver, URL and credential values come from the rewritten entries xplanner.properties / xplanner-custom.properties that carry the known MySQL patch; the upstream values cannot be separated. P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-04: the cited value is read from xplanner-custom.properties (rewritten entry, known patch target); upstream value not determinable. P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks A-C-076; open residual scope R-45 (e)).</t>
   </si>
   <si>
     <t>The hibernate.* settings of the property files other than the four connection values (dialect, show_sql, second-level and query cache, query substitutions) and the hibernate.dbcp.* pool settings are not passed to the web application's session factory or connection pool, so they are expected to have no effect there: the dialect is resolved by Hibernate itself, no second-level or query cache is configured, and the pool uses its defaults.</t>
@@ -913,43 +913,43 @@
     <t>Pool connects with the configured driver, URL and account; Hibernate settings from the property files do not appear in the web session factory (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/spring-beans.xml:60-69 (dataSource receives only ${hibernate.connection.driver_class}, url, username and password plus defaultAutoCommit) and :77-81 (sessionFactory AnnotationSessionFactoryBean with dataSource, packagesToScan and mappingLocations only; no hibernateProperties); no hibernate.properties or hibernate.cfg.xml in the WAR or at any JAR root (search; positive control ehcache-failsafe.xml in ehcache-1.2.3.jar). Consumers by name (.migration-tmp/stage-01/out/config-consumers-06.txt): hibernate.dialect only SystemInfo#getDatabaseInfo (display) and class com.technoetic.xplanner.db.hibernate.HibernateHelper#initializeConfiguration (Configuration.addProperties, a separate factory built only by #initializeHibernate, whose only outside caller is TomcatUserImporter#main); hibernate.show_sql only HsqlServer#isTraceOn; hibernate.query.substitutions only UseBeansTag#initializeQueryTranslations (the tag applies it to its own queries); hibernate.cache.* and hibernate.dbcp.* have no consumer. Keys: WAR:WEB-INF/classes/xplanner.properties:10,57-58,202-203,207-218; WAR:WEB-INF/classes/xplanner-custom.properties:15,19. Which dialect Hibernate picks and pool defaults are framework behavior (GAP-011). Provenance: all three files are rewritten entries (GAP-005 P-01, P-03, P-05). Source: stage-02-pass-004 F-003. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/db/hibernate/HibernateHelper.java HibernateHelper#initializeConfiguration. WAR: classes byte-identical to the v1.1a4 release; patched spring-beans.xml (WAR governs; the SVN copy is withheld). The source confirms that the property-file settings reach only the separate HibernateHelper configuration; which defaults the web session factory and pool then use is framework behavior. Live question: Does the running web application show no second-level or query cache and the default pool limits?</t>
-  </si>
-  <si>
-    <t>In the default, alternate (--), Danish, German, Japanese and Russian bundles, format.date is yyyy-MM-dd and format.datetime is yyyy-MM-dd HH:mm; they apply to the consumers that take the pattern from the session locale (the formatKey date displays, the calendar buttons and the saving of time entries). Exceptions: the history view (row 186), and the editor form converters, which validate and show dates with the patterns of the server default locale for every user (row 89).</t>
+    <t>WAR:WEB-INF/classes/spring-beans.xml:60-69 (dataSource receives only ${hibernate.connection.driver_class}, url, username and password plus defaultAutoCommit) and :77-81 (sessionFactory AnnotationSessionFactoryBean with dataSource, packagesToScan and mappingLocations only; no hibernateProperties); no hibernate.properties or hibernate.cfg.xml in the WAR or at any JAR root (search; positive control ehcache-failsafe.xml in ehcache-1.2.3.jar). Consumers by name (.migration-tmp/stage-01/out/config-consumers-06.txt): hibernate.dialect only SystemInfo#getDatabaseInfo (display) and class com.technoetic.xplanner.db.hibernate.HibernateHelper#initializeConfiguration (Configuration.addProperties, a separate factory built only by #initializeHibernate, whose only outside caller is TomcatUserImporter#main); hibernate.show_sql only HsqlServer#isTraceOn; hibernate.query.substitutions only UseBeansTag#initializeQueryTranslations (the tag applies it to its own queries); hibernate.cache.* and hibernate.dbcp.* have no consumer. Keys: WAR:WEB-INF/classes/xplanner.properties:10,57-58,202-203,207-218; WAR:WEB-INF/classes/xplanner-custom.properties:15,19. Which dialect Hibernate picks and pool defaults are framework behavior (GAP-011). Provenance: all three files are rewritten entries (GAP-005 P-01, P-03, P-05). Source: stage-02-pass-004 F-003. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/db/hibernate/HibernateHelper.java HibernateHelper#initializeConfiguration. WAR: classes byte-identical to the v1.1a4 release; patched spring-beans.xml (WAR governs; the SVN copy is withheld). The source confirms that the property-file settings reach only the separate HibernateHelper configuration; which defaults the web session factory and pool then use is framework behavior. Live question: Does the running web application show no second-level or query cache and the default pool limits? Stage 3 W001 live answer (BA-001-13, MC-C-12): "Query cache: disabled" although the property file enables it; "Second-level cache: enabled" does not decide. The cache provider and pool limits are not in the log extract (A-C-077). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks A-C-077; open residual scope R-45 (e)).</t>
+  </si>
+  <si>
+    <t>In the default, alternate (--), Danish, German, Japanese and Russian bundles, format.date is yyyy-MM-dd and format.datetime is yyyy-MM-dd HH:mm; they apply to the consumers that take the pattern from the session locale (the formatKey date displays, the time editor display, hint and Insert Time, and the saving of time entries). The iteration editor Calendar buttons pass format.date to a script function that the page does not load, so they insert no date (W001, row 71). Exceptions: the history view (row 186), and the editor form converters, which validate and show dates with the patterns of the server default locale for every user (row 89).</t>
   </si>
   <si>
     <t>Date formats follow the UI locale bundle.</t>
   </si>
   <si>
-    <t>Date displays with formatKey, the calendar buttons and saved time entries use yyyy-MM-dd in these session locales; editor validation and the iteration editor date fields use the server default locale's pattern (Inferred for the runtime effect).</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/classes/ResourceBundle.properties:8-9, ResourceBundle--.properties:5-6, ResourceBundle_da.properties:7-8, ResourceBundle_de.properties:8-9, ResourceBundle_ja.properties:12,14, ResourceBundle_ru.properties:9-10 (format.date, format.datetime); consumers editIteration.jsp, timesheet.jsp, editTimeEntries.jsp, UpdateTimeAction (format.date / format.datetime keys). Corrected in BA-001-03 (F-003): all 10 bundles compared. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag. WAR: the WAR bundles govern (the WAR copies of the da, es, fr, it and pt_br bundles differ from the SVN copies). The bundle patterns are confirmed for the format.date and format.datetime consumers, but not for every date display: the history view (history.jsp:61,106) uses xplanner:formatDate without a pattern, so FormatDateTag falls back to its built-in pattern "EEE MMM dd k:mm:ss z" (bytecode listing agrees). Resolves carried pass-009 F-002 statically; the observed format stays a live check. Live question: Which date format does the history view show after a fresh start for two sessions with different Accept-Language values? Correction (BA-001-12, pass-010 F-003): narrowed to the session-locale consumers. The editor form converters are static: SRC:src/com/technoetic/xplanner/forms/AbstractEditorForm.java AbstractEditorForm#initConverters, #getResources, #convertToDate, #convertToDateTime fills dateConverter and dateTimeConverter once from format.date and format.datetime of the server default locale's bundle (Struts MessageResources#getMessage(String) passes no locale, so the default locale taken from Locale.getDefault() when the resources were constructed applies (struts-1.2.9.jar listing), and XPlannerMessageResources#getMessage hands that locale to the Spring message source; SRC:src/net/sf/xplanner/struts/XPlannerMessageResources.java XPlannerMessageResources#getMessage), and decimalConverter with SRC:src/com/technoetic/xplanner/format/DecimalFormat.java DecimalFormat#DecimalFormat, whose parser uses the Accept-Language locale of the first request that calls initConverters (IterationEditorForm#validate, TimeEditorForm#validate or IdSearchAction#doExecute). SRC:src/com/technoetic/xplanner/forms/TaskEditorForm.java TaskEditorForm#validate keeps its own static date converter built the same way. Consumers: SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate, #toString, #reset (start and end dates are shown and parsed with the static converter; reset clears it and the next initConverters call rebuilds it from the same server-default pattern), SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#valideRow (dates, date-times and durations), TaskEditorForm#validate (created date). Session-locale consumers: SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#getDateFormat, #getDateTimeFormat (saving time entries), the calendar buttons (WAR:WEB-INF/jsp/edit/editIteration.jsp:52-57) and the formatKey displays of FormatDateTag. Bytecode listings agree. The runtime effect is Inferred.</t>
-  </si>
-  <si>
-    <t>In the Spanish, French, Italian and Brazilian Portuguese bundles, format.date is dd-MM-yyyy; the Spanish format.datetime is dd-MM-yyyy HH:MM, which uses the month letters in the minutes position. They apply to the session-locale consumers (row 69); the history view (row 186) and the editor form converters (row 89) are exceptions.</t>
+    <t>Date displays with formatKey, the time editor display and Insert Time, and saved time entries use yyyy-MM-dd in these session locales (observed in en and de; da, ja, ru and "--" not exercised); editor validation and the iteration editor date fields use the server default locale's pattern (Inferred for the runtime effect). The iteration editor Calendar buttons insert nothing: the click throws "showCalendar is not defined" and the image button submits the form; only the jQuery picker inserts dates (yyyy-MM-dd) (W001).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/classes/ResourceBundle.properties:8-9, ResourceBundle--.properties:5-6, ResourceBundle_da.properties:7-8, ResourceBundle_de.properties:8-9, ResourceBundle_ja.properties:12,14, ResourceBundle_ru.properties:9-10 (format.date, format.datetime); consumers editIteration.jsp, timesheet.jsp, editTimeEntries.jsp, UpdateTimeAction (format.date / format.datetime keys). Corrected in BA-001-03 (F-003): all 10 bundles compared. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag. WAR: the WAR bundles govern (the WAR copies of the da, es, fr, it and pt_br bundles differ from the SVN copies). The bundle patterns are confirmed for the format.date and format.datetime consumers, but not for every date display: the history view (history.jsp:61,106) uses xplanner:formatDate without a pattern, so FormatDateTag falls back to its built-in pattern "EEE MMM dd k:mm:ss z" (bytecode listing agrees). Resolves carried pass-009 F-002 statically; the observed format stays a live check. Live question: Which date format does the history view show after a fresh start for two sessions with different Accept-Language values? Correction (BA-001-12, pass-010 F-003): narrowed to the session-locale consumers. The editor form converters are static: SRC:src/com/technoetic/xplanner/forms/AbstractEditorForm.java AbstractEditorForm#initConverters, #getResources, #convertToDate, #convertToDateTime fills dateConverter and dateTimeConverter once from format.date and format.datetime of the server default locale's bundle (Struts MessageResources#getMessage(String) passes no locale, so the default locale taken from Locale.getDefault() when the resources were constructed applies (struts-1.2.9.jar listing), and XPlannerMessageResources#getMessage hands that locale to the Spring message source; SRC:src/net/sf/xplanner/struts/XPlannerMessageResources.java XPlannerMessageResources#getMessage), and decimalConverter with SRC:src/com/technoetic/xplanner/format/DecimalFormat.java DecimalFormat#DecimalFormat, whose parser uses the Accept-Language locale of the first request that calls initConverters (IterationEditorForm#validate, TimeEditorForm#validate or IdSearchAction#doExecute). SRC:src/com/technoetic/xplanner/forms/TaskEditorForm.java TaskEditorForm#validate keeps its own static date converter built the same way. Consumers: SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate, #toString, #reset (start and end dates are shown and parsed with the static converter; reset clears it and the next initConverters call rebuilds it from the same server-default pattern), SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#valideRow (dates, date-times and durations), TaskEditorForm#validate (created date). Session-locale consumers: SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#getDateFormat, #getDateTimeFormat (saving time entries), the calendar buttons (WAR:WEB-INF/jsp/edit/editIteration.jsp:52-57) and the formatKey displays of FormatDateTag. Bytecode listings agree. The runtime effect is Inferred. Stage 3 W001 (BA-001-13, MC-A-15, W001-F-17): the iteration editor loads jquery, jquery-ui, global.js and tooltip.js only; calendar.js is included only by the two timesheet pages. A Calendar click throws "ReferenceError: showCalendar is not defined" and submits the form, in en (E-C-028) and es (E-C-030). The en and de time editor hint "YYYY-MM-DD HH:MM" and Insert Time pattern "yyyy-MM-dd HH:mm" (C-C-003). Stage 3 W001 live answer (BA-001-13, MC-C-13): Both sessions (de first, then en) and later es sessions show "Mi Sep 30 19:45:16 UTC": the built-in pattern in the locale of the first requester (de). No fresh restart was done, so the first render since start-up is not proven (C-C-001). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks A-C-078, C-C-001, C-C-002, C-C-003, C-C-004, F-C-010; open residual scope R-26 (d), R-33 (e)).</t>
+  </si>
+  <si>
+    <t>In the Spanish, French, Italian and Brazilian Portuguese bundles, format.date is dd-MM-yyyy; the Spanish format.datetime is "dd-MM-yyyy HH:MM " (with a trailing space), which uses the month letters in the minutes position. They apply to the session-locale consumers (row 69): in an es session the time editor shows its hint and Insert Time output and saves entries with this pattern, so an entry typed as the hint reads passes validation and then fails at save with HTTP 500, and an entry shaped like the Insert Time output is saved with its minutes replaced (W001). The history view (row 186) and the editor form converters (row 89) are exceptions.</t>
   </si>
   <si>
     <t>Locale-dependent date entry and display; the Spanish pattern prints the month where minutes are expected.</t>
   </si>
   <si>
-    <t>dd-MM-yyyy dates on the session-locale consumers for these locales; Spanish date-times show the month number in place of minutes (runtime unverified).</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/classes/ResourceBundle_es.properties:7-8, ResourceBundle_fr.properties:5-6, ResourceBundle_it.properties:11-12, ResourceBundle_pt_br.properties:8-9. Source: stage-02-pass-001 F-003. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag. WAR: the WAR bundles govern (the WAR copies of the es, fr, it and pt_br bundles differ from the SVN copies). As row 69: the history view does not use these patterns. Resolves carried pass-009 F-002 statically. Correction (BA-001-12, pass-010 F-003): narrowed as row 69: the editor form converters use the server default locale's patterns, not these bundles, unless that is the server default locale.</t>
-  </si>
-  <si>
-    <t>The jQuery date picker attached to date fields always inserts yyyy-MM-dd, and the iteration editor calendar button inserts the session bundle's format.date, while the iteration editor parses both with the static converter built from the server default locale's format.date. Whether a picked date is accepted therefore depends on the server default locale, not the session locale; the converter is lenient, so a date in the other order is read as a different date rather than rejected (Inferred).</t>
+    <t>dd-MM-yyyy dates on the session-locale consumers for these locales; Spanish date-times show the month number in place of minutes. es time editor (W001): hint "DD-MM-YYYY HH:MM"; Insert Time produced "30-09-2026 23:09 " at 23:14 (month in the minutes place, trailing space); an entry typed as "30-09-2026 12:00" passed validation and failed with HTTP 500 (ParseException at UpdateTimeAction.java:145), nothing saved; an entry "30-09-2026 12:09 " was saved as 12:00 (minutes lost). fr, it and pt_br were not exercised.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/classes/ResourceBundle_es.properties:7-8, ResourceBundle_fr.properties:5-6, ResourceBundle_it.properties:11-12, ResourceBundle_pt_br.properties:8-9. Source: stage-02-pass-001 F-003. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag. WAR: the WAR bundles govern (the WAR copies of the es, fr, it and pt_br bundles differ from the SVN copies). As row 69: the history view does not use these patterns. Resolves carried pass-009 F-002 statically. Correction (BA-001-12, pass-010 F-003): narrowed as row 69: the editor form converters use the server default locale's patterns, not these bundles, unless that is the server default locale. Stage 3 W001 (BA-001-13, MC-A-16, W001-F-18): C-C-003 (en, de and es sessions; the Insert Time output was computed offline from the served script) and E-C-033 (es, real browser). en and de round trips are unchanged. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks A-C-079, F-C-011; open residual scope R-26 (d)).</t>
+  </si>
+  <si>
+    <t>The jQuery date picker attached to date fields always inserts yyyy-MM-dd. The iteration editor Calendar buttons call showCalendar(id, format.date), a function that the page never defines (calendar.js is included only by the two timesheet pages), so a click throws a ReferenceError, inserts nothing and submits the form (W001). The iteration editor parses dates with the static converter built from the server default locale's format.date; the converter is lenient, so a typed date in the other order is read as a different date rather than rejected.</t>
   </si>
   <si>
     <t>Conflict between two date pickers for non-ISO locales.</t>
   </si>
   <si>
-    <t>On a server whose default locale bundle uses yyyy-MM-dd, a date from the jQuery picker parses in every session, and a dd-MM-yyyy date from the calendar button of an es, fr, it or pt_br session is read with the server pattern as a different date; on a server with a dd-MM-yyyy default the reverse applies (runtime unverified).</t>
-  </si>
-  <si>
-    <t>WAR:js/global.js:39 (.dateField datepicker dateFormat yy-mm-dd); WAR:WEB-INF/jsp/edit/editIteration.jsp:54,57 (class dateField plus showCalendar with format.date); class IterationEditorForm#validate (iteration.editor.bad_start_date). Source: stage-02-pass-001 F-003. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release; js/global.js and editIteration.jsp identical to the SVN webapp copies. The picker format and the locale pattern are as recorded; whether a picked date is rejected is browser and locale behavior. Live question: In an es, fr, it or pt_br session, is a date picked with the jQuery picker rejected as "Start date is invalid."? Correction (BA-001-12, pass-010 F-003): the BA-001-11 note ("the locale pattern [is] as recorded") and its live question are superseded. The editor form converters are static: SRC:src/com/technoetic/xplanner/forms/AbstractEditorForm.java AbstractEditorForm#initConverters, #getResources, #convertToDate, #convertToDateTime fills dateConverter and dateTimeConverter once from format.date and format.datetime of the server default locale's bundle (Struts MessageResources#getMessage(String) passes no locale, so the default locale taken from Locale.getDefault() when the resources were constructed applies (struts-1.2.9.jar listing), and XPlannerMessageResources#getMessage hands that locale to the Spring message source; SRC:src/net/sf/xplanner/struts/XPlannerMessageResources.java XPlannerMessageResources#getMessage), and decimalConverter with SRC:src/com/technoetic/xplanner/format/DecimalFormat.java DecimalFormat#DecimalFormat, whose parser uses the Accept-Language locale of the first request that calls initConverters (IterationEditorForm#validate, TimeEditorForm#validate or IdSearchAction#doExecute). SRC:src/com/technoetic/xplanner/forms/TaskEditorForm.java TaskEditorForm#validate keeps its own static date converter built the same way. Consumers: SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate, #toString, #reset (start and end dates are shown and parsed with the static converter; reset clears it and the next initConverters call rebuilds it from the same server-default pattern), SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#valideRow (dates, date-times and durations), TaskEditorForm#validate (created date). Session-locale consumers: SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#getDateFormat, #getDateTimeFormat (saving time entries), the calendar buttons (WAR:WEB-INF/jsp/edit/editIteration.jsp:52-57) and the formatKey displays of FormatDateTag. Bytecode listings agree. The runtime effect is Inferred. New live question: on a server with a known default locale, which start date does the iteration editor store for a date from the jQuery picker and for one from the calendar button in an es session?</t>
+    <t>On this server (default bundle yyyy-MM-dd) a date picked with the jQuery picker is stored as picked in en and es sessions; the Calendar buttons insert nothing and submit the form ("Missing iteration name." when the name is empty); a typed dd-MM-yyyy date (02-11-2026) is stored as a different date (0008-05-18), not rejected (W001). fr, it and pt_br were not tested with the picker, and a server with a dd-MM-yyyy default was not observed.</t>
+  </si>
+  <si>
+    <t>WAR:js/global.js:39 (.dateField datepicker dateFormat yy-mm-dd); WAR:WEB-INF/jsp/edit/editIteration.jsp:54,57 (class dateField plus showCalendar with format.date); class IterationEditorForm#validate (iteration.editor.bad_start_date). Source: stage-02-pass-001 F-003. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release; js/global.js and editIteration.jsp identical to the SVN webapp copies. The picker format and the locale pattern are as recorded; whether a picked date is rejected is browser and locale behavior. Live question: In an es, fr, it or pt_br session, is a date picked with the jQuery picker rejected as "Start date is invalid."? Correction (BA-001-12, pass-010 F-003): the BA-001-11 note ("the locale pattern [is] as recorded") and its live question are superseded. The editor form converters are static: SRC:src/com/technoetic/xplanner/forms/AbstractEditorForm.java AbstractEditorForm#initConverters, #getResources, #convertToDate, #convertToDateTime fills dateConverter and dateTimeConverter once from format.date and format.datetime of the server default locale's bundle (Struts MessageResources#getMessage(String) passes no locale, so the default locale taken from Locale.getDefault() when the resources were constructed applies (struts-1.2.9.jar listing), and XPlannerMessageResources#getMessage hands that locale to the Spring message source; SRC:src/net/sf/xplanner/struts/XPlannerMessageResources.java XPlannerMessageResources#getMessage), and decimalConverter with SRC:src/com/technoetic/xplanner/format/DecimalFormat.java DecimalFormat#DecimalFormat, whose parser uses the Accept-Language locale of the first request that calls initConverters (IterationEditorForm#validate, TimeEditorForm#validate or IdSearchAction#doExecute). SRC:src/com/technoetic/xplanner/forms/TaskEditorForm.java TaskEditorForm#validate keeps its own static date converter built the same way. Consumers: SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate, #toString, #reset (start and end dates are shown and parsed with the static converter; reset clears it and the next initConverters call rebuilds it from the same server-default pattern), SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#valideRow (dates, date-times and durations), TaskEditorForm#validate (created date). Session-locale consumers: SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#getDateFormat, #getDateTimeFormat (saving time entries), the calendar buttons (WAR:WEB-INF/jsp/edit/editIteration.jsp:52-57) and the formatKey displays of FormatDateTag. Bytecode listings agree. The runtime effect is Inferred. New live question: on a server with a known default locale, which start date does the iteration editor store for a date from the jQuery picker and for one from the calendar button in an es session? Stage 3 W001 (BA-001-13, MC-A-15, W001-F-17): E-C-028 (en) and E-C-030 (es: onclick showCalendar('startDate', 'dd-MM-yyyy'), ReferenceError, form submitted, no value inserted). The calendar-button half of the BA-001-12 expectation does not occur; the dd-MM-yyyy misreading applies to typed dates only (C-C-005). Part E named the cells by shifted columns (E, G, I); the W001 lead mapped them to D, F and H. Status stays Inferred (fr, it, pt_br and another server default not observed). Stage 3 W001 live answer (BA-001-13, MC-C-14): es: no. The picker inserts yyyy-MM-dd and the date is stored as picked. A typed dd-MM-yyyy date is read as a different date (02-11-2026 stored as 0008-05-18), not rejected. The Calendar button inserts nothing (E-F-01). fr, it and pt_br were not tested with the picker (C-C-005, E-C-029, E-C-030). The D/F correction is under W001-F-17. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks A-C-080, C-C-005, E-C-027, E-C-028, E-C-029, E-C-030, F-C-012; open residual scope R-26 (d)).</t>
   </si>
   <si>
     <t>Request parameters under /do/* are decoded as UTF-8.</t>
@@ -961,7 +961,7 @@
     <t>Non-ASCII input round-trips in forms.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:121-128,178-181 (RequestCharacterEncodingFilter, requestCharacterEncoding UTF-8, /do/*). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/filters/RequestCharacterEncodingFilter.java RequestCharacterEncodingFilter#doFilter. WAR: classes byte-identical to the v1.1a4 release. The filter sets the configured request encoding before the chain.</t>
+    <t>WAR:WEB-INF/web.xml:121-128,178-181 (RequestCharacterEncodingFilter, requestCharacterEncoding UTF-8, /do/*). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/filters/RequestCharacterEncodingFilter.java RequestCharacterEncodingFilter#doFilter. WAR: classes byte-identical to the v1.1a4 release. The filter sets the configured request encoding before the chain. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks A-C-081).</t>
   </si>
   <si>
     <t>Activity logging</t>
@@ -976,7 +976,7 @@
     <t>Log lines START/END with duration in xplanner-plus-activity.log, which is written into the web application root, a publicly served location with no security filter; the container is expected to serve it to anyone (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:54-57,130-133 (ActivityLogFilter on /do/*); WAR:WEB-INF/classes/log4j-war.xml:44-55 (ACTIVITY_FILE ${xplanner-plus.root}/xplanner-plus-activity.log); class com.technoetic.xplanner.filters.ActivityLogFilter#doFilter. Public location (BA-001-06): the ACTIVITY_FILE appender writes ${xplanner-plus.root}/xplanner-plus-activity.log (WAR:WEB-INF/classes/log4j-war.xml:44-58, used by the ActivityLogFilter category at :54-58); webAppRootKey sets xplanner-plus.root to the web application root (WAR:WEB-INF/web.xml:45-52). class ActivityLogFilterHelper reads getUserId, getRemoteAddr, getRequestURI and getQueryString. No security filter covers the web root (web.xml:155-176). Static serving of web-root files is container behavior (GAP-011). A 2011 copy of this file also ships in the WAR (GAP-013). Observed risk only (Q3 deferred). Source: stage-02-pass-004 F-005. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/filters/ActivityLogFilter.java ActivityLogFilter#doFilter. WAR: classes byte-identical to the v1.1a4 release. A start and an end record are logged around every filtered request.</t>
+    <t>WAR:WEB-INF/web.xml:54-57,130-133 (ActivityLogFilter on /do/*); WAR:WEB-INF/classes/log4j-war.xml:44-55 (ACTIVITY_FILE ${xplanner-plus.root}/xplanner-plus-activity.log); class com.technoetic.xplanner.filters.ActivityLogFilter#doFilter. Public location (BA-001-06): the ACTIVITY_FILE appender writes ${xplanner-plus.root}/xplanner-plus-activity.log (WAR:WEB-INF/classes/log4j-war.xml:44-58, used by the ActivityLogFilter category at :54-58); webAppRootKey sets xplanner-plus.root to the web application root (WAR:WEB-INF/web.xml:45-52). class ActivityLogFilterHelper reads getUserId, getRemoteAddr, getRequestURI and getQueryString. No security filter covers the web root (web.xml:155-176). Static serving of web-root files is container behavior (GAP-011). A 2011 copy of this file also ships in the WAR (GAP-013). Observed risk only (Q3 deferred). Source: stage-02-pass-004 F-005. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/filters/ActivityLogFilter.java ActivityLogFilter#doFilter. WAR: classes byte-identical to the v1.1a4 release. A start and an end record are logged around every filtered request. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks A-C-082; open residual scope R-44 (e)).</t>
   </si>
   <si>
     <t>UF-005</t>
@@ -997,7 +997,7 @@
     <t>Table of projects with links to project and current iteration; "people" and "aggregate timesheet" links.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:179; WAR:WEB-INF/action-servlet.xml:29-31 (DispatchForward, authorizationRequired=false); WAR:WEB-INF/jsp/view/projects.jsp:32-167 (useBeans order "is_hidden,name asc"; iterations where "? between startDate and endDate"). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/struts-config.xml:179; WAR:WEB-INF/action-servlet.xml:29-31 (DispatchForward, authorizationRequired=false); WAR:WEB-INF/jsp/view/projects.jsp:32-167 (useBeans order "is_hidden,name asc"; iterations where "? between startDate and endDate"). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-034, B-C-001, B-C-002).</t>
   </si>
   <si>
     <t>Users who may hide projects see an extra "hidden" column with yes/no; hidden projects are sorted after visible ones but are not styled differently.</t>
@@ -1009,7 +1009,7 @@
     <t>Hidden column visible only with hide permission; hidden projects listed last.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/projects.jsp:137-142 (isUserAuthorizedForAny permissions="hide") and :33 (order "is_hidden,name asc"). The class HiddenRowDecorator declared at :65-75 is never passed to the table: the writableTable at :82-84 has no rowDecorator attribute, and the name occurs only at :66 (CHK-003). Corrected in BA-001-04 (Source: stage-02-pass-002 F-006). Server-side enforcement (CHK-002, BA-001-04): the column is display-level only; hiding a project goes through EditProjectAction, which performs no server-side permission check (rows 29-30). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/jsp/view/projects.jsp:137-142 (isUserAuthorizedForAny permissions="hide") and :33 (order "is_hidden,name asc"). The class HiddenRowDecorator declared at :65-75 is never passed to the table: the writableTable at :82-84 has no rowDecorator attribute, and the name occurs only at :66 (CHK-003). Corrected in BA-001-04 (Source: stage-02-pass-002 F-006). Server-side enforcement (CHK-002, BA-001-04): the column is display-level only; hiding a project goes through EditProjectAction, which performs no server-side permission check (rows 29-30). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks setup-C-019, B-C-003, E-C-012, E-C-013, E-C-014, E-C-015, F-C-002; open residual scope R-24 (d)).</t>
   </si>
   <si>
     <t>When no readable project exists the page shows a "no projects" message.</t>
@@ -1021,7 +1021,7 @@
     <t>Message projects.none.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/projects.jsp:147-150. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/jsp/view/projects.jsp:147-150. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-001).</t>
   </si>
   <si>
     <t>Create project</t>
@@ -1036,7 +1036,7 @@
     <t>Project saved; user returned to the projects list.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/projects.jsp:153-158 (link /do/edit/project under create.project); WAR:WEB-INF/struts-config.xml:195; WAR:WEB-INF/action-servlet.xml:72-76 (EditProjectAction); WAR:WEB-INF/jsp/edit/editProject.jsp:42-112. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditProjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editProject.jsp writes the raw request parameters oid (48), returnto (52) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/project that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Project object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). EditProjectAction#saveForm calls the same #populateObject. No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute (reached from EditProjectAction#doExecute) redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/actions/EditProjectAction.java EditProjectAction#saveForm, #doExecute; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject, #doExecute. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
+    <t>WAR:WEB-INF/jsp/view/projects.jsp:153-158 (link /do/edit/project under create.project); WAR:WEB-INF/struts-config.xml:195; WAR:WEB-INF/action-servlet.xml:72-76 (EditProjectAction); WAR:WEB-INF/jsp/edit/editProject.jsp:42-112. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditProjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editProject.jsp writes the raw request parameters oid (48), returnto (52) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/project that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Project object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). EditProjectAction#saveForm calls the same #populateObject. No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute (reached from EditProjectAction#doExecute) redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/actions/EditProjectAction.java EditProjectAction#saveForm, #doExecute; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject, #doExecute. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-005, setup-C-060, B-C-004, B-C-005, B-C-006).</t>
   </si>
   <si>
     <t>A project without a name is rejected.</t>
@@ -1048,7 +1048,7 @@
     <t>Editor redisplayed with "Missing project name."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.ProjectEditorForm#validate (string project.editor.missing_name). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/ProjectEditorForm.java ProjectEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release. The name is required on submit, except for the add and delete receiver actions.</t>
+    <t>class com.technoetic.xplanner.forms.ProjectEditorForm#validate (string project.editor.missing_name). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/ProjectEditorForm.java ProjectEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release. The name is required on submit, except for the add and delete receiver actions. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-007).</t>
   </si>
   <si>
     <t>Project options (wiki URL, send missing-time notification, escape brackets) are stored as per-project attributes when they differ from the global defaults in the property files (or the project already has the attribute); a value equal to the default is not stored.</t>
@@ -1060,7 +1060,7 @@
     <t>Options persist and are re-shown when editing.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.actions.EditProjectAction#saveForm/#saveOrUpdateAttribute (strings "twiki.scheme.wiki", "xplanner.project.send.notification", "xplanner.escape.brackets"); db-changelog.xml table attribute. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/EditProjectAction.java EditProjectAction#saveForm, #saveOrUpdateAttribute. WAR: classes byte-identical to the v1.1a4 release. An option is written as a project attribute only when the project already has that attribute, or when the new value is not empty and differs from the global default in the property files (or there is no default); a value equal to the default is not stored and the default keeps applying. The branches match the bytecode listing.</t>
+    <t>class com.technoetic.xplanner.actions.EditProjectAction#saveForm/#saveOrUpdateAttribute (strings "twiki.scheme.wiki", "xplanner.project.send.notification", "xplanner.escape.brackets"); db-changelog.xml table attribute. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/EditProjectAction.java EditProjectAction#saveForm, #saveOrUpdateAttribute. WAR: classes byte-identical to the v1.1a4 release. An option is written as a project attribute only when the project already has that attribute, or when the new value is not empty and differs from the global default in the property files (or there is no default); a value equal to the default is not stored and the default keeps applying. The branches match the bytecode listing. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks B-C-008; open residual scope R-39 (e)).</t>
   </si>
   <si>
     <t>Edit project</t>
@@ -1075,7 +1075,7 @@
     <t>Editor titled "Edit project: &lt;name&gt;" with Update/Reset; changes saved.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:28-34,76-80,104-106; class DomainMetaDataRepository#init (project edit -&gt; /do/edit/project, permission admin.edit). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditProjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 78 applies to every /do/edit/project request, and also to /do/edit/roles, whose action type is Project (row 35) (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
+    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:28-34,76-80,104-106; class DomainMetaDataRepository#init (project edit -&gt; /do/edit/project, permission admin.edit). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditProjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 78 applies to every /do/edit/project request, and also to /do/edit/roles, whose action type is Project (row 35) (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-009, B-C-010).</t>
   </si>
   <si>
     <t>Delete project</t>
@@ -1090,31 +1090,31 @@
     <t>Browser confirm "Do you want to delete project '&lt;name&gt;'?"; the project and its iterations, stories, tasks and time entries removed; orphan notes remain (runtime unverified).</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (delete -&gt; /do/delete/project, permission sysadmin.delete, onclick action.delete.confirmation); WAR:WEB-INF/struts-config.xml:197; WAR:WEB-INF/action-servlet.xml:78-82 (DeleteObjectAction#doExecute: CommonDao.delete). Cascades (CHK-003): net.sf.xplanner.domain.Project#getIterations @OneToMany(cascade=ALL), #getBacklog @OneToOne(cascade=REMOVE), Iteration#getUserStories, UserStory#getTasks, Task#getTimeEntries @OneToMany(cascade=REMOVE); The notification-receiver links (Project#getNotificationReceivers @ManyToMany, join table notification_receivers) and the project attributes (@ElementCollection, table attribute) are removed with the project row. Note refers to objects by attachedToId without a mapping; NoteHelper#deleteNotesFor is called from HibernateObjectRepository#delete, which the web delete path (DeleteObjectAction#doExecute -&gt; CommonDao.delete) does not reach. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute; SRC:src/net/sf/xplanner/domain/Project.java Project#getIterations; SRC:src/net/sf/xplanner/domain/Iteration.java Iteration#getUserStories; SRC:src/net/sf/xplanner/domain/UserStory.java UserStory#getTasks; SRC:src/net/sf/xplanner/domain/Task.java Task#getTimeEntries. WAR: classes byte-identical to the v1.1a4 release. The cascade annotations of the source match the recorded ones (ALL on project iterations, REMOVE on stories, tasks and time entries).</t>
+    <t>class DomainMetaDataRepository#init (delete -&gt; /do/delete/project, permission sysadmin.delete, onclick action.delete.confirmation); WAR:WEB-INF/struts-config.xml:197; WAR:WEB-INF/action-servlet.xml:78-82 (DeleteObjectAction#doExecute: CommonDao.delete). Cascades (CHK-003): net.sf.xplanner.domain.Project#getIterations @OneToMany(cascade=ALL), #getBacklog @OneToOne(cascade=REMOVE), Iteration#getUserStories, UserStory#getTasks, Task#getTimeEntries @OneToMany(cascade=REMOVE); The notification-receiver links (Project#getNotificationReceivers @ManyToMany, join table notification_receivers) and the project attributes (@ElementCollection, table attribute) are removed with the project row. Note refers to objects by attachedToId without a mapping; NoteHelper#deleteNotesFor is called from HibernateObjectRepository#delete, which the web delete path (DeleteObjectAction#doExecute -&gt; CommonDao.delete) does not reach. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute; SRC:src/net/sf/xplanner/domain/Project.java Project#getIterations; SRC:src/net/sf/xplanner/domain/Iteration.java Iteration#getUserStories; SRC:src/net/sf/xplanner/domain/UserStory.java UserStory#getTasks; SRC:src/net/sf/xplanner/domain/Task.java Task#getTimeEntries. WAR: classes byte-identical to the v1.1a4 release. The cascade annotations of the source match the recorded ones (ALL on project iterations, REMOVE on stories, tasks and time entries). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks B-C-011, B-C-012, E-C-019; open residual scope R-40 (e)).</t>
   </si>
   <si>
     <t>View project</t>
   </si>
   <si>
-    <t>The project page shows the description and a sortable, paged (10 per page) iteration table with ID, name, start/end dates, days worked and story count, newest first.</t>
+    <t>The project page shows the description and a sortable, paged (10 per page) iteration table with ID, name, start/end dates, days worked and story count. By default the table is sorted by its 5th rendered column, descending, within the current page only: End Date for users who see the Actions column, Days Worked for viewers (W001); with 11 iterations the newest was on page 2.</t>
   </si>
   <si>
     <t>Overview of a project's timeline.</t>
   </si>
   <si>
-    <t>Iteration table with edit/delete icons by permission; "create iteration", "people", export and history links.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/struts-config.xml:181-183; WAR:WEB-INF/action-servlet.xml:33-37; WAR:WEB-INF/jsp/view/project.jsp:41-70 (writableTable pagesize 10, defaultsort 5 descending) and :87-105 (links /do/edit/iteration, /do/view/people, exportLinks.jsp, /do/view/history). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>Iteration table, 10 per page, sorted by default by the 5th rendered column descending within the page (End Date with the Actions column, Days Worked for viewers); edit/delete icons by permission; "create iteration", "people", export and history links.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/struts-config.xml:181-183; WAR:WEB-INF/action-servlet.xml:33-37; WAR:WEB-INF/jsp/view/project.jsp:41-70 (writableTable pagesize 10, defaultsort 5 descending) and :87-105 (links /do/edit/iteration, /do/view/people, exportLinks.jsp, /do/view/history). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Stage 3 W001 (BA-001-13, MC-A-17, W001-F-19): B-C-013 (row order per role), B-C-014 (11 iterations: page 1 P10..P01, page 2 P11), B-C-015 (sort links and default order for viewer and editor). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-036, B-C-013, B-C-014, B-C-015).</t>
   </si>
   <si>
     <t>A project without iterations shows a "no iterations" message.</t>
   </si>
   <si>
-    <t>Message iterations.none.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/project.jsp:73-75 (logic:equal name="iterationCount" value="0"); no iterationCount bean is defined on the page, so the message display is unverified. Source reconciliation (BA-001-11, A4): runtime-only. none: no Java class or other JSP of the source tree sets iterationCount. WAR: project.jsp identical to the SVN webapp copy. The source confirms that nothing defines the bean the page compares; what Struts logic:equal then does is framework behavior. Live question: What does the project page show for a project without iterations?</t>
+    <t>Message iterations.none is not shown: live, a project without iterations shows the heading, the description and the links (People, Export, History; Create Iteration and Edit by role) and no "No iterations for this project." message, for all four roles (W001).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/project.jsp:73-75 (logic:equal name="iterationCount" value="0"); no iterationCount bean is defined on the page, so the message display is unverified. Source reconciliation (BA-001-11, A4): runtime-only. none: no Java class or other JSP of the source tree sets iterationCount. WAR: project.jsp identical to the SVN webapp copy. The source confirms that nothing defines the bean the page compares; what Struts logic:equal then does is framework behavior. Live question: What does the project page show for a project without iterations? Stage 3 W001 (BA-001-13, MC-A-18, W001-F-20): setup-C-037 (S3 Shared before any iteration) and B-C-016 (S3-B Planning, all four roles: message absent, no iteration table). The status stays Partial: deciding No would need the iterationCount condition of project.jsp re-read from source, which BA-001-13 does not do (no new research). Stage 3 W001 live answer (BA-001-13, MC-C-15): The heading, the description and the links (People, Export, History; Create Iteration and Edit by role); no "No iterations" message (setup-C-037, B-C-016). The D/F correction is under W001-F-20. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-037, B-C-016).</t>
   </si>
   <si>
     <t>Missing time entry notification receivers</t>
@@ -1129,7 +1129,7 @@
     <t>Person selected and "Add" pressed; the person appears in the receivers list.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:115-158 (select personToAddId, action addTimeNotification); class EditProjectAction#doExecute (forward /do/edit/project/notification); WAR:WEB-INF/struts-config.xml:368-372; class com.technoetic.xplanner.actions.UpdateTimeNotificationReceivers#doAction; db-changelog.xml table notification_receivers. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); UpdateTimeNotificationReceivers performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/UpdateTimeNotificationReceivers.java UpdateTimeNotificationReceivers#doAction. WAR: classes byte-identical to the v1.1a4 release. The add action appends the selected person to the project's receivers.</t>
+    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:115-158 (select personToAddId, action addTimeNotification); class EditProjectAction#doExecute (forward /do/edit/project/notification); WAR:WEB-INF/struts-config.xml:368-372; class com.technoetic.xplanner.actions.UpdateTimeNotificationReceivers#doAction; db-changelog.xml table notification_receivers. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); UpdateTimeNotificationReceivers performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/UpdateTimeNotificationReceivers.java UpdateTimeNotificationReceivers#doAction. WAR: classes byte-identical to the v1.1a4 release. The add action appends the selected person to the project's receivers. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-017, B-C-018).</t>
   </si>
   <si>
     <t>A receiver can be removed with the delete icon.</t>
@@ -1141,7 +1141,7 @@
     <t>Person disappears from the receivers list.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:20-25,146 (deleteNotifiedPerson, action delTimeNotification); class UpdateTimeNotificationReceivers (string "delTimeNotification"). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/UpdateTimeNotificationReceivers.java UpdateTimeNotificationReceivers#doAction. WAR: classes byte-identical to the v1.1a4 release. The delete action removes the selected person from the receivers.</t>
+    <t>WAR:WEB-INF/jsp/edit/editProject.jsp:20-25,146 (deleteNotifiedPerson, action delTimeNotification); class UpdateTimeNotificationReceivers (string "delTimeNotification"). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/UpdateTimeNotificationReceivers.java UpdateTimeNotificationReceivers#doAction. WAR: classes byte-identical to the v1.1a4 release. The delete action removes the selected person from the receivers. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-019, B-C-020).</t>
   </si>
   <si>
     <t>UF-006</t>
@@ -1162,19 +1162,19 @@
     <t>Iteration saved under the project; user returned.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/project.jsp:87-90 (link /do/edit/iteration); WAR:WEB-INF/struts-config.xml:241-243; WAR:WEB-INF/action-servlet.xml:177-181 (EditIterationAction); WAR:WEB-INF/jsp/edit/editIteration.jsp; class EditIterationAction#beforeObjectCommit (strings "Create", Project). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editIteration.jsp writes the raw request parameters oid (31), returnto (34), fkey (36,37) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/iteration that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Iteration object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/EditIterationAction.java EditIterationAction#beforeObjectCommit. WAR: classes byte-identical to the v1.1a4 release. A created iteration gets its project, the inactive status and zero days worked.</t>
-  </si>
-  <si>
-    <t>Missing name, unparsable dates, or an end date that does not follow the start date are rejected.</t>
+    <t>WAR:WEB-INF/jsp/view/project.jsp:87-90 (link /do/edit/iteration); WAR:WEB-INF/struts-config.xml:241-243; WAR:WEB-INF/action-servlet.xml:177-181 (EditIterationAction); WAR:WEB-INF/jsp/edit/editIteration.jsp; class EditIterationAction#beforeObjectCommit (strings "Create", Project). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editIteration.jsp writes the raw request parameters oid (31), returnto (34), fkey (36,37) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/iteration that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Iteration object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/EditIterationAction.java EditIterationAction#beforeObjectCommit. WAR: classes byte-identical to the v1.1a4 release. A created iteration gets its project, the inactive status and zero days worked. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-038, B-C-021, B-C-022).</t>
+  </si>
+  <si>
+    <t>A missing name, or an end date that does not follow the start date, is rejected. Dates are parsed leniently: out-of-range month and day values roll over and trailing characters after a valid date prefix are ignored, so only input that does not start with a date is rejected as an invalid date (W001).</t>
   </si>
   <si>
     <t>Iterations need a name and a valid positive date interval.</t>
   </si>
   <si>
-    <t>Messages "Missing iteration name.", "Start date is invalid.", "End date is invalid.", "Iteration must be a positive time interval."</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.forms.IterationEditorForm#validate (strings iteration.editor.missing_name, bad_start_date, bad_end_date) and #requirePositiveInterval (iteration.editor.nonpositive_interval); WAR:WEB-INF/classes/ResourceBundle.properties:265. Corrected in BA-001-04 (Source: stage-02-pass-002 F-001). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; iteration.editor.nonpositive_interval: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release. Name and both dates are required and the interval must be positive. Correction (BA-001-12, pass-010 F-003): the accepted date and date-time patterns are those of the server default locale's bundle, not of the active (session) bundle as stated above: IterationEditorForm#validate parses with the static converters. The editor form converters are static: SRC:src/com/technoetic/xplanner/forms/AbstractEditorForm.java AbstractEditorForm#initConverters, #getResources, #convertToDate, #convertToDateTime fills dateConverter and dateTimeConverter once from format.date and format.datetime of the server default locale's bundle (Struts MessageResources#getMessage(String) passes no locale, so the default locale taken from Locale.getDefault() when the resources were constructed applies (struts-1.2.9.jar listing), and XPlannerMessageResources#getMessage hands that locale to the Spring message source; SRC:src/net/sf/xplanner/struts/XPlannerMessageResources.java XPlannerMessageResources#getMessage), and decimalConverter with SRC:src/com/technoetic/xplanner/format/DecimalFormat.java DecimalFormat#DecimalFormat, whose parser uses the Accept-Language locale of the first request that calls initConverters (IterationEditorForm#validate, TimeEditorForm#validate or IdSearchAction#doExecute). SRC:src/com/technoetic/xplanner/forms/TaskEditorForm.java TaskEditorForm#validate keeps its own static date converter built the same way. Consumers: SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate, #toString, #reset (start and end dates are shown and parsed with the static converter; reset clears it and the next initConverters call rebuilds it from the same server-default pattern), SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#valideRow (dates, date-times and durations), TaskEditorForm#validate (created date). Session-locale consumers: SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#getDateFormat, #getDateTimeFormat (saving time entries), the calendar buttons (WAR:WEB-INF/jsp/edit/editIteration.jsp:52-57) and the formatKey displays of FormatDateTag. Bytecode listings agree. The runtime effect is Inferred.</t>
+    <t>Messages "Missing iteration name.", "Iteration must be a positive time interval." and, only for input that does not start with a date (for example not-a-date), "Start date is invalid." / "End date is invalid.". Live examples (W001): end 2026-99-99x and start 2026-99-99 stored as 2034-06-07, end 2026-11-31 as 2026-12-01, start 2026-11-09abc as 2026-11-09.</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.IterationEditorForm#validate (strings iteration.editor.missing_name, bad_start_date, bad_end_date) and #requirePositiveInterval (iteration.editor.nonpositive_interval); WAR:WEB-INF/classes/ResourceBundle.properties:265. Corrected in BA-001-04 (Source: stage-02-pass-002 F-001). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; iteration.editor.nonpositive_interval: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release. Name and both dates are required and the interval must be positive. Correction (BA-001-12, pass-010 F-003): the accepted date and date-time patterns are those of the server default locale's bundle, not of the active (session) bundle as stated above: IterationEditorForm#validate parses with the static converters. The editor form converters are static: SRC:src/com/technoetic/xplanner/forms/AbstractEditorForm.java AbstractEditorForm#initConverters, #getResources, #convertToDate, #convertToDateTime fills dateConverter and dateTimeConverter once from format.date and format.datetime of the server default locale's bundle (Struts MessageResources#getMessage(String) passes no locale, so the default locale taken from Locale.getDefault() when the resources were constructed applies (struts-1.2.9.jar listing), and XPlannerMessageResources#getMessage hands that locale to the Spring message source; SRC:src/net/sf/xplanner/struts/XPlannerMessageResources.java XPlannerMessageResources#getMessage), and decimalConverter with SRC:src/com/technoetic/xplanner/format/DecimalFormat.java DecimalFormat#DecimalFormat, whose parser uses the Accept-Language locale of the first request that calls initConverters (IterationEditorForm#validate, TimeEditorForm#validate or IdSearchAction#doExecute). SRC:src/com/technoetic/xplanner/forms/TaskEditorForm.java TaskEditorForm#validate keeps its own static date converter built the same way. Consumers: SRC:src/com/technoetic/xplanner/forms/IterationEditorForm.java IterationEditorForm#validate, #toString, #reset (start and end dates are shown and parsed with the static converter; reset clears it and the next initConverters call rebuilds it from the same server-default pattern), SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#valideRow (dates, date-times and durations), TaskEditorForm#validate (created date). Session-locale consumers: SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#getDateFormat, #getDateTimeFormat (saving time entries), the calendar buttons (WAR:WEB-INF/jsp/edit/editIteration.jsp:52-57) and the formatKey displays of FormatDateTag. Bytecode listings agree. The runtime effect is Inferred. Stage 3 W001 (BA-001-13, MC-A-19, W001-F-21): B-C-023 (five Create submits: missing name, not-a-date start, end before start and end equal to start rejected with their messages; end 2026-99-99x accepted) and B-C-024 (stored dates of the accepted submits). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks B-C-023, B-C-024).</t>
   </si>
   <si>
     <t>Edit iteration</t>
@@ -1189,7 +1189,7 @@
     <t>Editor with Update/Reset; changes saved.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editIteration.jsp (logic:present oid: status display, daysWorked input); class DomainMetaDataRepository#init (iteration edit, permission edit). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 88 applies to every /do/edit/iteration request (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
+    <t>WAR:WEB-INF/jsp/edit/editIteration.jsp (logic:present oid: status display, daysWorked input); class DomainMetaDataRepository#init (iteration edit, permission edit). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 88 applies to every /do/edit/iteration request (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-025, B-C-026).</t>
   </si>
   <si>
     <t>Delete iteration</t>
@@ -1204,7 +1204,7 @@
     <t>Confirm prompt; iteration, stories, tasks and time entries removed (runtime unverified).</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (iteration delete, onclick action.delete.confirmation); WAR:WEB-INF/struts-config.xml:257; WAR:WEB-INF/action-servlet.xml:196-200; db-changelog.xml permission id 19 (editor, delete, system.project.iteration, positive=false). Cascades: Iteration#getUserStories, UserStory#getTasks, Task#getTimeEntries @OneToMany(cascade=REMOVE). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002, F-007). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute; SRC:src/net/sf/xplanner/domain/Iteration.java Iteration#getUserStories. WAR: classes byte-identical to the v1.1a4 release. The cascades match the source annotations.</t>
+    <t>class DomainMetaDataRepository#init (iteration delete, onclick action.delete.confirmation); WAR:WEB-INF/struts-config.xml:257; WAR:WEB-INF/action-servlet.xml:196-200; db-changelog.xml permission id 19 (editor, delete, system.project.iteration, positive=false). Cascades: Iteration#getUserStories, UserStory#getTasks, Task#getTimeEntries @OneToMany(cascade=REMOVE). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002, F-007). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute; SRC:src/net/sf/xplanner/domain/Iteration.java Iteration#getUserStories. WAR: classes byte-identical to the v1.1a4 release. The cascades match the source annotations. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks setup-C-025, B-C-027, B-C-028, E-C-016, E-C-017; open residual scope R-40 (e)).</t>
   </si>
   <si>
     <t>View iteration stories</t>
@@ -1219,7 +1219,7 @@
     <t>Story table with per-story action icons by permission; zero values highlighted.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:203-205; WAR:WEB-INF/jsp/view/iteration.jsp:20-176; WAR:WEB-INF/jsp/layout/iterationTileParams.jsp:15-41; WAR:WEB-INF/jsp/view/iteration/progress.jsp. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/struts-config.xml:203-205; WAR:WEB-INF/jsp/view/iteration.jsp:20-176; WAR:WEB-INF/jsp/layout/iterationTileParams.jsp:15-41; WAR:WEB-INF/jsp/view/iteration/progress.jsp. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-044, B-C-029, B-C-030).</t>
   </si>
   <si>
     <t>An iteration without stories shows a "no stories" message.</t>
@@ -1228,7 +1228,7 @@
     <t>Message stories.none.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/iteration.jsp:166-168. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/jsp/view/iteration.jsp:166-168. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-039, B-C-031).</t>
   </si>
   <si>
     <t>The progress bar is rendered as HTML by default (xplanner.progressbar.impl=html); the actual-hours column is hidden when the image implementation is configured.</t>
@@ -1240,7 +1240,7 @@
     <t>HTML progress bars and actual hours column in the shipped configuration.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/xplanner.properties:133; WAR:WEB-INF/jsp/view/iteration.jsp:115-121. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/classes/xplanner.properties:133; WAR:WEB-INF/jsp/view/iteration.jsp:115-121. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks B-C-032, F-C-007; open residual scope R-31 (e)).</t>
   </si>
   <si>
     <t>Reorder stories</t>
@@ -1255,7 +1255,7 @@
     <t>After "save order" the page reloads with stories in the new order.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/iteration.jsp:33-36,79-89,160-162 (form /do/edit/reorderstories, orderNo inputs); WAR:WEB-INF/struts-config.xml:357-362; class com.technoetic.xplanner.actions.ReorderStoriesAction. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); ReorderStoriesAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed at class level. SRC:src/com/technoetic/xplanner/actions/ReorderStoriesAction.java ReorderStoriesAction. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes exist and nothing read contradicts the claim.</t>
+    <t>WAR:WEB-INF/jsp/view/iteration.jsp:33-36,79-89,160-162 (form /do/edit/reorderstories, orderNo inputs); WAR:WEB-INF/struts-config.xml:357-362; class com.technoetic.xplanner.actions.ReorderStoriesAction. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); ReorderStoriesAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed at class level. SRC:src/com/technoetic/xplanner/actions/ReorderStoriesAction.java ReorderStoriesAction. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes exist and nothing read contradicts the claim. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-033, B-C-034).</t>
   </si>
   <si>
     <t>A non-numeric order number is rejected.</t>
@@ -1267,7 +1267,7 @@
     <t>Message "Invalid order number &lt;n&gt; entered" on the iteration page.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.ReorderStoriesForm#validate (string story.editor.invalid.order.number); struts-config.xml:360 (error -&gt; iteration.jsp). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/ReorderStoriesForm.java ReorderStoriesForm#validate. WAR: classes byte-identical to the v1.1a4 release. Each order value must parse as a number.</t>
+    <t>class com.technoetic.xplanner.forms.ReorderStoriesForm#validate (string story.editor.invalid.order.number); struts-config.xml:360 (error -&gt; iteration.jsp). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/ReorderStoriesForm.java ReorderStoriesForm#validate. WAR: classes byte-identical to the v1.1a4 release. Each order value must parse as a number. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-035).</t>
   </si>
   <si>
     <t>Move multiple stories</t>
@@ -1279,10 +1279,10 @@
     <t>Bulk re-planning.</t>
   </si>
   <si>
-    <t>Move page with target iteration select; selected stories moved; redirect to /do/view/iteration?oid=&lt;source&gt;.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/iteration.jsp:38-40,60-64 (selected[] checkboxes, submitMoveMultiple); WAR:WEB-INF/struts-config.xml:364-366; WAR:WEB-INF/jsp/edit/moveStories.jsp; class com.technoetic.xplanner.actions.MoveStoriesAction (string "/do/view/iteration?oid="). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); MoveStoriesAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/MoveStoriesAction.java MoveStoriesAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. Each selected story is moved, both iterations are reordered and the browser is redirected to the source iteration.</t>
+    <t>Move page with target iteration select; selected stories moved; redirect to /do/view/iteration?oid=&lt;source&gt;. The target select lists the iterations of all projects the user can see (14 options across five projects for an editor in W001), with the first option pre-selected; whether a user without a role on a project also sees its iterations was not tested.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/iteration.jsp:38-40,60-64 (selected[] checkboxes, submitMoveMultiple); WAR:WEB-INF/struts-config.xml:364-366; WAR:WEB-INF/jsp/edit/moveStories.jsp; class com.technoetic.xplanner.actions.MoveStoriesAction (string "/do/view/iteration?oid="). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); MoveStoriesAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/MoveStoriesAction.java MoveStoriesAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. Each selected story is moved, both iterations are reordered and the browser is redirected to the source iteration. Stage 3 W001 (BA-001-13, MC-B-03, W001-F-22): Move Stories page: 14 iteration options from five projects, targetIterationId pre-set to the first (an S3 Shared iteration); the move itself matched (B-C-036). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks B-C-036, B-C-037).</t>
   </si>
   <si>
     <t>Start iteration</t>
@@ -1297,7 +1297,7 @@
     <t>Iteration becomes active and opening data samples are taken; the page "Start Iteration: &lt;name&gt;" with "Do you want to start the iteration?" and OK/Cancel appears only in the two cases above.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (start -&gt; start/iteration, permission edit); WAR:WEB-INF/struts-config.xml:245-248; WAR:WEB-INF/jsp/edit/editIterationStatus.jsp:43-47 (message_1 only when UpdateTimeAction.isFromUpdateTime) and :58-60 (message_4); WAR:WEB-INF/classes/ResourceBundle.properties:272,275; class StartIterationAction#beforeObjectCommit ("started", DataSampler.generateOpeningDataSamples). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); StartIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-005). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; iteration.status.editor.message_4 is defined only in the default and "--" bundles. Bundles without the key fall back to the default text (framework behavior, GAP-011). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editIterationStatus.jsp writes the raw request parameters fkey (34), returnto (35) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Script context (BA-001-09, pass-007 F-002, check (i)): the page binds returnto from the request (WAR:WEB-INF/jsp/edit/editIterationStatus.jsp:32, bean:parameter) and writes it unescaped after the context path into the JavaScript string of the Cancel button's onclick handler (document.location='&lt;context path&gt;&lt;returnto&gt;', :70). A crafted value can end the string and add script, and it chooses where Cancel leads on the same host. The page is the input and forward of /do/start/iteration and /do/close/iteration (WAR:WEB-INF/struts-config.xml:119-120,245,251) (Inferred; observed risk only, Q3 deferred; Q3 facts). Inventory: .migration-tmp/stage-01/out/script-sinks-09.txt. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/actions/StartIterationAction.java StartIterationAction#doExecute, #beforeObjectCommit; SRC:src/net/sf/xplanner/domain/Iteration.java Iteration#close, #start. WAR: classes byte-identical to the v1.1a4 release. The confirmation page is shown only when another iteration of the project is active (row 99) or when the request comes from time entry (row 100); otherwise the first request starts the iteration at once and redirects to returnto or the projects list. The action first calls Iteration#close (status inactive) and the hook then calls Iteration#start, so the iteration ends active (bytecode listing: Iteration.close at offsets 173 and 285).</t>
+    <t>class DomainMetaDataRepository#init (start -&gt; start/iteration, permission edit); WAR:WEB-INF/struts-config.xml:245-248; WAR:WEB-INF/jsp/edit/editIterationStatus.jsp:43-47 (message_1 only when UpdateTimeAction.isFromUpdateTime) and :58-60 (message_4); WAR:WEB-INF/classes/ResourceBundle.properties:272,275; class StartIterationAction#beforeObjectCommit ("started", DataSampler.generateOpeningDataSamples). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); StartIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-005). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; iteration.status.editor.message_4 is defined only in the default and "--" bundles. Bundles without the key fall back to the default text (framework behavior, GAP-011). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editIterationStatus.jsp writes the raw request parameters fkey (34), returnto (35) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Script context (BA-001-09, pass-007 F-002, check (i)): the page binds returnto from the request (WAR:WEB-INF/jsp/edit/editIterationStatus.jsp:32, bean:parameter) and writes it unescaped after the context path into the JavaScript string of the Cancel button's onclick handler (document.location='&lt;context path&gt;&lt;returnto&gt;', :70). A crafted value can end the string and add script, and it chooses where Cancel leads on the same host. The page is the input and forward of /do/start/iteration and /do/close/iteration (WAR:WEB-INF/struts-config.xml:119-120,245,251) (Inferred; observed risk only, Q3 deferred; Q3 facts). Inventory: .migration-tmp/stage-01/out/script-sinks-09.txt. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/actions/StartIterationAction.java StartIterationAction#doExecute, #beforeObjectCommit; SRC:src/net/sf/xplanner/domain/Iteration.java Iteration#close, #start. WAR: classes byte-identical to the v1.1a4 release. The confirmation page is shown only when another iteration of the project is active (row 99) or when the request comes from time entry (row 100); otherwise the first request starts the iteration at once and redirects to returnto or the projects list. The action first calls Iteration#close (status inactive) and the hook then calls Iteration#start, so the iteration ends active (bytecode listing: Iteration.close at offsets 173 and 285). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-040, B-C-038, B-C-039).</t>
   </si>
   <si>
     <t>If other iterations are still started, the page proposes closing them (checked by default).</t>
@@ -1309,7 +1309,7 @@
     <t>Message "...{n} started iteration(s) need(s) to be closed." with "Close started iterations?" checkbox.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editIterationStatus.jsp (startedIterationsNr, closeIterations checkbox); ResourceBundle.properties iteration.status.editor.message_2/3; class StartIterationAction ("startedIterationsNr"). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/StartIterationAction.java StartIterationAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. With started iterations in the project the action counts them and shows the start page; a confirmed start with the checkbox closes them.</t>
+    <t>WAR:WEB-INF/jsp/edit/editIterationStatus.jsp (startedIterationsNr, closeIterations checkbox); ResourceBundle.properties iteration.status.editor.message_2/3; class StartIterationAction ("startedIterationsNr"). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/StartIterationAction.java StartIterationAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. With started iterations in the project the action counts them and shows the start page; a confirmed start with the checkbox closes them. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-040).</t>
   </si>
   <si>
     <t>Entering time on a task of a not-yet-started iteration first asks to start the iteration and then continues to the time entry.</t>
@@ -1321,7 +1321,7 @@
     <t>Start page with message "The iteration has not been started yet"; after OK the saved time form is processed.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.actions.UpdateTimeAction#isIterationStarted/#doExecute (strings "/do/start/iteration", "from_edit/time", "UpdateTimeAction.savedForm"); WAR:WEB-INF/struts-config.xml:247 (forward edit/time); editIterationStatus.jsp (UpdateTimeAction.isFromUpdateTime). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#doExecute, #isIterationStarted; SRC:src/com/technoetic/xplanner/actions/StartIterationAction.java StartIterationAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. A submitted time form for a task of an inactive iteration is saved in the session and forwarded to /do/start/iteration; after the confirmation the start action forwards to the time editor in wizard mode.</t>
+    <t>class com.technoetic.xplanner.actions.UpdateTimeAction#isIterationStarted/#doExecute (strings "/do/start/iteration", "from_edit/time", "UpdateTimeAction.savedForm"); WAR:WEB-INF/struts-config.xml:247 (forward edit/time); editIterationStatus.jsp (UpdateTimeAction.isFromUpdateTime). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#doExecute, #isIterationStarted; SRC:src/com/technoetic/xplanner/actions/StartIterationAction.java StartIterationAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. A submitted time form for a task of an inactive iteration is saved in the session and forwarded to /do/start/iteration; after the confirmation the start action forwards to the time editor in wizard mode. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-041).</t>
   </si>
   <si>
     <t>Close iteration and continue unfinished stories</t>
@@ -1333,22 +1333,22 @@
     <t>End the time box and carry over remaining work.</t>
   </si>
   <si>
-    <t>Iteration set inactive; data sample taken; redirect to the continue-unfinished-stories page.</t>
-  </si>
-  <si>
-    <t>class DomainMetaDataRepository#init (close -&gt; close/iteration); WAR:WEB-INF/struts-config.xml:251-255 (forward onclose -&gt; /do/continue/unfinished/stories); class CloseIterationAction ("closed", "onclose"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); CloseIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Redirect target (BA-001-08, pass-006 F-002, check (e)): CloseIterationAction#doExecute redirects to the fixed onclose forward (/do/continue/unfinished/stories) and appends "?iterationId=", the iteration id, "&amp;" and the returnto request value unencoded to it, followed by "?oid=" and "&amp;fkey=" parts (bytecode listing), so the host of this redirect is fixed; the continue step (ContinueUnfinishedStoriesAction#doExecute) then redirects to its own returnto parameter unchanged (Inferred; observed risk only, Q3 deferred; Q3 facts). Script context (BA-001-09, pass-007 F-002): the close confirmation uses the same page, WAR:WEB-INF/jsp/edit/editIterationStatus.jsp (WAR:WEB-INF/struts-config.xml:120,251), whose Cancel button writes the returnto request value unescaped into its onclick script (:70; row 98; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/CloseIterationAction.java CloseIterationAction#doExecute, #beforeObjectCommit. WAR: classes byte-identical to the v1.1a4 release. An active iteration is set inactive (closing samples in the hook) and the browser goes to the continue page.</t>
-  </si>
-  <si>
-    <t>On the continue page the user selects a future iteration and confirms; unfinished stories are continued there.</t>
+    <t>Iteration set inactive; data sample taken; redirect to the continue-unfinished-stories page. The redirect Location carries iterationId but no projectId ("/do/continue/unfinished/stories?iterationId=&lt;id&gt;&amp;/do/view/iteration?oid=&lt;id&gt;?oid=&lt;id&gt;&amp;fkey=&lt;id&gt;"), so the continue page shows "No Future Iteration Available." even when the project has later iterations (W001).</t>
+  </si>
+  <si>
+    <t>class DomainMetaDataRepository#init (close -&gt; close/iteration); WAR:WEB-INF/struts-config.xml:251-255 (forward onclose -&gt; /do/continue/unfinished/stories); class CloseIterationAction ("closed", "onclose"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); CloseIterationAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Redirect target (BA-001-08, pass-006 F-002, check (e)): CloseIterationAction#doExecute redirects to the fixed onclose forward (/do/continue/unfinished/stories) and appends "?iterationId=", the iteration id, "&amp;" and the returnto request value unencoded to it, followed by "?oid=" and "&amp;fkey=" parts (bytecode listing), so the host of this redirect is fixed; the continue step (ContinueUnfinishedStoriesAction#doExecute) then redirects to its own returnto parameter unchanged (Inferred; observed risk only, Q3 deferred; Q3 facts). Script context (BA-001-09, pass-007 F-002): the close confirmation uses the same page, WAR:WEB-INF/jsp/edit/editIterationStatus.jsp (WAR:WEB-INF/struts-config.xml:120,251), whose Cancel button writes the returnto request value unescaped into its onclick script (:70; row 98; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/CloseIterationAction.java CloseIterationAction#doExecute, #beforeObjectCommit. WAR: classes byte-identical to the v1.1a4 release. An active iteration is set inactive (closing samples in the hook) and the browser goes to the continue page. Stage 3 W001 (BA-001-13, MC-A-20, W001-F-23): Close as editor and as viewer: 302 to the Location above, iteration not started afterwards (B-C-042, B-C-043); the continue page without projectId shows "No Future Iteration Available.", with projectId=222 the target select (5 later iterations) and Ok/Cancel (B-C-045). The data sample at close was not observed (residual R-25). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks B-C-042, B-C-043, F-C-009; open residual scope R-25 (d)).</t>
+  </si>
+  <si>
+    <t>On the continue page the user selects a future iteration and confirms; unfinished stories are continued there. In this baseline the confirmation answers HTTP 500 and continues nothing (W001).</t>
   </si>
   <si>
     <t>Carry-over of incomplete stories.</t>
   </si>
   <si>
-    <t>Target select with OK/Cancel; continued stories appear in the target iteration.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/struts-config.xml:277-279; WAR:WEB-INF/jsp/edit/continueUnfinishedStories.jsp; class ContinueUnfinishedStoriesAction#continueIteration. Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/continueUnfinishedStories.jsp writes the raw request parameters fkey (32) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ContinueUnfinishedStoriesAction.java ContinueUnfinishedStoriesAction#continueIteration. WAR: classes byte-identical to the v1.1a4 release. With a target iteration the unfinished stories are continued there.</t>
+    <t>Target select with OK/Cancel, shown only when projectId is in the URL (after Close the page shows "No Future Iteration Available.", row 101); continued stories appear in the target iteration (source). Live (W001): the continue submission answers HTTP 500 (HibernateException "Illegal attempt to associate a collection with two open sessions"), no continuation story is created and the stories stay unchanged.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/struts-config.xml:277-279; WAR:WEB-INF/jsp/edit/continueUnfinishedStories.jsp; class ContinueUnfinishedStoriesAction#continueIteration. Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/continueUnfinishedStories.jsp writes the raw request parameters fkey (32) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ContinueUnfinishedStoriesAction.java ContinueUnfinishedStoriesAction#continueIteration. WAR: classes byte-identical to the v1.1a4 release. With a target iteration the unfinished stories are continued there. Stage 3 W001 (BA-001-13, MC-A-20, MC-A-21, W001-F-23, W001-F-24): B-C-044 (OK on the page reached from Close: nothing continued), B-C-045 (target select only with projectId), B-C-046 (OK with projectId: HTTP 500, two open sessions; stories unchanged). Status Yes -&gt; Partial (R-G2). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks B-C-044, B-C-045, B-C-046).</t>
   </si>
   <si>
     <t>If no future iteration exists, the page says so.</t>
@@ -1360,7 +1360,7 @@
     <t>Message "No Future Iteration Available."</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/continueUnfinishedStories.jsp (iterationLoader.getIterationOptions(...).size() == 0; key iteration.status.editor.no_future_iteration). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/jsp/edit/continueUnfinishedStories.jsp (iterationLoader.getIterationOptions(...).size() == 0; key iteration.status.editor.no_future_iteration). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-047).</t>
   </si>
   <si>
     <t>Choosing the same iteration is rejected.</t>
@@ -1372,7 +1372,7 @@
     <t>Message "You cannot continue in the same iteration. Please choose a different one."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.ContinueUnfinishedStoriesForm#validate (string iteration.status.editor.continue_in_same_iteration). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/ContinueUnfinishedStoriesForm.java ContinueUnfinishedStoriesForm#validate. WAR: classes byte-identical to the v1.1a4 release. The same iteration is rejected on OK.</t>
+    <t>class com.technoetic.xplanner.forms.ContinueUnfinishedStoriesForm#validate (string iteration.status.editor.continue_in_same_iteration). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/ContinueUnfinishedStoriesForm.java ContinueUnfinishedStoriesForm#validate. WAR: classes byte-identical to the v1.1a4 release. The same iteration is rejected on OK. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-048).</t>
   </si>
   <si>
     <t>Tabbed iteration view</t>
@@ -1387,22 +1387,22 @@
     <t>Request expected to fail (missing JSP).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:199-201 (forward display -&gt; /WEB-INF/jsp/view/iterationTabs.jsp, ABSENT); WAR:WEB-INF/action-servlet.xml:84-88 (ViewObjectAction type Iteration); no live link found (linkgraph.txt). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ViewObjectAction.java ViewObjectAction#doExecute. WAR: classes byte-identical to the v1.1a4 release; iterationTabs.jsp absent from both the WAR and the SVN webapp. The action forwards to the display path, whose JSP is missing.</t>
+    <t>WAR:WEB-INF/struts-config.xml:199-201 (forward display -&gt; /WEB-INF/jsp/view/iterationTabs.jsp, ABSENT); WAR:WEB-INF/action-servlet.xml:84-88 (ViewObjectAction type Iteration); no live link found (linkgraph.txt). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ViewObjectAction.java ViewObjectAction#doExecute. WAR: classes byte-identical to the v1.1a4 release; iterationTabs.jsp absent from both the WAR and the SVN webapp. The action forwards to the display path, whose JSP is missing. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-049).</t>
   </si>
   <si>
     <t>View all tasks of an iteration</t>
   </si>
   <si>
-    <t>The iteration task view lists all tasks grouped by story with order, story, task, ID, acceptor, status icon, original estimate, estimate, actual, remaining, disposition and type, plus a legend.</t>
+    <t>The iteration task view lists all tasks with order, story, task, ID, acceptor, status icon, original estimate, estimate, actual, remaining, disposition and type, plus a legend. By default the table is sorted by its 7th column (for the viewer the original estimate, ascending), so tasks of one story can be interleaved with other stories; the story name is omitted only when the preceding row has the same story (W001).</t>
   </si>
   <si>
     <t>See all work items of the time box.</t>
   </si>
   <si>
-    <t>Grouped sortable task table with legend (started, completed, unassigned, unestimated).</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/struts-config.xml:211-213; WAR:WEB-INF/jsp/view/iterationTasks.jsp; links from WAR:WEB-INF/jsp/view/iteration/links.jsp:29 and globalLinks.jsp:22. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>Sortable task table, sorted by default by its 7th column, with legend (started, completed, unassigned, unestimated).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/struts-config.xml:211-213; WAR:WEB-INF/jsp/view/iterationTasks.jsp; links from WAR:WEB-INF/jsp/view/iteration/links.jsp:29 and globalLinks.jsp:22. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Stage 3 W001 (BA-001-13, MC-A-22, W001-F-25): All Tasks of S3-B I1 Current read as the viewer: rows in original-estimate order with tasks of story S1 interleaved; columns and legend as mapped (B-C-050). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks B-C-050).</t>
   </si>
   <si>
     <t>Iteration metrics</t>
@@ -1417,7 +1417,7 @@
     <t>Page layout with developer table, paired/unpaired bars and legend; in this baseline the figures are expected to be empty or zero.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:219-221; WAR:WEB-INF/action-servlet.xml:114-118 (ViewIterationMetricsAction); WAR:WEB-INF/jsp/view/iterationMetrics.jsp:19-90; mappings/Metrics.xml query iterationHoursWorkedQuery. BA-001-03 impact sweep: ViewIterationMetricsAction#doExecute passes #getRepository(mapping, request) to IterationMetrics#setIterationRepository, and #getRepository returns null (bytecode listing: aconst_null, areturn); IterationMetrics#calculateDeveloperMetrics first calls #getIterationObject, which calls load on that repository, so the developer calculation is expected to fail with a null reference that IterationMetrics#analyze catches and logs; the page then shows zero totals and empty developer tables (runtime unverified). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/ViewIterationMetricsAction.java ViewIterationMetricsAction#getRepository; SRC:src/com/technoetic/xplanner/metrics/IterationMetrics.java IterationMetrics#analyze, #calculateDeveloperMetrics. WAR: classes byte-identical to the v1.1a4 release. GetRepository returns null in the source as in the bytecode (the repository lookup is commented out); the page result is a runtime effect. Live question: Does the iteration metrics page show zero totals and empty developer tables?</t>
+    <t>WAR:WEB-INF/struts-config.xml:219-221; WAR:WEB-INF/action-servlet.xml:114-118 (ViewIterationMetricsAction); WAR:WEB-INF/jsp/view/iterationMetrics.jsp:19-90; mappings/Metrics.xml query iterationHoursWorkedQuery. BA-001-03 impact sweep: ViewIterationMetricsAction#doExecute passes #getRepository(mapping, request) to IterationMetrics#setIterationRepository, and #getRepository returns null (bytecode listing: aconst_null, areturn); IterationMetrics#calculateDeveloperMetrics first calls #getIterationObject, which calls load on that repository, so the developer calculation is expected to fail with a null reference that IterationMetrics#analyze catches and logs; the page then shows zero totals and empty developer tables (runtime unverified). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/ViewIterationMetricsAction.java ViewIterationMetricsAction#getRepository; SRC:src/com/technoetic/xplanner/metrics/IterationMetrics.java IterationMetrics#analyze, #calculateDeveloperMetrics. WAR: classes byte-identical to the v1.1a4 release. GetRepository returns null in the source as in the bytecode (the repository lookup is commented out); the page result is a runtime effect. Live question: Does the iteration metrics page show zero totals and empty developer tables? Stage 3 W001 live answer (BA-001-13, MC-C-16): Yes: Total Person Hours Worked 0.0, paired percentage 0.0%, "Nothing found to display.", although time was recorded (B-C-051). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-051).</t>
   </si>
   <si>
     <t>A second table shows per developer accepted hours (story and task), own worked hours, remaining hours and a worked-of-accepted bar.</t>
@@ -1429,7 +1429,7 @@
     <t>Accepted-hours table with bars; expected empty in this baseline for the same reason.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/iterationMetrics.jsp:96-175. BA-001-03 impact sweep: ViewIterationMetricsAction#doExecute passes #getRepository(mapping, request) to IterationMetrics#setIterationRepository, and #getRepository returns null (bytecode listing: aconst_null, areturn); IterationMetrics#calculateDeveloperMetrics first calls #getIterationObject, which calls load on that repository, so the developer calculation is expected to fail with a null reference that IterationMetrics#analyze catches and logs; the page then shows zero totals and empty developer tables (runtime unverified). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/ViewIterationMetricsAction.java ViewIterationMetricsAction#getRepository. WAR: classes byte-identical to the v1.1a4 release. Same cause as row 107. Live question: Is the accepted-hours table empty?</t>
+    <t>WAR:WEB-INF/jsp/view/iterationMetrics.jsp:96-175. BA-001-03 impact sweep: ViewIterationMetricsAction#doExecute passes #getRepository(mapping, request) to IterationMetrics#setIterationRepository, and #getRepository returns null (bytecode listing: aconst_null, areturn); IterationMetrics#calculateDeveloperMetrics first calls #getIterationObject, which calls load on that repository, so the developer calculation is expected to fail with a null reference that IterationMetrics#analyze catches and logs; the page then shows zero totals and empty developer tables (runtime unverified). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/ViewIterationMetricsAction.java ViewIterationMetricsAction#getRepository. WAR: classes byte-identical to the v1.1a4 release. Same cause as row 107. Live question: Is the accepted-hours table empty? Stage 3 W001 live answer (BA-001-13, MC-C-17): Yes: "Nothing found to display." (B-C-052). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-052).</t>
   </si>
   <si>
     <t>Iteration statistics charts</t>
@@ -1444,7 +1444,7 @@
     <t>Cewolf-rendered 3D pie charts and the progress and burn-down line chart images.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/iteration/globalLinks.jsp:33-37; WAR:WEB-INF/struts-config.xml:223-225; WAR:WEB-INF/action-servlet.xml:120-124; WAR:WEB-INF/classes/xplanner.properties:66-73,197; WAR:WEB-INF/jsp/view/iterationStatistics.jsp:46-230 (cewolf charts); WAR:WEB-INF/web.xml:211-225,293-296 (CewolfServlet /cewolf/*). Chart sweep (BA-001-05): live charts in WAR:WEB-INF/jsp/view/iterationStatistics.jsp: taskTypeChart, taskDispositionChart, taskTypeEstimatedHoursChart, taskDispositionEstimatedHoursChart, taskTypeActualHoursChart, taskDispositionActualHoursChart (pie3d, lines 46-112); velocityChart (:123-153, flag xplanner.effort.chart.velocity), velocityChart2 progress chart (:155-191, flag xplanner.effort.chart.progress), burnDownChart (:193-228, flag xplanner.effort.chart.burndown); flags at WAR:WEB-INF/classes/xplanner.properties:66-68 (burndown and progress displayed, velocity notDisplayed). Corrected in BA-001-05 (Source: stage-02-pass-003 F-004). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/jsp/view/iteration/globalLinks.jsp:33-37; WAR:WEB-INF/struts-config.xml:223-225; WAR:WEB-INF/action-servlet.xml:120-124; WAR:WEB-INF/classes/xplanner.properties:66-73,197; WAR:WEB-INF/jsp/view/iterationStatistics.jsp:46-230 (cewolf charts); WAR:WEB-INF/web.xml:211-225,293-296 (CewolfServlet /cewolf/*). Chart sweep (BA-001-05): live charts in WAR:WEB-INF/jsp/view/iterationStatistics.jsp: taskTypeChart, taskDispositionChart, taskTypeEstimatedHoursChart, taskDispositionEstimatedHoursChart, taskTypeActualHoursChart, taskDispositionActualHoursChart (pie3d, lines 46-112); velocityChart (:123-153, flag xplanner.effort.chart.velocity), velocityChart2 progress chart (:155-191, flag xplanner.effort.chart.progress), burnDownChart (:193-228, flag xplanner.effort.chart.burndown); flags at WAR:WEB-INF/classes/xplanner.properties:66-68 (burndown and progress displayed, velocity notDisplayed). Corrected in BA-001-05 (Source: stage-02-pass-003 F-004). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-053).</t>
   </si>
   <si>
     <t>A progress line chart plots the iteration's estimated and actual hours from the stored data samples; it is shown while xplanner.effort.chart.progress is "displayed", which is the shipped value.</t>
@@ -1456,7 +1456,7 @@
     <t>Line chart "velocityChart2" with the aspects estimatedHours and actualHours; weekends included per xplanner.effort.chart.include.weekends.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/iterationStatistics.jsp:155-191 (propertyEqual key xplanner.effort.chart.progress value displayed; jsp:useBean velocityData2 class com.technoetic.xplanner.charts.DataSampleData, aspects estimatedHours,actualHours at :163-165; cewolf:chart velocityChart2 type line); WAR:WEB-INF/classes/xplanner.properties:67 (xplanner.effort.chart.progress=displayed), :73 (include.weekends=true). Data comes from the data samples (row 112). Provenance: property value from a rewritten entry (GAP-005 P-03). Source: stage-02-pass-003 F-004. Source reconciliation (BA-001-11, A4): confirmed at class level. SRC:src/com/technoetic/xplanner/charts/DataSampleData.java DataSampleData. WAR: classes byte-identical to the v1.1a4 release; values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes exist and nothing read contradicts the claim.</t>
+    <t>WAR:WEB-INF/jsp/view/iterationStatistics.jsp:155-191 (propertyEqual key xplanner.effort.chart.progress value displayed; jsp:useBean velocityData2 class com.technoetic.xplanner.charts.DataSampleData, aspects estimatedHours,actualHours at :163-165; cewolf:chart velocityChart2 type line); WAR:WEB-INF/classes/xplanner.properties:67 (xplanner.effort.chart.progress=displayed), :73 (include.weekends=true). Data comes from the data samples (row 112). Provenance: property value from a rewritten entry (GAP-005 P-03). Source: stage-02-pass-003 F-004. Source reconciliation (BA-001-11, A4): confirmed at class level. SRC:src/com/technoetic/xplanner/charts/DataSampleData.java DataSampleData. WAR: classes byte-identical to the v1.1a4 release; values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes exist and nothing read contradicts the claim. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-054).</t>
   </si>
   <si>
     <t>Velocity charts appear only if xplanner.effort.chart.velocity is "displayed" (shipped: notDisplayed); weekends are included in charts (include.weekends=true).</t>
@@ -1468,7 +1468,7 @@
     <t>No velocity chart in the shipped configuration.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/xplanner.properties:66-73; WAR:WEB-INF/jsp/view/iterationStatistics.jsp:123-153 (propertyEqual xplanner.effort.chart.velocity, velocityChart). Citation range narrowed in BA-001-05 (was 122-196, which also spanned the progress and burn-down blocks). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/classes/xplanner.properties:66-73; WAR:WEB-INF/jsp/view/iterationStatistics.jsp:123-153 (propertyEqual xplanner.effort.chart.velocity, velocityChart). Citation range narrowed in BA-001-05 (was 122-196, which also spanned the progress and burn-down blocks). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-055).</t>
   </si>
   <si>
     <t>The burn-down and progress charts depend on stored data samples; samples are written at iteration start/close and by the manual sampling action, while the nightly Quartz sampling trigger is not scheduled.</t>
@@ -1480,7 +1480,7 @@
     <t>Burn-down and progress charts may be sparse between start and close.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/spring-beans.xml:343-383 (datasamplingJob, datasamplingTrigger) and :385-402 (SchedulerFactoryBean commented out); references from classes StartIterationAction and CloseIterationAction to DataSampler; test-action-servlet.xml:4-7. Both charts use class com.technoetic.xplanner.charts.DataSampleData (WAR:WEB-INF/jsp/view/iterationStatistics.jsp:163-165 aspects estimatedHours,actualHours; :202-205 aspect remainingHours). Corrected in BA-001-05 (Source: stage-02-pass-003 F-004). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/StartIterationAction.java StartIterationAction#beforeObjectCommit; SRC:src/com/technoetic/xplanner/actions/CloseIterationAction.java CloseIterationAction#beforeObjectCommit, #closeIteration. WAR: classes byte-identical to the v1.1a4 release; patched spring-beans.xml with the Quartz scheduler commented out (WAR governs). Opening samples are generated when an iteration starts and closing samples when an active iteration is closed; nothing else schedules sampling in the WAR configuration. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>WAR:WEB-INF/classes/spring-beans.xml:343-383 (datasamplingJob, datasamplingTrigger) and :385-402 (SchedulerFactoryBean commented out); references from classes StartIterationAction and CloseIterationAction to DataSampler; test-action-servlet.xml:4-7. Both charts use class com.technoetic.xplanner.charts.DataSampleData (WAR:WEB-INF/jsp/view/iterationStatistics.jsp:163-165 aspects estimatedHours,actualHours; :202-205 aspect remainingHours). Corrected in BA-001-05 (Source: stage-02-pass-003 F-004). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/StartIterationAction.java StartIterationAction#beforeObjectCommit; SRC:src/com/technoetic/xplanner/actions/CloseIterationAction.java CloseIterationAction#beforeObjectCommit, #closeIteration. WAR: classes byte-identical to the v1.1a4 release; patched spring-beans.xml with the Quartz scheduler commented out (WAR governs). Opening samples are generated when an iteration starts and closing samples when an active iteration is closed; nothing else schedules sampling in the WAR configuration. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream. Stage 3 W001 live answer (BA-001-13, MC-C-25): no nightly sample is taken at 23:55 (L-C-008; no Quartz scheduler, D-C-017); the start sample was observed (B-C-056). The manual sampling action was not run: residual R-30, candidate outside the core (owner decision at Stage 4). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks B-C-056, E-C-025, F-C-004, L-C-008; open residual scope R-30 (e), candidate outside the core (owner decision at Stage 4)).</t>
   </si>
   <si>
     <t>Iteration accuracy</t>
@@ -1495,7 +1495,7 @@
     <t>Two summary tables with tooltips and a per-story table.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:227-229; WAR:WEB-INF/jsp/view/iterationAccuracy.jsp:21-186. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/struts-config.xml:227-229; WAR:WEB-INF/jsp/view/iterationAccuracy.jsp:21-186. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-057).</t>
   </si>
   <si>
     <t>Iteration task board (dashboard)</t>
@@ -1510,7 +1510,7 @@
     <t>Story rows with task cards in three columns; cards can be dragged, but the drag only moves page elements and saves nothing.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/iteration/globalLinks.jsp:14-18 (xplanner:link to /do/view/dashboard with paramId iterationId, only if iteration.active); class com.technoetic.xplanner.tags.LinkTag#addNavigationParameters puts fkey = the tag attribute fkey when set, otherwise the current request's oid, and adds returnto and projectId when enabled (bytecode listing), so on /do/view/iteration*?oid=&lt;id&gt; the link carries fkey=&lt;id&gt;; WAR:WEB-INF/struts-config.xml:386; WAR:WEB-INF/jsp/view/dashboard.jsp:101-103 (column titles not started, in progress, done) and :131-132 ($.getJSON rest/view/iteration/${param.fkey}/userstories, row 223); no update call in dashboard.jsp. Corrected in BA-001-06 (Source: stage-02-pass-004 F-002): the earlier "parameter mismatch" did not account for the fkey parameter that the link tag adds. Request-value flow (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/view/dashboard.jsp:132 writes ${param.fkey} into a JavaScript string with EL (enabled under the Servlet 2.4 descriptor) without escaping, so the request value is reflected into the script (Inferred; observed risk only, Q3 deferred). Source: stage-02-pass-005 F-003. Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/tags/LinkTag.java LinkTag#addNavigationParameters. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
+    <t>WAR:WEB-INF/jsp/view/iteration/globalLinks.jsp:14-18 (xplanner:link to /do/view/dashboard with paramId iterationId, only if iteration.active); class com.technoetic.xplanner.tags.LinkTag#addNavigationParameters puts fkey = the tag attribute fkey when set, otherwise the current request's oid, and adds returnto and projectId when enabled (bytecode listing), so on /do/view/iteration*?oid=&lt;id&gt; the link carries fkey=&lt;id&gt;; WAR:WEB-INF/struts-config.xml:386; WAR:WEB-INF/jsp/view/dashboard.jsp:101-103 (column titles not started, in progress, done) and :131-132 ($.getJSON rest/view/iteration/${param.fkey}/userstories, row 223); no update call in dashboard.jsp. Corrected in BA-001-06 (Source: stage-02-pass-004 F-002): the earlier "parameter mismatch" did not account for the fkey parameter that the link tag adds. Request-value flow (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/view/dashboard.jsp:132 writes ${param.fkey} into a JavaScript string with EL (enabled under the Servlet 2.4 descriptor) without escaping, so the request value is reflected into the script (Inferred; observed risk only, Q3 deferred). Source: stage-02-pass-005 F-003. Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/tags/LinkTag.java LinkTag#addNavigationParameters. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-058, E-C-031).</t>
   </si>
   <si>
     <t>Import stories from a spreadsheet</t>
@@ -1522,10 +1522,10 @@
     <t>Bring an existing backlog into XPlanner.</t>
   </si>
   <si>
-    <t>Result "Imported &lt;n&gt; stories"; stories created.</t>
-  </si>
-  <si>
-    <t>class DomainMetaDataRepository#init (importStories -&gt; import/stories); WAR:WEB-INF/struts-config.xml:332-346; WAR:WEB-INF/action-servlet.xml:361-368 (ImportStoriesAction, SpreadsheetStoryImporter); WAR:WEB-INF/jsp/import/stories.jsp; xplanner.properties:277-284 (default headers). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); ImportStoriesAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/import/stories.jsp writes the raw request parameters returnto (32), oid (36) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init. WAR: classes byte-identical to the v1.1a4 release; values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>Result "Imported &lt;n&gt; stories"; stories created (source). Live (W001): every Import Stories submission, multipart as the served form posts it, answers HTTP 500 (NullPointerException at SessionImpl.get via CommonDao.getById and EditObjectAction) before validation or file reading, also with fkey, projectId and oid in the URL; no story is imported, no message is shown and no settings cookie is written.</t>
+  </si>
+  <si>
+    <t>class DomainMetaDataRepository#init (importStories -&gt; import/stories); WAR:WEB-INF/struts-config.xml:332-346; WAR:WEB-INF/action-servlet.xml:361-368 (ImportStoriesAction, SpreadsheetStoryImporter); WAR:WEB-INF/jsp/import/stories.jsp; xplanner.properties:277-284 (default headers). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); ImportStoriesAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/import/stories.jsp writes the raw request parameters returnto (32), oid (36) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init. WAR: classes byte-identical to the v1.1a4 release; values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. Stage 3 W001 (BA-001-13, MC-A-23, W001-F-26): B-C-059 (valid synthetic file: 500, no story), B-C-060 (served action and action URL with fkey/projectId: same NullPointerException). Status Yes -&gt; Partial. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks B-C-059, B-C-060).</t>
   </si>
   <si>
     <t>Missing required inputs are rejected before import.</t>
@@ -1534,10 +1534,10 @@
     <t>Import needs a file and column mapping.</t>
   </si>
   <si>
-    <t>Messages for missing worksheet name, title, end date or priority header, completed status, or file.</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.forms.ImportStoriesForm#validate and ImportForm#validate (import.status.worksheet_name, no_title_column, no_end_date_column, no_priority_column, no_completed_story_status, no_import_file). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/ImportStoriesForm.java ImportStoriesForm#validate, #isNotEmpty; SRC:src/com/technoetic/xplanner/forms/ImportForm.java ImportForm#validate. WAR: classes byte-identical to the v1.1a4 release. Worksheet name, title, end-date and priority columns and (with the option) the completed status are required; the helper named isNotEmpty returns StringUtils.isEmpty, so the checks are correct despite the name (bytecode listing agrees).</t>
+    <t>Messages for missing worksheet name, title, end date or priority header, completed status, or file (source). Live (W001): each of these submissions answers the same HTTP 500 (row 115), so no message is shown.</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.ImportStoriesForm#validate and ImportForm#validate (import.status.worksheet_name, no_title_column, no_end_date_column, no_priority_column, no_completed_story_status, no_import_file). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/ImportStoriesForm.java ImportStoriesForm#validate, #isNotEmpty; SRC:src/com/technoetic/xplanner/forms/ImportForm.java ImportForm#validate. WAR: classes byte-identical to the v1.1a4 release. Worksheet name, title, end-date and priority columns and (with the option) the completed status are required; the helper named isNotEmpty returns StringUtils.isEmpty, so the checks are correct despite the name (bytecode listing agrees). Stage 3 W001 (BA-001-13, MC-A-23, W001-F-26): six submissions, each with one input empty: all HTTP 500, no message (B-C-061). Status Yes -&gt; Partial. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks B-C-061).</t>
   </si>
   <si>
     <t>Import errors for a missing worksheet, missing header, missing required field or corrupt file are shown on the import page.</t>
@@ -1546,10 +1546,10 @@
     <t>Actionable feedback on bad files.</t>
   </si>
   <si>
-    <t>Messages "Could not find worksheet named ...", "Could not find a column with ... as the header...", "Some stories did not have ... specified.", "...appears to be corrupt."</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.actions.ImportStoriesAction#execute: exception handlers (bytecode exception table) catch importer.WrongImportFileSpreadsheetImporterException, MissingFieldSpreadsheetImporterException, MissingColumnHeaderSpreadsheetImporterException and importer.spreadsheet.MissingWorksheetException and save import.status.corrupted_file, missing_required_field, wrong_header and worksheet_not_found. The Struts mapping for the non-existent com.technoetic.xplanner.importer.MissingWorksheetException (WAR:WEB-INF/struts-config.xml:343-345) is therefore redundant, not a defect of the behavior. Corrected in BA-001-04 (Source: stage-02-pass-002 F-008). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ImportStoriesAction.java ImportStoriesAction#execute. WAR: classes byte-identical to the v1.1a4 release. The four importer exceptions become global errors on the import page.</t>
+    <t>Messages "Could not find worksheet named ...", "Could not find a column with ... as the header...", "Some stories did not have ... specified.", "...appears to be corrupt." (source). Live (W001): each case answers the same HTTP 500 (row 115) and no message is shown.</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.actions.ImportStoriesAction#execute: exception handlers (bytecode exception table) catch importer.WrongImportFileSpreadsheetImporterException, MissingFieldSpreadsheetImporterException, MissingColumnHeaderSpreadsheetImporterException and importer.spreadsheet.MissingWorksheetException and save import.status.corrupted_file, missing_required_field, wrong_header and worksheet_not_found. The Struts mapping for the non-existent com.technoetic.xplanner.importer.MissingWorksheetException (WAR:WEB-INF/struts-config.xml:343-345) is therefore redundant, not a defect of the behavior. Corrected in BA-001-04 (Source: stage-02-pass-002 F-008). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ImportStoriesAction.java ImportStoriesAction#execute. WAR: classes byte-identical to the v1.1a4 release. The four importer exceptions become global errors on the import page. Stage 3 W001 (BA-001-13, MC-A-23, W001-F-26): missing worksheet, missing header, missing required field and a corrupt file: all HTTP 500, no message, nothing imported (B-C-062). Status Yes -&gt; Partial. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks B-C-062).</t>
   </si>
   <si>
     <t>Optionally only incomplete stories are imported: rows whose status is "C" (ignoring case) are skipped; the completed-status field must be filled in but does not change this value.</t>
@@ -1558,10 +1558,10 @@
     <t>Avoid importing finished work.</t>
   </si>
   <si>
-    <t>Completed rows skipped when the checkbox is set.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/import/stories.jsp (onlyIncomplete, completedStatus); xplanner.properties:284 (import.spreadsheet.completedStoryStatus=C); class SpreadsheetStoryImporter. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/importer/SpreadsheetStoryImporter.java SpreadsheetStoryImporter#importStories; SRC:src/com/technoetic/xplanner/forms/ImportStoriesForm.java ImportStoriesForm#validate; SRC:src/com/technoetic/xplanner/actions/ImportStoriesAction.java ImportStoriesAction#setCookies. WAR: classes byte-identical to the v1.1a4 release. With the option set, the importer skips rows whose status equals "C" ignoring case; this value is hard-coded (bytecode listing: ldc "C", equalsIgnoreCase). The completed-status field is only required by the form validation and kept in a cookie; it does not change the filter. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>Completed rows skipped when the checkbox is set (source). Live (W001): the import with the checkbox set answers HTTP 500 (row 115) and imports nothing.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/import/stories.jsp (onlyIncomplete, completedStatus); xplanner.properties:284 (import.spreadsheet.completedStoryStatus=C); class SpreadsheetStoryImporter. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/importer/SpreadsheetStoryImporter.java SpreadsheetStoryImporter#importStories; SRC:src/com/technoetic/xplanner/forms/ImportStoriesForm.java ImportStoriesForm#validate; SRC:src/com/technoetic/xplanner/actions/ImportStoriesAction.java ImportStoriesAction#setCookies. WAR: classes byte-identical to the v1.1a4 release. With the option set, the importer skips rows whose status equals "C" ignoring case; this value is hard-coded (bytecode listing: ldc "C", equalsIgnoreCase). The completed-status field is only required by the form validation and kept in a cookie; it does not change the filter. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. Stage 3 W001 (BA-001-13, MC-A-23, W001-F-26): upload with "only incomplete" checked and completed status "X": HTTP 500, no story, no cookie (B-C-063). Status Yes -&gt; Partial. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks B-C-063).</t>
   </si>
   <si>
     <t>After an import the worksheet name, column headers, only-incomplete choice and completed status are saved in browser cookies, and the next import form is pre-filled from those cookies before the property defaults.</t>
@@ -1570,10 +1570,10 @@
     <t>The import settings are remembered per browser.</t>
   </si>
   <si>
-    <t>Import form pre-filled with the last used settings.</t>
-  </si>
-  <si>
-    <t>class ImportStoriesAction#setCookies (cookie names import.spreadsheet.worksheet.name, .story.title.column.header, .iteration.end.date.column.header, .story.estimate.column.header, .story.priority.column.header, .story.status.column.header, .onlyIncomplete, .completedStoryStatus), called from EditObjectAction#doExecute after #saveForm; #populateForm with #getValueFromCookieOrProperties (defaults WAR:WEB-INF/classes/xplanner.properties:278-284; provenance of these default values as in row 115, GAP-005 P-03). Source: stage-02-pass-002 F-008. Cookie lifetime and flags (BA-001-07, mechanism (b)): ImportStoriesAction#addCookie uses the same CookieSupport#createCookie (max-age 2147483647 seconds, no Secure flag, no path). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/ImportStoriesAction.java ImportStoriesAction#setCookies, #addCookie, #populateForm, #getValueFromCookieOrProperties; SRC:src/com/technoetic/xplanner/util/CookieSupport.java CookieSupport#createCookie. WAR: classes byte-identical to the v1.1a4 release. The eight settings are written as cookies after an import and read back, before the property defaults, when the form is shown.</t>
+    <t>Import form pre-filled with the last used settings (source). Live (W001): no import completes (row 115), so no settings cookie is written and the re-opened form shows the property defaults.</t>
+  </si>
+  <si>
+    <t>class ImportStoriesAction#setCookies (cookie names import.spreadsheet.worksheet.name, .story.title.column.header, .iteration.end.date.column.header, .story.estimate.column.header, .story.priority.column.header, .story.status.column.header, .onlyIncomplete, .completedStoryStatus), called from EditObjectAction#doExecute after #saveForm; #populateForm with #getValueFromCookieOrProperties (defaults WAR:WEB-INF/classes/xplanner.properties:278-284; provenance of these default values as in row 115, GAP-005 P-03). Source: stage-02-pass-002 F-008. Cookie lifetime and flags (BA-001-07, mechanism (b)): ImportStoriesAction#addCookie uses the same CookieSupport#createCookie (max-age 2147483647 seconds, no Secure flag, no path). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/ImportStoriesAction.java ImportStoriesAction#setCookies, #addCookie, #populateForm, #getValueFromCookieOrProperties; SRC:src/com/technoetic/xplanner/util/CookieSupport.java CookieSupport#createCookie. WAR: classes byte-identical to the v1.1a4 release. The eight settings are written as cookies after an import and read back, before the property defaults, when the form is shown. Stage 3 W001 (BA-001-13, MC-A-23, W001-F-26): the re-opened form shows the property defaults and the client holds no cookie besides the session (B-C-064; part B blocked, reclassified as observed by the W001 lead). Status Yes -&gt; Partial. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks B-C-064).</t>
   </si>
   <si>
     <t>UF-007</t>
@@ -1585,16 +1585,16 @@
     <t>Create user story</t>
   </si>
   <si>
-    <t>An editor can create a story in an iteration with name, disposition (planned, carried over, added), customer, tracker, status (draft..accepted), priority, order, estimated hours and description.</t>
+    <t>An editor can create a story in an iteration with name, disposition (planned, carried over, added), customer, tracker, status (draft..accepted), priority, order, estimated hours and description. Live (W001): the disposition and status chosen in the editor are not persisted.</t>
   </si>
   <si>
     <t>Capture a unit of customer value.</t>
   </si>
   <si>
-    <t>Story saved in the iteration; user returned to the iteration page.</t>
-  </si>
-  <si>
-    <t>class DomainMetaDataRepository#init (createStory -&gt; edit/userstory); WAR:WEB-INF/struts-config.xml:269-271; WAR:WEB-INF/action-servlet.xml:220-224 (EditStoryAction); WAR:WEB-INF/jsp/edit/editStory.jsp; classes com.technoetic.xplanner.domain.StoryStatus, StoryDisposition (enumeration strings). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editStory.jsp writes the raw request parameters oid (37), fkey (41,44), returnto (43) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/userstory that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new UserStory object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). With merge=true the story validator also skips its name, estimate and priority checks (row 124). No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init; SRC:src/com/technoetic/xplanner/domain/StoryStatus.java StoryStatus; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject, #doExecute. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
+    <t>Story saved in the iteration; user returned to the iteration page. The disposition and status chosen in the editor are not stored: the story keeps Planned and Draft (W001).</t>
+  </si>
+  <si>
+    <t>class DomainMetaDataRepository#init (createStory -&gt; edit/userstory); WAR:WEB-INF/struts-config.xml:269-271; WAR:WEB-INF/action-servlet.xml:220-224 (EditStoryAction); WAR:WEB-INF/jsp/edit/editStory.jsp; classes com.technoetic.xplanner.domain.StoryStatus, StoryDisposition (enumeration strings). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editStory.jsp writes the raw request parameters oid (37), fkey (41,44), returnto (43) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/userstory that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new UserStory object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). With merge=true the story validator also skips its name, estimate and priority checks (row 124). No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init; SRC:src/com/technoetic/xplanner/domain/StoryStatus.java StoryStatus; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject, #doExecute. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Stage 3 W001 (BA-001-13, MC-A-24, W001-F-27): created with added/defined (setup-C-042) and with carriedOver/estimated (B-C-065): shown as Planned/Draft. Status Yes -&gt; Partial (R-G2). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-041, setup-C-042, B-C-065, B-C-066).</t>
   </si>
   <si>
     <t>A new story defaults to priority 4.</t>
@@ -1606,7 +1606,7 @@
     <t>Priority field pre-filled with 4.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/xplanner.properties:150 (xplanner.story.defaultpriority=4); class UserStoryEditorForm (DEFAULT_PRIORITY_KEY, string "xplanner.story.defaultpriority"). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/UserStoryEditorForm.java UserStoryEditorForm#reset, #resetPriority. WAR: classes byte-identical to the v1.1a4 release; default priority from the patched WAR xplanner.properties (WAR governs). Reset sets the priority from xplanner.story.defaultpriority, or from the class default when the key is missing. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/classes/xplanner.properties:150 (xplanner.story.defaultpriority=4); class UserStoryEditorForm (DEFAULT_PRIORITY_KEY, string "xplanner.story.defaultpriority"). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/UserStoryEditorForm.java UserStoryEditorForm#reset, #resetPriority. WAR: classes byte-identical to the v1.1a4 release; default priority from the patched WAR xplanner.properties (WAR governs). Reset sets the priority from xplanner.story.defaultpriority, or from the class default when the key is missing. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-043, B-C-067).</t>
   </si>
   <si>
     <t>A missing name, a negative estimate or a non-numeric priority is rejected.</t>
@@ -1618,34 +1618,34 @@
     <t>Messages "Missing story name.", "Please provide an estimate greater than or equal to zero.", "Please provide a numeric priority."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.UserStoryEditorForm#validate (story.editor.missing_name, negative_estimated_hours, invalid_priority). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/UserStoryEditorForm.java UserStoryEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release. Without merge the name, a non-negative estimate and a numeric priority are required.</t>
-  </si>
-  <si>
-    <t>A story editor request that carries merge=true skips the name, estimate and priority checks, is rejected only when the target iteration equals the current one, and otherwise binds its request parameters directly onto the story; no page of the WAR posts merge=true to the story editor, so this applies to direct requests.</t>
+    <t>class com.technoetic.xplanner.forms.UserStoryEditorForm#validate (story.editor.missing_name, negative_estimated_hours, invalid_priority). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/UserStoryEditorForm.java UserStoryEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release. Without merge the name, a non-negative estimate and a numeric priority are required. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-068).</t>
+  </si>
+  <si>
+    <t>A story editor request that carries merge=true skips the name, estimate and priority checks and is rejected with the same-iteration message when its targetIterationId parameter equals the current iteration or is missing; with a different targetIterationId it binds its request parameters directly onto the story (observed for priority, estimate and description) and does not move the story. Without fkey and projectId the request answers HTTP 500. No page of the WAR posts merge=true to the story editor, so this applies to direct requests (W001).</t>
   </si>
   <si>
     <t>Documents the second validation branch of the story editor.</t>
   </si>
   <si>
-    <t>Message "Cannot move or continue story in same iteration." for merge=true with the same iteration; otherwise no validation message, and the story properties named by request parameters are set without the form copy (runtime unverified).</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.forms.UserStoryEditorForm#validate (bytecode listing: #isMerge false -&gt; story.editor.missing_name, negative_estimated_hours, #validateIsNumber invalid_priority; #isMerge true -&gt; story.editor.same_iteration when targetIterationId equals iterationId). The hidden merge field occurs only in moveContinueStory.jsp, moveContinueTask.jsp, continueUnfinishedStories.jsp and task.jsp, none of which posts to /do/edit/userstory (WAR:WEB-INF/jsp/edit/moveContinueStory.jsp:20,24). CHK-005 (BA-001-05). Source: stage-02-pass-003 F-003. Request binding (BA-001-08, pass-006 F-001): with merge=true, EditObjectAction#populateObject calls org.apache.struts.util.RequestUtils.populate onto the story instead of copying the form and resolving its many-to-one references (bytecode listing), so any writable story property named by a parameter is set, including properties the editor does not show; together with the skipped checks, unvalidated values reach the saved story (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/forms/UserStoryEditorForm.java UserStoryEditorForm#validate; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject. WAR: classes byte-identical to the v1.1a4 release. The two validation branches are confirmed; which properties the binding sets is commons-beanutils behavior (GAP-011). Live question: Does a direct story-editor request with merge=true and an extra property parameter change that property?</t>
+    <t>Message "Cannot move or continue story in same iteration." when targetIterationId is missing or equals the current iteration; with another targetIterationId: 302 without a validation message, the named properties set without the form copy (priority 9, estimate -5.0 and the description in W001, so a negative estimate is stored) and the story stays in its iteration; without fkey and projectId: HTTP 500.</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.UserStoryEditorForm#validate (bytecode listing: #isMerge false -&gt; story.editor.missing_name, negative_estimated_hours, #validateIsNumber invalid_priority; #isMerge true -&gt; story.editor.same_iteration when targetIterationId equals iterationId). The hidden merge field occurs only in moveContinueStory.jsp, moveContinueTask.jsp, continueUnfinishedStories.jsp and task.jsp, none of which posts to /do/edit/userstory (WAR:WEB-INF/jsp/edit/moveContinueStory.jsp:20,24). CHK-005 (BA-001-05). Source: stage-02-pass-003 F-003. Request binding (BA-001-08, pass-006 F-001): with merge=true, EditObjectAction#populateObject calls org.apache.struts.util.RequestUtils.populate onto the story instead of copying the form and resolving its many-to-one references (bytecode listing), so any writable story property named by a parameter is set, including properties the editor does not show; together with the skipped checks, unvalidated values reach the saved story (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/forms/UserStoryEditorForm.java UserStoryEditorForm#validate; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject. WAR: classes byte-identical to the v1.1a4 release. The two validation branches are confirmed; which properties the binding sets is commons-beanutils behavior (GAP-011). Live question: Does a direct story-editor request with merge=true and an extra property parameter change that property? Stage 3 W001 (BA-001-13, MC-A-25, W001-F-28): B-C-069 (no fkey/projectId: HTTP 500), B-C-070 (with fkey/projectId and only iterationId: same-iteration message every time), B-C-071 (targetIterationId as the move page uses it). Status Inferred -&gt; Yes on this live observation. Stage 3 W001 live answer (BA-001-13, MC-C-18): Yes, when targetIterationId differs from the current iteration: priority 9, estimate -5.0 and the description were bound without validation; the story stayed in its iteration (B-C-069, B-C-070, B-C-071). The D/F correction is under W001-F-28. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks B-C-069, B-C-070, B-C-071).</t>
   </si>
   <si>
     <t>Edit user story</t>
   </si>
   <si>
-    <t>An editor can update a story's fields.</t>
+    <t>An editor can update a story's fields. Live (W001): disposition and status changes are not persisted, and the edit form pre-selects neither stored value.</t>
   </si>
   <si>
     <t>Refine stories as understanding grows.</t>
   </si>
   <si>
-    <t>Editor titled for the story with Update/Reset; changes saved.</t>
-  </si>
-  <si>
-    <t>class DomainMetaDataRepository#init (story edit -&gt; /do/edit/userstory, permission edit); WAR:WEB-INF/jsp/edit/editStory.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 121 applies to every /do/edit/userstory request (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
+    <t>Editor titled for the story with Update/Reset; changes saved, except the disposition and status, which stay Planned and Draft; the edit form pre-selects neither the stored disposition nor the stored status (W001).</t>
+  </si>
+  <si>
+    <t>class DomainMetaDataRepository#init (story edit -&gt; /do/edit/userstory, permission edit); WAR:WEB-INF/jsp/edit/editStory.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 121 applies to every /do/edit/userstory request (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Stage 3 W001 (BA-001-13, MC-A-24, W001-F-27): updates to defined/added (setup-C-047) and to implemented/planned (B-C-072): 302, the other fields saved, disposition and status unchanged. Status Yes -&gt; Partial (R-G2). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-047, B-C-072, B-C-073).</t>
   </si>
   <si>
     <t>Delete user story</t>
@@ -1660,7 +1660,7 @@
     <t>Confirm prompt; story, tasks and time entries removed (runtime unverified).</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (story delete -&gt; /do/delete/userstory, action.delete.confirmation); WAR:WEB-INF/struts-config.xml:285; WAR:WEB-INF/action-servlet.xml:256-260. Cascades: UserStory#getTasks, Task#getTimeEntries @OneToMany(cascade=REMOVE). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute; SRC:src/net/sf/xplanner/domain/UserStory.java UserStory#getTasks. WAR: classes byte-identical to the v1.1a4 release. The cascades match the source annotations.</t>
+    <t>class DomainMetaDataRepository#init (story delete -&gt; /do/delete/userstory, action.delete.confirmation); WAR:WEB-INF/struts-config.xml:285; WAR:WEB-INF/action-servlet.xml:256-260. Cascades: UserStory#getTasks, Task#getTimeEntries @OneToMany(cascade=REMOVE). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute; SRC:src/net/sf/xplanner/domain/UserStory.java UserStory#getTasks. WAR: classes byte-identical to the v1.1a4 release. The cascades match the source annotations. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks B-C-074, E-C-018; open residual scope R-40 (e)).</t>
   </si>
   <si>
     <t>View user story</t>
@@ -1675,7 +1675,7 @@
     <t>Story summary card and task table with action icons; "create task", export and history links.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:265-267; WAR:WEB-INF/jsp/view/userstory.jsp. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/struts-config.xml:265-267; WAR:WEB-INF/jsp/view/userstory.jsp. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-045, B-C-075).</t>
   </si>
   <si>
     <t>A story without tasks shows a "no tasks" message.</t>
@@ -1684,7 +1684,7 @@
     <t>Message story.no_tasks.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/userstory.jsp (story.no_tasks). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/jsp/view/userstory.jsp (story.no_tasks). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-046).</t>
   </si>
   <si>
     <t>Move or continue a story</t>
@@ -1699,19 +1699,19 @@
     <t>Move/Continue page with target iteration; story moved.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (movecontinue -&gt; /do/move/continue/userstory); WAR:WEB-INF/struts-config.xml:273-275; WAR:WEB-INF/jsp/edit/moveContinueStory.jsp; class MoveContinueStoryAction#saveForm ("Move"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); MoveContinueStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/moveContinueStory.jsp writes the raw request parameters fkey (25) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001): the Move/Continue page posts merge=true together with oid, iterationId, fkey, action and returnto (WAR:WEB-INF/jsp/edit/moveContinueStory.jsp:20-28); MoveContinueStoryAction#saveForm calls EditObjectAction#populateObject, which binds every request parameter onto the story with org.apache.struts.util.RequestUtils.populate before the move (bytecode listing; Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect (F-002): MoveContinueStoryAction#doExecute then redirects to the returnto request value unchanged (Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init; SRC:src/com/technoetic/xplanner/actions/MoveContinueStoryAction.java MoveContinueStoryAction#saveForm, #doExecute; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
-  </si>
-  <si>
-    <t>Continue creates a continuation of the story in the target iteration for the unfinished work, with cross-references in the descriptions.</t>
+    <t>class DomainMetaDataRepository#init (movecontinue -&gt; /do/move/continue/userstory); WAR:WEB-INF/struts-config.xml:273-275; WAR:WEB-INF/jsp/edit/moveContinueStory.jsp; class MoveContinueStoryAction#saveForm ("Move"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); MoveContinueStoryAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/moveContinueStory.jsp writes the raw request parameters fkey (25) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001): the Move/Continue page posts merge=true together with oid, iterationId, fkey, action and returnto (WAR:WEB-INF/jsp/edit/moveContinueStory.jsp:20-28); MoveContinueStoryAction#saveForm calls EditObjectAction#populateObject, which binds every request parameter onto the story with org.apache.struts.util.RequestUtils.populate before the move (bytecode listing; Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect (F-002): MoveContinueStoryAction#doExecute then redirects to the returnto request value unchanged (Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init; SRC:src/com/technoetic/xplanner/actions/MoveContinueStoryAction.java MoveContinueStoryAction#saveForm, #doExecute; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-076, B-C-077).</t>
+  </si>
+  <si>
+    <t>Continue creates a continuation of the story in the target iteration for the unfinished work, with cross-references in the descriptions. In this baseline Continue answers HTTP 500 (two open sessions) and creates no continuation; story Move works (W001).</t>
   </si>
   <si>
     <t>Carry over incomplete work while keeping history.</t>
   </si>
   <si>
-    <t>New continued story in target; descriptions reference the origin/continuation.</t>
-  </si>
-  <si>
-    <t>class MoveContinueStoryAction#saveForm ("Continue"); classes com.technoetic.xplanner.actions.StoryContinuer, TaskContinuer (strings continue.description.from/to); ResourceBundle.properties task.continued.to/from. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/Continuer.java Continuer#continueObject, #updateDescriptionAndHistory; SRC:src/com/technoetic/xplanner/actions/StoryContinuer.java StoryContinuer#doContinueObject. WAR: classes byte-identical to the v1.1a4 release. The continuation gets the remaining task-based hours, a disposition from the target iteration state and continuations of the unfinished tasks; both descriptions and the history receive the cross-references.</t>
+    <t>New continued story in target; descriptions reference the origin/continuation (source). Live (W001): Continue on the story Move/Continue page answers HTTP 500 and creates no continuation story; the original story is unchanged.</t>
+  </si>
+  <si>
+    <t>class MoveContinueStoryAction#saveForm ("Continue"); classes com.technoetic.xplanner.actions.StoryContinuer, TaskContinuer (strings continue.description.from/to); ResourceBundle.properties task.continued.to/from. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/Continuer.java Continuer#continueObject, #updateDescriptionAndHistory; SRC:src/com/technoetic/xplanner/actions/StoryContinuer.java StoryContinuer#doContinueObject. WAR: classes byte-identical to the v1.1a4 release. The continuation gets the remaining task-based hours, a disposition from the target iteration state and continuations of the unfinished tasks; both descriptions and the history receive the cross-references. Stage 3 W001 (BA-001-13, MC-A-21, W001-F-24): Continue on "S3-B S8 Continue" to S3-B I2 Next: POST 500, no continuation (B-C-078); the error page names HibernateException "Illegal attempt to associate a collection with two open sessions" (B-C-098). Status Yes -&gt; Partial (R-G2). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks B-C-078).</t>
   </si>
   <si>
     <t>Moving or continuing into the same iteration is rejected.</t>
@@ -1723,7 +1723,7 @@
     <t>Message "Cannot move or continue story in same iteration."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.MoveContinueStoryForm#validate (story.editor.same_iteration). The check runs on the merge branch of MoveContinueStoryForm#validate, which is the branch the move/continue page posts (row 132 covers the other branch). BA-001-05. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/MoveContinueStoryForm.java MoveContinueStoryForm#validate. WAR: classes byte-identical to the v1.1a4 release. With merge the target iteration must differ.</t>
+    <t>class com.technoetic.xplanner.forms.MoveContinueStoryForm#validate (story.editor.same_iteration). The check runs on the merge branch of MoveContinueStoryForm#validate, which is the branch the move/continue page posts (row 132 covers the other branch). BA-001-05. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/MoveContinueStoryForm.java MoveContinueStoryForm#validate. WAR: classes byte-identical to the v1.1a4 release. With merge the target iteration must differ. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-079).</t>
   </si>
   <si>
     <t>A move/continue story request without merge=true and without a name is rejected; the move/continue page always posts merge=true, so this applies to direct requests.</t>
@@ -1735,7 +1735,7 @@
     <t>Message "Missing story name." (runtime unverified).</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.MoveContinueStoryForm#validate (bytecode listing: #isMerge false -&gt; story.editor.missing_name; #isMerge true -&gt; story.editor.same_iteration); WAR:WEB-INF/jsp/edit/moveContinueStory.jsp:20,24 (form to /do/move/continue/userstory with hidden merge=true). CHK-005 (BA-001-05). Source: stage-02-pass-003 F-003. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/MoveContinueStoryForm.java MoveContinueStoryForm#validate. WAR: classes byte-identical to the v1.1a4 release. Without merge the name is required; with merge only the target iteration is checked.</t>
+    <t>class com.technoetic.xplanner.forms.MoveContinueStoryForm#validate (bytecode listing: #isMerge false -&gt; story.editor.missing_name; #isMerge true -&gt; story.editor.same_iteration); WAR:WEB-INF/jsp/edit/moveContinueStory.jsp:20,24 (form to /do/move/continue/userstory with hidden merge=true). CHK-005 (BA-001-05). Source: stage-02-pass-003 F-003. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/MoveContinueStoryForm.java MoveContinueStoryForm#validate. WAR: classes byte-identical to the v1.1a4 release. Without merge the name is required; with merge only the target iteration is checked. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-080).</t>
   </si>
   <si>
     <t>UF-008</t>
@@ -1747,16 +1747,16 @@
     <t>Create task</t>
   </si>
   <si>
-    <t>An editor can create a task under a story with name, type (feature, debt, defect, functional test, acceptance test, overhead), disposition, acceptor, estimated hours and description.</t>
+    <t>An editor can create a task under a story with name, type (feature, debt, defect, functional test, acceptance test, overhead), disposition, acceptor, estimated hours and description. Live (W001): the disposition chosen in the editor is not stored on create.</t>
   </si>
   <si>
     <t>Break stories into assignable work.</t>
   </si>
   <si>
-    <t>Task saved; user returned to the story.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/userstory.jsp (link /do/edit/task, story.link.create_task); WAR:WEB-INF/struts-config.xml:291; WAR:WEB-INF/action-servlet.xml:268-272 (EditTaskAction); WAR:WEB-INF/jsp/edit/editTask.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editTask.jsp writes the raw request parameters oid (31), returnto (34), fkey (36,37) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/task that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Task object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). EditTaskAction#populateObject calls the parent method. With merge=true the task validator skips its name and estimate checks (row 137). The complete and reopen buttons of the task page post merge=true (rows 140-141); any other parameter added to such a request is bound as well (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute (reached from EditTaskAction#doExecute) redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/actions/EditTaskAction.java EditTaskAction#populateObject, #doExecute; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject, #doExecute. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
+    <t>Task saved; user returned to the story. The disposition chosen in the editor is not stored on create: a task created with the pre-selected "discovered" is shown as "Planned" (W001).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/userstory.jsp (link /do/edit/task, story.link.create_task); WAR:WEB-INF/struts-config.xml:291; WAR:WEB-INF/action-servlet.xml:268-272 (EditTaskAction); WAR:WEB-INF/jsp/edit/editTask.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editTask.jsp writes the raw request parameters oid (31), returnto (34), fkey (36,37) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/task that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Task object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). EditTaskAction#populateObject calls the parent method. With merge=true the task validator skips its name and estimate checks (row 137). The complete and reopen buttons of the task page post merge=true (rows 140-141); any other parameter added to such a request is bound as well (Inferred; observed risk only, Q3 deferred; Q3 facts). Redirect target (BA-001-08, pass-006 F-002, check (e)): EditObjectAction#doExecute (reached from EditTaskAction#doExecute) redirects to the returnto request value unchanged (new ActionForward(returnto, true)); only a missing value selects a mapping forward instead, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/actions/EditTaskAction.java EditTaskAction#populateObject, #doExecute; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject, #doExecute. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Stage 3 W001 (BA-001-13, MC-A-26, W001-F-29): setup-C-049 and B-C-081 (pre-selected disposition submitted, task shown as Planned). Status Yes -&gt; Partial (R-G2). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-048, setup-C-049, B-C-081, B-C-082).</t>
   </si>
   <si>
     <t>The task type is stored as a message label, not a code: the type options carry label text as their values, resolved without the user's locale, so the stored value follows the server default locale. The labels differ between bundles.</t>
@@ -1768,10 +1768,10 @@
     <t>Type select shows the user's language; the stored value is the server-default-locale label (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editTask.jsp:52-69 (html:option value=messages.getMessage("task.type.feature") ... "task.type.overhead", no locale argument); class net.sf.xplanner.struts.XPlannerMessageResources#getMessage delegates to the Spring MessageSource (null locale falls back to the JVM default, framework behavior, GAP-011). Per bundle (CHK-004, .migration-tmp/stage-01/out/task-type-labels.json): the default and "--" bundles use Feature, Defect, Debt, FTest, ATest, Overhead; da, de, es, fr, it, ja and ru differ from the default for at least one type; pt_br matches except that it has no overhead key; da, es, fr and pt_br define no task.type.overhead (fallback to the default). Corrected in BA-001-04 (Source: stage-02-pass-002 F-009). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/net/sf/xplanner/struts/XPlannerMessageResources.java XPlannerMessageResources#getMessage. WAR: classes byte-identical to the v1.1a4 release; editTask.jsp identical to the SVN webapp copy. The page asks for the label without a locale; the stored value then follows the Spring message source and the JVM default locale (framework behavior). Live question: Which type value is stored for a task created in a de session on a server whose default locale is English?</t>
-  </si>
-  <si>
-    <t>The default disposition of a new task is "discovered" when its story is started or its iteration is active, and "planned" otherwise.</t>
+    <t>WAR:WEB-INF/jsp/edit/editTask.jsp:52-69 (html:option value=messages.getMessage("task.type.feature") ... "task.type.overhead", no locale argument); class net.sf.xplanner.struts.XPlannerMessageResources#getMessage delegates to the Spring MessageSource (null locale falls back to the JVM default, framework behavior, GAP-011). Per bundle (CHK-004, .migration-tmp/stage-01/out/task-type-labels.json): the default and "--" bundles use Feature, Defect, Debt, FTest, ATest, Overhead; da, de, es, fr, it, ja and ru differ from the default for at least one type; pt_br matches except that it has no overhead key; da, es, fr and pt_br define no task.type.overhead (fallback to the default). Corrected in BA-001-04 (Source: stage-02-pass-002 F-009). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/net/sf/xplanner/struts/XPlannerMessageResources.java XPlannerMessageResources#getMessage. WAR: classes byte-identical to the v1.1a4 release; editTask.jsp identical to the SVN webapp copy. The page asks for the label without a locale; the stored value then follows the Spring message source and the JVM default locale (framework behavior). Live question: Which type value is stored for a task created in a de session on a server whose default locale is English? Stage 3 W001 live answer (BA-001-13, MC-C-19): The English label "Debt" is stored for the option shown as "Rückstand" (B-C-083). Status Inferred -&gt; Yes on this live observation (server default locale English). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-050, B-C-083).</t>
+  </si>
+  <si>
+    <t>The disposition pre-selected in the editor for a new task is "discovered" when its story is started or its iteration is active, and "planned" otherwise; the chosen value is not stored on create (row 134, W001).</t>
   </si>
   <si>
     <t>Distinguishes planned from added/discovered work.</t>
@@ -1780,16 +1780,16 @@
     <t>Disposition pre-selected.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.actions.EditTaskAction#setTaskDisposition/#getTaskDisposition (UserStory, Iteration). Rule not decompiled. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/EditTaskAction.java EditTaskAction#setTaskDisposition, #getTaskDisposition; SRC:src/net/sf/xplanner/domain/Iteration.java Iteration#getNewTaskDisposition. WAR: classes byte-identical to the v1.1a4 release. The rule is now visible: for a new task (no oid, form not submitted) the disposition is "discovered" when the story is started or the iteration is active, otherwise "planned".</t>
-  </si>
-  <si>
-    <t>A missing name, a negative estimate or an invalid created date is rejected.</t>
-  </si>
-  <si>
-    <t>Messages "Missing task name.", "Please provide an estimate greater than or equal to zero.", "Created date is invalid."</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.forms.TaskEditorForm#validate (task.editor.missing_name, negative_estimated_hours, bad_created_date). Merge branch (CHK-005, BA-001-05): TaskEditorForm#validate checks the created date first and skips the name and estimate checks when merge=true, which the complete and reopen buttons post (WAR:WEB-INF/jsp/view/task.jsp:76-79,87-90). Request binding (BA-001-08, pass-006 F-001): the same merge=true requests are bound onto the task by EditObjectAction#populateObject with org.apache.struts.util.RequestUtils.populate instead of the form copy (EditTaskAction#populateObject calls the parent), so the skipped name and estimate checks leave any task property named by a parameter unvalidated (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/TaskEditorForm.java TaskEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release. A given created date must parse; without merge the name and a non-negative estimate are required.</t>
+    <t>class com.technoetic.xplanner.actions.EditTaskAction#setTaskDisposition/#getTaskDisposition (UserStory, Iteration). Rule not decompiled. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/EditTaskAction.java EditTaskAction#setTaskDisposition, #getTaskDisposition; SRC:src/net/sf/xplanner/domain/Iteration.java Iteration#getNewTaskDisposition. WAR: classes byte-identical to the v1.1a4 release. The rule is now visible: for a new task (no oid, form not submitted) the disposition is "discovered" when the story is started or the iteration is active, otherwise "planned". Stage 3 W001 (BA-001-13, MC-A-26, W001-F-29): the pre-selection follows this rule in both branches (B-C-084); the requirement is limited to the pre-selection because the stored disposition differs (row 134). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-051, B-C-084).</t>
+  </si>
+  <si>
+    <t>A missing name, a negative estimate or an invalid created date is rejected. The task editor has no created-date field, so the created-date check applies only to a createdDateString parameter added to a direct request (W001).</t>
+  </si>
+  <si>
+    <t>Messages "Missing task name.", "Please provide an estimate greater than or equal to zero." and, for a direct createdDateString parameter only, "Created date is invalid."</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.TaskEditorForm#validate (task.editor.missing_name, negative_estimated_hours, bad_created_date). Merge branch (CHK-005, BA-001-05): TaskEditorForm#validate checks the created date first and skips the name and estimate checks when merge=true, which the complete and reopen buttons post (WAR:WEB-INF/jsp/view/task.jsp:76-79,87-90). Request binding (BA-001-08, pass-006 F-001): the same merge=true requests are bound onto the task by EditObjectAction#populateObject with org.apache.struts.util.RequestUtils.populate instead of the form copy (EditTaskAction#populateObject calls the parent), so the skipped name and estimate checks leave any task property named by a parameter unvalidated (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/TaskEditorForm.java TaskEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release. A given created date must parse; without merge the name and a non-negative estimate are required. Stage 3 W001 (BA-001-13, MC-A-27, W001-F-30): the three messages were shown; the Define/Edit Task form has no created-date field (B-C-085). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks B-C-085).</t>
   </si>
   <si>
     <t>Task e-mail notification</t>
@@ -1801,10 +1801,10 @@
     <t>Keeps assignees informed.</t>
   </si>
   <si>
-    <t>E-mail "Task was created." or "Task was updated." to the editor and, when the task has an acceptor, to the acceptor, with task and assignee details; the old-assignee value is taken from the new acceptor, so after a reassignment it shows the new assignee (runtime unverified).</t>
-  </si>
-  <si>
-    <t>class EditTaskAction#sendNotification (templates com/technoetic/xplanner/mail/velocity/email_notification_task_created.vm and ..._updated.vm; EmailNotificationSupport.compileEmail/sendNotifications); WAR:WEB-INF/classes/EmailResourceBundle.properties task.created.*, task.updated.*; recipients not determinable statically. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/actions/EditTaskAction.java EditTaskAction#sendNotification; SRC:src/com/technoetic/xplanner/mail/EmailNotificationSupport.java EmailNotificationSupport#compileEmail. WAR: classes byte-identical to the v1.1a4 release. The recipients are determinable: mail is compiled only after a redirecting save by a signed-in user, for the editor and, when the task has an acceptor, for the acceptor. The "old assignee" is always derived from the new acceptor id (bytecode listing agrees), so it names the new assignee whenever one is set. Delivery depends on SMTP. Live question: Are the created and updated mails delivered to the editor and the acceptor, and which old assignee does an updated mail show after a reassignment?</t>
+    <t>E-mail "Task was created." or "Task was updated.", one per recipient, to the saving user and, when the task has an acceptor, to the current acceptor (one mail when they are the same person); the story tracker and a previous acceptor are not notified; the "creator:" line shows the saving user, also on updates; the task link is built from xplanner.application.url (http://localhost:8080/xplanner/do/view/task?oid=&lt;id&gt;); the old-assignee value is taken from the new acceptor, so after a reassignment "Assigned to" shows the new assignee in both columns (W001, adapted mail environment). Sending depends on fetching xplanner.application.url + /css/email.css (row 202, GAP-008): when the fetch fails, as in the original deployment condition of W001, no mail is sent, the error is only logged and the task change is still saved.</t>
+  </si>
+  <si>
+    <t>class EditTaskAction#sendNotification (templates com/technoetic/xplanner/mail/velocity/email_notification_task_created.vm and ..._updated.vm; EmailNotificationSupport.compileEmail/sendNotifications); WAR:WEB-INF/classes/EmailResourceBundle.properties task.created.*, task.updated.*; recipients not determinable statically. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/actions/EditTaskAction.java EditTaskAction#sendNotification; SRC:src/com/technoetic/xplanner/mail/EmailNotificationSupport.java EmailNotificationSupport#compileEmail. WAR: classes byte-identical to the v1.1a4 release. The recipients are determinable: mail is compiled only after a redirecting save by a signed-in user, for the editor and, when the task has an acceptor, for the acceptor. The "old assignee" is always derived from the new acceptor id (bytecode listing agrees), so it names the new assignee whenever one is set. Delivery depends on SMTP. Live question: Are the created and updated mails delivered to the editor and the acceptor, and which old assignee does an updated mail show after a reassignment? Stage 3 W001 (BA-001-13, MC-B-04, W001-F-31): original deployment condition (before 20:03:44Z): each task notification failed while fetching http://localhost:8080/xplanner/css/email.css (FileNotFoundException, logged as "Error sending email"), no mail reached the sink, and the task create and update themselves succeeded (setup-C-059, part setup blocked, reclassified as observed; B-C-086). The cause is the configured application URL (/xplanner) versus the deployed context path (/xplanner-legacy), a property of this deployment (GAP-008; Data And Integrations, outbound HTTP row; row 202). Stage 3 W001 (BA-001-13, MC-B-05, W001-F-32): adapted mail environment (static email.css): four task actions with the recipients and texts above (B-C-087). Status stays Inferred: delivery depends on the deployment's application URL, and the mapped mails were observed only in the adapted environment. Stage 3 W001 live answer (BA-001-13, MC-C-20): Original deployment condition: no mail (email.css fetch fails). Adapted environment: one mail each to the saving user and the current acceptor; after a reassignment "Assigned to" shows the new assignee in both columns (setup-C-059, B-C-086, B-C-087). The D/F correction is under W001-F-31. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-059, B-C-086, B-C-087).</t>
   </si>
   <si>
     <t>Edit task</t>
@@ -1819,7 +1819,7 @@
     <t>Task editor with Update/Reset; changes saved.</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (task edit -&gt; /do/edit/task); WAR:WEB-INF/jsp/edit/editTask.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 134 applies to every /do/edit/task request (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
+    <t>class DomainMetaDataRepository#init (task edit -&gt; /do/edit/task); WAR:WEB-INF/jsp/edit/editTask.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 134 applies to every /do/edit/task request (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-088, B-C-089).</t>
   </si>
   <si>
     <t>Complete or reopen task</t>
@@ -1831,10 +1831,10 @@
     <t>Signal work is done.</t>
   </si>
   <si>
-    <t>"Complete" button; task becomes completed; page reloads.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/task.jsp:86-95 (form /do/edit/task, action Update, merge true, completed true). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Mechanism (BA-001-08, pass-006 F-001): the completion takes effect through the merge=true binding, not through the task form: EditObjectAction#populateObject calls org.apache.struts.util.RequestUtils.populate, which sets Task#setCompleted from the posted completed=true (WAR:WEB-INF/jsp/view/task.jsp:87-94); any further parameter added to the request is bound onto the task as well (Inferred; Q3 facts). After the save, EditObjectAction#doExecute redirects to the posted returnto value (F-002). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject, #doExecute; SRC:src/net/sf/xplanner/domain/Task.java Task#setCompleted. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
+    <t>"Complete Task" button; its form posts oid, action=Update, merge=true and completed=true to /do/edit/task (the generic-editor merge binding, Q3 facts; compare row 124); task becomes completed; page reloads.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/task.jsp:86-95 (form /do/edit/task, action Update, merge true, completed true). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Mechanism (BA-001-08, pass-006 F-001): the completion takes effect through the merge=true binding, not through the task form: EditObjectAction#populateObject calls org.apache.struts.util.RequestUtils.populate, which sets Task#setCompleted from the posted completed=true (WAR:WEB-INF/jsp/view/task.jsp:87-94); any further parameter added to the request is bound onto the task as well (Inferred; Q3 facts). After the save, EditObjectAction#doExecute redirects to the posted returnto value (F-002). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject, #doExecute; SRC:src/net/sf/xplanner/domain/Task.java Task#setCompleted. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Stage 3 W001 (BA-001-13, MC-A-28, W001-F-33): setup-C-053 and B-C-090 (button "Complete Task", fields oid, action=Update, merge=true, returnto, completed=true; 302 to the task page). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-053, B-C-090, B-C-091).</t>
   </si>
   <si>
     <t>A completed task can be reopened.</t>
@@ -1843,10 +1843,10 @@
     <t>Correct premature completion.</t>
   </si>
   <si>
-    <t>"Reopen" button; task becomes open again.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/task.jsp:75-84 (completed false). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Mechanism (BA-001-08, pass-006 F-001): the reopen form posts merge=true and completed=false (WAR:WEB-INF/jsp/view/task.jsp:76-83), so the change is made by the same RequestUtils.populate binding as in row 140 (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>"Reopen Task" button (form with merge=true and completed=false); task becomes open again.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/task.jsp:75-84 (completed false). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditTaskAction performs no server-side permission check that gates the change (the only authorization call on the EditTaskAction path is the recipient lookup inside the e-mail notification), so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Mechanism (BA-001-08, pass-006 F-001): the reopen form posts merge=true and completed=false (WAR:WEB-INF/jsp/view/task.jsp:76-83), so the change is made by the same RequestUtils.populate binding as in row 140 (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Stage 3 W001 (BA-001-13, MC-A-28, W001-F-33): setup-C-054 and B-C-092 (button "Reopen Task", completed=false; shown to editor, admin and system administrator, not to the viewer). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-054, B-C-092, B-C-093).</t>
   </si>
   <si>
     <t>Delete task</t>
@@ -1861,7 +1861,7 @@
     <t>Confirm prompt; task and its time entries removed (runtime unverified).</t>
   </si>
   <si>
-    <t>class DomainMetaDataRepository#init (task delete -&gt; /do/delete/task, action.delete.confirmation); WAR:WEB-INF/struts-config.xml:304; WAR:WEB-INF/action-servlet.xml:300-304. Cascade: Task#getTimeEntries @OneToMany(cascade=REMOVE). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute; SRC:src/net/sf/xplanner/domain/Task.java Task#getTimeEntries. WAR: classes byte-identical to the v1.1a4 release. The cascade matches the source annotation.</t>
+    <t>class DomainMetaDataRepository#init (task delete -&gt; /do/delete/task, action.delete.confirmation); WAR:WEB-INF/struts-config.xml:304; WAR:WEB-INF/action-servlet.xml:300-304. Cascade: Task#getTimeEntries @OneToMany(cascade=REMOVE). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteObjectAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Corrected in BA-001-04 (Source: stage-02-pass-002 F-002). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DeleteObjectAction.java DeleteObjectAction#doExecute; SRC:src/net/sf/xplanner/domain/Task.java Task#getTimeEntries. WAR: classes byte-identical to the v1.1a4 release. The cascade matches the source annotation. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks B-C-094, B-C-095).</t>
   </si>
   <si>
     <t>View task</t>
@@ -1876,22 +1876,22 @@
     <t>Task card and time-log table; action links (edit, delete, move/continue, time) by permission; export and history links.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:287-289; WAR:WEB-INF/jsp/view/task.jsp. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/struts-config.xml:287-289; WAR:WEB-INF/jsp/view/task.jsp. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks setup-C-052, B-C-096).</t>
   </si>
   <si>
     <t>Move or continue a task</t>
   </si>
   <si>
-    <t>An editor can move a task to another story.</t>
+    <t>An editor can move a task to another story. In this baseline every move/continue task submission answers HTTP 500 and nothing is moved (W001).</t>
   </si>
   <si>
     <t>Re-assign work to the right story.</t>
   </si>
   <si>
-    <t>Move/Continue page with target story; history records "moved".</t>
-  </si>
-  <si>
-    <t>class DomainMetaDataRepository#init (task movecontinue -&gt; /do/move/continue/task); WAR:WEB-INF/struts-config.xml:293-295; WAR:WEB-INF/jsp/edit/moveContinueTask.jsp; class MoveContinueTaskAction#saveForm ("Move", "task.moved.from.to", "moved out", "moved in"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); MoveContinueTaskAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/moveContinueTask.jsp writes the raw request parameters fkey (25) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init; SRC:src/com/technoetic/xplanner/actions/MoveContinueTaskAction.java MoveContinueTaskAction#saveForm. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
+    <t>Move/Continue page with target story, listing the stories of all projects the user can see (14 options across five projects in W001; first option pre-selected); history records "moved" (source). Live (W001): every POST to /do/move/continue/task answers HTTP 500 (IllegalStateException "No Hibernate Session bound to thread") before validation: the task stays in its story, no history row is written and no message is shown; the GET page renders.</t>
+  </si>
+  <si>
+    <t>class DomainMetaDataRepository#init (task movecontinue -&gt; /do/move/continue/task); WAR:WEB-INF/struts-config.xml:293-295; WAR:WEB-INF/jsp/edit/moveContinueTask.jsp; class MoveContinueTaskAction#saveForm ("Move", "task.moved.from.to", "moved out", "moved in"). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); MoveContinueTaskAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/moveContinueTask.jsp writes the raw request parameters fkey (25) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/domain/DomainMetaDataRepository.java DomainMetaDataRepository#init; SRC:src/com/technoetic/xplanner/actions/MoveContinueTaskAction.java MoveContinueTaskAction#saveForm. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Stage 3 W001 (BA-001-13, MC-A-29, MC-B-03, W001-F-22, W001-F-34): Move to another story, with and without projectId: HTTP 500, task unchanged, history empty (B-C-097, B-C-098); target options from five projects (B-C-099). Whether a user without a role on a project also sees its stories was not tested. Status Yes -&gt; Partial (R-G2). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks B-C-097, B-C-098, B-C-099).</t>
   </si>
   <si>
     <t>Continue copies the unfinished task into the target story with cross-referenced descriptions.</t>
@@ -1900,19 +1900,19 @@
     <t>Carry over remaining effort.</t>
   </si>
   <si>
-    <t>New task "Continued from task:&lt;id&gt;".</t>
-  </si>
-  <si>
-    <t>class MoveContinueTaskAction#saveForm ("Continue"); class TaskContinuer; ResourceBundle.properties task.continued.to/from. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/TaskContinuer.java TaskContinuer#doContinueObject; SRC:src/com/technoetic/xplanner/actions/Continuer.java Continuer#continueObject, #updateDescriptionAndHistory. WAR: classes byte-identical to the v1.1a4 release. The continued task gets the remaining hours as its estimate, no acceptor and no time entries, and the original task is postponed; descriptions and history receive the cross-references.</t>
+    <t>New task "Continued from task:&lt;id&gt;" (source). Live (W001): Continue answers HTTP 500; no task is created and the original is unchanged.</t>
+  </si>
+  <si>
+    <t>class MoveContinueTaskAction#saveForm ("Continue"); class TaskContinuer; ResourceBundle.properties task.continued.to/from. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/TaskContinuer.java TaskContinuer#doContinueObject; SRC:src/com/technoetic/xplanner/actions/Continuer.java Continuer#continueObject, #updateDescriptionAndHistory. WAR: classes byte-identical to the v1.1a4 release. The continued task gets the remaining hours as its estimate, no acceptor and no time entries, and the original task is postponed; descriptions and history receive the cross-references. Stage 3 W001 (BA-001-13, MC-A-29, W001-F-34): Continue of T1 to S2 Beta: POST 500, no new task (B-C-100). Status Yes -&gt; Partial (R-G2). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks B-C-100).</t>
   </si>
   <si>
     <t>Moving or continuing into the same story is rejected.</t>
   </si>
   <si>
-    <t>Validation message task.editor.same_story.</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.forms.MoveContinueTaskForm#validate (merge branch: task.editor.same_story; the non-merge branch task.editor.missing_name is row 147). Wording corrected in BA-001-05 (Source: stage-02-pass-003 F-003). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/MoveContinueTaskForm.java MoveContinueTaskForm#validate. WAR: classes byte-identical to the v1.1a4 release. With merge the target story must differ.</t>
+    <t>Validation message task.editor.same_story (source; the key has no text in the default bundle, part B static note). Live (W001): a same-story Move answers HTTP 500 before validation, so no message is shown.</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.MoveContinueTaskForm#validate (merge branch: task.editor.same_story; the non-merge branch task.editor.missing_name is row 147). Wording corrected in BA-001-05 (Source: stage-02-pass-003 F-003). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/MoveContinueTaskForm.java MoveContinueTaskForm#validate. WAR: classes byte-identical to the v1.1a4 release. With merge the target story must differ. Stage 3 W001 (BA-001-13, MC-A-29, W001-F-34): Move of T1 to its own story: POST 500, no message (B-C-101). Status Yes -&gt; Partial (R-G2). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks B-C-101).</t>
   </si>
   <si>
     <t>A move/continue task request without merge=true and without a name is rejected; the move/continue page always posts merge=true, so this applies to direct requests.</t>
@@ -1921,10 +1921,10 @@
     <t>Documents the non-merge branch of the task move/continue form.</t>
   </si>
   <si>
-    <t>Message "Missing task name." (runtime unverified).</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.forms.MoveContinueTaskForm#validate (bytecode listing: #isMerge false -&gt; task.editor.missing_name; #isMerge true -&gt; task.editor.same_story); WAR:WEB-INF/jsp/edit/moveContinueTask.jsp:21,24 (form to /do/move/continue/task with hidden merge=true). CHK-005 (BA-001-05), wording point of pass-003 F-003. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/MoveContinueTaskForm.java MoveContinueTaskForm#validate. WAR: classes byte-identical to the v1.1a4 release. Without merge the name is required; with merge only the target story is checked.</t>
+    <t>Message "Missing task name." (source). Live (W001): the direct request answers HTTP 500; the message is not shown and the task stays in its story.</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.MoveContinueTaskForm#validate (bytecode listing: #isMerge false -&gt; task.editor.missing_name; #isMerge true -&gt; task.editor.same_story); WAR:WEB-INF/jsp/edit/moveContinueTask.jsp:21,24 (form to /do/move/continue/task with hidden merge=true). CHK-005 (BA-001-05), wording point of pass-003 F-003. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/MoveContinueTaskForm.java MoveContinueTaskForm#validate. WAR: classes byte-identical to the v1.1a4 release. Without merge the name is required; with merge only the target story is checked. Stage 3 W001 (BA-001-13, MC-A-29, W001-F-34): POST without merge and without name: 500, message not shown (B-C-102). Status Yes -&gt; Partial (R-G2). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks B-C-102).</t>
   </si>
   <si>
     <t>UF-009</t>
@@ -1942,10 +1942,10 @@
     <t>Track actual effort, including pair programming.</t>
   </si>
   <si>
-    <t>Time grid with an empty new row; "Insert Time" fills current time; Update saves; redirect to the task page.</t>
-  </si>
-  <si>
-    <t>class DomainMetaDataRepository#init (edittime -&gt; /do/edit/time); WAR:WEB-INF/struts-config.xml:350-355; WAR:WEB-INF/action-servlet.xml:376-378 (UpdateTimeAction); WAR:WEB-INF/jsp/edit/editTimeEntries.jsp; WAR:editTimeEntries.js; WAR:time.js. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); UpdateTimeAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editTimeEntries.jsp writes the raw request parameters oid (59), returnto (61), fkey (63,64) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Redirect target (BA-001-08, pass-006 F-002, check (e)): UpdateTimeAction#doUpdateTimeAction (and #doUpdateEstimateAction for the estimate action) redirects to the returnto value posted by the time editor, unchanged (new ActionForward(returnto, true)); there is no fallback for a missing value, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#doUpdateTimeAction. WAR: classes byte-identical to the v1.1a4 release. New rows with a start time or a duration are saved, existing rows are edited or deleted, and the browser is redirected to returnto.</t>
+    <t>Time grid with an empty new row; "Insert Time" fills current time; Update saves; redirect to the task page. In es sessions the time editor uses the Spanish date-time pattern (row 70): an entry typed as the hint reads fails at save with HTTP 500 and an entry shaped like the Insert Time output loses its minutes (W001); en and de round trips are unchanged.</t>
+  </si>
+  <si>
+    <t>class DomainMetaDataRepository#init (edittime -&gt; /do/edit/time); WAR:WEB-INF/struts-config.xml:350-355; WAR:WEB-INF/action-servlet.xml:376-378 (UpdateTimeAction); WAR:WEB-INF/jsp/edit/editTimeEntries.jsp; WAR:editTimeEntries.js; WAR:time.js. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); UpdateTimeAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editTimeEntries.jsp writes the raw request parameters oid (59), returnto (61), fkey (63,64) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Redirect target (BA-001-08, pass-006 F-002, check (e)): UpdateTimeAction#doUpdateTimeAction (and #doUpdateEstimateAction for the estimate action) redirects to the returnto value posted by the time editor, unchanged (new ActionForward(returnto, true)); there is no fallback for a missing value, and the value is not validated (bytecode listing). The bundled Struts RequestProcessor#processForwardConfig adds the context path only to values that start with "/", so an absolute URL in returnto sends the browser to another host after the action completes (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#doUpdateTimeAction. WAR: classes byte-identical to the v1.1a4 release. New rows with a start time or a duration are saved, existing rows are edited or deleted, and the browser is redirected to returnto. Stage 3 W001 (BA-001-13, MC-A-16, W001-F-18): C-C-003, E-C-033; en and de saves and an unchanged resubmit kept dates and durations (C-C-003). The es defect is recorded as a locale exception (row 70); the editor itself was observed working in en and de (setup-C-055, C-C-006, E-C-032), so the status is unchanged. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-055, C-C-003, C-C-006, C-C-007, C-C-008, E-C-032, E-C-033, F-C-013; open residual scope R-26 (d)).</t>
   </si>
   <si>
     <t>Existing entries can be edited or marked for deletion in the same grid.</t>
@@ -1957,7 +1957,7 @@
     <t>Delete checkbox per row; changes saved on Update.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/edit/editTimeEntries.jsp (deleted[row] checkbox). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/jsp/edit/editTimeEntries.jsp (deleted[row] checkbox). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-009).</t>
   </si>
   <si>
     <t>The remaining-hours field recalculates as durations change and updates the task estimate on save.</t>
@@ -1966,19 +1966,19 @@
     <t>Keeps remaining effort current.</t>
   </si>
   <si>
-    <t>Remaining hours shown (red when negative); task estimate updated.</t>
-  </si>
-  <si>
-    <t>WAR:editTimeEntries.js:9-19,65-67 (remainingHours recalculation); class UpdateTimeAction#doUpdateTimeAction (TimeEditorForm.getRemainingHours, Task.setEstimatedHours). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#doUpdateTimeAction. WAR: classes byte-identical to the v1.1a4 release; editTimeEntries.js identical to the SVN webapp copy. On save, when the remaining hours are given and not negative, the task estimate becomes the effort of the form's entries plus the remaining hours.</t>
+    <t>Remaining hours recalculated when the start, end or duration of an entry changes or an entry is deleted (Insert Time alone does not trigger it); a negative result is shown as 0 and the "remaining hours" label turns red; task estimate updated on save (W001).</t>
+  </si>
+  <si>
+    <t>WAR:editTimeEntries.js:9-19,65-67 (remainingHours recalculation); class UpdateTimeAction#doUpdateTimeAction (TimeEditorForm.getRemainingHours, Task.setEstimatedHours). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#doUpdateTimeAction. WAR: classes byte-identical to the v1.1a4 release; editTimeEntries.js identical to the SVN webapp copy. On save, when the remaining hours are given and not negative, the task estimate becomes the effort of the form's entries plus the remaining hours. Stage 3 W001 (BA-001-13, MC-A-30, W001-F-35): durations 1, 3 and 1 typed in the new row: 1.5 -&gt; 0.5, then 0 with the label remainingHoursLabel red, then 0.5 (E-C-034); the estimate update on save (E-C-035). Part E named column G; the expected result is column F. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-056, C-C-010, E-C-034, E-C-035).</t>
   </si>
   <si>
     <t>Unparsable date/time or number input in a time entry row is rejected.</t>
   </si>
   <si>
-    <t>Time editor redisplayed with "Can't parse the supplied date/time value." or "Can't parse the supplied number." (forward "error").</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.unparsable_time, edittime.error.unparsable_number; WAR:WEB-INF/classes/ResourceBundle.properties:675-676; WAR:WEB-INF/struts-config.xml:353-354 (error -&gt; editTimeEntries.jsp). Corrected in BA-001-04 (Source: stage-02-pass-002 F-001; the validator is the form, not UpdateTimeAction). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.unparsable_time: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). edittime.error.unparsable_number is missing in es and fr. Bundles without the key fall back to the default text (framework behavior, GAP-011). The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#valideRow. WAR: classes byte-identical to the v1.1a4 release. Start, end and report date are converted with the unparsable-time key and the duration with the unparsable-number key, as recorded.</t>
+    <t>Time editor redisplayed with "Can't parse the supplied date/time value." or "Can't parse the supplied number." (forward "error"). In es sessions a value that the session pattern cannot parse passes the TimeEditorForm validation (server default locale patterns, row 89) and then fails in UpdateTimeAction with HTTP 500 instead of showing a message (W001).</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.unparsable_time, edittime.error.unparsable_number; WAR:WEB-INF/classes/ResourceBundle.properties:675-676; WAR:WEB-INF/struts-config.xml:353-354 (error -&gt; editTimeEntries.jsp). Corrected in BA-001-04 (Source: stage-02-pass-002 F-001; the validator is the form, not UpdateTimeAction). Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.unparsable_time: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). edittime.error.unparsable_number is missing in es and fr. Bundles without the key fall back to the default text (framework behavior, GAP-011). The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#valideRow. WAR: classes byte-identical to the v1.1a4 release. Start, end and report date are converted with the unparsable-time key and the duration with the unparsable-number key, as recorded. Stage 3 W001 (BA-001-13, MC-A-16, W001-F-18): es: "30-09-2026 12:00" passed validation and failed with java.text.ParseException at UpdateTimeAction.doUpdateTimeAction(UpdateTimeAction.java:145) (C-C-003). In en the unparsable start "not-a-date" and the duration "abc" redisplay the editor with the message (C-C-011, C-C-012), so the status is unchanged. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks C-C-003, C-C-011, C-C-012).</t>
   </si>
   <si>
     <t>A time entry row other than the last one that lacks a start or an end time and has no duration is rejected, as is any row with an end time and a duration but no start time; in the last row a start time alone is accepted.</t>
@@ -1990,7 +1990,7 @@
     <t>Message "Missing start or end time."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.missing_time; WAR:WEB-INF/classes/ResourceBundle.properties:677. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.missing_time: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. The missing-time check (#1) applies to every row except the last one: a row that lacks a start or an end time and has no duration is rejected; a row with an end time, no start time and a duration is also rejected (#6). In the last row a start time without end time or duration is not rejected and is saved as an entry without end time (UpdateTimeAction#doUpdateTimeAction saves a new row when it has a start time or a duration).</t>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.missing_time; WAR:WEB-INF/classes/ResourceBundle.properties:677. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.missing_time: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. The missing-time check (#1) applies to every row except the last one: a row that lacks a start or an end time and has no duration is rejected; a row with an end time, no start time and a duration is also rejected (#6). In the last row a start time without end time or duration is not rejected and is saved as an entry without end time (UpdateTimeAction#doUpdateTimeAction saves a new row when it has a start time or a duration). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-013).</t>
   </si>
   <si>
     <t>A time entry row without any person is rejected.</t>
@@ -2002,7 +2002,7 @@
     <t>Message "No person is specified in a time entry."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.missing_person; ResourceBundle.properties:678. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.missing_person: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. A row that has an id, a start or end time, or a positive duration, but neither person, is rejected with the missing-person key.</t>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.missing_person; ResourceBundle.properties:678. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.missing_person: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. A row that has an id, a start or end time, or a positive duration, but neither person, is rejected with the missing-person key. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-014).</t>
   </si>
   <si>
     <t>A time entry row with a start time that names the same person as both pair members is rejected; a duration-only row is not checked.</t>
@@ -2014,7 +2014,7 @@
     <t>Message "Must specify different people for time entry."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.same_people; ResourceBundle.properties:681. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.same_people: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. The same-people check runs only when a person is present and the row has a start time: a duration-only row with the same person twice is not rejected.</t>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.same_people; ResourceBundle.properties:681. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.same_people: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. The same-people check runs only when a person is present and the row has a start time: a duration-only row with the same person twice is not rejected. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-015).</t>
   </si>
   <si>
     <t>A time entry row whose end is not after its start is rejected.</t>
@@ -2026,7 +2026,7 @@
     <t>Message "Negative or zero-length intervals are not allowed."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.negative_interval; ResourceBundle.properties:679. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.negative_interval: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. When start and end are both present and the end is not after the start, the negative-interval key is raised.</t>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.negative_interval; ResourceBundle.properties:679. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.negative_interval: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. When start and end are both present and the end is not after the start, the negative-interval key is raised. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-016).</t>
   </si>
   <si>
     <t>Time entry rows whose intervals overlap are rejected.</t>
@@ -2038,7 +2038,7 @@
     <t>Message "Overlapping intervals are not allowed."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.overlapping_interval; ResourceBundle.properties:680. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.overlapping_interval: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow; SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#isOverlapping. WAR: classes byte-identical to the v1.1a4 release. Rows whose interval does not end before its start are compared with the earlier rows of the same form; an overlap raises the overlapping-interval key.</t>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.overlapping_interval; ResourceBundle.properties:680. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.overlapping_interval: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow; SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#isOverlapping. WAR: classes byte-identical to the v1.1a4 release. Rows whose interval does not end before its start are compared with the earlier rows of the same form; an overlap raises the overlapping-interval key. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-017).</t>
   </si>
   <si>
     <t>The last (new) time entry row is rejected when it has both a start/end interval and a duration; the other rows are not checked for this.</t>
@@ -2050,7 +2050,7 @@
     <t>Message "Cannot specify both an interval and duration."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.both_interval_and_duration; ResourceBundle.properties:682. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.both_interval_and_duration is missing in es. Bundles without the key fall back to the default text (framework behavior, GAP-011). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. The interval-and-duration check (#7) applies only to the last row; in other rows a start time, an end time and a duration together are accepted.</t>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.both_interval_and_duration; ResourceBundle.properties:682. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.both_interval_and_duration is missing in es. Bundles without the key fall back to the default text (framework behavior, GAP-011). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. The interval-and-duration check (#7) applies only to the last row; in other rows a start time, an end time and a duration together are accepted. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-018).</t>
   </si>
   <si>
     <t>A time entry row without a report date is rejected.</t>
@@ -2062,7 +2062,7 @@
     <t>Message "Missing reported date."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.missing_report_date; ResourceBundle.properties:683. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.missing_report_date is defined only in the default, "--", de, it, ja and ru bundles. Bundles without the key fall back to the default text (framework behavior, GAP-011). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. Every row except an empty last row and a deleted row needs a report date.</t>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.missing_report_date; ResourceBundle.properties:683. Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.missing_report_date is defined only in the default, "--", de, it, ja and ru bundles. Bundles without the key fall back to the default text (framework behavior, GAP-011). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. Every row except an empty last row and a deleted row needs a report date. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-019).</t>
   </si>
   <si>
     <t>A time entry description longer than the allowed maximum is rejected.</t>
@@ -2074,22 +2074,22 @@
     <t>Message "The time entry description is too long."</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.long_description; ResourceBundle.properties:684; the description input carries maxlength TimeEditorForm.MAX_DESCRIPTION_LENGTH (WAR:WEB-INF/jsp/edit/editTimeEntries.jsp). Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.long_description: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. A description longer than MAX_DESCRIPTION_LENGTH raises the long-description key.</t>
+    <t>class com.technoetic.xplanner.forms.TimeEditorForm#valideRow (bytecode constants; condition inferred from the key and message): edittime.error.long_description; ResourceBundle.properties:684; the description input carries maxlength TimeEditorForm.MAX_DESCRIPTION_LENGTH (WAR:WEB-INF/jsp/edit/editTimeEntries.jsp). Source: stage-02-pass-002 F-001. Locale variants (CHK-004, BA-001-04): quoted texts are from the default bundle; edittime.error.long_description: the key is defined in all 10 bundles (default, "--", da, de, es, fr, it, ja, pt_br, ru). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/forms/TimeEditorForm.java TimeEditorForm#validate, #valideRow. WAR: classes byte-identical to the v1.1a4 release. A description longer than MAX_DESCRIPTION_LENGTH raises the long-description key. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-020).</t>
   </si>
   <si>
     <t>Re-estimate task (legacy page)</t>
   </si>
   <si>
-    <t>A task re-estimate page exists that shows actual and estimated hours and submits a new estimate, recording "Estimate changed from x to y" in history.</t>
+    <t>A task re-estimate page is mapped at /do/edit/task/estimate, but its action is a plain Struts Action: a GET answers HTTP 200 with an empty body, so no page is shown (W001). The estimate update and its "Estimate changed from x to y" history entry work only through a direct POST of the editTaskEstimate.jsp fields to /do/edit/time with action=UPDATE_ESTIMATE (W001).</t>
   </si>
   <si>
     <t>Adjust estimates when actual exceeds plan.</t>
   </si>
   <si>
-    <t>Page reachable only by URL; the mapped action class is a plain Struts Action.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/struts-config.xml:130,301-302 (global forward edit/task/estimate; action /edit/task/estimate); WAR:WEB-INF/action-servlet.xml:298 (org.apache.struts.action.Action); WAR:WEB-INF/jsp/edit/editTaskEstimate.jsp (UPDATE_ESTIMATE); class UpdateTimeAction#doUpdateEstimateAction ("reestimated", "Estimate changed from "). No class references the forward (grep over class dumps). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editTaskEstimate.jsp writes the raw request parameters fkey (43), returnto (45), oid (48) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#doUpdateEstimateAction. WAR: classes byte-identical to the v1.1a4 release. The estimate update and its history text exist, but the page's action mapping uses a plain Struts Action.</t>
+    <t>/do/edit/task/estimate returns an empty 200 response; a direct POST of the estimate fields to /do/edit/time updates the estimate and writes the "reestimated" history entry (W001).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/struts-config.xml:130,301-302 (global forward edit/task/estimate; action /edit/task/estimate); WAR:WEB-INF/action-servlet.xml:298 (org.apache.struts.action.Action); WAR:WEB-INF/jsp/edit/editTaskEstimate.jsp (UPDATE_ESTIMATE); class UpdateTimeAction#doUpdateEstimateAction ("reestimated", "Estimate changed from "). No class references the forward (grep over class dumps). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editTaskEstimate.jsp writes the raw request parameters fkey (43), returnto (45), oid (48) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/UpdateTimeAction.java UpdateTimeAction#doUpdateEstimateAction. WAR: classes byte-identical to the v1.1a4 release. The estimate update and its history text exist, but the page's action mapping uses a plain Struts Action. Stage 3 W001 (BA-001-13, MC-A-31, W001-F-36): GET: 200, 0 bytes; direct POST (estimate 6.0, action UPDATE_ESTIMATE): 302, estimate 6.0 (4.0), history "Estimate changed from 4.0 to 6.0" (C-C-021). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks C-C-021).</t>
   </si>
   <si>
     <t>Personal timesheet</t>
@@ -2101,19 +2101,19 @@
     <t>Report personal effort.</t>
   </si>
   <si>
-    <t>Summary table with total, daily table, and pie charts by project, iteration and story.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/person.jsp (link /do/view/timesheet); WAR:WEB-INF/struts-config.xml:374-378; class ViewTimesheetAction; WAR:calendar/calendar-i18n.jsp, WAR:calendar/calendar.js (date picker); WAR:WEB-INF/jsp/view/timesheet.jsp (cewolf charts personTimesheetProjectChart, ...IterationChart, ...StoryChart). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ViewTimesheetAction.java ViewTimesheetAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. The timesheet of the posted person and period is queried and shown.</t>
+    <t>Summary table with total, daily table, and pie charts by project, iteration and story. The entry point from the person page is unavailable while that page answers HTTP 500 (row 40, W001); /do/view/timesheet?oid=&lt;id&gt; works by its own URL.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/person.jsp (link /do/view/timesheet); WAR:WEB-INF/struts-config.xml:374-378; class ViewTimesheetAction; WAR:calendar/calendar-i18n.jsp, WAR:calendar/calendar.js (date picker); WAR:WEB-INF/jsp/view/timesheet.jsp (cewolf charts personTimesheetProjectChart, ...IterationChart, ...StoryChart). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ViewTimesheetAction.java ViewTimesheetAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. The timesheet of the posted person and period is queried and shown. Stage 3 W001 (BA-001-13, MC-A-09, W001-F-10): the own person page answered HTTP 500, so its Timesheet link was not reachable (setup-C-058); the timesheet itself works by URL (C-C-022, C-C-024). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks setup-C-057, setup-C-058, C-C-022).</t>
   </si>
   <si>
     <t>An unparsable period date is rejected.</t>
   </si>
   <si>
-    <t>Message "Can't parse the supplied date value."</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.forms.PersonTimesheetForm#validate (timesheet.error.unparsable_date). Locale variants (CHK-004, BA-001-04): The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/PersonTimesheetForm.java PersonTimesheetForm#validate. WAR: classes byte-identical to the v1.1a4 release. An unparsable start or end date raises the unparsable-date key; the pattern comes from format.date in the request (Accept-Language) locale.</t>
+    <t>No message is displayed: the page returns with the default period (W001: 2026-09-27 to 2026-10-03) and no error markup, so the unparsable-date key raised by validate() (static, below) is not shown.</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.PersonTimesheetForm#validate (timesheet.error.unparsable_date). Locale variants (CHK-004, BA-001-04): The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/PersonTimesheetForm.java PersonTimesheetForm#validate. WAR: classes byte-identical to the v1.1a4 release. An unparsable start or end date raises the unparsable-date key; the pattern comes from format.date in the request (Accept-Language) locale. Stage 3 W001 (BA-001-13, MC-A-32, W001-F-37): start date "not-a-date" and empty: 200, no message, no error markup, default period (C-C-023). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks C-C-023).</t>
   </si>
   <si>
     <t>The personal timesheet applies no permission filter: any signed-in user can open any person's timesheet by its oid.</t>
@@ -2125,7 +2125,7 @@
     <t>Timesheet of the requested person is shown to any signed-in user (runtime unverified).</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.actions.ViewTimesheetAction: no authorization call reachable (.migration-tmp/stage-01/out/authtrace.json); the "timesheet" link on WAR:WEB-INF/jsp/view/person.jsp is not permission-gated. BA-001-03 impact sweep of F-007. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/ViewTimesheetAction.java ViewTimesheetAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. The action queries the timesheet of the posted person id with no authorizer call.</t>
+    <t>class com.technoetic.xplanner.actions.ViewTimesheetAction: no authorization call reachable (.migration-tmp/stage-01/out/authtrace.json); the "timesheet" link on WAR:WEB-INF/jsp/view/person.jsp is not permission-gated. BA-001-03 impact sweep of F-007. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/ViewTimesheetAction.java ViewTimesheetAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. The action queries the timesheet of the posted person id with no authorizer call. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-024).</t>
   </si>
   <si>
     <t>Aggregate timesheet</t>
@@ -2140,10 +2140,13 @@
     <t>Multi-select of people, date range, summary tables and three pie charts.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/projects.jsp:164 (link /do/view/aggregateTimesheet); WAR:WEB-INF/struts-config.xml:380-384; class ViewAggregateTimesheetAction (HQL people.hidden = false order by name); WAR:WEB-INF/jsp/view/aggregateTimesheet.jsp. Request-value flow (BA-001-07, mechanism (b)): the posted selectedPeople values (AggregateTimesheetForm#setSelectedPeople, String[]) are passed to AggregateTimesheetQuery#setPersonIds; #getTimesheet appends each element unchanged into "AND person.id IN (...)", substitutes it for the placeholder "AND 1=1" with String#replaceAll and runs Session.iterate with only the two dates bound (bytecode listing). The query text is kept in a static field that each call re-initialises, so concurrent requests may share it (Inferred). AggregateTimesheetForm#validate checks only the dates. Mapping WAR:WEB-INF/struts-config.xml:380-384, any signed-in user. Exploitability is not established (static only). Observed risk only (Q3 deferred). Source: stage-02-pass-005 F-002. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/db/AggregateTimesheetQuery.java AggregateTimesheetQuery#getTimesheet. WAR: classes byte-identical to the v1.1a4 release. The query groups hours by project, iteration and story for the selected people and period.</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.forms.AggregateTimesheetForm#validate (timesheet.error.unparsable_date). Locale variants (CHK-004, BA-001-04): The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/AggregateTimesheetForm.java AggregateTimesheetForm#validate. WAR: classes byte-identical to the v1.1a4 release. An unparsable date raises the unparsable-date key.</t>
+    <t>WAR:WEB-INF/jsp/view/projects.jsp:164 (link /do/view/aggregateTimesheet); WAR:WEB-INF/struts-config.xml:380-384; class ViewAggregateTimesheetAction (HQL people.hidden = false order by name); WAR:WEB-INF/jsp/view/aggregateTimesheet.jsp. Request-value flow (BA-001-07, mechanism (b)): the posted selectedPeople values (AggregateTimesheetForm#setSelectedPeople, String[]) are passed to AggregateTimesheetQuery#setPersonIds; #getTimesheet appends each element unchanged into "AND person.id IN (...)", substitutes it for the placeholder "AND 1=1" with String#replaceAll and runs Session.iterate with only the two dates bound (bytecode listing). The query text is kept in a static field that each call re-initialises, so concurrent requests may share it (Inferred). AggregateTimesheetForm#validate checks only the dates. Mapping WAR:WEB-INF/struts-config.xml:380-384, any signed-in user. Exploitability is not established (static only). Observed risk only (Q3 deferred). Source: stage-02-pass-005 F-002. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/db/AggregateTimesheetQuery.java AggregateTimesheetQuery#getTimesheet. WAR: classes byte-identical to the v1.1a4 release. The query groups hours by project, iteration and story for the selected people and period. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-025).</t>
+  </si>
+  <si>
+    <t>No message is displayed: the form returns the default period and "Nothing found to display." with no error markup (W001), so the unparsable-date key raised by validate() (static, below) is not shown.</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.AggregateTimesheetForm#validate (timesheet.error.unparsable_date). Locale variants (CHK-004, BA-001-04): The accepted date and date-time patterns follow format.date and format.datetime of the active bundle and differ per locale (rows 69-71). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/forms/AggregateTimesheetForm.java AggregateTimesheetForm#validate. WAR: classes byte-identical to the v1.1a4 release. An unparsable date raises the unparsable-date key. Stage 3 W001 (BA-001-13, MC-A-32, W001-F-37): start date "not-a-date" and "2026/13/45x": 200, no message, no error markup, default period (C-C-026). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks C-C-026).</t>
   </si>
   <si>
     <t>The aggregate timesheet includes only hours on projects the viewing user may read.</t>
@@ -2155,7 +2158,7 @@
     <t>Rows and charts cover readable projects only.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.db.AggregateTimesheetQuery#getTimesheet (SystemAuthorizer.get, Authorizer.hasPermission with "system.project" and "read"); path ViewAggregateTimesheetAction#doExecute in .migration-tmp/stage-01/out/authtrace.json. Source: stage-02-pass-001 F-007. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/db/AggregateTimesheetQuery.java AggregateTimesheetQuery#getTimesheet. WAR: classes byte-identical to the v1.1a4 release. Each result row is added only when the viewing user has read permission on its project.</t>
+    <t>class com.technoetic.xplanner.db.AggregateTimesheetQuery#getTimesheet (SystemAuthorizer.get, Authorizer.hasPermission with "system.project" and "read"); path ViewAggregateTimesheetAction#doExecute in .migration-tmp/stage-01/out/authtrace.json. Source: stage-02-pass-001 F-007. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/db/AggregateTimesheetQuery.java AggregateTimesheetQuery#getTimesheet. WAR: classes byte-identical to the v1.1a4 release. Each result row is added only when the viewing user has read permission on its project. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-027, E-C-001, E-C-002, E-C-003, E-C-004).</t>
   </si>
   <si>
     <t>UF-010</t>
@@ -2167,16 +2170,16 @@
     <t>Add note to an object</t>
   </si>
   <si>
-    <t>On project, iteration, story and task pages a user with note edit permission can add a note with subject, author, body and an optional file attachment.</t>
+    <t>On project, iteration, story and task pages a user with note edit permission can add a note with subject, author, body and an optional file attachment. In this baseline a note with a file attachment cannot be saved (W001).</t>
   </si>
   <si>
     <t>Record decisions and share files in context.</t>
   </si>
   <si>
-    <t>Note editor (multipart form); after save the note appears in the Notes section of the object page.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/layout/viewLayout.jsp:114-116 (include view/notes.jsp in tiles:view pages); WAR:WEB-INF/jsp/view/notes.jsp:20-23 (isNoteEditor = hasPermission(..., "note", 0, "edit")) and link /do/edit/note?attachedToId=; WAR:WEB-INF/struts-config.xml:306-307; WAR:WEB-INF/action-servlet.xml:306-313 (EditNoteAction, virtualFileSystem); WAR:WEB-INF/jsp/edit/editNote.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request-value flow (BA-001-07, mechanism (b)): the note list included in these pages reads the oid request parameter (WAR:WEB-INF/jsp/view/notes.jsp:13, bean:parameter) and concatenates it into the useBeans where clause "attachedToId=" + oid (:14-15), which UseBeansTag#doEndTag appends into the HQL text; this is the same pattern as the time-log query of WAR:WEB-INF/jsp/view/task.jsp:101-103 (Q3 facts). Exploitability is not established (static only; observed risk only, Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editNote.jsp writes the raw request parameters oid (31), returnto (35,106), projectId (37), attachedToId (39), formFileName (82) [parameter (lines); line 106 passes returnto as the page attribute of html:link] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/note that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Note object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). EditNoteAction#populateObject calls the parent method before it stores the attachment. No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/actions/EditNoteAction.java EditNoteAction#populateObject; SRC:src/com/technoetic/xplanner/tags/db/UseBeansTag.java UseBeansTag#doEndTag; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
+    <t>Note editor (multipart form); after save the note appears in the Notes section of the object page. With a file attachment the save answers HTTP 500 (ConstraintViolationException, foreign key noteAttachments, note.attachment_id -&gt; xfile.id): no note and no file are stored (W001, Runtime: live-observed on this runtime; may depend on this runtime (Tomcat 9 / JRE 8, MySQL 5.7); whether the original installation behaves the same is not established).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/layout/viewLayout.jsp:114-116 (include view/notes.jsp in tiles:view pages); WAR:WEB-INF/jsp/view/notes.jsp:20-23 (isNoteEditor = hasPermission(..., "note", 0, "edit")) and link /do/edit/note?attachedToId=; WAR:WEB-INF/struts-config.xml:306-307; WAR:WEB-INF/action-servlet.xml:306-313 (EditNoteAction, virtualFileSystem); WAR:WEB-INF/jsp/edit/editNote.jsp. Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request-value flow (BA-001-07, mechanism (b)): the note list included in these pages reads the oid request parameter (WAR:WEB-INF/jsp/view/notes.jsp:13, bean:parameter) and concatenates it into the useBeans where clause "attachedToId=" + oid (:14-15), which UseBeansTag#doEndTag appends into the HQL text; this is the same pattern as the time-log query of WAR:WEB-INF/jsp/view/task.jsp:101-103 (Q3 facts). Exploitability is not established (static only; observed risk only, Q3 deferred). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editNote.jsp writes the raw request parameters oid (31), returnto (35,106), projectId (37), attachedToId (39), formFileName (82) [parameter (lines); line 106 passes returnto as the page attribute of html:link] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Request binding (BA-001-08, pass-006 F-001, check (d)): a request to /do/edit/note that carries merge=true is not copied from the form; class EditObjectAction#populateObject compares the merge parameter with "true" and then calls org.apache.struts.util.RequestUtils.populate onto the loaded or new Note object, skipping the form copy (#copyProperties) and the many-to-one resolution (#populateManyToOneRelationships) (bytecode listing). Every request parameter that names a writable property of the object is set; no property list restricts the set, and nested property names are resolved by the bundled commons-beanutils (framework behavior, GAP-011). EditNoteAction#populateObject calls the parent method before it stores the attachment. No page posts merge=true to this editor, so this applies to direct requests (Inferred; observed risk only, Q3 deferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/com/technoetic/xplanner/actions/EditNoteAction.java EditNoteAction#populateObject; SRC:src/com/technoetic/xplanner/tags/db/UseBeansTag.java UseBeansTag#doEndTag; SRC:src/com/technoetic/xplanner/actions/EditObjectAction.java EditObjectAction#populateObject. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Stage 3 W001 (BA-001-13, MC-A-33, W001-F-38): two notes with synthetic files (one without body): both HTTP 500 with the foreign-key violation, no note listed (C-C-030). Status Yes -&gt; Partial (R-G2). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks C-C-028, C-C-029, C-C-030).</t>
   </si>
   <si>
     <t>A note without subject or author is rejected; a note without body is rejected only when no file is attached.</t>
@@ -2185,10 +2188,10 @@
     <t>Notes must be meaningful and attributed.</t>
   </si>
   <si>
-    <t>Messages "Missing subject.", "Missing author.", "Missing body."</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.forms.NoteEditorForm#validate (note.editor.missing_subject, missing_author, missing_body). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/forms/NoteEditorForm.java NoteEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release. Subject and author are always required, but the body only when no file is attached.</t>
+    <t>Messages "Missing subject.", "Missing author.", "Missing body." (source). On this runtime they are never shown: a note editor submission that fails validation answers HTTP 500 (java.lang.AbstractMethodError, MultipartRequestWrapper.getServletContext()) and saves nothing (W001; container-dependent, the bundled Struts 1.2 multipart wrapper on a Servlet 3+ container; may depend on this runtime (Tomcat 9)). The body-optional-with-file rule cannot occur in this baseline, because no note with a file can be saved (row 169, MC-A-33).</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.forms.NoteEditorForm#validate (note.editor.missing_subject, missing_author, missing_body). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/forms/NoteEditorForm.java NoteEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release. Subject and author are always required, but the body only when no file is attached. Stage 3 W001 (BA-001-13, MC-A-34, MC-A-33, W001-F-39, W001-F-38): empty subject, authorId 0, and empty body with an empty file part: all HTTP 500 AbstractMethodError, nothing saved (C-C-031); a note with a file and no body failed with the attachment error (C-C-032, part C blocked, reclassified as observed by the W001 lead). Status Yes -&gt; Partial (R-G2). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks C-C-031, C-C-032).</t>
   </si>
   <si>
     <t>Each note with an attachment shows the attachment name and a "References:" count, which is the number of notes that point to the same file.</t>
@@ -2197,10 +2200,10 @@
     <t>Shows how many notes share one attached file.</t>
   </si>
   <si>
-    <t>"Attachment" link and "References: &lt;n&gt;" on the note.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/notes.jsp:80-92 (link /do/download/attachment, notes.label.attachment.count, note.getAttachmentCount()); class net.sf.xplanner.domain.Note#getAttachmentCount runs "select note from Note note where note.file.id=" + file id and returns the list size (bytecode listing); label WAR:WEB-INF/classes/ResourceBundle.properties:545 ("References:"); DownloadAttachmentAction counts nothing. Label per bundle (CHK-004): "References:" in the default, "--" and ja bundles, "Referenzen:" in de; the other bundles have no key and fall back to the default. Corrected in BA-001-04 (Source: stage-02-pass-002 F-004). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/net/sf/xplanner/domain/Note.java Note#getAttachmentCount. WAR: classes byte-identical to the v1.1a4 release. The count is the number of notes whose file id equals this note's file id.</t>
+    <t>"Attachment" link and "References: &lt;n&gt;" on the note (source); neither occurs in this baseline, because no attachment can be stored (row 169, W001).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/notes.jsp:80-92 (link /do/download/attachment, notes.label.attachment.count, note.getAttachmentCount()); class net.sf.xplanner.domain.Note#getAttachmentCount runs "select note from Note note where note.file.id=" + file id and returns the list size (bytecode listing); label WAR:WEB-INF/classes/ResourceBundle.properties:545 ("References:"); DownloadAttachmentAction counts nothing. Label per bundle (CHK-004): "References:" in the default, "--" and ja bundles, "Referenzen:" in de; the other bundles have no key and fall back to the default. Corrected in BA-001-04 (Source: stage-02-pass-002 F-004). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/net/sf/xplanner/domain/Note.java Note#getAttachmentCount. WAR: classes byte-identical to the v1.1a4 release. The count is the number of notes whose file id equals this note's file id. Stage 3 W001 (BA-001-13, MC-A-33, W001-F-38): C-C-033 was not executed (not-checked): the behavior is unavailable because the upload fails (C-C-030, C-C-034). Status Yes -&gt; Partial (R-G2). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks C-C-030, C-C-033, C-C-034).</t>
   </si>
   <si>
     <t>An uploaded attachment is stored in the application virtual file system under /attachments/project/&lt;projectId&gt;; the file bytes are kept in the database as a BLOB (table xfile, column data), and directories are rows of table xdir.</t>
@@ -2209,37 +2212,37 @@
     <t>Attachments are kept with the project, inside the database.</t>
   </si>
   <si>
-    <t>Attachment readable via the download link; the first attachment of a project also creates the root directory and the /attachments/project/&lt;projectId&gt; directory rows (runtime unverified).</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.actions.EditNoteAction#populateObject (strings "/attachments/project/", "Saving note: filename="; calls FileSystem.getDirectory, FileSystem.createFile, Note.setFile); class com.technoetic.xplanner.file.FileSystemImpl#createFile (Hibernate.createBlob, File.setData); class net.sf.xplanner.domain.File field data (@Lob, @Column(name="data", length=1000000000)); WAR:WEB-INF/classes/spring-beans.xml:263 (virtualFileSystem FileSystemImpl); WAR:WEB-INF/classes/db-changelog.xml:234 (xfile.data LONGBLOB). Corrected in BA-001-03 (stage-02-pass-001 F-008). Directory creation on first use (BA-001-07, mechanism (c)): EditNoteAction#populateObject calls FileSystem#getDirectory("/attachments/project/&lt;id&gt;"); FileSystemImpl#getDirectory(String) calls #getRootDirectory, which saves, flushes and refreshes a new root Directory when none exists, and calls #createDirectory for each missing path segment (bytecode listings). The file system is wired into /edit/note explicitly (WAR:WEB-INF/action-servlet.xml:306-309). Source: stage-02-pass-005 F-005. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/EditNoteAction.java EditNoteAction#populateObject; SRC:src/com/technoetic/xplanner/file/FileSystemImpl.java FileSystemImpl#createFile. WAR: classes byte-identical to the v1.1a4 release. The file bytes are stored as a BLOB in a File row of the directory /attachments/project/&lt;projectId&gt; (the projectId request parameter, 0 when missing). Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>Attachment readable via the download link; the first attachment of a project also creates the root directory and the /attachments/project/&lt;projectId&gt; directory rows (source, runtime unverified). Live (W001): the upload fails at the note insert with the note -&gt; xfile foreign key violation, so no attachment, reference count or download exists in this baseline; database rows were not inspected (may depend on this runtime (Tomcat 9 / JRE 8, MySQL 5.7)).</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.actions.EditNoteAction#populateObject (strings "/attachments/project/", "Saving note: filename="; calls FileSystem.getDirectory, FileSystem.createFile, Note.setFile); class com.technoetic.xplanner.file.FileSystemImpl#createFile (Hibernate.createBlob, File.setData); class net.sf.xplanner.domain.File field data (@Lob, @Column(name="data", length=1000000000)); WAR:WEB-INF/classes/spring-beans.xml:263 (virtualFileSystem FileSystemImpl); WAR:WEB-INF/classes/db-changelog.xml:234 (xfile.data LONGBLOB). Corrected in BA-001-03 (stage-02-pass-001 F-008). Directory creation on first use (BA-001-07, mechanism (c)): EditNoteAction#populateObject calls FileSystem#getDirectory("/attachments/project/&lt;id&gt;"); FileSystemImpl#getDirectory(String) calls #getRootDirectory, which saves, flushes and refreshes a new root Directory when none exists, and calls #createDirectory for each missing path segment (bytecode listings). The file system is wired into /edit/note explicitly (WAR:WEB-INF/action-servlet.xml:306-309). Source: stage-02-pass-005 F-005. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/EditNoteAction.java EditNoteAction#populateObject; SRC:src/com/technoetic/xplanner/file/FileSystemImpl.java FileSystemImpl#createFile. WAR: classes byte-identical to the v1.1a4 release. The file bytes are stored as a BLOB in a File row of the directory /attachments/project/&lt;projectId&gt; (the projectId request parameter, 0 when missing). Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream. Stage 3 W001 (BA-001-13, MC-A-33, W001-F-38): C-C-034. Status Yes -&gt; Partial, as proposed. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks C-C-034).</t>
   </si>
   <si>
     <t>Edit and delete note</t>
   </si>
   <si>
-    <t>An authorized user can edit a note.</t>
+    <t>An authorized user can edit a note. For an editor without the author select (a non-administrator), the editor posts the editing user as authorId in a hidden field, so the save reassigns the note's author to the editing user (W001).</t>
   </si>
   <si>
     <t>Correct notes.</t>
   </si>
   <si>
-    <t>Note editor pre-filled; changes saved.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/notes.jsp (isUserAuthorized note edit; link /do/edit/note). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 169 applies to every /do/edit/note request (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
-  </si>
-  <si>
-    <t>An authorized user can delete a note after confirming "Do you want to delete note &lt;subject&gt;".</t>
+    <t>Note editor pre-filled; changes saved; for a non-administrator editor the note's author becomes the editing user (W001).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/notes.jsp (isUserAuthorized note edit; link /do/edit/note). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); EditNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Request binding (BA-001-08, pass-006 F-001): the merge=true binding of row 169 applies to every /do/edit/note request (Inferred; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Stage 3 W001 (BA-001-13, MC-B-06, W001-F-40): the edit link of note 499 (author: viewer) opened as editor: hidden authorId carries the editor; after the save the author is the editor (C-C-035). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks C-C-035).</t>
+  </si>
+  <si>
+    <t>An authorized user can delete a note after confirming "Do you want to delete note &lt;subject&gt;". In this baseline the note is not removed (W001).</t>
   </si>
   <si>
     <t>Remove obsolete notes.</t>
   </si>
   <si>
-    <t>Confirm prompt; note removed; its attachment file removed too unless another note references it.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/notes.jsp (link /do/delete/note with confirm); WAR:WEB-INF/struts-config.xml:309; class com.technoetic.xplanner.actions.DeleteNoteAction#doExecute calls NoteHelper#deleteNote, which deletes the attached file only when no other note references it (query "select note from Note note where note.file.id= ?", size check), then the note (bytecode listing; BA-001-04 cascade sweep). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/db/NoteHelper.java NoteHelper#deleteNote. WAR: classes byte-identical to the v1.1a4 release. The note is deleted, and its file only when no other note refers to it.</t>
+    <t>Confirm prompt; in this baseline /do/delete/note then redirects (302 to returnto) without deleting the note, for editor and viewer requests (W001). The claim that its attachment file is removed too unless another note references it stays static.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/notes.jsp (link /do/delete/note with confirm); WAR:WEB-INF/struts-config.xml:309; class com.technoetic.xplanner.actions.DeleteNoteAction#doExecute calls NoteHelper#deleteNote, which deletes the attached file only when no other note references it (query "select note from Note note where note.file.id= ?", size check), then the note (bytecode listing; BA-001-04 cascade sweep). Server-side enforcement (CHK-002, BA-001-04): the condition is display-level only (link, field or button shown by JSP permission tags); DeleteNoteAction performs no server-side permission check, so a direct request succeeds for any signed-in user (rows 29-30; .migration-tmp/stage-01/out/authtrace.json). Observed risk only (Q3 deferred). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/db/NoteHelper.java NoteHelper#deleteNote. WAR: classes byte-identical to the v1.1a4 release. The note is deleted, and its file only when no other note refers to it. Stage 3 W001 (BA-001-13, MC-A-35, W001-F-41): onclick confirm text as mapped; both requests answered 302 to the task, the note stays listed and its editor still opens (C-C-036); part E left nine orphan notes for the same reason. Status Yes -&gt; Partial (R-G2). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks C-C-036).</t>
   </si>
   <si>
     <t>Download attachment</t>
@@ -2251,10 +2254,10 @@
     <t>Retrieve shared files.</t>
   </si>
   <si>
-    <t>File streamed with Content-disposition filename.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/notes.jsp (link /do/download/attachment?oid=); WAR:WEB-INF/struts-config.xml:311; class com.technoetic.xplanner.actions.DownloadAttachmentAction (strings "Content-disposition", "note;filename="). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DownloadAttachmentAction.java DownloadAttachmentAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. The file of the note is written to the response with its content type and name.</t>
+    <t>File streamed with Content-disposition filename (source); no download occurs in this baseline, because no attachment can be stored (row 169, W001).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/notes.jsp (link /do/download/attachment?oid=); WAR:WEB-INF/struts-config.xml:311; class com.technoetic.xplanner.actions.DownloadAttachmentAction (strings "Content-disposition", "note;filename="). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/DownloadAttachmentAction.java DownloadAttachmentAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. The file of the note is written to the response with its content type and name. Stage 3 W001 (BA-001-13, MC-A-33, W001-F-38): C-C-037 was not executed (not-checked): no attachment can be stored (C-C-030, C-C-034). Status Yes -&gt; Partial (R-G2). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks C-C-030, C-C-034, C-C-037).</t>
   </si>
   <si>
     <t>File manager (directories)</t>
@@ -2269,7 +2272,7 @@
     <t>Pages reachable by URL only; every file-manager operation, including the default listing, is expected to fail with a null reference because the file system is never injected into the action (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:401-403; WAR:WEB-INF/action-servlet.xml:396 (FileManagerAction); WAR:WEB-INF/jsp/view/directory.jsp; class FileManagerAction#doExecute (actions list, upload, download, delete, mkdir, rmdir). Only self-links from directory.jsp were found (linkgraph.txt); entry is by URL. Delete cascade sweep (BA-001-04): class com.technoetic.xplanner.file.FileSystemImpl#deleteFile and #deleteDirectory run an HQL delete by id without cascading; net.sf.xplanner.domain.Directory maps files and subdirectories without cascade. The foreign keys WAR:WEB-INF/classes/db-changelog.xml:259 (note.attachment_id -&gt; xfile), :266 (xdir.parent_id -&gt; xdir) and :267 (xfile.dir_id -&gt; xdir) are expected to make the database reject deleting a file that a note references or a directory that is not empty (runtime unverified). Wiring and read-path writes (BA-001-07, mechanisms (a) and (c)): the bean /view/directory (WAR:WEB-INF/action-servlet.xml:396) has no properties; FileManagerAction#setFileSystem would need a bean named fileSystem, but the file system bean is named virtualFileSystem (WAR:WEB-INF/classes/spring-beans.xml:263; provenance P-05) and is wired explicitly only into /edit/note (action-servlet.xml:306-309). FileManagerAction#doExecute reads the field for every action (list, upload, download, delete, mkdir, rmdir), so the first call is expected to fail. The write-on-read of FileSystemImpl#getRootDirectory (it saves, flushes and refreshes a new root Directory when none exists) is therefore not expected to be reached from GET /do/view/directory. Corrected in BA-001-07 (Source: stage-02-pass-005 F-005, narrowed). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/FileManagerAction.java FileManagerAction#doExecute, #setFileSystem. WAR: classes byte-identical to the v1.1a4 release. The setter has no annotation and no bean named fileSystem exists; the null-reference outcome is a runtime effect. Live question: Does /do/view/directory fail on the default listing?</t>
+    <t>WAR:WEB-INF/struts-config.xml:401-403; WAR:WEB-INF/action-servlet.xml:396 (FileManagerAction); WAR:WEB-INF/jsp/view/directory.jsp; class FileManagerAction#doExecute (actions list, upload, download, delete, mkdir, rmdir). Only self-links from directory.jsp were found (linkgraph.txt); entry is by URL. Delete cascade sweep (BA-001-04): class com.technoetic.xplanner.file.FileSystemImpl#deleteFile and #deleteDirectory run an HQL delete by id without cascading; net.sf.xplanner.domain.Directory maps files and subdirectories without cascade. The foreign keys WAR:WEB-INF/classes/db-changelog.xml:259 (note.attachment_id -&gt; xfile), :266 (xdir.parent_id -&gt; xdir) and :267 (xfile.dir_id -&gt; xdir) are expected to make the database reject deleting a file that a note references or a directory that is not empty (runtime unverified). Wiring and read-path writes (BA-001-07, mechanisms (a) and (c)): the bean /view/directory (WAR:WEB-INF/action-servlet.xml:396) has no properties; FileManagerAction#setFileSystem would need a bean named fileSystem, but the file system bean is named virtualFileSystem (WAR:WEB-INF/classes/spring-beans.xml:263; provenance P-05) and is wired explicitly only into /edit/note (action-servlet.xml:306-309). FileManagerAction#doExecute reads the field for every action (list, upload, download, delete, mkdir, rmdir), so the first call is expected to fail. The write-on-read of FileSystemImpl#getRootDirectory (it saves, flushes and refreshes a new root Directory when none exists) is therefore not expected to be reached from GET /do/view/directory. Corrected in BA-001-07 (Source: stage-02-pass-005 F-005, narrowed). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/FileManagerAction.java FileManagerAction#doExecute, #setFileSystem. WAR: classes byte-identical to the v1.1a4 release. The setter has no annotation and no bean named fileSystem exists; the null-reference outcome is a runtime effect. Live question: Does /do/view/directory fail on the default listing? Stage 3 W001 live answer (BA-001-13, MC-C-21): Yes: HTTP 500, NullPointerException at FileManagerAction.doExecute(FileManagerAction.java:40) (C-C-038). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-038).</t>
   </si>
   <si>
     <t>UF-011</t>
@@ -2290,7 +2293,7 @@
     <t>Results page "Search results - &lt;text&gt;" with type, ID, title (links to object or to the object a note is attached to) and match.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:22-35 (form /do/search/content, searchedContent, restrictToProjectId); WAR:WEB-INF/struts-config.xml:415-417; class ContentSearchAction (search.content.globalScopeEnable); WAR:WEB-INF/classes/xplanner.properties:287; WAR:WEB-INF/classes/spring-beans.xml:210-226; WAR:WEB-INF/jsp/view/searchResults.jsp. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute. WAR: classes byte-identical to the v1.1a4 release; search.content.globalScopeEnable=true in the WAR xplanner.properties. With the global scope the whole database is searched; a numeric search text also adds the object with that id first (row 180). Correction (BA-001-12, pass-010 F-002): the object added first for a numeric text is the one found by SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search; IdSearchHelper#search tries Project, Iteration, UserStory, Task, Person and Note in that order and, when the object is a Note, returns Note#getParent instead: the object whose id is the note's attached-to id, looked up the same way (a failed lookup gives null). For a note's id the parent object is added, not the note (SRC:src/net/sf/xplanner/domain/Note.java Note#getParent; SRC:src/com/technoetic/xplanner/tags/DomainContext.java DomainContext#getNoteTarget; SRC:src/com/technoetic/xplanner/db/OLDIdSearchHelper.java OLDIdSearchHelper#search; bytecode listings agree: instanceof Note, getParent; the thread session is bound by SRC:src/com/technoetic/xplanner/db/hibernate/HibernateSessionFilter.java HibernateSessionFilter#doFilter before the filter chain, mapped at /* (WAR:WEB-INF/web.xml:147-152)). See row 180. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:22-35 (form /do/search/content, searchedContent, restrictToProjectId); WAR:WEB-INF/struts-config.xml:415-417; class ContentSearchAction (search.content.globalScopeEnable); WAR:WEB-INF/classes/xplanner.properties:287; WAR:WEB-INF/classes/spring-beans.xml:210-226; WAR:WEB-INF/jsp/view/searchResults.jsp. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute. WAR: classes byte-identical to the v1.1a4 release; search.content.globalScopeEnable=true in the WAR xplanner.properties. With the global scope the whole database is searched; a numeric search text also adds the object with that id first (row 180). Correction (BA-001-12, pass-010 F-002): the object added first for a numeric text is the one found by SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search; IdSearchHelper#search tries Project, Iteration, UserStory, Task, Person and Note in that order and, when the object is a Note, returns Note#getParent instead: the object whose id is the note's attached-to id, looked up the same way (a failed lookup gives null). For a note's id the parent object is added, not the note (SRC:src/net/sf/xplanner/domain/Note.java Note#getParent; SRC:src/com/technoetic/xplanner/tags/DomainContext.java DomainContext#getNoteTarget; SRC:src/com/technoetic/xplanner/db/OLDIdSearchHelper.java OLDIdSearchHelper#search; bytecode listings agree: instanceof Note, getParent; the thread session is bound by SRC:src/com/technoetic/xplanner/db/hibernate/HibernateSessionFilter.java HibernateSessionFilter#doFilter before the filter chain, mapped at /* (WAR:WEB-INF/web.xml:147-152)). See row 180. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-039).</t>
   </si>
   <si>
     <t>A search without results shows an empty-results message.</t>
@@ -2302,7 +2305,7 @@
     <t>Message empty.search.results.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/view/searchResults.jsp (empty.search.results). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/jsp/view/searchResults.jsp (empty.search.results). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-040).</t>
   </si>
   <si>
     <t>Text matches are filtered to objects the searching user may read; a numeric search text also puts the object with that id at the top of the results (for the id of a note, the note's parent object), without a read check.</t>
@@ -2314,7 +2317,7 @@
     <t>Only readable matches are listed.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.db.ContentSearchHelper#search calls #excludeResultsBasedOnUserPermissions, which filters with #getAuthorizationPredicate -&gt; class com.technoetic.xplanner.actions.SearchResultAuthorizationPredicate#evaluate/#isResultReadableByUser (SystemAuthorizer.get, Authorizer.hasPermission, string "read"). Source: stage-02-pass-001 F-007. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/db/ContentSearchHelper.java ContentSearchHelper#search, #excludeResultsBasedOnUserPermissions; SRC:src/com/technoetic/xplanner/actions/SearchResultAuthorizationPredicate.java SearchResultAuthorizationPredicate#isResultReadableByUser; SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute; SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search. WAR: classes byte-identical to the v1.1a4 release; search.content.globalScopeEnable=true in the WAR xplanner.properties. Text matches are filtered by read permission. After the filter, when the search text is a number and the scope is global (the WAR value), ContentSearchAction adds the object with that id at the top of the results without a permission check (bytecode listing agrees). Correction (BA-001-12, pass-010 F-002): method-level reading of the corrected claim: SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search; SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute (adds the returned object at position 0 when it is Nameable, with no authorizer call); SRC:src/net/sf/xplanner/domain/Note.java Note#getParent; SRC:src/com/technoetic/xplanner/tags/DomainContext.java DomainContext#getNoteTarget; SRC:src/com/technoetic/xplanner/db/OLDIdSearchHelper.java OLDIdSearchHelper#search. IdSearchHelper#search tries Project, Iteration, UserStory, Task, Person and Note in that order and, when the object is a Note, returns Note#getParent instead: the object whose id is the note's attached-to id, looked up the same way (a failed lookup gives null). Bytecode listings agree; the thread session is bound by SRC:src/com/technoetic/xplanner/db/hibernate/HibernateSessionFilter.java HibernateSessionFilter#doFilter before the filter chain, mapped at /* (WAR:WEB-INF/web.xml:147-152). Status stays Yes on this reading.</t>
+    <t>class com.technoetic.xplanner.db.ContentSearchHelper#search calls #excludeResultsBasedOnUserPermissions, which filters with #getAuthorizationPredicate -&gt; class com.technoetic.xplanner.actions.SearchResultAuthorizationPredicate#evaluate/#isResultReadableByUser (SystemAuthorizer.get, Authorizer.hasPermission, string "read"). Source: stage-02-pass-001 F-007. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/db/ContentSearchHelper.java ContentSearchHelper#search, #excludeResultsBasedOnUserPermissions; SRC:src/com/technoetic/xplanner/actions/SearchResultAuthorizationPredicate.java SearchResultAuthorizationPredicate#isResultReadableByUser; SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute; SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search. WAR: classes byte-identical to the v1.1a4 release; search.content.globalScopeEnable=true in the WAR xplanner.properties. Text matches are filtered by read permission. After the filter, when the search text is a number and the scope is global (the WAR value), ContentSearchAction adds the object with that id at the top of the results without a permission check (bytecode listing agrees). Correction (BA-001-12, pass-010 F-002): method-level reading of the corrected claim: SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search; SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute (adds the returned object at position 0 when it is Nameable, with no authorizer call); SRC:src/net/sf/xplanner/domain/Note.java Note#getParent; SRC:src/com/technoetic/xplanner/tags/DomainContext.java DomainContext#getNoteTarget; SRC:src/com/technoetic/xplanner/db/OLDIdSearchHelper.java OLDIdSearchHelper#search. IdSearchHelper#search tries Project, Iteration, UserStory, Task, Person and Note in that order and, when the object is a Note, returns Note#getParent instead: the object whose id is the note's attached-to id, looked up the same way (a failed lookup gives null). Bytecode listings agree; the thread session is bound by SRC:src/com/technoetic/xplanner/db/hibernate/HibernateSessionFilter.java HibernateSessionFilter#doFilter before the filter chain, mapped at /* (WAR:WEB-INF/web.xml:147-152). Status stays Yes on this reading. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-041, C-C-042, E-C-005, E-C-006, E-C-007, E-C-008).</t>
   </si>
   <si>
     <t>Submitting an empty search yields an error.</t>
@@ -2323,10 +2326,10 @@
     <t>Guides the user to enter text.</t>
   </si>
   <si>
-    <t>General error page "Invalid content specified for search.: missing content" (text in the Accept-Language locale; bundles without contentsearch.invalid_id fall back to the default text).</t>
-  </si>
-  <si>
-    <t>class ContentSearchAction#produceException (strings "missing content", "contentsearch.invalid_id"). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute, #produceException. WAR: classes byte-identical to the v1.1a4 release. An empty search text forwards to the general error page with the message of contentsearch.invalid_id followed by ": missing content", resolved in the request (Accept-Language) locale; the key is missing in da, es, fr, it, pt_br and ru.</t>
+    <t>General error page "An error has occurred." without the contentsearch.invalid_id text ("Invalid content specified for search.: missing content" is not shown), in en and de sessions (W001).</t>
+  </si>
+  <si>
+    <t>class ContentSearchAction#produceException (strings "missing content", "contentsearch.invalid_id"). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute, #produceException. WAR: classes byte-identical to the v1.1a4 release. An empty search text forwards to the general error page with the message of contentsearch.invalid_id followed by ": missing content", resolved in the request (Accept-Language) locale; the key is missing in da, es, fr, it, pt_br and ru. Stage 3 W001 (BA-001-13, MC-A-36, W001-F-42): empty header search: 200, general error page, 0 matches for "Invalid content specified" and "missing content" (C-C-043). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks C-C-043).</t>
   </si>
   <si>
     <t>Jump to object by ID</t>
@@ -2341,7 +2344,7 @@
     <t>Search results headed by the object with that id (for a note's id, the note's parent); a request to /do/search/id?searchedId=&lt;id&gt; redirects to /do/view/&lt;type&gt;?oid=&lt;id&gt; of the found object, which for a note's id are the parent's type and id.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:46 (tooltip "search by word or ID"); class ContentSearchAction (setIdSearchHelper); class IdSearchAction (strings "/do/view/", "?oid="); WAR:WEB-INF/struts-config.xml:141,413 (search/id). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute; SRC:src/com/technoetic/xplanner/actions/IdSearchAction.java IdSearchAction#doExecute. WAR: classes byte-identical to the v1.1a4 release; baseHeader.jsp of the WAR (differs from the SVN copy; WAR governs). The header search box posts to /do/search/content: a numeric text lists the object with that id first among the search results, without a redirect. The redirecting ID search (/do/search/id, IdSearchAction) is linked from no page of the WAR. Correction (BA-001-12, pass-010 F-002): method-level reading of the corrected claim: SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search; SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute; SRC:src/com/technoetic/xplanner/actions/IdSearchAction.java IdSearchAction#doExecute (builds the redirect from the class of the returned object through DomainMetaDataRepository#classToTypeName and from its getId); SRC:src/net/sf/xplanner/domain/Note.java Note#getParent; SRC:src/com/technoetic/xplanner/tags/DomainContext.java DomainContext#getNoteTarget; SRC:src/com/technoetic/xplanner/db/OLDIdSearchHelper.java OLDIdSearchHelper#search. IdSearchHelper#search tries Project, Iteration, UserStory, Task, Person and Note in that order and, when the object is a Note, returns Note#getParent instead: the object whose id is the note's attached-to id, looked up the same way (a failed lookup gives null). Bytecode listings agree; the thread session is bound by SRC:src/com/technoetic/xplanner/db/hibernate/HibernateSessionFilter.java HibernateSessionFilter#doFilter before the filter chain, mapped at /* (WAR:WEB-INF/web.xml:147-152). Status stays Yes on this reading.</t>
+    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:46 (tooltip "search by word or ID"); class ContentSearchAction (setIdSearchHelper); class IdSearchAction (strings "/do/view/", "?oid="); WAR:WEB-INF/struts-config.xml:141,413 (search/id). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute; SRC:src/com/technoetic/xplanner/actions/IdSearchAction.java IdSearchAction#doExecute. WAR: classes byte-identical to the v1.1a4 release; baseHeader.jsp of the WAR (differs from the SVN copy; WAR governs). The header search box posts to /do/search/content: a numeric text lists the object with that id first among the search results, without a redirect. The redirecting ID search (/do/search/id, IdSearchAction) is linked from no page of the WAR. Correction (BA-001-12, pass-010 F-002): method-level reading of the corrected claim: SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search; SRC:src/com/technoetic/xplanner/actions/ContentSearchAction.java ContentSearchAction#doExecute; SRC:src/com/technoetic/xplanner/actions/IdSearchAction.java IdSearchAction#doExecute (builds the redirect from the class of the returned object through DomainMetaDataRepository#classToTypeName and from its getId); SRC:src/net/sf/xplanner/domain/Note.java Note#getParent; SRC:src/com/technoetic/xplanner/tags/DomainContext.java DomainContext#getNoteTarget; SRC:src/com/technoetic/xplanner/db/OLDIdSearchHelper.java OLDIdSearchHelper#search. IdSearchHelper#search tries Project, Iteration, UserStory, Task, Person and Note in that order and, when the object is a Note, returns Note#getParent instead: the object whose id is the note's attached-to id, looked up the same way (a failed lookup gives null). Bytecode listings agree; the thread session is bound by SRC:src/com/technoetic/xplanner/db/hibernate/HibernateSessionFilter.java HibernateSessionFilter#doFilter before the filter chain, mapped at /* (WAR:WEB-INF/web.xml:147-152). Status stays Yes on this reading. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-044).</t>
   </si>
   <si>
     <t>A missing, malformed or unknown ID shows an error.</t>
@@ -2353,7 +2356,7 @@
     <t>Messages idsearch.error.missingId, badId, idNotFound.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.actions.IdSearchAction#doExecute (idsearch.error.missingId, idsearch.error.badId, idsearch.error.idNotFound). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/IdSearchAction.java IdSearchAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. An empty, non-numeric or unknown id returns the general error forward with the three keys; they exist only in the default and "--" bundles.</t>
+    <t>class com.technoetic.xplanner.actions.IdSearchAction#doExecute (idsearch.error.missingId, idsearch.error.badId, idsearch.error.idNotFound). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/IdSearchAction.java IdSearchAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. An empty, non-numeric or unknown id returns the general error forward with the three keys; they exist only in the default and "--" bundles. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-045).</t>
   </si>
   <si>
     <t>Jumping by ID applies no read-permission check, unlike text search; the target view page does not check either.</t>
@@ -2365,7 +2368,7 @@
     <t>Any existing object ID opens the page of that object, or for a note's ID the page of the note's parent, for any signed-in user (runtime unverified).</t>
   </si>
   <si>
-    <t>classes IdSearchAction and ViewObjectAction: no authorization call reachable (.migration-tmp/stage-01/out/authtrace.json). BA-001-03 impact sweep of F-001 and F-007. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/IdSearchAction.java IdSearchAction#doExecute; SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search; SRC:src/com/technoetic/xplanner/actions/ViewObjectAction.java ViewObjectAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. Neither the ID search nor the view action calls an authorizer. Correction (BA-001-12, pass-010 F-002): the page opened is that of the object returned by SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search; for a note's id this is the note's parent (SRC:src/net/sf/xplanner/domain/Note.java Note#getParent; SRC:src/com/technoetic/xplanner/tags/DomainContext.java DomainContext#getNoteTarget; SRC:src/com/technoetic/xplanner/db/OLDIdSearchHelper.java OLDIdSearchHelper#search). The missing read check is unchanged.</t>
+    <t>classes IdSearchAction and ViewObjectAction: no authorization call reachable (.migration-tmp/stage-01/out/authtrace.json). BA-001-03 impact sweep of F-001 and F-007. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/IdSearchAction.java IdSearchAction#doExecute; SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search; SRC:src/com/technoetic/xplanner/actions/ViewObjectAction.java ViewObjectAction#doExecute. WAR: classes byte-identical to the v1.1a4 release. Neither the ID search nor the view action calls an authorizer. Correction (BA-001-12, pass-010 F-002): the page opened is that of the object returned by SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search; for a note's id this is the note's parent (SRC:src/net/sf/xplanner/domain/Note.java Note#getParent; SRC:src/com/technoetic/xplanner/tags/DomainContext.java DomainContext#getNoteTarget; SRC:src/com/technoetic/xplanner/db/OLDIdSearchHelper.java OLDIdSearchHelper#search). The missing read check is unchanged. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-046, E-C-009, E-C-010, E-C-011).</t>
   </si>
   <si>
     <t>Breadcrumb navigation</t>
@@ -2380,7 +2383,7 @@
     <t>Breadcrumb links above the page content.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/tags/breadcrumb.tag; class net.sf.xplanner.tags.NavigationBarTag#render (strings "navigation.top", project, iteration, userstory, task, feature); layouts viewLayout.jsp:59, defaultLayout.jsp:44, defaultEditLayout.jsp:55. Request-driven lookup (BA-001-10, pass-008 F-002 lead, check (l)): NavigationBarTag#doEndTag reads the request parameter oid, or else fkey. Because breadcrumb.tag passes type="${objectType}", which is an empty string when the attribute is unset, #setObject(int) looks the id up with IdSearchHelper#search (Session#get over Project, Iteration, UserStory, Task, Person and Note; WAR:WEB-INF/classes/spring-dao.xml:61) and applies no permission check. The link texts are the stored names of the hierarchy and are printed with unescaped EL (WAR:WEB-INF/tags/breadcrumb.tag:15,18). On signed-in pages this adds no exposure beyond the missing read checks (rows 29-30); on the public login and error pages it runs before sign-in (rows 8, 56; Inferred; GAP-007; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/net/sf/xplanner/tags/NavigationBarTag.java NavigationBarTag#render, #doEndTag; SRC:src/com/technoetic/xplanner/tags/NavigationBarTag.java NavigationBarTag#doEndTag; SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim.</t>
+    <t>WAR:WEB-INF/tags/breadcrumb.tag; class net.sf.xplanner.tags.NavigationBarTag#render (strings "navigation.top", project, iteration, userstory, task, feature); layouts viewLayout.jsp:59, defaultLayout.jsp:44, defaultEditLayout.jsp:55. Request-driven lookup (BA-001-10, pass-008 F-002 lead, check (l)): NavigationBarTag#doEndTag reads the request parameter oid, or else fkey. Because breadcrumb.tag passes type="${objectType}", which is an empty string when the attribute is unset, #setObject(int) looks the id up with IdSearchHelper#search (Session#get over Project, Iteration, UserStory, Task, Person and Note; WAR:WEB-INF/classes/spring-dao.xml:61) and applies no permission check. The link texts are the stored names of the hierarchy and are printed with unescaped EL (WAR:WEB-INF/tags/breadcrumb.tag:15,18). On signed-in pages this adds no exposure beyond the missing read checks (rows 29-30); on the public login and error pages it runs before sign-in (rows 8, 56; Inferred; GAP-007; Q3 facts). Source reconciliation (BA-001-11, A4): confirmed at name level. SRC:src/net/sf/xplanner/tags/NavigationBarTag.java NavigationBarTag#render, #doEndTag; SRC:src/com/technoetic/xplanner/tags/NavigationBarTag.java NavigationBarTag#doEndTag; SRC:src/com/technoetic/xplanner/db/IdSearchHelper.java IdSearchHelper#search. WAR: classes byte-identical to the v1.1a4 release. The claim rests on the WAR descriptors, JSPs and bytecode already cited; the cited source classes and methods exist by name and nothing read contradicts the claim. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-047).</t>
   </si>
   <si>
     <t>Object and project history</t>
@@ -2392,22 +2395,22 @@
     <t>Audit trail of recorded changes.</t>
   </si>
   <si>
-    <t>Sortable history table; the container view adds object type and name links. The "when" dates use the built-in pattern "EEE MMM dd k:mm:ss z" in the Accept-Language locale of the first request after start-up that renders a history date, for every later user (Inferred).</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/project.jsp:99-104, iteration/globalLinks.jsp:41-45, userstory.jsp, task.jsp (links /do/view/history, container flag for projects); WAR:WEB-INF/struts-config.xml:396-398; WAR:WEB-INF/jsp/view/history.jsp:30-32 (HistorySupport#getEvents) and :71-73 (#getContainerEvents); class com.technoetic.xplanner.history.HistorySupport#getContainerEvents (strings "created", "deleted"); WAR:WEB-INF/classes/spring-dao.xml:63-65 (historySupport); db-changelog.xml table history. Corrected in BA-001-03 (stage-02-pass-001 F-002). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/history/HistorySupport.java HistorySupport#getEvents, #getContainerEvents; SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag. WAR: classes byte-identical to the v1.1a4 release; history.jsp of the WAR (differs from the SVN copy, which calls HistorySupport statically; the WAR page calls the historySupport bean; WAR governs). The "when" column (history.jsp:61,106) uses xplanner:formatDate without format or formatKey: FormatDateTag uses its built-in pattern "EEE MMM dd k:mm:ss z" and keeps one SimpleDateFormat per pattern in a static, unsynchronized map, created with request.getLocale() (Accept-Language) of the first request after start-up, so later users see day and month names in that first locale (bytecode listing agrees). Resolves carried pass-009 F-002 statically (Inferred for the runtime effect). Live question: After a fresh start, which language do the history dates show for a second session with a different Accept-Language? Correction (BA-001-12, pass-010 F-003): the formatter for the built-in pattern is created by the first request that renders a history date (the only formatDate uses without format or formatKey are WAR:WEB-INF/jsp/view/history.jsp:61,106), not by the first request after start-up. SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag.</t>
-  </si>
-  <si>
-    <t>History is written only by these entry points: web iteration start and close, story move/continue (including multi-move and continue unfinished stories), task move/continue and task re-estimate; and every SOAP add, update and remove ("created", "updated", "deleted"). Web create, edit and delete of projects, iterations, stories, tasks, notes, people and settings write no history.</t>
+    <t>Sortable history table; the container view adds object type and name links. The "when" dates use the built-in pattern "EEE MMM dd k:mm:ss z" in the Accept-Language locale of the first request after start-up that renders a history date, for every later user (Inferred). The column headings (action, by, when, description; in the container view also type and name) are always in the server default locale: history.jsp takes them through messages.getMessage(key) without a locale, while the page title and heading follow the session bundle; the es bundle has no history keys and falls back to English (W001).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/project.jsp:99-104, iteration/globalLinks.jsp:41-45, userstory.jsp, task.jsp (links /do/view/history, container flag for projects); WAR:WEB-INF/struts-config.xml:396-398; WAR:WEB-INF/jsp/view/history.jsp:30-32 (HistorySupport#getEvents) and :71-73 (#getContainerEvents); class com.technoetic.xplanner.history.HistorySupport#getContainerEvents (strings "created", "deleted"); WAR:WEB-INF/classes/spring-dao.xml:63-65 (historySupport); db-changelog.xml table history. Corrected in BA-001-03 (stage-02-pass-001 F-002). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/history/HistorySupport.java HistorySupport#getEvents, #getContainerEvents; SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag. WAR: classes byte-identical to the v1.1a4 release; history.jsp of the WAR (differs from the SVN copy, which calls HistorySupport statically; the WAR page calls the historySupport bean; WAR governs). The "when" column (history.jsp:61,106) uses xplanner:formatDate without format or formatKey: FormatDateTag uses its built-in pattern "EEE MMM dd k:mm:ss z" and keeps one SimpleDateFormat per pattern in a static, unsynchronized map, created with request.getLocale() (Accept-Language) of the first request after start-up, so later users see day and month names in that first locale (bytecode listing agrees). Resolves carried pass-009 F-002 statically (Inferred for the runtime effect). Live question: After a fresh start, which language do the history dates show for a second session with a different Accept-Language? Correction (BA-001-12, pass-010 F-003): the formatter for the built-in pattern is created by the first request that renders a history date (the only formatDate uses without format or formatKey are WAR:WEB-INF/jsp/view/history.jsp:61,106), not by the first request after start-up. SRC:src/com/technoetic/xplanner/tags/FormatDateTag.java FormatDateTag#doStartTag. Stage 3 W001 (BA-001-13, MC-B-07, W001-F-43): history views in en, de and es sessions: title and h1 follow the session bundle ("Historie"/"Ereignis" in de), the column headings stay English although the de bundle defines them (C-C-049); the same for other dt:table column titles and the displaytag banner (C-C-002). WAR:WEB-INF/jsp/view/history.jsp:52-63,97-111 (column titles from messages.getMessage without a locale). Stage 3 W001 live answer (BA-001-13, MC-C-22): The first requester's locale (German day names) for every later session; no fresh restart was done (see row 69) (C-C-001, C-C-002). The restart case stays residual (R-33). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks C-C-001, C-C-002, C-C-048, C-C-049; open residual scope R-33 (e)).</t>
+  </si>
+  <si>
+    <t>History is written only by these entry points: web iteration start and close, story move/continue (including multi-move and continue unfinished stories), task move/continue and task re-estimate; and every SOAP add, update and remove ("created", "updated", "deleted"). Web create, edit and delete of projects, iterations, stories, tasks, notes, people and settings write no history. In this baseline the task move/continue entry points write no history, because they fail with HTTP 500 before saving (row 144, W001).</t>
   </si>
   <si>
     <t>Explains which changes appear in the audit trail; web edits leave none, and the container view therefore shows only SOAP-made creations and deletions.</t>
   </si>
   <si>
-    <t>No history entry after a web edit or delete (runtime unverified).</t>
-  </si>
-  <si>
-    <t>Callers of com.technoetic.xplanner.history.HistorySupport#saveEvent reachable per entry point in .migration-tmp/stage-01/out/authtrace.json: StartIterationAction, CloseIterationAction, MoveContinueStoryAction, MoveStoriesAction and ContinueUnfinishedStoriesAction (via MoveContinueStory and Continuer), MoveContinueTaskAction, UpdateTimeAction#doUpdateEstimateAction ("reestimated"), SOAP XPlanner#addObject/#updateObject/#removeObject (#saveHistory; strings "created", "updated", "deleted"); none from EditObjectAction or DeleteObjectAction, which only publish events that no registered listener receives. Source: stage-02-pass-001 F-002. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/history/HistorySupport.java HistorySupport#saveEvent (callers: StartIterationAction, CloseIterationAction, Continuer, MoveContinueStory, MoveContinueTaskAction, UpdateTimeAction, soap/XPlanner); SRC:src/net/sf/xplanner/events/EventManager.java EventManager (publishes Spring application events); SRC:src/net/sf/xplanner/email/EmailPerChangeListener.java (the only ApplicationListener; no bean). WAR: classes byte-identical to the v1.1a4 release. The source callers of saveEvent are exactly the recorded entry points; the generic web edit and delete only publish events, and no listener bean receives them.</t>
+    <t>No history entry after a web create or edit (observed in W001; a web delete was not observed); task Move and Continue write none either, because they fail with HTTP 500 before saving (row 144).</t>
+  </si>
+  <si>
+    <t>Callers of com.technoetic.xplanner.history.HistorySupport#saveEvent reachable per entry point in .migration-tmp/stage-01/out/authtrace.json: StartIterationAction, CloseIterationAction, MoveContinueStoryAction, MoveStoriesAction and ContinueUnfinishedStoriesAction (via MoveContinueStory and Continuer), MoveContinueTaskAction, UpdateTimeAction#doUpdateEstimateAction ("reestimated"), SOAP XPlanner#addObject/#updateObject/#removeObject (#saveHistory; strings "created", "updated", "deleted"); none from EditObjectAction or DeleteObjectAction, which only publish events that no registered listener receives. Source: stage-02-pass-001 F-002. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/history/HistorySupport.java HistorySupport#saveEvent (callers: StartIterationAction, CloseIterationAction, Continuer, MoveContinueStory, MoveContinueTaskAction, UpdateTimeAction, soap/XPlanner); SRC:src/net/sf/xplanner/events/EventManager.java EventManager (publishes Spring application events); SRC:src/net/sf/xplanner/email/EmailPerChangeListener.java (the only ApplicationListener; no bean). WAR: classes byte-identical to the v1.1a4 release. The source callers of saveEvent are exactly the recorded entry points; the generic web edit and delete only publish events, and no listener bean receives them. Stage 3 W001 (BA-001-13, MC-A-29, W001-F-34): C-C-050: no history for web creates and a task edit; "started", "moved" (with moved out/in) and "reestimated" written; task Move and Continue answer HTTP 500 (MoveContinueTaskAction.saveForm) and write nothing. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks C-C-050).</t>
   </si>
   <si>
     <t>My status page</t>
@@ -2422,7 +2425,7 @@
     <t>Page /setting/me/status/&lt;personId&gt; with the same sections as the person page.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:17 (link ${appUrl}/setting/me/status/${person.id}); class net.sf.xplanner.web.MePage (@RequestMapping "/me/status/{id}", view "view/meStatus"); WAR:WEB-INF/jsp/view/meStatus.jsp; WAR:WEB-INF/classes/spring-web.xml. The link base appUrl comes from xplanner.application.url (class net.sf.xplanner.context.ContextLoaderListener; effective value http://localhost:8080/xplanner in xplanner-custom.properties:30), so the link target depends on that configured URL. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/net/sf/xplanner/web/MePage.java MePage. WAR: classes byte-identical to the v1.1a4 release; baseHeader.jsp of the WAR links through xplanner:link with the application URL (the SVN copy uses html:link; WAR governs). The controller is component-scanned with its DAO and repository fields autowired. Provenance (fixed baseline, see reconnaissance GAP-005): P-04: the cited value is read from xplanner-custom.properties (rewritten entry, known patch target); upstream value not determinable.</t>
+    <t>WAR:WEB-INF/jsp/common/baseHeader.jsp:17 (link ${appUrl}/setting/me/status/${person.id}); class net.sf.xplanner.web.MePage (@RequestMapping "/me/status/{id}", view "view/meStatus"); WAR:WEB-INF/jsp/view/meStatus.jsp; WAR:WEB-INF/classes/spring-web.xml. The link base appUrl comes from xplanner.application.url (class net.sf.xplanner.context.ContextLoaderListener; effective value http://localhost:8080/xplanner in xplanner-custom.properties:30), so the link target depends on that configured URL. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/net/sf/xplanner/web/MePage.java MePage. WAR: classes byte-identical to the v1.1a4 release; baseHeader.jsp of the WAR links through xplanner:link with the application URL (the SVN copy uses html:link; WAR governs). The controller is component-scanned with its DAO and repository fields autowired. Provenance (fixed baseline, see reconnaissance GAP-005): P-04: the cited value is read from xplanner-custom.properties (rewritten entry, known patch target); upstream value not determinable. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-051).</t>
   </si>
   <si>
     <t>Wiki-style formatting of descriptions</t>
@@ -2437,7 +2440,7 @@
     <t>Formatted HTML with links; bracket escaping can be enabled per project.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/xplanner.tld (twiki -&gt; com.technoetic.xplanner.tags.TwikiTag); WAR:WEB-INF/classes/xplanner.properties:92-127 (twiki.scheme.*, GenericWikiAdapter); package com.technoetic.xplanner.wiki (11 classes). Server-side request (BA-001-06): TwikiTag builds com.technoetic.xplanner.wiki.TwikiFormat, which instantiates the adapter class named by twiki.wikiadapter (WAR:WEB-INF/classes/xplanner.properties:113, GenericWikiAdapter) and calls ExternalWikiAdapter#formatWikiWord for each WikiWord; GenericWikiAdapter#formatWikiWord calls #isTopicExisting, which opens new URL(topic.url.existing with the word).openStream() (:114, http://localhost:9090/vqw/...) and reads it; no connect or read timeout is set. Existing topics are cached; an IOException returns false, so the word is rendered as a new-topic link and is requested again on the next rendering (bytecode listing with exception table). Rendering a description with a WikiWord is therefore expected to make an outbound HTTP request and to wait for it (runtime unverified). Provenance of the URL: GAP-005 P-03. Source: stage-02-pass-004 F-006. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/tags/TwikiTag.java TwikiTag; SRC:src/com/technoetic/xplanner/wiki/TwikiFormat.java TwikiFormat#format; SRC:src/com/technoetic/xplanner/wiki/GenericWikiAdapter.java GenericWikiAdapter#formatWikiWord. WAR: classes byte-identical to the v1.1a4 release; wiki settings from the patched WAR xplanner.properties. The rendering path is as recorded; the result of the many format rules and of the external wiki lookup is not established without rendering. Live question: How are a description with TWiki markup, a WikiWord and an object link (story:&lt;id&gt;) rendered? Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/xplanner.tld (twiki -&gt; com.technoetic.xplanner.tags.TwikiTag); WAR:WEB-INF/classes/xplanner.properties:92-127 (twiki.scheme.*, GenericWikiAdapter); package com.technoetic.xplanner.wiki (11 classes). Server-side request (BA-001-06): TwikiTag builds com.technoetic.xplanner.wiki.TwikiFormat, which instantiates the adapter class named by twiki.wikiadapter (WAR:WEB-INF/classes/xplanner.properties:113, GenericWikiAdapter) and calls ExternalWikiAdapter#formatWikiWord for each WikiWord; GenericWikiAdapter#formatWikiWord calls #isTopicExisting, which opens new URL(topic.url.existing with the word).openStream() (:114, http://localhost:9090/vqw/...) and reads it; no connect or read timeout is set. Existing topics are cached; an IOException returns false, so the word is rendered as a new-topic link and is requested again on the next rendering (bytecode listing with exception table). Rendering a description with a WikiWord is therefore expected to make an outbound HTTP request and to wait for it (runtime unverified). Provenance of the URL: GAP-005 P-03. Source: stage-02-pass-004 F-006. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/tags/TwikiTag.java TwikiTag; SRC:src/com/technoetic/xplanner/wiki/TwikiFormat.java TwikiFormat#format; SRC:src/com/technoetic/xplanner/wiki/GenericWikiAdapter.java GenericWikiAdapter#formatWikiWord. WAR: classes byte-identical to the v1.1a4 release; wiki settings from the patched WAR xplanner.properties. The rendering path is as recorded; the result of the many format rules and of the external wiki lookup is not established without rendering. Live question: How are a description with TWiki markup, a WikiWord and an object link (story:&lt;id&gt;) rendered? Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. Stage 3 W001 live answer (BA-001-13, MC-C-23): Bold, italic and fixed text become HTML; the WikiWord gets a "?" link to the external wiki edit page (localhost:9090); story:&lt;id&gt; and task:&lt;id&gt; become links with the object names; [[...]] stays literal (C-C-052). The status stays Inferred: per-project bracket escaping (R-27) and the server-side topic lookup (R-47) were not observed. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks C-C-052, F-C-014; open residual scope R-27 (d), R-47 (e)).</t>
   </si>
   <si>
     <t>Editors show a formatting-help link to a TWiki formatting reference page.</t>
@@ -2449,7 +2452,7 @@
     <t>Help page describing the markup.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/common/formattingHelpLink.jsp (hard-coded /xplanner/do/view/twikiformat, which does not match the WAR context path /xplanner-plus in META-INF/context.xml); WAR:WEB-INF/struts-config.xml:177; WAR:WEB-INF/jsp/view/twikiformat.jsp. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: JSP and descriptor fact. WAR: formattingHelpLink.jsp and META-INF/context.xml identical to the SVN webapp copies. The link hard-codes /xplanner while the context path is /xplanner-plus.</t>
+    <t>WAR:WEB-INF/jsp/common/formattingHelpLink.jsp (hard-coded /xplanner/do/view/twikiformat, which does not match the WAR context path /xplanner-plus in META-INF/context.xml); WAR:WEB-INF/struts-config.xml:177; WAR:WEB-INF/jsp/view/twikiformat.jsp. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: JSP and descriptor fact. WAR: formattingHelpLink.jsp and META-INF/context.xml identical to the SVN webapp copies. The link hard-codes /xplanner while the context path is /xplanner-plus. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-053).</t>
   </si>
   <si>
     <t>Switch page width</t>
@@ -2464,7 +2467,7 @@
     <t>Page toggles between normal and wide layout; preference persists across pages via browser localStorage.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/common/footer.jsp:11-14 (page_footer, wider.png, label); WAR:js/global.js:1-10 (click on .page_footer toggles class wide, localStorage.widescreen); included by layouts defaultLayout.jsp:41 and defaultEditLayout.jsp:52. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/jsp/common/footer.jsp:11-14 (page_footer, wider.png, label); WAR:js/global.js:1-10 (click on .page_footer toggles class wide, localStorage.widescreen); included by layouts defaultLayout.jsp:41 and defaultEditLayout.jsp:52. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-054, E-C-026).</t>
   </si>
   <si>
     <t>Any page built with the xplanner:content tag is rendered with the print layout (no header, no footer) when the request carries a print parameter, for example ?print=true; no page links to this mode, so it is reachable by URL only.</t>
@@ -2476,7 +2479,7 @@
     <t>Page body without the header and footer tiles.</t>
   </si>
   <si>
-    <t>class com.technoetic.xplanner.tags.ContentTag#doStartTag calls PrintLinkTag#isInPrintMode, which returns true when ServletRequest.getParameter("print") is not null, and then inserts the Tiles definition "tiles:print" (bytecode listings); WAR:WEB-INF/tiles-definitions.xml:23-28 (tiles:print extends tiles:view with displayMode print and empty header and footer). xplanner:content has 43 live opening tags in 43 JSPs (comment-blanked count); the printLink tag (WAR:WEB-INF/xplanner.tld:707-708) is used by no JSP. Request-parameter sweep of all tag classes (.migration-tmp/stage-01/out/render-side-effects-06.txt): print is the only parameter that switches the layout. Source: stage-02-pass-004 F-004. Related switch (BA-001-07, mechanism (b)): the Spring MVC Tiles definition viewLayout (WAR:WEB-INF/tiles-pages.xml:6) uses WAR:WEB-INF/jsp/layout/viewLayoutNew.jsp, which compares ${param.mode} with print (:15) and then omits the sections guarded by isScreenMode (:47, :84, :93); the value is compared only, not written. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/tags/ContentTag.java ContentTag#doStartTag; SRC:src/com/technoetic/xplanner/tags/PrintLinkTag.java PrintLinkTag#isInPrintMode. WAR: classes byte-identical to the v1.1a4 release. Any non-null print parameter selects tiles:print; otherwise a missing definition becomes tiles:default and a caller-given one is kept.</t>
+    <t>class com.technoetic.xplanner.tags.ContentTag#doStartTag calls PrintLinkTag#isInPrintMode, which returns true when ServletRequest.getParameter("print") is not null, and then inserts the Tiles definition "tiles:print" (bytecode listings); WAR:WEB-INF/tiles-definitions.xml:23-28 (tiles:print extends tiles:view with displayMode print and empty header and footer). xplanner:content has 43 live opening tags in 43 JSPs (comment-blanked count); the printLink tag (WAR:WEB-INF/xplanner.tld:707-708) is used by no JSP. Request-parameter sweep of all tag classes (.migration-tmp/stage-01/out/render-side-effects-06.txt): print is the only parameter that switches the layout. Source: stage-02-pass-004 F-004. Related switch (BA-001-07, mechanism (b)): the Spring MVC Tiles definition viewLayout (WAR:WEB-INF/tiles-pages.xml:6) uses WAR:WEB-INF/jsp/layout/viewLayoutNew.jsp, which compares ${param.mode} with print (:15) and then omits the sections guarded by isScreenMode (:47, :84, :93); the value is compared only, not written. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/tags/ContentTag.java ContentTag#doStartTag; SRC:src/com/technoetic/xplanner/tags/PrintLinkTag.java PrintLinkTag#isInPrintMode. WAR: classes byte-identical to the v1.1a4 release. Any non-null print parameter selects tiles:print; otherwise a missing definition becomes tiles:default and a caller-given one is kept. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-055).</t>
   </si>
   <si>
     <t>Share on social networks</t>
@@ -2491,7 +2494,7 @@
     <t>Twitter and Facebook share icons open the external sites; no like widget, no LinkedIn link.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/jsp/layout/viewLayout.jsp:73-88 (twitter.com/home?status=..., facebook.com/dialog/feed with app_id and page URL) and :92-95 (HTML comment "&lt;!-- a class=\"in\" ... &lt;/span --&gt;" enclosing the LinkedIn link, the connect.facebook.net script and fb:like); the same comment in WAR:WEB-INF/jsp/layout/viewLayoutNew.jsp:114-117. Corrected in BA-001-04 (Source: stage-02-pass-002 F-003). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/jsp/layout/viewLayout.jsp:73-88 (twitter.com/home?status=..., facebook.com/dialog/feed with app_id and page URL) and :92-95 (HTML comment "&lt;!-- a class=\"in\" ... &lt;/span --&gt;" enclosing the LinkedIn link, the connect.facebook.net script and fb:like); the same comment in WAR:WEB-INF/jsp/layout/viewLayoutNew.jsp:114-117. Corrected in BA-001-04 (Source: stage-02-pass-002 F-003). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks C-C-056; open residual scope R-36 (e)).</t>
   </si>
   <si>
     <t>Features (story features)</t>
@@ -2506,7 +2509,7 @@
     <t>Pages reachable only by URL; runtime behaviour expected to fail.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:185-187,207-209,215-217,259-263; WAR:WEB-INF/action-servlet.xml:96-100,202-212 (type net.sf.xplanner.domain.Feature - class ABSENT from WAR); class com.technoetic.xplanner.domain.Feature has no @Entity; WAR:WEB-INF/classes/mappings/Feature.xml not loaded (spring-beans.xml:80 loads only Metrics.xml); iteration/links.jsp:32-35 commented; pages WAR:WEB-INF/jsp/view/projectFeatures.jsp, WAR:WEB-INF/jsp/view/iterationFeatures.jsp, WAR:WEB-INF/jsp/view/feature.jsp (uses com.technoetic.xplanner.domain.Feature), WAR:WEB-INF/jsp/edit/editFeature.jsp; class FeatureEditorForm#validate (feature.editor.missing_name). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editFeature.jsp writes the raw request parameters oid (29), returnto (32), fkey (34,35) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/domain/Feature.java Feature (no @Entity); SRC:src/com/technoetic/xplanner/forms/FeatureEditorForm.java FeatureEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release; net.sf.xplanner.domain.Feature absent from both the WAR and the SVN source. The type named by the action beans does not exist in the source either, and the old Feature class is not mapped. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the "not mapped" conclusion rests on spring-beans.xml:80 (rewritten entry) and is corroborated independently by the compiled class com.technoetic.xplanner.db.hibernate.HibernateHelper, whose mapped-class list also omits this class.</t>
+    <t>WAR:WEB-INF/struts-config.xml:185-187,207-209,215-217,259-263; WAR:WEB-INF/action-servlet.xml:96-100,202-212 (type net.sf.xplanner.domain.Feature - class ABSENT from WAR); class com.technoetic.xplanner.domain.Feature has no @Entity; WAR:WEB-INF/classes/mappings/Feature.xml not loaded (spring-beans.xml:80 loads only Metrics.xml); iteration/links.jsp:32-35 commented; pages WAR:WEB-INF/jsp/view/projectFeatures.jsp, WAR:WEB-INF/jsp/view/iterationFeatures.jsp, WAR:WEB-INF/jsp/view/feature.jsp (uses com.technoetic.xplanner.domain.Feature), WAR:WEB-INF/jsp/edit/editFeature.jsp; class FeatureEditorForm#validate (feature.editor.missing_name). Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/edit/editFeature.jsp writes the raw request parameters oid (29), returnto (32), fkey (34,35) [parameter (lines)] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/domain/Feature.java Feature (no @Entity); SRC:src/com/technoetic/xplanner/forms/FeatureEditorForm.java FeatureEditorForm#validate. WAR: classes byte-identical to the v1.1a4 release; net.sf.xplanner.domain.Feature absent from both the WAR and the SVN source. The type named by the action beans does not exist in the source either, and the old Feature class is not mapped. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the "not mapped" conclusion rests on spring-beans.xml:80 (rewritten entry) and is corroborated independently by the compiled class com.technoetic.xplanner.db.hibernate.HibernateHelper, whose mapped-class list also omits this class. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks C-C-057).</t>
   </si>
   <si>
     <t>UF-012</t>
@@ -2524,10 +2527,10 @@
     <t>Serialise code integrations in an XP team.</t>
   </si>
   <si>
-    <t>Integration page with Start/Finished/Cancel buttons and a join form.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/struts-config.xml:388-394; WAR:WEB-INF/action-servlet.xml:390-392; WAR:WEB-INF/jsp/view/integrations.jsp; class com.technoetic.xplanner.actions.IntegrationAction (action.join, action.start, action.finish, action.cancel, action.leave). The used class com.technoetic.xplanner.domain.Integration has no @Entity and mappings/Integration.xml is not loaded; no live link to /do/view/integrations found. Server-side enforcement (CHK-002, BA-001-04): the view (DispatchForward) requires a projectId and system.project read (row 28); the join/start/finish/cancel/leave requests (IntegrationAction) perform no server-side permission check that gates the change (the only authorization call on the path is the recipient lookup inside the e-mail notifier), and the "integrate" condition only hides the buttons. Query property paths (BA-001-05): IntegrationAction#getIntegrationsInState and the three useBeans tags of WAR:WEB-INF/jsp/view/integrations.jsp (lines 23, 29, 155) query com.technoetic.xplanner.domain.Integration, which is not a mapped entity (GAP-004). Sweep of pass-003 F-001. Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/view/integrations.jsp writes the raw request parameters projectId (36) [parameter (lines); lines 26, 32 and 160 bind it as a query parameter] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/domain/Integration.java Integration (no @Entity); SRC:src/com/technoetic/xplanner/actions/IntegrationAction.java IntegrationAction#onJoinRequest, #onStartRequest. WAR: classes byte-identical to the v1.1a4 release; src/mappings/Integration.xml exists in the source but is not loaded by the WAR spring-beans.xml. The page and actions exist; the entity is neither annotated nor mapped by a loaded file. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the "not mapped" conclusion rests on spring-beans.xml:80 (rewritten entry) and is corroborated independently by the compiled class com.technoetic.xplanner.db.hibernate.HibernateHelper, whose mapped-class list also omits this class.</t>
+    <t>HTTP 500 error page (JspTagException, IllegalArgumentException "No positional parameters in query: from com.technoetic.xplanner.domain.Integration where state = ? and projectId = ?"): the queue page never renders in this baseline, and every /do/edit/integrations request (join, start, finish, cancel, leave) fails the same way, for viewer and editor (W001).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/struts-config.xml:388-394; WAR:WEB-INF/action-servlet.xml:390-392; WAR:WEB-INF/jsp/view/integrations.jsp; class com.technoetic.xplanner.actions.IntegrationAction (action.join, action.start, action.finish, action.cancel, action.leave). The used class com.technoetic.xplanner.domain.Integration has no @Entity and mappings/Integration.xml is not loaded; no live link to /do/view/integrations found. Server-side enforcement (CHK-002, BA-001-04): the view (DispatchForward) requires a projectId and system.project read (row 28); the join/start/finish/cancel/leave requests (IntegrationAction) perform no server-side permission check that gates the change (the only authorization call on the path is the recipient lookup inside the e-mail notifier), and the "integrate" condition only hides the buttons. Query property paths (BA-001-05): IntegrationAction#getIntegrationsInState and the three useBeans tags of WAR:WEB-INF/jsp/view/integrations.jsp (lines 23, 29, 155) query com.technoetic.xplanner.domain.Integration, which is not a mapped entity (GAP-004). Sweep of pass-003 F-001. Reflected request values (BA-001-07, mechanism (b)): WAR:WEB-INF/jsp/view/integrations.jsp writes the raw request parameters projectId (36) [parameter (lines); lines 26, 32 and 160 bind it as a query parameter] into the page with &lt;%= %&gt;, mostly as hidden input values, without HTML escaping; a crafted link is expected to inject markup into the page (Inferred; observed risk only, Q3 deferred). Inventory: .migration-tmp/stage-01/out/request-echo-07.txt. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/domain/Integration.java Integration (no @Entity); SRC:src/com/technoetic/xplanner/actions/IntegrationAction.java IntegrationAction#onJoinRequest, #onStartRequest. WAR: classes byte-identical to the v1.1a4 release; src/mappings/Integration.xml exists in the source but is not loaded by the WAR spring-beans.xml. The page and actions exist; the entity is neither annotated nor mapped by a loaded file. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the "not mapped" conclusion rests on spring-beans.xml:80 (rewritten entry) and is corroborated independently by the compiled class com.technoetic.xplanner.db.hibernate.HibernateHelper, whose mapped-class list also omits this class. Stage 3 W001 (BA-001-13, MC-A-37, W001-F-44): D-C-002 (editor), D-C-003 (viewer), D-C-004 (the full request sequence), D-C-005 (viewer join; part D blocked, reclassified as observed by the W001 lead). This confirms GAP-004 live: the unmapped Integration entity makes the queue non-functional. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks D-C-001, D-C-002, D-C-003, D-C-004, D-C-005).</t>
   </si>
   <si>
     <t>Joining without selecting a person or starting while another integration is active shows an error.</t>
@@ -2536,22 +2539,22 @@
     <t>Queue integrity.</t>
   </si>
   <si>
-    <t>Messages integrations.error.noperson / integrations.error.alreadyactive.</t>
-  </si>
-  <si>
-    <t>class IntegrationAction#onJoinRequest ("integrations.error.noperson"), #onStartRequest ("integrations.error.alreadyactive"). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/IntegrationAction.java IntegrationAction#onJoinRequest, #onStartRequest. WAR: classes byte-identical to the v1.1a4 release. A join without a person (empty or "0") and a start while an integration is active return the error forward with the two keys.</t>
-  </si>
-  <si>
-    <t>Integration events notify listeners; the configured listener sends e-mail (suppressed with a nonotify parameter).</t>
+    <t>Messages integrations.error.noperson / integrations.error.alreadyactive (source keys). Live (W001): a join without a person answers HTTP 500, because the error forward renders the failing integrations page (row 196), so no message is shown; no integration can become active, so the "already active" case cannot occur.</t>
+  </si>
+  <si>
+    <t>class IntegrationAction#onJoinRequest ("integrations.error.noperson"), #onStartRequest ("integrations.error.alreadyactive"). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/actions/IntegrationAction.java IntegrationAction#onJoinRequest, #onStartRequest. WAR: classes byte-identical to the v1.1a4 release. A join without a person (empty or "0") and a start while an integration is active return the error forward with the two keys. Stage 3 W001 (BA-001-13, MC-A-38, W001-F-45): D-C-006 (personId 0: HTTP 500, message absent) and D-C-007 (start after the joins: HTTP 500; part D blocked, reclassified as observed). Status Yes -&gt; Partial. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks D-C-006, D-C-007).</t>
+  </si>
+  <si>
+    <t>Integration events notify listeners: IntegrationAction fires only the ready event (on finish, cancel or leave when another integration is waiting), not on join or start, and the configured listener sends e-mail (suppressed with a nonotify parameter) (part D source note, static). In this baseline no event occurs, because the queue actions fail (row 196, W001).</t>
   </si>
   <si>
     <t>Team is informed of integration state.</t>
   </si>
   <si>
-    <t>E-mail on integration events.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/classes/xplanner.properties:86-87 (xplanner.integration.listeners=IntegrationEmailNotifier); class IntegrationAction#init/#fireIntegrationEvent/#isNotificationEnabled ("nonotify"). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/IntegrationAction.java IntegrationAction#init, #fireIntegrationEvent, #isNotificationEnabled; SRC:src/com/technoetic/xplanner/actions/IntegrationEmailNotifier.java IntegrationEmailNotifier. WAR: classes byte-identical to the v1.1a4 release; listener list from the patched WAR xplanner.properties. The listeners named in the property are instantiated with Class.forName (not by Spring) and receive every event; the e-mail itself depends on SMTP. Live question: Is an e-mail sent when an integration is joined and started, and suppressed with nonotify? Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>E-mail on the ready event (source). Live (W001, adapted mail environment): no integration e-mail, because every queue request fails with HTTP 500 (row 196) before any event; suppression by nonotify cannot be told apart.</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/classes/xplanner.properties:86-87 (xplanner.integration.listeners=IntegrationEmailNotifier); class IntegrationAction#init/#fireIntegrationEvent/#isNotificationEnabled ("nonotify"). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/IntegrationAction.java IntegrationAction#init, #fireIntegrationEvent, #isNotificationEnabled; SRC:src/com/technoetic/xplanner/actions/IntegrationEmailNotifier.java IntegrationEmailNotifier. WAR: classes byte-identical to the v1.1a4 release; listener list from the patched WAR xplanner.properties. The listeners named in the property are instantiated with Class.forName (not by Spring) and receive every event; the e-mail itself depends on SMTP. Live question: Is an e-mail sent when an integration is joined and started, and suppressed with nonotify? Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. Stage 3 W001 (BA-001-13, MC-A-39, W001-F-46): full join/start/finish/cancel/leave sequence after the mail adaptation, with and without nonotify: no message with the integration subject (D-C-009, D-C-010). Under the original condition no integration event occurred; the logged email.css failures came from task notifications only (D-C-008). Part D source note: IntegrationEmailNotifier does not use the stylesheet formatter. Status Inferred -&gt; Partial (R-G2). Stage 3 W001 live answer (BA-001-13, MC-C-24): No e-mail in this baseline: join and start fail with HTTP 500 before any event. Suppression by nonotify cannot be told apart because no event fires (D-C-008, D-C-009, D-C-010). The D/F correction is under W001-F-46. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks D-C-008, D-C-009, D-C-010).</t>
   </si>
   <si>
     <t>UF-013</t>
@@ -2563,28 +2566,28 @@
     <t>Daily missing time entry reminder</t>
   </si>
   <si>
-    <t>Every day at 00:05 the system e-mails acceptors of tasks with no time entry after a cut-off, asking them to enter time.</t>
+    <t>Every day at 00:05 the system is meant to e-mail acceptors of tasks with no time entry after a cut-off, asking them to enter time. In this baseline the job runs at 00:05 (twice, inferred from two send attempts per recipient, row 65), but every send fails before the recipient is set (LazyInitializationException on Person.getEmail outside a session, then MessagingException "error setting recipient"), so no reminder is sent and the error is only logged (W001).</t>
   </si>
   <si>
     <t>Keeps actuals complete.</t>
   </si>
   <si>
-    <t>E-mail "XPlanner time entry reminder." listing tasks.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/classes/spring-beans.xml:362-367 (task:scheduled missingTimeEntryNotifier execute cron "0 5 0 * * *"); class com.technoetic.xplanner.mail.MissingTimeEntryNotifier#execute/#sendMissingTimeEntryReminderToAcceptors; ResourceBundle.properties job.emailnotifier.subjectForAcceptors; mappings/Metrics.xml TimeEntryEmailNotificationToAcceptors. Loading (BA-001-05): the task:scheduled registration sits in spring-beans.xml, which both Spring contexts load (row 65), so two schedulers are expected to run the job, and each acceptor is expected to receive the reminder twice (Inferred, runtime unverified). Source: stage-02-pass-003 F-002. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/mail/MissingTimeEntryNotifier.java MissingTimeEntryNotifier#execute, #sendMissingTimeEntryReminderToAcceptors. WAR: classes byte-identical to the v1.1a4 release; patched spring-beans.xml (WAR governs). The cut-off is hard-coded to the previous midnight; the schedule, the double registration and the delivery are runtime effects. Live question: At 00:05, are reminders sent, and are they sent twice? Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
-  </si>
-  <si>
-    <t>The same job e-mails project notification receivers listing people who may have forgotten to enter time the previous working day.</t>
+    <t>E-mail "XPlanner time entry reminder." listing tasks (source). Live (W001, adapted mail environment): none is sent; each attempt is logged as "Error sending email" and the sink received 0 messages. The failure is in recipient resolution, before the stylesheet fetch (lead interpretation).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/classes/spring-beans.xml:362-367 (task:scheduled missingTimeEntryNotifier execute cron "0 5 0 * * *"); class com.technoetic.xplanner.mail.MissingTimeEntryNotifier#execute/#sendMissingTimeEntryReminderToAcceptors; ResourceBundle.properties job.emailnotifier.subjectForAcceptors; mappings/Metrics.xml TimeEntryEmailNotificationToAcceptors. Loading (BA-001-05): the task:scheduled registration sits in spring-beans.xml, which both Spring contexts load (row 65), so two schedulers are expected to run the job, and each acceptor is expected to receive the reminder twice (Inferred, runtime unverified). Source: stage-02-pass-003 F-002. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/mail/MissingTimeEntryNotifier.java MissingTimeEntryNotifier#execute, #sendMissingTimeEntryReminderToAcceptors. WAR: classes byte-identical to the v1.1a4 release; patched spring-beans.xml (WAR governs). The cut-off is hard-coded to the previous midnight; the schedule, the double registration and the delivery are runtime effects. Live question: At 00:05, are reminders sent, and are they sent twice? Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream. Stage 3 W001 (BA-001-13, MC-A-40, W001-F-47): the 00:05 job fired at 00:05:00Z; 2 reminder attempts for the prepared acceptor, each failing as above (L-C-006). Status Inferred -&gt; Partial. Stage 3 W001 live answer (BA-001-13, MC-C-26): Not sent: the job fired at 00:05:00Z and attempted the reminder twice for the prepared acceptor (consistent with a doubled job, inferred), and each attempt failed with LazyInitializationException on Person.getEmail ("no Session"); 0 mails (L-C-005, L-C-006). The D/F correction is under W001-F-47. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks D-C-011, L-C-006).</t>
+  </si>
+  <si>
+    <t>The same job is meant to e-mail project notification receivers listing people who may have forgotten to enter time the previous working day. In this baseline every report send fails the same way as the reminder (row 200), so no report is sent and the error is only logged (W001).</t>
   </si>
   <si>
     <t>Project leads follow up.</t>
   </si>
   <si>
-    <t>E-mail "XPlanner project time entry status."</t>
-  </si>
-  <si>
-    <t>class MissingTimeEntryNotifier#sendMissingTimeEntryReportToLeads; ResourceBundle.properties job.emailnotifier.subjectForProjectLeeds, bodyheaderForProjectLeeds; mappings/Metrics.xml TimeEntryEmailNotificationToProjectSpecificLeads; project option sendemail (editProject.jsp). Loading (BA-001-05): because the job is registered in both Spring contexts (row 65), receivers are expected to get the report twice (Inferred, runtime unverified). Source: stage-02-pass-003 F-002. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/mail/MissingTimeEntryNotifier.java MissingTimeEntryNotifier#execute, #sendMissingTimeEntryReportToLeads. WAR: classes byte-identical to the v1.1a4 release; patched spring-beans.xml (WAR governs). The same run sends the report to the leads; the delivery is a runtime effect. Live question: Do the notification receivers of a project with the option on receive the report, and twice?</t>
+    <t>E-mail "XPlanner project time entry status." (source). Live (W001, adapted mail environment): none is sent; the report was attempted twice for the recipient and each attempt failed with the same LazyInitializationException and MessagingException; 0 messages.</t>
+  </si>
+  <si>
+    <t>class MissingTimeEntryNotifier#sendMissingTimeEntryReportToLeads; ResourceBundle.properties job.emailnotifier.subjectForProjectLeeds, bodyheaderForProjectLeeds; mappings/Metrics.xml TimeEntryEmailNotificationToProjectSpecificLeads; project option sendemail (editProject.jsp). Loading (BA-001-05): because the job is registered in both Spring contexts (row 65), receivers are expected to get the report twice (Inferred, runtime unverified). Source: stage-02-pass-003 F-002. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/mail/MissingTimeEntryNotifier.java MissingTimeEntryNotifier#execute, #sendMissingTimeEntryReportToLeads. WAR: classes byte-identical to the v1.1a4 release; patched spring-beans.xml (WAR governs). The same run sends the report to the leads; the delivery is a runtime effect. Live question: Do the notification receivers of a project with the option on receive the report, and twice? Stage 3 W001 (BA-001-13, MC-A-40, W001-F-47): MissingTimeEntryNotifier.sendMissingTimeEntryReportToLeads failed twice for the report recipient (L-C-007). Status Inferred -&gt; Partial. Stage 3 W001 live answer (BA-001-13, MC-C-27): No: the report was attempted twice for the recipient and each attempt failed the same way; 0 mails (L-C-005, L-C-007). The D/F correction is under W001-F-47. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks D-C-012, L-C-007).</t>
   </si>
   <si>
     <t>Before each notification e-mail is composed, the application fetches the stylesheet xplanner.application.url + "/css/email.css" over HTTP and embeds it in the message.</t>
@@ -2593,10 +2596,10 @@
     <t>E-mail appearance depends on the application reaching its own configured URL (effective value http://localhost:8080/xplanner, which may not match the deployed context).</t>
   </si>
   <si>
-    <t>Styled e-mail when the URL is reachable; otherwise the style is expected to be missing or the e-mail to fail (runtime unverified).</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.mail.EmailFormatterImpl#formatEmailEntry (strings "xplanner.application.url", "/css/email.css", "style"; calls com.technoetic.xplanner.util.HttpClient#getPage); caller EmailNotificationSupport; WAR:css/email.css; WAR:WEB-INF/classes/xplanner-custom.properties:30. Source: stage-02-pass-001 F-006. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/mail/EmailFormatterImpl.java EmailFormatterImpl#formatEmailEntry (both variants). WAR: classes byte-identical to the v1.1a4 release; application URL from the patched WAR xplanner-custom.properties. Both variants fetch the stylesheet from the application URL before merging the template; the effect of an unreachable URL depends on HttpClient and the network. Live question: With the application URL unreachable from the server, is a notification sent without style, delayed or not sent?</t>
+    <t>Styled e-mail when the URL is reachable (W001, adapted environment: the served stylesheet is embedded in a style element); when the stylesheet URL is not reachable the e-mail is not sent: the send throws FileNotFoundException and is logged as "Error sending email" (W001, original deployment condition).</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.mail.EmailFormatterImpl#formatEmailEntry (strings "xplanner.application.url", "/css/email.css", "style"; calls com.technoetic.xplanner.util.HttpClient#getPage); caller EmailNotificationSupport; WAR:css/email.css; WAR:WEB-INF/classes/xplanner-custom.properties:30. Source: stage-02-pass-001 F-006. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/mail/EmailFormatterImpl.java EmailFormatterImpl#formatEmailEntry (both variants). WAR: classes byte-identical to the v1.1a4 release; application URL from the patched WAR xplanner-custom.properties. Both variants fetch the stylesheet from the application URL before merging the template; the effect of an unreachable URL depends on HttpClient and the network. Live question: With the application URL unreachable from the server, is a notification sent without style, delayed or not sent? Stage 3 W001 live answer (BA-001-13, MC-C-28): Not sent: the send throws FileNotFoundException for the stylesheet URL and is logged as "Error sending email"; no mail reaches the sink. With the stylesheet reachable (adapted) the mail is styled (D-C-013, D-C-014). Status Inferred -&gt; Yes on this live observation. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-013, D-C-014).</t>
   </si>
   <si>
     <t>Mail is sent through the configured SMTP server (localhost:25, from xplanner@xplannerplus.org in the shipped properties).</t>
@@ -2605,10 +2608,10 @@
     <t>Operational dependency for all e-mail.</t>
   </si>
   <si>
-    <t>No e-mail without a reachable SMTP server.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/classes/xplanner.properties:78-80; WAR:WEB-INF/classes/xplanner-custom.properties:30-34; package com.technoetic.xplanner.mail (EmailMessageImpl, SmtpAuthenticator). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR xplanner.properties, xplanner-custom.properties (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-04: the cited value is read from xplanner-custom.properties (rewritten entry, known patch target); upstream value not determinable.</t>
+    <t>No e-mail without a reachable SMTP server; the triggering change is still saved and the user sees no error, because the failure (javax.mail ConnectException "Connection refused") is only logged (W001).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/classes/xplanner.properties:78-80; WAR:WEB-INF/classes/xplanner-custom.properties:30-34; package com.technoetic.xplanner.mail (EmailMessageImpl, SmtpAuthenticator). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR xplanner.properties, xplanner-custom.properties (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. P-04: the cited value is read from xplanner-custom.properties (rewritten entry, known patch target); upstream value not determinable. Stage 3 W001 live answer (BA-001-13, MC-C-29): with the mail sink stopped (Codex-decided check performed by PM, attempt 2; attempt 1 invalid): the task POST answered 302 and the task was saved; the send failed with javax.mail ConnectException "Connection refused" in the app log; no error reached the user; no mail. Controls before and after: one mail delivered (L-C-009). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-015, D-C-016, L-C-009).</t>
   </si>
   <si>
     <t>Data sampling for burn-down</t>
@@ -2623,7 +2626,7 @@
     <t>No nightly samples in the shipped configuration.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/spring-beans.xml:343-360 (datasamplingJob), :369-383 (trigger "0 55 23 ? 1-12 *"), :385-402 (SchedulerFactoryBean commented out); class com.technoetic.xplanner.charts.DataSamplingJob; WAR:WEB-INF/test-action-servlet.xml:4-7. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/charts/DataSamplingJob.java DataSamplingJob. WAR: patched spring-beans.xml with the scheduler factory commented out (WAR governs). The job class exists, but the WAR configuration registers no scheduler for its trigger. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>WAR:WEB-INF/classes/spring-beans.xml:343-360 (datasamplingJob), :369-383 (trigger "0 55 23 ? 1-12 *"), :385-402 (SchedulerFactoryBean commented out); class com.technoetic.xplanner.charts.DataSamplingJob; WAR:WEB-INF/test-action-servlet.xml:4-7. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/charts/DataSamplingJob.java DataSamplingJob. WAR: patched spring-beans.xml with the scheduler factory commented out (WAR governs). The job class exists, but the WAR configuration registers no scheduler for its trigger. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream. Stage 3 W001 live answer (BA-001-13, MC-C-25): no nightly sample is taken: no data sample was written at 23:55 (datasample held 48 rows at 00:07Z; the same count before 23:55 is a PM statement) (L-C-008); the startup log shows no Quartz scheduler and the database has no qrtz tables (D-C-017). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-017, D-C-018, L-C-008).</t>
   </si>
   <si>
     <t>If iteration.automatically.extend.endDate were true, sampling would extend the end date of unclosed iterations (shipped: false).</t>
@@ -2635,7 +2638,7 @@
     <t>No automatic extension with shipped properties.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/xplanner.properties:314; class com.technoetic.xplanner.charts.DataSamplerImpl ("iteration.automatically.extend.endDate", "Extend iteration end day to "). Wiring (BA-001-07, mechanism (a)): DataSamplerImpl#extendIterationEndDateIfNeeded uses the hibernateOperations property only when the flag is true; the bean dataSampler (WAR:WEB-INF/classes/spring-beans.xml:303, autowire byName) finds no bean named hibernateOperations, so enabling the flag is expected to fail with a null reference (Inferred). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/charts/DataSamplerImpl.java DataSamplerImpl#extendIterationEndDateIfNeeded. WAR: classes byte-identical to the v1.1a4 release; flag false in the patched WAR xplanner.properties. The end date is extended only when the flag is true and the iteration is active with a past end date; with the shipped value nothing is extended. The expected failure with the flag enabled stays Inferred (wiring). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>WAR:WEB-INF/classes/xplanner.properties:314; class com.technoetic.xplanner.charts.DataSamplerImpl ("iteration.automatically.extend.endDate", "Extend iteration end day to "). Wiring (BA-001-07, mechanism (a)): DataSamplerImpl#extendIterationEndDateIfNeeded uses the hibernateOperations property only when the flag is true; the bean dataSampler (WAR:WEB-INF/classes/spring-beans.xml:303, autowire byName) finds no bean named hibernateOperations, so enabling the flag is expected to fail with a null reference (Inferred). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/charts/DataSamplerImpl.java DataSamplerImpl#extendIterationEndDateIfNeeded. WAR: classes byte-identical to the v1.1a4 release; flag false in the patched WAR xplanner.properties. The end date is extended only when the flag is true and the iteration is active with a past end date; with the shipped value nothing is extended. The expected failure with the flag enabled stays Inferred (wiring). Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: partially verified; checks D-C-019, D-C-020, F-C-008; open residual scope R-32 (e)).</t>
   </si>
   <si>
     <t>Per-change e-mail listener</t>
@@ -2650,7 +2653,7 @@
     <t>No e-mail per object change.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/classes/spring-beans.xml:404-406 (eventBus EventManager); class net.sf.xplanner.email.EmailPerChangeListener (no annotation, no bean definition in any Spring XML - grep of WAR XML for EmailPerChangeListener returned no match while the same grep found eventBus). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/net/sf/xplanner/email/EmailPerChangeListener.java EmailPerChangeListener (implements ApplicationListener, no annotation); SRC:src/net/sf/xplanner/events/EventManager.java EventManager. WAR: classes byte-identical to the v1.1a4 release; component scans only net.sf.xplanner.rest (spring-beans.xml:50) and net.sf.xplanner.web (spring-web.xml:12). Events are published as Spring application events; the listener is neither annotated nor defined as a bean, and no scan covers its package. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>WAR:WEB-INF/classes/spring-beans.xml:404-406 (eventBus EventManager); class net.sf.xplanner.email.EmailPerChangeListener (no annotation, no bean definition in any Spring XML - grep of WAR XML for EmailPerChangeListener returned no match while the same grep found eventBus). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/net/sf/xplanner/email/EmailPerChangeListener.java EmailPerChangeListener (implements ApplicationListener, no annotation); SRC:src/net/sf/xplanner/events/EventManager.java EventManager. WAR: classes byte-identical to the v1.1a4 release; component scans only net.sf.xplanner.rest (spring-beans.xml:50) and net.sf.xplanner.web (spring-web.xml:12). Events are published as Spring application events; the listener is neither annotated nor defined as a bean, and no scan covers its package. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-021).</t>
   </si>
   <si>
     <t>UF-014</t>
@@ -2668,10 +2671,10 @@
     <t>Take data out of XPlanner.</t>
   </si>
   <si>
-    <t>Overlib pop-up with format links such as XML, MPX, MSPDI, PDF, Report.</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/jsp/view/exportLinks.jsp:16-40 (formats filtered by findActionConfig("/export/"+name+"/"+format)); WAR:WEB-INF/classes/xplanner.properties:145 (xml,mpx,mspdi,pdf,jrpdf). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value.</t>
+    <t>Overlib pop-up (link "Export", caption "Format:") with the format links per object type: project XML, MPX, MSPDI; iteration XML, MPX, MSPDI, PDF, JRPDF; story and task PDF, JRPDF; person JRPDF (W001).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/jsp/view/exportLinks.jsp:16-40 (formats filtered by findActionConfig("/export/"+name+"/"+format)); WAR:WEB-INF/classes/xplanner.properties:145 (xml,mpx,mspdi,pdf,jrpdf). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies); values from the patched WAR xplanner.properties (WAR governs). The claim rests on the WAR descriptors and JSPs already cited. Provenance (fixed baseline, see reconnaissance GAP-005): P-03: the cited value is read from xplanner.properties, one of 3 WAR entries rewritten after packaging (ZIP version-needed 2.0 versus 1.0 for the other 1087 entries); no content sign shows this key changed, but it is not guaranteed to be the upstream value. Stage 3 W001 (BA-001-13, MC-A-41, W001-F-48): export links read on project 224, iteration 234, story 256, task 270 and person 209; the jrpdf label is "JRPDF" (key export.jrpdf) (D-C-022). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks D-C-022, D-C-023).</t>
   </si>
   <si>
     <t>Export project</t>
@@ -2686,7 +2689,7 @@
     <t>Download export.xml (text/xml), export.mpx (application/mpx) or export.xml (application/mspdi).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:189-193; WAR:WEB-INF/action-servlet.xml:45-70; classes com.technoetic.xplanner.export.XmlExporter, MpxExporter, MspdiExporter (Content-type and filename strings); WAR:WEB-INF/lib/mpxj-3.0.1.jar. Content (BA-001-08, pass-006 F-003, check (f)): besides the selected project, all three formats contain every person of the system. XmlExporter#export runs the unconditional query "from person in class net.sf.xplanner.domain.Person" and writes the result as the people of the document (XmlExporter$XPlannerData#setPeople); XmlExporter#configureBindings hides the person password and lastUpdateTime, so the other readable person properties (for example id, name, user ID, e-mail, phone, initials, hidden flag and description) are expected in the file (Betwixt, exact set Inferred). MpxExporter#export and MspdiExporter#export load all persons into MpxExporter$ResourceRegistry, which adds each one as a resource with its name only (Person#getName). The export actions have no server-side permission check (rows 29-30). Inferred; observed fact for Stage 9, Q3 deferred. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/export/XmlExporter.java XmlExporter#export; SRC:src/com/technoetic/xplanner/export/MpxExporter.java MpxExporter#export. WAR: classes byte-identical to the v1.1a4 release. Both exporters load all persons (the XML file as people, MPX and MSPDI as resources), as recorded.</t>
+    <t>WAR:WEB-INF/struts-config.xml:189-193; WAR:WEB-INF/action-servlet.xml:45-70; classes com.technoetic.xplanner.export.XmlExporter, MpxExporter, MspdiExporter (Content-type and filename strings); WAR:WEB-INF/lib/mpxj-3.0.1.jar. Content (BA-001-08, pass-006 F-003, check (f)): besides the selected project, all three formats contain every person of the system. XmlExporter#export runs the unconditional query "from person in class net.sf.xplanner.domain.Person" and writes the result as the people of the document (XmlExporter$XPlannerData#setPeople); XmlExporter#configureBindings hides the person password and lastUpdateTime, so the other readable person properties (for example id, name, user ID, e-mail, phone, initials, hidden flag and description) are expected in the file (Betwixt, exact set Inferred). MpxExporter#export and MspdiExporter#export load all persons into MpxExporter$ResourceRegistry, which adds each one as a resource with its name only (Person#getName). The export actions have no server-side permission check (rows 29-30). Inferred; observed fact for Stage 9, Q3 deferred. Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/export/XmlExporter.java XmlExporter#export; SRC:src/com/technoetic/xplanner/export/MpxExporter.java MpxExporter#export. WAR: classes byte-identical to the v1.1a4 release. Both exporters load all persons (the XML file as people, MPX and MSPDI as resources), as recorded. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-024, D-C-025, D-C-026).</t>
   </si>
   <si>
     <t>Export iteration</t>
@@ -2701,7 +2704,7 @@
     <t>Downloads export.xml, export.mpx, export.xml, export.pdf.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:231-237; WAR:WEB-INF/action-servlet.xml:132-166; class com.technoetic.xplanner.export.PdfExporter ("application/pdf", "export.pdf"); WAR:WEB-INF/lib/itext-1.01.jar. Content (BA-001-08, pass-006 F-003, check (f)): the XML, MPX and MSPDI files contain every person of the system, as in row 209 (the same exporter beans, WAR:WEB-INF/action-servlet.xml:132-166). The PDF listing (PdfExporter) shows only the names of the customers and acceptors of the exported stories and tasks (Person#getName), no person list (Inferred). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/export/XmlExporter.java XmlExporter#export; SRC:src/com/technoetic/xplanner/export/PdfExporter.java PdfExporter. WAR: classes byte-identical to the v1.1a4 release. As row 209 for XML, MPX and MSPDI; the PDF exporter lists the iteration's stories and tasks.</t>
+    <t>WAR:WEB-INF/struts-config.xml:231-237; WAR:WEB-INF/action-servlet.xml:132-166; class com.technoetic.xplanner.export.PdfExporter ("application/pdf", "export.pdf"); WAR:WEB-INF/lib/itext-1.01.jar. Content (BA-001-08, pass-006 F-003, check (f)): the XML, MPX and MSPDI files contain every person of the system, as in row 209 (the same exporter beans, WAR:WEB-INF/action-servlet.xml:132-166). The PDF listing (PdfExporter) shows only the names of the customers and acceptors of the exported stories and tasks (Person#getName), no person list (Inferred). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/export/XmlExporter.java XmlExporter#export; SRC:src/com/technoetic/xplanner/export/PdfExporter.java PdfExporter. WAR: classes byte-identical to the v1.1a4 release. As row 209 for XML, MPX and MSPDI; the PDF exporter lists the iteration's stories and tasks. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-027, D-C-028).</t>
   </si>
   <si>
     <t>An iteration JasperReports PDF (jrpdf) report is offered but its report template is missing from the WAR.</t>
@@ -2713,7 +2716,7 @@
     <t>report.pdf expected; generation expected to fail.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:239; WAR:WEB-INF/action-servlet.xml:168-175 (reportExporter); class com.technoetic.xplanner.export.PdfReportExporter (template com/technoetic/xplanner/export/reports/JRIteration.jrxml) - no *.jrxml or *.jasper in the WAR or its JARs (search also matched JRXml* classes, proving the pattern works). Query property paths (BA-001-05): class PdfReportExporter$PersonDataSource and $UserStoryDataSource also query "task.story", which Task does not map, so the person and story reports would fail even with templates present. Sweep of pass-003 F-001. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/export/PdfReportExporter.java PdfReportExporter (loads the templates with getResourceAsStream); SRC:src/com/technoetic/xplanner/export/reports/JRIteration.jrxml. WAR: classes byte-identical to the v1.1a4 release; the four report templates exist in the SVN source (src/com/technoetic/xplanner/export/reports/JR*.jrxml) but not in the WAR (WAR governs). The template is missing from the delivered package only: the release build did not include the SVN templates. For the WAR the generation is still expected to fail.</t>
+    <t>WAR:WEB-INF/struts-config.xml:239; WAR:WEB-INF/action-servlet.xml:168-175 (reportExporter); class com.technoetic.xplanner.export.PdfReportExporter (template com/technoetic/xplanner/export/reports/JRIteration.jrxml) - no *.jrxml or *.jasper in the WAR or its JARs (search also matched JRXml* classes, proving the pattern works). Query property paths (BA-001-05): class PdfReportExporter$PersonDataSource and $UserStoryDataSource also query "task.story", which Task does not map, so the person and story reports would fail even with templates present. Sweep of pass-003 F-001. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/export/PdfReportExporter.java PdfReportExporter (loads the templates with getResourceAsStream); SRC:src/com/technoetic/xplanner/export/reports/JRIteration.jrxml. WAR: classes byte-identical to the v1.1a4 release; the four report templates exist in the SVN source (src/com/technoetic/xplanner/export/reports/JR*.jrxml) but not in the WAR (WAR governs). The template is missing from the delivered package only: the release build did not include the SVN templates. For the WAR the generation is still expected to fail. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-029).</t>
   </si>
   <si>
     <t>Export story, task and person</t>
@@ -2728,7 +2731,7 @@
     <t>export.pdf download.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:281,297; WAR:WEB-INF/action-servlet.xml:238-245,280-287 (pdfExporter). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
+    <t>WAR:WEB-INF/struts-config.xml:281,297; WAR:WEB-INF/action-servlet.xml:238-245,280-287 (pdfExporter). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-030).</t>
   </si>
   <si>
     <t>Story, task and person JasperReports reports (jrpdf) are offered but their templates are missing.</t>
@@ -2737,7 +2740,7 @@
     <t>Formatted reports.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/struts-config.xml:283,299,315; WAR:WEB-INF/action-servlet.xml:247-254,289-296,333-340; class PdfReportExporter (JRStory.jrxml, JRTask.jrxml, JRPerson.jrxml absent). Query property paths (BA-001-05): the story and person report data sources (PdfReportExporter$UserStoryDataSource "task.story = ?", $PersonDataSource "task.story = story.id") use a property that Task does not map. Sweep of pass-003 F-001. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/export/PdfReportExporter.java PdfReportExporter; SRC:src/com/technoetic/xplanner/export/reports/JRStory.jrxml, JRTask.jrxml, JRPerson.jrxml. WAR: classes byte-identical to the v1.1a4 release; JRStory, JRTask and JRPerson.jrxml exist in the SVN source but not in the WAR (WAR governs). As row 211: the templates exist in the source tree but were not packaged; the task.story query defect remains.</t>
+    <t>WAR:WEB-INF/struts-config.xml:283,299,315; WAR:WEB-INF/action-servlet.xml:247-254,289-296,333-340; class PdfReportExporter (JRStory.jrxml, JRTask.jrxml, JRPerson.jrxml absent). Query property paths (BA-001-05): the story and person report data sources (PdfReportExporter$UserStoryDataSource "task.story = ?", $PersonDataSource "task.story = story.id") use a property that Task does not map. Sweep of pass-003 F-001. Source reconciliation (BA-001-11, A4): correction needed, corrected in this row. SRC:src/com/technoetic/xplanner/export/PdfReportExporter.java PdfReportExporter; SRC:src/com/technoetic/xplanner/export/reports/JRStory.jrxml, JRTask.jrxml, JRPerson.jrxml. WAR: classes byte-identical to the v1.1a4 release; JRStory, JRTask and JRPerson.jrxml exist in the SVN source but not in the WAR (WAR governs). As row 211: the templates exist in the source tree but were not packaged; the task.story query defect remains. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-031, D-C-032, D-C-033).</t>
   </si>
   <si>
     <t>UF-015</t>
@@ -2758,7 +2761,7 @@
     <t>SOAP responses with ProjectData, IterationData, UserStoryData, TaskData, TimeEntryData, NoteData, PersonData beans; 401 challenge "Basic realm=XPlanner" without credentials.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:206-209,298-306 (AxisServlet /servlet/AxisServlet and /soap/*), :111-119,168-171 (BasicSecurityFilter on /soap/*); WAR:WEB-INF/server-config.wsdd:25-28,44-51 (service XPlanner, class com.technoetic.xplanner.soap.XPlanner, 8 bean mappings); class BasicSecurityFilter#challenge ("WWW-Authenticate", "Basic realm=\"XPlanner\""). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/security/filter/BasicSecurityFilter.java BasicSecurityFilter#onAuthenticationFailure, #challenge. WAR: classes byte-identical to the v1.1a4 release. An unauthenticated SOAP request is answered with a Basic challenge.</t>
+    <t>WAR:WEB-INF/web.xml:206-209,298-306 (AxisServlet /servlet/AxisServlet and /soap/*), :111-119,168-171 (BasicSecurityFilter on /soap/*); WAR:WEB-INF/server-config.wsdd:25-28,44-51 (service XPlanner, class com.technoetic.xplanner.soap.XPlanner, 8 bean mappings); class BasicSecurityFilter#challenge ("WWW-Authenticate", "Basic realm=\"XPlanner\""). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/com/technoetic/xplanner/security/filter/BasicSecurityFilter.java BasicSecurityFilter#onAuthenticationFailure, #challenge. WAR: classes byte-identical to the v1.1a4 release. An unauthenticated SOAP request is answered with a Basic challenge. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-034, D-C-035).</t>
   </si>
   <si>
     <t>The same Axis servlet is also mapped at /servlet/AxisServlet, where no Basic security filter is applied.</t>
@@ -2767,10 +2770,10 @@
     <t>Records an unprotected alternate endpoint.</t>
   </si>
   <si>
-    <t>SOAP reachable without the filter at the alternate path (runtime unverified).</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/web.xml:298-301 (servlet-mapping /servlet/AxisServlet) versus filter mappings :168-176 (/soap/*, /ical/* only). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact); status Inferred -&gt; Yes. none: descriptor fact, no Java involved. WAR: web.xml identical to the SVN webapp copy. The servlet mapping /servlet/AxisServlet has no security filter mapping. Correction (BA-001-12, pass-010 F-004): the BA-001-11 change to Yes had no evidence that was new since the Inferred status. Its only basis is the descriptor fact already cited (WAR:WEB-INF/web.xml:168-176,299-302); no method-level reading of the Axis servlet or of its handler chain was made, and no rule permits a descriptor-only status change. Status returned Yes -&gt; Inferred; the descriptor fact stands.</t>
+    <t>SOAP reachable without credentials at the alternate path (W001): a GET lists the XPlanner and Version services with all operations; with the service namespace and SOAPAction the calls execute: object operations fault "no user principal in session", getProjects returns null, getVersion works, and the attribute operations run anonymously (an anonymous setAttribute was persisted on story 256).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/web.xml:298-301 (servlet-mapping /servlet/AxisServlet) versus filter mappings :168-176 (/soap/*, /ical/* only). Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact); status Inferred -&gt; Yes. none: descriptor fact, no Java involved. WAR: web.xml identical to the SVN webapp copy. The servlet mapping /servlet/AxisServlet has no security filter mapping. Correction (BA-001-12, pass-010 F-004): the BA-001-11 change to Yes had no evidence that was new since the Inferred status. Its only basis is the descriptor fact already cited (WAR:WEB-INF/web.xml:168-176,299-302); no method-level reading of the Axis servlet or of its handler chain was made, and no rule permits a descriptor-only status change. Status returned Yes -&gt; Inferred; the descriptor fact stands. Stage 3 W001 (BA-001-13, MC-A-42, W001-F-49): D-C-036 (without a namespace or SOAPAction the call faults "could not find a target service"). Security-relevant (GAP-007, Q3 deferred). Status Inferred -&gt; Yes on this live observation, new since the BA-001-12 return. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks D-C-036, D-C-037).</t>
   </si>
   <si>
     <t>An Axis "Version" service reports the Axis version.</t>
@@ -2782,19 +2785,19 @@
     <t>getVersion response.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/server-config.wsdd:29-32. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited.</t>
-  </si>
-  <si>
-    <t>SOAP operations check the caller's permission on each object (read for get operations, create/edit/delete for changes); the five attribute operations (setAttribute, getAttribute, deleteAttribute, getAttributes, getAttributesWithPrefix) have no permission check.</t>
+    <t>WAR:WEB-INF/server-config.wsdd:29-32. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: descriptor or JSP fact, no Java decides it. WAR: WAR descriptors and JSPs (71 of 73 JSPs identical to the SVN webapp copies). The claim rests on the WAR descriptors and JSPs already cited. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-038).</t>
+  </si>
+  <si>
+    <t>SOAP operations check the caller's permission on each object (read for get operations, create/edit/delete for changes); the five attribute operations (setAttribute, getAttribute, deleteAttribute, getAttributes, getAttributesWithPrefix) have no permission check, so any caller can use them, including unauthenticated calls through /servlet/AxisServlet (row 216, W001).</t>
   </si>
   <si>
     <t>Unlike the web actions, the SOAP channel enforces object permissions, except for attributes.</t>
   </si>
   <si>
-    <t>Messages such as "no permission to update object"; lists contain only accessible objects; attribute calls succeed for any authenticated caller (runtime unverified).</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.soap.XPlanner#hasPermission via #getObject, #getObjects/#selectAccessibleObjects, #addObject, #updateObject, #removeObject (strings "no permission to create object", "no permission to update object", "no permission to delete object"); no authorization call reachable from the attribute operations (.migration-tmp/stage-01/out/authtrace.json). BA-001-03 impact sweep of F-001. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/soap/XPlanner.java XPlanner#hasPermission, #setAttribute, #getAttribute, #deleteAttribute, #getAttributes, #getAttributesWithPrefix. WAR: classes byte-identical to the v1.1a4 release. Object operations call hasPermission; the attribute operations delegate straight to the attribute repository.</t>
+    <t>Messages such as "no permission to update object"; lists contain only accessible objects; attribute calls run for any caller, including unauthenticated calls through /servlet/AxisServlet (W001). getAttribute always returns a SOAP fault (TypeMismatchException: expected AttributeId, got Attribute); getAttributes works and getAttributesWithPrefix returns the keys with the prefix removed (W001).</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.soap.XPlanner#hasPermission via #getObject, #getObjects/#selectAccessibleObjects, #addObject, #updateObject, #removeObject (strings "no permission to create object", "no permission to update object", "no permission to delete object"); no authorization call reachable from the attribute operations (.migration-tmp/stage-01/out/authtrace.json). BA-001-03 impact sweep of F-001. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/soap/XPlanner.java XPlanner#hasPermission, #setAttribute, #getAttribute, #deleteAttribute, #getAttributes, #getAttributesWithPrefix. WAR: classes byte-identical to the v1.1a4 release. Object operations call hasPermission; the attribute operations delegate straight to the attribute repository. Stage 3 W001 (BA-001-13, MC-A-42, MC-A-43, W001-F-49, W001-F-50): anonymous setAttribute persisted (D-C-036); viewer setAttribute succeeded and getAttributes of an unreadable project returned an empty map without a fault; getAttribute faults for every caller (D-C-044); object permission checks observed (D-C-042). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks D-C-039, D-C-040, D-C-041, D-C-042, D-C-043, D-C-044).</t>
   </si>
   <si>
     <t>A JAX-WS endpoint net.sf.xplanner.soap.XPlanner is declared but not active (servlet commented out, class absent).</t>
@@ -2809,7 +2812,7 @@
     <t>No</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/sun-jaxws.xml:3; WAR:WEB-INF/web.xml:183-185,273-282 (WSServlet commented); class net.sf.xplanner.soap.XPlanner ABSENT. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: net.sf.xplanner.soap.XPlanner is absent from the SVN source as from the WAR. WAR: sun-jaxws.xml identical to the SVN webapp copy. The declared endpoint class exists nowhere.</t>
+    <t>WAR:WEB-INF/sun-jaxws.xml:3; WAR:WEB-INF/web.xml:183-185,273-282 (WSServlet commented); class net.sf.xplanner.soap.XPlanner ABSENT. Source reconciliation (BA-001-11, A4): confirmed (descriptor or JSP fact). none: net.sf.xplanner.soap.XPlanner is absent from the SVN source as from the WAR. WAR: sun-jaxws.xml identical to the SVN webapp copy. The declared endpoint class exists nowhere. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-045).</t>
   </si>
   <si>
     <t>SOAP read operations</t>
@@ -2821,25 +2824,25 @@
     <t>Read access to planning data.</t>
   </si>
   <si>
-    <t>Operations getProjects, getProject, getIterations, getIteration, getUserStories, getUserStory, getTasks, getTask, getCurrentTasksForPerson, getPlannedTasksForPerson, getTimeEntries, getTimeEntry, getNote, getNotesForObject, getPerson, getPeople, getAttribute, getAttributes, getAttributesWithPrefix; getCurrentIteration expected to return a SOAP fault (runtime unverified).</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.soap.XPlanner public methods (43 public operations enumerated in .migration-tmp/stage-01/out/enumeration.json); #selectAccessibleObjects/#hasPermission (permission filtering). Query property paths (BA-001-05): XPlanner#getCurrentIteration passes "object.startDate &lt;= ? and object.endDate &gt;= ? and object.projectId = ?" to #getObjects, which builds "from net.sf.xplanner.domain.Iteration where " + condition without declaring an alias; Iteration maps project (@ManyToOne) but no projectId. #getObjects logs "error loading objects" and rethrows. #getNotesForObject uses "attachedTo_Id = &lt;id&gt;", an unqualified column name (Note maps attachedToId, column attachedTo_id) whose treatment is framework behavior (GAP-011, Stage 3). Source: stage-02-pass-003 F-001. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/soap/XPlanner.java XPlanner#getCurrentIteration, #getObjects. WAR: classes byte-identical to the v1.1a4 release. The source confirms the condition text; how Hibernate treats it is framework behavior. Live question: Does getCurrentIteration return a SOAP fault, and does getNotesForObject return the notes of an object?</t>
+    <t>Operations getProjects, getProject, getIterations, getIteration, getUserStories, getUserStory, getTasks, getTask, getCurrentTasksForPerson, getPlannedTasksForPerson, getTimeEntries, getTimeEntry, getNote, getNotesForObject, getPerson, getPeople, getAttribute, getAttributes, getAttributesWithPrefix return data, but the parent id fields of the returned beans (IterationData.projectId, UserStoryData.iterationId, TaskData.storyId, TimeEntryData.taskId) are 0; getAttribute always returns a SOAP fault (TypeMismatchException); getAttributesWithPrefix returns the keys without the prefix; getCurrentIteration returns a SOAP fault (W001).</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.soap.XPlanner public methods (43 public operations enumerated in .migration-tmp/stage-01/out/enumeration.json); #selectAccessibleObjects/#hasPermission (permission filtering). Query property paths (BA-001-05): XPlanner#getCurrentIteration passes "object.startDate &lt;= ? and object.endDate &gt;= ? and object.projectId = ?" to #getObjects, which builds "from net.sf.xplanner.domain.Iteration where " + condition without declaring an alias; Iteration maps project (@ManyToOne) but no projectId. #getObjects logs "error loading objects" and rethrows. #getNotesForObject uses "attachedTo_Id = &lt;id&gt;", an unqualified column name (Note maps attachedToId, column attachedTo_id) whose treatment is framework behavior (GAP-011, Stage 3). Source: stage-02-pass-003 F-001. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/soap/XPlanner.java XPlanner#getCurrentIteration, #getObjects. WAR: classes byte-identical to the v1.1a4 release. The source confirms the condition text; how Hibernate treats it is framework behavior. Live question: Does getCurrentIteration return a SOAP fault, and does getNotesForObject return the notes of an object? Stage 3 W001 (BA-001-13, MC-A-43, MC-B-08, W001-F-50, W001-F-51): all read operations answered with data, parent references 0 (D-C-046); getAttribute TypeMismatchException, getAttributesWithPrefix without prefix (D-C-044, D-C-049). Status Inferred -&gt; Partial (R-G2: getAttribute fails and the parent ids are lost). Stage 3 W001 live answer (BA-001-13, MC-C-30): getCurrentIteration faults (QuerySyntaxException near the undeclared alias "object"); getNotesForObject returns the notes of the story (D-C-047, D-C-048). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks D-C-046, D-C-047, D-C-048, D-C-049).</t>
   </si>
   <si>
     <t>SOAP write operations</t>
   </si>
   <si>
-    <t>Clients can add, update and remove projects, iterations, stories, tasks, time entries, notes and people, and set/delete object attributes, subject to permissions, with history recorded.</t>
+    <t>Clients can add, update and remove projects, iterations, stories, tasks, time entries, notes and people, and set/delete object attributes, subject to permissions, with history recorded (source). Live (W001): addIteration faults (TransientObjectException, Project) and addTask faults (ConstraintViolationException); addUserStory and addTimeEntry return an id but create the object without its parent (the story has no iteration, so only the system administrator can still read or remove it; the time entry is not attached to the task); addProject, addNote, addPerson, all update and all remove operations work; removeProject leaves the project's notes; deleteAttribute faults (QueryException, targetId).</t>
   </si>
   <si>
     <t>Automated maintenance of planning data.</t>
   </si>
   <si>
-    <t>Operations addX/update/removeX, setAttribute, deleteAttribute.</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.soap.XPlanner (addProject ... removePerson, update(*Data), setAttribute, deleteAttribute; #saveHistory, #hasPermission). Server-side enforcement (CHK-002, BA-001-04): enforced on the server by XPlanner#hasPermission for the object operations; the attribute operations have no check (row 218). Delete cascade sweep (BA-001-04): XPlanner#removeObject calls Session.delete, so the mapping cascades of the web deletes apply (rows 82, 91, 126, 142) and notes attached to the removed object are not deleted (NoteHelper#deleteNotesFor is not reached). Query property paths (BA-001-05): deleteAttribute calls AttributeRepositoryImpl#delete with "from a in net.sf.xplanner.domain.Attribute where a.targetId = ? and a.name = ?"; Attribute keeps targetId and name in its embedded id (#getAttributeId, @EmbeddedId; #getName is @Transient), so a.targetId and a.name are not mapped paths and deleteAttribute is expected to fail. setAttribute and getAttributes use unqualified targetId and name (framework behavior, GAP-011). Sweep of pass-003 F-001. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/soap/XPlanner.java XPlanner#addObject, #updateObject, #removeObject, #saveHistory; SRC:src/com/technoetic/xplanner/domain/repository/AttributeRepositoryImpl.java AttributeRepositoryImpl#delete. WAR: classes byte-identical to the v1.1a4 release. Permission checks and history on the object operations are confirmed; the delete cascades and the deleteAttribute query depend on Hibernate. Live question: Does SOAP removeProject leave the project notes, and does deleteAttribute fail?</t>
+    <t>Operations addX/update/removeX, setAttribute, deleteAttribute, with the per-operation outcomes stated in the requirement (W001).</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.soap.XPlanner (addProject ... removePerson, update(*Data), setAttribute, deleteAttribute; #saveHistory, #hasPermission). Server-side enforcement (CHK-002, BA-001-04): enforced on the server by XPlanner#hasPermission for the object operations; the attribute operations have no check (row 218). Delete cascade sweep (BA-001-04): XPlanner#removeObject calls Session.delete, so the mapping cascades of the web deletes apply (rows 82, 91, 126, 142) and notes attached to the removed object are not deleted (NoteHelper#deleteNotesFor is not reached). Query property paths (BA-001-05): deleteAttribute calls AttributeRepositoryImpl#delete with "from a in net.sf.xplanner.domain.Attribute where a.targetId = ? and a.name = ?"; Attribute keeps targetId and name in its embedded id (#getAttributeId, @EmbeddedId; #getName is @Transient), so a.targetId and a.name are not mapped paths and deleteAttribute is expected to fail. setAttribute and getAttributes use unqualified targetId and name (framework behavior, GAP-011). Sweep of pass-003 F-001. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/soap/XPlanner.java XPlanner#addObject, #updateObject, #removeObject, #saveHistory; SRC:src/com/technoetic/xplanner/domain/repository/AttributeRepositoryImpl.java AttributeRepositoryImpl#delete. WAR: classes byte-identical to the v1.1a4 release. Permission checks and history on the object operations are confirmed; the delete cascades and the deleteAttribute query depend on Hibernate. Live question: Does SOAP removeProject leave the project notes, and does deleteAttribute fail? Stage 3 W001 (BA-001-13, MC-A-44, W001-F-52): D-C-051 (addIteration, editor and system administrator), D-C-052 (addUserStory without iteration), D-C-053 (addTask), D-C-054 (addTimeEntry not attached; getTimeEntry and removeTimeEntry of it fault NullPointerException). Status Inferred -&gt; Partial. Stage 3 W001 live answer (BA-001-13, MC-C-31): Yes to both: the note of a removed project is still returned, and deleteAttribute faults (QueryException, targetId) (D-C-050, D-C-058). The D/F correction is under W001-F-52. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks D-C-050, D-C-051, D-C-052, D-C-053, D-C-054, D-C-055, D-C-056, D-C-057, D-C-058).</t>
   </si>
   <si>
     <t>UF-016</t>
@@ -2860,7 +2863,7 @@
     <t>XML/JSON payloads (ProjectView, UserStoryView[]).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:256-263,288-291 (Jersey SpringServlet /rest/*, POJOMappingFeature); class net.sf.xplanner.rest.ViewService (@Path "/view", "/project/{projectId}", "/iteration/{iterationId}/userstories", @Produces application/xml, application/json); WAR:WEB-INF/classes/spring-beans.xml:50 (component-scan net.sf.xplanner.rest). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/net/sf/xplanner/rest/ViewService.java ViewService#getProject, #getUserStories. WAR: classes byte-identical to the v1.1a4 release. The two GET resources return the project view and the story views as XML or JSON. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream.</t>
+    <t>WAR:WEB-INF/web.xml:256-263,288-291 (Jersey SpringServlet /rest/*, POJOMappingFeature); class net.sf.xplanner.rest.ViewService (@Path "/view", "/project/{projectId}", "/iteration/{iterationId}/userstories", @Produces application/xml, application/json); WAR:WEB-INF/classes/spring-beans.xml:50 (component-scan net.sf.xplanner.rest). Source reconciliation (BA-001-11, A4): confirmed at method level. SRC:src/net/sf/xplanner/rest/ViewService.java ViewService#getProject, #getUserStories. WAR: classes byte-identical to the v1.1a4 release. The two GET resources return the project view and the story views as XML or JSON. Provenance (fixed baseline, see reconnaissance GAP-005): P-05: the cited wiring is in spring-beans.xml, a rewritten entry that also carries the P-02 patch; the rest of the file is not guaranteed upstream. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-059).</t>
   </si>
   <si>
     <t>GET /rest/view returns a plain-text response.</t>
@@ -2872,7 +2875,7 @@
     <t>text/plain body.</t>
   </si>
   <si>
-    <t>class ViewService#getIt (@GET, @Produces text/plain). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/net/sf/xplanner/rest/ViewService.java ViewService#getIt. WAR: classes byte-identical to the v1.1a4 release. GET /rest/view returns a constant text/plain string.</t>
+    <t>class ViewService#getIt (@GET, @Produces text/plain). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/net/sf/xplanner/rest/ViewService.java ViewService#getIt. WAR: classes byte-identical to the v1.1a4 release. GET /rest/view returns a constant text/plain string. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-060).</t>
   </si>
   <si>
     <t>No security filter is mapped to /rest/*.</t>
@@ -2884,7 +2887,7 @@
     <t>Endpoints reachable without authentication (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:130-181 (no filter-mapping for /rest/*). BA-001-03 impact sweep of F-001: ViewService, UpdateService, ViewManager and UpdateManager reach no authorization call either (.migration-tmp/stage-01/out/authtrace.json). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/net/sf/xplanner/rest/ViewService.java ViewService; SRC:src/net/sf/xplanner/rest/UpdateService.java UpdateService; SRC:src/net/sf/xplanner/rest/ViewManager.java ViewManager; SRC:src/net/sf/xplanner/rest/UpdateManager.java UpdateManager. WAR: web.xml identical to the SVN webapp copy. No filter mapping covers /rest/* and none of the REST classes calls an authorizer.</t>
+    <t>WAR:WEB-INF/web.xml:130-181 (no filter-mapping for /rest/*). BA-001-03 impact sweep of F-001: ViewService, UpdateService, ViewManager and UpdateManager reach no authorization call either (.migration-tmp/stage-01/out/authtrace.json). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/net/sf/xplanner/rest/ViewService.java ViewService; SRC:src/net/sf/xplanner/rest/UpdateService.java UpdateService; SRC:src/net/sf/xplanner/rest/ViewManager.java ViewManager; SRC:src/net/sf/xplanner/rest/UpdateManager.java UpdateManager. WAR: web.xml identical to the SVN webapp copy. No filter mapping covers /rest/* and none of the REST classes calls an authorizer. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-061).</t>
   </si>
   <si>
     <t>REST task status update</t>
@@ -2896,10 +2899,10 @@
     <t>Lets clients update task progress.</t>
   </si>
   <si>
-    <t>Result "Task updated", "Task not found", "Task status not changed" or "Moving Task to not started not implemented".</t>
-  </si>
-  <si>
-    <t>class net.sf.xplanner.rest.UpdateService (@Path "/update", @POST "/task/{taskId}/status", @FormParam status, originalEstimate); class net.sf.xplanner.rest.UpdateManager#updateTaskStatus (result strings); class net.sf.xplanner.domain.enums.TaskStatus. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/net/sf/xplanner/rest/UpdateService.java UpdateService#post; SRC:src/net/sf/xplanner/rest/UpdateManager.java UpdateManager#updateTaskStatus. WAR: classes byte-identical to the v1.1a4 release. The four results are returned as recorded: not found, unchanged status, not-started not implemented, otherwise started (with the original estimate) or completed and saved.</t>
+    <t>Result "Task updated", "Task not found", "Task status not changed" or "Moving Task to not started not implemented"; an unrecognized status value is answered like notStarted (code 402). The results are JSON objects {"code","decription","error"} (the field name is spelled "decription") with codes 0, 401, 402 and 404 (W001).</t>
+  </si>
+  <si>
+    <t>class net.sf.xplanner.rest.UpdateService (@Path "/update", @POST "/task/{taskId}/status", @FormParam status, originalEstimate); class net.sf.xplanner.rest.UpdateManager#updateTaskStatus (result strings); class net.sf.xplanner.domain.enums.TaskStatus. Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/net/sf/xplanner/rest/UpdateService.java UpdateService#post; SRC:src/net/sf/xplanner/rest/UpdateManager.java UpdateManager#updateTaskStatus. WAR: classes byte-identical to the v1.1a4 release. The four results are returned as recorded: not found, unchanged status, not-started not implemented, otherwise started (with the original estimate) or completed and saved. Stage 3 W001 (BA-001-13, MC-B-09, W001-F-53): status=bogus answered code 402 (D-C-063); started, repeated start, notStarted, completed and an unknown id answered codes 0, 401, 402, 0 and 404 (D-C-062). An XML form of the update result was not observed. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks D-C-062, D-C-063).</t>
   </si>
   <si>
     <t>UF-017</t>
@@ -2920,7 +2923,7 @@
     <t>Expected: the first query fails, "ical error" is logged and the servlet answers with sendError and the exception message; no VCALENDAR body (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:251-254,308-311 (iCalServlet /ical/*), :173-176 (BasicSecurityFilter /ical/*); class com.technoetic.xplanner.ical.iCalServlet#doGet, #generateTaskData, #generateTimeEntryData (HQL and VCALENDAR strings). Locale dependence (CHK-004, BA-001-04): the "non-overhead" filter compares the stored type with task.type.overhead from java.util.ResourceBundle.getBundle("ResourceBundle"), i.e. the JVM default locale (class iCalServlet#generateTaskData); overhead tasks saved under a different label are included (row 135). Query property paths (BA-001-05): class iCalServlet#generateTimeEntryData (called first, before #generateTaskData) and #generateTaskData pass HQL containing "task.story = story.id" to Session.find; net.sf.xplanner.domain.Task maps the story only as userStory (#getUserStory, @ManyToOne @JoinColumn story_id) and has no story property; mappings/Task.xml is not loaded (WAR:WEB-INF/classes/spring-beans.xml:77-81). The exception propagates to #doGet, whose handler logs "ical error" and calls HttpServletResponse.sendError (bytecode listing with exception table). The query failure itself is framework behavior (Hibernate rejects an unresolvable property path; GAP-011). Corrected in BA-001-05 (Source: stage-02-pass-003 F-001). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/ical/iCalServlet.java iCalServlet#doGet, #generateTimeEntryData, #generateTaskData. WAR: classes byte-identical to the v1.1a4 release. The queries use task.story as recorded; whether Hibernate rejects them is framework behavior. Live question: Does GET /ical/&lt;own userId&gt;.ics return an error instead of a calendar?</t>
+    <t>WAR:WEB-INF/web.xml:251-254,308-311 (iCalServlet /ical/*), :173-176 (BasicSecurityFilter /ical/*); class com.technoetic.xplanner.ical.iCalServlet#doGet, #generateTaskData, #generateTimeEntryData (HQL and VCALENDAR strings). Locale dependence (CHK-004, BA-001-04): the "non-overhead" filter compares the stored type with task.type.overhead from java.util.ResourceBundle.getBundle("ResourceBundle"), i.e. the JVM default locale (class iCalServlet#generateTaskData); overhead tasks saved under a different label are included (row 135). Query property paths (BA-001-05): class iCalServlet#generateTimeEntryData (called first, before #generateTaskData) and #generateTaskData pass HQL containing "task.story = story.id" to Session.find; net.sf.xplanner.domain.Task maps the story only as userStory (#getUserStory, @ManyToOne @JoinColumn story_id) and has no story property; mappings/Task.xml is not loaded (WAR:WEB-INF/classes/spring-beans.xml:77-81). The exception propagates to #doGet, whose handler logs "ical error" and calls HttpServletResponse.sendError (bytecode listing with exception table). The query failure itself is framework behavior (Hibernate rejects an unresolvable property path; GAP-011). Corrected in BA-001-05 (Source: stage-02-pass-003 F-001). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/ical/iCalServlet.java iCalServlet#doGet, #generateTimeEntryData, #generateTaskData. WAR: classes byte-identical to the v1.1a4 release. The queries use task.story as recorded; whether Hibernate rejects them is framework behavior. Live question: Does GET /ical/&lt;own userId&gt;.ics return an error instead of a calendar? Stage 3 W001 live answer (BA-001-13, MC-C-32): Yes: HTTP 500 with the query exception message ("could not resolve property: story"), no VCALENDAR, for all four roles; without credentials 401 Basic (D-C-064, D-C-065). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-064, D-C-065).</t>
   </si>
   <si>
     <t>Requests without a file name or without the .ics suffix are rejected.</t>
@@ -2932,7 +2935,7 @@
     <t>Messages "No iCal file requested." / "No .ics suffix for requested iCal file."</t>
   </si>
   <si>
-    <t>class iCalServlet#doGet (strings "No iCal file requested.", "No .ics suffix for requested iCal file."). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/ical/iCalServlet.java iCalServlet#doGet. WAR: classes byte-identical to the v1.1a4 release. A missing file name and a missing .ics suffix return HTTP 400 with the two messages.</t>
+    <t>class iCalServlet#doGet (strings "No iCal file requested.", "No .ics suffix for requested iCal file."). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/ical/iCalServlet.java iCalServlet#doGet. WAR: classes byte-identical to the v1.1a4 release. A missing file name and a missing .ics suffix return HTTP 400 with the two messages. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-066).</t>
   </si>
   <si>
     <t>Requesting another person's calendar requires admin.edit on system.person.</t>
@@ -2944,7 +2947,7 @@
     <t>Message "No authorization for accessing calendar for &lt;user&gt;".</t>
   </si>
   <si>
-    <t>class iCalServlet#doGet (strings "system.person", "admin.edit", "No authorization for accessing calendar for "). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/ical/iCalServlet.java iCalServlet#doGet. WAR: classes byte-identical to the v1.1a4 release. For another user's calendar the servlet requires admin.edit on system.person for some project (checked against the caller's own person id) and otherwise returns HTTP 403 with the message.</t>
+    <t>class iCalServlet#doGet (strings "system.person", "admin.edit", "No authorization for accessing calendar for "). Source reconciliation (BA-001-11, A4): confirmed at method level; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/ical/iCalServlet.java iCalServlet#doGet. WAR: classes byte-identical to the v1.1a4 release. For another user's calendar the servlet requires admin.edit on system.person for some project (checked against the caller's own person id) and otherwise returns HTTP 403 with the message. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-067, D-C-068).</t>
   </si>
   <si>
     <t>UF-018</t>
@@ -2962,10 +2965,10 @@
     <t>Read-only access from early mobile phones.</t>
   </si>
   <si>
-    <t>WML cards with links to the underlying objects (hard-coded /xplanner path). Submitting the WAP login is expected to fail with a null reference, and a view request that carries a projectId is expected to fail the same way, because these actions are created by Struts without Spring injection (runtime unverified).</t>
-  </si>
-  <si>
-    <t>WAR:WEB-INF/mobile-struts-config.xml:20-49 (7 actions); WAR:WEB-INF/jsp/wap/login.jsp, projects.jsp, project.jsp, iteration.jsp, story.jsp, task.jsp, person.jsp; WAR:WEB-INF/web.xml:98-109,155-158 (MobileSecurityFilter /do/mobile/*); WAR:WEB-INF/mobile-security.xml. All WML links hard-code /xplanner/do/mobile/..., which does not match the WAR context path /xplanner-plus. Wiring (BA-001-07, mechanism (a)): the seven mappings of WAR:WEB-INF/mobile-struts-config.xml:20-49 have no bean in action-servlet.xml; the Spring request processor falls back to the Struts-created instance (framework behavior, GAP-011), which receives no injection. AuthenticationAction#execute uses the authenticator field, set only by #setAuthenticator; DispatchForward#execute uses the authorizer field, set only by #setAuthorizer (sweep .migration-tmp/stage-01/out/wiring-07.txt, wiring-impact-07.txt). Corrected in BA-001-07 (Source: stage-02-pass-005 F-004). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/AuthenticationAction.java AuthenticationAction#execute (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/actions/DispatchForward.java DispatchForward#execute. WAR: classes byte-identical to the v1.1a4 release; WAP JSPs identical to the SVN webapp copies. Both actions depend on injected fields that the Struts-created instances do not receive; the outcome is a runtime effect. Live question: Does a WAP login submission fail with an error page?</t>
+    <t>WML cards with links to the underlying objects (hard-coded /xplanner path), as the pages are written. In this baseline every WAP login request fails with HTTP 500 (NullPointerException at AuthenticationAction.execute:47), including the display of the login card inside a signed-in web session, so no WAP action serves a WML page; views without projectId answer 404 (row 234) and with projectId HTTP 500 (W001).</t>
+  </si>
+  <si>
+    <t>WAR:WEB-INF/mobile-struts-config.xml:20-49 (7 actions); WAR:WEB-INF/jsp/wap/login.jsp, projects.jsp, project.jsp, iteration.jsp, story.jsp, task.jsp, person.jsp; WAR:WEB-INF/web.xml:98-109,155-158 (MobileSecurityFilter /do/mobile/*); WAR:WEB-INF/mobile-security.xml. All WML links hard-code /xplanner/do/mobile/..., which does not match the WAR context path /xplanner-plus. Wiring (BA-001-07, mechanism (a)): the seven mappings of WAR:WEB-INF/mobile-struts-config.xml:20-49 have no bean in action-servlet.xml; the Spring request processor falls back to the Struts-created instance (framework behavior, GAP-011), which receives no injection. AuthenticationAction#execute uses the authenticator field, set only by #setAuthenticator; DispatchForward#execute uses the authorizer field, set only by #setAuthorizer (sweep .migration-tmp/stage-01/out/wiring-07.txt, wiring-impact-07.txt). Corrected in BA-001-07 (Source: stage-02-pass-005 F-004). Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/AuthenticationAction.java AuthenticationAction#execute (withheld file, cited by path only); SRC:src/com/technoetic/xplanner/actions/DispatchForward.java DispatchForward#execute. WAR: classes byte-identical to the v1.1a4 release; WAP JSPs identical to the SVN webapp copies. Both actions depend on injected fields that the Struts-created instances do not receive; the outcome is a runtime effect. Live question: Does a WAP login submission fail with an error page? Stage 3 W001 (BA-001-13, MC-A-45, W001-F-54): GET /do/mobile/login twice and with ?action=authenticate: each HTTP 500 at AuthenticationAction.java:47, no WML (D-C-069). Stage 3 W001 live answer (BA-001-13, MC-C-33): Yes: HTTP 500, NullPointerException at AuthenticationAction.execute:47, for the submission and even for the login card display (D-C-069, D-C-070). The D/F correction is under W001-F-54. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks D-C-069, D-C-070).</t>
   </si>
   <si>
     <t>The general web security filter also covers /do/mobile/* and does not bypass /do/mobile/login, so an unauthenticated mobile login request is redirected to the HTML login.</t>
@@ -2977,7 +2980,7 @@
     <t>Redirect to /do/login before the mobile login is reached.</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/web.xml:155-163 (MobileSecurityFilter /do/mobile/* then WebSecurityFilter /do/*); WAR:WEB-INF/security.xml:2-6 (no /do/mobile/login bypass); class SecurityConfiguration#isSecureRequest. The viewer/editor/admin roles listed in WAR:WEB-INF/mobile-security.xml:11-15 are never evaluated (SecurityConfiguration#isAuthorized has no caller; stage-02-pass-001 F-004). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/filter/AbstractSecurityFilter.java AbstractSecurityFilter#doFilter; SRC:src/com/technoetic/xplanner/security/config/SecurityConfiguration.java SecurityConfiguration#isSecureRequest; SRC:src/com/technoetic/xplanner/security/filter/FormSecurityFilter.java FormSecurityFilter#onAuthenticationFailure. WAR: web.xml, security.xml and mobile-security.xml identical to the SVN webapp copies. Both filters are FormSecurityFilter instances; a request is secure unless it matches the filter's own bypass list. The mobile filter bypasses /do/mobile/login, but the web filter on /do/* uses security.xml, which does not, so an unauthenticated mobile login request is redirected to /do/login.</t>
+    <t>WAR:WEB-INF/web.xml:155-163 (MobileSecurityFilter /do/mobile/* then WebSecurityFilter /do/*); WAR:WEB-INF/security.xml:2-6 (no /do/mobile/login bypass); class SecurityConfiguration#isSecureRequest. The viewer/editor/admin roles listed in WAR:WEB-INF/mobile-security.xml:11-15 are never evaluated (SecurityConfiguration#isAuthorized has no caller; stage-02-pass-001 F-004). Source reconciliation (BA-001-11, A4): correction needed, corrected in this row; status Inferred -&gt; Yes. SRC:src/com/technoetic/xplanner/security/filter/AbstractSecurityFilter.java AbstractSecurityFilter#doFilter; SRC:src/com/technoetic/xplanner/security/config/SecurityConfiguration.java SecurityConfiguration#isSecureRequest; SRC:src/com/technoetic/xplanner/security/filter/FormSecurityFilter.java FormSecurityFilter#onAuthenticationFailure. WAR: web.xml, security.xml and mobile-security.xml identical to the SVN webapp copies. Both filters are FormSecurityFilter instances; a request is secure unless it matches the filter's own bypass list. The mobile filter bypasses /do/mobile/login, but the web filter on /do/* uses security.xml, which does not, so an unauthenticated mobile login request is redirected to /do/login. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-071).</t>
   </si>
   <si>
     <t>The WAP view actions are DispatchForward actions with authorization required (the default); the WML links pass only oid, so without a projectId parameter each view is expected to forward to the not-authorized page (absent) instead of the WML card.</t>
@@ -2989,7 +2992,7 @@
     <t>Not-authorized forward instead of the project, iteration, story, task or person card (runtime unverified).</t>
   </si>
   <si>
-    <t>WAR:WEB-INF/mobile-struts-config.xml:27-49 (type DispatchForward, no Spring bean and no authorizationRequired override); class DispatchForward#&lt;init&gt; (isAuthorizationRequired true) and #execute ("no project identifier supplied for secure access", forward "security/notAuthorized"); WAR:WEB-INF/jsp/wap/projects.jsp, project.jsp (links with oid only). Depends on Spring DelegatingTilesRequestProcessor falling back to the mapping type when no bean exists (framework behavior, GAP-011). BA-001-03 impact sweep of F-001. Null dependency (BA-001-07): because the Struts-created DispatchForward has no authorizer, a request that does carry a non-zero projectId is expected to fail with a null reference in #execute at Authorizer.hasPermission; without projectId the not-authorized forward described here remains the outcome. Source: stage-02-pass-005 F-004. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/DispatchForward.java DispatchForward#execute, #isSecure. WAR: classes byte-identical to the v1.1a4 release. The authorization-required default and the missing projectId branch are confirmed; the fallback to the mapping type without a bean is framework behavior. Live question: Which page does /do/mobile/view/project?oid=&lt;id&gt; show after a mobile login?</t>
+    <t>WAR:WEB-INF/mobile-struts-config.xml:27-49 (type DispatchForward, no Spring bean and no authorizationRequired override); class DispatchForward#&lt;init&gt; (isAuthorizationRequired true) and #execute ("no project identifier supplied for secure access", forward "security/notAuthorized"); WAR:WEB-INF/jsp/wap/projects.jsp, project.jsp (links with oid only). Depends on Spring DelegatingTilesRequestProcessor falling back to the mapping type when no bean exists (framework behavior, GAP-011). BA-001-03 impact sweep of F-001. Null dependency (BA-001-07): because the Struts-created DispatchForward has no authorizer, a request that does carry a non-zero projectId is expected to fail with a null reference in #execute at Authorizer.hasPermission; without projectId the not-authorized forward described here remains the outcome. Source: stage-02-pass-005 F-004. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/actions/DispatchForward.java DispatchForward#execute, #isSecure. WAR: classes byte-identical to the v1.1a4 release. The authorization-required default and the missing projectId branch are confirmed; the fallback to the mapping type without a bean is framework behavior. Live question: Which page does /do/mobile/view/project?oid=&lt;id&gt; show after a mobile login? Stage 3 W001 live answer (BA-001-13, MC-C-34): No mobile login is possible (row 232). In a web session the view answers 404 (notAuthorized.jsp missing); with projectId it answers HTTP 500 (NullPointerException in DispatchForward) (D-C-072, D-C-073). Status Inferred -&gt; Yes on this live observation: without projectId the view forwards to the absent not-authorized page. Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: live-verified; checks D-C-072, D-C-073).</t>
   </si>
 </sst>
 </file>
@@ -4560,7 +4563,7 @@
         <v>168</v>
       </c>
       <c r="G38" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H38" s="23" t="s">
         <v>169</v>
@@ -4618,7 +4621,7 @@
         <v>177</v>
       </c>
       <c r="G40" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H40" s="23" t="s">
         <v>178</v>
@@ -4760,7 +4763,7 @@
         <v>198</v>
       </c>
       <c r="G45" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H45" s="23" t="s">
         <v>199</v>
@@ -4846,7 +4849,7 @@
         <v>211</v>
       </c>
       <c r="G48" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H48" s="23" t="s">
         <v>212</v>
@@ -4962,7 +4965,7 @@
         <v>229</v>
       </c>
       <c r="G52" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H52" s="23" t="s">
         <v>230</v>
@@ -5102,7 +5105,7 @@
         <v>249</v>
       </c>
       <c r="G57" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H57" s="23" t="s">
         <v>250</v>
@@ -6394,7 +6397,7 @@
         <v>443</v>
       </c>
       <c r="G102" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H102" s="23" t="s">
         <v>444</v>
@@ -6772,7 +6775,7 @@
         <v>502</v>
       </c>
       <c r="G115" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H115" s="23" t="s">
         <v>503</v>
@@ -6800,7 +6803,7 @@
         <v>506</v>
       </c>
       <c r="G116" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H116" s="23" t="s">
         <v>507</v>
@@ -6828,7 +6831,7 @@
         <v>510</v>
       </c>
       <c r="G117" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H117" s="23" t="s">
         <v>511</v>
@@ -6856,7 +6859,7 @@
         <v>514</v>
       </c>
       <c r="G118" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H118" s="23" t="s">
         <v>515</v>
@@ -6884,7 +6887,7 @@
         <v>518</v>
       </c>
       <c r="G119" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H119" s="23" t="s">
         <v>519</v>
@@ -6938,7 +6941,7 @@
         <v>525</v>
       </c>
       <c r="G121" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H121" s="23" t="s">
         <v>526</v>
@@ -7022,7 +7025,7 @@
         <v>537</v>
       </c>
       <c r="G124" s="23" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="H124" s="23" t="s">
         <v>538</v>
@@ -7052,7 +7055,7 @@
         <v>542</v>
       </c>
       <c r="G125" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H125" s="23" t="s">
         <v>543</v>
@@ -7198,7 +7201,7 @@
         <v>564</v>
       </c>
       <c r="G130" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H130" s="23" t="s">
         <v>565</v>
@@ -7308,7 +7311,7 @@
         <v>579</v>
       </c>
       <c r="G134" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H134" s="23" t="s">
         <v>580</v>
@@ -7336,7 +7339,7 @@
         <v>583</v>
       </c>
       <c r="G135" s="23" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="H135" s="23" t="s">
         <v>584</v>
@@ -7600,7 +7603,7 @@
         <v>624</v>
       </c>
       <c r="G144" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H144" s="23" t="s">
         <v>625</v>
@@ -7628,7 +7631,7 @@
         <v>628</v>
       </c>
       <c r="G145" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H145" s="23" t="s">
         <v>629</v>
@@ -7656,7 +7659,7 @@
         <v>631</v>
       </c>
       <c r="G146" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H146" s="23" t="s">
         <v>632</v>
@@ -7684,7 +7687,7 @@
         <v>635</v>
       </c>
       <c r="G147" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H147" s="23" t="s">
         <v>636</v>
@@ -8217,13 +8220,13 @@
         <v>532</v>
       </c>
       <c r="F166" s="23" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
       <c r="G166" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H166" s="23" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="I166" s="23"/>
       <c r="J166" s="23"/>
@@ -8239,19 +8242,19 @@
         <v>39</v>
       </c>
       <c r="D167" s="23" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="E167" s="23" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="F167" s="23" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="G167" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H167" s="23" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="I167" s="23"/>
       <c r="J167" s="23"/>
@@ -8262,10 +8265,10 @@
     </row>
     <row r="168" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A168" s="20" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B168" s="20" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="C168" s="20" t="s">
         <v>30</v>
@@ -8287,25 +8290,25 @@
     <row r="169" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A169" s="21"/>
       <c r="B169" s="22" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="C169" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D169" s="23" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="E169" s="23" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="F169" s="23" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="G169" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H169" s="23" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="I169" s="23"/>
       <c r="J169" s="23"/>
@@ -8321,19 +8324,19 @@
         <v>39</v>
       </c>
       <c r="D170" s="23" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="E170" s="23" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="F170" s="23" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="G170" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H170" s="23" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="I170" s="23"/>
       <c r="J170" s="23"/>
@@ -8349,19 +8352,19 @@
         <v>39</v>
       </c>
       <c r="D171" s="23" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="E171" s="23" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="F171" s="23" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="G171" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H171" s="23" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="I171" s="23"/>
       <c r="J171" s="23"/>
@@ -8377,19 +8380,19 @@
         <v>39</v>
       </c>
       <c r="D172" s="23" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="E172" s="23" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="F172" s="23" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="G172" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H172" s="23" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="I172" s="23"/>
       <c r="J172" s="23"/>
@@ -8401,25 +8404,25 @@
     <row r="173" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A173" s="21"/>
       <c r="B173" s="22" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="C173" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D173" s="23" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="E173" s="23" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="F173" s="23" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="G173" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H173" s="23" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="I173" s="23"/>
       <c r="J173" s="23"/>
@@ -8435,19 +8438,19 @@
         <v>39</v>
       </c>
       <c r="D174" s="23" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="E174" s="23" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="F174" s="23" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="G174" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H174" s="23" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="I174" s="23"/>
       <c r="J174" s="23"/>
@@ -8459,25 +8462,25 @@
     <row r="175" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A175" s="21"/>
       <c r="B175" s="22" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="C175" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D175" s="23" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="E175" s="23" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="F175" s="23" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="G175" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H175" s="23" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="I175" s="23"/>
       <c r="J175" s="23"/>
@@ -8489,25 +8492,25 @@
     <row r="176" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A176" s="21"/>
       <c r="B176" s="22" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="C176" s="21" t="s">
         <v>39</v>
       </c>
       <c r="D176" s="23" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="E176" s="23" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="F176" s="23" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="G176" s="23" t="s">
         <v>99</v>
       </c>
       <c r="H176" s="23" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="I176" s="23"/>
       <c r="J176" s="23"/>
@@ -8518,10 +8521,10 @@
     </row>
     <row r="177" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A177" s="20" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B177" s="20" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="C177" s="20" t="s">
         <v>30</v>
@@ -8543,25 +8546,25 @@
     <row r="178" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A178" s="21"/>
       <c r="B178" s="22" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="C178" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D178" s="23" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="E178" s="23" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="F178" s="23" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="G178" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H178" s="23" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="I178" s="23"/>
       <c r="J178" s="23"/>
@@ -8577,19 +8580,19 @@
         <v>39</v>
       </c>
       <c r="D179" s="23" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="E179" s="23" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="F179" s="23" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="G179" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H179" s="23" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="I179" s="23"/>
       <c r="J179" s="23"/>
@@ -8605,19 +8608,19 @@
         <v>39</v>
       </c>
       <c r="D180" s="23" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="E180" s="23" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="F180" s="23" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="G180" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H180" s="23" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="I180" s="23"/>
       <c r="J180" s="23"/>
@@ -8633,19 +8636,19 @@
         <v>39</v>
       </c>
       <c r="D181" s="23" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="E181" s="23" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="F181" s="23" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="G181" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H181" s="23" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="I181" s="23"/>
       <c r="J181" s="23"/>
@@ -8657,25 +8660,25 @@
     <row r="182" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A182" s="21"/>
       <c r="B182" s="22" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="C182" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D182" s="23" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="E182" s="23" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="F182" s="23" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="G182" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H182" s="23" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="I182" s="23"/>
       <c r="J182" s="23"/>
@@ -8691,19 +8694,19 @@
         <v>39</v>
       </c>
       <c r="D183" s="23" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="E183" s="23" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="F183" s="23" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="G183" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H183" s="23" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="I183" s="23"/>
       <c r="J183" s="23"/>
@@ -8719,19 +8722,19 @@
         <v>39</v>
       </c>
       <c r="D184" s="23" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="E184" s="23" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="F184" s="23" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="G184" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H184" s="23" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="I184" s="23"/>
       <c r="J184" s="23"/>
@@ -8743,25 +8746,25 @@
     <row r="185" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A185" s="21"/>
       <c r="B185" s="22" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="C185" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D185" s="23" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="E185" s="23" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="F185" s="23" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="G185" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H185" s="23" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="I185" s="23"/>
       <c r="J185" s="23"/>
@@ -8773,25 +8776,25 @@
     <row r="186" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A186" s="21"/>
       <c r="B186" s="22" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="C186" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D186" s="23" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="E186" s="23" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="F186" s="23" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="G186" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H186" s="23" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="I186" s="23"/>
       <c r="J186" s="23"/>
@@ -8807,19 +8810,19 @@
         <v>90</v>
       </c>
       <c r="D187" s="23" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E187" s="23" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="F187" s="23" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="G187" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H187" s="23" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="I187" s="23"/>
       <c r="J187" s="23"/>
@@ -8831,25 +8834,25 @@
     <row r="188" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A188" s="21"/>
       <c r="B188" s="22" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="C188" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D188" s="23" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="E188" s="23" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="F188" s="23" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="G188" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H188" s="23" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="I188" s="23"/>
       <c r="J188" s="23"/>
@@ -8861,25 +8864,25 @@
     <row r="189" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A189" s="21"/>
       <c r="B189" s="22" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="C189" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D189" s="23" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="E189" s="23" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="F189" s="23" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="G189" s="23" t="s">
         <v>51</v>
       </c>
       <c r="H189" s="23" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="I189" s="23"/>
       <c r="J189" s="23"/>
@@ -8895,19 +8898,19 @@
         <v>39</v>
       </c>
       <c r="D190" s="23" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="E190" s="23" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="F190" s="23" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="G190" s="23" t="s">
         <v>99</v>
       </c>
       <c r="H190" s="23" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="I190" s="23"/>
       <c r="J190" s="23"/>
@@ -8919,25 +8922,25 @@
     <row r="191" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A191" s="21"/>
       <c r="B191" s="22" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="C191" s="21" t="s">
         <v>39</v>
       </c>
       <c r="D191" s="23" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="E191" s="23" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="F191" s="23" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="G191" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H191" s="23" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="I191" s="23"/>
       <c r="J191" s="23"/>
@@ -8953,19 +8956,19 @@
         <v>39</v>
       </c>
       <c r="D192" s="23" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="E192" s="23" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="F192" s="23" t="s">
-        <v>819</v>
+        <v>820</v>
       </c>
       <c r="G192" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H192" s="23" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="I192" s="23"/>
       <c r="J192" s="23"/>
@@ -8977,25 +8980,25 @@
     <row r="193" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A193" s="21"/>
       <c r="B193" s="22" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="C193" s="21" t="s">
         <v>39</v>
       </c>
       <c r="D193" s="23" t="s">
-        <v>822</v>
+        <v>823</v>
       </c>
       <c r="E193" s="23" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="F193" s="23" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
       <c r="G193" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H193" s="23" t="s">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="I193" s="23"/>
       <c r="J193" s="23"/>
@@ -9007,25 +9010,25 @@
     <row r="194" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A194" s="21"/>
       <c r="B194" s="22" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="C194" s="21" t="s">
         <v>39</v>
       </c>
       <c r="D194" s="23" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="E194" s="23" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="F194" s="23" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="G194" s="23" t="s">
         <v>99</v>
       </c>
       <c r="H194" s="23" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="I194" s="23"/>
       <c r="J194" s="23"/>
@@ -9036,10 +9039,10 @@
     </row>
     <row r="195" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A195" s="20" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="B195" s="20" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="C195" s="20" t="s">
         <v>30</v>
@@ -9061,25 +9064,25 @@
     <row r="196" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A196" s="21"/>
       <c r="B196" s="22" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="C196" s="21" t="s">
         <v>39</v>
       </c>
       <c r="D196" s="23" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="E196" s="23" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="F196" s="23" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="G196" s="23" t="s">
         <v>99</v>
       </c>
       <c r="H196" s="23" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="I196" s="23"/>
       <c r="J196" s="23"/>
@@ -9095,19 +9098,19 @@
         <v>39</v>
       </c>
       <c r="D197" s="23" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="E197" s="23" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="F197" s="23" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="G197" s="23" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H197" s="23" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="I197" s="23"/>
       <c r="J197" s="23"/>
@@ -9123,19 +9126,19 @@
         <v>90</v>
       </c>
       <c r="D198" s="23" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E198" s="23" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="F198" s="23" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="G198" s="23" t="s">
-        <v>51</v>
+        <v>99</v>
       </c>
       <c r="H198" s="23" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="I198" s="23"/>
       <c r="J198" s="23"/>
@@ -9146,10 +9149,10 @@
     </row>
     <row r="199" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A199" s="20" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="B199" s="20" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="C199" s="20" t="s">
         <v>30</v>
@@ -9171,25 +9174,25 @@
     <row r="200" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A200" s="21"/>
       <c r="B200" s="22" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="C200" s="21" t="s">
         <v>90</v>
       </c>
       <c r="D200" s="23" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="E200" s="23" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="F200" s="23" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="G200" s="23" t="s">
-        <v>51</v>
+        <v>99</v>
       </c>
       <c r="H200" s="23" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="I200" s="23"/>
       <c r="J200" s="23"/>
@@ -9205,19 +9208,19 @@
         <v>90</v>
       </c>
       <c r="D201" s="23" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="E201" s="23" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="F201" s="23" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="G201" s="23" t="s">
-        <v>51</v>
+        <v>99</v>
       </c>
       <c r="H201" s="23" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="I201" s="23"/>
       <c r="J201" s="23"/>
@@ -9233,19 +9236,19 @@
         <v>90</v>
       </c>
       <c r="D202" s="23" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="E202" s="23" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="F202" s="23" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="G202" s="23" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="H202" s="23" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="I202" s="23"/>
       <c r="J202" s="23"/>
@@ -9261,19 +9264,19 @@
         <v>90</v>
       </c>
       <c r="D203" s="23" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="E203" s="23" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="F203" s="23" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="G203" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H203" s="23" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="I203" s="23"/>
       <c r="J203" s="23"/>
@@ -9285,25 +9288,25 @@
     <row r="204" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A204" s="21"/>
       <c r="B204" s="22" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="C204" s="21" t="s">
         <v>90</v>
       </c>
       <c r="D204" s="23" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="E204" s="23" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="F204" s="23" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="G204" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H204" s="23" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="I204" s="23"/>
       <c r="J204" s="23"/>
@@ -9319,19 +9322,19 @@
         <v>90</v>
       </c>
       <c r="D205" s="23" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="E205" s="23" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="F205" s="23" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="G205" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H205" s="23" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="I205" s="23"/>
       <c r="J205" s="23"/>
@@ -9343,25 +9346,25 @@
     <row r="206" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A206" s="21"/>
       <c r="B206" s="22" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="C206" s="21" t="s">
         <v>90</v>
       </c>
       <c r="D206" s="23" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="E206" s="23" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="F206" s="23" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="G206" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H206" s="23" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="I206" s="23"/>
       <c r="J206" s="23"/>
@@ -9372,10 +9375,10 @@
     </row>
     <row r="207" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A207" s="20" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="B207" s="20" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="C207" s="20" t="s">
         <v>30</v>
@@ -9397,25 +9400,25 @@
     <row r="208" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A208" s="21"/>
       <c r="B208" s="22" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="C208" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D208" s="23" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="E208" s="23" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="F208" s="23" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="G208" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H208" s="23" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="I208" s="23"/>
       <c r="J208" s="23"/>
@@ -9427,25 +9430,25 @@
     <row r="209" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A209" s="21"/>
       <c r="B209" s="22" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="C209" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D209" s="23" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="E209" s="23" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="F209" s="23" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="G209" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H209" s="23" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="I209" s="23"/>
       <c r="J209" s="23"/>
@@ -9457,25 +9460,25 @@
     <row r="210" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A210" s="21"/>
       <c r="B210" s="22" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="C210" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D210" s="23" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
       <c r="E210" s="23" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="F210" s="23" t="s">
-        <v>894</v>
+        <v>895</v>
       </c>
       <c r="G210" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H210" s="23" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
       <c r="I210" s="23"/>
       <c r="J210" s="23"/>
@@ -9491,19 +9494,19 @@
         <v>39</v>
       </c>
       <c r="D211" s="23" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="E211" s="23" t="s">
-        <v>897</v>
+        <v>898</v>
       </c>
       <c r="F211" s="23" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="G211" s="23" t="s">
         <v>99</v>
       </c>
       <c r="H211" s="23" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="I211" s="23"/>
       <c r="J211" s="23"/>
@@ -9515,25 +9518,25 @@
     <row r="212" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A212" s="21"/>
       <c r="B212" s="22" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="C212" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D212" s="23" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="E212" s="23" t="s">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="F212" s="23" t="s">
-        <v>903</v>
+        <v>904</v>
       </c>
       <c r="G212" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H212" s="23" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="I212" s="23"/>
       <c r="J212" s="23"/>
@@ -9549,19 +9552,19 @@
         <v>39</v>
       </c>
       <c r="D213" s="23" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="E213" s="23" t="s">
-        <v>906</v>
+        <v>907</v>
       </c>
       <c r="F213" s="23" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="G213" s="23" t="s">
         <v>99</v>
       </c>
       <c r="H213" s="23" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="I213" s="23"/>
       <c r="J213" s="23"/>
@@ -9572,10 +9575,10 @@
     </row>
     <row r="214" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A214" s="20" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="B214" s="20" t="s">
-        <v>909</v>
+        <v>910</v>
       </c>
       <c r="C214" s="20" t="s">
         <v>30</v>
@@ -9597,25 +9600,25 @@
     <row r="215" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A215" s="21"/>
       <c r="B215" s="22" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="C215" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D215" s="23" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="E215" s="23" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="F215" s="23" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="G215" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H215" s="23" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="I215" s="23"/>
       <c r="J215" s="23"/>
@@ -9631,19 +9634,19 @@
         <v>39</v>
       </c>
       <c r="D216" s="23" t="s">
-        <v>915</v>
+        <v>916</v>
       </c>
       <c r="E216" s="23" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="F216" s="23" t="s">
-        <v>917</v>
+        <v>918</v>
       </c>
       <c r="G216" s="23" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="H216" s="23" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
       <c r="I216" s="23"/>
       <c r="J216" s="23"/>
@@ -9659,19 +9662,19 @@
         <v>39</v>
       </c>
       <c r="D217" s="23" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="E217" s="23" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
       <c r="F217" s="23" t="s">
-        <v>921</v>
+        <v>922</v>
       </c>
       <c r="G217" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H217" s="23" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="I217" s="23"/>
       <c r="J217" s="23"/>
@@ -9687,19 +9690,19 @@
         <v>39</v>
       </c>
       <c r="D218" s="23" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
       <c r="E218" s="23" t="s">
-        <v>924</v>
+        <v>925</v>
       </c>
       <c r="F218" s="23" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="G218" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H218" s="23" t="s">
-        <v>926</v>
+        <v>927</v>
       </c>
       <c r="I218" s="23"/>
       <c r="J218" s="23"/>
@@ -9715,19 +9718,19 @@
         <v>90</v>
       </c>
       <c r="D219" s="23" t="s">
-        <v>927</v>
+        <v>928</v>
       </c>
       <c r="E219" s="23" t="s">
-        <v>928</v>
+        <v>929</v>
       </c>
       <c r="F219" s="23" t="s">
-        <v>929</v>
+        <v>930</v>
       </c>
       <c r="G219" s="23" t="s">
-        <v>930</v>
+        <v>931</v>
       </c>
       <c r="H219" s="23" t="s">
-        <v>931</v>
+        <v>932</v>
       </c>
       <c r="I219" s="23"/>
       <c r="J219" s="23"/>
@@ -9739,25 +9742,25 @@
     <row r="220" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A220" s="21"/>
       <c r="B220" s="22" t="s">
-        <v>932</v>
+        <v>933</v>
       </c>
       <c r="C220" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D220" s="23" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="E220" s="23" t="s">
-        <v>934</v>
+        <v>935</v>
       </c>
       <c r="F220" s="23" t="s">
-        <v>935</v>
+        <v>936</v>
       </c>
       <c r="G220" s="23" t="s">
-        <v>51</v>
+        <v>99</v>
       </c>
       <c r="H220" s="23" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="I220" s="23"/>
       <c r="J220" s="23"/>
@@ -9769,25 +9772,25 @@
     <row r="221" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A221" s="21"/>
       <c r="B221" s="22" t="s">
-        <v>937</v>
+        <v>938</v>
       </c>
       <c r="C221" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D221" s="23" t="s">
-        <v>938</v>
+        <v>939</v>
       </c>
       <c r="E221" s="23" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="F221" s="23" t="s">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="G221" s="23" t="s">
-        <v>51</v>
+        <v>99</v>
       </c>
       <c r="H221" s="23" t="s">
-        <v>941</v>
+        <v>942</v>
       </c>
       <c r="I221" s="23"/>
       <c r="J221" s="23"/>
@@ -9798,10 +9801,10 @@
     </row>
     <row r="222" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A222" s="20" t="s">
-        <v>942</v>
+        <v>943</v>
       </c>
       <c r="B222" s="20" t="s">
-        <v>943</v>
+        <v>944</v>
       </c>
       <c r="C222" s="20" t="s">
         <v>30</v>
@@ -9823,25 +9826,25 @@
     <row r="223" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A223" s="21"/>
       <c r="B223" s="22" t="s">
-        <v>944</v>
+        <v>945</v>
       </c>
       <c r="C223" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D223" s="23" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
       <c r="E223" s="23" t="s">
-        <v>946</v>
+        <v>947</v>
       </c>
       <c r="F223" s="23" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="G223" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H223" s="23" t="s">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="I223" s="23"/>
       <c r="J223" s="23"/>
@@ -9857,19 +9860,19 @@
         <v>39</v>
       </c>
       <c r="D224" s="23" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="E224" s="23" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="F224" s="23" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="G224" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H224" s="23" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="I224" s="23"/>
       <c r="J224" s="23"/>
@@ -9885,19 +9888,19 @@
         <v>39</v>
       </c>
       <c r="D225" s="23" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="E225" s="23" t="s">
-        <v>954</v>
+        <v>955</v>
       </c>
       <c r="F225" s="23" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="G225" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H225" s="23" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
       <c r="I225" s="23"/>
       <c r="J225" s="23"/>
@@ -9909,25 +9912,25 @@
     <row r="226" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A226" s="21"/>
       <c r="B226" s="22" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="C226" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D226" s="23" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="E226" s="23" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
       <c r="F226" s="23" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="G226" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H226" s="23" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="I226" s="23"/>
       <c r="J226" s="23"/>
@@ -9938,10 +9941,10 @@
     </row>
     <row r="227" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A227" s="20" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="B227" s="20" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="C227" s="20" t="s">
         <v>30</v>
@@ -9963,25 +9966,25 @@
     <row r="228" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A228" s="21"/>
       <c r="B228" s="22" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="C228" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D228" s="23" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="E228" s="23" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="F228" s="23" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="G228" s="23" t="s">
         <v>99</v>
       </c>
       <c r="H228" s="23" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="I228" s="23"/>
       <c r="J228" s="23"/>
@@ -9997,19 +10000,19 @@
         <v>39</v>
       </c>
       <c r="D229" s="23" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="E229" s="23" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="F229" s="23" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="G229" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H229" s="23" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="I229" s="23"/>
       <c r="J229" s="23"/>
@@ -10025,19 +10028,19 @@
         <v>39</v>
       </c>
       <c r="D230" s="23" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="E230" s="23" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="F230" s="23" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="G230" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H230" s="23" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="I230" s="23"/>
       <c r="J230" s="23"/>
@@ -10048,10 +10051,10 @@
     </row>
     <row r="231" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A231" s="20" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="B231" s="20" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="C231" s="20" t="s">
         <v>30</v>
@@ -10073,25 +10076,25 @@
     <row r="232" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A232" s="21"/>
       <c r="B232" s="22" t="s">
-        <v>979</v>
+        <v>980</v>
       </c>
       <c r="C232" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D232" s="23" t="s">
-        <v>980</v>
+        <v>981</v>
       </c>
       <c r="E232" s="23" t="s">
-        <v>981</v>
+        <v>982</v>
       </c>
       <c r="F232" s="23" t="s">
-        <v>982</v>
+        <v>983</v>
       </c>
       <c r="G232" s="23" t="s">
         <v>99</v>
       </c>
       <c r="H232" s="23" t="s">
-        <v>983</v>
+        <v>984</v>
       </c>
       <c r="I232" s="23"/>
       <c r="J232" s="23"/>
@@ -10107,19 +10110,19 @@
         <v>39</v>
       </c>
       <c r="D233" s="23" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="E233" s="23" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
       <c r="F233" s="23" t="s">
-        <v>986</v>
+        <v>987</v>
       </c>
       <c r="G233" s="23" t="s">
         <v>37</v>
       </c>
       <c r="H233" s="23" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
       <c r="I233" s="23"/>
       <c r="J233" s="23"/>
@@ -10135,19 +10138,19 @@
         <v>39</v>
       </c>
       <c r="D234" s="23" t="s">
-        <v>988</v>
+        <v>989</v>
       </c>
       <c r="E234" s="23" t="s">
-        <v>989</v>
+        <v>990</v>
       </c>
       <c r="F234" s="23" t="s">
-        <v>990</v>
+        <v>991</v>
       </c>
       <c r="G234" s="23" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="H234" s="23" t="s">
-        <v>991</v>
+        <v>992</v>
       </c>
       <c r="I234" s="23"/>
       <c r="J234" s="23"/>

</xml_diff>

<commit_message>
Stage 1 BA-001-14: narrow correction of F220 (Stage 4 map hole MH-01)
Finding-driven return from Stage 4. F220 no longer lists getAttribute among
the SOAP read operations that return data; it states that getAttribute always
faults (W001 D-C-044, D-C-049, W001-F-50, MC-A-43). The tied H220 wording is
narrowed the same way. Only row 220 changed; no status change; target
decisions I-N, Rev 1, other rows, the reconnaissance and sealed records are
untouched; the 7 open pass-013 findings stay open. Next: a fresh
correction-validation, then back to Stage 4.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -3179,10 +3179,10 @@
     <t>Read access to planning data.</t>
   </si>
   <si>
-    <t>Operations getProjects, getProject, getIterations, getIteration, getUserStories, getUserStory, getTasks, getTask, getCurrentTasksForPerson, getPlannedTasksForPerson, getTimeEntries, getTimeEntry, getNote, getNotesForObject, getPerson, getPeople, getAttribute, getAttributes, getAttributesWithPrefix return data, but the parent id fields of the returned beans (IterationData.projectId, UserStoryData.iterationId, TaskData.storyId, TimeEntryData.taskId) are 0; getAttribute always returns a SOAP fault (TypeMismatchException); getAttributesWithPrefix returns the keys without the prefix; getCurrentIteration returns a SOAP fault (W001).</t>
-  </si>
-  <si>
-    <t>class com.technoetic.xplanner.soap.XPlanner public methods (43 public operations enumerated in .migration-tmp/stage-01/out/enumeration.json); #selectAccessibleObjects/#hasPermission (permission filtering). Query property paths (BA-001-05): XPlanner#getCurrentIteration passes "object.startDate &lt;= ? and object.endDate &gt;= ? and object.projectId = ?" to #getObjects, which builds "from net.sf.xplanner.domain.Iteration where " + condition without declaring an alias; Iteration maps project (@ManyToOne) but no projectId. #getObjects logs "error loading objects" and rethrows. #getNotesForObject uses "attachedTo_Id = &lt;id&gt;", an unqualified column name (Note maps attachedToId, column attachedTo_id) whose treatment is framework behavior (GAP-011, Stage 3). Source: stage-02-pass-003 F-001. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/soap/XPlanner.java XPlanner#getCurrentIteration, #getObjects. WAR: classes byte-identical to the v1.1a4 release. The source confirms the condition text; how Hibernate treats it is framework behavior. Live question: Does getCurrentIteration return a SOAP fault, and does getNotesForObject return the notes of an object? Stage 3 W001 (BA-001-13, MC-A-43, MC-B-08, W001-F-50, W001-F-51): all read operations answered with data, parent references 0 (D-C-046); getAttribute TypeMismatchException, getAttributesWithPrefix without prefix (D-C-044, D-C-049). Status Inferred -&gt; Partial (R-G2: getAttribute fails and the parent ids are lost). Stage 3 W001 live answer (BA-001-13, MC-C-30): getCurrentIteration faults (QuerySyntaxException near the undeclared alias "object"); getNotesForObject returns the notes of the story (D-C-047, D-C-048). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks D-C-046, D-C-047, D-C-048, D-C-049).</t>
+    <t>Operations getProjects, getProject, getIterations, getIteration, getUserStories, getUserStory, getTasks, getTask, getCurrentTasksForPerson, getPlannedTasksForPerson, getTimeEntries, getTimeEntry, getNote, getNotesForObject, getPerson, getPeople, getAttributes, getAttributesWithPrefix return data, but the parent id fields of the returned beans (IterationData.projectId, UserStoryData.iterationId, TaskData.storyId, TimeEntryData.taskId) are 0; getAttributesWithPrefix returns the keys without the prefix; getAttribute does not return data: it always returns a SOAP fault (TypeMismatchException); getCurrentIteration returns a SOAP fault (W001).</t>
+  </si>
+  <si>
+    <t>class com.technoetic.xplanner.soap.XPlanner public methods (43 public operations enumerated in .migration-tmp/stage-01/out/enumeration.json); #selectAccessibleObjects/#hasPermission (permission filtering). Query property paths (BA-001-05): XPlanner#getCurrentIteration passes "object.startDate &lt;= ? and object.endDate &gt;= ? and object.projectId = ?" to #getObjects, which builds "from net.sf.xplanner.domain.Iteration where " + condition without declaring an alias; Iteration maps project (@ManyToOne) but no projectId. #getObjects logs "error loading objects" and rethrows. #getNotesForObject uses "attachedTo_Id = &lt;id&gt;", an unqualified column name (Note maps attachedToId, column attachedTo_id) whose treatment is framework behavior (GAP-011, Stage 3). Source: stage-02-pass-003 F-001. Source reconciliation (BA-001-11, A4): runtime-only. SRC:src/com/technoetic/xplanner/soap/XPlanner.java XPlanner#getCurrentIteration, #getObjects. WAR: classes byte-identical to the v1.1a4 release. The source confirms the condition text; how Hibernate treats it is framework behavior. Live question: Does getCurrentIteration return a SOAP fault, and does getNotesForObject return the notes of an object? Stage 3 W001 (BA-001-13, MC-A-43, MC-B-08, W001-F-50, W001-F-51): the read operations listed in F220 other than getAttribute answered with data, parent references 0 (D-C-046); getAttribute TypeMismatchException, getAttributesWithPrefix without prefix (D-C-044, D-C-049). Status Inferred -&gt; Partial (R-G2: getAttribute fails and the parent ids are lost). Stage 3 W001 live answer (BA-001-13, MC-C-30): getCurrentIteration faults (QuerySyntaxException near the undeclared alias "object"); getNotesForObject returns the notes of the story (D-C-047, D-C-048). Stage 4 MH-01 correction (BA-001-14): getAttribute is no longer listed among the operations that return data, because it always faults (D-C-044, D-C-049, W001-F-50, MC-A-43). Runtime: live-observed (Stage 3 W001, analysis/stages/stage-03/walkthrough-001.md; W001 row verdict: difference; checks D-C-046, D-C-047, D-C-048, D-C-049).</t>
   </si>
   <si>
     <t>SOAP write operations</t>
@@ -4419,7 +4419,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O234"/>
+  <dimension ref="A1:N234"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="1" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="10.625" customWidth="1"/>
@@ -4437,7 +4437,7 @@
     <col min="14" max="14" width="48.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20.25" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" ht="20.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4455,7 +4455,7 @@
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -4473,7 +4473,7 @@
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
     </row>
-    <row r="3" ht="31.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" ht="31.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -4491,7 +4491,7 @@
       <c r="M3" s="5"/>
       <c r="N3" s="5"/>
     </row>
-    <row r="4" ht="54" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="54" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
@@ -4523,7 +4523,7 @@
       <c r="M4" s="9"/>
       <c r="N4" s="9"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>11</v>
       </c>
@@ -4545,7 +4545,7 @@
       <c r="M5" s="13"/>
       <c r="N5" s="14"/>
     </row>
-    <row r="6" ht="37.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" ht="37.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
         <v>14</v>
       </c>
@@ -4589,7 +4589,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="20" t="s">
         <v>28</v>
       </c>
@@ -4613,7 +4613,7 @@
       <c r="M7" s="20"/>
       <c r="N7" s="20"/>
     </row>
-    <row r="8" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="8" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A8" s="21"/>
       <c r="B8" s="22" t="s">
         <v>32</v>
@@ -4645,7 +4645,7 @@
       <c r="M8" s="23"/>
       <c r="N8" s="23"/>
     </row>
-    <row r="9" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="9" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A9" s="21"/>
       <c r="B9" s="21"/>
       <c r="C9" s="21" t="s">
@@ -4675,7 +4675,7 @@
       <c r="M9" s="23"/>
       <c r="N9" s="23"/>
     </row>
-    <row r="10" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="10" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A10" s="21"/>
       <c r="B10" s="21"/>
       <c r="C10" s="21" t="s">
@@ -4705,7 +4705,7 @@
       <c r="M10" s="23"/>
       <c r="N10" s="23"/>
     </row>
-    <row r="11" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="11" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A11" s="21"/>
       <c r="B11" s="21"/>
       <c r="C11" s="21" t="s">
@@ -4735,7 +4735,7 @@
       <c r="M11" s="23"/>
       <c r="N11" s="23"/>
     </row>
-    <row r="12" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="12" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A12" s="21"/>
       <c r="B12" s="22" t="s">
         <v>57</v>
@@ -4767,7 +4767,7 @@
       <c r="M12" s="23"/>
       <c r="N12" s="23"/>
     </row>
-    <row r="13" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="13" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A13" s="21"/>
       <c r="B13" s="21"/>
       <c r="C13" s="21" t="s">
@@ -4797,7 +4797,7 @@
       <c r="M13" s="23"/>
       <c r="N13" s="23"/>
     </row>
-    <row r="14" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="14" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A14" s="21"/>
       <c r="B14" s="21"/>
       <c r="C14" s="21" t="s">
@@ -4827,7 +4827,7 @@
       <c r="M14" s="23"/>
       <c r="N14" s="23"/>
     </row>
-    <row r="15" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="15" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A15" s="21"/>
       <c r="B15" s="22" t="s">
         <v>72</v>
@@ -4861,7 +4861,7 @@
       </c>
       <c r="N15" s="24"/>
     </row>
-    <row r="16" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="16" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A16" s="21"/>
       <c r="B16" s="21"/>
       <c r="C16" s="21" t="s">
@@ -4893,7 +4893,7 @@
       </c>
       <c r="N16" s="24"/>
     </row>
-    <row r="17" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="17" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A17" s="21"/>
       <c r="B17" s="22" t="s">
         <v>82</v>
@@ -4925,7 +4925,7 @@
       <c r="M17" s="23"/>
       <c r="N17" s="23"/>
     </row>
-    <row r="18" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="18" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A18" s="21"/>
       <c r="B18" s="21"/>
       <c r="C18" s="21" t="s">
@@ -4955,7 +4955,7 @@
       <c r="M18" s="23"/>
       <c r="N18" s="23"/>
     </row>
-    <row r="19" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="19" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A19" s="21"/>
       <c r="B19" s="22" t="s">
         <v>92</v>
@@ -4987,7 +4987,7 @@
       <c r="M19" s="23"/>
       <c r="N19" s="23"/>
     </row>
-    <row r="20" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="20" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A20" s="21"/>
       <c r="B20" s="22" t="s">
         <v>97</v>
@@ -5019,7 +5019,7 @@
       <c r="M20" s="23"/>
       <c r="N20" s="23"/>
     </row>
-    <row r="21" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="21" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A21" s="21"/>
       <c r="B21" s="22" t="s">
         <v>103</v>
@@ -5053,7 +5053,7 @@
       </c>
       <c r="N21" s="24"/>
     </row>
-    <row r="22" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
         <v>110</v>
       </c>
@@ -5077,7 +5077,7 @@
       <c r="M22" s="20"/>
       <c r="N22" s="20"/>
     </row>
-    <row r="23" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="23" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A23" s="21"/>
       <c r="B23" s="22" t="s">
         <v>112</v>
@@ -5109,7 +5109,7 @@
       <c r="M23" s="23"/>
       <c r="N23" s="23"/>
     </row>
-    <row r="24" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="24" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A24" s="21"/>
       <c r="B24" s="21"/>
       <c r="C24" s="21" t="s">
@@ -5139,7 +5139,7 @@
       <c r="M24" s="23"/>
       <c r="N24" s="23"/>
     </row>
-    <row r="25" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="25" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A25" s="21"/>
       <c r="B25" s="21"/>
       <c r="C25" s="21" t="s">
@@ -5169,7 +5169,7 @@
       <c r="M25" s="23"/>
       <c r="N25" s="23"/>
     </row>
-    <row r="26" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="26" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A26" s="21"/>
       <c r="B26" s="22" t="s">
         <v>127</v>
@@ -5201,7 +5201,7 @@
       <c r="M26" s="23"/>
       <c r="N26" s="23"/>
     </row>
-    <row r="27" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="27" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A27" s="21"/>
       <c r="B27" s="21"/>
       <c r="C27" s="21" t="s">
@@ -5231,7 +5231,7 @@
       <c r="M27" s="23"/>
       <c r="N27" s="23"/>
     </row>
-    <row r="28" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="28" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A28" s="21"/>
       <c r="B28" s="21"/>
       <c r="C28" s="21" t="s">
@@ -5261,7 +5261,7 @@
       <c r="M28" s="23"/>
       <c r="N28" s="23"/>
     </row>
-    <row r="29" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="29" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A29" s="21"/>
       <c r="B29" s="22" t="s">
         <v>142</v>
@@ -5293,7 +5293,7 @@
       <c r="M29" s="23"/>
       <c r="N29" s="23"/>
     </row>
-    <row r="30" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="30" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A30" s="21"/>
       <c r="B30" s="21"/>
       <c r="C30" s="21" t="s">
@@ -5323,7 +5323,7 @@
       <c r="M30" s="23"/>
       <c r="N30" s="23"/>
     </row>
-    <row r="31" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="31" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A31" s="21"/>
       <c r="B31" s="21"/>
       <c r="C31" s="21" t="s">
@@ -5353,7 +5353,7 @@
       <c r="M31" s="23"/>
       <c r="N31" s="23"/>
     </row>
-    <row r="32" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="32" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A32" s="21"/>
       <c r="B32" s="21"/>
       <c r="C32" s="21" t="s">
@@ -5383,7 +5383,7 @@
       <c r="M32" s="23"/>
       <c r="N32" s="23"/>
     </row>
-    <row r="33" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="33" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A33" s="21"/>
       <c r="B33" s="22" t="s">
         <v>161</v>
@@ -5415,7 +5415,7 @@
       <c r="M33" s="23"/>
       <c r="N33" s="23"/>
     </row>
-    <row r="34" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="34" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A34" s="21"/>
       <c r="B34" s="21"/>
       <c r="C34" s="21" t="s">
@@ -5445,7 +5445,7 @@
       <c r="M34" s="23"/>
       <c r="N34" s="23"/>
     </row>
-    <row r="35" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="35" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A35" s="21"/>
       <c r="B35" s="22" t="s">
         <v>171</v>
@@ -5477,7 +5477,7 @@
       <c r="M35" s="23"/>
       <c r="N35" s="23"/>
     </row>
-    <row r="36" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="20" t="s">
         <v>177</v>
       </c>
@@ -5501,7 +5501,7 @@
       <c r="M36" s="20"/>
       <c r="N36" s="20"/>
     </row>
-    <row r="37" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="37" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A37" s="21"/>
       <c r="B37" s="22" t="s">
         <v>179</v>
@@ -5533,7 +5533,7 @@
       <c r="M37" s="23"/>
       <c r="N37" s="23"/>
     </row>
-    <row r="38" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="38" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A38" s="21"/>
       <c r="B38" s="21"/>
       <c r="C38" s="21" t="s">
@@ -5563,7 +5563,7 @@
       <c r="M38" s="23"/>
       <c r="N38" s="23"/>
     </row>
-    <row r="39" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="39" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A39" s="21"/>
       <c r="B39" s="21"/>
       <c r="C39" s="21" t="s">
@@ -5593,7 +5593,7 @@
       <c r="M39" s="23"/>
       <c r="N39" s="23"/>
     </row>
-    <row r="40" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="40" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A40" s="21"/>
       <c r="B40" s="22" t="s">
         <v>194</v>
@@ -5625,7 +5625,7 @@
       <c r="M40" s="23"/>
       <c r="N40" s="23"/>
     </row>
-    <row r="41" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="41" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A41" s="21"/>
       <c r="B41" s="21"/>
       <c r="C41" s="21" t="s">
@@ -5655,7 +5655,7 @@
       <c r="M41" s="23"/>
       <c r="N41" s="23"/>
     </row>
-    <row r="42" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="42" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A42" s="21"/>
       <c r="B42" s="21"/>
       <c r="C42" s="21" t="s">
@@ -5685,7 +5685,7 @@
       <c r="M42" s="23"/>
       <c r="N42" s="23"/>
     </row>
-    <row r="43" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="43" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A43" s="21"/>
       <c r="B43" s="22" t="s">
         <v>208</v>
@@ -5717,7 +5717,7 @@
       <c r="M43" s="23"/>
       <c r="N43" s="23"/>
     </row>
-    <row r="44" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="44" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A44" s="21"/>
       <c r="B44" s="21"/>
       <c r="C44" s="21" t="s">
@@ -5747,7 +5747,7 @@
       <c r="M44" s="23"/>
       <c r="N44" s="23"/>
     </row>
-    <row r="45" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="45" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A45" s="21"/>
       <c r="B45" s="21"/>
       <c r="C45" s="21" t="s">
@@ -5777,7 +5777,7 @@
       <c r="M45" s="23"/>
       <c r="N45" s="23"/>
     </row>
-    <row r="46" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="46" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A46" s="21"/>
       <c r="B46" s="22" t="s">
         <v>223</v>
@@ -5809,7 +5809,7 @@
       <c r="M46" s="23"/>
       <c r="N46" s="23"/>
     </row>
-    <row r="47" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="47" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A47" s="21"/>
       <c r="B47" s="21"/>
       <c r="C47" s="21" t="s">
@@ -5839,7 +5839,7 @@
       <c r="M47" s="23"/>
       <c r="N47" s="23"/>
     </row>
-    <row r="48" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="48" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A48" s="21"/>
       <c r="B48" s="21"/>
       <c r="C48" s="21" t="s">
@@ -5869,7 +5869,7 @@
       <c r="M48" s="23"/>
       <c r="N48" s="23"/>
     </row>
-    <row r="49" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="49" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A49" s="21"/>
       <c r="B49" s="22" t="s">
         <v>238</v>
@@ -5901,7 +5901,7 @@
       <c r="M49" s="23"/>
       <c r="N49" s="23"/>
     </row>
-    <row r="50" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="50" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A50" s="21"/>
       <c r="B50" s="22" t="s">
         <v>244</v>
@@ -5935,7 +5935,7 @@
       </c>
       <c r="N50" s="24"/>
     </row>
-    <row r="51" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="51" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A51" s="21"/>
       <c r="B51" s="21"/>
       <c r="C51" s="21" t="s">
@@ -5967,7 +5967,7 @@
       </c>
       <c r="N51" s="24"/>
     </row>
-    <row r="52" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="52" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A52" s="21"/>
       <c r="B52" s="21"/>
       <c r="C52" s="21" t="s">
@@ -5999,7 +5999,7 @@
       </c>
       <c r="N52" s="24"/>
     </row>
-    <row r="53" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="53" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A53" s="21"/>
       <c r="B53" s="21"/>
       <c r="C53" s="21" t="s">
@@ -6031,7 +6031,7 @@
       </c>
       <c r="N53" s="24"/>
     </row>
-    <row r="54" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="20" t="s">
         <v>262</v>
       </c>
@@ -6055,7 +6055,7 @@
       <c r="M54" s="20"/>
       <c r="N54" s="20"/>
     </row>
-    <row r="55" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="55" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A55" s="21"/>
       <c r="B55" s="22" t="s">
         <v>264</v>
@@ -6087,7 +6087,7 @@
       <c r="M55" s="23"/>
       <c r="N55" s="23"/>
     </row>
-    <row r="56" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="56" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A56" s="21"/>
       <c r="B56" s="22" t="s">
         <v>270</v>
@@ -6119,7 +6119,7 @@
       <c r="M56" s="23"/>
       <c r="N56" s="23"/>
     </row>
-    <row r="57" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="57" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A57" s="21"/>
       <c r="B57" s="21"/>
       <c r="C57" s="21" t="s">
@@ -6149,7 +6149,7 @@
       <c r="M57" s="23"/>
       <c r="N57" s="23"/>
     </row>
-    <row r="58" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="58" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A58" s="21"/>
       <c r="B58" s="22" t="s">
         <v>281</v>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="N58" s="24"/>
     </row>
-    <row r="59" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="59" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A59" s="21"/>
       <c r="B59" s="22" t="s">
         <v>287</v>
@@ -6215,7 +6215,7 @@
       <c r="M59" s="23"/>
       <c r="N59" s="23"/>
     </row>
-    <row r="60" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="60" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A60" s="21"/>
       <c r="B60" s="21"/>
       <c r="C60" s="21" t="s">
@@ -6245,7 +6245,7 @@
       <c r="M60" s="23"/>
       <c r="N60" s="23"/>
     </row>
-    <row r="61" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="61" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A61" s="21"/>
       <c r="B61" s="22" t="s">
         <v>298</v>
@@ -6277,7 +6277,7 @@
       <c r="M61" s="23"/>
       <c r="N61" s="23"/>
     </row>
-    <row r="62" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="62" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A62" s="21"/>
       <c r="B62" s="21"/>
       <c r="C62" s="21" t="s">
@@ -6307,7 +6307,7 @@
       <c r="M62" s="23"/>
       <c r="N62" s="23"/>
     </row>
-    <row r="63" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="63" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A63" s="21"/>
       <c r="B63" s="21"/>
       <c r="C63" s="21" t="s">
@@ -6337,7 +6337,7 @@
       <c r="M63" s="23"/>
       <c r="N63" s="23"/>
     </row>
-    <row r="64" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="64" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A64" s="21"/>
       <c r="B64" s="22" t="s">
         <v>314</v>
@@ -6369,7 +6369,7 @@
       <c r="M64" s="23"/>
       <c r="N64" s="23"/>
     </row>
-    <row r="65" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="65" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A65" s="21"/>
       <c r="B65" s="21"/>
       <c r="C65" s="21" t="s">
@@ -6399,7 +6399,7 @@
       <c r="M65" s="23"/>
       <c r="N65" s="23"/>
     </row>
-    <row r="66" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="66" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A66" s="21"/>
       <c r="B66" s="21"/>
       <c r="C66" s="21" t="s">
@@ -6429,7 +6429,7 @@
       <c r="M66" s="23"/>
       <c r="N66" s="23"/>
     </row>
-    <row r="67" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="67" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A67" s="21"/>
       <c r="B67" s="22" t="s">
         <v>330</v>
@@ -6461,7 +6461,7 @@
       <c r="M67" s="23"/>
       <c r="N67" s="23"/>
     </row>
-    <row r="68" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="68" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A68" s="21"/>
       <c r="B68" s="21"/>
       <c r="C68" s="21" t="s">
@@ -6491,7 +6491,7 @@
       <c r="M68" s="23"/>
       <c r="N68" s="23"/>
     </row>
-    <row r="69" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="69" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A69" s="21"/>
       <c r="B69" s="21"/>
       <c r="C69" s="21" t="s">
@@ -6521,7 +6521,7 @@
       <c r="M69" s="23"/>
       <c r="N69" s="23"/>
     </row>
-    <row r="70" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="70" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A70" s="21"/>
       <c r="B70" s="21"/>
       <c r="C70" s="21" t="s">
@@ -6553,7 +6553,7 @@
       </c>
       <c r="N70" s="24"/>
     </row>
-    <row r="71" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="71" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A71" s="21"/>
       <c r="B71" s="21"/>
       <c r="C71" s="21" t="s">
@@ -6583,7 +6583,7 @@
       <c r="M71" s="23"/>
       <c r="N71" s="23"/>
     </row>
-    <row r="72" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="72" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A72" s="21"/>
       <c r="B72" s="21"/>
       <c r="C72" s="21" t="s">
@@ -6613,7 +6613,7 @@
       <c r="M72" s="23"/>
       <c r="N72" s="23"/>
     </row>
-    <row r="73" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="73" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A73" s="21"/>
       <c r="B73" s="22" t="s">
         <v>360</v>
@@ -6645,7 +6645,7 @@
       <c r="M73" s="23"/>
       <c r="N73" s="23"/>
     </row>
-    <row r="74" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="74" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A74" s="20" t="s">
         <v>366</v>
       </c>
@@ -6669,7 +6669,7 @@
       <c r="M74" s="20"/>
       <c r="N74" s="20"/>
     </row>
-    <row r="75" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="75" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A75" s="21"/>
       <c r="B75" s="22" t="s">
         <v>368</v>
@@ -6701,7 +6701,7 @@
       <c r="M75" s="23"/>
       <c r="N75" s="23"/>
     </row>
-    <row r="76" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="76" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A76" s="21"/>
       <c r="B76" s="21"/>
       <c r="C76" s="21" t="s">
@@ -6731,7 +6731,7 @@
       <c r="M76" s="23"/>
       <c r="N76" s="23"/>
     </row>
-    <row r="77" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="77" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A77" s="21"/>
       <c r="B77" s="21"/>
       <c r="C77" s="21" t="s">
@@ -6761,7 +6761,7 @@
       <c r="M77" s="23"/>
       <c r="N77" s="23"/>
     </row>
-    <row r="78" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="78" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A78" s="21"/>
       <c r="B78" s="22" t="s">
         <v>382</v>
@@ -6793,7 +6793,7 @@
       <c r="M78" s="23"/>
       <c r="N78" s="23"/>
     </row>
-    <row r="79" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="79" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A79" s="21"/>
       <c r="B79" s="21"/>
       <c r="C79" s="21" t="s">
@@ -6823,7 +6823,7 @@
       <c r="M79" s="23"/>
       <c r="N79" s="23"/>
     </row>
-    <row r="80" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="80" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A80" s="21"/>
       <c r="B80" s="21"/>
       <c r="C80" s="21" t="s">
@@ -6853,7 +6853,7 @@
       <c r="M80" s="23"/>
       <c r="N80" s="23"/>
     </row>
-    <row r="81" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="81" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A81" s="21"/>
       <c r="B81" s="22" t="s">
         <v>396</v>
@@ -6885,7 +6885,7 @@
       <c r="M81" s="23"/>
       <c r="N81" s="23"/>
     </row>
-    <row r="82" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="82" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A82" s="21"/>
       <c r="B82" s="22" t="s">
         <v>401</v>
@@ -6917,7 +6917,7 @@
       <c r="M82" s="23"/>
       <c r="N82" s="23"/>
     </row>
-    <row r="83" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="83" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A83" s="21"/>
       <c r="B83" s="22" t="s">
         <v>407</v>
@@ -6949,7 +6949,7 @@
       <c r="M83" s="23"/>
       <c r="N83" s="23"/>
     </row>
-    <row r="84" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="84" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A84" s="21"/>
       <c r="B84" s="21"/>
       <c r="C84" s="21" t="s">
@@ -6979,7 +6979,7 @@
       <c r="M84" s="23"/>
       <c r="N84" s="23"/>
     </row>
-    <row r="85" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="85" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A85" s="21"/>
       <c r="B85" s="22" t="s">
         <v>417</v>
@@ -7013,7 +7013,7 @@
       </c>
       <c r="N85" s="24"/>
     </row>
-    <row r="86" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="86" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A86" s="21"/>
       <c r="B86" s="21"/>
       <c r="C86" s="21" t="s">
@@ -7045,7 +7045,7 @@
       </c>
       <c r="N86" s="24"/>
     </row>
-    <row r="87" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="87" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A87" s="20" t="s">
         <v>427</v>
       </c>
@@ -7069,7 +7069,7 @@
       <c r="M87" s="20"/>
       <c r="N87" s="20"/>
     </row>
-    <row r="88" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="88" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A88" s="21"/>
       <c r="B88" s="22" t="s">
         <v>429</v>
@@ -7101,7 +7101,7 @@
       <c r="M88" s="23"/>
       <c r="N88" s="23"/>
     </row>
-    <row r="89" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="89" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A89" s="21"/>
       <c r="B89" s="21"/>
       <c r="C89" s="21" t="s">
@@ -7131,7 +7131,7 @@
       <c r="M89" s="23"/>
       <c r="N89" s="23"/>
     </row>
-    <row r="90" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="90" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A90" s="21"/>
       <c r="B90" s="22" t="s">
         <v>439</v>
@@ -7163,7 +7163,7 @@
       <c r="M90" s="23"/>
       <c r="N90" s="23"/>
     </row>
-    <row r="91" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="91" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A91" s="21"/>
       <c r="B91" s="22" t="s">
         <v>444</v>
@@ -7195,7 +7195,7 @@
       <c r="M91" s="23"/>
       <c r="N91" s="23"/>
     </row>
-    <row r="92" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="92" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A92" s="21"/>
       <c r="B92" s="22" t="s">
         <v>450</v>
@@ -7227,7 +7227,7 @@
       <c r="M92" s="23"/>
       <c r="N92" s="23"/>
     </row>
-    <row r="93" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="93" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A93" s="21"/>
       <c r="B93" s="21"/>
       <c r="C93" s="21" t="s">
@@ -7257,7 +7257,7 @@
       <c r="M93" s="23"/>
       <c r="N93" s="23"/>
     </row>
-    <row r="94" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="94" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A94" s="21"/>
       <c r="B94" s="21"/>
       <c r="C94" s="21" t="s">
@@ -7287,7 +7287,7 @@
       <c r="M94" s="23"/>
       <c r="N94" s="23"/>
     </row>
-    <row r="95" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="95" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A95" s="21"/>
       <c r="B95" s="22" t="s">
         <v>463</v>
@@ -7319,7 +7319,7 @@
       <c r="M95" s="23"/>
       <c r="N95" s="23"/>
     </row>
-    <row r="96" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="96" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A96" s="21"/>
       <c r="B96" s="21"/>
       <c r="C96" s="21" t="s">
@@ -7349,7 +7349,7 @@
       <c r="M96" s="23"/>
       <c r="N96" s="23"/>
     </row>
-    <row r="97" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="97" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A97" s="21"/>
       <c r="B97" s="22" t="s">
         <v>472</v>
@@ -7381,7 +7381,7 @@
       <c r="M97" s="23"/>
       <c r="N97" s="23"/>
     </row>
-    <row r="98" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="98" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A98" s="21"/>
       <c r="B98" s="22" t="s">
         <v>478</v>
@@ -7413,7 +7413,7 @@
       <c r="M98" s="23"/>
       <c r="N98" s="23"/>
     </row>
-    <row r="99" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="99" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A99" s="21"/>
       <c r="B99" s="21"/>
       <c r="C99" s="21" t="s">
@@ -7443,7 +7443,7 @@
       <c r="M99" s="23"/>
       <c r="N99" s="23"/>
     </row>
-    <row r="100" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="100" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A100" s="21"/>
       <c r="B100" s="21"/>
       <c r="C100" s="21" t="s">
@@ -7473,7 +7473,7 @@
       <c r="M100" s="23"/>
       <c r="N100" s="23"/>
     </row>
-    <row r="101" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="101" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A101" s="21"/>
       <c r="B101" s="22" t="s">
         <v>491</v>
@@ -7505,7 +7505,7 @@
       <c r="M101" s="23"/>
       <c r="N101" s="23"/>
     </row>
-    <row r="102" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="102" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A102" s="21"/>
       <c r="B102" s="21"/>
       <c r="C102" s="21" t="s">
@@ -7535,7 +7535,7 @@
       <c r="M102" s="23"/>
       <c r="N102" s="23"/>
     </row>
-    <row r="103" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="103" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A103" s="21"/>
       <c r="B103" s="21"/>
       <c r="C103" s="21" t="s">
@@ -7565,7 +7565,7 @@
       <c r="M103" s="23"/>
       <c r="N103" s="23"/>
     </row>
-    <row r="104" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="104" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A104" s="21"/>
       <c r="B104" s="21"/>
       <c r="C104" s="21" t="s">
@@ -7595,7 +7595,7 @@
       <c r="M104" s="23"/>
       <c r="N104" s="23"/>
     </row>
-    <row r="105" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="105" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A105" s="21"/>
       <c r="B105" s="22" t="s">
         <v>510</v>
@@ -7627,7 +7627,7 @@
       <c r="M105" s="23"/>
       <c r="N105" s="23"/>
     </row>
-    <row r="106" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="106" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A106" s="21"/>
       <c r="B106" s="22" t="s">
         <v>516</v>
@@ -7659,7 +7659,7 @@
       <c r="M106" s="23"/>
       <c r="N106" s="23"/>
     </row>
-    <row r="107" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="107" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A107" s="21"/>
       <c r="B107" s="22" t="s">
         <v>522</v>
@@ -7693,7 +7693,7 @@
       </c>
       <c r="N107" s="24"/>
     </row>
-    <row r="108" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="108" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A108" s="21"/>
       <c r="B108" s="21"/>
       <c r="C108" s="21" t="s">
@@ -7725,7 +7725,7 @@
       </c>
       <c r="N108" s="24"/>
     </row>
-    <row r="109" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="109" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A109" s="21"/>
       <c r="B109" s="22" t="s">
         <v>532</v>
@@ -7757,7 +7757,7 @@
       <c r="M109" s="23"/>
       <c r="N109" s="23"/>
     </row>
-    <row r="110" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="110" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A110" s="21"/>
       <c r="B110" s="21"/>
       <c r="C110" s="21" t="s">
@@ -7787,7 +7787,7 @@
       <c r="M110" s="23"/>
       <c r="N110" s="23"/>
     </row>
-    <row r="111" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="111" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A111" s="21"/>
       <c r="B111" s="21"/>
       <c r="C111" s="21" t="s">
@@ -7817,7 +7817,7 @@
       <c r="M111" s="23"/>
       <c r="N111" s="23"/>
     </row>
-    <row r="112" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="112" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A112" s="21"/>
       <c r="B112" s="21"/>
       <c r="C112" s="21" t="s">
@@ -7847,7 +7847,7 @@
       <c r="M112" s="23"/>
       <c r="N112" s="23"/>
     </row>
-    <row r="113" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="113" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A113" s="21"/>
       <c r="B113" s="22" t="s">
         <v>550</v>
@@ -7879,7 +7879,7 @@
       <c r="M113" s="23"/>
       <c r="N113" s="23"/>
     </row>
-    <row r="114" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="114" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A114" s="21"/>
       <c r="B114" s="22" t="s">
         <v>555</v>
@@ -7911,7 +7911,7 @@
       <c r="M114" s="23"/>
       <c r="N114" s="23"/>
     </row>
-    <row r="115" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="115" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A115" s="21"/>
       <c r="B115" s="22" t="s">
         <v>561</v>
@@ -7945,7 +7945,7 @@
       </c>
       <c r="N115" s="24"/>
     </row>
-    <row r="116" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="116" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A116" s="21"/>
       <c r="B116" s="21"/>
       <c r="C116" s="21" t="s">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="N116" s="24"/>
     </row>
-    <row r="117" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="117" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A117" s="21"/>
       <c r="B117" s="21"/>
       <c r="C117" s="21" t="s">
@@ -8009,7 +8009,7 @@
       </c>
       <c r="N117" s="24"/>
     </row>
-    <row r="118" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="118" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A118" s="21"/>
       <c r="B118" s="21"/>
       <c r="C118" s="21" t="s">
@@ -8041,7 +8041,7 @@
       </c>
       <c r="N118" s="24"/>
     </row>
-    <row r="119" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="119" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A119" s="21"/>
       <c r="B119" s="21"/>
       <c r="C119" s="21" t="s">
@@ -8073,7 +8073,7 @@
       </c>
       <c r="N119" s="24"/>
     </row>
-    <row r="120" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="120" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A120" s="20" t="s">
         <v>583</v>
       </c>
@@ -8097,7 +8097,7 @@
       <c r="M120" s="20"/>
       <c r="N120" s="20"/>
     </row>
-    <row r="121" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="121" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A121" s="21"/>
       <c r="B121" s="22" t="s">
         <v>585</v>
@@ -8129,7 +8129,7 @@
       <c r="M121" s="23"/>
       <c r="N121" s="23"/>
     </row>
-    <row r="122" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="122" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A122" s="21"/>
       <c r="B122" s="21"/>
       <c r="C122" s="21" t="s">
@@ -8159,7 +8159,7 @@
       <c r="M122" s="23"/>
       <c r="N122" s="23"/>
     </row>
-    <row r="123" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="123" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A123" s="21"/>
       <c r="B123" s="21"/>
       <c r="C123" s="21" t="s">
@@ -8189,7 +8189,7 @@
       <c r="M123" s="23"/>
       <c r="N123" s="23"/>
     </row>
-    <row r="124" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="124" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A124" s="21"/>
       <c r="B124" s="21"/>
       <c r="C124" s="21" t="s">
@@ -8219,7 +8219,7 @@
       <c r="M124" s="23"/>
       <c r="N124" s="23"/>
     </row>
-    <row r="125" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="125" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A125" s="21"/>
       <c r="B125" s="22" t="s">
         <v>604</v>
@@ -8251,7 +8251,7 @@
       <c r="M125" s="23"/>
       <c r="N125" s="23"/>
     </row>
-    <row r="126" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="126" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A126" s="21"/>
       <c r="B126" s="22" t="s">
         <v>610</v>
@@ -8283,7 +8283,7 @@
       <c r="M126" s="23"/>
       <c r="N126" s="23"/>
     </row>
-    <row r="127" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="127" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A127" s="21"/>
       <c r="B127" s="22" t="s">
         <v>616</v>
@@ -8315,7 +8315,7 @@
       <c r="M127" s="23"/>
       <c r="N127" s="23"/>
     </row>
-    <row r="128" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="128" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A128" s="21"/>
       <c r="B128" s="21"/>
       <c r="C128" s="21" t="s">
@@ -8345,7 +8345,7 @@
       <c r="M128" s="23"/>
       <c r="N128" s="23"/>
     </row>
-    <row r="129" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="129" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A129" s="21"/>
       <c r="B129" s="22" t="s">
         <v>624</v>
@@ -8377,7 +8377,7 @@
       <c r="M129" s="23"/>
       <c r="N129" s="23"/>
     </row>
-    <row r="130" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="130" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A130" s="21"/>
       <c r="B130" s="21"/>
       <c r="C130" s="21" t="s">
@@ -8407,7 +8407,7 @@
       <c r="M130" s="23"/>
       <c r="N130" s="23"/>
     </row>
-    <row r="131" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="131" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A131" s="21"/>
       <c r="B131" s="21"/>
       <c r="C131" s="21" t="s">
@@ -8437,7 +8437,7 @@
       <c r="M131" s="23"/>
       <c r="N131" s="23"/>
     </row>
-    <row r="132" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="132" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A132" s="21"/>
       <c r="B132" s="21"/>
       <c r="C132" s="21" t="s">
@@ -8467,7 +8467,7 @@
       <c r="M132" s="23"/>
       <c r="N132" s="23"/>
     </row>
-    <row r="133" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="133" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A133" s="20" t="s">
         <v>642</v>
       </c>
@@ -8491,7 +8491,7 @@
       <c r="M133" s="20"/>
       <c r="N133" s="20"/>
     </row>
-    <row r="134" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="134" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A134" s="21"/>
       <c r="B134" s="22" t="s">
         <v>644</v>
@@ -8523,7 +8523,7 @@
       <c r="M134" s="23"/>
       <c r="N134" s="23"/>
     </row>
-    <row r="135" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="135" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A135" s="21"/>
       <c r="B135" s="21"/>
       <c r="C135" s="21" t="s">
@@ -8553,7 +8553,7 @@
       <c r="M135" s="23"/>
       <c r="N135" s="23"/>
     </row>
-    <row r="136" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="136" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A136" s="21"/>
       <c r="B136" s="21"/>
       <c r="C136" s="21" t="s">
@@ -8583,7 +8583,7 @@
       <c r="M136" s="23"/>
       <c r="N136" s="23"/>
     </row>
-    <row r="137" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="137" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A137" s="21"/>
       <c r="B137" s="21"/>
       <c r="C137" s="21" t="s">
@@ -8613,7 +8613,7 @@
       <c r="M137" s="23"/>
       <c r="N137" s="23"/>
     </row>
-    <row r="138" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="138" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A138" s="21"/>
       <c r="B138" s="22" t="s">
         <v>664</v>
@@ -8645,7 +8645,7 @@
       <c r="M138" s="23"/>
       <c r="N138" s="23"/>
     </row>
-    <row r="139" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="139" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A139" s="21"/>
       <c r="B139" s="22" t="s">
         <v>670</v>
@@ -8677,7 +8677,7 @@
       <c r="M139" s="23"/>
       <c r="N139" s="23"/>
     </row>
-    <row r="140" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="140" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A140" s="21"/>
       <c r="B140" s="22" t="s">
         <v>675</v>
@@ -8709,7 +8709,7 @@
       <c r="M140" s="23"/>
       <c r="N140" s="23"/>
     </row>
-    <row r="141" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="141" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A141" s="21"/>
       <c r="B141" s="21"/>
       <c r="C141" s="21" t="s">
@@ -8739,7 +8739,7 @@
       <c r="M141" s="23"/>
       <c r="N141" s="23"/>
     </row>
-    <row r="142" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="142" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A142" s="21"/>
       <c r="B142" s="22" t="s">
         <v>685</v>
@@ -8771,7 +8771,7 @@
       <c r="M142" s="23"/>
       <c r="N142" s="23"/>
     </row>
-    <row r="143" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="143" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A143" s="21"/>
       <c r="B143" s="22" t="s">
         <v>691</v>
@@ -8803,7 +8803,7 @@
       <c r="M143" s="23"/>
       <c r="N143" s="23"/>
     </row>
-    <row r="144" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="144" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A144" s="21"/>
       <c r="B144" s="22" t="s">
         <v>697</v>
@@ -8835,7 +8835,7 @@
       <c r="M144" s="23"/>
       <c r="N144" s="23"/>
     </row>
-    <row r="145" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="145" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A145" s="21"/>
       <c r="B145" s="21"/>
       <c r="C145" s="21" t="s">
@@ -8865,7 +8865,7 @@
       <c r="M145" s="23"/>
       <c r="N145" s="23"/>
     </row>
-    <row r="146" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="146" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A146" s="21"/>
       <c r="B146" s="21"/>
       <c r="C146" s="21" t="s">
@@ -8895,7 +8895,7 @@
       <c r="M146" s="23"/>
       <c r="N146" s="23"/>
     </row>
-    <row r="147" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="147" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A147" s="21"/>
       <c r="B147" s="21"/>
       <c r="C147" s="21" t="s">
@@ -8925,7 +8925,7 @@
       <c r="M147" s="23"/>
       <c r="N147" s="23"/>
     </row>
-    <row r="148" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="148" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A148" s="20" t="s">
         <v>715</v>
       </c>
@@ -8949,7 +8949,7 @@
       <c r="M148" s="20"/>
       <c r="N148" s="20"/>
     </row>
-    <row r="149" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="149" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A149" s="21"/>
       <c r="B149" s="22" t="s">
         <v>717</v>
@@ -8981,7 +8981,7 @@
       <c r="M149" s="23"/>
       <c r="N149" s="23"/>
     </row>
-    <row r="150" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="150" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A150" s="21"/>
       <c r="B150" s="21"/>
       <c r="C150" s="21" t="s">
@@ -9011,7 +9011,7 @@
       <c r="M150" s="23"/>
       <c r="N150" s="23"/>
     </row>
-    <row r="151" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="151" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A151" s="21"/>
       <c r="B151" s="21"/>
       <c r="C151" s="21" t="s">
@@ -9041,7 +9041,7 @@
       <c r="M151" s="23"/>
       <c r="N151" s="23"/>
     </row>
-    <row r="152" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="152" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A152" s="21"/>
       <c r="B152" s="21"/>
       <c r="C152" s="21" t="s">
@@ -9071,7 +9071,7 @@
       <c r="M152" s="23"/>
       <c r="N152" s="23"/>
     </row>
-    <row r="153" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="153" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A153" s="21"/>
       <c r="B153" s="21"/>
       <c r="C153" s="21" t="s">
@@ -9101,7 +9101,7 @@
       <c r="M153" s="23"/>
       <c r="N153" s="23"/>
     </row>
-    <row r="154" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="154" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A154" s="21"/>
       <c r="B154" s="21"/>
       <c r="C154" s="21" t="s">
@@ -9131,7 +9131,7 @@
       <c r="M154" s="23"/>
       <c r="N154" s="23"/>
     </row>
-    <row r="155" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="155" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A155" s="21"/>
       <c r="B155" s="21"/>
       <c r="C155" s="21" t="s">
@@ -9161,7 +9161,7 @@
       <c r="M155" s="23"/>
       <c r="N155" s="23"/>
     </row>
-    <row r="156" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="156" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A156" s="21"/>
       <c r="B156" s="21"/>
       <c r="C156" s="21" t="s">
@@ -9191,7 +9191,7 @@
       <c r="M156" s="23"/>
       <c r="N156" s="23"/>
     </row>
-    <row r="157" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="157" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A157" s="21"/>
       <c r="B157" s="21"/>
       <c r="C157" s="21" t="s">
@@ -9221,7 +9221,7 @@
       <c r="M157" s="23"/>
       <c r="N157" s="23"/>
     </row>
-    <row r="158" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="158" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A158" s="21"/>
       <c r="B158" s="21"/>
       <c r="C158" s="21" t="s">
@@ -9251,7 +9251,7 @@
       <c r="M158" s="23"/>
       <c r="N158" s="23"/>
     </row>
-    <row r="159" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="159" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A159" s="21"/>
       <c r="B159" s="21"/>
       <c r="C159" s="21" t="s">
@@ -9281,7 +9281,7 @@
       <c r="M159" s="23"/>
       <c r="N159" s="23"/>
     </row>
-    <row r="160" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="160" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A160" s="21"/>
       <c r="B160" s="21"/>
       <c r="C160" s="21" t="s">
@@ -9311,7 +9311,7 @@
       <c r="M160" s="23"/>
       <c r="N160" s="23"/>
     </row>
-    <row r="161" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="161" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A161" s="21"/>
       <c r="B161" s="22" t="s">
         <v>767</v>
@@ -9343,7 +9343,7 @@
       <c r="M161" s="23"/>
       <c r="N161" s="23"/>
     </row>
-    <row r="162" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="162" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A162" s="21"/>
       <c r="B162" s="22" t="s">
         <v>773</v>
@@ -9375,7 +9375,7 @@
       <c r="M162" s="23"/>
       <c r="N162" s="23"/>
     </row>
-    <row r="163" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="163" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A163" s="21"/>
       <c r="B163" s="21"/>
       <c r="C163" s="21" t="s">
@@ -9405,7 +9405,7 @@
       <c r="M163" s="23"/>
       <c r="N163" s="23"/>
     </row>
-    <row r="164" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="164" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A164" s="21"/>
       <c r="B164" s="21"/>
       <c r="C164" s="21" t="s">
@@ -9435,7 +9435,7 @@
       <c r="M164" s="23"/>
       <c r="N164" s="23"/>
     </row>
-    <row r="165" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="165" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A165" s="21"/>
       <c r="B165" s="22" t="s">
         <v>788</v>
@@ -9467,7 +9467,7 @@
       <c r="M165" s="23"/>
       <c r="N165" s="23"/>
     </row>
-    <row r="166" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="166" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A166" s="21"/>
       <c r="B166" s="21"/>
       <c r="C166" s="21" t="s">
@@ -9497,7 +9497,7 @@
       <c r="M166" s="23"/>
       <c r="N166" s="23"/>
     </row>
-    <row r="167" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="167" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A167" s="21"/>
       <c r="B167" s="21"/>
       <c r="C167" s="21" t="s">
@@ -9527,7 +9527,7 @@
       <c r="M167" s="23"/>
       <c r="N167" s="23"/>
     </row>
-    <row r="168" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="168" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A168" s="20" t="s">
         <v>800</v>
       </c>
@@ -9551,7 +9551,7 @@
       <c r="M168" s="20"/>
       <c r="N168" s="20"/>
     </row>
-    <row r="169" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="169" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A169" s="21"/>
       <c r="B169" s="22" t="s">
         <v>802</v>
@@ -9583,7 +9583,7 @@
       <c r="M169" s="23"/>
       <c r="N169" s="23"/>
     </row>
-    <row r="170" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="170" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A170" s="21"/>
       <c r="B170" s="21"/>
       <c r="C170" s="21" t="s">
@@ -9613,7 +9613,7 @@
       <c r="M170" s="23"/>
       <c r="N170" s="23"/>
     </row>
-    <row r="171" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="171" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A171" s="21"/>
       <c r="B171" s="21"/>
       <c r="C171" s="21" t="s">
@@ -9645,7 +9645,7 @@
       </c>
       <c r="N171" s="24"/>
     </row>
-    <row r="172" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="172" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A172" s="21"/>
       <c r="B172" s="21"/>
       <c r="C172" s="21" t="s">
@@ -9677,7 +9677,7 @@
       </c>
       <c r="N172" s="24"/>
     </row>
-    <row r="173" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="173" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A173" s="21"/>
       <c r="B173" s="22" t="s">
         <v>822</v>
@@ -9709,7 +9709,7 @@
       <c r="M173" s="23"/>
       <c r="N173" s="23"/>
     </row>
-    <row r="174" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="174" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A174" s="21"/>
       <c r="B174" s="21"/>
       <c r="C174" s="21" t="s">
@@ -9739,7 +9739,7 @@
       <c r="M174" s="23"/>
       <c r="N174" s="23"/>
     </row>
-    <row r="175" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="175" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A175" s="21"/>
       <c r="B175" s="22" t="s">
         <v>833</v>
@@ -9773,7 +9773,7 @@
       </c>
       <c r="N175" s="24"/>
     </row>
-    <row r="176" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="176" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A176" s="21"/>
       <c r="B176" s="22" t="s">
         <v>838</v>
@@ -9805,7 +9805,7 @@
       <c r="M176" s="23"/>
       <c r="N176" s="23"/>
     </row>
-    <row r="177" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="177" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A177" s="20" t="s">
         <v>844</v>
       </c>
@@ -9829,7 +9829,7 @@
       <c r="M177" s="20"/>
       <c r="N177" s="20"/>
     </row>
-    <row r="178" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="178" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A178" s="21"/>
       <c r="B178" s="22" t="s">
         <v>846</v>
@@ -9861,7 +9861,7 @@
       <c r="M178" s="23"/>
       <c r="N178" s="23"/>
     </row>
-    <row r="179" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="179" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A179" s="21"/>
       <c r="B179" s="21"/>
       <c r="C179" s="21" t="s">
@@ -9891,7 +9891,7 @@
       <c r="M179" s="23"/>
       <c r="N179" s="23"/>
     </row>
-    <row r="180" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="180" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A180" s="21"/>
       <c r="B180" s="21"/>
       <c r="C180" s="21" t="s">
@@ -9921,7 +9921,7 @@
       <c r="M180" s="23"/>
       <c r="N180" s="23"/>
     </row>
-    <row r="181" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="181" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A181" s="21"/>
       <c r="B181" s="21"/>
       <c r="C181" s="21" t="s">
@@ -9951,7 +9951,7 @@
       <c r="M181" s="23"/>
       <c r="N181" s="23"/>
     </row>
-    <row r="182" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="182" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A182" s="21"/>
       <c r="B182" s="22" t="s">
         <v>865</v>
@@ -9983,7 +9983,7 @@
       <c r="M182" s="23"/>
       <c r="N182" s="23"/>
     </row>
-    <row r="183" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="183" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A183" s="21"/>
       <c r="B183" s="21"/>
       <c r="C183" s="21" t="s">
@@ -10013,7 +10013,7 @@
       <c r="M183" s="23"/>
       <c r="N183" s="23"/>
     </row>
-    <row r="184" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="184" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A184" s="21"/>
       <c r="B184" s="21"/>
       <c r="C184" s="21" t="s">
@@ -10043,7 +10043,7 @@
       <c r="M184" s="23"/>
       <c r="N184" s="23"/>
     </row>
-    <row r="185" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="185" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A185" s="21"/>
       <c r="B185" s="22" t="s">
         <v>879</v>
@@ -10075,7 +10075,7 @@
       <c r="M185" s="23"/>
       <c r="N185" s="23"/>
     </row>
-    <row r="186" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="186" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A186" s="21"/>
       <c r="B186" s="22" t="s">
         <v>885</v>
@@ -10107,7 +10107,7 @@
       <c r="M186" s="23"/>
       <c r="N186" s="23"/>
     </row>
-    <row r="187" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="187" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A187" s="21"/>
       <c r="B187" s="21"/>
       <c r="C187" s="21" t="s">
@@ -10137,7 +10137,7 @@
       <c r="M187" s="23"/>
       <c r="N187" s="23"/>
     </row>
-    <row r="188" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="188" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A188" s="21"/>
       <c r="B188" s="22" t="s">
         <v>896</v>
@@ -10169,7 +10169,7 @@
       <c r="M188" s="23"/>
       <c r="N188" s="23"/>
     </row>
-    <row r="189" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="189" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A189" s="21"/>
       <c r="B189" s="22" t="s">
         <v>901</v>
@@ -10201,7 +10201,7 @@
       <c r="M189" s="23"/>
       <c r="N189" s="23"/>
     </row>
-    <row r="190" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="190" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A190" s="21"/>
       <c r="B190" s="21"/>
       <c r="C190" s="21" t="s">
@@ -10231,7 +10231,7 @@
       <c r="M190" s="23"/>
       <c r="N190" s="23"/>
     </row>
-    <row r="191" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="191" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A191" s="21"/>
       <c r="B191" s="22" t="s">
         <v>912</v>
@@ -10263,7 +10263,7 @@
       <c r="M191" s="23"/>
       <c r="N191" s="23"/>
     </row>
-    <row r="192" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="192" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A192" s="21"/>
       <c r="B192" s="21"/>
       <c r="C192" s="21" t="s">
@@ -10293,7 +10293,7 @@
       <c r="M192" s="23"/>
       <c r="N192" s="23"/>
     </row>
-    <row r="193" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="193" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A193" s="21"/>
       <c r="B193" s="22" t="s">
         <v>923</v>
@@ -10325,7 +10325,7 @@
       <c r="M193" s="23"/>
       <c r="N193" s="23"/>
     </row>
-    <row r="194" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="194" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A194" s="21"/>
       <c r="B194" s="22" t="s">
         <v>929</v>
@@ -10357,7 +10357,7 @@
       <c r="M194" s="23"/>
       <c r="N194" s="23"/>
     </row>
-    <row r="195" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="195" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A195" s="20" t="s">
         <v>935</v>
       </c>
@@ -10381,7 +10381,7 @@
       <c r="M195" s="20"/>
       <c r="N195" s="20"/>
     </row>
-    <row r="196" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="196" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A196" s="21"/>
       <c r="B196" s="22" t="s">
         <v>937</v>
@@ -10413,7 +10413,7 @@
       <c r="M196" s="23"/>
       <c r="N196" s="23"/>
     </row>
-    <row r="197" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="197" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A197" s="21"/>
       <c r="B197" s="21"/>
       <c r="C197" s="21" t="s">
@@ -10443,7 +10443,7 @@
       <c r="M197" s="23"/>
       <c r="N197" s="23"/>
     </row>
-    <row r="198" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="198" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A198" s="21"/>
       <c r="B198" s="21"/>
       <c r="C198" s="21" t="s">
@@ -10473,7 +10473,7 @@
       <c r="M198" s="23"/>
       <c r="N198" s="23"/>
     </row>
-    <row r="199" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="199" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A199" s="20" t="s">
         <v>951</v>
       </c>
@@ -10497,7 +10497,7 @@
       <c r="M199" s="20"/>
       <c r="N199" s="20"/>
     </row>
-    <row r="200" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="200" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A200" s="21"/>
       <c r="B200" s="22" t="s">
         <v>953</v>
@@ -10531,7 +10531,7 @@
       </c>
       <c r="N200" s="24"/>
     </row>
-    <row r="201" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="201" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A201" s="21"/>
       <c r="B201" s="21"/>
       <c r="C201" s="21" t="s">
@@ -10563,7 +10563,7 @@
       </c>
       <c r="N201" s="24"/>
     </row>
-    <row r="202" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="202" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A202" s="21"/>
       <c r="B202" s="21"/>
       <c r="C202" s="21" t="s">
@@ -10593,7 +10593,7 @@
       <c r="M202" s="23"/>
       <c r="N202" s="23"/>
     </row>
-    <row r="203" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="203" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A203" s="21"/>
       <c r="B203" s="21"/>
       <c r="C203" s="21" t="s">
@@ -10623,7 +10623,7 @@
       <c r="M203" s="23"/>
       <c r="N203" s="23"/>
     </row>
-    <row r="204" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="204" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A204" s="21"/>
       <c r="B204" s="22" t="s">
         <v>973</v>
@@ -10655,7 +10655,7 @@
       <c r="M204" s="23"/>
       <c r="N204" s="23"/>
     </row>
-    <row r="205" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="205" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A205" s="21"/>
       <c r="B205" s="21"/>
       <c r="C205" s="21" t="s">
@@ -10685,7 +10685,7 @@
       <c r="M205" s="23"/>
       <c r="N205" s="23"/>
     </row>
-    <row r="206" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="206" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A206" s="21"/>
       <c r="B206" s="22" t="s">
         <v>984</v>
@@ -10717,7 +10717,7 @@
       <c r="M206" s="23"/>
       <c r="N206" s="23"/>
     </row>
-    <row r="207" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="207" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A207" s="20" t="s">
         <v>990</v>
       </c>
@@ -10741,7 +10741,7 @@
       <c r="M207" s="20"/>
       <c r="N207" s="20"/>
     </row>
-    <row r="208" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="208" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A208" s="21"/>
       <c r="B208" s="22" t="s">
         <v>992</v>
@@ -10773,7 +10773,7 @@
       <c r="M208" s="23"/>
       <c r="N208" s="23"/>
     </row>
-    <row r="209" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="209" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A209" s="21"/>
       <c r="B209" s="22" t="s">
         <v>998</v>
@@ -10805,7 +10805,7 @@
       <c r="M209" s="23"/>
       <c r="N209" s="23"/>
     </row>
-    <row r="210" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="210" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A210" s="21"/>
       <c r="B210" s="22" t="s">
         <v>1004</v>
@@ -10837,7 +10837,7 @@
       <c r="M210" s="23"/>
       <c r="N210" s="23"/>
     </row>
-    <row r="211" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="211" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A211" s="21"/>
       <c r="B211" s="21"/>
       <c r="C211" s="21" t="s">
@@ -10867,7 +10867,7 @@
       <c r="M211" s="23"/>
       <c r="N211" s="23"/>
     </row>
-    <row r="212" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="212" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A212" s="21"/>
       <c r="B212" s="22" t="s">
         <v>1014</v>
@@ -10899,7 +10899,7 @@
       <c r="M212" s="23"/>
       <c r="N212" s="23"/>
     </row>
-    <row r="213" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="213" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A213" s="21"/>
       <c r="B213" s="21"/>
       <c r="C213" s="21" t="s">
@@ -10929,7 +10929,7 @@
       <c r="M213" s="23"/>
       <c r="N213" s="23"/>
     </row>
-    <row r="214" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="214" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A214" s="20" t="s">
         <v>1023</v>
       </c>
@@ -10953,7 +10953,7 @@
       <c r="M214" s="20"/>
       <c r="N214" s="20"/>
     </row>
-    <row r="215" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="215" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A215" s="21"/>
       <c r="B215" s="22" t="s">
         <v>1025</v>
@@ -10987,7 +10987,7 @@
       </c>
       <c r="N215" s="24"/>
     </row>
-    <row r="216" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="216" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A216" s="21"/>
       <c r="B216" s="21"/>
       <c r="C216" s="21" t="s">
@@ -11017,7 +11017,7 @@
       <c r="M216" s="23"/>
       <c r="N216" s="23"/>
     </row>
-    <row r="217" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="217" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A217" s="21"/>
       <c r="B217" s="21"/>
       <c r="C217" s="21" t="s">
@@ -11047,7 +11047,7 @@
       <c r="M217" s="23"/>
       <c r="N217" s="23"/>
     </row>
-    <row r="218" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="218" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A218" s="21"/>
       <c r="B218" s="21"/>
       <c r="C218" s="21" t="s">
@@ -11079,7 +11079,7 @@
       </c>
       <c r="N218" s="24"/>
     </row>
-    <row r="219" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="219" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A219" s="21"/>
       <c r="B219" s="21"/>
       <c r="C219" s="21" t="s">
@@ -11109,7 +11109,7 @@
       <c r="M219" s="23"/>
       <c r="N219" s="23"/>
     </row>
-    <row r="220" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="220" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A220" s="21"/>
       <c r="B220" s="22" t="s">
         <v>1051</v>
@@ -11143,7 +11143,7 @@
       </c>
       <c r="N220" s="24"/>
     </row>
-    <row r="221" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="221" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A221" s="21"/>
       <c r="B221" s="22" t="s">
         <v>1056</v>
@@ -11177,7 +11177,7 @@
       </c>
       <c r="N221" s="24"/>
     </row>
-    <row r="222" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="222" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A222" s="20" t="s">
         <v>1061</v>
       </c>
@@ -11201,7 +11201,7 @@
       <c r="M222" s="20"/>
       <c r="N222" s="20"/>
     </row>
-    <row r="223" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="223" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A223" s="21"/>
       <c r="B223" s="22" t="s">
         <v>1063</v>
@@ -11233,7 +11233,7 @@
       <c r="M223" s="23"/>
       <c r="N223" s="23"/>
     </row>
-    <row r="224" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="224" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A224" s="21"/>
       <c r="B224" s="21"/>
       <c r="C224" s="21" t="s">
@@ -11263,7 +11263,7 @@
       <c r="M224" s="23"/>
       <c r="N224" s="23"/>
     </row>
-    <row r="225" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="225" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A225" s="21"/>
       <c r="B225" s="21"/>
       <c r="C225" s="21" t="s">
@@ -11293,7 +11293,7 @@
       <c r="M225" s="23"/>
       <c r="N225" s="23"/>
     </row>
-    <row r="226" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="226" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A226" s="21"/>
       <c r="B226" s="22" t="s">
         <v>1079</v>
@@ -11327,7 +11327,7 @@
       </c>
       <c r="N226" s="24"/>
     </row>
-    <row r="227" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="227" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A227" s="25" t="s">
         <v>1085</v>
       </c>
@@ -11351,7 +11351,7 @@
       <c r="M227" s="25"/>
       <c r="N227" s="25"/>
     </row>
-    <row r="228" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="228" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A228" s="21"/>
       <c r="B228" s="22" t="s">
         <v>1088</v>
@@ -11385,7 +11385,7 @@
       </c>
       <c r="N228" s="24"/>
     </row>
-    <row r="229" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="229" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A229" s="21"/>
       <c r="B229" s="21"/>
       <c r="C229" s="21" t="s">
@@ -11417,7 +11417,7 @@
       </c>
       <c r="N229" s="24"/>
     </row>
-    <row r="230" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="230" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A230" s="21"/>
       <c r="B230" s="21"/>
       <c r="C230" s="21" t="s">
@@ -11449,7 +11449,7 @@
       </c>
       <c r="N230" s="24"/>
     </row>
-    <row r="231" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="231" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A231" s="20" t="s">
         <v>1102</v>
       </c>
@@ -11473,7 +11473,7 @@
       <c r="M231" s="20"/>
       <c r="N231" s="20"/>
     </row>
-    <row r="232" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="232" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A232" s="21"/>
       <c r="B232" s="22" t="s">
         <v>1104</v>
@@ -11505,7 +11505,7 @@
       <c r="M232" s="23"/>
       <c r="N232" s="23"/>
     </row>
-    <row r="233" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="233" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A233" s="21"/>
       <c r="B233" s="21"/>
       <c r="C233" s="21" t="s">
@@ -11535,7 +11535,7 @@
       <c r="M233" s="23"/>
       <c r="N233" s="23"/>
     </row>
-    <row r="234" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="234" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A234" s="21"/>
       <c r="B234" s="21"/>
       <c r="C234" s="21" t="s">
@@ -11584,7 +11584,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O61"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -11597,7 +11597,7 @@
     <col min="9" max="9" width="64" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" ht="40" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
         <v>1118</v>
       </c>
@@ -11626,7 +11626,7 @@
         <v>1125</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
         <v>1126</v>
       </c>
@@ -11655,7 +11655,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="27" t="s">
         <v>1133</v>
       </c>
@@ -11684,7 +11684,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
         <v>1136</v>
       </c>
@@ -11713,7 +11713,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="28" t="s">
         <v>1139</v>
       </c>
@@ -11742,7 +11742,7 @@
         <v>1143</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="29" t="s">
         <v>1144</v>
       </c>
@@ -11771,7 +11771,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="27" t="s">
         <v>1149</v>
       </c>
@@ -11800,7 +11800,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="27" t="s">
         <v>1152</v>
       </c>
@@ -11829,7 +11829,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
         <v>1155</v>
       </c>
@@ -11858,7 +11858,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="27" t="s">
         <v>1158</v>
       </c>
@@ -11887,7 +11887,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="29" t="s">
         <v>1160</v>
       </c>
@@ -11916,7 +11916,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
         <v>1162</v>
       </c>
@@ -11945,7 +11945,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
         <v>1165</v>
       </c>
@@ -11974,7 +11974,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="29" t="s">
         <v>1167</v>
       </c>
@@ -12003,7 +12003,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="28" t="s">
         <v>1169</v>
       </c>
@@ -12032,7 +12032,7 @@
         <v>1172</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
         <v>1173</v>
       </c>
@@ -12061,7 +12061,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="29" t="s">
         <v>1176</v>
       </c>
@@ -12090,7 +12090,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
         <v>1178</v>
       </c>
@@ -12119,7 +12119,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="28" t="s">
         <v>1181</v>
       </c>
@@ -12148,7 +12148,7 @@
         <v>1172</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
         <v>1183</v>
       </c>
@@ -12177,7 +12177,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
         <v>1186</v>
       </c>
@@ -12206,7 +12206,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="27" t="s">
         <v>1188</v>
       </c>
@@ -12235,7 +12235,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="29" t="s">
         <v>1191</v>
       </c>
@@ -12264,7 +12264,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="27" t="s">
         <v>1193</v>
       </c>
@@ -12293,7 +12293,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="28" t="s">
         <v>1196</v>
       </c>
@@ -12322,7 +12322,7 @@
         <v>1172</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="29" t="s">
         <v>1198</v>
       </c>
@@ -12351,7 +12351,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="28" t="s">
         <v>1200</v>
       </c>
@@ -12380,7 +12380,7 @@
         <v>1172</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="27" t="s">
         <v>1203</v>
       </c>
@@ -12409,7 +12409,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="29" t="s">
         <v>1206</v>
       </c>
@@ -12438,7 +12438,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="27" t="s">
         <v>1208</v>
       </c>
@@ -12467,7 +12467,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="27" t="s">
         <v>1211</v>
       </c>
@@ -12496,7 +12496,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="28" t="s">
         <v>1214</v>
       </c>
@@ -12525,7 +12525,7 @@
         <v>1172</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="29" t="s">
         <v>1216</v>
       </c>
@@ -12554,7 +12554,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="27" t="s">
         <v>1218</v>
       </c>
@@ -12583,7 +12583,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="28" t="s">
         <v>1221</v>
       </c>
@@ -12612,7 +12612,7 @@
         <v>1143</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="29" t="s">
         <v>1223</v>
       </c>
@@ -12641,7 +12641,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="27" t="s">
         <v>1225</v>
       </c>
@@ -12670,7 +12670,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="27" t="s">
         <v>1228</v>
       </c>
@@ -12699,7 +12699,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="29" t="s">
         <v>1230</v>
       </c>
@@ -12728,7 +12728,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="29" t="s">
         <v>1232</v>
       </c>
@@ -12757,7 +12757,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="27" t="s">
         <v>1235</v>
       </c>
@@ -12786,7 +12786,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="27" t="s">
         <v>1238</v>
       </c>
@@ -12815,7 +12815,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="29" t="s">
         <v>1240</v>
       </c>
@@ -12844,7 +12844,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="28" t="s">
         <v>1242</v>
       </c>
@@ -12873,7 +12873,7 @@
         <v>1143</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="29" t="s">
         <v>1245</v>
       </c>
@@ -12902,7 +12902,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="27" t="s">
         <v>1247</v>
       </c>
@@ -12931,7 +12931,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="28" t="s">
         <v>1250</v>
       </c>
@@ -12960,7 +12960,7 @@
         <v>1143</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="27" t="s">
         <v>1252</v>
       </c>
@@ -12989,7 +12989,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="29" t="s">
         <v>1254</v>
       </c>
@@ -13018,7 +13018,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="28" t="s">
         <v>1256</v>
       </c>
@@ -13047,7 +13047,7 @@
         <v>1143</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="29" t="s">
         <v>1259</v>
       </c>
@@ -13076,7 +13076,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="27" t="s">
         <v>1262</v>
       </c>
@@ -13105,7 +13105,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="27" t="s">
         <v>1266</v>
       </c>
@@ -13134,7 +13134,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
         <v>1269</v>
       </c>
@@ -13163,7 +13163,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="27" t="s">
         <v>1272</v>
       </c>
@@ -13192,7 +13192,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="27" t="s">
         <v>1275</v>
       </c>
@@ -13221,7 +13221,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="27" t="s">
         <v>1278</v>
       </c>
@@ -13250,7 +13250,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="27" t="s">
         <v>1281</v>
       </c>
@@ -13279,7 +13279,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="27" t="s">
         <v>1284</v>
       </c>
@@ -13308,7 +13308,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="27" t="s">
         <v>1287</v>
       </c>
@@ -13337,7 +13337,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="27" t="s">
         <v>1290</v>
       </c>

</xml_diff>